<commit_message>
Add Thai mutual-fund NAVs via SEC Thailand Open API
- pipeline/fetch_thai_nav.py: Fund Factsheet (abbr->proj_id, cached) + Fund Daily
  Info (dailynav last_val); exact+punctuation-insensitive matching; 8-day NAV
  walk-back; graceful carry-forward when keys unset or fund unmatched
- fetch_prices.py: prices Thai MFs from SEC with real NAV date; only unmatched carry fwd
- weekly.yml: SEC_FUND_FACTSHEET_KEY / SEC_FUND_DAILY_INFO_KEY via Actions secrets
- README: SEC subscription + setup docs

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -14241,13 +14241,13 @@
         <v>46172</v>
       </c>
       <c r="C6" s="75" t="n">
-        <v>23446173</v>
+        <v>23445398</v>
       </c>
       <c r="D6" s="75" t="n">
         <v>19595542</v>
       </c>
       <c r="E6" s="75" t="n">
-        <v>3850630</v>
+        <v>3849855</v>
       </c>
       <c r="F6" s="76" t="n">
         <v>0.1965</v>
@@ -14259,7 +14259,7 @@
         <v>2859438</v>
       </c>
       <c r="I6" s="75" t="n">
-        <v>1317330</v>
+        <v>1316555</v>
       </c>
       <c r="J6" s="77" t="n">
         <v>32.43</v>
@@ -18233,7 +18233,7 @@
         </is>
       </c>
       <c r="E73" s="41" t="n">
-        <v>82.7</v>
+        <v>82.81</v>
       </c>
       <c r="F73" s="42" t="inlineStr">
         <is>
@@ -18270,7 +18270,7 @@
         </is>
       </c>
       <c r="E74" s="41" t="n">
-        <v>673.88</v>
+        <v>672.33</v>
       </c>
       <c r="F74" s="42" t="inlineStr">
         <is>
@@ -18307,7 +18307,7 @@
         </is>
       </c>
       <c r="E75" s="41" t="n">
-        <v>73532</v>
+        <v>73502</v>
       </c>
       <c r="F75" s="42" t="inlineStr">
         <is>
@@ -18344,7 +18344,7 @@
         </is>
       </c>
       <c r="E76" s="41" t="n">
-        <v>0.008004000000000001</v>
+        <v>0.008047</v>
       </c>
       <c r="F76" s="42" t="inlineStr">
         <is>
@@ -18381,7 +18381,7 @@
         </is>
       </c>
       <c r="E77" s="41" t="n">
-        <v>0.012855</v>
+        <v>0.012723</v>
       </c>
       <c r="F77" s="42" t="inlineStr">
         <is>
@@ -18418,7 +18418,7 @@
         </is>
       </c>
       <c r="E78" s="41" t="n">
-        <v>82.28</v>
+        <v>82.27</v>
       </c>
       <c r="F78" s="42" t="inlineStr">
         <is>
@@ -18529,7 +18529,7 @@
         </is>
       </c>
       <c r="E81" s="41" t="n">
-        <v>0.016095</v>
+        <v>0.016008</v>
       </c>
       <c r="F81" s="42" t="inlineStr">
         <is>
@@ -18566,7 +18566,7 @@
         </is>
       </c>
       <c r="E82" s="41" t="n">
-        <v>3.386081</v>
+        <v>3.392243</v>
       </c>
       <c r="F82" s="42" t="inlineStr">
         <is>
@@ -18603,7 +18603,7 @@
         </is>
       </c>
       <c r="E83" s="41" t="n">
-        <v>29.121297</v>
+        <v>29.098628</v>
       </c>
       <c r="F83" s="42" t="inlineStr">
         <is>
@@ -18640,7 +18640,7 @@
         </is>
       </c>
       <c r="E84" s="41" t="n">
-        <v>0.138974</v>
+        <v>0.139166</v>
       </c>
       <c r="F84" s="42" t="inlineStr">
         <is>
@@ -18677,7 +18677,7 @@
         </is>
       </c>
       <c r="E85" s="41" t="n">
-        <v>21853.9284</v>
+        <v>21803.6619</v>
       </c>
       <c r="F85" s="42" t="inlineStr">
         <is>
@@ -18714,7 +18714,7 @@
         </is>
       </c>
       <c r="E86" s="41" t="n">
-        <v>2384642.76</v>
+        <v>2383669.86</v>
       </c>
       <c r="F86" s="42" t="inlineStr">
         <is>
@@ -18751,7 +18751,7 @@
         </is>
       </c>
       <c r="E87" s="41" t="n">
-        <v>3.265117</v>
+        <v>3.267744</v>
       </c>
       <c r="F87" s="42" t="inlineStr">
         <is>
@@ -18788,7 +18788,7 @@
         </is>
       </c>
       <c r="E88" s="41" t="n">
-        <v>65340.9369</v>
+        <v>65340.2883</v>
       </c>
       <c r="F88" s="42" t="inlineStr">
         <is>
@@ -18825,7 +18825,7 @@
         </is>
       </c>
       <c r="E89" s="41" t="n">
-        <v>25.988235</v>
+        <v>25.981392</v>
       </c>
       <c r="F89" s="42" t="inlineStr">
         <is>
@@ -18862,7 +18862,7 @@
         </is>
       </c>
       <c r="E90" s="41" t="n">
-        <v>73532</v>
+        <v>73502</v>
       </c>
       <c r="F90" s="42" t="inlineStr">
         <is>
@@ -18899,7 +18899,7 @@
         </is>
       </c>
       <c r="E91" s="41" t="n">
-        <v>18.48</v>
+        <v>18.59</v>
       </c>
       <c r="F91" s="42" t="inlineStr">
         <is>
@@ -19010,7 +19010,7 @@
         </is>
       </c>
       <c r="E94" s="41" t="n">
-        <v>0.008004000000000001</v>
+        <v>0.008047</v>
       </c>
       <c r="F94" s="42" t="inlineStr">
         <is>
@@ -19047,7 +19047,7 @@
         </is>
       </c>
       <c r="E95" s="41" t="n">
-        <v>82.28</v>
+        <v>82.27</v>
       </c>
       <c r="F95" s="42" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Weekly dashboard rebuild — 2026-05-30 (SEC NAVs live)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -14241,25 +14241,25 @@
         <v>46172</v>
       </c>
       <c r="C6" s="75" t="n">
-        <v>23445398</v>
+        <v>23462387</v>
       </c>
       <c r="D6" s="75" t="n">
         <v>19595542</v>
       </c>
       <c r="E6" s="75" t="n">
-        <v>3849855</v>
+        <v>3866844</v>
       </c>
       <c r="F6" s="76" t="n">
-        <v>0.1965</v>
+        <v>0.1973</v>
       </c>
       <c r="G6" s="75" t="n">
-        <v>19269405</v>
+        <v>19269313</v>
       </c>
       <c r="H6" s="75" t="n">
         <v>2859438</v>
       </c>
       <c r="I6" s="75" t="n">
-        <v>1316555</v>
+        <v>1333636</v>
       </c>
       <c r="J6" s="77" t="n">
         <v>32.43</v>
@@ -18233,7 +18233,7 @@
         </is>
       </c>
       <c r="E73" s="41" t="n">
-        <v>82.94</v>
+        <v>83.08</v>
       </c>
       <c r="F73" s="42" t="inlineStr">
         <is>
@@ -18270,7 +18270,7 @@
         </is>
       </c>
       <c r="E74" s="41" t="n">
-        <v>694.91</v>
+        <v>704.77</v>
       </c>
       <c r="F74" s="42" t="inlineStr">
         <is>
@@ -18307,7 +18307,7 @@
         </is>
       </c>
       <c r="E75" s="41" t="n">
-        <v>73803</v>
+        <v>73855</v>
       </c>
       <c r="F75" s="42" t="inlineStr">
         <is>
@@ -18344,7 +18344,7 @@
         </is>
       </c>
       <c r="E76" s="41" t="n">
-        <v>0.008011000000000001</v>
+        <v>0.008023000000000001</v>
       </c>
       <c r="F76" s="42" t="inlineStr">
         <is>
@@ -18381,7 +18381,7 @@
         </is>
       </c>
       <c r="E77" s="41" t="n">
-        <v>0.012743</v>
+        <v>0.01268</v>
       </c>
       <c r="F77" s="42" t="inlineStr">
         <is>
@@ -18418,7 +18418,7 @@
         </is>
       </c>
       <c r="E78" s="41" t="n">
-        <v>82.55</v>
+        <v>82.75</v>
       </c>
       <c r="F78" s="42" t="inlineStr">
         <is>
@@ -18455,7 +18455,7 @@
         </is>
       </c>
       <c r="E79" s="41" t="n">
-        <v>2</v>
+        <v>2.01</v>
       </c>
       <c r="F79" s="42" t="inlineStr">
         <is>
@@ -18529,7 +18529,7 @@
         </is>
       </c>
       <c r="E81" s="41" t="n">
-        <v>0.016139</v>
+        <v>0.016161</v>
       </c>
       <c r="F81" s="42" t="inlineStr">
         <is>
@@ -18566,7 +18566,7 @@
         </is>
       </c>
       <c r="E82" s="41" t="n">
-        <v>3.397529</v>
+        <v>3.408393</v>
       </c>
       <c r="F82" s="42" t="inlineStr">
         <is>
@@ -18603,7 +18603,7 @@
         </is>
       </c>
       <c r="E83" s="41" t="n">
-        <v>29.439143</v>
+        <v>29.520186</v>
       </c>
       <c r="F83" s="42" t="inlineStr">
         <is>
@@ -18640,7 +18640,7 @@
         </is>
       </c>
       <c r="E84" s="41" t="n">
-        <v>0.136593</v>
+        <v>0.135964</v>
       </c>
       <c r="F84" s="42" t="inlineStr">
         <is>
@@ -18677,7 +18677,7 @@
         </is>
       </c>
       <c r="E85" s="41" t="n">
-        <v>22535.9313</v>
+        <v>22855.6911</v>
       </c>
       <c r="F85" s="42" t="inlineStr">
         <is>
@@ -18714,7 +18714,7 @@
         </is>
       </c>
       <c r="E86" s="41" t="n">
-        <v>2393431.29</v>
+        <v>2395117.65</v>
       </c>
       <c r="F86" s="42" t="inlineStr">
         <is>
@@ -18751,7 +18751,7 @@
         </is>
       </c>
       <c r="E87" s="41" t="n">
-        <v>3.283408</v>
+        <v>3.288434</v>
       </c>
       <c r="F87" s="42" t="inlineStr">
         <is>
@@ -18788,7 +18788,7 @@
         </is>
       </c>
       <c r="E88" s="41" t="n">
-        <v>65597.45819999999</v>
+        <v>65654.535</v>
       </c>
       <c r="F88" s="42" t="inlineStr">
         <is>
@@ -18825,7 +18825,7 @@
         </is>
       </c>
       <c r="E89" s="41" t="n">
-        <v>26.150417</v>
+        <v>26.067007</v>
       </c>
       <c r="F89" s="42" t="inlineStr">
         <is>
@@ -18862,7 +18862,7 @@
         </is>
       </c>
       <c r="E90" s="41" t="n">
-        <v>73803</v>
+        <v>73855</v>
       </c>
       <c r="F90" s="42" t="inlineStr">
         <is>
@@ -18899,7 +18899,7 @@
         </is>
       </c>
       <c r="E91" s="41" t="n">
-        <v>18.33</v>
+        <v>18.53</v>
       </c>
       <c r="F91" s="42" t="inlineStr">
         <is>
@@ -19010,7 +19010,7 @@
         </is>
       </c>
       <c r="E94" s="41" t="n">
-        <v>0.008011000000000001</v>
+        <v>0.008023000000000001</v>
       </c>
       <c r="F94" s="42" t="inlineStr">
         <is>
@@ -19047,7 +19047,7 @@
         </is>
       </c>
       <c r="E95" s="41" t="n">
-        <v>82.55</v>
+        <v>82.75</v>
       </c>
       <c r="F95" s="42" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
v2 dashboard: clean institutional tabbed redesign
Major overhaul, promoted from the approved design prototype:
- 5 tabs: Overview · Allocation · Holdings · Performance · Risk
- clean institutional light system: tabular numerals, neutral grays, single green accent
- Overview: KPIs with week-over-week deltas + sparklines, allocation ribbon, top movers
- Holdings: searchable / sortable / filterable dense table (all positions)
- Risk: single-name concentration, top-5/10 weight, effective holdings (1/HHI),
  currency exposure (THB vs USD), risk-posture band
- Performance/WoW use REAL accumulating Weekly Snapshot history; graceful
  'history is building' state until a 2nd weekly point exists
- configurable logo_text; mobile-responsive (scrollable tabs, single-col KPIs)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -14271,16 +14271,38 @@
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="54">
-      <c r="B7" s="74" t="n"/>
-      <c r="C7" s="75" t="n"/>
-      <c r="D7" s="75" t="n"/>
-      <c r="E7" s="75" t="n"/>
-      <c r="F7" s="76" t="n"/>
-      <c r="G7" s="75" t="n"/>
-      <c r="H7" s="75" t="n"/>
-      <c r="I7" s="75" t="n"/>
-      <c r="J7" s="77" t="n"/>
-      <c r="K7" s="40" t="n"/>
+      <c r="B7" s="74" t="n">
+        <v>46173</v>
+      </c>
+      <c r="C7" s="75" t="n">
+        <v>23470248</v>
+      </c>
+      <c r="D7" s="75" t="n">
+        <v>19595542</v>
+      </c>
+      <c r="E7" s="75" t="n">
+        <v>3874706</v>
+      </c>
+      <c r="F7" s="76" t="n">
+        <v>0.1977</v>
+      </c>
+      <c r="G7" s="75" t="n">
+        <v>19269313</v>
+      </c>
+      <c r="H7" s="75" t="n">
+        <v>2859438</v>
+      </c>
+      <c r="I7" s="75" t="n">
+        <v>1341497</v>
+      </c>
+      <c r="J7" s="77" t="n">
+        <v>32.43</v>
+      </c>
+      <c r="K7" s="40" t="inlineStr">
+        <is>
+          <t>Auto weekly snapshot</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="54">
       <c r="B8" s="74" t="n"/>
@@ -15562,7 +15584,7 @@
         </is>
       </c>
       <c r="C5" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="D5" s="32" t="inlineStr">
         <is>
@@ -15581,7 +15603,7 @@
       </c>
       <c r="D6" s="32" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-05-30</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-05-31</t>
         </is>
       </c>
     </row>
@@ -16909,7 +16931,7 @@
         </is>
       </c>
       <c r="G37" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H37" s="42" t="inlineStr">
         <is>
@@ -16946,7 +16968,7 @@
         </is>
       </c>
       <c r="G38" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H38" s="42" t="inlineStr">
         <is>
@@ -16983,7 +17005,7 @@
         </is>
       </c>
       <c r="G39" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H39" s="42" t="inlineStr">
         <is>
@@ -17020,7 +17042,7 @@
         </is>
       </c>
       <c r="G40" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H40" s="42" t="inlineStr">
         <is>
@@ -17094,7 +17116,7 @@
         </is>
       </c>
       <c r="G42" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H42" s="42" t="inlineStr">
         <is>
@@ -17131,7 +17153,7 @@
         </is>
       </c>
       <c r="G43" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H43" s="42" t="inlineStr">
         <is>
@@ -17168,7 +17190,7 @@
         </is>
       </c>
       <c r="G44" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H44" s="42" t="inlineStr">
         <is>
@@ -17205,7 +17227,7 @@
         </is>
       </c>
       <c r="G45" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H45" s="42" t="inlineStr">
         <is>
@@ -17242,7 +17264,7 @@
         </is>
       </c>
       <c r="G46" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H46" s="42" t="inlineStr">
         <is>
@@ -17279,7 +17301,7 @@
         </is>
       </c>
       <c r="G47" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H47" s="42" t="inlineStr">
         <is>
@@ -17316,7 +17338,7 @@
         </is>
       </c>
       <c r="G48" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H48" s="42" t="inlineStr">
         <is>
@@ -17353,7 +17375,7 @@
         </is>
       </c>
       <c r="G49" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H49" s="42" t="inlineStr">
         <is>
@@ -17390,7 +17412,7 @@
         </is>
       </c>
       <c r="G50" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H50" s="42" t="inlineStr">
         <is>
@@ -17427,7 +17449,7 @@
         </is>
       </c>
       <c r="G51" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H51" s="42" t="inlineStr">
         <is>
@@ -17464,7 +17486,7 @@
         </is>
       </c>
       <c r="G52" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H52" s="42" t="inlineStr">
         <is>
@@ -17501,7 +17523,7 @@
         </is>
       </c>
       <c r="G53" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H53" s="42" t="inlineStr">
         <is>
@@ -17538,7 +17560,7 @@
         </is>
       </c>
       <c r="G54" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H54" s="42" t="inlineStr">
         <is>
@@ -17575,7 +17597,7 @@
         </is>
       </c>
       <c r="G55" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H55" s="42" t="inlineStr">
         <is>
@@ -17612,7 +17634,7 @@
         </is>
       </c>
       <c r="G56" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H56" s="42" t="inlineStr">
         <is>
@@ -17649,7 +17671,7 @@
         </is>
       </c>
       <c r="G57" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H57" s="42" t="inlineStr">
         <is>
@@ -17686,7 +17708,7 @@
         </is>
       </c>
       <c r="G58" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H58" s="42" t="inlineStr">
         <is>
@@ -17723,7 +17745,7 @@
         </is>
       </c>
       <c r="G59" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H59" s="42" t="inlineStr">
         <is>
@@ -17760,7 +17782,7 @@
         </is>
       </c>
       <c r="G60" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H60" s="42" t="inlineStr">
         <is>
@@ -17797,7 +17819,7 @@
         </is>
       </c>
       <c r="G61" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H61" s="42" t="inlineStr">
         <is>
@@ -17834,7 +17856,7 @@
         </is>
       </c>
       <c r="G62" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H62" s="42" t="inlineStr">
         <is>
@@ -17871,7 +17893,7 @@
         </is>
       </c>
       <c r="G63" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H63" s="42" t="inlineStr">
         <is>
@@ -17908,7 +17930,7 @@
         </is>
       </c>
       <c r="G64" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H64" s="42" t="inlineStr">
         <is>
@@ -17945,7 +17967,7 @@
         </is>
       </c>
       <c r="G65" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H65" s="42" t="inlineStr">
         <is>
@@ -17982,7 +18004,7 @@
         </is>
       </c>
       <c r="G66" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H66" s="42" t="inlineStr">
         <is>
@@ -18019,7 +18041,7 @@
         </is>
       </c>
       <c r="G67" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H67" s="42" t="inlineStr">
         <is>
@@ -18056,7 +18078,7 @@
         </is>
       </c>
       <c r="G68" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H68" s="42" t="inlineStr">
         <is>
@@ -18093,7 +18115,7 @@
         </is>
       </c>
       <c r="G69" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H69" s="42" t="inlineStr">
         <is>
@@ -18130,7 +18152,7 @@
         </is>
       </c>
       <c r="G70" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H70" s="42" t="inlineStr">
         <is>
@@ -18167,7 +18189,7 @@
         </is>
       </c>
       <c r="G71" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H71" s="42" t="inlineStr">
         <is>
@@ -18204,7 +18226,7 @@
         </is>
       </c>
       <c r="G72" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H72" s="42" t="inlineStr">
         <is>
@@ -18233,7 +18255,7 @@
         </is>
       </c>
       <c r="E73" s="41" t="n">
-        <v>83.08</v>
+        <v>82.70999999999999</v>
       </c>
       <c r="F73" s="42" t="inlineStr">
         <is>
@@ -18241,7 +18263,7 @@
         </is>
       </c>
       <c r="G73" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H73" s="42" t="inlineStr">
         <is>
@@ -18270,7 +18292,7 @@
         </is>
       </c>
       <c r="E74" s="41" t="n">
-        <v>704.77</v>
+        <v>722.79</v>
       </c>
       <c r="F74" s="42" t="inlineStr">
         <is>
@@ -18278,7 +18300,7 @@
         </is>
       </c>
       <c r="G74" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H74" s="42" t="inlineStr">
         <is>
@@ -18307,7 +18329,7 @@
         </is>
       </c>
       <c r="E75" s="41" t="n">
-        <v>73855</v>
+        <v>73920</v>
       </c>
       <c r="F75" s="42" t="inlineStr">
         <is>
@@ -18315,7 +18337,7 @@
         </is>
       </c>
       <c r="G75" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H75" s="42" t="inlineStr">
         <is>
@@ -18344,7 +18366,7 @@
         </is>
       </c>
       <c r="E76" s="41" t="n">
-        <v>0.008023000000000001</v>
+        <v>0.007985000000000001</v>
       </c>
       <c r="F76" s="42" t="inlineStr">
         <is>
@@ -18352,7 +18374,7 @@
         </is>
       </c>
       <c r="G76" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H76" s="42" t="inlineStr">
         <is>
@@ -18381,7 +18403,7 @@
         </is>
       </c>
       <c r="E77" s="41" t="n">
-        <v>0.01268</v>
+        <v>0.013265</v>
       </c>
       <c r="F77" s="42" t="inlineStr">
         <is>
@@ -18389,7 +18411,7 @@
         </is>
       </c>
       <c r="G77" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H77" s="42" t="inlineStr">
         <is>
@@ -18418,7 +18440,7 @@
         </is>
       </c>
       <c r="E78" s="41" t="n">
-        <v>82.75</v>
+        <v>82.8</v>
       </c>
       <c r="F78" s="42" t="inlineStr">
         <is>
@@ -18426,7 +18448,7 @@
         </is>
       </c>
       <c r="G78" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H78" s="42" t="inlineStr">
         <is>
@@ -18455,7 +18477,7 @@
         </is>
       </c>
       <c r="E79" s="41" t="n">
-        <v>2.01</v>
+        <v>1.99</v>
       </c>
       <c r="F79" s="42" t="inlineStr">
         <is>
@@ -18463,7 +18485,7 @@
         </is>
       </c>
       <c r="G79" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H79" s="42" t="inlineStr">
         <is>
@@ -18500,7 +18522,7 @@
         </is>
       </c>
       <c r="G80" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H80" s="42" t="inlineStr">
         <is>
@@ -18529,7 +18551,7 @@
         </is>
       </c>
       <c r="E81" s="41" t="n">
-        <v>0.016161</v>
+        <v>0.016039</v>
       </c>
       <c r="F81" s="42" t="inlineStr">
         <is>
@@ -18537,7 +18559,7 @@
         </is>
       </c>
       <c r="G81" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H81" s="42" t="inlineStr">
         <is>
@@ -18566,7 +18588,7 @@
         </is>
       </c>
       <c r="E82" s="41" t="n">
-        <v>3.408393</v>
+        <v>3.367077</v>
       </c>
       <c r="F82" s="42" t="inlineStr">
         <is>
@@ -18574,7 +18596,7 @@
         </is>
       </c>
       <c r="G82" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H82" s="42" t="inlineStr">
         <is>
@@ -18603,7 +18625,7 @@
         </is>
       </c>
       <c r="E83" s="41" t="n">
-        <v>29.520186</v>
+        <v>29.579695</v>
       </c>
       <c r="F83" s="42" t="inlineStr">
         <is>
@@ -18611,7 +18633,7 @@
         </is>
       </c>
       <c r="G83" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H83" s="42" t="inlineStr">
         <is>
@@ -18640,7 +18662,7 @@
         </is>
       </c>
       <c r="E84" s="41" t="n">
-        <v>0.135964</v>
+        <v>0.13623</v>
       </c>
       <c r="F84" s="42" t="inlineStr">
         <is>
@@ -18648,7 +18670,7 @@
         </is>
       </c>
       <c r="G84" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H84" s="42" t="inlineStr">
         <is>
@@ -18677,7 +18699,7 @@
         </is>
       </c>
       <c r="E85" s="41" t="n">
-        <v>22855.6911</v>
+        <v>23440.0797</v>
       </c>
       <c r="F85" s="42" t="inlineStr">
         <is>
@@ -18685,7 +18707,7 @@
         </is>
       </c>
       <c r="G85" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H85" s="42" t="inlineStr">
         <is>
@@ -18714,7 +18736,7 @@
         </is>
       </c>
       <c r="E86" s="41" t="n">
-        <v>2395117.65</v>
+        <v>2397225.6</v>
       </c>
       <c r="F86" s="42" t="inlineStr">
         <is>
@@ -18722,7 +18744,7 @@
         </is>
       </c>
       <c r="G86" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H86" s="42" t="inlineStr">
         <is>
@@ -18751,7 +18773,7 @@
         </is>
       </c>
       <c r="E87" s="41" t="n">
-        <v>3.288434</v>
+        <v>3.263658</v>
       </c>
       <c r="F87" s="42" t="inlineStr">
         <is>
@@ -18759,7 +18781,7 @@
         </is>
       </c>
       <c r="G87" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H87" s="42" t="inlineStr">
         <is>
@@ -18788,7 +18810,7 @@
         </is>
       </c>
       <c r="E88" s="41" t="n">
-        <v>65654.535</v>
+        <v>65637.3471</v>
       </c>
       <c r="F88" s="42" t="inlineStr">
         <is>
@@ -18796,7 +18818,7 @@
         </is>
       </c>
       <c r="G88" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H88" s="42" t="inlineStr">
         <is>
@@ -18825,7 +18847,7 @@
         </is>
       </c>
       <c r="E89" s="41" t="n">
-        <v>26.067007</v>
+        <v>26.188425</v>
       </c>
       <c r="F89" s="42" t="inlineStr">
         <is>
@@ -18833,7 +18855,7 @@
         </is>
       </c>
       <c r="G89" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H89" s="42" t="inlineStr">
         <is>
@@ -18862,7 +18884,7 @@
         </is>
       </c>
       <c r="E90" s="41" t="n">
-        <v>73855</v>
+        <v>73920</v>
       </c>
       <c r="F90" s="42" t="inlineStr">
         <is>
@@ -18870,7 +18892,7 @@
         </is>
       </c>
       <c r="G90" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H90" s="42" t="inlineStr">
         <is>
@@ -18899,7 +18921,7 @@
         </is>
       </c>
       <c r="E91" s="41" t="n">
-        <v>18.53</v>
+        <v>18.24</v>
       </c>
       <c r="F91" s="42" t="inlineStr">
         <is>
@@ -18907,7 +18929,7 @@
         </is>
       </c>
       <c r="G91" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H91" s="42" t="inlineStr">
         <is>
@@ -19010,7 +19032,7 @@
         </is>
       </c>
       <c r="E94" s="41" t="n">
-        <v>0.008023000000000001</v>
+        <v>0.007985000000000001</v>
       </c>
       <c r="F94" s="42" t="inlineStr">
         <is>
@@ -19018,7 +19040,7 @@
         </is>
       </c>
       <c r="G94" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H94" s="42" t="inlineStr">
         <is>
@@ -19047,7 +19069,7 @@
         </is>
       </c>
       <c r="E95" s="41" t="n">
-        <v>82.75</v>
+        <v>82.8</v>
       </c>
       <c r="F95" s="42" t="inlineStr">
         <is>
@@ -19055,7 +19077,7 @@
         </is>
       </c>
       <c r="G95" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H95" s="42" t="inlineStr">
         <is>
@@ -19092,7 +19114,7 @@
         </is>
       </c>
       <c r="G96" s="74" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="H96" s="42" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Fix Thai fund share-class pins (NAV accuracy)
User cross-checked SCBKEQTG against the SCBAM website: NAV 28.2028 (28 May,
accumulation class), but it was pinned to class SCBKEQTGE (28.7313) because the
workbook's original NAV matched that class. The original workbook NAVs were
entered for the wrong share class on 5 funds. Re-pinned each to the class whose
name exactly matches the workbook label, verified vs SEC /v2/fund:
  SCBKEQTG    SCBKEQTGE  -> SCBKEQTG     (28.2028, matches website)
  K-USA-A(D)  K-USA-SSF  -> K-USA-A(D)   (12.1230)
  SCBSEMI(A)  SCBSEMI(SSF)-> SCBSEMI(A)  (37.6341)
  SCBTAPX(25D) SCBTAPX(LTFA)-> SCBTAPX(25D)(12.4460)
  UOBSG-N     UOBSG-D    -> UOBSG-N      (29.0432)
Net portfolio impact -243k -> total now THB 23,227,220 (+18.5%).
Reset the brief test history so the chart shows no artificial dip.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -14237,72 +14237,28 @@
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="54">
-      <c r="B6" s="74" t="n">
-        <v>46172</v>
-      </c>
-      <c r="C6" s="75" t="n">
-        <v>23462387</v>
-      </c>
-      <c r="D6" s="75" t="n">
-        <v>19595542</v>
-      </c>
-      <c r="E6" s="75" t="n">
-        <v>3866844</v>
-      </c>
-      <c r="F6" s="76" t="n">
-        <v>0.1973</v>
-      </c>
-      <c r="G6" s="75" t="n">
-        <v>19269313</v>
-      </c>
-      <c r="H6" s="75" t="n">
-        <v>2859438</v>
-      </c>
-      <c r="I6" s="75" t="n">
-        <v>1333636</v>
-      </c>
-      <c r="J6" s="77" t="n">
-        <v>32.43</v>
-      </c>
-      <c r="K6" s="40" t="inlineStr">
-        <is>
-          <t>Auto weekly snapshot</t>
-        </is>
-      </c>
+      <c r="B6" s="74" t="n"/>
+      <c r="C6" s="75" t="n"/>
+      <c r="D6" s="75" t="n"/>
+      <c r="E6" s="75" t="n"/>
+      <c r="F6" s="76" t="n"/>
+      <c r="G6" s="75" t="n"/>
+      <c r="H6" s="75" t="n"/>
+      <c r="I6" s="75" t="n"/>
+      <c r="J6" s="77" t="n"/>
+      <c r="K6" s="40" t="n"/>
     </row>
     <row r="7" ht="15" customHeight="1" s="54">
-      <c r="B7" s="74" t="n">
-        <v>46173</v>
-      </c>
-      <c r="C7" s="75" t="n">
-        <v>23470248</v>
-      </c>
-      <c r="D7" s="75" t="n">
-        <v>19595542</v>
-      </c>
-      <c r="E7" s="75" t="n">
-        <v>3874706</v>
-      </c>
-      <c r="F7" s="76" t="n">
-        <v>0.1977</v>
-      </c>
-      <c r="G7" s="75" t="n">
-        <v>19269313</v>
-      </c>
-      <c r="H7" s="75" t="n">
-        <v>2859438</v>
-      </c>
-      <c r="I7" s="75" t="n">
-        <v>1341497</v>
-      </c>
-      <c r="J7" s="77" t="n">
-        <v>32.43</v>
-      </c>
-      <c r="K7" s="40" t="inlineStr">
-        <is>
-          <t>Auto weekly snapshot</t>
-        </is>
-      </c>
+      <c r="B7" s="74" t="n"/>
+      <c r="C7" s="75" t="n"/>
+      <c r="D7" s="75" t="n"/>
+      <c r="E7" s="75" t="n"/>
+      <c r="F7" s="76" t="n"/>
+      <c r="G7" s="75" t="n"/>
+      <c r="H7" s="75" t="n"/>
+      <c r="I7" s="75" t="n"/>
+      <c r="J7" s="77" t="n"/>
+      <c r="K7" s="40" t="n"/>
     </row>
     <row r="8" ht="15" customHeight="1" s="54">
       <c r="B8" s="74" t="n"/>
@@ -15739,7 +15695,7 @@
         </is>
       </c>
       <c r="E5" s="41" t="n">
-        <v>24.8415</v>
+        <v>25.0666</v>
       </c>
       <c r="F5" s="42" t="inlineStr">
         <is>
@@ -15747,7 +15703,7 @@
         </is>
       </c>
       <c r="G5" s="74" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="H5" s="42" t="inlineStr">
         <is>
@@ -15776,7 +15732,7 @@
         </is>
       </c>
       <c r="E6" s="41" t="n">
-        <v>10.6846</v>
+        <v>10.6848</v>
       </c>
       <c r="F6" s="42" t="inlineStr">
         <is>
@@ -15784,7 +15740,7 @@
         </is>
       </c>
       <c r="G6" s="74" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="H6" s="42" t="inlineStr">
         <is>
@@ -15813,7 +15769,7 @@
         </is>
       </c>
       <c r="E7" s="41" t="n">
-        <v>7.2284</v>
+        <v>7.1689</v>
       </c>
       <c r="F7" s="42" t="inlineStr">
         <is>
@@ -15821,7 +15777,7 @@
         </is>
       </c>
       <c r="G7" s="74" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="H7" s="42" t="inlineStr">
         <is>
@@ -15850,7 +15806,7 @@
         </is>
       </c>
       <c r="E8" s="41" t="n">
-        <v>9.7121</v>
+        <v>9.7524</v>
       </c>
       <c r="F8" s="42" t="inlineStr">
         <is>
@@ -15858,7 +15814,7 @@
         </is>
       </c>
       <c r="G8" s="74" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="H8" s="42" t="inlineStr">
         <is>
@@ -15887,7 +15843,7 @@
         </is>
       </c>
       <c r="E9" s="41" t="n">
-        <v>9.3271</v>
+        <v>9.3216</v>
       </c>
       <c r="F9" s="42" t="inlineStr">
         <is>
@@ -15895,7 +15851,7 @@
         </is>
       </c>
       <c r="G9" s="74" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="H9" s="42" t="inlineStr">
         <is>
@@ -15924,7 +15880,7 @@
         </is>
       </c>
       <c r="E10" s="41" t="n">
-        <v>13.3005</v>
+        <v>13.2248</v>
       </c>
       <c r="F10" s="42" t="inlineStr">
         <is>
@@ -15932,7 +15888,7 @@
         </is>
       </c>
       <c r="G10" s="74" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="H10" s="42" t="inlineStr">
         <is>
@@ -15961,7 +15917,7 @@
         </is>
       </c>
       <c r="E11" s="41" t="n">
-        <v>13.0648</v>
+        <v>13.0748</v>
       </c>
       <c r="F11" s="42" t="inlineStr">
         <is>
@@ -15969,7 +15925,7 @@
         </is>
       </c>
       <c r="G11" s="74" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="H11" s="42" t="inlineStr">
         <is>
@@ -15998,7 +15954,7 @@
         </is>
       </c>
       <c r="E12" s="41" t="n">
-        <v>26.2958</v>
+        <v>26.4159</v>
       </c>
       <c r="F12" s="42" t="inlineStr">
         <is>
@@ -16006,7 +15962,7 @@
         </is>
       </c>
       <c r="G12" s="74" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="H12" s="42" t="inlineStr">
         <is>
@@ -16035,7 +15991,7 @@
         </is>
       </c>
       <c r="E13" s="41" t="n">
-        <v>35.9715</v>
+        <v>35.9236</v>
       </c>
       <c r="F13" s="42" t="inlineStr">
         <is>
@@ -16043,7 +15999,7 @@
         </is>
       </c>
       <c r="G13" s="74" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="H13" s="42" t="inlineStr">
         <is>
@@ -16072,7 +16028,7 @@
         </is>
       </c>
       <c r="E14" s="41" t="n">
-        <v>25.2468</v>
+        <v>25.2351</v>
       </c>
       <c r="F14" s="42" t="inlineStr">
         <is>
@@ -16080,7 +16036,7 @@
         </is>
       </c>
       <c r="G14" s="74" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="H14" s="42" t="inlineStr">
         <is>
@@ -16109,7 +16065,7 @@
         </is>
       </c>
       <c r="E15" s="41" t="n">
-        <v>14.8272</v>
+        <v>14.8144</v>
       </c>
       <c r="F15" s="42" t="inlineStr">
         <is>
@@ -16117,7 +16073,7 @@
         </is>
       </c>
       <c r="G15" s="74" t="n">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="H15" s="42" t="inlineStr">
         <is>
@@ -16146,7 +16102,7 @@
         </is>
       </c>
       <c r="E16" s="41" t="n">
-        <v>80.66759999999999</v>
+        <v>80.6575</v>
       </c>
       <c r="F16" s="42" t="inlineStr">
         <is>
@@ -16154,7 +16110,7 @@
         </is>
       </c>
       <c r="G16" s="74" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="H16" s="42" t="inlineStr">
         <is>
@@ -16183,7 +16139,7 @@
         </is>
       </c>
       <c r="E17" s="41" t="n">
-        <v>52.8982</v>
+        <v>52.9188</v>
       </c>
       <c r="F17" s="42" t="inlineStr">
         <is>
@@ -16191,7 +16147,7 @@
         </is>
       </c>
       <c r="G17" s="74" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="H17" s="42" t="inlineStr">
         <is>
@@ -16220,7 +16176,7 @@
         </is>
       </c>
       <c r="E18" s="41" t="n">
-        <v>16.3952</v>
+        <v>16.418</v>
       </c>
       <c r="F18" s="42" t="inlineStr">
         <is>
@@ -16228,7 +16184,7 @@
         </is>
       </c>
       <c r="G18" s="74" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="H18" s="42" t="inlineStr">
         <is>
@@ -16257,7 +16213,7 @@
         </is>
       </c>
       <c r="E19" s="41" t="n">
-        <v>23.3976</v>
+        <v>23.3983</v>
       </c>
       <c r="F19" s="42" t="inlineStr">
         <is>
@@ -16265,7 +16221,7 @@
         </is>
       </c>
       <c r="G19" s="74" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="H19" s="42" t="inlineStr">
         <is>
@@ -16294,7 +16250,7 @@
         </is>
       </c>
       <c r="E20" s="41" t="n">
-        <v>41.3279</v>
+        <v>41.5536</v>
       </c>
       <c r="F20" s="42" t="inlineStr">
         <is>
@@ -16302,7 +16258,7 @@
         </is>
       </c>
       <c r="G20" s="74" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="H20" s="42" t="inlineStr">
         <is>
@@ -16331,7 +16287,7 @@
         </is>
       </c>
       <c r="E21" s="41" t="n">
-        <v>13.6222</v>
+        <v>13.3525</v>
       </c>
       <c r="F21" s="42" t="inlineStr">
         <is>
@@ -16339,7 +16295,7 @@
         </is>
       </c>
       <c r="G21" s="74" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="H21" s="42" t="inlineStr">
         <is>
@@ -16368,7 +16324,7 @@
         </is>
       </c>
       <c r="E22" s="41" t="n">
-        <v>13.0596</v>
+        <v>13.1196</v>
       </c>
       <c r="F22" s="42" t="inlineStr">
         <is>
@@ -16376,7 +16332,7 @@
         </is>
       </c>
       <c r="G22" s="74" t="n">
-        <v>46168</v>
+        <v>46170</v>
       </c>
       <c r="H22" s="42" t="inlineStr">
         <is>
@@ -16405,7 +16361,7 @@
         </is>
       </c>
       <c r="E23" s="41" t="n">
-        <v>12.2836</v>
+        <v>12.2892</v>
       </c>
       <c r="F23" s="42" t="inlineStr">
         <is>
@@ -16413,7 +16369,7 @@
         </is>
       </c>
       <c r="G23" s="74" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="H23" s="42" t="inlineStr">
         <is>
@@ -16442,7 +16398,7 @@
         </is>
       </c>
       <c r="E24" s="41" t="n">
-        <v>16.3863</v>
+        <v>12.123</v>
       </c>
       <c r="F24" s="42" t="inlineStr">
         <is>
@@ -16450,7 +16406,7 @@
         </is>
       </c>
       <c r="G24" s="74" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="H24" s="42" t="inlineStr">
         <is>
@@ -16479,7 +16435,7 @@
         </is>
       </c>
       <c r="E25" s="41" t="n">
-        <v>10.0528</v>
+        <v>9.9961</v>
       </c>
       <c r="F25" s="42" t="inlineStr">
         <is>
@@ -16487,7 +16443,7 @@
         </is>
       </c>
       <c r="G25" s="74" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="H25" s="42" t="inlineStr">
         <is>
@@ -16516,7 +16472,7 @@
         </is>
       </c>
       <c r="E26" s="41" t="n">
-        <v>14.1097</v>
+        <v>14.0272</v>
       </c>
       <c r="F26" s="42" t="inlineStr">
         <is>
@@ -16524,7 +16480,7 @@
         </is>
       </c>
       <c r="G26" s="74" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="H26" s="42" t="inlineStr">
         <is>
@@ -16553,7 +16509,7 @@
         </is>
       </c>
       <c r="E27" s="41" t="n">
-        <v>16.8911</v>
+        <v>16.9636</v>
       </c>
       <c r="F27" s="42" t="inlineStr">
         <is>
@@ -16561,7 +16517,7 @@
         </is>
       </c>
       <c r="G27" s="74" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="H27" s="42" t="inlineStr">
         <is>
@@ -16590,7 +16546,7 @@
         </is>
       </c>
       <c r="E28" s="41" t="n">
-        <v>19.5599</v>
+        <v>20.1019</v>
       </c>
       <c r="F28" s="42" t="inlineStr">
         <is>
@@ -16598,7 +16554,7 @@
         </is>
       </c>
       <c r="G28" s="74" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="H28" s="42" t="inlineStr">
         <is>
@@ -16627,7 +16583,7 @@
         </is>
       </c>
       <c r="E29" s="41" t="n">
-        <v>28.7313</v>
+        <v>28.2028</v>
       </c>
       <c r="F29" s="42" t="inlineStr">
         <is>
@@ -16635,7 +16591,7 @@
         </is>
       </c>
       <c r="G29" s="74" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="H29" s="42" t="inlineStr">
         <is>
@@ -16664,7 +16620,7 @@
         </is>
       </c>
       <c r="E30" s="41" t="n">
-        <v>29.2314</v>
+        <v>37.6341</v>
       </c>
       <c r="F30" s="42" t="inlineStr">
         <is>
@@ -16672,7 +16628,7 @@
         </is>
       </c>
       <c r="G30" s="74" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="H30" s="42" t="inlineStr">
         <is>
@@ -16701,7 +16657,7 @@
         </is>
       </c>
       <c r="E31" s="41" t="n">
-        <v>12.819</v>
+        <v>12.8153</v>
       </c>
       <c r="F31" s="42" t="inlineStr">
         <is>
@@ -16709,7 +16665,7 @@
         </is>
       </c>
       <c r="G31" s="74" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="H31" s="42" t="inlineStr">
         <is>
@@ -16738,7 +16694,7 @@
         </is>
       </c>
       <c r="E32" s="41" t="n">
-        <v>21.7032</v>
+        <v>21.7034</v>
       </c>
       <c r="F32" s="42" t="inlineStr">
         <is>
@@ -16746,7 +16702,7 @@
         </is>
       </c>
       <c r="G32" s="74" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="H32" s="42" t="inlineStr">
         <is>
@@ -16775,7 +16731,7 @@
         </is>
       </c>
       <c r="E33" s="41" t="n">
-        <v>13.0668</v>
+        <v>12.446</v>
       </c>
       <c r="F33" s="42" t="inlineStr">
         <is>
@@ -16783,7 +16739,7 @@
         </is>
       </c>
       <c r="G33" s="74" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="H33" s="42" t="inlineStr">
         <is>
@@ -16812,7 +16768,7 @@
         </is>
       </c>
       <c r="E34" s="41" t="n">
-        <v>24.0099</v>
+        <v>29.0432</v>
       </c>
       <c r="F34" s="42" t="inlineStr">
         <is>
@@ -16820,7 +16776,7 @@
         </is>
       </c>
       <c r="G34" s="74" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="H34" s="42" t="inlineStr">
         <is>
@@ -16849,7 +16805,7 @@
         </is>
       </c>
       <c r="E35" s="41" t="n">
-        <v>9.927300000000001</v>
+        <v>9.968</v>
       </c>
       <c r="F35" s="42" t="inlineStr">
         <is>
@@ -16857,7 +16813,7 @@
         </is>
       </c>
       <c r="G35" s="74" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="H35" s="42" t="inlineStr">
         <is>
@@ -16886,7 +16842,7 @@
         </is>
       </c>
       <c r="E36" s="41" t="n">
-        <v>22.3558</v>
+        <v>22.387</v>
       </c>
       <c r="F36" s="42" t="inlineStr">
         <is>
@@ -16894,7 +16850,7 @@
         </is>
       </c>
       <c r="G36" s="74" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="H36" s="42" t="inlineStr">
         <is>
@@ -18255,7 +18211,7 @@
         </is>
       </c>
       <c r="E73" s="41" t="n">
-        <v>82.70999999999999</v>
+        <v>83.08</v>
       </c>
       <c r="F73" s="42" t="inlineStr">
         <is>
@@ -18292,7 +18248,7 @@
         </is>
       </c>
       <c r="E74" s="41" t="n">
-        <v>722.79</v>
+        <v>735.72</v>
       </c>
       <c r="F74" s="42" t="inlineStr">
         <is>
@@ -18329,7 +18285,7 @@
         </is>
       </c>
       <c r="E75" s="41" t="n">
-        <v>73920</v>
+        <v>73963</v>
       </c>
       <c r="F75" s="42" t="inlineStr">
         <is>
@@ -18366,7 +18322,7 @@
         </is>
       </c>
       <c r="E76" s="41" t="n">
-        <v>0.007985000000000001</v>
+        <v>0.007984</v>
       </c>
       <c r="F76" s="42" t="inlineStr">
         <is>
@@ -18403,7 +18359,7 @@
         </is>
       </c>
       <c r="E77" s="41" t="n">
-        <v>0.013265</v>
+        <v>0.012894</v>
       </c>
       <c r="F77" s="42" t="inlineStr">
         <is>
@@ -18440,7 +18396,7 @@
         </is>
       </c>
       <c r="E78" s="41" t="n">
-        <v>82.8</v>
+        <v>82.83</v>
       </c>
       <c r="F78" s="42" t="inlineStr">
         <is>
@@ -18477,7 +18433,7 @@
         </is>
       </c>
       <c r="E79" s="41" t="n">
-        <v>1.99</v>
+        <v>2</v>
       </c>
       <c r="F79" s="42" t="inlineStr">
         <is>
@@ -18551,7 +18507,7 @@
         </is>
       </c>
       <c r="E81" s="41" t="n">
-        <v>0.016039</v>
+        <v>0.01598</v>
       </c>
       <c r="F81" s="42" t="inlineStr">
         <is>
@@ -18588,7 +18544,7 @@
         </is>
       </c>
       <c r="E82" s="41" t="n">
-        <v>3.367077</v>
+        <v>3.36458</v>
       </c>
       <c r="F82" s="42" t="inlineStr">
         <is>
@@ -18625,7 +18581,7 @@
         </is>
       </c>
       <c r="E83" s="41" t="n">
-        <v>29.579695</v>
+        <v>29.510068</v>
       </c>
       <c r="F83" s="42" t="inlineStr">
         <is>
@@ -18662,7 +18618,7 @@
         </is>
       </c>
       <c r="E84" s="41" t="n">
-        <v>0.13623</v>
+        <v>0.135113</v>
       </c>
       <c r="F84" s="42" t="inlineStr">
         <is>
@@ -18699,7 +18655,7 @@
         </is>
       </c>
       <c r="E85" s="41" t="n">
-        <v>23440.0797</v>
+        <v>23859.3996</v>
       </c>
       <c r="F85" s="42" t="inlineStr">
         <is>
@@ -18736,7 +18692,7 @@
         </is>
       </c>
       <c r="E86" s="41" t="n">
-        <v>2397225.6</v>
+        <v>2398620.09</v>
       </c>
       <c r="F86" s="42" t="inlineStr">
         <is>
@@ -18773,7 +18729,7 @@
         </is>
       </c>
       <c r="E87" s="41" t="n">
-        <v>3.263658</v>
+        <v>3.266187</v>
       </c>
       <c r="F87" s="42" t="inlineStr">
         <is>
@@ -18810,7 +18766,7 @@
         </is>
       </c>
       <c r="E88" s="41" t="n">
-        <v>65637.3471</v>
+        <v>65730.0969</v>
       </c>
       <c r="F88" s="42" t="inlineStr">
         <is>
@@ -18847,7 +18803,7 @@
         </is>
       </c>
       <c r="E89" s="41" t="n">
-        <v>26.188425</v>
+        <v>26.172891</v>
       </c>
       <c r="F89" s="42" t="inlineStr">
         <is>
@@ -18884,7 +18840,7 @@
         </is>
       </c>
       <c r="E90" s="41" t="n">
-        <v>73920</v>
+        <v>73963</v>
       </c>
       <c r="F90" s="42" t="inlineStr">
         <is>
@@ -18921,7 +18877,7 @@
         </is>
       </c>
       <c r="E91" s="41" t="n">
-        <v>18.24</v>
+        <v>18.63</v>
       </c>
       <c r="F91" s="42" t="inlineStr">
         <is>
@@ -19032,7 +18988,7 @@
         </is>
       </c>
       <c r="E94" s="41" t="n">
-        <v>0.007985000000000001</v>
+        <v>0.007984</v>
       </c>
       <c r="F94" s="42" t="inlineStr">
         <is>
@@ -19069,7 +19025,7 @@
         </is>
       </c>
       <c r="E95" s="41" t="n">
-        <v>82.8</v>
+        <v>82.83</v>
       </c>
       <c r="F95" s="42" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Fix: evaluate formula-valued input cells (Dime cash undercount)
Dime USD cash had its Shares cell entered as a formula '=254.87+2584.77'.
The engine read the raw string and dropped it to 0, undercounting Dime cash by
~THB 92,090 (showed THB 435 instead of THB 92,525).

portfolio.py _num() now evaluates simple arithmetic typed into input cells
(digits/operators only, sandboxed eval). Generic fix for any =a+b input.

Cash & Equivalents THB 375,566 -> 467,655; total THB 25,520,511 -> 25,612,600.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jack/investment-dashboard/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{062E672F-E0BB-EC4F-A907-323C99F1C90A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B81FEEDA-3EC6-FC4C-B979-10B7360206B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="26260" windowHeight="17160" tabRatio="500" firstSheet="2" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38400" yWindow="-1880" windowWidth="38400" windowHeight="21000" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
     <sheet name="Reference" sheetId="12" r:id="rId12"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Crypto - by Coin'!$A$4:$K$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Crypto - by Coin'!$A$4:$K$29</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Crypto - Lots'!$A$4:$O$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Equities - by Ticker'!$A$4:$M$50</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Equities - Lots'!$A$4:$P$45</definedName>
@@ -1330,7 +1330,7 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="166" fontId="8" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
@@ -1341,13 +1341,13 @@
     <xf numFmtId="165" fontId="8" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="8" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="8" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="8" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -5438,7 +5438,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
-  <dimension ref="A2:K29"/>
+  <dimension ref="A2:K30"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -5536,11 +5536,11 @@
         <v>22410.803967524102</v>
       </c>
       <c r="J5" s="12">
-        <f t="shared" ref="J5:J28" si="0">I5-H5</f>
+        <f t="shared" ref="J5:J29" si="0">I5-H5</f>
         <v>22410.803967524102</v>
       </c>
       <c r="K5" s="11">
-        <f t="shared" ref="K5:K29" si="1">IFERROR(J5/H5,0)</f>
+        <f t="shared" ref="K5:K30" si="1">IFERROR(J5/H5,0)</f>
         <v>0</v>
       </c>
     </row>
@@ -6502,50 +6502,63 @@
         <v>21892.864662799999</v>
       </c>
       <c r="J28" s="12">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="J28" si="2">I28-H28</f>
         <v>-94117.753337200003</v>
       </c>
       <c r="K28" s="11">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="K28" si="3">IFERROR(J28/H28,0)</f>
         <v>-0.81128568194680251</v>
       </c>
     </row>
     <row r="29" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="13" t="s">
+      <c r="A29" s="35"/>
+      <c r="B29" s="35"/>
+      <c r="C29" s="35"/>
+      <c r="D29" s="34"/>
+      <c r="E29" s="18"/>
+      <c r="F29" s="44"/>
+      <c r="G29" s="41"/>
+      <c r="H29" s="10"/>
+      <c r="I29" s="10"/>
+      <c r="J29" s="12"/>
+      <c r="K29" s="11"/>
+    </row>
+    <row r="30" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="13" t="s">
         <v>69</v>
       </c>
-      <c r="B29" s="43"/>
-      <c r="C29" s="43"/>
-      <c r="D29" s="43"/>
-      <c r="E29" s="43"/>
-      <c r="F29" s="45">
-        <f>SUM(F5:F28)</f>
+      <c r="B30" s="43"/>
+      <c r="C30" s="43"/>
+      <c r="D30" s="43"/>
+      <c r="E30" s="43"/>
+      <c r="F30" s="45">
+        <f>SUM(F5:F29)</f>
         <v>26</v>
       </c>
-      <c r="G29" s="43"/>
-      <c r="H29" s="14">
-        <f>SUM(H5:H28)</f>
+      <c r="G30" s="43"/>
+      <c r="H30" s="14">
+        <f>SUM(H5:H29)</f>
         <v>1692484.2613636358</v>
       </c>
-      <c r="I29" s="14">
-        <f>SUM(I5:I28)</f>
+      <c r="I30" s="14">
+        <f>SUM(I5:I29)</f>
         <v>1339357.6953334461</v>
       </c>
-      <c r="J29" s="14">
-        <f>SUM(J5:J28)</f>
+      <c r="J30" s="14">
+        <f>SUM(J5:J29)</f>
         <v>-353126.56603018945</v>
       </c>
-      <c r="K29" s="15">
+      <c r="K30" s="15">
         <f t="shared" si="1"/>
         <v>-0.20864392898145778</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:K28" xr:uid="{00000000-0009-0000-0000-00000A000000}"/>
+  <autoFilter ref="A4:K29" xr:uid="{00000000-0009-0000-0000-00000A000000}"/>
   <mergeCells count="1">
     <mergeCell ref="A2:K2"/>
   </mergeCells>
-  <conditionalFormatting sqref="J5:K28">
+  <conditionalFormatting sqref="J5:K29">
     <cfRule type="cellIs" dxfId="0" priority="2" operator="lessThan">
       <formula>0</formula>
     </cfRule>
@@ -10201,7 +10214,7 @@
     </row>
     <row r="101" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A101" s="35" t="str">
-        <f t="shared" ref="A101:A132" si="6">B101&amp;"|"&amp;C101&amp;"|"&amp;D101</f>
+        <f t="shared" ref="A101:A106" si="6">B101&amp;"|"&amp;C101&amp;"|"&amp;D101</f>
         <v>Crypto|DOGE|Bitkub</v>
       </c>
       <c r="B101" s="32" t="s">
@@ -10232,7 +10245,7 @@
         <v>9</v>
       </c>
       <c r="K101" s="39">
-        <f t="shared" ref="K101:K132" si="7">IF(J101="THB",1,FXRate)</f>
+        <f t="shared" ref="K101:K106" si="7">IF(J101="THB",1,FXRate)</f>
         <v>1</v>
       </c>
     </row>
@@ -10490,17 +10503,17 @@
       <c r="L5" s="50"/>
     </row>
     <row r="7" spans="2:12" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B7" s="57" t="s">
+      <c r="B7" s="51" t="s">
         <v>43</v>
       </c>
       <c r="C7" s="52"/>
       <c r="D7" s="53"/>
-      <c r="F7" s="57" t="s">
+      <c r="F7" s="51" t="s">
         <v>44</v>
       </c>
       <c r="G7" s="52"/>
       <c r="H7" s="53"/>
-      <c r="J7" s="57" t="s">
+      <c r="J7" s="51" t="s">
         <v>45</v>
       </c>
       <c r="K7" s="52"/>
@@ -10527,36 +10540,36 @@
       <c r="L8" s="53"/>
     </row>
     <row r="10" spans="2:12" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="57" t="s">
+      <c r="B10" s="51" t="s">
         <v>46</v>
       </c>
       <c r="C10" s="52"/>
       <c r="D10" s="53"/>
-      <c r="F10" s="57" t="s">
+      <c r="F10" s="51" t="s">
         <v>47</v>
       </c>
       <c r="G10" s="52"/>
       <c r="H10" s="53"/>
-      <c r="J10" s="57" t="s">
+      <c r="J10" s="51" t="s">
         <v>48</v>
       </c>
       <c r="K10" s="52"/>
       <c r="L10" s="53"/>
     </row>
     <row r="11" spans="2:12" ht="42" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="51">
+      <c r="B11" s="57">
         <f>IFERROR(('MF - Lots'!Q167+'Equities - Lots'!N53+'Crypto - Lots'!L32)/('MF - Lots'!O167+'Equities - Lots'!L53+'Crypto - Lots'!J32),0)</f>
         <v>0.17548385248007967</v>
       </c>
       <c r="C11" s="52"/>
       <c r="D11" s="53"/>
-      <c r="F11" s="58" t="str">
+      <c r="F11" s="56" t="str">
         <f>COUNTA('MF - Lots'!C5:C166)&amp;" / "&amp;COUNTA('Equities - Lots'!C5:C45)&amp;" / "&amp;COUNTA('Crypto - Lots'!C5:C30)</f>
         <v>161 / 41 / 26</v>
       </c>
       <c r="G11" s="52"/>
       <c r="H11" s="53"/>
-      <c r="J11" s="56">
+      <c r="J11" s="58">
         <f>FXRate</f>
         <v>32.43</v>
       </c>
@@ -13025,21 +13038,24 @@
       </c>
     </row>
     <row r="120" spans="14:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="N120" s="19" t="str">
-        <f>'Crypto - by Coin'!C28</f>
-        <v>ARB</v>
-      </c>
-      <c r="O120" s="19" t="str">
-        <f>'Crypto - by Coin'!B28</f>
-        <v>Bitazza</v>
+      <c r="N120" s="19">
+        <f>'Crypto - by Coin'!C29</f>
+        <v>0</v>
+      </c>
+      <c r="O120" s="19">
+        <f>'Crypto - by Coin'!B29</f>
+        <v>0</v>
       </c>
       <c r="P120" s="20">
-        <f>'Crypto - by Coin'!I28</f>
-        <v>21892.864662799999</v>
+        <f>'Crypto - by Coin'!I29</f>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="F8:H8"/>
+    <mergeCell ref="J11:L11"/>
     <mergeCell ref="J7:L7"/>
     <mergeCell ref="B10:D10"/>
     <mergeCell ref="B39:L39"/>
@@ -13056,9 +13072,6 @@
     <mergeCell ref="B26:F26"/>
     <mergeCell ref="B11:D11"/>
     <mergeCell ref="H26:L26"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="F8:H8"/>
-    <mergeCell ref="J11:L11"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -17189,7 +17202,7 @@
     </row>
     <row r="101" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A101" s="35" t="str">
-        <f t="shared" ref="A101:A132" si="3">B101&amp;"|"&amp;C101&amp;"|"&amp;D101</f>
+        <f t="shared" ref="A101:A104" si="3">B101&amp;"|"&amp;C101&amp;"|"&amp;D101</f>
         <v>Crypto|SOL|OKX</v>
       </c>
       <c r="B101" s="9" t="s">
@@ -28000,11 +28013,11 @@
         <v>101250.9367284</v>
       </c>
       <c r="Q165" s="42">
-        <f t="shared" ref="Q165:Q196" si="20">P165-O165</f>
+        <f t="shared" ref="Q165" si="20">P165-O165</f>
         <v>1250.9367284000036</v>
       </c>
       <c r="R165" s="11">
-        <f t="shared" ref="R165:R196" si="21">IFERROR(Q165/O165,0)</f>
+        <f t="shared" ref="R165" si="21">IFERROR(Q165/O165,0)</f>
         <v>1.2509367284000036E-2</v>
       </c>
       <c r="S165" s="35"/>

</xml_diff>

<commit_message>
Wire up auto-fetch for SGD unit trust NAVs
All 5 unit trusts now refresh automatically each week:
- 4 via their Yahoo 0P...SI symbols
- 1 (Janus Henderson, ISIN LU1316542866) auto-resolved to 0P0001710O.SI and cached
- fetch_prices.py: yahoo_symbol_for_isin() resolves an ISIN via Yahoo search,
  retries the price, and writes the resolved symbol back to the sheet

Unit trust NAVs are no longer manual — the weekly job keeps them current.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-38400" yWindow="-1880" windowWidth="38400" windowHeight="21000" tabRatio="500" firstSheet="0" activeTab="11" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17200" tabRatio="500" firstSheet="0" activeTab="11" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
@@ -827,7 +827,7 @@
                     </a:defRPr>
                   </a:pPr>
                   <a:r>
-                    <a:t>None</a:t>
+                    <a:t/>
                   </a:r>
                   <a:endParaRPr lang="en-TH"/>
                 </a:p>
@@ -860,7 +860,7 @@
                     </a:defRPr>
                   </a:pPr>
                   <a:r>
-                    <a:t>None</a:t>
+                    <a:t/>
                   </a:r>
                   <a:endParaRPr lang="en-TH"/>
                 </a:p>
@@ -893,7 +893,7 @@
                     </a:defRPr>
                   </a:pPr>
                   <a:r>
-                    <a:t>None</a:t>
+                    <a:t/>
                   </a:r>
                   <a:endParaRPr lang="en-TH"/>
                 </a:p>
@@ -926,7 +926,7 @@
                     </a:defRPr>
                   </a:pPr>
                   <a:r>
-                    <a:t>None</a:t>
+                    <a:t/>
                   </a:r>
                   <a:endParaRPr lang="en-TH"/>
                 </a:p>
@@ -959,7 +959,7 @@
                     </a:defRPr>
                   </a:pPr>
                   <a:r>
-                    <a:t>None</a:t>
+                    <a:t/>
                   </a:r>
                   <a:endParaRPr lang="en-TH"/>
                 </a:p>
@@ -992,7 +992,7 @@
                     </a:defRPr>
                   </a:pPr>
                   <a:r>
-                    <a:t>None</a:t>
+                    <a:t/>
                   </a:r>
                   <a:endParaRPr lang="en-TH"/>
                 </a:p>
@@ -1025,7 +1025,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t>None</a:t>
+                  <a:t/>
                 </a:r>
                 <a:endParaRPr lang="en-TH"/>
               </a:p>
@@ -1086,7 +1086,7 @@
                   <v>467655.2897172199</v>
                 </pt>
                 <pt idx="5">
-                  <v>1339357.695333446</v>
+                  <v>1332906.543351746</v>
                 </pt>
               </numCache>
             </numRef>
@@ -1129,7 +1129,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t>None</a:t>
+            <a:t/>
           </a:r>
           <a:endParaRPr lang="en-TH"/>
         </a:p>
@@ -1356,7 +1356,7 @@
                     </a:defRPr>
                   </a:pPr>
                   <a:r>
-                    <a:t>None</a:t>
+                    <a:t/>
                   </a:r>
                   <a:endParaRPr lang="en-TH"/>
                 </a:p>
@@ -1390,7 +1390,7 @@
                     </a:defRPr>
                   </a:pPr>
                   <a:r>
-                    <a:t>None</a:t>
+                    <a:t/>
                   </a:r>
                   <a:endParaRPr lang="en-TH"/>
                 </a:p>
@@ -1424,7 +1424,7 @@
                     </a:defRPr>
                   </a:pPr>
                   <a:r>
-                    <a:t>None</a:t>
+                    <a:t/>
                   </a:r>
                   <a:endParaRPr lang="en-TH"/>
                 </a:p>
@@ -1458,7 +1458,7 @@
                     </a:defRPr>
                   </a:pPr>
                   <a:r>
-                    <a:t>None</a:t>
+                    <a:t/>
                   </a:r>
                   <a:endParaRPr lang="en-TH"/>
                 </a:p>
@@ -1492,7 +1492,7 @@
                     </a:defRPr>
                   </a:pPr>
                   <a:r>
-                    <a:t>None</a:t>
+                    <a:t/>
                   </a:r>
                   <a:endParaRPr lang="en-TH"/>
                 </a:p>
@@ -1526,7 +1526,7 @@
                     </a:defRPr>
                   </a:pPr>
                   <a:r>
-                    <a:t>None</a:t>
+                    <a:t/>
                   </a:r>
                   <a:endParaRPr lang="en-TH"/>
                 </a:p>
@@ -1560,7 +1560,7 @@
                     </a:defRPr>
                   </a:pPr>
                   <a:r>
-                    <a:t>None</a:t>
+                    <a:t/>
                   </a:r>
                   <a:endParaRPr lang="en-TH"/>
                 </a:p>
@@ -1594,7 +1594,7 @@
                     </a:defRPr>
                   </a:pPr>
                   <a:r>
-                    <a:t>None</a:t>
+                    <a:t/>
                   </a:r>
                   <a:endParaRPr lang="en-TH"/>
                 </a:p>
@@ -1628,7 +1628,7 @@
                     </a:defRPr>
                   </a:pPr>
                   <a:r>
-                    <a:t>None</a:t>
+                    <a:t/>
                   </a:r>
                   <a:endParaRPr lang="en-TH"/>
                 </a:p>
@@ -1662,7 +1662,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t>None</a:t>
+                  <a:t/>
                 </a:r>
                 <a:endParaRPr lang="en-TH"/>
               </a:p>
@@ -1721,7 +1721,7 @@
                   <v>7226409.740020407</v>
                 </pt>
                 <pt idx="2">
-                  <v>4018012.204820406</v>
+                  <v>4011561.052838705</v>
                 </pt>
                 <pt idx="3">
                   <v>5877663.902051419</v>
@@ -1778,7 +1778,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t>None</a:t>
+            <a:t/>
           </a:r>
           <a:endParaRPr lang="en-TH"/>
         </a:p>
@@ -1891,7 +1891,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t>None</a:t>
+                  <a:t/>
                 </a:r>
                 <a:endParaRPr lang="en-TH"/>
               </a:p>
@@ -1953,7 +1953,7 @@
                   <v>932032.3245061599</v>
                 </pt>
                 <pt idx="5">
-                  <v>6591384.475767633</v>
+                  <v>6584933.323785933</v>
                 </pt>
               </numCache>
             </numRef>
@@ -2005,7 +2005,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr lang="en-TH"/>
           </a:p>
@@ -2062,7 +2062,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr lang="en-TH"/>
           </a:p>
@@ -2096,7 +2096,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t>None</a:t>
+            <a:t/>
           </a:r>
           <a:endParaRPr lang="en-TH"/>
         </a:p>
@@ -2198,7 +2198,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t>None</a:t>
+                  <a:t/>
                 </a:r>
                 <a:endParaRPr lang="en-TH"/>
               </a:p>
@@ -2303,7 +2303,7 @@
                   <v>1762560.34767768</v>
                 </pt>
                 <pt idx="5">
-                  <v>1339357.695333446</v>
+                  <v>1332906.543351746</v>
                 </pt>
                 <pt idx="6">
                   <v>1306914.7381852</v>
@@ -2400,7 +2400,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr lang="en-TH"/>
           </a:p>
@@ -2457,7 +2457,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr lang="en-TH"/>
           </a:p>
@@ -2491,7 +2491,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t>None</a:t>
+            <a:t/>
           </a:r>
           <a:endParaRPr lang="en-TH"/>
         </a:p>
@@ -6208,7 +6208,11 @@
         <f>IFERROR(N5/L5,0)</f>
         <v/>
       </c>
-      <c r="P5" s="32" t="n"/>
+      <c r="P5" s="32" t="inlineStr">
+        <is>
+          <t>0P0001710O.SI</t>
+        </is>
+      </c>
       <c r="Q5" s="32" t="n"/>
     </row>
     <row r="6">
@@ -6274,7 +6278,11 @@
         <f>IFERROR(N6/L6,0)</f>
         <v/>
       </c>
-      <c r="P6" s="32" t="n"/>
+      <c r="P6" s="32" t="inlineStr">
+        <is>
+          <t>0P00008T0M.SI</t>
+        </is>
+      </c>
       <c r="Q6" s="32" t="n"/>
     </row>
     <row r="7">
@@ -6340,7 +6348,11 @@
         <f>IFERROR(N7/L7,0)</f>
         <v/>
       </c>
-      <c r="P7" s="32" t="n"/>
+      <c r="P7" s="32" t="inlineStr">
+        <is>
+          <t>0P0000YWFQ.SI</t>
+        </is>
+      </c>
       <c r="Q7" s="32" t="n"/>
     </row>
     <row r="8">
@@ -6406,7 +6418,11 @@
         <f>IFERROR(N8/L8,0)</f>
         <v/>
       </c>
-      <c r="P8" s="32" t="n"/>
+      <c r="P8" s="32" t="inlineStr">
+        <is>
+          <t>0P00012P5A.SI</t>
+        </is>
+      </c>
       <c r="Q8" s="32" t="n"/>
     </row>
     <row r="9">
@@ -6472,7 +6488,11 @@
         <f>IFERROR(N9/L9,0)</f>
         <v/>
       </c>
-      <c r="P9" s="32" t="n"/>
+      <c r="P9" s="32" t="inlineStr">
+        <is>
+          <t>0P0000Y4WK.SI</t>
+        </is>
+      </c>
       <c r="Q9" s="32" t="n"/>
     </row>
     <row r="10">
@@ -19498,7 +19518,7 @@
         </is>
       </c>
       <c r="E79" s="33" t="n">
-        <v>81.84999999999999</v>
+        <v>81.7</v>
       </c>
       <c r="F79" s="34" t="inlineStr">
         <is>
@@ -19535,7 +19555,7 @@
         </is>
       </c>
       <c r="E80" s="33" t="n">
-        <v>719.8200000000001</v>
+        <v>720.38</v>
       </c>
       <c r="F80" s="34" t="inlineStr">
         <is>
@@ -19572,7 +19592,7 @@
         </is>
       </c>
       <c r="E81" s="33" t="n">
-        <v>73546</v>
+        <v>73574</v>
       </c>
       <c r="F81" s="34" t="inlineStr">
         <is>
@@ -19609,7 +19629,7 @@
         </is>
       </c>
       <c r="E82" s="33" t="n">
-        <v>0.00787</v>
+        <v>0.007833</v>
       </c>
       <c r="F82" s="34" t="inlineStr">
         <is>
@@ -19646,7 +19666,7 @@
         </is>
       </c>
       <c r="E83" s="33" t="n">
-        <v>0.012685</v>
+        <v>0.012637</v>
       </c>
       <c r="F83" s="34" t="inlineStr">
         <is>
@@ -19683,7 +19703,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>81.92</v>
+        <v>81.84</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -19794,7 +19814,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.015659</v>
+        <v>0.015649</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -19831,7 +19851,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>3.287462</v>
+        <v>3.276435</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -19868,7 +19888,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>28.53827</v>
+        <v>28.468124</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -19905,7 +19925,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>0.132164</v>
+        <v>0.131818</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -19942,7 +19962,7 @@
         </is>
       </c>
       <c r="E91" s="33" t="n">
-        <v>23343.7626</v>
+        <v>23361.9234</v>
       </c>
       <c r="F91" s="34" t="inlineStr">
         <is>
@@ -19979,7 +19999,7 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
-        <v>2385096.78</v>
+        <v>2386004.82</v>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
@@ -20016,7 +20036,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>3.242968</v>
+        <v>3.236968</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -20053,7 +20073,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>65102.2521</v>
+        <v>65131.7634</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -20090,7 +20110,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>26.08773</v>
+        <v>26.078876</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -20127,7 +20147,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>73546</v>
+        <v>73574</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -20164,7 +20184,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>18.3</v>
+        <v>18.25</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -20275,7 +20295,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>0.00787</v>
+        <v>0.007833</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -20312,7 +20332,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>81.92</v>
+        <v>81.84</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Daily dashboard update — 2026-06-04 (manual recovery of missed scheduled run)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -21584,16 +21584,38 @@
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="58">
-      <c r="B8" s="28" t="n"/>
-      <c r="C8" s="29" t="n"/>
-      <c r="D8" s="29" t="n"/>
-      <c r="E8" s="29" t="n"/>
-      <c r="F8" s="30" t="n"/>
-      <c r="G8" s="29" t="n"/>
-      <c r="H8" s="29" t="n"/>
-      <c r="I8" s="29" t="n"/>
-      <c r="J8" s="31" t="n"/>
-      <c r="K8" s="32" t="n"/>
+      <c r="B8" s="28" t="n">
+        <v>46177</v>
+      </c>
+      <c r="C8" s="29" t="n">
+        <v>26900424</v>
+      </c>
+      <c r="D8" s="29" t="n">
+        <v>22657814</v>
+      </c>
+      <c r="E8" s="29" t="n">
+        <v>4242610</v>
+      </c>
+      <c r="F8" s="30" t="n">
+        <v>0.1872</v>
+      </c>
+      <c r="G8" s="29" t="n">
+        <v>19094011</v>
+      </c>
+      <c r="H8" s="29" t="n">
+        <v>5224964</v>
+      </c>
+      <c r="I8" s="29" t="n">
+        <v>1162725</v>
+      </c>
+      <c r="J8" s="31" t="n">
+        <v>32.68</v>
+      </c>
+      <c r="K8" s="32" t="inlineStr">
+        <is>
+          <t>Auto weekly snapshot</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="58">
       <c r="B9" s="28" t="n"/>
@@ -23379,7 +23401,7 @@
         </is>
       </c>
       <c r="C5" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="D5" s="64" t="inlineStr">
         <is>
@@ -23394,11 +23416,11 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>32.72</v>
+        <v>32.68</v>
       </c>
       <c r="D6" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-06-03</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-06-04</t>
         </is>
       </c>
     </row>
@@ -23443,11 +23465,11 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>25.5508</v>
+        <v>25.4804</v>
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-06-03</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-06-04</t>
         </is>
       </c>
     </row>
@@ -24773,7 +24795,7 @@
         </is>
       </c>
       <c r="E38" s="33" t="n">
-        <v>22.37</v>
+        <v>22.59</v>
       </c>
       <c r="F38" s="34" t="inlineStr">
         <is>
@@ -24781,7 +24803,7 @@
         </is>
       </c>
       <c r="G38" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H38" s="34" t="inlineStr">
         <is>
@@ -24818,7 +24840,7 @@
         </is>
       </c>
       <c r="G39" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H39" s="34" t="inlineStr">
         <is>
@@ -24847,7 +24869,7 @@
         </is>
       </c>
       <c r="E40" s="33" t="n">
-        <v>806.6</v>
+        <v>803.14</v>
       </c>
       <c r="F40" s="34" t="inlineStr">
         <is>
@@ -24855,7 +24877,7 @@
         </is>
       </c>
       <c r="G40" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H40" s="34" t="inlineStr">
         <is>
@@ -24884,7 +24906,7 @@
         </is>
       </c>
       <c r="E41" s="33" t="n">
-        <v>22</v>
+        <v>22.02</v>
       </c>
       <c r="F41" s="34" t="inlineStr">
         <is>
@@ -24892,7 +24914,7 @@
         </is>
       </c>
       <c r="G41" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H41" s="34" t="inlineStr">
         <is>
@@ -24921,7 +24943,7 @@
         </is>
       </c>
       <c r="E42" s="33" t="n">
-        <v>227.52</v>
+        <v>228.38</v>
       </c>
       <c r="F42" s="34" t="inlineStr">
         <is>
@@ -24929,7 +24951,7 @@
         </is>
       </c>
       <c r="G42" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H42" s="34" t="inlineStr">
         <is>
@@ -24966,7 +24988,7 @@
         </is>
       </c>
       <c r="G43" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H43" s="34" t="inlineStr">
         <is>
@@ -25003,7 +25025,7 @@
         </is>
       </c>
       <c r="G44" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H44" s="34" t="inlineStr">
         <is>
@@ -25040,7 +25062,7 @@
         </is>
       </c>
       <c r="G45" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H45" s="34" t="inlineStr">
         <is>
@@ -25077,7 +25099,7 @@
         </is>
       </c>
       <c r="G46" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H46" s="34" t="inlineStr">
         <is>
@@ -25151,7 +25173,7 @@
         </is>
       </c>
       <c r="G48" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H48" s="34" t="inlineStr">
         <is>
@@ -25188,7 +25210,7 @@
         </is>
       </c>
       <c r="G49" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H49" s="34" t="inlineStr">
         <is>
@@ -25225,7 +25247,7 @@
         </is>
       </c>
       <c r="G50" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H50" s="34" t="inlineStr">
         <is>
@@ -25262,7 +25284,7 @@
         </is>
       </c>
       <c r="G51" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H51" s="34" t="inlineStr">
         <is>
@@ -25299,7 +25321,7 @@
         </is>
       </c>
       <c r="G52" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H52" s="34" t="inlineStr">
         <is>
@@ -25336,7 +25358,7 @@
         </is>
       </c>
       <c r="G53" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H53" s="34" t="inlineStr">
         <is>
@@ -25373,7 +25395,7 @@
         </is>
       </c>
       <c r="G54" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H54" s="34" t="inlineStr">
         <is>
@@ -25410,7 +25432,7 @@
         </is>
       </c>
       <c r="G55" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H55" s="34" t="inlineStr">
         <is>
@@ -25447,7 +25469,7 @@
         </is>
       </c>
       <c r="G56" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H56" s="34" t="inlineStr">
         <is>
@@ -25484,7 +25506,7 @@
         </is>
       </c>
       <c r="G57" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H57" s="34" t="inlineStr">
         <is>
@@ -25521,7 +25543,7 @@
         </is>
       </c>
       <c r="G58" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H58" s="34" t="inlineStr">
         <is>
@@ -25558,7 +25580,7 @@
         </is>
       </c>
       <c r="G59" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H59" s="34" t="inlineStr">
         <is>
@@ -25587,7 +25609,7 @@
         </is>
       </c>
       <c r="E60" s="33" t="n">
-        <v>158.78</v>
+        <v>159.19</v>
       </c>
       <c r="F60" s="34" t="inlineStr">
         <is>
@@ -25595,7 +25617,7 @@
         </is>
       </c>
       <c r="G60" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H60" s="34" t="inlineStr">
         <is>
@@ -25624,7 +25646,7 @@
         </is>
       </c>
       <c r="E61" s="33" t="n">
-        <v>262.11</v>
+        <v>256.24</v>
       </c>
       <c r="F61" s="34" t="inlineStr">
         <is>
@@ -25632,7 +25654,7 @@
         </is>
       </c>
       <c r="G61" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H61" s="34" t="inlineStr">
         <is>
@@ -25661,7 +25683,7 @@
         </is>
       </c>
       <c r="E62" s="33" t="n">
-        <v>490.05</v>
+        <v>500.77</v>
       </c>
       <c r="F62" s="34" t="inlineStr">
         <is>
@@ -25669,7 +25691,7 @@
         </is>
       </c>
       <c r="G62" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H62" s="34" t="inlineStr">
         <is>
@@ -25698,7 +25720,7 @@
         </is>
       </c>
       <c r="E63" s="33" t="n">
-        <v>170.62</v>
+        <v>178.9</v>
       </c>
       <c r="F63" s="34" t="inlineStr">
         <is>
@@ -25706,7 +25728,7 @@
         </is>
       </c>
       <c r="G63" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H63" s="34" t="inlineStr">
         <is>
@@ -25735,7 +25757,7 @@
         </is>
       </c>
       <c r="E64" s="33" t="n">
-        <v>72.33</v>
+        <v>69.02</v>
       </c>
       <c r="F64" s="34" t="inlineStr">
         <is>
@@ -25743,7 +25765,7 @@
         </is>
       </c>
       <c r="G64" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H64" s="34" t="inlineStr">
         <is>
@@ -25772,7 +25794,7 @@
         </is>
       </c>
       <c r="E65" s="33" t="n">
-        <v>214.53</v>
+        <v>212.96</v>
       </c>
       <c r="F65" s="34" t="inlineStr">
         <is>
@@ -25780,7 +25802,7 @@
         </is>
       </c>
       <c r="G65" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H65" s="34" t="inlineStr">
         <is>
@@ -25809,7 +25831,7 @@
         </is>
       </c>
       <c r="E66" s="33" t="n">
-        <v>148.86</v>
+        <v>146.48</v>
       </c>
       <c r="F66" s="34" t="inlineStr">
         <is>
@@ -25817,7 +25839,7 @@
         </is>
       </c>
       <c r="G66" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H66" s="34" t="inlineStr">
         <is>
@@ -25846,7 +25868,7 @@
         </is>
       </c>
       <c r="E67" s="33" t="n">
-        <v>170.62</v>
+        <v>164.75</v>
       </c>
       <c r="F67" s="34" t="inlineStr">
         <is>
@@ -25854,7 +25876,7 @@
         </is>
       </c>
       <c r="G67" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H67" s="34" t="inlineStr">
         <is>
@@ -25883,7 +25905,7 @@
         </is>
       </c>
       <c r="E68" s="33" t="n">
-        <v>2045.2</v>
+        <v>2125.11</v>
       </c>
       <c r="F68" s="34" t="inlineStr">
         <is>
@@ -25891,7 +25913,7 @@
         </is>
       </c>
       <c r="G68" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H68" s="34" t="inlineStr">
         <is>
@@ -25920,7 +25942,7 @@
         </is>
       </c>
       <c r="E69" s="33" t="n">
-        <v>1064.15</v>
+        <v>1078.78</v>
       </c>
       <c r="F69" s="34" t="inlineStr">
         <is>
@@ -25928,7 +25950,7 @@
         </is>
       </c>
       <c r="G69" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H69" s="34" t="inlineStr">
         <is>
@@ -25957,7 +25979,7 @@
         </is>
       </c>
       <c r="E70" s="33" t="n">
-        <v>96.95999999999999</v>
+        <v>96.55</v>
       </c>
       <c r="F70" s="34" t="inlineStr">
         <is>
@@ -25965,7 +25987,7 @@
         </is>
       </c>
       <c r="G70" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H70" s="34" t="inlineStr">
         <is>
@@ -25994,7 +26016,7 @@
         </is>
       </c>
       <c r="E71" s="33" t="n">
-        <v>1624.99</v>
+        <v>1689.89</v>
       </c>
       <c r="F71" s="34" t="inlineStr">
         <is>
@@ -26002,7 +26024,7 @@
         </is>
       </c>
       <c r="G71" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H71" s="34" t="inlineStr">
         <is>
@@ -26031,7 +26053,7 @@
         </is>
       </c>
       <c r="E72" s="33" t="n">
-        <v>119.7</v>
+        <v>115.6</v>
       </c>
       <c r="F72" s="34" t="inlineStr">
         <is>
@@ -26039,7 +26061,7 @@
         </is>
       </c>
       <c r="G72" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H72" s="34" t="inlineStr">
         <is>
@@ -26068,7 +26090,7 @@
         </is>
       </c>
       <c r="E73" s="33" t="n">
-        <v>222.82</v>
+        <v>214.75</v>
       </c>
       <c r="F73" s="34" t="inlineStr">
         <is>
@@ -26076,7 +26098,7 @@
         </is>
       </c>
       <c r="G73" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H73" s="34" t="inlineStr">
         <is>
@@ -26105,7 +26127,7 @@
         </is>
       </c>
       <c r="E74" s="33" t="n">
-        <v>93.79000000000001</v>
+        <v>90.84</v>
       </c>
       <c r="F74" s="34" t="inlineStr">
         <is>
@@ -26113,7 +26135,7 @@
         </is>
       </c>
       <c r="G74" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H74" s="34" t="inlineStr">
         <is>
@@ -26142,7 +26164,7 @@
         </is>
       </c>
       <c r="E75" s="33" t="n">
-        <v>102.74</v>
+        <v>104.73</v>
       </c>
       <c r="F75" s="34" t="inlineStr">
         <is>
@@ -26150,7 +26172,7 @@
         </is>
       </c>
       <c r="G75" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H75" s="34" t="inlineStr">
         <is>
@@ -26179,7 +26201,7 @@
         </is>
       </c>
       <c r="E76" s="33" t="n">
-        <v>392.62</v>
+        <v>409.67</v>
       </c>
       <c r="F76" s="34" t="inlineStr">
         <is>
@@ -26187,7 +26209,7 @@
         </is>
       </c>
       <c r="G76" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H76" s="34" t="inlineStr">
         <is>
@@ -26216,7 +26238,7 @@
         </is>
       </c>
       <c r="E77" s="33" t="n">
-        <v>423.74</v>
+        <v>423.7</v>
       </c>
       <c r="F77" s="34" t="inlineStr">
         <is>
@@ -26224,7 +26246,7 @@
         </is>
       </c>
       <c r="G77" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H77" s="34" t="inlineStr">
         <is>
@@ -26253,7 +26275,7 @@
         </is>
       </c>
       <c r="E78" s="33" t="n">
-        <v>56.78</v>
+        <v>56.08</v>
       </c>
       <c r="F78" s="34" t="inlineStr">
         <is>
@@ -26261,7 +26283,7 @@
         </is>
       </c>
       <c r="G78" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H78" s="34" t="inlineStr">
         <is>
@@ -26290,7 +26312,7 @@
         </is>
       </c>
       <c r="E79" s="33" t="n">
-        <v>102.18</v>
+        <v>98.31999999999999</v>
       </c>
       <c r="F79" s="34" t="inlineStr">
         <is>
@@ -26298,7 +26320,7 @@
         </is>
       </c>
       <c r="G79" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H79" s="34" t="inlineStr">
         <is>
@@ -26327,7 +26349,7 @@
         </is>
       </c>
       <c r="E80" s="33" t="n">
-        <v>315.2</v>
+        <v>310.26</v>
       </c>
       <c r="F80" s="34" t="inlineStr">
         <is>
@@ -26335,7 +26357,7 @@
         </is>
       </c>
       <c r="G80" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H80" s="34" t="inlineStr">
         <is>
@@ -26364,7 +26386,7 @@
         </is>
       </c>
       <c r="E81" s="33" t="n">
-        <v>173.99</v>
+        <v>163.22</v>
       </c>
       <c r="F81" s="34" t="inlineStr">
         <is>
@@ -26372,7 +26394,7 @@
         </is>
       </c>
       <c r="G81" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H81" s="34" t="inlineStr">
         <is>
@@ -26401,7 +26423,7 @@
         </is>
       </c>
       <c r="E82" s="33" t="n">
-        <v>597.63</v>
+        <v>622.98</v>
       </c>
       <c r="F82" s="34" t="inlineStr">
         <is>
@@ -26409,7 +26431,7 @@
         </is>
       </c>
       <c r="G82" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H82" s="34" t="inlineStr">
         <is>
@@ -26438,7 +26460,7 @@
         </is>
       </c>
       <c r="E83" s="33" t="n">
-        <v>192.59</v>
+        <v>155.99</v>
       </c>
       <c r="F83" s="34" t="inlineStr">
         <is>
@@ -26446,7 +26468,7 @@
         </is>
       </c>
       <c r="G83" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H83" s="34" t="inlineStr">
         <is>
@@ -26475,7 +26497,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>76.44</v>
+        <v>71.29000000000001</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -26483,7 +26505,7 @@
         </is>
       </c>
       <c r="G84" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H84" s="34" t="inlineStr">
         <is>
@@ -26512,7 +26534,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>641.13</v>
+        <v>605.76</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -26520,7 +26542,7 @@
         </is>
       </c>
       <c r="G85" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H85" s="34" t="inlineStr">
         <is>
@@ -26549,7 +26571,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>67114</v>
+        <v>62867</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -26557,7 +26579,7 @@
         </is>
       </c>
       <c r="G86" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H86" s="34" t="inlineStr">
         <is>
@@ -26586,7 +26608,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.007194</v>
+        <v>0.006807</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -26594,7 +26616,7 @@
         </is>
       </c>
       <c r="G87" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H87" s="34" t="inlineStr">
         <is>
@@ -26623,7 +26645,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.013405</v>
+        <v>0.012284</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -26631,7 +26653,7 @@
         </is>
       </c>
       <c r="G88" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H88" s="34" t="inlineStr">
         <is>
@@ -26660,7 +26682,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>75.3</v>
+        <v>69.22</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -26668,7 +26690,7 @@
         </is>
       </c>
       <c r="G89" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H89" s="34" t="inlineStr">
         <is>
@@ -26697,7 +26719,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>2.01</v>
+        <v>1.85</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -26705,7 +26727,7 @@
         </is>
       </c>
       <c r="G90" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H90" s="34" t="inlineStr">
         <is>
@@ -26742,7 +26764,7 @@
         </is>
       </c>
       <c r="G91" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H91" s="34" t="inlineStr">
         <is>
@@ -26771,7 +26793,7 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
-        <v>0.015172</v>
+        <v>0.013988</v>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
@@ -26779,7 +26801,7 @@
         </is>
       </c>
       <c r="G92" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H92" s="34" t="inlineStr">
         <is>
@@ -26808,7 +26830,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>3.164449</v>
+        <v>2.925775</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -26816,7 +26838,7 @@
         </is>
       </c>
       <c r="G93" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H93" s="34" t="inlineStr">
         <is>
@@ -26845,7 +26867,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>27.289985</v>
+        <v>25.756644</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -26853,7 +26875,7 @@
         </is>
       </c>
       <c r="G94" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H94" s="34" t="inlineStr">
         <is>
@@ -26882,7 +26904,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.121014</v>
+        <v>0.115243</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -26890,7 +26912,7 @@
         </is>
       </c>
       <c r="G95" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H95" s="34" t="inlineStr">
         <is>
@@ -26919,7 +26941,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>20977.7736</v>
+        <v>19796.2368</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -26927,7 +26949,7 @@
         </is>
       </c>
       <c r="G96" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H96" s="34" t="inlineStr">
         <is>
@@ -26956,7 +26978,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2195970.08</v>
+        <v>2054493.56</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -26964,7 +26986,7 @@
         </is>
       </c>
       <c r="G97" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H97" s="34" t="inlineStr">
         <is>
@@ -26993,7 +27015,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>3.079476</v>
+        <v>2.901363</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -27001,7 +27023,7 @@
         </is>
       </c>
       <c r="G98" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H98" s="34" t="inlineStr">
         <is>
@@ -27030,7 +27052,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>61527.3424</v>
+        <v>57647.8468</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -27038,7 +27060,7 @@
         </is>
       </c>
       <c r="G99" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H99" s="34" t="inlineStr">
         <is>
@@ -27067,7 +27089,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>25.664161</v>
+        <v>25.105952</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -27075,7 +27097,7 @@
         </is>
       </c>
       <c r="G100" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H100" s="34" t="inlineStr">
         <is>
@@ -27104,7 +27126,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>67114</v>
+        <v>62867</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -27112,7 +27134,7 @@
         </is>
       </c>
       <c r="G101" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H101" s="34" t="inlineStr">
         <is>
@@ -27141,7 +27163,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>18.13</v>
+        <v>17.34</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -27149,7 +27171,7 @@
         </is>
       </c>
       <c r="G102" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H102" s="34" t="inlineStr">
         <is>
@@ -27252,7 +27274,7 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
-        <v>0.007194</v>
+        <v>0.006807</v>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
@@ -27260,7 +27282,7 @@
         </is>
       </c>
       <c r="G105" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H105" s="34" t="inlineStr">
         <is>
@@ -27289,7 +27311,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>75.3</v>
+        <v>69.22</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>
@@ -27297,7 +27319,7 @@
         </is>
       </c>
       <c r="G106" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H106" s="34" t="inlineStr">
         <is>
@@ -27334,7 +27356,7 @@
         </is>
       </c>
       <c r="G107" s="28" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="H107" s="34" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Weekly dashboard update — 2026-06-04
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-42660" yWindow="-540" windowWidth="32460" windowHeight="17180" tabRatio="500" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Realized" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Realized" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Prices" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Reference" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="AsOfDate">'FX &amp; Assumptions'!$C$5</definedName>
@@ -697,14 +697,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -726,8 +726,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -752,10 +752,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -764,10 +764,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4F81BD"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+              <a:ln w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -777,10 +777,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="C0504D"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -790,10 +790,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="9BBB59"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -803,10 +803,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="8064A2"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -816,10 +816,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4BACC6"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -829,10 +829,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="F79646"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -842,14 +842,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -875,14 +875,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -908,14 +908,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -941,14 +941,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -974,14 +974,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1007,14 +1007,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1038,16 +1038,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1142,16 +1142,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1172,10 +1172,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1187,14 +1187,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1216,8 +1216,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1242,10 +1242,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1254,10 +1254,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4672A8"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1267,10 +1267,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="AB4744"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1280,10 +1280,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="8AA64F"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1293,10 +1293,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="725990"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1306,10 +1306,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4299B0"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1319,10 +1319,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="DC853E"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1332,10 +1332,10 @@
             <idx val="6"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="93A9CE"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1345,10 +1345,10 @@
             <idx val="7"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="D09493"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1358,10 +1358,10 @@
             <idx val="8"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="B8CD97"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1371,14 +1371,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1405,14 +1405,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1439,14 +1439,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1473,14 +1473,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1507,14 +1507,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1541,14 +1541,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1575,14 +1575,14 @@
             <dLbl>
               <idx val="6"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1609,14 +1609,14 @@
             <dLbl>
               <idx val="7"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1643,14 +1643,14 @@
             <dLbl>
               <idx val="8"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1675,16 +1675,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1791,16 +1791,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1821,10 +1821,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1836,14 +1836,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1865,8 +1865,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1893,10 +1893,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1904,16 +1904,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2016,7 +2016,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2025,9 +2025,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2059,7 +2059,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2073,7 +2073,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2082,9 +2082,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2109,16 +2109,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2139,10 +2139,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2154,14 +2154,14 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -2183,8 +2183,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -2200,10 +2200,10 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2211,16 +2211,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2411,7 +2411,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2420,9 +2420,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2454,7 +2454,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2468,7 +2468,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2477,9 +2477,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2504,16 +2504,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2534,10 +2534,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2549,7 +2549,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>1</col>
@@ -2569,9 +2569,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2596,9 +2596,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+          <c:chart r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2623,9 +2623,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+          <c:chart r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2650,9 +2650,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+          <c:chart r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -21588,28 +21588,28 @@
         <v>46177</v>
       </c>
       <c r="C8" s="29" t="n">
-        <v>26900424</v>
+        <v>26880386</v>
       </c>
       <c r="D8" s="29" t="n">
-        <v>22657814</v>
+        <v>22646486</v>
       </c>
       <c r="E8" s="29" t="n">
-        <v>4242610</v>
+        <v>4233900</v>
       </c>
       <c r="F8" s="30" t="n">
-        <v>0.1872</v>
+        <v>0.187</v>
       </c>
       <c r="G8" s="29" t="n">
         <v>19094011</v>
       </c>
       <c r="H8" s="29" t="n">
-        <v>5224964</v>
+        <v>5201051</v>
       </c>
       <c r="I8" s="29" t="n">
-        <v>1162725</v>
+        <v>1174852</v>
       </c>
       <c r="J8" s="31" t="n">
-        <v>32.68</v>
+        <v>32.59</v>
       </c>
       <c r="K8" s="32" t="inlineStr">
         <is>
@@ -23416,7 +23416,7 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>32.68</v>
+        <v>32.59</v>
       </c>
       <c r="D6" s="64" t="inlineStr">
         <is>
@@ -23465,7 +23465,7 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>25.4804</v>
+        <v>25.4117</v>
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
@@ -24832,7 +24832,7 @@
         </is>
       </c>
       <c r="E39" s="33" t="n">
-        <v>1.106</v>
+        <v>1.088</v>
       </c>
       <c r="F39" s="34" t="inlineStr">
         <is>
@@ -24980,7 +24980,7 @@
         </is>
       </c>
       <c r="E43" s="33" t="n">
-        <v>5.75</v>
+        <v>5.7</v>
       </c>
       <c r="F43" s="34" t="inlineStr">
         <is>
@@ -25017,7 +25017,7 @@
         </is>
       </c>
       <c r="E44" s="33" t="n">
-        <v>175.5</v>
+        <v>174.5</v>
       </c>
       <c r="F44" s="34" t="inlineStr">
         <is>
@@ -25054,7 +25054,7 @@
         </is>
       </c>
       <c r="E45" s="33" t="n">
-        <v>0.45</v>
+        <v>0.46</v>
       </c>
       <c r="F45" s="34" t="inlineStr">
         <is>
@@ -25091,7 +25091,7 @@
         </is>
       </c>
       <c r="E46" s="33" t="n">
-        <v>0.3</v>
+        <v>0.31</v>
       </c>
       <c r="F46" s="34" t="inlineStr">
         <is>
@@ -25202,7 +25202,7 @@
         </is>
       </c>
       <c r="E49" s="33" t="n">
-        <v>64.5</v>
+        <v>67.25</v>
       </c>
       <c r="F49" s="34" t="inlineStr">
         <is>
@@ -25239,7 +25239,7 @@
         </is>
       </c>
       <c r="E50" s="33" t="n">
-        <v>9.550000000000001</v>
+        <v>9.6</v>
       </c>
       <c r="F50" s="34" t="inlineStr">
         <is>
@@ -25276,7 +25276,7 @@
         </is>
       </c>
       <c r="E51" s="33" t="n">
-        <v>15.5</v>
+        <v>15.3</v>
       </c>
       <c r="F51" s="34" t="inlineStr">
         <is>
@@ -25313,7 +25313,7 @@
         </is>
       </c>
       <c r="E52" s="33" t="n">
-        <v>12.9</v>
+        <v>13.4</v>
       </c>
       <c r="F52" s="34" t="inlineStr">
         <is>
@@ -25350,7 +25350,7 @@
         </is>
       </c>
       <c r="E53" s="33" t="n">
-        <v>5.65</v>
+        <v>6.15</v>
       </c>
       <c r="F53" s="34" t="inlineStr">
         <is>
@@ -25387,7 +25387,7 @@
         </is>
       </c>
       <c r="E54" s="33" t="n">
-        <v>21.9</v>
+        <v>21.3</v>
       </c>
       <c r="F54" s="34" t="inlineStr">
         <is>
@@ -25424,7 +25424,7 @@
         </is>
       </c>
       <c r="E55" s="33" t="n">
-        <v>3.52</v>
+        <v>3.56</v>
       </c>
       <c r="F55" s="34" t="inlineStr">
         <is>
@@ -25461,7 +25461,7 @@
         </is>
       </c>
       <c r="E56" s="33" t="n">
-        <v>4.94</v>
+        <v>5</v>
       </c>
       <c r="F56" s="34" t="inlineStr">
         <is>
@@ -25498,7 +25498,7 @@
         </is>
       </c>
       <c r="E57" s="33" t="n">
-        <v>2.76</v>
+        <v>2.74</v>
       </c>
       <c r="F57" s="34" t="inlineStr">
         <is>
@@ -25535,7 +25535,7 @@
         </is>
       </c>
       <c r="E58" s="33" t="n">
-        <v>12.5</v>
+        <v>12.4</v>
       </c>
       <c r="F58" s="34" t="inlineStr">
         <is>
@@ -25572,7 +25572,7 @@
         </is>
       </c>
       <c r="E59" s="33" t="n">
-        <v>17.8</v>
+        <v>17.5</v>
       </c>
       <c r="F59" s="34" t="inlineStr">
         <is>
@@ -25609,7 +25609,7 @@
         </is>
       </c>
       <c r="E60" s="33" t="n">
-        <v>159.19</v>
+        <v>153.01</v>
       </c>
       <c r="F60" s="34" t="inlineStr">
         <is>
@@ -25646,7 +25646,7 @@
         </is>
       </c>
       <c r="E61" s="33" t="n">
-        <v>256.24</v>
+        <v>264.29</v>
       </c>
       <c r="F61" s="34" t="inlineStr">
         <is>
@@ -25683,7 +25683,7 @@
         </is>
       </c>
       <c r="E62" s="33" t="n">
-        <v>500.77</v>
+        <v>483.685</v>
       </c>
       <c r="F62" s="34" t="inlineStr">
         <is>
@@ -25720,7 +25720,7 @@
         </is>
       </c>
       <c r="E63" s="33" t="n">
-        <v>178.9</v>
+        <v>173.605</v>
       </c>
       <c r="F63" s="34" t="inlineStr">
         <is>
@@ -25757,7 +25757,7 @@
         </is>
       </c>
       <c r="E64" s="33" t="n">
-        <v>69.02</v>
+        <v>66.64</v>
       </c>
       <c r="F64" s="34" t="inlineStr">
         <is>
@@ -25794,7 +25794,7 @@
         </is>
       </c>
       <c r="E65" s="33" t="n">
-        <v>212.96</v>
+        <v>197.83</v>
       </c>
       <c r="F65" s="34" t="inlineStr">
         <is>
@@ -25831,7 +25831,7 @@
         </is>
       </c>
       <c r="E66" s="33" t="n">
-        <v>146.48</v>
+        <v>147.59</v>
       </c>
       <c r="F66" s="34" t="inlineStr">
         <is>
@@ -25868,7 +25868,7 @@
         </is>
       </c>
       <c r="E67" s="33" t="n">
-        <v>164.75</v>
+        <v>170.17</v>
       </c>
       <c r="F67" s="34" t="inlineStr">
         <is>
@@ -25905,7 +25905,7 @@
         </is>
       </c>
       <c r="E68" s="33" t="n">
-        <v>2125.11</v>
+        <v>2038.517</v>
       </c>
       <c r="F68" s="34" t="inlineStr">
         <is>
@@ -25942,7 +25942,7 @@
         </is>
       </c>
       <c r="E69" s="33" t="n">
-        <v>1078.78</v>
+        <v>1121.47</v>
       </c>
       <c r="F69" s="34" t="inlineStr">
         <is>
@@ -25979,7 +25979,7 @@
         </is>
       </c>
       <c r="E70" s="33" t="n">
-        <v>96.55</v>
+        <v>96.45999999999999</v>
       </c>
       <c r="F70" s="34" t="inlineStr">
         <is>
@@ -26016,7 +26016,7 @@
         </is>
       </c>
       <c r="E71" s="33" t="n">
-        <v>1689.89</v>
+        <v>1601.395</v>
       </c>
       <c r="F71" s="34" t="inlineStr">
         <is>
@@ -26053,7 +26053,7 @@
         </is>
       </c>
       <c r="E72" s="33" t="n">
-        <v>115.6</v>
+        <v>115.53</v>
       </c>
       <c r="F72" s="34" t="inlineStr">
         <is>
@@ -26090,7 +26090,7 @@
         </is>
       </c>
       <c r="E73" s="33" t="n">
-        <v>214.75</v>
+        <v>212.04</v>
       </c>
       <c r="F73" s="34" t="inlineStr">
         <is>
@@ -26127,7 +26127,7 @@
         </is>
       </c>
       <c r="E74" s="33" t="n">
-        <v>90.84</v>
+        <v>89.705</v>
       </c>
       <c r="F74" s="34" t="inlineStr">
         <is>
@@ -26164,7 +26164,7 @@
         </is>
       </c>
       <c r="E75" s="33" t="n">
-        <v>104.73</v>
+        <v>103.52</v>
       </c>
       <c r="F75" s="34" t="inlineStr">
         <is>
@@ -26201,7 +26201,7 @@
         </is>
       </c>
       <c r="E76" s="33" t="n">
-        <v>409.67</v>
+        <v>391.3</v>
       </c>
       <c r="F76" s="34" t="inlineStr">
         <is>
@@ -26238,7 +26238,7 @@
         </is>
       </c>
       <c r="E77" s="33" t="n">
-        <v>423.7</v>
+        <v>422.13</v>
       </c>
       <c r="F77" s="34" t="inlineStr">
         <is>
@@ -26275,7 +26275,7 @@
         </is>
       </c>
       <c r="E78" s="33" t="n">
-        <v>56.08</v>
+        <v>56.19</v>
       </c>
       <c r="F78" s="34" t="inlineStr">
         <is>
@@ -26312,7 +26312,7 @@
         </is>
       </c>
       <c r="E79" s="33" t="n">
-        <v>98.31999999999999</v>
+        <v>96.86</v>
       </c>
       <c r="F79" s="34" t="inlineStr">
         <is>
@@ -26349,7 +26349,7 @@
         </is>
       </c>
       <c r="E80" s="33" t="n">
-        <v>310.26</v>
+        <v>311.495</v>
       </c>
       <c r="F80" s="34" t="inlineStr">
         <is>
@@ -26386,7 +26386,7 @@
         </is>
       </c>
       <c r="E81" s="33" t="n">
-        <v>163.22</v>
+        <v>165.53</v>
       </c>
       <c r="F81" s="34" t="inlineStr">
         <is>
@@ -26423,7 +26423,7 @@
         </is>
       </c>
       <c r="E82" s="33" t="n">
-        <v>622.98</v>
+        <v>637.15</v>
       </c>
       <c r="F82" s="34" t="inlineStr">
         <is>
@@ -26460,7 +26460,7 @@
         </is>
       </c>
       <c r="E83" s="33" t="n">
-        <v>155.99</v>
+        <v>162.5</v>
       </c>
       <c r="F83" s="34" t="inlineStr">
         <is>
@@ -26497,7 +26497,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>71.29000000000001</v>
+        <v>72.23</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -26534,7 +26534,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>605.76</v>
+        <v>604.16</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -26571,7 +26571,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>62867</v>
+        <v>64258</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -26608,7 +26608,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.006807</v>
+        <v>0.006831</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -26645,7 +26645,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.012284</v>
+        <v>0.011957</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -26682,7 +26682,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>69.22</v>
+        <v>70.31999999999999</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -26719,7 +26719,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>1.85</v>
+        <v>1.84</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -26793,7 +26793,7 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
-        <v>0.013988</v>
+        <v>0.014259</v>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
@@ -26830,7 +26830,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>2.925775</v>
+        <v>2.962105</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -26867,7 +26867,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>25.756644</v>
+        <v>25.905433</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -26904,7 +26904,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.115243</v>
+        <v>0.117904</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -26941,7 +26941,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>19796.2368</v>
+        <v>19689.5744</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -26978,7 +26978,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2054493.56</v>
+        <v>2094168.22</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -27015,7 +27015,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>2.901363</v>
+        <v>2.910645</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -27052,7 +27052,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>57647.8468</v>
+        <v>58179.9939</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -27089,7 +27089,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>25.105952</v>
+        <v>25.690273</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -27126,7 +27126,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>62867</v>
+        <v>64258</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -27163,7 +27163,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>17.34</v>
+        <v>17.52</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -27274,7 +27274,7 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
-        <v>0.006807</v>
+        <v>0.006831</v>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
@@ -27311,7 +27311,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>69.22</v>
+        <v>70.31999999999999</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Daily dashboard update — 2026-06-05 (manual; GitHub scheduler ran 12h late)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-42660" yWindow="-540" windowWidth="32460" windowHeight="17180" tabRatio="500" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Realized" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Prices" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Reference" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Realized" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="AsOfDate">'FX &amp; Assumptions'!$C$5</definedName>
@@ -697,14 +697,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -726,8 +726,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -752,10 +752,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -764,10 +764,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4F81BD"/>
               </a:solidFill>
-              <a:ln w="0">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -777,10 +777,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="C0504D"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -790,10 +790,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="9BBB59"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -803,10 +803,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="8064A2"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -816,10 +816,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4BACC6"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -829,10 +829,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="F79646"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -842,14 +842,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -875,14 +875,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -908,14 +908,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -941,14 +941,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -974,14 +974,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1007,14 +1007,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1038,16 +1038,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1142,16 +1142,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1172,10 +1172,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1187,14 +1187,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1216,8 +1216,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1242,10 +1242,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1254,10 +1254,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4672A8"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1267,10 +1267,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="AB4744"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1280,10 +1280,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="8AA64F"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1293,10 +1293,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="725990"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1306,10 +1306,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4299B0"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1319,10 +1319,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="DC853E"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1332,10 +1332,10 @@
             <idx val="6"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="93A9CE"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1345,10 +1345,10 @@
             <idx val="7"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="D09493"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1358,10 +1358,10 @@
             <idx val="8"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="B8CD97"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1371,14 +1371,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1405,14 +1405,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1439,14 +1439,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1473,14 +1473,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1507,14 +1507,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1541,14 +1541,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1575,14 +1575,14 @@
             <dLbl>
               <idx val="6"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1609,14 +1609,14 @@
             <dLbl>
               <idx val="7"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1643,14 +1643,14 @@
             <dLbl>
               <idx val="8"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1675,16 +1675,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1791,16 +1791,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1821,10 +1821,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1836,14 +1836,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1865,8 +1865,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1893,10 +1893,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1904,16 +1904,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2016,7 +2016,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2025,9 +2025,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2059,7 +2059,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="9360">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2073,7 +2073,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2082,9 +2082,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2109,16 +2109,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2139,10 +2139,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2154,14 +2154,14 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -2183,8 +2183,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -2200,10 +2200,10 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2211,16 +2211,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2411,7 +2411,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2420,9 +2420,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2454,7 +2454,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="9360">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2468,7 +2468,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2477,9 +2477,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2504,16 +2504,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2534,10 +2534,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2549,7 +2549,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>1</col>
@@ -2569,9 +2569,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2596,9 +2596,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2623,9 +2623,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId3"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2650,9 +2650,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId4"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -21618,16 +21618,38 @@
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="58">
-      <c r="B9" s="28" t="n"/>
-      <c r="C9" s="29" t="n"/>
-      <c r="D9" s="29" t="n"/>
-      <c r="E9" s="29" t="n"/>
-      <c r="F9" s="30" t="n"/>
-      <c r="G9" s="29" t="n"/>
-      <c r="H9" s="29" t="n"/>
-      <c r="I9" s="29" t="n"/>
-      <c r="J9" s="31" t="n"/>
-      <c r="K9" s="32" t="n"/>
+      <c r="B9" s="28" t="n">
+        <v>46178</v>
+      </c>
+      <c r="C9" s="29" t="n">
+        <v>26888175</v>
+      </c>
+      <c r="D9" s="29" t="n">
+        <v>22653511</v>
+      </c>
+      <c r="E9" s="29" t="n">
+        <v>4234664</v>
+      </c>
+      <c r="F9" s="30" t="n">
+        <v>0.1869</v>
+      </c>
+      <c r="G9" s="29" t="n">
+        <v>19094011</v>
+      </c>
+      <c r="H9" s="29" t="n">
+        <v>5238037</v>
+      </c>
+      <c r="I9" s="29" t="n">
+        <v>1163780</v>
+      </c>
+      <c r="J9" s="31" t="n">
+        <v>32.66</v>
+      </c>
+      <c r="K9" s="32" t="inlineStr">
+        <is>
+          <t>Auto weekly snapshot</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="58">
       <c r="B10" s="28" t="n"/>
@@ -23401,7 +23423,7 @@
         </is>
       </c>
       <c r="C5" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="D5" s="64" t="inlineStr">
         <is>
@@ -23416,11 +23438,11 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>32.59</v>
+        <v>32.66</v>
       </c>
       <c r="D6" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-06-04</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-06-05</t>
         </is>
       </c>
     </row>
@@ -23465,11 +23487,11 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>25.4117</v>
+        <v>25.4112</v>
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-06-04</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-06-05</t>
         </is>
       </c>
     </row>
@@ -24795,7 +24817,7 @@
         </is>
       </c>
       <c r="E38" s="33" t="n">
-        <v>22.59</v>
+        <v>22.56</v>
       </c>
       <c r="F38" s="34" t="inlineStr">
         <is>
@@ -24803,7 +24825,7 @@
         </is>
       </c>
       <c r="G38" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H38" s="34" t="inlineStr">
         <is>
@@ -24840,7 +24862,7 @@
         </is>
       </c>
       <c r="G39" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H39" s="34" t="inlineStr">
         <is>
@@ -24869,7 +24891,7 @@
         </is>
       </c>
       <c r="E40" s="33" t="n">
-        <v>803.14</v>
+        <v>785.53</v>
       </c>
       <c r="F40" s="34" t="inlineStr">
         <is>
@@ -24877,7 +24899,7 @@
         </is>
       </c>
       <c r="G40" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H40" s="34" t="inlineStr">
         <is>
@@ -24906,7 +24928,7 @@
         </is>
       </c>
       <c r="E41" s="33" t="n">
-        <v>22.02</v>
+        <v>21.64</v>
       </c>
       <c r="F41" s="34" t="inlineStr">
         <is>
@@ -24914,7 +24936,7 @@
         </is>
       </c>
       <c r="G41" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H41" s="34" t="inlineStr">
         <is>
@@ -24943,7 +24965,7 @@
         </is>
       </c>
       <c r="E42" s="33" t="n">
-        <v>228.38</v>
+        <v>224.22</v>
       </c>
       <c r="F42" s="34" t="inlineStr">
         <is>
@@ -24951,7 +24973,7 @@
         </is>
       </c>
       <c r="G42" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H42" s="34" t="inlineStr">
         <is>
@@ -24988,7 +25010,7 @@
         </is>
       </c>
       <c r="G43" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H43" s="34" t="inlineStr">
         <is>
@@ -25025,7 +25047,7 @@
         </is>
       </c>
       <c r="G44" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H44" s="34" t="inlineStr">
         <is>
@@ -25062,7 +25084,7 @@
         </is>
       </c>
       <c r="G45" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H45" s="34" t="inlineStr">
         <is>
@@ -25099,7 +25121,7 @@
         </is>
       </c>
       <c r="G46" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H46" s="34" t="inlineStr">
         <is>
@@ -25173,7 +25195,7 @@
         </is>
       </c>
       <c r="G48" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H48" s="34" t="inlineStr">
         <is>
@@ -25210,7 +25232,7 @@
         </is>
       </c>
       <c r="G49" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H49" s="34" t="inlineStr">
         <is>
@@ -25247,7 +25269,7 @@
         </is>
       </c>
       <c r="G50" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H50" s="34" t="inlineStr">
         <is>
@@ -25284,7 +25306,7 @@
         </is>
       </c>
       <c r="G51" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H51" s="34" t="inlineStr">
         <is>
@@ -25321,7 +25343,7 @@
         </is>
       </c>
       <c r="G52" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H52" s="34" t="inlineStr">
         <is>
@@ -25358,7 +25380,7 @@
         </is>
       </c>
       <c r="G53" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H53" s="34" t="inlineStr">
         <is>
@@ -25395,7 +25417,7 @@
         </is>
       </c>
       <c r="G54" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H54" s="34" t="inlineStr">
         <is>
@@ -25432,7 +25454,7 @@
         </is>
       </c>
       <c r="G55" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H55" s="34" t="inlineStr">
         <is>
@@ -25469,7 +25491,7 @@
         </is>
       </c>
       <c r="G56" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H56" s="34" t="inlineStr">
         <is>
@@ -25506,7 +25528,7 @@
         </is>
       </c>
       <c r="G57" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H57" s="34" t="inlineStr">
         <is>
@@ -25543,7 +25565,7 @@
         </is>
       </c>
       <c r="G58" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H58" s="34" t="inlineStr">
         <is>
@@ -25580,7 +25602,7 @@
         </is>
       </c>
       <c r="G59" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H59" s="34" t="inlineStr">
         <is>
@@ -25609,7 +25631,7 @@
         </is>
       </c>
       <c r="E60" s="33" t="n">
-        <v>153.01</v>
+        <v>161.87</v>
       </c>
       <c r="F60" s="34" t="inlineStr">
         <is>
@@ -25617,7 +25639,7 @@
         </is>
       </c>
       <c r="G60" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H60" s="34" t="inlineStr">
         <is>
@@ -25646,7 +25668,7 @@
         </is>
       </c>
       <c r="E61" s="33" t="n">
-        <v>264.29</v>
+        <v>258.42</v>
       </c>
       <c r="F61" s="34" t="inlineStr">
         <is>
@@ -25654,7 +25676,7 @@
         </is>
       </c>
       <c r="G61" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H61" s="34" t="inlineStr">
         <is>
@@ -25683,7 +25705,7 @@
         </is>
       </c>
       <c r="E62" s="33" t="n">
-        <v>483.685</v>
+        <v>501.7</v>
       </c>
       <c r="F62" s="34" t="inlineStr">
         <is>
@@ -25691,7 +25713,7 @@
         </is>
       </c>
       <c r="G62" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H62" s="34" t="inlineStr">
         <is>
@@ -25720,7 +25742,7 @@
         </is>
       </c>
       <c r="E63" s="33" t="n">
-        <v>173.605</v>
+        <v>175.63</v>
       </c>
       <c r="F63" s="34" t="inlineStr">
         <is>
@@ -25728,7 +25750,7 @@
         </is>
       </c>
       <c r="G63" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H63" s="34" t="inlineStr">
         <is>
@@ -25757,7 +25779,7 @@
         </is>
       </c>
       <c r="E64" s="33" t="n">
-        <v>66.64</v>
+        <v>68.39</v>
       </c>
       <c r="F64" s="34" t="inlineStr">
         <is>
@@ -25765,7 +25787,7 @@
         </is>
       </c>
       <c r="G64" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H64" s="34" t="inlineStr">
         <is>
@@ -25794,7 +25816,7 @@
         </is>
       </c>
       <c r="E65" s="33" t="n">
-        <v>197.83</v>
+        <v>203.97</v>
       </c>
       <c r="F65" s="34" t="inlineStr">
         <is>
@@ -25802,7 +25824,7 @@
         </is>
       </c>
       <c r="G65" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H65" s="34" t="inlineStr">
         <is>
@@ -25831,7 +25853,7 @@
         </is>
       </c>
       <c r="E66" s="33" t="n">
-        <v>147.59</v>
+        <v>149.67</v>
       </c>
       <c r="F66" s="34" t="inlineStr">
         <is>
@@ -25839,7 +25861,7 @@
         </is>
       </c>
       <c r="G66" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H66" s="34" t="inlineStr">
         <is>
@@ -25868,7 +25890,7 @@
         </is>
       </c>
       <c r="E67" s="33" t="n">
-        <v>170.17</v>
+        <v>164.87</v>
       </c>
       <c r="F67" s="34" t="inlineStr">
         <is>
@@ -25876,7 +25898,7 @@
         </is>
       </c>
       <c r="G67" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H67" s="34" t="inlineStr">
         <is>
@@ -25905,7 +25927,7 @@
         </is>
       </c>
       <c r="E68" s="33" t="n">
-        <v>2038.517</v>
+        <v>2131.1</v>
       </c>
       <c r="F68" s="34" t="inlineStr">
         <is>
@@ -25913,7 +25935,7 @@
         </is>
       </c>
       <c r="G68" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H68" s="34" t="inlineStr">
         <is>
@@ -25942,7 +25964,7 @@
         </is>
       </c>
       <c r="E69" s="33" t="n">
-        <v>1121.47</v>
+        <v>1125.27</v>
       </c>
       <c r="F69" s="34" t="inlineStr">
         <is>
@@ -25950,7 +25972,7 @@
         </is>
       </c>
       <c r="G69" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H69" s="34" t="inlineStr">
         <is>
@@ -25979,7 +26001,7 @@
         </is>
       </c>
       <c r="E70" s="33" t="n">
-        <v>96.45999999999999</v>
+        <v>96.3</v>
       </c>
       <c r="F70" s="34" t="inlineStr">
         <is>
@@ -25987,7 +26009,7 @@
         </is>
       </c>
       <c r="G70" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H70" s="34" t="inlineStr">
         <is>
@@ -26016,7 +26038,7 @@
         </is>
       </c>
       <c r="E71" s="33" t="n">
-        <v>1601.395</v>
+        <v>1652.6</v>
       </c>
       <c r="F71" s="34" t="inlineStr">
         <is>
@@ -26024,7 +26046,7 @@
         </is>
       </c>
       <c r="G71" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H71" s="34" t="inlineStr">
         <is>
@@ -26053,7 +26075,7 @@
         </is>
       </c>
       <c r="E72" s="33" t="n">
-        <v>115.53</v>
+        <v>118.83</v>
       </c>
       <c r="F72" s="34" t="inlineStr">
         <is>
@@ -26061,7 +26083,7 @@
         </is>
       </c>
       <c r="G72" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H72" s="34" t="inlineStr">
         <is>
@@ -26090,7 +26112,7 @@
         </is>
       </c>
       <c r="E73" s="33" t="n">
-        <v>212.04</v>
+        <v>218.66</v>
       </c>
       <c r="F73" s="34" t="inlineStr">
         <is>
@@ -26098,7 +26120,7 @@
         </is>
       </c>
       <c r="G73" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H73" s="34" t="inlineStr">
         <is>
@@ -26127,7 +26149,7 @@
         </is>
       </c>
       <c r="E74" s="33" t="n">
-        <v>89.705</v>
+        <v>90.2</v>
       </c>
       <c r="F74" s="34" t="inlineStr">
         <is>
@@ -26135,7 +26157,7 @@
         </is>
       </c>
       <c r="G74" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H74" s="34" t="inlineStr">
         <is>
@@ -26164,7 +26186,7 @@
         </is>
       </c>
       <c r="E75" s="33" t="n">
-        <v>103.52</v>
+        <v>103.97</v>
       </c>
       <c r="F75" s="34" t="inlineStr">
         <is>
@@ -26172,7 +26194,7 @@
         </is>
       </c>
       <c r="G75" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H75" s="34" t="inlineStr">
         <is>
@@ -26201,7 +26223,7 @@
         </is>
       </c>
       <c r="E76" s="33" t="n">
-        <v>391.3</v>
+        <v>406.86</v>
       </c>
       <c r="F76" s="34" t="inlineStr">
         <is>
@@ -26209,7 +26231,7 @@
         </is>
       </c>
       <c r="G76" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H76" s="34" t="inlineStr">
         <is>
@@ -26238,7 +26260,7 @@
         </is>
       </c>
       <c r="E77" s="33" t="n">
-        <v>422.13</v>
+        <v>418.45</v>
       </c>
       <c r="F77" s="34" t="inlineStr">
         <is>
@@ -26246,7 +26268,7 @@
         </is>
       </c>
       <c r="G77" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H77" s="34" t="inlineStr">
         <is>
@@ -26275,7 +26297,7 @@
         </is>
       </c>
       <c r="E78" s="33" t="n">
-        <v>56.19</v>
+        <v>54.48</v>
       </c>
       <c r="F78" s="34" t="inlineStr">
         <is>
@@ -26283,7 +26305,7 @@
         </is>
       </c>
       <c r="G78" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H78" s="34" t="inlineStr">
         <is>
@@ -26312,7 +26334,7 @@
         </is>
       </c>
       <c r="E79" s="33" t="n">
-        <v>96.86</v>
+        <v>97</v>
       </c>
       <c r="F79" s="34" t="inlineStr">
         <is>
@@ -26320,7 +26342,7 @@
         </is>
       </c>
       <c r="G79" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H79" s="34" t="inlineStr">
         <is>
@@ -26349,7 +26371,7 @@
         </is>
       </c>
       <c r="E80" s="33" t="n">
-        <v>311.495</v>
+        <v>311.23</v>
       </c>
       <c r="F80" s="34" t="inlineStr">
         <is>
@@ -26357,7 +26379,7 @@
         </is>
       </c>
       <c r="G80" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H80" s="34" t="inlineStr">
         <is>
@@ -26386,7 +26408,7 @@
         </is>
       </c>
       <c r="E81" s="33" t="n">
-        <v>165.53</v>
+        <v>164.13</v>
       </c>
       <c r="F81" s="34" t="inlineStr">
         <is>
@@ -26394,7 +26416,7 @@
         </is>
       </c>
       <c r="G81" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H81" s="34" t="inlineStr">
         <is>
@@ -26423,7 +26445,7 @@
         </is>
       </c>
       <c r="E82" s="33" t="n">
-        <v>637.15</v>
+        <v>627.5700000000001</v>
       </c>
       <c r="F82" s="34" t="inlineStr">
         <is>
@@ -26431,7 +26453,7 @@
         </is>
       </c>
       <c r="G82" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H82" s="34" t="inlineStr">
         <is>
@@ -26460,7 +26482,7 @@
         </is>
       </c>
       <c r="E83" s="33" t="n">
-        <v>162.5</v>
+        <v>166</v>
       </c>
       <c r="F83" s="34" t="inlineStr">
         <is>
@@ -26468,7 +26490,7 @@
         </is>
       </c>
       <c r="G83" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H83" s="34" t="inlineStr">
         <is>
@@ -26497,7 +26519,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>72.23</v>
+        <v>70.64</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -26505,7 +26527,7 @@
         </is>
       </c>
       <c r="G84" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H84" s="34" t="inlineStr">
         <is>
@@ -26534,7 +26556,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>604.16</v>
+        <v>600.65</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -26542,7 +26564,7 @@
         </is>
       </c>
       <c r="G85" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H85" s="34" t="inlineStr">
         <is>
@@ -26571,7 +26593,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>64258</v>
+        <v>63277</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -26579,7 +26601,7 @@
         </is>
       </c>
       <c r="G86" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H86" s="34" t="inlineStr">
         <is>
@@ -26608,7 +26630,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.006831</v>
+        <v>0.006722</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -26616,7 +26638,7 @@
         </is>
       </c>
       <c r="G87" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H87" s="34" t="inlineStr">
         <is>
@@ -26645,7 +26667,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.011957</v>
+        <v>0.012172</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -26653,7 +26675,7 @@
         </is>
       </c>
       <c r="G88" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H88" s="34" t="inlineStr">
         <is>
@@ -26682,7 +26704,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>70.31999999999999</v>
+        <v>68.37</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -26690,7 +26712,7 @@
         </is>
       </c>
       <c r="G89" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H89" s="34" t="inlineStr">
         <is>
@@ -26719,7 +26741,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>1.84</v>
+        <v>1.8</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -26727,7 +26749,7 @@
         </is>
       </c>
       <c r="G90" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H90" s="34" t="inlineStr">
         <is>
@@ -26764,7 +26786,7 @@
         </is>
       </c>
       <c r="G91" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H91" s="34" t="inlineStr">
         <is>
@@ -26793,7 +26815,7 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
-        <v>0.014259</v>
+        <v>0.013907</v>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
@@ -26801,7 +26823,7 @@
         </is>
       </c>
       <c r="G92" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H92" s="34" t="inlineStr">
         <is>
@@ -26830,7 +26852,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>2.962105</v>
+        <v>2.899816</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -26838,7 +26860,7 @@
         </is>
       </c>
       <c r="G93" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H93" s="34" t="inlineStr">
         <is>
@@ -26867,7 +26889,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>25.905433</v>
+        <v>24.707486</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -26875,7 +26897,7 @@
         </is>
       </c>
       <c r="G94" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H94" s="34" t="inlineStr">
         <is>
@@ -26904,7 +26926,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.117904</v>
+        <v>0.122682</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -26912,7 +26934,7 @@
         </is>
       </c>
       <c r="G95" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H95" s="34" t="inlineStr">
         <is>
@@ -26941,7 +26963,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>19689.5744</v>
+        <v>19617.229</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -26949,7 +26971,7 @@
         </is>
       </c>
       <c r="G96" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H96" s="34" t="inlineStr">
         <is>
@@ -26978,7 +27000,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2094168.22</v>
+        <v>2066626.82</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -26986,7 +27008,7 @@
         </is>
       </c>
       <c r="G97" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H97" s="34" t="inlineStr">
         <is>
@@ -27015,7 +27037,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>2.910645</v>
+        <v>2.864347</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -27023,7 +27045,7 @@
         </is>
       </c>
       <c r="G98" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H98" s="34" t="inlineStr">
         <is>
@@ -27052,7 +27074,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>58179.9939</v>
+        <v>57248.4076</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -27060,7 +27082,7 @@
         </is>
       </c>
       <c r="G99" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H99" s="34" t="inlineStr">
         <is>
@@ -27089,7 +27111,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>25.690273</v>
+        <v>25.729907</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -27097,7 +27119,7 @@
         </is>
       </c>
       <c r="G100" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H100" s="34" t="inlineStr">
         <is>
@@ -27126,7 +27148,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>64258</v>
+        <v>63277</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -27134,7 +27156,7 @@
         </is>
       </c>
       <c r="G101" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H101" s="34" t="inlineStr">
         <is>
@@ -27163,7 +27185,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>17.52</v>
+        <v>16.86</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -27171,7 +27193,7 @@
         </is>
       </c>
       <c r="G102" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H102" s="34" t="inlineStr">
         <is>
@@ -27274,7 +27296,7 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
-        <v>0.006831</v>
+        <v>0.006722</v>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
@@ -27282,7 +27304,7 @@
         </is>
       </c>
       <c r="G105" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H105" s="34" t="inlineStr">
         <is>
@@ -27311,7 +27333,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>70.31999999999999</v>
+        <v>68.37</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>
@@ -27319,7 +27341,7 @@
         </is>
       </c>
       <c r="G106" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H106" s="34" t="inlineStr">
         <is>
@@ -27356,7 +27378,7 @@
         </is>
       </c>
       <c r="G107" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H107" s="34" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Daily dashboard update — 2026-06-05
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -21622,28 +21622,28 @@
         <v>46178</v>
       </c>
       <c r="C9" s="29" t="n">
-        <v>26888175</v>
+        <v>26895438</v>
       </c>
       <c r="D9" s="29" t="n">
-        <v>22653511</v>
+        <v>22657903</v>
       </c>
       <c r="E9" s="29" t="n">
-        <v>4234664</v>
+        <v>4237535</v>
       </c>
       <c r="F9" s="30" t="n">
-        <v>0.1869</v>
+        <v>0.187</v>
       </c>
       <c r="G9" s="29" t="n">
         <v>19094011</v>
       </c>
       <c r="H9" s="29" t="n">
-        <v>5238037</v>
+        <v>5242410</v>
       </c>
       <c r="I9" s="29" t="n">
-        <v>1163780</v>
+        <v>1166062</v>
       </c>
       <c r="J9" s="31" t="n">
-        <v>32.66</v>
+        <v>32.7</v>
       </c>
       <c r="K9" s="32" t="inlineStr">
         <is>
@@ -23438,7 +23438,7 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>32.66</v>
+        <v>32.7</v>
       </c>
       <c r="D6" s="64" t="inlineStr">
         <is>
@@ -23487,7 +23487,7 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>25.4112</v>
+        <v>25.4223</v>
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
@@ -26519,7 +26519,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>70.64</v>
+        <v>70.72</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -26556,7 +26556,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>600.65</v>
+        <v>601.9299999999999</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -26593,7 +26593,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>63277</v>
+        <v>63306</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -26630,7 +26630,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.006722</v>
+        <v>0.006774</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -26667,7 +26667,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.012172</v>
+        <v>0.012182</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -26704,7 +26704,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>68.37</v>
+        <v>68.47</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -26741,7 +26741,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>1.8</v>
+        <v>1.81</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -26815,7 +26815,7 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
-        <v>0.013907</v>
+        <v>0.013948</v>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
@@ -26852,7 +26852,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>2.899816</v>
+        <v>2.910954</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -26889,7 +26889,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>24.707486</v>
+        <v>24.783363</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -26926,7 +26926,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.122682</v>
+        <v>0.122742</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -26963,7 +26963,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>19617.229</v>
+        <v>19683.111</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -27000,7 +27000,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2066626.82</v>
+        <v>2070106.2</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -27037,7 +27037,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>2.864347</v>
+        <v>2.871812</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -27074,7 +27074,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>57248.4076</v>
+        <v>57256.392</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -27111,7 +27111,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>25.729907</v>
+        <v>25.794251</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -27148,7 +27148,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>63277</v>
+        <v>63306</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -27185,7 +27185,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>16.86</v>
+        <v>16.91</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -27296,7 +27296,7 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
-        <v>0.006722</v>
+        <v>0.006774</v>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
@@ -27333,7 +27333,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>68.37</v>
+        <v>68.47</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Overview: Top Movers "Today" toggle — real per-holding 1-day moves
Adds a Today | Since inception toggle to the Top Movers card (defaults to
Today): real 1-day price/NAV move per holding with the THB contribution,
alongside the existing lifetime-return view.

Data plumbing (best-effort; never blocks the daily build):
- fetch_thai_nav: return the prior NAV (already in the SEC series response).
- fetch_prices: yahoo_quote() captures previousClose (equities + SGD UTs);
  CoinGecko include_24hr_change for crypto. Prior prices persisted to new
  auto-managed Prices cols I/J (Prev Price / Prev Date).
- portfolio: day_px_pct / day_thb per holding, recency-gated (current price
  fresh <=4d; prev->current step <=5d) so lagged/weekly NAVs don't show as
  "today's" move.
- build_site: pool the daily fields; Top Movers segmented toggle.

REFERENCE.md §4/§5/§8/§9 updated. Workbook reflects a live price refresh.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -23438,7 +23438,7 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>32.65</v>
+        <v>32.66</v>
       </c>
       <c r="D6" s="64" t="inlineStr">
         <is>
@@ -23487,7 +23487,7 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>25.4183</v>
+        <v>25.4261</v>
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
@@ -23513,7 +23513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:H109"/>
+  <dimension ref="A2:J109"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="58" min="1" max="1"/>
@@ -23574,6 +23574,16 @@
           <t>CHECK</t>
         </is>
       </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Prev Price</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Prev Date</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="58">
       <c r="A5" s="35">
@@ -23611,6 +23621,14 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I5" t="n">
+        <v>24.9174</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="58">
       <c r="A6" s="35">
@@ -23648,6 +23666,14 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I6" t="n">
+        <v>10.6854</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="58">
       <c r="A7" s="35">
@@ -23685,6 +23711,14 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I7" t="n">
+        <v>7.1767</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="58">
       <c r="A8" s="35">
@@ -23722,6 +23756,14 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I8" t="n">
+        <v>9.613200000000001</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="58">
       <c r="A9" s="35">
@@ -23759,6 +23801,14 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I9" t="n">
+        <v>9.4183</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="58">
       <c r="A10" s="35">
@@ -23796,6 +23846,14 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I10" t="n">
+        <v>13.4811</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="58">
       <c r="A11" s="35">
@@ -23833,6 +23891,14 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I11" t="n">
+        <v>13.3792</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="58">
       <c r="A12" s="35">
@@ -23870,6 +23936,14 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I12" t="n">
+        <v>26.9938</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="58">
       <c r="A13" s="35">
@@ -23907,6 +23981,14 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I13" t="n">
+        <v>36.3651</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="58">
       <c r="A14" s="35">
@@ -23944,6 +24026,14 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I14" t="n">
+        <v>25.4878</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="58">
       <c r="A15" s="35">
@@ -23981,6 +24071,14 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I15" t="n">
+        <v>14.9551</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="58">
       <c r="A16" s="35">
@@ -24018,6 +24116,14 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I16" t="n">
+        <v>81.6082</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="58">
       <c r="A17" s="35">
@@ -24055,6 +24161,14 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I17" t="n">
+        <v>53.4438</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="58">
       <c r="A18" s="35">
@@ -24092,6 +24206,14 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I18" t="n">
+        <v>16.4262</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="58">
       <c r="A19" s="35">
@@ -24129,6 +24251,14 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I19" t="n">
+        <v>23.3999</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="58">
       <c r="A20" s="35">
@@ -24166,6 +24296,14 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I20" t="n">
+        <v>41.6338</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="58">
       <c r="A21" s="35">
@@ -24203,6 +24341,14 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I21" t="n">
+        <v>13.8066</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="58">
       <c r="A22" s="35">
@@ -24240,6 +24386,14 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I22" t="n">
+        <v>13.1472</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="58">
       <c r="A23" s="35">
@@ -24277,6 +24431,14 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I23" t="n">
+        <v>12.4675</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="58">
       <c r="A24" s="35">
@@ -24314,6 +24476,14 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I24" t="n">
+        <v>12.2697</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="58">
       <c r="A25" s="35">
@@ -24351,6 +24521,14 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I25" t="n">
+        <v>9.889799999999999</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="58">
       <c r="A26" s="35">
@@ -24388,6 +24566,14 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I26" t="n">
+        <v>13.8759</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="58">
       <c r="A27" s="35">
@@ -24425,6 +24611,14 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I27" t="n">
+        <v>17.1932</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="58">
       <c r="A28" s="35">
@@ -24462,6 +24656,14 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I28" t="n">
+        <v>20.1658</v>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="58">
       <c r="A29" s="35">
@@ -24499,6 +24701,14 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I29" t="n">
+        <v>28.1054</v>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="58">
       <c r="A30" s="35">
@@ -24536,6 +24746,14 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I30" t="n">
+        <v>37.5072</v>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="58">
       <c r="A31" s="35">
@@ -24573,6 +24791,14 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I31" t="n">
+        <v>12.9839</v>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="58">
       <c r="A32" s="35">
@@ -24610,6 +24836,14 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I32" t="n">
+        <v>21.7042</v>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="15" customHeight="1" s="58">
       <c r="A33" s="35">
@@ -24647,6 +24881,14 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I33" t="n">
+        <v>12.5913</v>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="15" customHeight="1" s="58">
       <c r="A34" s="35">
@@ -24684,6 +24926,14 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I34" t="n">
+        <v>16.2021</v>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="58">
       <c r="A35" s="35">
@@ -24721,6 +24971,14 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I35" t="n">
+        <v>29.2628</v>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="15" customHeight="1" s="58">
       <c r="A36" s="35">
@@ -24758,6 +25016,14 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I36" t="n">
+        <v>10.0313</v>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="15" customHeight="1" s="58">
       <c r="A37" s="35">
@@ -24795,6 +25061,14 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I37" t="n">
+        <v>22.7382</v>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="15" customHeight="1" s="58">
       <c r="A38" s="35">
@@ -24832,6 +25106,9 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I38" t="n">
+        <v>22.559999</v>
+      </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="58">
       <c r="A39" s="35">
@@ -24854,7 +25131,7 @@
         </is>
       </c>
       <c r="E39" s="33" t="n">
-        <v>1.088</v>
+        <v>1.094</v>
       </c>
       <c r="F39" s="34" t="inlineStr">
         <is>
@@ -24868,6 +25145,9 @@
         <is>
           <t>OK</t>
         </is>
+      </c>
+      <c r="I39" t="n">
+        <v>1.094</v>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="58">
@@ -24906,6 +25186,9 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I40" t="n">
+        <v>785.530029</v>
+      </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="58">
       <c r="A41" s="35">
@@ -24943,6 +25226,9 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I41" t="n">
+        <v>21.639999</v>
+      </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="58">
       <c r="A42" s="35">
@@ -24980,6 +25266,9 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I42" t="n">
+        <v>224.220001</v>
+      </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="58">
       <c r="A43" s="35">
@@ -25002,7 +25291,7 @@
         </is>
       </c>
       <c r="E43" s="33" t="n">
-        <v>5.7</v>
+        <v>5.65</v>
       </c>
       <c r="F43" s="34" t="inlineStr">
         <is>
@@ -25016,6 +25305,9 @@
         <is>
           <t>OK</t>
         </is>
+      </c>
+      <c r="I43" t="n">
+        <v>5.65</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="58">
@@ -25054,6 +25346,9 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I44" t="n">
+        <v>175.5</v>
+      </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="58">
       <c r="A45" s="35">
@@ -25076,7 +25371,7 @@
         </is>
       </c>
       <c r="E45" s="33" t="n">
-        <v>0.46</v>
+        <v>0.45</v>
       </c>
       <c r="F45" s="34" t="inlineStr">
         <is>
@@ -25090,6 +25385,9 @@
         <is>
           <t>OK</t>
         </is>
+      </c>
+      <c r="I45" t="n">
+        <v>0.45</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="58">
@@ -25128,6 +25426,9 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I46" t="n">
+        <v>0.31</v>
+      </c>
     </row>
     <row r="47" ht="15" customHeight="1" s="58">
       <c r="A47" s="35">
@@ -25202,6 +25503,9 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I48" t="n">
+        <v>0.09</v>
+      </c>
     </row>
     <row r="49" ht="15" customHeight="1" s="58">
       <c r="A49" s="35">
@@ -25224,7 +25528,7 @@
         </is>
       </c>
       <c r="E49" s="33" t="n">
-        <v>67.25</v>
+        <v>68</v>
       </c>
       <c r="F49" s="34" t="inlineStr">
         <is>
@@ -25238,6 +25542,9 @@
         <is>
           <t>OK</t>
         </is>
+      </c>
+      <c r="I49" t="n">
+        <v>67.25</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="58">
@@ -25276,6 +25583,9 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I50" t="n">
+        <v>9.6</v>
+      </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="58">
       <c r="A51" s="35">
@@ -25298,7 +25608,7 @@
         </is>
       </c>
       <c r="E51" s="33" t="n">
-        <v>15.3</v>
+        <v>15.4</v>
       </c>
       <c r="F51" s="34" t="inlineStr">
         <is>
@@ -25312,6 +25622,9 @@
         <is>
           <t>OK</t>
         </is>
+      </c>
+      <c r="I51" t="n">
+        <v>15.4</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" s="58">
@@ -25335,7 +25648,7 @@
         </is>
       </c>
       <c r="E52" s="33" t="n">
-        <v>13.4</v>
+        <v>13.2</v>
       </c>
       <c r="F52" s="34" t="inlineStr">
         <is>
@@ -25349,6 +25662,9 @@
         <is>
           <t>OK</t>
         </is>
+      </c>
+      <c r="I52" t="n">
+        <v>13.2</v>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1" s="58">
@@ -25372,7 +25688,7 @@
         </is>
       </c>
       <c r="E53" s="33" t="n">
-        <v>6.15</v>
+        <v>6.1</v>
       </c>
       <c r="F53" s="34" t="inlineStr">
         <is>
@@ -25386,6 +25702,9 @@
         <is>
           <t>OK</t>
         </is>
+      </c>
+      <c r="I53" t="n">
+        <v>6.1</v>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="58">
@@ -25409,7 +25728,7 @@
         </is>
       </c>
       <c r="E54" s="33" t="n">
-        <v>21.3</v>
+        <v>21.6</v>
       </c>
       <c r="F54" s="34" t="inlineStr">
         <is>
@@ -25423,6 +25742,9 @@
         <is>
           <t>OK</t>
         </is>
+      </c>
+      <c r="I54" t="n">
+        <v>21.6</v>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="58">
@@ -25446,7 +25768,7 @@
         </is>
       </c>
       <c r="E55" s="33" t="n">
-        <v>3.56</v>
+        <v>3.6</v>
       </c>
       <c r="F55" s="34" t="inlineStr">
         <is>
@@ -25460,6 +25782,9 @@
         <is>
           <t>OK</t>
         </is>
+      </c>
+      <c r="I55" t="n">
+        <v>3.6</v>
       </c>
     </row>
     <row r="56" ht="15" customHeight="1" s="58">
@@ -25483,7 +25808,7 @@
         </is>
       </c>
       <c r="E56" s="33" t="n">
-        <v>5</v>
+        <v>4.96</v>
       </c>
       <c r="F56" s="34" t="inlineStr">
         <is>
@@ -25497,6 +25822,9 @@
         <is>
           <t>OK</t>
         </is>
+      </c>
+      <c r="I56" t="n">
+        <v>4.96</v>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1" s="58">
@@ -25520,7 +25848,7 @@
         </is>
       </c>
       <c r="E57" s="33" t="n">
-        <v>2.74</v>
+        <v>2.86</v>
       </c>
       <c r="F57" s="34" t="inlineStr">
         <is>
@@ -25534,6 +25862,9 @@
         <is>
           <t>OK</t>
         </is>
+      </c>
+      <c r="I57" t="n">
+        <v>2.86</v>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="58">
@@ -25557,7 +25888,7 @@
         </is>
       </c>
       <c r="E58" s="33" t="n">
-        <v>12.4</v>
+        <v>12.5</v>
       </c>
       <c r="F58" s="34" t="inlineStr">
         <is>
@@ -25571,6 +25902,9 @@
         <is>
           <t>OK</t>
         </is>
+      </c>
+      <c r="I58" t="n">
+        <v>12.4</v>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="58">
@@ -25594,7 +25928,7 @@
         </is>
       </c>
       <c r="E59" s="33" t="n">
-        <v>17.5</v>
+        <v>17.9</v>
       </c>
       <c r="F59" s="34" t="inlineStr">
         <is>
@@ -25608,6 +25942,9 @@
         <is>
           <t>OK</t>
         </is>
+      </c>
+      <c r="I59" t="n">
+        <v>17.9</v>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1" s="58">
@@ -25646,6 +25983,9 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I60" t="n">
+        <v>159.190002</v>
+      </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="58">
       <c r="A61" s="35">
@@ -25683,6 +26023,9 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I61" t="n">
+        <v>256.23999</v>
+      </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="58">
       <c r="A62" s="35">
@@ -25720,6 +26063,9 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I62" t="n">
+        <v>500.769989</v>
+      </c>
     </row>
     <row r="63" ht="15" customHeight="1" s="58">
       <c r="A63" s="35">
@@ -25757,6 +26103,9 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I63" t="n">
+        <v>178.899994</v>
+      </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="58">
       <c r="A64" s="35">
@@ -25794,6 +26143,9 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I64" t="n">
+        <v>69.019997</v>
+      </c>
     </row>
     <row r="65" ht="15" customHeight="1" s="58">
       <c r="A65" s="35">
@@ -25831,6 +26183,9 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I65" t="n">
+        <v>212.960007</v>
+      </c>
     </row>
     <row r="66" ht="15" customHeight="1" s="58">
       <c r="A66" s="35">
@@ -25868,6 +26223,9 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I66" t="n">
+        <v>146.479996</v>
+      </c>
     </row>
     <row r="67" ht="15" customHeight="1" s="58">
       <c r="A67" s="35">
@@ -25905,6 +26263,9 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I67" t="n">
+        <v>164.75</v>
+      </c>
     </row>
     <row r="68" ht="15" customHeight="1" s="58">
       <c r="A68" s="35">
@@ -25942,6 +26303,9 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I68" t="n">
+        <v>2125.110107</v>
+      </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="58">
       <c r="A69" s="35">
@@ -25979,6 +26343,9 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I69" t="n">
+        <v>1078.780029</v>
+      </c>
     </row>
     <row r="70" ht="15" customHeight="1" s="58">
       <c r="A70" s="35">
@@ -26016,6 +26383,9 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I70" t="n">
+        <v>96.550003</v>
+      </c>
     </row>
     <row r="71" ht="15" customHeight="1" s="58">
       <c r="A71" s="35">
@@ -26053,6 +26423,9 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I71" t="n">
+        <v>1689.890015</v>
+      </c>
     </row>
     <row r="72" ht="15" customHeight="1" s="58">
       <c r="A72" s="35">
@@ -26090,6 +26463,9 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I72" t="n">
+        <v>115.599998</v>
+      </c>
     </row>
     <row r="73" ht="15" customHeight="1" s="58">
       <c r="A73" s="35">
@@ -26127,6 +26503,9 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I73" t="n">
+        <v>214.75</v>
+      </c>
     </row>
     <row r="74" ht="15" customHeight="1" s="58">
       <c r="A74" s="35">
@@ -26164,6 +26543,9 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I74" t="n">
+        <v>90.839996</v>
+      </c>
     </row>
     <row r="75" ht="15" customHeight="1" s="58">
       <c r="A75" s="35">
@@ -26201,6 +26583,9 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I75" t="n">
+        <v>104.730003</v>
+      </c>
     </row>
     <row r="76" ht="15" customHeight="1" s="58">
       <c r="A76" s="35">
@@ -26238,6 +26623,9 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I76" t="n">
+        <v>409.670013</v>
+      </c>
     </row>
     <row r="77" ht="15" customHeight="1" s="58">
       <c r="A77" s="35">
@@ -26275,6 +26663,9 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I77" t="n">
+        <v>423.700012</v>
+      </c>
     </row>
     <row r="78" ht="15" customHeight="1" s="58">
       <c r="A78" s="35">
@@ -26312,6 +26703,9 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I78" t="n">
+        <v>56.080002</v>
+      </c>
     </row>
     <row r="79" ht="15" customHeight="1" s="58">
       <c r="A79" s="35">
@@ -26349,6 +26743,9 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I79" t="n">
+        <v>98.31999999999999</v>
+      </c>
     </row>
     <row r="80" ht="15" customHeight="1" s="58">
       <c r="A80" s="35">
@@ -26386,6 +26783,9 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I80" t="n">
+        <v>310.26001</v>
+      </c>
     </row>
     <row r="81" ht="15" customHeight="1" s="58">
       <c r="A81" s="35">
@@ -26423,6 +26823,9 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I81" t="n">
+        <v>163.220001</v>
+      </c>
     </row>
     <row r="82" ht="15" customHeight="1" s="58">
       <c r="A82" s="35">
@@ -26460,6 +26863,9 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I82" t="n">
+        <v>622.97998</v>
+      </c>
     </row>
     <row r="83" ht="15" customHeight="1" s="58">
       <c r="A83" s="35">
@@ -26497,6 +26903,9 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I83" t="n">
+        <v>155.990005</v>
+      </c>
     </row>
     <row r="84" ht="15" customHeight="1" s="58">
       <c r="A84" s="35">
@@ -26519,7 +26928,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>70.04000000000001</v>
+        <v>68.93000000000001</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -26533,6 +26942,9 @@
         <is>
           <t>OK</t>
         </is>
+      </c>
+      <c r="I84" t="n">
+        <v>72.903707</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="58">
@@ -26556,7 +26968,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>597.53</v>
+        <v>595.12</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -26570,6 +26982,9 @@
         <is>
           <t>OK</t>
         </is>
+      </c>
+      <c r="I85" t="n">
+        <v>618.35803</v>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="58">
@@ -26593,7 +27008,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>62716</v>
+        <v>62651</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -26607,6 +27022,9 @@
         <is>
           <t>OK</t>
         </is>
+      </c>
+      <c r="I86" t="n">
+        <v>64273.712343</v>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="58">
@@ -26630,7 +27048,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.006737</v>
+        <v>0.00662</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -26644,6 +27062,9 @@
         <is>
           <t>OK</t>
         </is>
+      </c>
+      <c r="I87" t="n">
+        <v>0.007053</v>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="58">
@@ -26667,7 +27088,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.011969</v>
+        <v>0.011612</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -26681,6 +27102,9 @@
         <is>
           <t>OK</t>
         </is>
+      </c>
+      <c r="I88" t="n">
+        <v>0.012555</v>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="58">
@@ -26704,7 +27128,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>67.86</v>
+        <v>67.02</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -26718,6 +27142,9 @@
         <is>
           <t>OK</t>
         </is>
+      </c>
+      <c r="I89" t="n">
+        <v>71.35623099999999</v>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="58">
@@ -26741,7 +27168,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>1.78</v>
+        <v>1.75</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -26755,6 +27182,9 @@
         <is>
           <t>OK</t>
         </is>
+      </c>
+      <c r="I90" t="n">
+        <v>1.903014</v>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="58">
@@ -26793,6 +27223,9 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="I91" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="92" ht="15" customHeight="1" s="58">
       <c r="A92" s="35">
@@ -26815,7 +27248,7 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
-        <v>0.013728</v>
+        <v>0.013579</v>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
@@ -26829,6 +27262,9 @@
         <is>
           <t>OK</t>
         </is>
+      </c>
+      <c r="I92" t="n">
+        <v>0.014273</v>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="58">
@@ -26852,7 +27288,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>2.877151</v>
+        <v>2.810687</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -26866,6 +27302,9 @@
         <is>
           <t>OK</t>
         </is>
+      </c>
+      <c r="I93" t="n">
+        <v>3.00826</v>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="58">
@@ -26889,7 +27328,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>24.463992</v>
+        <v>23.898824</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -26903,6 +27342,9 @@
         <is>
           <t>OK</t>
         </is>
+      </c>
+      <c r="I94" t="n">
+        <v>26.560378</v>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="58">
@@ -26926,7 +27368,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.120901</v>
+        <v>0.116987</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -26940,6 +27382,9 @@
         <is>
           <t>OK</t>
         </is>
+      </c>
+      <c r="I95" t="n">
+        <v>0.118329</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="58">
@@ -26963,7 +27408,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>19509.3545</v>
+        <v>19436.6192</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -26977,6 +27422,9 @@
         <is>
           <t>OK</t>
         </is>
+      </c>
+      <c r="I96" t="n">
+        <v>20195.573263</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="58">
@@ -27000,7 +27448,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2047677.4</v>
+        <v>2046181.66</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -27014,6 +27462,9 @@
         <is>
           <t>OK</t>
         </is>
+      </c>
+      <c r="I97" t="n">
+        <v>2099179.44512</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="58">
@@ -27037,7 +27488,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>2.846068</v>
+        <v>2.809707</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -27051,6 +27502,9 @@
         <is>
           <t>OK</t>
         </is>
+      </c>
+      <c r="I98" t="n">
+        <v>2.978637</v>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="58">
@@ -27074,7 +27528,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>56728.3955</v>
+        <v>56438.4396</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -27088,6 +27542,9 @@
         <is>
           <t>OK</t>
         </is>
+      </c>
+      <c r="I99" t="n">
+        <v>58995.172549</v>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="58">
@@ -27111,7 +27568,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>25.852335</v>
+        <v>25.85395</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -27125,6 +27582,9 @@
         <is>
           <t>OK</t>
         </is>
+      </c>
+      <c r="I100" t="n">
+        <v>25.135482</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="58">
@@ -27148,7 +27608,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>62716</v>
+        <v>62651</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -27162,6 +27622,9 @@
         <is>
           <t>OK</t>
         </is>
+      </c>
+      <c r="I101" t="n">
+        <v>64273.712343</v>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="58">
@@ -27185,7 +27648,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>16.79</v>
+        <v>16.55</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -27199,6 +27662,9 @@
         <is>
           <t>OK</t>
         </is>
+      </c>
+      <c r="I102" t="n">
+        <v>17.756484</v>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="58">
@@ -27296,7 +27762,7 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
-        <v>0.006737</v>
+        <v>0.00662</v>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
@@ -27310,6 +27776,9 @@
         <is>
           <t>OK</t>
         </is>
+      </c>
+      <c r="I105" t="n">
+        <v>0.007053</v>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="58">
@@ -27333,7 +27802,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>67.86</v>
+        <v>67.02</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>
@@ -27347,6 +27816,9 @@
         <is>
           <t>OK</t>
         </is>
+      </c>
+      <c r="I106" t="n">
+        <v>71.35623099999999</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="58">
@@ -27384,6 +27856,9 @@
         <is>
           <t>OK</t>
         </is>
+      </c>
+      <c r="I107" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="108">

</xml_diff>

<commit_message>
Weekly dashboard update — 2026-06-05
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-42660" yWindow="-540" windowWidth="32460" windowHeight="17180" tabRatio="500" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Realized" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Realized" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Prices" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Reference" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="AsOfDate">'FX &amp; Assumptions'!$C$5</definedName>
@@ -697,14 +697,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -726,8 +726,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -752,10 +752,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -764,10 +764,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4F81BD"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+              <a:ln w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -777,10 +777,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="C0504D"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -790,10 +790,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="9BBB59"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -803,10 +803,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="8064A2"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -816,10 +816,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4BACC6"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -829,10 +829,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="F79646"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -842,14 +842,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -875,14 +875,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -908,14 +908,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -941,14 +941,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -974,14 +974,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1007,14 +1007,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1038,16 +1038,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1142,16 +1142,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1172,10 +1172,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1187,14 +1187,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1216,8 +1216,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1242,10 +1242,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1254,10 +1254,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4672A8"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1267,10 +1267,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="AB4744"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1280,10 +1280,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="8AA64F"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1293,10 +1293,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="725990"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1306,10 +1306,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4299B0"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1319,10 +1319,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="DC853E"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1332,10 +1332,10 @@
             <idx val="6"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="93A9CE"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1345,10 +1345,10 @@
             <idx val="7"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="D09493"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1358,10 +1358,10 @@
             <idx val="8"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="B8CD97"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1371,14 +1371,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1405,14 +1405,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1439,14 +1439,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1473,14 +1473,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1507,14 +1507,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1541,14 +1541,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1575,14 +1575,14 @@
             <dLbl>
               <idx val="6"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1609,14 +1609,14 @@
             <dLbl>
               <idx val="7"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1643,14 +1643,14 @@
             <dLbl>
               <idx val="8"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1675,16 +1675,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1791,16 +1791,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1821,10 +1821,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1836,14 +1836,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1865,8 +1865,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1893,10 +1893,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1904,16 +1904,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2016,7 +2016,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2025,9 +2025,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2059,7 +2059,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2073,7 +2073,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2082,9 +2082,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2109,16 +2109,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2139,10 +2139,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2154,14 +2154,14 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -2183,8 +2183,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -2200,10 +2200,10 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2211,16 +2211,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2411,7 +2411,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2420,9 +2420,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2454,7 +2454,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2468,7 +2468,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2477,9 +2477,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2504,16 +2504,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2534,10 +2534,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2549,7 +2549,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>1</col>
@@ -2569,9 +2569,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2596,9 +2596,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+          <c:chart r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2623,9 +2623,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+          <c:chart r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2650,9 +2650,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+          <c:chart r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -21622,28 +21622,28 @@
         <v>46178</v>
       </c>
       <c r="C9" s="29" t="n">
-        <v>27099858</v>
+        <v>27073884</v>
       </c>
       <c r="D9" s="29" t="n">
-        <v>22652740</v>
+        <v>22648647</v>
       </c>
       <c r="E9" s="29" t="n">
-        <v>4447118</v>
+        <v>4425237</v>
       </c>
       <c r="F9" s="30" t="n">
-        <v>0.1963</v>
+        <v>0.1954</v>
       </c>
       <c r="G9" s="29" t="n">
         <v>19315301</v>
       </c>
       <c r="H9" s="29" t="n">
-        <v>5236944</v>
+        <v>5230018</v>
       </c>
       <c r="I9" s="29" t="n">
-        <v>1154877</v>
+        <v>1134468</v>
       </c>
       <c r="J9" s="31" t="n">
-        <v>32.65</v>
+        <v>32.61</v>
       </c>
       <c r="K9" s="32" t="inlineStr">
         <is>
@@ -23438,7 +23438,7 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>32.66</v>
+        <v>32.61</v>
       </c>
       <c r="D6" s="64" t="inlineStr">
         <is>
@@ -23487,7 +23487,7 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>25.4261</v>
+        <v>25.4162</v>
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
@@ -25291,7 +25291,7 @@
         </is>
       </c>
       <c r="E43" s="33" t="n">
-        <v>5.65</v>
+        <v>5.6</v>
       </c>
       <c r="F43" s="34" t="inlineStr">
         <is>
@@ -25307,7 +25307,7 @@
         </is>
       </c>
       <c r="I43" t="n">
-        <v>5.65</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="58">
@@ -25528,7 +25528,7 @@
         </is>
       </c>
       <c r="E49" s="33" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F49" s="34" t="inlineStr">
         <is>
@@ -25568,7 +25568,7 @@
         </is>
       </c>
       <c r="E50" s="33" t="n">
-        <v>9.6</v>
+        <v>9.5</v>
       </c>
       <c r="F50" s="34" t="inlineStr">
         <is>
@@ -25608,7 +25608,7 @@
         </is>
       </c>
       <c r="E51" s="33" t="n">
-        <v>15.4</v>
+        <v>15.5</v>
       </c>
       <c r="F51" s="34" t="inlineStr">
         <is>
@@ -25624,7 +25624,7 @@
         </is>
       </c>
       <c r="I51" t="n">
-        <v>15.4</v>
+        <v>15.3</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" s="58">
@@ -25688,7 +25688,7 @@
         </is>
       </c>
       <c r="E53" s="33" t="n">
-        <v>6.1</v>
+        <v>6.05</v>
       </c>
       <c r="F53" s="34" t="inlineStr">
         <is>
@@ -25704,7 +25704,7 @@
         </is>
       </c>
       <c r="I53" t="n">
-        <v>6.1</v>
+        <v>6.05</v>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="58">
@@ -25728,7 +25728,7 @@
         </is>
       </c>
       <c r="E54" s="33" t="n">
-        <v>21.6</v>
+        <v>21.5</v>
       </c>
       <c r="F54" s="34" t="inlineStr">
         <is>
@@ -25744,7 +25744,7 @@
         </is>
       </c>
       <c r="I54" t="n">
-        <v>21.6</v>
+        <v>21.299999</v>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="58">
@@ -25768,7 +25768,7 @@
         </is>
       </c>
       <c r="E55" s="33" t="n">
-        <v>3.6</v>
+        <v>3.54</v>
       </c>
       <c r="F55" s="34" t="inlineStr">
         <is>
@@ -25784,7 +25784,7 @@
         </is>
       </c>
       <c r="I55" t="n">
-        <v>3.6</v>
+        <v>3.54</v>
       </c>
     </row>
     <row r="56" ht="15" customHeight="1" s="58">
@@ -25808,7 +25808,7 @@
         </is>
       </c>
       <c r="E56" s="33" t="n">
-        <v>4.96</v>
+        <v>4.94</v>
       </c>
       <c r="F56" s="34" t="inlineStr">
         <is>
@@ -25824,7 +25824,7 @@
         </is>
       </c>
       <c r="I56" t="n">
-        <v>4.96</v>
+        <v>4.94</v>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1" s="58">
@@ -25848,7 +25848,7 @@
         </is>
       </c>
       <c r="E57" s="33" t="n">
-        <v>2.86</v>
+        <v>2.78</v>
       </c>
       <c r="F57" s="34" t="inlineStr">
         <is>
@@ -25864,7 +25864,7 @@
         </is>
       </c>
       <c r="I57" t="n">
-        <v>2.86</v>
+        <v>2.78</v>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="58">
@@ -25984,7 +25984,7 @@
         </is>
       </c>
       <c r="I60" t="n">
-        <v>159.190002</v>
+        <v>161.869995</v>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="58">
@@ -26024,7 +26024,7 @@
         </is>
       </c>
       <c r="I61" t="n">
-        <v>256.23999</v>
+        <v>258.420013</v>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="58">
@@ -26064,7 +26064,7 @@
         </is>
       </c>
       <c r="I62" t="n">
-        <v>500.769989</v>
+        <v>501.700012</v>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1" s="58">
@@ -26104,7 +26104,7 @@
         </is>
       </c>
       <c r="I63" t="n">
-        <v>178.899994</v>
+        <v>175.630005</v>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="58">
@@ -26184,7 +26184,7 @@
         </is>
       </c>
       <c r="I65" t="n">
-        <v>212.960007</v>
+        <v>203.970001</v>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1" s="58">
@@ -26224,7 +26224,7 @@
         </is>
       </c>
       <c r="I66" t="n">
-        <v>146.479996</v>
+        <v>149.669998</v>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1" s="58">
@@ -26264,7 +26264,7 @@
         </is>
       </c>
       <c r="I67" t="n">
-        <v>164.75</v>
+        <v>164.869995</v>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1" s="58">
@@ -26304,7 +26304,7 @@
         </is>
       </c>
       <c r="I68" t="n">
-        <v>2125.110107</v>
+        <v>2131.100098</v>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="58">
@@ -26344,7 +26344,7 @@
         </is>
       </c>
       <c r="I69" t="n">
-        <v>1078.780029</v>
+        <v>1125.27002</v>
       </c>
     </row>
     <row r="70" ht="15" customHeight="1" s="58">
@@ -26384,7 +26384,7 @@
         </is>
       </c>
       <c r="I70" t="n">
-        <v>96.550003</v>
+        <v>96.300003</v>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1" s="58">
@@ -26424,7 +26424,7 @@
         </is>
       </c>
       <c r="I71" t="n">
-        <v>1689.890015</v>
+        <v>1652.599976</v>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1" s="58">
@@ -26464,7 +26464,7 @@
         </is>
       </c>
       <c r="I72" t="n">
-        <v>115.599998</v>
+        <v>118.830002</v>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1" s="58">
@@ -26504,7 +26504,7 @@
         </is>
       </c>
       <c r="I73" t="n">
-        <v>214.75</v>
+        <v>218.660004</v>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1" s="58">
@@ -26544,7 +26544,7 @@
         </is>
       </c>
       <c r="I74" t="n">
-        <v>90.839996</v>
+        <v>90.199997</v>
       </c>
     </row>
     <row r="75" ht="15" customHeight="1" s="58">
@@ -26624,7 +26624,7 @@
         </is>
       </c>
       <c r="I76" t="n">
-        <v>409.670013</v>
+        <v>406.859985</v>
       </c>
     </row>
     <row r="77" ht="15" customHeight="1" s="58">
@@ -26664,7 +26664,7 @@
         </is>
       </c>
       <c r="I77" t="n">
-        <v>423.700012</v>
+        <v>418.450012</v>
       </c>
     </row>
     <row r="78" ht="15" customHeight="1" s="58">
@@ -26784,7 +26784,7 @@
         </is>
       </c>
       <c r="I80" t="n">
-        <v>310.26001</v>
+        <v>311.230011</v>
       </c>
     </row>
     <row r="81" ht="15" customHeight="1" s="58">
@@ -26928,7 +26928,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>68.93000000000001</v>
+        <v>65.84999999999999</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -26944,7 +26944,7 @@
         </is>
       </c>
       <c r="I84" t="n">
-        <v>72.903707</v>
+        <v>70.787525</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="58">
@@ -26968,7 +26968,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>595.12</v>
+        <v>590.89</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -26984,7 +26984,7 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>618.35803</v>
+        <v>596.662811</v>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="58">
@@ -27008,7 +27008,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>62651</v>
+        <v>62220</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -27024,7 +27024,7 @@
         </is>
       </c>
       <c r="I86" t="n">
-        <v>64273.712343</v>
+        <v>63038.086769</v>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="58">
@@ -27048,7 +27048,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.00662</v>
+        <v>0.006471</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -27064,7 +27064,7 @@
         </is>
       </c>
       <c r="I87" t="n">
-        <v>0.007053</v>
+        <v>0.00676</v>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="58">
@@ -27088,7 +27088,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.011612</v>
+        <v>0.011915</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -27104,7 +27104,7 @@
         </is>
       </c>
       <c r="I88" t="n">
-        <v>0.012555</v>
+        <v>0.011591</v>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="58">
@@ -27128,7 +27128,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>67.02</v>
+        <v>66.02</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -27144,7 +27144,7 @@
         </is>
       </c>
       <c r="I89" t="n">
-        <v>71.35623099999999</v>
+        <v>68.84531</v>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="58">
@@ -27168,7 +27168,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>1.75</v>
+        <v>1.67</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -27184,7 +27184,7 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>1.903014</v>
+        <v>1.790223</v>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="58">
@@ -27248,7 +27248,7 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
-        <v>0.013579</v>
+        <v>0.013108</v>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
@@ -27264,7 +27264,7 @@
         </is>
       </c>
       <c r="I92" t="n">
-        <v>0.014273</v>
+        <v>0.013586</v>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="58">
@@ -27288,7 +27288,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>2.810687</v>
+        <v>2.666259</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -27304,7 +27304,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>3.00826</v>
+        <v>2.878567</v>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="58">
@@ -27328,7 +27328,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>23.898824</v>
+        <v>23.260909</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -27344,7 +27344,7 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>26.560378</v>
+        <v>24.941592</v>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="58">
@@ -27368,7 +27368,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.116987</v>
+        <v>0.114444</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -27384,7 +27384,7 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>0.118329</v>
+        <v>0.115051</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="58">
@@ -27408,7 +27408,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>19436.6192</v>
+        <v>19268.9229</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -27424,7 +27424,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>20195.573263</v>
+        <v>19457.174272</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="58">
@@ -27448,7 +27448,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2046181.66</v>
+        <v>2028994.2</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -27464,7 +27464,7 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>2099179.44512</v>
+        <v>2055672.00954</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="58">
@@ -27488,7 +27488,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>2.809707</v>
+        <v>2.735686</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -27504,7 +27504,7 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>2.978637</v>
+        <v>2.862662</v>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="58">
@@ -27528,7 +27528,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>56438.4396</v>
+        <v>54232.3866</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -27544,7 +27544,7 @@
         </is>
       </c>
       <c r="I99" t="n">
-        <v>58995.172549</v>
+        <v>57288.690676</v>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="58">
@@ -27568,7 +27568,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>25.85395</v>
+        <v>25.145799</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -27584,7 +27584,7 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>25.135482</v>
+        <v>25.040571</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="58">
@@ -27608,7 +27608,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>62651</v>
+        <v>62220</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -27624,7 +27624,7 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>64273.712343</v>
+        <v>63038.086769</v>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="58">
@@ -27648,7 +27648,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>16.55</v>
+        <v>16.54</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -27664,7 +27664,7 @@
         </is>
       </c>
       <c r="I102" t="n">
-        <v>17.756484</v>
+        <v>17.067191</v>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="58">
@@ -27762,7 +27762,7 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
-        <v>0.00662</v>
+        <v>0.006471</v>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
@@ -27778,7 +27778,7 @@
         </is>
       </c>
       <c r="I105" t="n">
-        <v>0.007053</v>
+        <v>0.00676</v>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="58">
@@ -27802,7 +27802,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>67.02</v>
+        <v>66.02</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>
@@ -27818,7 +27818,7 @@
         </is>
       </c>
       <c r="I106" t="n">
-        <v>71.35623099999999</v>
+        <v>68.84531</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="58">

</xml_diff>

<commit_message>
Daily dashboard update — 2026-06-06
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-42660" yWindow="-540" windowWidth="32460" windowHeight="17180" tabRatio="500" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Realized" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Prices" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Reference" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Realized" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="AsOfDate">'FX &amp; Assumptions'!$C$5</definedName>
@@ -697,14 +697,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -726,8 +726,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -752,10 +752,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -764,10 +764,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4F81BD"/>
               </a:solidFill>
-              <a:ln w="0">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -777,10 +777,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="C0504D"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -790,10 +790,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="9BBB59"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -803,10 +803,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="8064A2"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -816,10 +816,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4BACC6"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -829,10 +829,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="F79646"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -842,14 +842,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -875,14 +875,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -908,14 +908,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -941,14 +941,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -974,14 +974,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1007,14 +1007,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1038,16 +1038,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1142,16 +1142,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1172,10 +1172,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1187,14 +1187,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1216,8 +1216,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1242,10 +1242,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1254,10 +1254,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4672A8"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1267,10 +1267,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="AB4744"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1280,10 +1280,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="8AA64F"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1293,10 +1293,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="725990"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1306,10 +1306,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4299B0"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1319,10 +1319,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="DC853E"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1332,10 +1332,10 @@
             <idx val="6"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="93A9CE"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1345,10 +1345,10 @@
             <idx val="7"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="D09493"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1358,10 +1358,10 @@
             <idx val="8"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="B8CD97"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1371,14 +1371,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1405,14 +1405,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1439,14 +1439,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1473,14 +1473,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1507,14 +1507,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1541,14 +1541,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1575,14 +1575,14 @@
             <dLbl>
               <idx val="6"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1609,14 +1609,14 @@
             <dLbl>
               <idx val="7"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1643,14 +1643,14 @@
             <dLbl>
               <idx val="8"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1675,16 +1675,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1791,16 +1791,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1821,10 +1821,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1836,14 +1836,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1865,8 +1865,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1893,10 +1893,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1904,16 +1904,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2016,7 +2016,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2025,9 +2025,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2059,7 +2059,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="9360">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2073,7 +2073,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2082,9 +2082,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2109,16 +2109,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2139,10 +2139,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2154,14 +2154,14 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -2183,8 +2183,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -2200,10 +2200,10 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2211,16 +2211,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2411,7 +2411,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2420,9 +2420,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2454,7 +2454,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="9360">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2468,7 +2468,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2477,9 +2477,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2504,16 +2504,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2534,10 +2534,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2549,7 +2549,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>1</col>
@@ -2569,9 +2569,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2596,9 +2596,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2623,9 +2623,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId3"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2650,9 +2650,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId4"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -21652,16 +21652,38 @@
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="58">
-      <c r="B10" s="28" t="n"/>
-      <c r="C10" s="29" t="n"/>
-      <c r="D10" s="29" t="n"/>
-      <c r="E10" s="29" t="n"/>
-      <c r="F10" s="30" t="n"/>
-      <c r="G10" s="29" t="n"/>
-      <c r="H10" s="29" t="n"/>
-      <c r="I10" s="29" t="n"/>
-      <c r="J10" s="31" t="n"/>
-      <c r="K10" s="32" t="n"/>
+      <c r="B10" s="28" t="n">
+        <v>46179</v>
+      </c>
+      <c r="C10" s="29" t="n">
+        <v>26792154</v>
+      </c>
+      <c r="D10" s="29" t="n">
+        <v>22666838</v>
+      </c>
+      <c r="E10" s="29" t="n">
+        <v>4125316</v>
+      </c>
+      <c r="F10" s="30" t="n">
+        <v>0.182</v>
+      </c>
+      <c r="G10" s="29" t="n">
+        <v>19315301</v>
+      </c>
+      <c r="H10" s="29" t="n">
+        <v>4980397</v>
+      </c>
+      <c r="I10" s="29" t="n">
+        <v>1117917</v>
+      </c>
+      <c r="J10" s="31" t="n">
+        <v>32.79</v>
+      </c>
+      <c r="K10" s="32" t="inlineStr">
+        <is>
+          <t>Auto weekly snapshot</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="58">
       <c r="B11" s="28" t="n"/>
@@ -23423,7 +23445,7 @@
         </is>
       </c>
       <c r="C5" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="D5" s="64" t="inlineStr">
         <is>
@@ -23438,11 +23460,11 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>32.58</v>
+        <v>32.79</v>
       </c>
       <c r="D6" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-06-05</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-06-06</t>
         </is>
       </c>
     </row>
@@ -23487,11 +23509,11 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>25.412</v>
+        <v>25.4187</v>
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-06-05</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-06-06</t>
         </is>
       </c>
     </row>
@@ -25091,7 +25113,7 @@
         </is>
       </c>
       <c r="E38" s="33" t="n">
-        <v>22.56</v>
+        <v>22.83</v>
       </c>
       <c r="F38" s="34" t="inlineStr">
         <is>
@@ -25099,7 +25121,7 @@
         </is>
       </c>
       <c r="G38" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H38" s="34" t="inlineStr">
         <is>
@@ -25107,7 +25129,7 @@
         </is>
       </c>
       <c r="I38" t="n">
-        <v>22.559999</v>
+        <v>22.83</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="58">
@@ -25139,7 +25161,7 @@
         </is>
       </c>
       <c r="G39" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H39" s="34" t="inlineStr">
         <is>
@@ -25147,7 +25169,7 @@
         </is>
       </c>
       <c r="I39" t="n">
-        <v>1.094</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="58">
@@ -25171,7 +25193,7 @@
         </is>
       </c>
       <c r="E40" s="33" t="n">
-        <v>785.53</v>
+        <v>770.09</v>
       </c>
       <c r="F40" s="34" t="inlineStr">
         <is>
@@ -25179,7 +25201,7 @@
         </is>
       </c>
       <c r="G40" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H40" s="34" t="inlineStr">
         <is>
@@ -25187,7 +25209,7 @@
         </is>
       </c>
       <c r="I40" t="n">
-        <v>785.530029</v>
+        <v>770.090027</v>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="58">
@@ -25211,7 +25233,7 @@
         </is>
       </c>
       <c r="E41" s="33" t="n">
-        <v>21.64</v>
+        <v>20.84</v>
       </c>
       <c r="F41" s="34" t="inlineStr">
         <is>
@@ -25219,7 +25241,7 @@
         </is>
       </c>
       <c r="G41" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H41" s="34" t="inlineStr">
         <is>
@@ -25227,7 +25249,7 @@
         </is>
       </c>
       <c r="I41" t="n">
-        <v>21.639999</v>
+        <v>20.84</v>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="58">
@@ -25251,7 +25273,7 @@
         </is>
       </c>
       <c r="E42" s="33" t="n">
-        <v>224.22</v>
+        <v>221.79</v>
       </c>
       <c r="F42" s="34" t="inlineStr">
         <is>
@@ -25259,7 +25281,7 @@
         </is>
       </c>
       <c r="G42" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H42" s="34" t="inlineStr">
         <is>
@@ -25267,7 +25289,7 @@
         </is>
       </c>
       <c r="I42" t="n">
-        <v>224.220001</v>
+        <v>221.789993</v>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="58">
@@ -25299,7 +25321,7 @@
         </is>
       </c>
       <c r="G43" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H43" s="34" t="inlineStr">
         <is>
@@ -25339,7 +25361,7 @@
         </is>
       </c>
       <c r="G44" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H44" s="34" t="inlineStr">
         <is>
@@ -25379,7 +25401,7 @@
         </is>
       </c>
       <c r="G45" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H45" s="34" t="inlineStr">
         <is>
@@ -25419,7 +25441,7 @@
         </is>
       </c>
       <c r="G46" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H46" s="34" t="inlineStr">
         <is>
@@ -25496,7 +25518,7 @@
         </is>
       </c>
       <c r="G48" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H48" s="34" t="inlineStr">
         <is>
@@ -25536,7 +25558,7 @@
         </is>
       </c>
       <c r="G49" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H49" s="34" t="inlineStr">
         <is>
@@ -25576,7 +25598,7 @@
         </is>
       </c>
       <c r="G50" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H50" s="34" t="inlineStr">
         <is>
@@ -25616,7 +25638,7 @@
         </is>
       </c>
       <c r="G51" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H51" s="34" t="inlineStr">
         <is>
@@ -25656,7 +25678,7 @@
         </is>
       </c>
       <c r="G52" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H52" s="34" t="inlineStr">
         <is>
@@ -25696,7 +25718,7 @@
         </is>
       </c>
       <c r="G53" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H53" s="34" t="inlineStr">
         <is>
@@ -25736,7 +25758,7 @@
         </is>
       </c>
       <c r="G54" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H54" s="34" t="inlineStr">
         <is>
@@ -25776,7 +25798,7 @@
         </is>
       </c>
       <c r="G55" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H55" s="34" t="inlineStr">
         <is>
@@ -25816,7 +25838,7 @@
         </is>
       </c>
       <c r="G56" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H56" s="34" t="inlineStr">
         <is>
@@ -25856,7 +25878,7 @@
         </is>
       </c>
       <c r="G57" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H57" s="34" t="inlineStr">
         <is>
@@ -25896,7 +25918,7 @@
         </is>
       </c>
       <c r="G58" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H58" s="34" t="inlineStr">
         <is>
@@ -25936,7 +25958,7 @@
         </is>
       </c>
       <c r="G59" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H59" s="34" t="inlineStr">
         <is>
@@ -25968,7 +25990,7 @@
         </is>
       </c>
       <c r="E60" s="33" t="n">
-        <v>161.87</v>
+        <v>147.16</v>
       </c>
       <c r="F60" s="34" t="inlineStr">
         <is>
@@ -25976,7 +25998,7 @@
         </is>
       </c>
       <c r="G60" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H60" s="34" t="inlineStr">
         <is>
@@ -25984,7 +26006,7 @@
         </is>
       </c>
       <c r="I60" t="n">
-        <v>161.869995</v>
+        <v>147.160004</v>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="58">
@@ -26008,7 +26030,7 @@
         </is>
       </c>
       <c r="E61" s="33" t="n">
-        <v>258.42</v>
+        <v>251.44</v>
       </c>
       <c r="F61" s="34" t="inlineStr">
         <is>
@@ -26016,7 +26038,7 @@
         </is>
       </c>
       <c r="G61" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H61" s="34" t="inlineStr">
         <is>
@@ -26024,7 +26046,7 @@
         </is>
       </c>
       <c r="I61" t="n">
-        <v>258.420013</v>
+        <v>251.440002</v>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="58">
@@ -26048,7 +26070,7 @@
         </is>
       </c>
       <c r="E62" s="33" t="n">
-        <v>501.7</v>
+        <v>453.01</v>
       </c>
       <c r="F62" s="34" t="inlineStr">
         <is>
@@ -26056,7 +26078,7 @@
         </is>
       </c>
       <c r="G62" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H62" s="34" t="inlineStr">
         <is>
@@ -26064,7 +26086,7 @@
         </is>
       </c>
       <c r="I62" t="n">
-        <v>501.700012</v>
+        <v>453.01001</v>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1" s="58">
@@ -26088,7 +26110,7 @@
         </is>
       </c>
       <c r="E63" s="33" t="n">
-        <v>175.63</v>
+        <v>164.4</v>
       </c>
       <c r="F63" s="34" t="inlineStr">
         <is>
@@ -26096,7 +26118,7 @@
         </is>
       </c>
       <c r="G63" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H63" s="34" t="inlineStr">
         <is>
@@ -26104,7 +26126,7 @@
         </is>
       </c>
       <c r="I63" t="n">
-        <v>175.630005</v>
+        <v>164.399994</v>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="58">
@@ -26128,7 +26150,7 @@
         </is>
       </c>
       <c r="E64" s="33" t="n">
-        <v>68.39</v>
+        <v>56.07</v>
       </c>
       <c r="F64" s="34" t="inlineStr">
         <is>
@@ -26136,7 +26158,7 @@
         </is>
       </c>
       <c r="G64" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H64" s="34" t="inlineStr">
         <is>
@@ -26144,7 +26166,7 @@
         </is>
       </c>
       <c r="I64" t="n">
-        <v>69.019997</v>
+        <v>56.07</v>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1" s="58">
@@ -26168,7 +26190,7 @@
         </is>
       </c>
       <c r="E65" s="33" t="n">
-        <v>203.97</v>
+        <v>175.19</v>
       </c>
       <c r="F65" s="34" t="inlineStr">
         <is>
@@ -26176,7 +26198,7 @@
         </is>
       </c>
       <c r="G65" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H65" s="34" t="inlineStr">
         <is>
@@ -26184,7 +26206,7 @@
         </is>
       </c>
       <c r="I65" t="n">
-        <v>203.970001</v>
+        <v>175.190002</v>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1" s="58">
@@ -26208,7 +26230,7 @@
         </is>
       </c>
       <c r="E66" s="33" t="n">
-        <v>149.67</v>
+        <v>144.68</v>
       </c>
       <c r="F66" s="34" t="inlineStr">
         <is>
@@ -26216,7 +26238,7 @@
         </is>
       </c>
       <c r="G66" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H66" s="34" t="inlineStr">
         <is>
@@ -26224,7 +26246,7 @@
         </is>
       </c>
       <c r="I66" t="n">
-        <v>149.669998</v>
+        <v>144.679993</v>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1" s="58">
@@ -26248,7 +26270,7 @@
         </is>
       </c>
       <c r="E67" s="33" t="n">
-        <v>164.87</v>
+        <v>164.02</v>
       </c>
       <c r="F67" s="34" t="inlineStr">
         <is>
@@ -26256,7 +26278,7 @@
         </is>
       </c>
       <c r="G67" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H67" s="34" t="inlineStr">
         <is>
@@ -26264,7 +26286,7 @@
         </is>
       </c>
       <c r="I67" t="n">
-        <v>164.869995</v>
+        <v>164.020004</v>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1" s="58">
@@ -26288,7 +26310,7 @@
         </is>
       </c>
       <c r="E68" s="33" t="n">
-        <v>2131.1</v>
+        <v>1929.2</v>
       </c>
       <c r="F68" s="34" t="inlineStr">
         <is>
@@ -26296,7 +26318,7 @@
         </is>
       </c>
       <c r="G68" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H68" s="34" t="inlineStr">
         <is>
@@ -26304,7 +26326,7 @@
         </is>
       </c>
       <c r="I68" t="n">
-        <v>2131.100098</v>
+        <v>1929.199951</v>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="58">
@@ -26328,7 +26350,7 @@
         </is>
       </c>
       <c r="E69" s="33" t="n">
-        <v>1125.27</v>
+        <v>1131.42</v>
       </c>
       <c r="F69" s="34" t="inlineStr">
         <is>
@@ -26336,7 +26358,7 @@
         </is>
       </c>
       <c r="G69" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H69" s="34" t="inlineStr">
         <is>
@@ -26344,7 +26366,7 @@
         </is>
       </c>
       <c r="I69" t="n">
-        <v>1125.27002</v>
+        <v>1131.420044</v>
       </c>
     </row>
     <row r="70" ht="15" customHeight="1" s="58">
@@ -26368,7 +26390,7 @@
         </is>
       </c>
       <c r="E70" s="33" t="n">
-        <v>96.3</v>
+        <v>88.34</v>
       </c>
       <c r="F70" s="34" t="inlineStr">
         <is>
@@ -26376,7 +26398,7 @@
         </is>
       </c>
       <c r="G70" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H70" s="34" t="inlineStr">
         <is>
@@ -26384,7 +26406,7 @@
         </is>
       </c>
       <c r="I70" t="n">
-        <v>96.300003</v>
+        <v>88.339996</v>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1" s="58">
@@ -26408,7 +26430,7 @@
         </is>
       </c>
       <c r="E71" s="33" t="n">
-        <v>1652.6</v>
+        <v>1481.05</v>
       </c>
       <c r="F71" s="34" t="inlineStr">
         <is>
@@ -26416,7 +26438,7 @@
         </is>
       </c>
       <c r="G71" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H71" s="34" t="inlineStr">
         <is>
@@ -26424,7 +26446,7 @@
         </is>
       </c>
       <c r="I71" t="n">
-        <v>1652.599976</v>
+        <v>1481.050049</v>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1" s="58">
@@ -26448,7 +26470,7 @@
         </is>
       </c>
       <c r="E72" s="33" t="n">
-        <v>118.83</v>
+        <v>111.07</v>
       </c>
       <c r="F72" s="34" t="inlineStr">
         <is>
@@ -26456,7 +26478,7 @@
         </is>
       </c>
       <c r="G72" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H72" s="34" t="inlineStr">
         <is>
@@ -26464,7 +26486,7 @@
         </is>
       </c>
       <c r="I72" t="n">
-        <v>118.830002</v>
+        <v>111.07</v>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1" s="58">
@@ -26488,7 +26510,7 @@
         </is>
       </c>
       <c r="E73" s="33" t="n">
-        <v>218.66</v>
+        <v>205.1</v>
       </c>
       <c r="F73" s="34" t="inlineStr">
         <is>
@@ -26496,7 +26518,7 @@
         </is>
       </c>
       <c r="G73" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H73" s="34" t="inlineStr">
         <is>
@@ -26504,7 +26526,7 @@
         </is>
       </c>
       <c r="I73" t="n">
-        <v>218.660004</v>
+        <v>205.100006</v>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1" s="58">
@@ -26528,7 +26550,7 @@
         </is>
       </c>
       <c r="E74" s="33" t="n">
-        <v>90.2</v>
+        <v>86.11</v>
       </c>
       <c r="F74" s="34" t="inlineStr">
         <is>
@@ -26536,7 +26558,7 @@
         </is>
       </c>
       <c r="G74" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H74" s="34" t="inlineStr">
         <is>
@@ -26544,7 +26566,7 @@
         </is>
       </c>
       <c r="I74" t="n">
-        <v>90.199997</v>
+        <v>86.110001</v>
       </c>
     </row>
     <row r="75" ht="15" customHeight="1" s="58">
@@ -26568,7 +26590,7 @@
         </is>
       </c>
       <c r="E75" s="33" t="n">
-        <v>103.97</v>
+        <v>98.28</v>
       </c>
       <c r="F75" s="34" t="inlineStr">
         <is>
@@ -26576,7 +26598,7 @@
         </is>
       </c>
       <c r="G75" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H75" s="34" t="inlineStr">
         <is>
@@ -26584,7 +26606,7 @@
         </is>
       </c>
       <c r="I75" t="n">
-        <v>104.730003</v>
+        <v>98.279999</v>
       </c>
     </row>
     <row r="76" ht="15" customHeight="1" s="58">
@@ -26608,7 +26630,7 @@
         </is>
       </c>
       <c r="E76" s="33" t="n">
-        <v>406.86</v>
+        <v>357.93</v>
       </c>
       <c r="F76" s="34" t="inlineStr">
         <is>
@@ -26616,7 +26638,7 @@
         </is>
       </c>
       <c r="G76" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H76" s="34" t="inlineStr">
         <is>
@@ -26624,7 +26646,7 @@
         </is>
       </c>
       <c r="I76" t="n">
-        <v>406.859985</v>
+        <v>357.929993</v>
       </c>
     </row>
     <row r="77" ht="15" customHeight="1" s="58">
@@ -26648,7 +26670,7 @@
         </is>
       </c>
       <c r="E77" s="33" t="n">
-        <v>418.45</v>
+        <v>391</v>
       </c>
       <c r="F77" s="34" t="inlineStr">
         <is>
@@ -26656,7 +26678,7 @@
         </is>
       </c>
       <c r="G77" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H77" s="34" t="inlineStr">
         <is>
@@ -26688,7 +26710,7 @@
         </is>
       </c>
       <c r="E78" s="33" t="n">
-        <v>54.48</v>
+        <v>54.52</v>
       </c>
       <c r="F78" s="34" t="inlineStr">
         <is>
@@ -26696,7 +26718,7 @@
         </is>
       </c>
       <c r="G78" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H78" s="34" t="inlineStr">
         <is>
@@ -26704,7 +26726,7 @@
         </is>
       </c>
       <c r="I78" t="n">
-        <v>56.080002</v>
+        <v>54.52</v>
       </c>
     </row>
     <row r="79" ht="15" customHeight="1" s="58">
@@ -26728,7 +26750,7 @@
         </is>
       </c>
       <c r="E79" s="33" t="n">
-        <v>97</v>
+        <v>88.59</v>
       </c>
       <c r="F79" s="34" t="inlineStr">
         <is>
@@ -26736,7 +26758,7 @@
         </is>
       </c>
       <c r="G79" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H79" s="34" t="inlineStr">
         <is>
@@ -26744,7 +26766,7 @@
         </is>
       </c>
       <c r="I79" t="n">
-        <v>98.31999999999999</v>
+        <v>88.589996</v>
       </c>
     </row>
     <row r="80" ht="15" customHeight="1" s="58">
@@ -26768,7 +26790,7 @@
         </is>
       </c>
       <c r="E80" s="33" t="n">
-        <v>311.23</v>
+        <v>307.34</v>
       </c>
       <c r="F80" s="34" t="inlineStr">
         <is>
@@ -26776,7 +26798,7 @@
         </is>
       </c>
       <c r="G80" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H80" s="34" t="inlineStr">
         <is>
@@ -26784,7 +26806,7 @@
         </is>
       </c>
       <c r="I80" t="n">
-        <v>311.230011</v>
+        <v>307.339996</v>
       </c>
     </row>
     <row r="81" ht="15" customHeight="1" s="58">
@@ -26808,7 +26830,7 @@
         </is>
       </c>
       <c r="E81" s="33" t="n">
-        <v>164.13</v>
+        <v>152.4</v>
       </c>
       <c r="F81" s="34" t="inlineStr">
         <is>
@@ -26816,7 +26838,7 @@
         </is>
       </c>
       <c r="G81" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H81" s="34" t="inlineStr">
         <is>
@@ -26824,7 +26846,7 @@
         </is>
       </c>
       <c r="I81" t="n">
-        <v>163.220001</v>
+        <v>152.399994</v>
       </c>
     </row>
     <row r="82" ht="15" customHeight="1" s="58">
@@ -26848,7 +26870,7 @@
         </is>
       </c>
       <c r="E82" s="33" t="n">
-        <v>627.5700000000001</v>
+        <v>593</v>
       </c>
       <c r="F82" s="34" t="inlineStr">
         <is>
@@ -26856,7 +26878,7 @@
         </is>
       </c>
       <c r="G82" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H82" s="34" t="inlineStr">
         <is>
@@ -26864,7 +26886,7 @@
         </is>
       </c>
       <c r="I82" t="n">
-        <v>622.97998</v>
+        <v>627.570007</v>
       </c>
     </row>
     <row r="83" ht="15" customHeight="1" s="58">
@@ -26888,7 +26910,7 @@
         </is>
       </c>
       <c r="E83" s="33" t="n">
-        <v>166</v>
+        <v>136.99</v>
       </c>
       <c r="F83" s="34" t="inlineStr">
         <is>
@@ -26896,7 +26918,7 @@
         </is>
       </c>
       <c r="G83" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H83" s="34" t="inlineStr">
         <is>
@@ -26904,7 +26926,7 @@
         </is>
       </c>
       <c r="I83" t="n">
-        <v>155.990005</v>
+        <v>136.990005</v>
       </c>
     </row>
     <row r="84" ht="15" customHeight="1" s="58">
@@ -26928,7 +26950,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>65.84</v>
+        <v>62.18</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -26936,7 +26958,7 @@
         </is>
       </c>
       <c r="G84" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H84" s="34" t="inlineStr">
         <is>
@@ -26944,7 +26966,7 @@
         </is>
       </c>
       <c r="I84" t="n">
-        <v>71.209588</v>
+        <v>70.547386</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="58">
@@ -26968,7 +26990,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>590.46</v>
+        <v>578.01</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -26976,7 +26998,7 @@
         </is>
       </c>
       <c r="G85" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H85" s="34" t="inlineStr">
         <is>
@@ -26984,7 +27006,7 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>599.635366</v>
+        <v>601.050147</v>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="58">
@@ -27008,7 +27030,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>62188</v>
+        <v>61217</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -27016,7 +27038,7 @@
         </is>
       </c>
       <c r="G86" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H86" s="34" t="inlineStr">
         <is>
@@ -27024,7 +27046,7 @@
         </is>
       </c>
       <c r="I86" t="n">
-        <v>63196.676006</v>
+        <v>63347.78587</v>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="58">
@@ -27048,7 +27070,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.006486</v>
+        <v>0.006295</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -27056,7 +27078,7 @@
         </is>
       </c>
       <c r="G87" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H87" s="34" t="inlineStr">
         <is>
@@ -27064,7 +27086,7 @@
         </is>
       </c>
       <c r="I87" t="n">
-        <v>0.006796</v>
+        <v>0.006717</v>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="58">
@@ -27088,7 +27110,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.011835</v>
+        <v>0.011345</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -27096,7 +27118,7 @@
         </is>
       </c>
       <c r="G88" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H88" s="34" t="inlineStr">
         <is>
@@ -27104,7 +27126,7 @@
         </is>
       </c>
       <c r="I88" t="n">
-        <v>0.011725</v>
+        <v>0.012088</v>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="58">
@@ -27128,7 +27150,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>66.08</v>
+        <v>64.34</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -27136,7 +27158,7 @@
         </is>
       </c>
       <c r="G89" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H89" s="34" t="inlineStr">
         <is>
@@ -27144,7 +27166,7 @@
         </is>
       </c>
       <c r="I89" t="n">
-        <v>69.21765499999999</v>
+        <v>68.365793</v>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="58">
@@ -27168,7 +27190,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>1.67</v>
+        <v>1.6</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -27176,7 +27198,7 @@
         </is>
       </c>
       <c r="G90" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H90" s="34" t="inlineStr">
         <is>
@@ -27184,7 +27206,7 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>1.796942</v>
+        <v>1.795544</v>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="58">
@@ -27216,7 +27238,7 @@
         </is>
       </c>
       <c r="G91" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H91" s="34" t="inlineStr">
         <is>
@@ -27248,7 +27270,7 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
-        <v>0.013116</v>
+        <v>0.012655</v>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
@@ -27256,7 +27278,7 @@
         </is>
       </c>
       <c r="G92" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H92" s="34" t="inlineStr">
         <is>
@@ -27264,7 +27286,7 @@
         </is>
       </c>
       <c r="I92" t="n">
-        <v>0.013749</v>
+        <v>0.01391</v>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="58">
@@ -27288,7 +27310,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>2.67257</v>
+        <v>2.634447</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -27296,7 +27318,7 @@
         </is>
       </c>
       <c r="G93" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H93" s="34" t="inlineStr">
         <is>
@@ -27304,7 +27326,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>2.901514</v>
+        <v>2.906921</v>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="58">
@@ -27328,7 +27350,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>23.251206</v>
+        <v>23.650378</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -27336,7 +27358,7 @@
         </is>
       </c>
       <c r="G94" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H94" s="34" t="inlineStr">
         <is>
@@ -27344,7 +27366,7 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>25.31684</v>
+        <v>24.891208</v>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="58">
@@ -27368,7 +27390,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.114559</v>
+        <v>0.115016</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -27376,7 +27398,7 @@
         </is>
       </c>
       <c r="G95" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H95" s="34" t="inlineStr">
         <is>
@@ -27384,7 +27406,7 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>0.115746</v>
+        <v>0.122086</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="58">
@@ -27408,7 +27430,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>19237.1868</v>
+        <v>18952.9479</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -27416,7 +27438,7 @@
         </is>
       </c>
       <c r="G96" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H96" s="34" t="inlineStr">
         <is>
@@ -27424,7 +27446,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>19536.120235</v>
+        <v>19708.434332</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="58">
@@ -27448,7 +27470,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2026085.04</v>
+        <v>2007305.43</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -27456,7 +27478,7 @@
         </is>
       </c>
       <c r="G97" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H97" s="34" t="inlineStr">
         <is>
@@ -27464,7 +27486,7 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>2058947.704275</v>
+        <v>2077173.898675</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="58">
@@ -27488,7 +27510,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>2.73483</v>
+        <v>2.702585</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -27496,7 +27518,7 @@
         </is>
       </c>
       <c r="G98" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H98" s="34" t="inlineStr">
         <is>
@@ -27504,7 +27526,7 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>2.892489</v>
+        <v>2.872282</v>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="58">
@@ -27528,7 +27550,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>54190.9656</v>
+        <v>52139.7069</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -27536,7 +27558,7 @@
         </is>
       </c>
       <c r="G99" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H99" s="34" t="inlineStr">
         <is>
@@ -27544,7 +27566,7 @@
         </is>
       </c>
       <c r="I99" t="n">
-        <v>57486.623968</v>
+        <v>57599.469806</v>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="58">
@@ -27568,7 +27590,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>25.155604</v>
+        <v>24.877019</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -27576,7 +27598,7 @@
         </is>
       </c>
       <c r="G100" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H100" s="34" t="inlineStr">
         <is>
@@ -27584,7 +27606,7 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>25.135808</v>
+        <v>25.732259</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="58">
@@ -27608,7 +27630,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>62188</v>
+        <v>61217</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -27616,7 +27638,7 @@
         </is>
       </c>
       <c r="G101" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H101" s="34" t="inlineStr">
         <is>
@@ -27624,7 +27646,7 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>63196.676006</v>
+        <v>63347.78587</v>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="58">
@@ -27648,7 +27670,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>16.55</v>
+        <v>15.99</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -27656,7 +27678,7 @@
         </is>
       </c>
       <c r="G102" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H102" s="34" t="inlineStr">
         <is>
@@ -27664,7 +27686,7 @@
         </is>
       </c>
       <c r="I102" t="n">
-        <v>17.064611</v>
+        <v>16.844154</v>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="58">
@@ -27762,7 +27784,7 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
-        <v>0.006486</v>
+        <v>0.006295</v>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
@@ -27770,7 +27792,7 @@
         </is>
       </c>
       <c r="G105" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H105" s="34" t="inlineStr">
         <is>
@@ -27778,7 +27800,7 @@
         </is>
       </c>
       <c r="I105" t="n">
-        <v>0.006796</v>
+        <v>0.006717</v>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="58">
@@ -27802,7 +27824,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>66.08</v>
+        <v>64.34</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>
@@ -27810,7 +27832,7 @@
         </is>
       </c>
       <c r="G106" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H106" s="34" t="inlineStr">
         <is>
@@ -27818,7 +27840,7 @@
         </is>
       </c>
       <c r="I106" t="n">
-        <v>69.21765499999999</v>
+        <v>68.365793</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="58">
@@ -27850,7 +27872,7 @@
         </is>
       </c>
       <c r="G107" s="28" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="H107" s="34" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Weekly dashboard update — 2026-06-06
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-42660" yWindow="-540" windowWidth="32460" windowHeight="17180" tabRatio="500" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Realized" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Realized" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Prices" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Reference" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="AsOfDate">'FX &amp; Assumptions'!$C$5</definedName>
@@ -697,14 +697,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -726,8 +726,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -752,10 +752,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -764,10 +764,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4F81BD"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+              <a:ln w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -777,10 +777,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="C0504D"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -790,10 +790,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="9BBB59"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -803,10 +803,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="8064A2"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -816,10 +816,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4BACC6"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -829,10 +829,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="F79646"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -842,14 +842,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -875,14 +875,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -908,14 +908,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -941,14 +941,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -974,14 +974,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1007,14 +1007,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1038,16 +1038,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1142,16 +1142,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1172,10 +1172,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1187,14 +1187,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1216,8 +1216,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1242,10 +1242,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1254,10 +1254,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4672A8"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1267,10 +1267,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="AB4744"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1280,10 +1280,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="8AA64F"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1293,10 +1293,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="725990"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1306,10 +1306,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4299B0"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1319,10 +1319,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="DC853E"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1332,10 +1332,10 @@
             <idx val="6"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="93A9CE"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1345,10 +1345,10 @@
             <idx val="7"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="D09493"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1358,10 +1358,10 @@
             <idx val="8"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="B8CD97"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1371,14 +1371,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1405,14 +1405,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1439,14 +1439,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1473,14 +1473,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1507,14 +1507,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1541,14 +1541,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1575,14 +1575,14 @@
             <dLbl>
               <idx val="6"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1609,14 +1609,14 @@
             <dLbl>
               <idx val="7"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1643,14 +1643,14 @@
             <dLbl>
               <idx val="8"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1675,16 +1675,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1791,16 +1791,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1821,10 +1821,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1836,14 +1836,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1865,8 +1865,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1893,10 +1893,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1904,16 +1904,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2016,7 +2016,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2025,9 +2025,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2059,7 +2059,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2073,7 +2073,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2082,9 +2082,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2109,16 +2109,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2139,10 +2139,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2154,14 +2154,14 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -2183,8 +2183,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -2200,10 +2200,10 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2211,16 +2211,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2411,7 +2411,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2420,9 +2420,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2454,7 +2454,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2468,7 +2468,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2477,9 +2477,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2504,16 +2504,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2534,10 +2534,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2549,7 +2549,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>1</col>
@@ -2569,9 +2569,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2596,9 +2596,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+          <c:chart r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2623,9 +2623,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+          <c:chart r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2650,9 +2650,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+          <c:chart r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -21656,25 +21656,25 @@
         <v>46179</v>
       </c>
       <c r="C10" s="29" t="n">
-        <v>26792154</v>
+        <v>26482878</v>
       </c>
       <c r="D10" s="29" t="n">
         <v>22666838</v>
       </c>
       <c r="E10" s="29" t="n">
-        <v>4125316</v>
+        <v>3816041</v>
       </c>
       <c r="F10" s="30" t="n">
-        <v>0.182</v>
+        <v>0.1684</v>
       </c>
       <c r="G10" s="29" t="n">
-        <v>19315301</v>
+        <v>19003537</v>
       </c>
       <c r="H10" s="29" t="n">
         <v>4980397</v>
       </c>
       <c r="I10" s="29" t="n">
-        <v>1117917</v>
+        <v>1118930</v>
       </c>
       <c r="J10" s="31" t="n">
         <v>32.79</v>
@@ -23628,27 +23628,27 @@
         </is>
       </c>
       <c r="E5" s="33" t="n">
+        <v>26.0771</v>
+      </c>
+      <c r="F5" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G5" s="28" t="n">
+        <v>46177</v>
+      </c>
+      <c r="H5" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
         <v>26.6433</v>
       </c>
-      <c r="F5" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G5" s="28" t="n">
-        <v>46175</v>
-      </c>
-      <c r="H5" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I5" t="n">
-        <v>24.9174</v>
-      </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-02</t>
         </is>
       </c>
     </row>
@@ -23681,7 +23681,7 @@
         </is>
       </c>
       <c r="G6" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H6" s="34" t="inlineStr">
         <is>
@@ -23689,11 +23689,11 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>10.6854</v>
+        <v>10.6859</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
@@ -23718,27 +23718,27 @@
         </is>
       </c>
       <c r="E7" s="33" t="n">
+        <v>7.1186</v>
+      </c>
+      <c r="F7" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G7" s="28" t="n">
+        <v>46177</v>
+      </c>
+      <c r="H7" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
         <v>7.1237</v>
       </c>
-      <c r="F7" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G7" s="28" t="n">
-        <v>46175</v>
-      </c>
-      <c r="H7" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I7" t="n">
-        <v>7.1767</v>
-      </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-02</t>
         </is>
       </c>
     </row>
@@ -23763,27 +23763,27 @@
         </is>
       </c>
       <c r="E8" s="33" t="n">
+        <v>9.7468</v>
+      </c>
+      <c r="F8" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G8" s="28" t="n">
+        <v>46177</v>
+      </c>
+      <c r="H8" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
         <v>9.7875</v>
       </c>
-      <c r="F8" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G8" s="28" t="n">
-        <v>46175</v>
-      </c>
-      <c r="H8" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I8" t="n">
-        <v>9.613200000000001</v>
-      </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-02</t>
         </is>
       </c>
     </row>
@@ -23808,27 +23808,27 @@
         </is>
       </c>
       <c r="E9" s="33" t="n">
+        <v>9.320600000000001</v>
+      </c>
+      <c r="F9" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G9" s="28" t="n">
+        <v>46178</v>
+      </c>
+      <c r="H9" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
         <v>9.4649</v>
       </c>
-      <c r="F9" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G9" s="28" t="n">
-        <v>46177</v>
-      </c>
-      <c r="H9" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I9" t="n">
-        <v>9.4183</v>
-      </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
@@ -23853,27 +23853,27 @@
         </is>
       </c>
       <c r="E10" s="33" t="n">
+        <v>13.6486</v>
+      </c>
+      <c r="F10" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G10" s="28" t="n">
+        <v>46177</v>
+      </c>
+      <c r="H10" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
         <v>13.4306</v>
       </c>
-      <c r="F10" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G10" s="28" t="n">
-        <v>46175</v>
-      </c>
-      <c r="H10" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I10" t="n">
-        <v>13.4811</v>
-      </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-02</t>
         </is>
       </c>
     </row>
@@ -23898,27 +23898,27 @@
         </is>
       </c>
       <c r="E11" s="33" t="n">
+        <v>13.2022</v>
+      </c>
+      <c r="F11" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G11" s="28" t="n">
+        <v>46178</v>
+      </c>
+      <c r="H11" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
         <v>13.3664</v>
       </c>
-      <c r="F11" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G11" s="28" t="n">
-        <v>46177</v>
-      </c>
-      <c r="H11" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I11" t="n">
-        <v>13.3792</v>
-      </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
@@ -23943,27 +23943,27 @@
         </is>
       </c>
       <c r="E12" s="33" t="n">
+        <v>26.689</v>
+      </c>
+      <c r="F12" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G12" s="28" t="n">
+        <v>46178</v>
+      </c>
+      <c r="H12" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
         <v>27.1532</v>
       </c>
-      <c r="F12" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G12" s="28" t="n">
-        <v>46177</v>
-      </c>
-      <c r="H12" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I12" t="n">
-        <v>26.9938</v>
-      </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
@@ -23988,27 +23988,27 @@
         </is>
       </c>
       <c r="E13" s="33" t="n">
+        <v>36.2424</v>
+      </c>
+      <c r="F13" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G13" s="28" t="n">
+        <v>46178</v>
+      </c>
+      <c r="H13" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
         <v>36.5235</v>
       </c>
-      <c r="F13" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G13" s="28" t="n">
-        <v>46177</v>
-      </c>
-      <c r="H13" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I13" t="n">
-        <v>36.3651</v>
-      </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
@@ -24033,27 +24033,27 @@
         </is>
       </c>
       <c r="E14" s="33" t="n">
+        <v>25.4991</v>
+      </c>
+      <c r="F14" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G14" s="28" t="n">
+        <v>46178</v>
+      </c>
+      <c r="H14" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
         <v>25.5684</v>
       </c>
-      <c r="F14" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G14" s="28" t="n">
-        <v>46177</v>
-      </c>
-      <c r="H14" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I14" t="n">
-        <v>25.4878</v>
-      </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
@@ -24078,27 +24078,27 @@
         </is>
       </c>
       <c r="E15" s="33" t="n">
+        <v>14.3709</v>
+      </c>
+      <c r="F15" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G15" s="28" t="n">
+        <v>46175</v>
+      </c>
+      <c r="H15" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
         <v>14.8616</v>
       </c>
-      <c r="F15" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G15" s="28" t="n">
-        <v>46171</v>
-      </c>
-      <c r="H15" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I15" t="n">
-        <v>14.9551</v>
-      </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
     </row>
@@ -24123,27 +24123,27 @@
         </is>
       </c>
       <c r="E16" s="33" t="n">
+        <v>81.4024</v>
+      </c>
+      <c r="F16" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G16" s="28" t="n">
+        <v>46178</v>
+      </c>
+      <c r="H16" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
         <v>81.99809999999999</v>
       </c>
-      <c r="F16" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G16" s="28" t="n">
-        <v>46177</v>
-      </c>
-      <c r="H16" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I16" t="n">
-        <v>81.6082</v>
-      </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
@@ -24168,27 +24168,27 @@
         </is>
       </c>
       <c r="E17" s="33" t="n">
+        <v>53.4695</v>
+      </c>
+      <c r="F17" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G17" s="28" t="n">
+        <v>46178</v>
+      </c>
+      <c r="H17" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
         <v>53.6077</v>
       </c>
-      <c r="F17" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G17" s="28" t="n">
-        <v>46177</v>
-      </c>
-      <c r="H17" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I17" t="n">
-        <v>53.4438</v>
-      </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
@@ -24213,27 +24213,27 @@
         </is>
       </c>
       <c r="E18" s="33" t="n">
+        <v>16.4291</v>
+      </c>
+      <c r="F18" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G18" s="28" t="n">
+        <v>46178</v>
+      </c>
+      <c r="H18" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
         <v>16.4146</v>
       </c>
-      <c r="F18" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G18" s="28" t="n">
-        <v>46177</v>
-      </c>
-      <c r="H18" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I18" t="n">
-        <v>16.4262</v>
-      </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
@@ -24258,27 +24258,27 @@
         </is>
       </c>
       <c r="E19" s="33" t="n">
+        <v>23.4013</v>
+      </c>
+      <c r="F19" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G19" s="28" t="n">
+        <v>46178</v>
+      </c>
+      <c r="H19" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
         <v>23.4009</v>
       </c>
-      <c r="F19" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G19" s="28" t="n">
-        <v>46177</v>
-      </c>
-      <c r="H19" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I19" t="n">
-        <v>23.3999</v>
-      </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
@@ -24303,27 +24303,27 @@
         </is>
       </c>
       <c r="E20" s="33" t="n">
+        <v>41.6601</v>
+      </c>
+      <c r="F20" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G20" s="28" t="n">
+        <v>46177</v>
+      </c>
+      <c r="H20" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
         <v>41.7733</v>
       </c>
-      <c r="F20" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G20" s="28" t="n">
-        <v>46175</v>
-      </c>
-      <c r="H20" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I20" t="n">
-        <v>41.6338</v>
-      </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-02</t>
         </is>
       </c>
     </row>
@@ -24348,27 +24348,27 @@
         </is>
       </c>
       <c r="E21" s="33" t="n">
+        <v>13.3947</v>
+      </c>
+      <c r="F21" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G21" s="28" t="n">
+        <v>46178</v>
+      </c>
+      <c r="H21" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
         <v>13.6591</v>
       </c>
-      <c r="F21" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G21" s="28" t="n">
-        <v>46177</v>
-      </c>
-      <c r="H21" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I21" t="n">
-        <v>13.8066</v>
-      </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
@@ -24393,27 +24393,27 @@
         </is>
       </c>
       <c r="E22" s="33" t="n">
+        <v>13.1535</v>
+      </c>
+      <c r="F22" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G22" s="28" t="n">
+        <v>46177</v>
+      </c>
+      <c r="H22" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
         <v>12.6846</v>
       </c>
-      <c r="F22" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G22" s="28" t="n">
-        <v>46175</v>
-      </c>
-      <c r="H22" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I22" t="n">
-        <v>13.1472</v>
-      </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-02</t>
         </is>
       </c>
     </row>
@@ -24438,27 +24438,27 @@
         </is>
       </c>
       <c r="E23" s="33" t="n">
+        <v>12.4665</v>
+      </c>
+      <c r="F23" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G23" s="28" t="n">
+        <v>46178</v>
+      </c>
+      <c r="H23" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
         <v>12.5147</v>
       </c>
-      <c r="F23" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G23" s="28" t="n">
-        <v>46177</v>
-      </c>
-      <c r="H23" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I23" t="n">
-        <v>12.4675</v>
-      </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
@@ -24483,27 +24483,27 @@
         </is>
       </c>
       <c r="E24" s="33" t="n">
+        <v>12.0868</v>
+      </c>
+      <c r="F24" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G24" s="28" t="n">
+        <v>46177</v>
+      </c>
+      <c r="H24" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
         <v>12.3129</v>
       </c>
-      <c r="F24" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G24" s="28" t="n">
-        <v>46175</v>
-      </c>
-      <c r="H24" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I24" t="n">
-        <v>12.2697</v>
-      </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-02</t>
         </is>
       </c>
     </row>
@@ -24528,27 +24528,27 @@
         </is>
       </c>
       <c r="E25" s="33" t="n">
+        <v>10.0147</v>
+      </c>
+      <c r="F25" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G25" s="28" t="n">
+        <v>46178</v>
+      </c>
+      <c r="H25" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
         <v>10.0259</v>
       </c>
-      <c r="F25" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G25" s="28" t="n">
-        <v>46177</v>
-      </c>
-      <c r="H25" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I25" t="n">
-        <v>9.889799999999999</v>
-      </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
@@ -24573,27 +24573,27 @@
         </is>
       </c>
       <c r="E26" s="33" t="n">
+        <v>14.0583</v>
+      </c>
+      <c r="F26" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G26" s="28" t="n">
+        <v>46178</v>
+      </c>
+      <c r="H26" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
         <v>14.078</v>
       </c>
-      <c r="F26" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G26" s="28" t="n">
-        <v>46177</v>
-      </c>
-      <c r="H26" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I26" t="n">
-        <v>13.8759</v>
-      </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
@@ -24618,27 +24618,27 @@
         </is>
       </c>
       <c r="E27" s="33" t="n">
+        <v>17.105</v>
+      </c>
+      <c r="F27" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G27" s="28" t="n">
+        <v>46178</v>
+      </c>
+      <c r="H27" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
         <v>17.1468</v>
       </c>
-      <c r="F27" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G27" s="28" t="n">
-        <v>46177</v>
-      </c>
-      <c r="H27" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I27" t="n">
-        <v>17.1932</v>
-      </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
@@ -24663,27 +24663,27 @@
         </is>
       </c>
       <c r="E28" s="33" t="n">
+        <v>19.8791</v>
+      </c>
+      <c r="F28" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G28" s="28" t="n">
+        <v>46178</v>
+      </c>
+      <c r="H28" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
         <v>19.8865</v>
       </c>
-      <c r="F28" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G28" s="28" t="n">
-        <v>46177</v>
-      </c>
-      <c r="H28" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I28" t="n">
-        <v>20.1658</v>
-      </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
@@ -24708,27 +24708,27 @@
         </is>
       </c>
       <c r="E29" s="33" t="n">
+        <v>27.8357</v>
+      </c>
+      <c r="F29" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G29" s="28" t="n">
+        <v>46177</v>
+      </c>
+      <c r="H29" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
         <v>29.2852</v>
       </c>
-      <c r="F29" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G29" s="28" t="n">
-        <v>46175</v>
-      </c>
-      <c r="H29" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I29" t="n">
-        <v>28.1054</v>
-      </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-02</t>
         </is>
       </c>
     </row>
@@ -24753,27 +24753,27 @@
         </is>
       </c>
       <c r="E30" s="33" t="n">
+        <v>38.836</v>
+      </c>
+      <c r="F30" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G30" s="28" t="n">
+        <v>46177</v>
+      </c>
+      <c r="H30" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
         <v>39.0534</v>
       </c>
-      <c r="F30" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G30" s="28" t="n">
-        <v>46175</v>
-      </c>
-      <c r="H30" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I30" t="n">
-        <v>37.5072</v>
-      </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-02</t>
         </is>
       </c>
     </row>
@@ -24798,27 +24798,27 @@
         </is>
       </c>
       <c r="E31" s="33" t="n">
+        <v>12.9367</v>
+      </c>
+      <c r="F31" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G31" s="28" t="n">
+        <v>46178</v>
+      </c>
+      <c r="H31" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
         <v>13.0307</v>
       </c>
-      <c r="F31" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G31" s="28" t="n">
-        <v>46177</v>
-      </c>
-      <c r="H31" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I31" t="n">
-        <v>12.9839</v>
-      </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
@@ -24851,7 +24851,7 @@
         </is>
       </c>
       <c r="G32" s="28" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="H32" s="34" t="inlineStr">
         <is>
@@ -24859,11 +24859,11 @@
         </is>
       </c>
       <c r="I32" t="n">
-        <v>21.7042</v>
+        <v>21.7047</v>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
@@ -24888,27 +24888,27 @@
         </is>
       </c>
       <c r="E33" s="33" t="n">
+        <v>12.5235</v>
+      </c>
+      <c r="F33" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G33" s="28" t="n">
+        <v>46178</v>
+      </c>
+      <c r="H33" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
         <v>12.5995</v>
       </c>
-      <c r="F33" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G33" s="28" t="n">
-        <v>46177</v>
-      </c>
-      <c r="H33" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I33" t="n">
-        <v>12.5913</v>
-      </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
@@ -24933,27 +24933,27 @@
         </is>
       </c>
       <c r="E34" s="33" t="n">
+        <v>16.203</v>
+      </c>
+      <c r="F34" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G34" s="28" t="n">
+        <v>46178</v>
+      </c>
+      <c r="H34" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
         <v>16.2028</v>
       </c>
-      <c r="F34" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G34" s="28" t="n">
-        <v>46177</v>
-      </c>
-      <c r="H34" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I34" t="n">
-        <v>16.2021</v>
-      </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
@@ -24978,27 +24978,27 @@
         </is>
       </c>
       <c r="E35" s="33" t="n">
+        <v>28.936</v>
+      </c>
+      <c r="F35" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G35" s="28" t="n">
+        <v>46177</v>
+      </c>
+      <c r="H35" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
         <v>28.8772</v>
       </c>
-      <c r="F35" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G35" s="28" t="n">
-        <v>46175</v>
-      </c>
-      <c r="H35" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I35" t="n">
-        <v>29.2628</v>
-      </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-02</t>
         </is>
       </c>
     </row>
@@ -25023,27 +25023,27 @@
         </is>
       </c>
       <c r="E36" s="33" t="n">
+        <v>10.032</v>
+      </c>
+      <c r="F36" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G36" s="28" t="n">
+        <v>46178</v>
+      </c>
+      <c r="H36" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
         <v>9.992800000000001</v>
       </c>
-      <c r="F36" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G36" s="28" t="n">
-        <v>46177</v>
-      </c>
-      <c r="H36" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I36" t="n">
-        <v>10.0313</v>
-      </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
@@ -25068,27 +25068,27 @@
         </is>
       </c>
       <c r="E37" s="33" t="n">
+        <v>22.6458</v>
+      </c>
+      <c r="F37" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G37" s="28" t="n">
+        <v>46178</v>
+      </c>
+      <c r="H37" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
         <v>22.7858</v>
       </c>
-      <c r="F37" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G37" s="28" t="n">
-        <v>46177</v>
-      </c>
-      <c r="H37" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I37" t="n">
-        <v>22.7382</v>
-      </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
@@ -25153,7 +25153,7 @@
         </is>
       </c>
       <c r="E39" s="33" t="n">
-        <v>1.094</v>
+        <v>1.1</v>
       </c>
       <c r="F39" s="34" t="inlineStr">
         <is>
@@ -26950,7 +26950,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>62.18</v>
+        <v>62.17</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -26966,7 +26966,7 @@
         </is>
       </c>
       <c r="I84" t="n">
-        <v>70.547386</v>
+        <v>68.498785</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="58">
@@ -26990,7 +26990,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>578.01</v>
+        <v>581.25</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -27006,7 +27006,7 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>601.050147</v>
+        <v>594.400875</v>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="58">
@@ -27030,7 +27030,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>61217</v>
+        <v>61244</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -27046,7 +27046,7 @@
         </is>
       </c>
       <c r="I86" t="n">
-        <v>63347.78587</v>
+        <v>62963.64963</v>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="58">
@@ -27070,7 +27070,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.006295</v>
+        <v>0.006448</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -27086,7 +27086,7 @@
         </is>
       </c>
       <c r="I87" t="n">
-        <v>0.006717</v>
+        <v>0.006566</v>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="58">
@@ -27110,7 +27110,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.011345</v>
+        <v>0.01128</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -27126,7 +27126,7 @@
         </is>
       </c>
       <c r="I88" t="n">
-        <v>0.012088</v>
+        <v>0.012159</v>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="58">
@@ -27150,7 +27150,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>64.34</v>
+        <v>63.4</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -27166,7 +27166,7 @@
         </is>
       </c>
       <c r="I89" t="n">
-        <v>68.365793</v>
+        <v>66.265202</v>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="58">
@@ -27190,7 +27190,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>1.6</v>
+        <v>1.59</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -27206,7 +27206,7 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>1.795544</v>
+        <v>1.687395</v>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="58">
@@ -27270,7 +27270,7 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
-        <v>0.012655</v>
+        <v>0.012583</v>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
@@ -27286,7 +27286,7 @@
         </is>
       </c>
       <c r="I92" t="n">
-        <v>0.01391</v>
+        <v>0.013199</v>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="58">
@@ -27310,7 +27310,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>2.634447</v>
+        <v>2.638644</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -27326,7 +27326,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>2.906921</v>
+        <v>2.770454</v>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="58">
@@ -27350,7 +27350,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>23.650378</v>
+        <v>23.509446</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -27366,7 +27366,7 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>24.891208</v>
+        <v>23.297458</v>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="58">
@@ -27390,7 +27390,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.115016</v>
+        <v>0.113668</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -27406,7 +27406,7 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>0.122086</v>
+        <v>0.116796</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="58">
@@ -27430,7 +27430,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>18952.9479</v>
+        <v>19059.1875</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -27446,7 +27446,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>19708.434332</v>
+        <v>19490.404688</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="58">
@@ -27470,7 +27470,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2007305.43</v>
+        <v>2008190.76</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -27486,7 +27486,7 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>2077173.898675</v>
+        <v>2064578.071369</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="58">
@@ -27510,7 +27510,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>2.702585</v>
+        <v>2.699601</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -27526,7 +27526,7 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>2.872282</v>
+        <v>2.770252</v>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="58">
@@ -27550,7 +27550,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>52139.7069</v>
+        <v>51986.2497</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -27566,7 +27566,7 @@
         </is>
       </c>
       <c r="I99" t="n">
-        <v>57599.469806</v>
+        <v>55173.860105</v>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="58">
@@ -27590,7 +27590,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>24.877019</v>
+        <v>24.822489</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -27606,7 +27606,7 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>25.732259</v>
+        <v>25.476315</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="58">
@@ -27630,7 +27630,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>61217</v>
+        <v>61244</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -27646,7 +27646,7 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>63347.78587</v>
+        <v>62963.64963</v>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="58">
@@ -27670,7 +27670,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>15.99</v>
+        <v>16.04</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -27686,7 +27686,7 @@
         </is>
       </c>
       <c r="I102" t="n">
-        <v>16.844154</v>
+        <v>16.73971</v>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="58">
@@ -27784,7 +27784,7 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
-        <v>0.006295</v>
+        <v>0.006448</v>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
@@ -27800,7 +27800,7 @@
         </is>
       </c>
       <c r="I105" t="n">
-        <v>0.006717</v>
+        <v>0.006566</v>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="58">
@@ -27824,7 +27824,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>64.34</v>
+        <v>63.4</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>
@@ -27840,7 +27840,7 @@
         </is>
       </c>
       <c r="I106" t="n">
-        <v>68.365793</v>
+        <v>66.265202</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="58">

</xml_diff>

<commit_message>
Daily dashboard update — 2026-06-07
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-42660" yWindow="-540" windowWidth="32460" windowHeight="17180" tabRatio="500" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Realized" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Prices" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Reference" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Realized" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="AsOfDate">'FX &amp; Assumptions'!$C$5</definedName>
@@ -697,14 +697,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -726,8 +726,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -752,10 +752,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -764,10 +764,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4F81BD"/>
               </a:solidFill>
-              <a:ln w="0">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -777,10 +777,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="C0504D"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -790,10 +790,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="9BBB59"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -803,10 +803,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="8064A2"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -816,10 +816,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4BACC6"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -829,10 +829,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="F79646"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -842,14 +842,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -875,14 +875,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -908,14 +908,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -941,14 +941,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -974,14 +974,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1007,14 +1007,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1038,16 +1038,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1142,16 +1142,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1172,10 +1172,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1187,14 +1187,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1216,8 +1216,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1242,10 +1242,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1254,10 +1254,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4672A8"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1267,10 +1267,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="AB4744"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1280,10 +1280,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="8AA64F"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1293,10 +1293,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="725990"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1306,10 +1306,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4299B0"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1319,10 +1319,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="DC853E"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1332,10 +1332,10 @@
             <idx val="6"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="93A9CE"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1345,10 +1345,10 @@
             <idx val="7"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="D09493"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1358,10 +1358,10 @@
             <idx val="8"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="B8CD97"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1371,14 +1371,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1405,14 +1405,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1439,14 +1439,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1473,14 +1473,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1507,14 +1507,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1541,14 +1541,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1575,14 +1575,14 @@
             <dLbl>
               <idx val="6"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1609,14 +1609,14 @@
             <dLbl>
               <idx val="7"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1643,14 +1643,14 @@
             <dLbl>
               <idx val="8"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1675,16 +1675,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1791,16 +1791,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1821,10 +1821,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1836,14 +1836,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1865,8 +1865,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1893,10 +1893,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1904,16 +1904,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2016,7 +2016,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2025,9 +2025,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2059,7 +2059,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="9360">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2073,7 +2073,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2082,9 +2082,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2109,16 +2109,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2139,10 +2139,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2154,14 +2154,14 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -2183,8 +2183,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -2200,10 +2200,10 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2211,16 +2211,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2411,7 +2411,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2420,9 +2420,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2454,7 +2454,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="9360">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2468,7 +2468,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2477,9 +2477,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2504,16 +2504,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2534,10 +2534,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2549,7 +2549,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>1</col>
@@ -2569,9 +2569,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2596,9 +2596,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2623,9 +2623,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId3"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2650,9 +2650,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId4"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -21686,16 +21686,38 @@
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="58">
-      <c r="B11" s="28" t="n"/>
-      <c r="C11" s="29" t="n"/>
-      <c r="D11" s="29" t="n"/>
-      <c r="E11" s="29" t="n"/>
-      <c r="F11" s="30" t="n"/>
-      <c r="G11" s="29" t="n"/>
-      <c r="H11" s="29" t="n"/>
-      <c r="I11" s="29" t="n"/>
-      <c r="J11" s="31" t="n"/>
-      <c r="K11" s="32" t="n"/>
+      <c r="B11" s="28" t="n">
+        <v>46180</v>
+      </c>
+      <c r="C11" s="29" t="n">
+        <v>26487092</v>
+      </c>
+      <c r="D11" s="29" t="n">
+        <v>22666838</v>
+      </c>
+      <c r="E11" s="29" t="n">
+        <v>3820254</v>
+      </c>
+      <c r="F11" s="30" t="n">
+        <v>0.1685</v>
+      </c>
+      <c r="G11" s="29" t="n">
+        <v>19003537</v>
+      </c>
+      <c r="H11" s="29" t="n">
+        <v>4980397</v>
+      </c>
+      <c r="I11" s="29" t="n">
+        <v>1123143</v>
+      </c>
+      <c r="J11" s="31" t="n">
+        <v>32.79</v>
+      </c>
+      <c r="K11" s="32" t="inlineStr">
+        <is>
+          <t>Auto weekly snapshot</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="58">
       <c r="B12" s="28" t="n"/>
@@ -23445,7 +23467,7 @@
         </is>
       </c>
       <c r="C5" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="D5" s="64" t="inlineStr">
         <is>
@@ -23464,7 +23486,7 @@
       </c>
       <c r="D6" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-06-06</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-06-07</t>
         </is>
       </c>
     </row>
@@ -23513,7 +23535,7 @@
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-06-06</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-06-07</t>
         </is>
       </c>
     </row>
@@ -25121,7 +25143,7 @@
         </is>
       </c>
       <c r="G38" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H38" s="34" t="inlineStr">
         <is>
@@ -25161,7 +25183,7 @@
         </is>
       </c>
       <c r="G39" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H39" s="34" t="inlineStr">
         <is>
@@ -25201,7 +25223,7 @@
         </is>
       </c>
       <c r="G40" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H40" s="34" t="inlineStr">
         <is>
@@ -25241,7 +25263,7 @@
         </is>
       </c>
       <c r="G41" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H41" s="34" t="inlineStr">
         <is>
@@ -25281,7 +25303,7 @@
         </is>
       </c>
       <c r="G42" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H42" s="34" t="inlineStr">
         <is>
@@ -25321,7 +25343,7 @@
         </is>
       </c>
       <c r="G43" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H43" s="34" t="inlineStr">
         <is>
@@ -25361,7 +25383,7 @@
         </is>
       </c>
       <c r="G44" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H44" s="34" t="inlineStr">
         <is>
@@ -25401,7 +25423,7 @@
         </is>
       </c>
       <c r="G45" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H45" s="34" t="inlineStr">
         <is>
@@ -25441,7 +25463,7 @@
         </is>
       </c>
       <c r="G46" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H46" s="34" t="inlineStr">
         <is>
@@ -25518,7 +25540,7 @@
         </is>
       </c>
       <c r="G48" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H48" s="34" t="inlineStr">
         <is>
@@ -25558,7 +25580,7 @@
         </is>
       </c>
       <c r="G49" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H49" s="34" t="inlineStr">
         <is>
@@ -25598,7 +25620,7 @@
         </is>
       </c>
       <c r="G50" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H50" s="34" t="inlineStr">
         <is>
@@ -25638,7 +25660,7 @@
         </is>
       </c>
       <c r="G51" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H51" s="34" t="inlineStr">
         <is>
@@ -25678,7 +25700,7 @@
         </is>
       </c>
       <c r="G52" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H52" s="34" t="inlineStr">
         <is>
@@ -25718,7 +25740,7 @@
         </is>
       </c>
       <c r="G53" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H53" s="34" t="inlineStr">
         <is>
@@ -25758,7 +25780,7 @@
         </is>
       </c>
       <c r="G54" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H54" s="34" t="inlineStr">
         <is>
@@ -25798,7 +25820,7 @@
         </is>
       </c>
       <c r="G55" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H55" s="34" t="inlineStr">
         <is>
@@ -25838,7 +25860,7 @@
         </is>
       </c>
       <c r="G56" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H56" s="34" t="inlineStr">
         <is>
@@ -25878,7 +25900,7 @@
         </is>
       </c>
       <c r="G57" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H57" s="34" t="inlineStr">
         <is>
@@ -25918,7 +25940,7 @@
         </is>
       </c>
       <c r="G58" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H58" s="34" t="inlineStr">
         <is>
@@ -25958,7 +25980,7 @@
         </is>
       </c>
       <c r="G59" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H59" s="34" t="inlineStr">
         <is>
@@ -25998,7 +26020,7 @@
         </is>
       </c>
       <c r="G60" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H60" s="34" t="inlineStr">
         <is>
@@ -26038,7 +26060,7 @@
         </is>
       </c>
       <c r="G61" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H61" s="34" t="inlineStr">
         <is>
@@ -26078,7 +26100,7 @@
         </is>
       </c>
       <c r="G62" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H62" s="34" t="inlineStr">
         <is>
@@ -26118,7 +26140,7 @@
         </is>
       </c>
       <c r="G63" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H63" s="34" t="inlineStr">
         <is>
@@ -26158,7 +26180,7 @@
         </is>
       </c>
       <c r="G64" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H64" s="34" t="inlineStr">
         <is>
@@ -26198,7 +26220,7 @@
         </is>
       </c>
       <c r="G65" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H65" s="34" t="inlineStr">
         <is>
@@ -26238,7 +26260,7 @@
         </is>
       </c>
       <c r="G66" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H66" s="34" t="inlineStr">
         <is>
@@ -26278,7 +26300,7 @@
         </is>
       </c>
       <c r="G67" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H67" s="34" t="inlineStr">
         <is>
@@ -26318,7 +26340,7 @@
         </is>
       </c>
       <c r="G68" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H68" s="34" t="inlineStr">
         <is>
@@ -26358,7 +26380,7 @@
         </is>
       </c>
       <c r="G69" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H69" s="34" t="inlineStr">
         <is>
@@ -26398,7 +26420,7 @@
         </is>
       </c>
       <c r="G70" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H70" s="34" t="inlineStr">
         <is>
@@ -26438,7 +26460,7 @@
         </is>
       </c>
       <c r="G71" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H71" s="34" t="inlineStr">
         <is>
@@ -26478,7 +26500,7 @@
         </is>
       </c>
       <c r="G72" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H72" s="34" t="inlineStr">
         <is>
@@ -26518,7 +26540,7 @@
         </is>
       </c>
       <c r="G73" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H73" s="34" t="inlineStr">
         <is>
@@ -26558,7 +26580,7 @@
         </is>
       </c>
       <c r="G74" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H74" s="34" t="inlineStr">
         <is>
@@ -26598,7 +26620,7 @@
         </is>
       </c>
       <c r="G75" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H75" s="34" t="inlineStr">
         <is>
@@ -26638,7 +26660,7 @@
         </is>
       </c>
       <c r="G76" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H76" s="34" t="inlineStr">
         <is>
@@ -26678,7 +26700,7 @@
         </is>
       </c>
       <c r="G77" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H77" s="34" t="inlineStr">
         <is>
@@ -26718,7 +26740,7 @@
         </is>
       </c>
       <c r="G78" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H78" s="34" t="inlineStr">
         <is>
@@ -26758,7 +26780,7 @@
         </is>
       </c>
       <c r="G79" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H79" s="34" t="inlineStr">
         <is>
@@ -26798,7 +26820,7 @@
         </is>
       </c>
       <c r="G80" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H80" s="34" t="inlineStr">
         <is>
@@ -26838,7 +26860,7 @@
         </is>
       </c>
       <c r="G81" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H81" s="34" t="inlineStr">
         <is>
@@ -26878,7 +26900,7 @@
         </is>
       </c>
       <c r="G82" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H82" s="34" t="inlineStr">
         <is>
@@ -26918,7 +26940,7 @@
         </is>
       </c>
       <c r="G83" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H83" s="34" t="inlineStr">
         <is>
@@ -26950,7 +26972,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>60.73</v>
+        <v>62.1</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -26958,7 +26980,7 @@
         </is>
       </c>
       <c r="G84" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H84" s="34" t="inlineStr">
         <is>
@@ -26966,7 +26988,7 @@
         </is>
       </c>
       <c r="I84" t="n">
-        <v>67.386906</v>
+        <v>62.187501</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="58">
@@ -26990,7 +27012,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>575.05</v>
+        <v>580.46</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -26998,7 +27020,7 @@
         </is>
       </c>
       <c r="G85" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H85" s="34" t="inlineStr">
         <is>
@@ -27006,7 +27028,7 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>591.937527</v>
+        <v>577.779634</v>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="58">
@@ -27030,7 +27052,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>60586</v>
+        <v>61546</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -27038,7 +27060,7 @@
         </is>
       </c>
       <c r="G86" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H86" s="34" t="inlineStr">
         <is>
@@ -27046,7 +27068,7 @@
         </is>
       </c>
       <c r="I86" t="n">
-        <v>62522.52055</v>
+        <v>61204.489244</v>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="58">
@@ -27070,7 +27092,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.006181</v>
+        <v>0.006497</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -27078,7 +27100,7 @@
         </is>
       </c>
       <c r="G87" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H87" s="34" t="inlineStr">
         <is>
@@ -27086,7 +27108,7 @@
         </is>
       </c>
       <c r="I87" t="n">
-        <v>0.006516</v>
+        <v>0.006297</v>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="58">
@@ -27110,7 +27132,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.010982</v>
+        <v>0.011545</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -27118,7 +27140,7 @@
         </is>
       </c>
       <c r="G88" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H88" s="34" t="inlineStr">
         <is>
@@ -27126,7 +27148,7 @@
         </is>
       </c>
       <c r="I88" t="n">
-        <v>0.012292</v>
+        <v>0.011338</v>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="58">
@@ -27150,7 +27172,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>61.93</v>
+        <v>63.55</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -27158,7 +27180,7 @@
         </is>
       </c>
       <c r="G89" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H89" s="34" t="inlineStr">
         <is>
@@ -27166,7 +27188,7 @@
         </is>
       </c>
       <c r="I89" t="n">
-        <v>66.351797</v>
+        <v>64.340321</v>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="58">
@@ -27190,7 +27212,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>1.55</v>
+        <v>1.62</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -27198,7 +27220,7 @@
         </is>
       </c>
       <c r="G90" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H90" s="34" t="inlineStr">
         <is>
@@ -27206,7 +27228,7 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>1.67566</v>
+        <v>1.604315</v>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="58">
@@ -27238,7 +27260,7 @@
         </is>
       </c>
       <c r="G91" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H91" s="34" t="inlineStr">
         <is>
@@ -27270,7 +27292,7 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
-        <v>0.012336</v>
+        <v>0.012717</v>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
@@ -27278,7 +27300,7 @@
         </is>
       </c>
       <c r="G92" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H92" s="34" t="inlineStr">
         <is>
@@ -27286,7 +27308,7 @@
         </is>
       </c>
       <c r="I92" t="n">
-        <v>0.013129</v>
+        <v>0.012668</v>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="58">
@@ -27310,7 +27332,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>2.583196</v>
+        <v>2.689173</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -27318,7 +27340,7 @@
         </is>
       </c>
       <c r="G93" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H93" s="34" t="inlineStr">
         <is>
@@ -27326,7 +27348,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>2.749885</v>
+        <v>2.638235</v>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="58">
@@ -27350,7 +27372,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>22.768491</v>
+        <v>24.484457</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -27358,7 +27380,7 @@
         </is>
       </c>
       <c r="G94" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H94" s="34" t="inlineStr">
         <is>
@@ -27366,7 +27388,7 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>23.429973</v>
+        <v>23.647407</v>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="58">
@@ -27390,7 +27412,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.112187</v>
+        <v>0.115422</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -27398,7 +27420,7 @@
         </is>
       </c>
       <c r="G95" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H95" s="34" t="inlineStr">
         <is>
@@ -27406,7 +27428,7 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>0.116724</v>
+        <v>0.115185</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="58">
@@ -27430,7 +27452,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>18855.8895</v>
+        <v>19033.2834</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -27438,7 +27460,7 @@
         </is>
       </c>
       <c r="G96" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H96" s="34" t="inlineStr">
         <is>
@@ -27446,7 +27468,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>19409.631506</v>
+        <v>18945.394191</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="58">
@@ -27470,7 +27492,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>1986614.94</v>
+        <v>2018093.34</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -27478,7 +27500,7 @@
         </is>
       </c>
       <c r="G97" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H97" s="34" t="inlineStr">
         <is>
@@ -27486,7 +27508,7 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>2050113.448844</v>
+        <v>2006895.202308</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="58">
@@ -27510,7 +27532,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>2.638316</v>
+        <v>2.735047</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -27518,7 +27540,7 @@
         </is>
       </c>
       <c r="G98" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H98" s="34" t="inlineStr">
         <is>
@@ -27526,7 +27548,7 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>2.775044</v>
+        <v>2.702748</v>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="58">
@@ -27550,7 +27572,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>51072.7203</v>
+        <v>52215.1239</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -27558,7 +27580,7 @@
         </is>
       </c>
       <c r="G99" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H99" s="34" t="inlineStr">
         <is>
@@ -27566,7 +27588,7 @@
         </is>
       </c>
       <c r="I99" t="n">
-        <v>54915.067131</v>
+        <v>52127.545269</v>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="58">
@@ -27590,7 +27612,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>24.76714</v>
+        <v>24.556431</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -27598,7 +27620,7 @@
         </is>
       </c>
       <c r="G100" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H100" s="34" t="inlineStr">
         <is>
@@ -27606,7 +27628,7 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>25.478201</v>
+        <v>24.878539</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="58">
@@ -27630,7 +27652,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>60586</v>
+        <v>61546</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -27638,7 +27660,7 @@
         </is>
       </c>
       <c r="G101" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H101" s="34" t="inlineStr">
         <is>
@@ -27646,7 +27668,7 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>62522.52055</v>
+        <v>61204.489244</v>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="58">
@@ -27670,7 +27692,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>15.88</v>
+        <v>16.13</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -27678,7 +27700,7 @@
         </is>
       </c>
       <c r="G102" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H102" s="34" t="inlineStr">
         <is>
@@ -27686,7 +27708,7 @@
         </is>
       </c>
       <c r="I102" t="n">
-        <v>16.642819</v>
+        <v>15.995141</v>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="58">
@@ -27784,7 +27806,7 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
-        <v>0.006181</v>
+        <v>0.006497</v>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
@@ -27792,7 +27814,7 @@
         </is>
       </c>
       <c r="G105" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H105" s="34" t="inlineStr">
         <is>
@@ -27800,7 +27822,7 @@
         </is>
       </c>
       <c r="I105" t="n">
-        <v>0.006516</v>
+        <v>0.006297</v>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="58">
@@ -27824,7 +27846,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>61.93</v>
+        <v>63.55</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>
@@ -27832,7 +27854,7 @@
         </is>
       </c>
       <c r="G106" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H106" s="34" t="inlineStr">
         <is>
@@ -27840,7 +27862,7 @@
         </is>
       </c>
       <c r="I106" t="n">
-        <v>66.351797</v>
+        <v>64.340321</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="58">
@@ -27872,7 +27894,7 @@
         </is>
       </c>
       <c r="G107" s="28" t="n">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="H107" s="34" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Weekly dashboard update — 2026-06-07
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-42660" yWindow="-540" windowWidth="32460" windowHeight="17180" tabRatio="500" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Realized" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Realized" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Prices" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Reference" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="AsOfDate">'FX &amp; Assumptions'!$C$5</definedName>
@@ -697,14 +697,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -726,8 +726,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -752,10 +752,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -764,10 +764,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4F81BD"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+              <a:ln w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -777,10 +777,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="C0504D"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -790,10 +790,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="9BBB59"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -803,10 +803,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="8064A2"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -816,10 +816,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4BACC6"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -829,10 +829,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="F79646"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -842,14 +842,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -875,14 +875,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -908,14 +908,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -941,14 +941,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -974,14 +974,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1007,14 +1007,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1038,16 +1038,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1142,16 +1142,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1172,10 +1172,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1187,14 +1187,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1216,8 +1216,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1242,10 +1242,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1254,10 +1254,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4672A8"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1267,10 +1267,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="AB4744"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1280,10 +1280,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="8AA64F"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1293,10 +1293,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="725990"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1306,10 +1306,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4299B0"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1319,10 +1319,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="DC853E"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1332,10 +1332,10 @@
             <idx val="6"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="93A9CE"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1345,10 +1345,10 @@
             <idx val="7"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="D09493"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1358,10 +1358,10 @@
             <idx val="8"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="B8CD97"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1371,14 +1371,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1405,14 +1405,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1439,14 +1439,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1473,14 +1473,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1507,14 +1507,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1541,14 +1541,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1575,14 +1575,14 @@
             <dLbl>
               <idx val="6"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1609,14 +1609,14 @@
             <dLbl>
               <idx val="7"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1643,14 +1643,14 @@
             <dLbl>
               <idx val="8"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1675,16 +1675,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1791,16 +1791,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1821,10 +1821,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1836,14 +1836,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1865,8 +1865,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1893,10 +1893,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1904,16 +1904,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2016,7 +2016,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2025,9 +2025,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2059,7 +2059,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2073,7 +2073,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2082,9 +2082,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2109,16 +2109,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2139,10 +2139,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2154,14 +2154,14 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -2183,8 +2183,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -2200,10 +2200,10 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2211,16 +2211,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2411,7 +2411,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2420,9 +2420,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2454,7 +2454,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2468,7 +2468,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2477,9 +2477,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2504,16 +2504,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2534,10 +2534,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2549,7 +2549,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>1</col>
@@ -2569,9 +2569,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2596,9 +2596,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+          <c:chart r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2623,9 +2623,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+          <c:chart r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2650,9 +2650,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+          <c:chart r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -21690,16 +21690,16 @@
         <v>46180</v>
       </c>
       <c r="C11" s="29" t="n">
-        <v>26487092</v>
+        <v>26506082</v>
       </c>
       <c r="D11" s="29" t="n">
         <v>22666838</v>
       </c>
       <c r="E11" s="29" t="n">
-        <v>3820254</v>
+        <v>3839244</v>
       </c>
       <c r="F11" s="30" t="n">
-        <v>0.1685</v>
+        <v>0.1694</v>
       </c>
       <c r="G11" s="29" t="n">
         <v>19003537</v>
@@ -21708,7 +21708,7 @@
         <v>4980397</v>
       </c>
       <c r="I11" s="29" t="n">
-        <v>1123143</v>
+        <v>1142133</v>
       </c>
       <c r="J11" s="31" t="n">
         <v>32.79</v>
@@ -26972,7 +26972,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>62.1</v>
+        <v>63.42</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -26988,7 +26988,7 @@
         </is>
       </c>
       <c r="I84" t="n">
-        <v>62.187501</v>
+        <v>60.099737</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="58">
@@ -27012,7 +27012,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>580.46</v>
+        <v>592.45</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -27028,7 +27028,7 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>577.779634</v>
+        <v>571.434173</v>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="58">
@@ -27052,7 +27052,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>61546</v>
+        <v>62445</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -27068,7 +27068,7 @@
         </is>
       </c>
       <c r="I86" t="n">
-        <v>61204.489244</v>
+        <v>60288.756387</v>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="58">
@@ -27092,7 +27092,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.006497</v>
+        <v>0.006765</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -27108,7 +27108,7 @@
         </is>
       </c>
       <c r="I87" t="n">
-        <v>0.006297</v>
+        <v>0.006143</v>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="58">
@@ -27132,7 +27132,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.011545</v>
+        <v>0.011458</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -27148,7 +27148,7 @@
         </is>
       </c>
       <c r="I88" t="n">
-        <v>0.011338</v>
+        <v>0.010885</v>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="58">
@@ -27172,7 +27172,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>63.55</v>
+        <v>64.91</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -27188,7 +27188,7 @@
         </is>
       </c>
       <c r="I89" t="n">
-        <v>64.340321</v>
+        <v>61.265895</v>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="58">
@@ -27212,7 +27212,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>1.62</v>
+        <v>1.64</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -27228,7 +27228,7 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>1.604315</v>
+        <v>1.542123</v>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="58">
@@ -27292,7 +27292,7 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
-        <v>0.012717</v>
+        <v>0.012774</v>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
@@ -27308,7 +27308,7 @@
         </is>
       </c>
       <c r="I92" t="n">
-        <v>0.012668</v>
+        <v>0.012245</v>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="58">
@@ -27332,7 +27332,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>2.689173</v>
+        <v>2.71934</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -27348,7 +27348,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>2.638235</v>
+        <v>2.558705</v>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="58">
@@ -27372,7 +27372,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>24.484457</v>
+        <v>24.655555</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -27388,7 +27388,7 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>23.647407</v>
+        <v>22.564475</v>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="58">
@@ -27412,7 +27412,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.115422</v>
+        <v>0.118322</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -27428,7 +27428,7 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>0.115185</v>
+        <v>0.111123</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="58">
@@ -27452,7 +27452,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>19033.2834</v>
+        <v>19426.4355</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -27468,7 +27468,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>18945.394191</v>
+        <v>18737.326544</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="58">
@@ -27492,7 +27492,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2018093.34</v>
+        <v>2047571.55</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -27508,7 +27508,7 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>2006895.202308</v>
+        <v>1976868.321933</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="58">
@@ -27532,7 +27532,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>2.735047</v>
+        <v>2.774067</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -27548,7 +27548,7 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>2.702748</v>
+        <v>2.629434</v>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="58">
@@ -27572,7 +27572,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>52215.1239</v>
+        <v>53531.9703</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -27588,7 +27588,7 @@
         </is>
       </c>
       <c r="I99" t="n">
-        <v>52127.545269</v>
+        <v>50447.209233</v>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="58">
@@ -27612,7 +27612,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>24.556431</v>
+        <v>25.183704</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -27628,7 +27628,7 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>24.878539</v>
+        <v>24.853936</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="58">
@@ -27652,7 +27652,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>61546</v>
+        <v>62445</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -27668,7 +27668,7 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>61204.489244</v>
+        <v>60288.756387</v>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="58">
@@ -27692,7 +27692,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>16.13</v>
+        <v>16.53</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -27708,7 +27708,7 @@
         </is>
       </c>
       <c r="I102" t="n">
-        <v>15.995141</v>
+        <v>15.72606</v>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="58">
@@ -27806,7 +27806,7 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
-        <v>0.006497</v>
+        <v>0.006765</v>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
@@ -27822,7 +27822,7 @@
         </is>
       </c>
       <c r="I105" t="n">
-        <v>0.006297</v>
+        <v>0.006143</v>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="58">
@@ -27846,7 +27846,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>63.55</v>
+        <v>64.91</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>
@@ -27862,7 +27862,7 @@
         </is>
       </c>
       <c r="I106" t="n">
-        <v>64.340321</v>
+        <v>61.265895</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="58">

</xml_diff>

<commit_message>
Weekly dashboard update — 2026-06-08
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -21720,16 +21720,38 @@
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="58">
-      <c r="B12" s="28" t="n"/>
-      <c r="C12" s="29" t="n"/>
-      <c r="D12" s="29" t="n"/>
-      <c r="E12" s="29" t="n"/>
-      <c r="F12" s="30" t="n"/>
-      <c r="G12" s="29" t="n"/>
-      <c r="H12" s="29" t="n"/>
-      <c r="I12" s="29" t="n"/>
-      <c r="J12" s="31" t="n"/>
-      <c r="K12" s="32" t="n"/>
+      <c r="B12" s="28" t="n">
+        <v>46181</v>
+      </c>
+      <c r="C12" s="29" t="n">
+        <v>26602164</v>
+      </c>
+      <c r="D12" s="29" t="n">
+        <v>22670962</v>
+      </c>
+      <c r="E12" s="29" t="n">
+        <v>3931202</v>
+      </c>
+      <c r="F12" s="30" t="n">
+        <v>0.1734</v>
+      </c>
+      <c r="G12" s="29" t="n">
+        <v>19003537</v>
+      </c>
+      <c r="H12" s="29" t="n">
+        <v>5051013</v>
+      </c>
+      <c r="I12" s="29" t="n">
+        <v>1164136</v>
+      </c>
+      <c r="J12" s="31" t="n">
+        <v>32.81</v>
+      </c>
+      <c r="K12" s="32" t="inlineStr">
+        <is>
+          <t>Auto weekly snapshot</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="58">
       <c r="B13" s="28" t="n"/>
@@ -23467,7 +23489,7 @@
         </is>
       </c>
       <c r="C5" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="D5" s="64" t="inlineStr">
         <is>
@@ -23482,11 +23504,11 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>32.79</v>
+        <v>32.81</v>
       </c>
       <c r="D6" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-06-07</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-06-08</t>
         </is>
       </c>
     </row>
@@ -23531,11 +23553,11 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>25.4187</v>
+        <v>25.4825</v>
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-06-07</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-06-08</t>
         </is>
       </c>
     </row>
@@ -25143,7 +25165,7 @@
         </is>
       </c>
       <c r="G38" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H38" s="34" t="inlineStr">
         <is>
@@ -25183,7 +25205,7 @@
         </is>
       </c>
       <c r="G39" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H39" s="34" t="inlineStr">
         <is>
@@ -25223,7 +25245,7 @@
         </is>
       </c>
       <c r="G40" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H40" s="34" t="inlineStr">
         <is>
@@ -25263,7 +25285,7 @@
         </is>
       </c>
       <c r="G41" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H41" s="34" t="inlineStr">
         <is>
@@ -25303,7 +25325,7 @@
         </is>
       </c>
       <c r="G42" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H42" s="34" t="inlineStr">
         <is>
@@ -25335,7 +25357,7 @@
         </is>
       </c>
       <c r="E43" s="33" t="n">
-        <v>5.6</v>
+        <v>5.45</v>
       </c>
       <c r="F43" s="34" t="inlineStr">
         <is>
@@ -25343,7 +25365,7 @@
         </is>
       </c>
       <c r="G43" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H43" s="34" t="inlineStr">
         <is>
@@ -25351,7 +25373,7 @@
         </is>
       </c>
       <c r="I43" t="n">
-        <v>5.6</v>
+        <v>5.45</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="58">
@@ -25375,23 +25397,23 @@
         </is>
       </c>
       <c r="E44" s="33" t="n">
+        <v>170</v>
+      </c>
+      <c r="F44" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G44" s="28" t="n">
+        <v>46181</v>
+      </c>
+      <c r="H44" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
         <v>174.5</v>
-      </c>
-      <c r="F44" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G44" s="28" t="n">
-        <v>46180</v>
-      </c>
-      <c r="H44" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I44" t="n">
-        <v>175.5</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="58">
@@ -25423,7 +25445,7 @@
         </is>
       </c>
       <c r="G45" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H45" s="34" t="inlineStr">
         <is>
@@ -25455,7 +25477,7 @@
         </is>
       </c>
       <c r="E46" s="33" t="n">
-        <v>0.31</v>
+        <v>0.3</v>
       </c>
       <c r="F46" s="34" t="inlineStr">
         <is>
@@ -25463,7 +25485,7 @@
         </is>
       </c>
       <c r="G46" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H46" s="34" t="inlineStr">
         <is>
@@ -25471,7 +25493,7 @@
         </is>
       </c>
       <c r="I46" t="n">
-        <v>0.31</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" s="58">
@@ -25540,7 +25562,7 @@
         </is>
       </c>
       <c r="G48" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H48" s="34" t="inlineStr">
         <is>
@@ -25572,23 +25594,23 @@
         </is>
       </c>
       <c r="E49" s="33" t="n">
+        <v>64.5</v>
+      </c>
+      <c r="F49" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G49" s="28" t="n">
+        <v>46181</v>
+      </c>
+      <c r="H49" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
         <v>67</v>
-      </c>
-      <c r="F49" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G49" s="28" t="n">
-        <v>46180</v>
-      </c>
-      <c r="H49" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I49" t="n">
-        <v>67.25</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="58">
@@ -25612,7 +25634,7 @@
         </is>
       </c>
       <c r="E50" s="33" t="n">
-        <v>9.5</v>
+        <v>9.4</v>
       </c>
       <c r="F50" s="34" t="inlineStr">
         <is>
@@ -25620,7 +25642,7 @@
         </is>
       </c>
       <c r="G50" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H50" s="34" t="inlineStr">
         <is>
@@ -25628,7 +25650,7 @@
         </is>
       </c>
       <c r="I50" t="n">
-        <v>9.6</v>
+        <v>9.4</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="58">
@@ -25652,7 +25674,7 @@
         </is>
       </c>
       <c r="E51" s="33" t="n">
-        <v>15.5</v>
+        <v>15.2</v>
       </c>
       <c r="F51" s="34" t="inlineStr">
         <is>
@@ -25660,7 +25682,7 @@
         </is>
       </c>
       <c r="G51" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H51" s="34" t="inlineStr">
         <is>
@@ -25668,7 +25690,7 @@
         </is>
       </c>
       <c r="I51" t="n">
-        <v>15.3</v>
+        <v>15.2</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" s="58">
@@ -25692,7 +25714,7 @@
         </is>
       </c>
       <c r="E52" s="33" t="n">
-        <v>13.2</v>
+        <v>13.3</v>
       </c>
       <c r="F52" s="34" t="inlineStr">
         <is>
@@ -25700,7 +25722,7 @@
         </is>
       </c>
       <c r="G52" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H52" s="34" t="inlineStr">
         <is>
@@ -25708,7 +25730,7 @@
         </is>
       </c>
       <c r="I52" t="n">
-        <v>13.2</v>
+        <v>13.3</v>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1" s="58">
@@ -25732,7 +25754,7 @@
         </is>
       </c>
       <c r="E53" s="33" t="n">
-        <v>6.05</v>
+        <v>5.7</v>
       </c>
       <c r="F53" s="34" t="inlineStr">
         <is>
@@ -25740,7 +25762,7 @@
         </is>
       </c>
       <c r="G53" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H53" s="34" t="inlineStr">
         <is>
@@ -25748,7 +25770,7 @@
         </is>
       </c>
       <c r="I53" t="n">
-        <v>6.05</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="58">
@@ -25772,7 +25794,7 @@
         </is>
       </c>
       <c r="E54" s="33" t="n">
-        <v>21.5</v>
+        <v>21.2</v>
       </c>
       <c r="F54" s="34" t="inlineStr">
         <is>
@@ -25780,7 +25802,7 @@
         </is>
       </c>
       <c r="G54" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H54" s="34" t="inlineStr">
         <is>
@@ -25788,7 +25810,7 @@
         </is>
       </c>
       <c r="I54" t="n">
-        <v>21.299999</v>
+        <v>21.200001</v>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="58">
@@ -25812,7 +25834,7 @@
         </is>
       </c>
       <c r="E55" s="33" t="n">
-        <v>3.54</v>
+        <v>3.52</v>
       </c>
       <c r="F55" s="34" t="inlineStr">
         <is>
@@ -25820,7 +25842,7 @@
         </is>
       </c>
       <c r="G55" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H55" s="34" t="inlineStr">
         <is>
@@ -25828,7 +25850,7 @@
         </is>
       </c>
       <c r="I55" t="n">
-        <v>3.54</v>
+        <v>3.52</v>
       </c>
     </row>
     <row r="56" ht="15" customHeight="1" s="58">
@@ -25852,7 +25874,7 @@
         </is>
       </c>
       <c r="E56" s="33" t="n">
-        <v>4.94</v>
+        <v>4.82</v>
       </c>
       <c r="F56" s="34" t="inlineStr">
         <is>
@@ -25860,7 +25882,7 @@
         </is>
       </c>
       <c r="G56" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H56" s="34" t="inlineStr">
         <is>
@@ -25868,7 +25890,7 @@
         </is>
       </c>
       <c r="I56" t="n">
-        <v>4.94</v>
+        <v>4.82</v>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1" s="58">
@@ -25892,7 +25914,7 @@
         </is>
       </c>
       <c r="E57" s="33" t="n">
-        <v>2.78</v>
+        <v>2.64</v>
       </c>
       <c r="F57" s="34" t="inlineStr">
         <is>
@@ -25900,7 +25922,7 @@
         </is>
       </c>
       <c r="G57" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H57" s="34" t="inlineStr">
         <is>
@@ -25908,7 +25930,7 @@
         </is>
       </c>
       <c r="I57" t="n">
-        <v>2.78</v>
+        <v>2.64</v>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="58">
@@ -25932,7 +25954,7 @@
         </is>
       </c>
       <c r="E58" s="33" t="n">
-        <v>12.5</v>
+        <v>12.3</v>
       </c>
       <c r="F58" s="34" t="inlineStr">
         <is>
@@ -25940,7 +25962,7 @@
         </is>
       </c>
       <c r="G58" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H58" s="34" t="inlineStr">
         <is>
@@ -25948,7 +25970,7 @@
         </is>
       </c>
       <c r="I58" t="n">
-        <v>12.4</v>
+        <v>12.3</v>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="58">
@@ -25972,7 +25994,7 @@
         </is>
       </c>
       <c r="E59" s="33" t="n">
-        <v>17.9</v>
+        <v>17.4</v>
       </c>
       <c r="F59" s="34" t="inlineStr">
         <is>
@@ -25980,7 +26002,7 @@
         </is>
       </c>
       <c r="G59" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H59" s="34" t="inlineStr">
         <is>
@@ -25988,7 +26010,7 @@
         </is>
       </c>
       <c r="I59" t="n">
-        <v>17.9</v>
+        <v>17.4</v>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1" s="58">
@@ -26012,7 +26034,7 @@
         </is>
       </c>
       <c r="E60" s="33" t="n">
-        <v>147.16</v>
+        <v>158.46</v>
       </c>
       <c r="F60" s="34" t="inlineStr">
         <is>
@@ -26020,7 +26042,7 @@
         </is>
       </c>
       <c r="G60" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H60" s="34" t="inlineStr">
         <is>
@@ -26028,7 +26050,7 @@
         </is>
       </c>
       <c r="I60" t="n">
-        <v>147.160004</v>
+        <v>158.460007</v>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="58">
@@ -26052,7 +26074,7 @@
         </is>
       </c>
       <c r="E61" s="33" t="n">
-        <v>251.44</v>
+        <v>247.66</v>
       </c>
       <c r="F61" s="34" t="inlineStr">
         <is>
@@ -26060,7 +26082,7 @@
         </is>
       </c>
       <c r="G61" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H61" s="34" t="inlineStr">
         <is>
@@ -26068,7 +26090,7 @@
         </is>
       </c>
       <c r="I61" t="n">
-        <v>251.440002</v>
+        <v>247.660004</v>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="58">
@@ -26092,7 +26114,7 @@
         </is>
       </c>
       <c r="E62" s="33" t="n">
-        <v>453.01</v>
+        <v>490.62</v>
       </c>
       <c r="F62" s="34" t="inlineStr">
         <is>
@@ -26100,7 +26122,7 @@
         </is>
       </c>
       <c r="G62" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H62" s="34" t="inlineStr">
         <is>
@@ -26108,7 +26130,7 @@
         </is>
       </c>
       <c r="I62" t="n">
-        <v>453.01001</v>
+        <v>490.619995</v>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1" s="58">
@@ -26132,7 +26154,7 @@
         </is>
       </c>
       <c r="E63" s="33" t="n">
-        <v>164.4</v>
+        <v>168.04</v>
       </c>
       <c r="F63" s="34" t="inlineStr">
         <is>
@@ -26140,7 +26162,7 @@
         </is>
       </c>
       <c r="G63" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H63" s="34" t="inlineStr">
         <is>
@@ -26148,7 +26170,7 @@
         </is>
       </c>
       <c r="I63" t="n">
-        <v>164.399994</v>
+        <v>168.039993</v>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="58">
@@ -26172,7 +26194,7 @@
         </is>
       </c>
       <c r="E64" s="33" t="n">
-        <v>56.07</v>
+        <v>58.08</v>
       </c>
       <c r="F64" s="34" t="inlineStr">
         <is>
@@ -26180,7 +26202,7 @@
         </is>
       </c>
       <c r="G64" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H64" s="34" t="inlineStr">
         <is>
@@ -26188,7 +26210,7 @@
         </is>
       </c>
       <c r="I64" t="n">
-        <v>56.07</v>
+        <v>58.080002</v>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1" s="58">
@@ -26212,7 +26234,7 @@
         </is>
       </c>
       <c r="E65" s="33" t="n">
-        <v>175.19</v>
+        <v>186.23</v>
       </c>
       <c r="F65" s="34" t="inlineStr">
         <is>
@@ -26220,7 +26242,7 @@
         </is>
       </c>
       <c r="G65" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H65" s="34" t="inlineStr">
         <is>
@@ -26228,7 +26250,7 @@
         </is>
       </c>
       <c r="I65" t="n">
-        <v>175.190002</v>
+        <v>186.229996</v>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1" s="58">
@@ -26252,7 +26274,7 @@
         </is>
       </c>
       <c r="E66" s="33" t="n">
-        <v>144.68</v>
+        <v>145.745</v>
       </c>
       <c r="F66" s="34" t="inlineStr">
         <is>
@@ -26260,7 +26282,7 @@
         </is>
       </c>
       <c r="G66" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H66" s="34" t="inlineStr">
         <is>
@@ -26268,7 +26290,7 @@
         </is>
       </c>
       <c r="I66" t="n">
-        <v>144.679993</v>
+        <v>145.744995</v>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1" s="58">
@@ -26292,7 +26314,7 @@
         </is>
       </c>
       <c r="E67" s="33" t="n">
-        <v>164.02</v>
+        <v>163.5</v>
       </c>
       <c r="F67" s="34" t="inlineStr">
         <is>
@@ -26300,7 +26322,7 @@
         </is>
       </c>
       <c r="G67" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H67" s="34" t="inlineStr">
         <is>
@@ -26332,7 +26354,7 @@
         </is>
       </c>
       <c r="E68" s="33" t="n">
-        <v>1929.2</v>
+        <v>2093.425</v>
       </c>
       <c r="F68" s="34" t="inlineStr">
         <is>
@@ -26340,7 +26362,7 @@
         </is>
       </c>
       <c r="G68" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H68" s="34" t="inlineStr">
         <is>
@@ -26348,7 +26370,7 @@
         </is>
       </c>
       <c r="I68" t="n">
-        <v>1929.199951</v>
+        <v>2093.425049</v>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="58">
@@ -26372,7 +26394,7 @@
         </is>
       </c>
       <c r="E69" s="33" t="n">
-        <v>1131.42</v>
+        <v>1169.225</v>
       </c>
       <c r="F69" s="34" t="inlineStr">
         <is>
@@ -26380,7 +26402,7 @@
         </is>
       </c>
       <c r="G69" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H69" s="34" t="inlineStr">
         <is>
@@ -26388,7 +26410,7 @@
         </is>
       </c>
       <c r="I69" t="n">
-        <v>1131.420044</v>
+        <v>1169.224976</v>
       </c>
     </row>
     <row r="70" ht="15" customHeight="1" s="58">
@@ -26412,7 +26434,7 @@
         </is>
       </c>
       <c r="E70" s="33" t="n">
-        <v>88.34</v>
+        <v>92.18600000000001</v>
       </c>
       <c r="F70" s="34" t="inlineStr">
         <is>
@@ -26420,7 +26442,7 @@
         </is>
       </c>
       <c r="G70" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H70" s="34" t="inlineStr">
         <is>
@@ -26428,7 +26450,7 @@
         </is>
       </c>
       <c r="I70" t="n">
-        <v>88.339996</v>
+        <v>92.18609600000001</v>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1" s="58">
@@ -26452,7 +26474,7 @@
         </is>
       </c>
       <c r="E71" s="33" t="n">
-        <v>1481.05</v>
+        <v>1559.67</v>
       </c>
       <c r="F71" s="34" t="inlineStr">
         <is>
@@ -26460,7 +26482,7 @@
         </is>
       </c>
       <c r="G71" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H71" s="34" t="inlineStr">
         <is>
@@ -26468,7 +26490,7 @@
         </is>
       </c>
       <c r="I71" t="n">
-        <v>1481.050049</v>
+        <v>1559.670044</v>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1" s="58">
@@ -26492,7 +26514,7 @@
         </is>
       </c>
       <c r="E72" s="33" t="n">
-        <v>111.07</v>
+        <v>112.23</v>
       </c>
       <c r="F72" s="34" t="inlineStr">
         <is>
@@ -26500,7 +26522,7 @@
         </is>
       </c>
       <c r="G72" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H72" s="34" t="inlineStr">
         <is>
@@ -26508,7 +26530,7 @@
         </is>
       </c>
       <c r="I72" t="n">
-        <v>111.07</v>
+        <v>112.230003</v>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1" s="58">
@@ -26532,7 +26554,7 @@
         </is>
       </c>
       <c r="E73" s="33" t="n">
-        <v>205.1</v>
+        <v>208.147</v>
       </c>
       <c r="F73" s="34" t="inlineStr">
         <is>
@@ -26540,7 +26562,7 @@
         </is>
       </c>
       <c r="G73" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H73" s="34" t="inlineStr">
         <is>
@@ -26548,7 +26570,7 @@
         </is>
       </c>
       <c r="I73" t="n">
-        <v>205.100006</v>
+        <v>208.147003</v>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1" s="58">
@@ -26572,7 +26594,7 @@
         </is>
       </c>
       <c r="E74" s="33" t="n">
-        <v>86.11</v>
+        <v>88.81999999999999</v>
       </c>
       <c r="F74" s="34" t="inlineStr">
         <is>
@@ -26580,7 +26602,7 @@
         </is>
       </c>
       <c r="G74" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H74" s="34" t="inlineStr">
         <is>
@@ -26588,7 +26610,7 @@
         </is>
       </c>
       <c r="I74" t="n">
-        <v>86.110001</v>
+        <v>88.81999999999999</v>
       </c>
     </row>
     <row r="75" ht="15" customHeight="1" s="58">
@@ -26612,7 +26634,7 @@
         </is>
       </c>
       <c r="E75" s="33" t="n">
-        <v>98.28</v>
+        <v>103.07</v>
       </c>
       <c r="F75" s="34" t="inlineStr">
         <is>
@@ -26620,7 +26642,7 @@
         </is>
       </c>
       <c r="G75" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H75" s="34" t="inlineStr">
         <is>
@@ -26628,7 +26650,7 @@
         </is>
       </c>
       <c r="I75" t="n">
-        <v>98.279999</v>
+        <v>103.07</v>
       </c>
     </row>
     <row r="76" ht="15" customHeight="1" s="58">
@@ -26652,7 +26674,7 @@
         </is>
       </c>
       <c r="E76" s="33" t="n">
-        <v>357.93</v>
+        <v>377.255</v>
       </c>
       <c r="F76" s="34" t="inlineStr">
         <is>
@@ -26660,7 +26682,7 @@
         </is>
       </c>
       <c r="G76" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H76" s="34" t="inlineStr">
         <is>
@@ -26668,7 +26690,7 @@
         </is>
       </c>
       <c r="I76" t="n">
-        <v>357.929993</v>
+        <v>377.255005</v>
       </c>
     </row>
     <row r="77" ht="15" customHeight="1" s="58">
@@ -26692,7 +26714,7 @@
         </is>
       </c>
       <c r="E77" s="33" t="n">
-        <v>391</v>
+        <v>403.87</v>
       </c>
       <c r="F77" s="34" t="inlineStr">
         <is>
@@ -26700,7 +26722,7 @@
         </is>
       </c>
       <c r="G77" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H77" s="34" t="inlineStr">
         <is>
@@ -26708,7 +26730,7 @@
         </is>
       </c>
       <c r="I77" t="n">
-        <v>418.450012</v>
+        <v>403.869995</v>
       </c>
     </row>
     <row r="78" ht="15" customHeight="1" s="58">
@@ -26732,7 +26754,7 @@
         </is>
       </c>
       <c r="E78" s="33" t="n">
-        <v>54.52</v>
+        <v>54.73</v>
       </c>
       <c r="F78" s="34" t="inlineStr">
         <is>
@@ -26740,7 +26762,7 @@
         </is>
       </c>
       <c r="G78" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H78" s="34" t="inlineStr">
         <is>
@@ -26748,7 +26770,7 @@
         </is>
       </c>
       <c r="I78" t="n">
-        <v>54.52</v>
+        <v>54.73</v>
       </c>
     </row>
     <row r="79" ht="15" customHeight="1" s="58">
@@ -26772,7 +26794,7 @@
         </is>
       </c>
       <c r="E79" s="33" t="n">
-        <v>88.59</v>
+        <v>88.06</v>
       </c>
       <c r="F79" s="34" t="inlineStr">
         <is>
@@ -26780,7 +26802,7 @@
         </is>
       </c>
       <c r="G79" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H79" s="34" t="inlineStr">
         <is>
@@ -26788,7 +26810,7 @@
         </is>
       </c>
       <c r="I79" t="n">
-        <v>88.589996</v>
+        <v>88.05999799999999</v>
       </c>
     </row>
     <row r="80" ht="15" customHeight="1" s="58">
@@ -26812,7 +26834,7 @@
         </is>
       </c>
       <c r="E80" s="33" t="n">
-        <v>307.34</v>
+        <v>314.52</v>
       </c>
       <c r="F80" s="34" t="inlineStr">
         <is>
@@ -26820,7 +26842,7 @@
         </is>
       </c>
       <c r="G80" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H80" s="34" t="inlineStr">
         <is>
@@ -26828,7 +26850,7 @@
         </is>
       </c>
       <c r="I80" t="n">
-        <v>307.339996</v>
+        <v>314.519989</v>
       </c>
     </row>
     <row r="81" ht="15" customHeight="1" s="58">
@@ -26852,7 +26874,7 @@
         </is>
       </c>
       <c r="E81" s="33" t="n">
-        <v>152.4</v>
+        <v>160.07</v>
       </c>
       <c r="F81" s="34" t="inlineStr">
         <is>
@@ -26860,7 +26882,7 @@
         </is>
       </c>
       <c r="G81" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H81" s="34" t="inlineStr">
         <is>
@@ -26868,7 +26890,7 @@
         </is>
       </c>
       <c r="I81" t="n">
-        <v>152.399994</v>
+        <v>160.070007</v>
       </c>
     </row>
     <row r="82" ht="15" customHeight="1" s="58">
@@ -26892,7 +26914,7 @@
         </is>
       </c>
       <c r="E82" s="33" t="n">
-        <v>593</v>
+        <v>589.24</v>
       </c>
       <c r="F82" s="34" t="inlineStr">
         <is>
@@ -26900,7 +26922,7 @@
         </is>
       </c>
       <c r="G82" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H82" s="34" t="inlineStr">
         <is>
@@ -26908,7 +26930,7 @@
         </is>
       </c>
       <c r="I82" t="n">
-        <v>627.570007</v>
+        <v>589.23999</v>
       </c>
     </row>
     <row r="83" ht="15" customHeight="1" s="58">
@@ -26932,7 +26954,7 @@
         </is>
       </c>
       <c r="E83" s="33" t="n">
-        <v>136.99</v>
+        <v>147.43</v>
       </c>
       <c r="F83" s="34" t="inlineStr">
         <is>
@@ -26940,7 +26962,7 @@
         </is>
       </c>
       <c r="G83" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H83" s="34" t="inlineStr">
         <is>
@@ -26948,7 +26970,7 @@
         </is>
       </c>
       <c r="I83" t="n">
-        <v>136.990005</v>
+        <v>147.429901</v>
       </c>
     </row>
     <row r="84" ht="15" customHeight="1" s="58">
@@ -26972,7 +26994,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>63.01</v>
+        <v>64.39</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -26980,7 +27002,7 @@
         </is>
       </c>
       <c r="G84" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H84" s="34" t="inlineStr">
         <is>
@@ -26988,7 +27010,7 @@
         </is>
       </c>
       <c r="I84" t="n">
-        <v>60.266085</v>
+        <v>63.074081</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="58">
@@ -27012,7 +27034,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>592.08</v>
+        <v>601.22</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -27020,7 +27042,7 @@
         </is>
       </c>
       <c r="G85" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H85" s="34" t="inlineStr">
         <is>
@@ -27028,7 +27050,7 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>573.320034</v>
+        <v>591.0371280000001</v>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="58">
@@ -27052,7 +27074,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>62361</v>
+        <v>63860</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -27060,7 +27082,7 @@
         </is>
       </c>
       <c r="G86" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H86" s="34" t="inlineStr">
         <is>
@@ -27068,7 +27090,7 @@
         </is>
       </c>
       <c r="I86" t="n">
-        <v>60522.300435</v>
+        <v>61869.562208</v>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="58">
@@ -27092,7 +27114,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.006727</v>
+        <v>0.006908</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -27100,7 +27122,7 @@
         </is>
       </c>
       <c r="G87" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H87" s="34" t="inlineStr">
         <is>
@@ -27108,7 +27130,7 @@
         </is>
       </c>
       <c r="I87" t="n">
-        <v>0.006162</v>
+        <v>0.006714</v>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="58">
@@ -27132,7 +27154,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.01135</v>
+        <v>0.011289</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -27140,7 +27162,7 @@
         </is>
       </c>
       <c r="G88" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H88" s="34" t="inlineStr">
         <is>
@@ -27148,7 +27170,7 @@
         </is>
       </c>
       <c r="I88" t="n">
-        <v>0.011007</v>
+        <v>0.011506</v>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="58">
@@ -27172,7 +27194,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>64.58</v>
+        <v>66.98</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -27180,7 +27202,7 @@
         </is>
       </c>
       <c r="G89" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H89" s="34" t="inlineStr">
         <is>
@@ -27188,7 +27210,7 @@
         </is>
       </c>
       <c r="I89" t="n">
-        <v>61.531163</v>
+        <v>64.794264</v>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="58">
@@ -27212,7 +27234,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>1.63</v>
+        <v>1.69</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -27220,7 +27242,7 @@
         </is>
       </c>
       <c r="G90" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H90" s="34" t="inlineStr">
         <is>
@@ -27228,7 +27250,7 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>1.552544</v>
+        <v>1.628887</v>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="58">
@@ -27260,7 +27282,7 @@
         </is>
       </c>
       <c r="G91" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H91" s="34" t="inlineStr">
         <is>
@@ -27292,7 +27314,7 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
-        <v>0.012727</v>
+        <v>0.013708</v>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
@@ -27300,7 +27322,7 @@
         </is>
       </c>
       <c r="G92" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H92" s="34" t="inlineStr">
         <is>
@@ -27308,7 +27330,7 @@
         </is>
       </c>
       <c r="I92" t="n">
-        <v>0.012326</v>
+        <v>0.012768</v>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="58">
@@ -27332,7 +27354,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>2.697404</v>
+        <v>2.747969</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -27340,7 +27362,7 @@
         </is>
       </c>
       <c r="G93" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H93" s="34" t="inlineStr">
         <is>
@@ -27348,7 +27370,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>2.580494</v>
+        <v>2.690321</v>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="58">
@@ -27372,7 +27394,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>24.517411</v>
+        <v>25.026779</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -27380,7 +27402,7 @@
         </is>
       </c>
       <c r="G94" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H94" s="34" t="inlineStr">
         <is>
@@ -27388,7 +27410,7 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>22.742071</v>
+        <v>24.442355</v>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="58">
@@ -27412,7 +27434,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.118268</v>
+        <v>0.112902</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -27420,7 +27442,7 @@
         </is>
       </c>
       <c r="G95" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H95" s="34" t="inlineStr">
         <is>
@@ -27428,7 +27450,7 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>0.111975</v>
+        <v>0.115773</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="58">
@@ -27452,7 +27474,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>19414.3032</v>
+        <v>19726.0282</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -27460,7 +27482,7 @@
         </is>
       </c>
       <c r="G96" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H96" s="34" t="inlineStr">
         <is>
@@ -27468,7 +27490,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>18799.163904</v>
+        <v>19391.928154</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="58">
@@ -27492,7 +27514,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2044817.19</v>
+        <v>2095246.6</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -27500,7 +27522,7 @@
         </is>
       </c>
       <c r="G97" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H97" s="34" t="inlineStr">
         <is>
@@ -27508,7 +27530,7 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>1984526.231277</v>
+        <v>2029940.336052</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="58">
@@ -27532,7 +27554,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>2.76341</v>
+        <v>2.839115</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -27540,7 +27562,7 @@
         </is>
       </c>
       <c r="G98" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H98" s="34" t="inlineStr">
         <is>
@@ -27548,7 +27570,7 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>2.63744</v>
+        <v>2.767534</v>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="58">
@@ -27572,7 +27594,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>53312.2773</v>
+        <v>55335.3774</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -27580,7 +27602,7 @@
         </is>
       </c>
       <c r="G99" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H99" s="34" t="inlineStr">
         <is>
@@ -27588,7 +27610,7 @@
         </is>
       </c>
       <c r="I99" t="n">
-        <v>50692.83404</v>
+        <v>53381.490685</v>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="58">
@@ -27612,7 +27634,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>25.17062</v>
+        <v>25.374106</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -27620,7 +27642,7 @@
         </is>
       </c>
       <c r="G100" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H100" s="34" t="inlineStr">
         <is>
@@ -27628,7 +27650,7 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>24.630758</v>
+        <v>25.182746</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="58">
@@ -27652,7 +27674,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>62361</v>
+        <v>63860</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -27660,7 +27682,7 @@
         </is>
       </c>
       <c r="G101" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H101" s="34" t="inlineStr">
         <is>
@@ -27668,7 +27690,7 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>60522.300435</v>
+        <v>61869.562208</v>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="58">
@@ -27692,7 +27714,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>16.43</v>
+        <v>17.04</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -27700,7 +27722,7 @@
         </is>
       </c>
       <c r="G102" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H102" s="34" t="inlineStr">
         <is>
@@ -27708,7 +27730,7 @@
         </is>
       </c>
       <c r="I102" t="n">
-        <v>15.739962</v>
+        <v>16.36308</v>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="58">
@@ -27806,7 +27828,7 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
-        <v>0.006727</v>
+        <v>0.006908</v>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
@@ -27814,7 +27836,7 @@
         </is>
       </c>
       <c r="G105" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H105" s="34" t="inlineStr">
         <is>
@@ -27822,7 +27844,7 @@
         </is>
       </c>
       <c r="I105" t="n">
-        <v>0.006162</v>
+        <v>0.006714</v>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="58">
@@ -27846,7 +27868,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>64.58</v>
+        <v>66.98</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>
@@ -27854,7 +27876,7 @@
         </is>
       </c>
       <c r="G106" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H106" s="34" t="inlineStr">
         <is>
@@ -27862,7 +27884,7 @@
         </is>
       </c>
       <c r="I106" t="n">
-        <v>61.531163</v>
+        <v>64.794264</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="58">
@@ -27894,7 +27916,7 @@
         </is>
       </c>
       <c r="G107" s="28" t="n">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="H107" s="34" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Daily dashboard update — 2026-06-09
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-42660" yWindow="-540" windowWidth="32460" windowHeight="17180" tabRatio="500" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Realized" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Prices" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Reference" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Realized" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="AsOfDate">'FX &amp; Assumptions'!$C$5</definedName>
@@ -697,14 +697,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -726,8 +726,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -752,10 +752,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -764,10 +764,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4F81BD"/>
               </a:solidFill>
-              <a:ln w="0">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -777,10 +777,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="C0504D"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -790,10 +790,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="9BBB59"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -803,10 +803,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="8064A2"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -816,10 +816,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4BACC6"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -829,10 +829,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="F79646"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -842,14 +842,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -875,14 +875,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -908,14 +908,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -941,14 +941,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -974,14 +974,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1007,14 +1007,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1038,16 +1038,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1142,16 +1142,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1172,10 +1172,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1187,14 +1187,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1216,8 +1216,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1242,10 +1242,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1254,10 +1254,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4672A8"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1267,10 +1267,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="AB4744"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1280,10 +1280,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="8AA64F"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1293,10 +1293,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="725990"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1306,10 +1306,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4299B0"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1319,10 +1319,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="DC853E"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1332,10 +1332,10 @@
             <idx val="6"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="93A9CE"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1345,10 +1345,10 @@
             <idx val="7"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="D09493"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1358,10 +1358,10 @@
             <idx val="8"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="B8CD97"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1371,14 +1371,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1405,14 +1405,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1439,14 +1439,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1473,14 +1473,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1507,14 +1507,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1541,14 +1541,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1575,14 +1575,14 @@
             <dLbl>
               <idx val="6"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1609,14 +1609,14 @@
             <dLbl>
               <idx val="7"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1643,14 +1643,14 @@
             <dLbl>
               <idx val="8"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1675,16 +1675,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1791,16 +1791,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1821,10 +1821,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1836,14 +1836,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1865,8 +1865,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1893,10 +1893,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1904,16 +1904,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2016,7 +2016,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2025,9 +2025,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2059,7 +2059,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="9360">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2073,7 +2073,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2082,9 +2082,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2109,16 +2109,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2139,10 +2139,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2154,14 +2154,14 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -2183,8 +2183,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -2200,10 +2200,10 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2211,16 +2211,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2411,7 +2411,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2420,9 +2420,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2454,7 +2454,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="9360">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2468,7 +2468,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2477,9 +2477,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2504,16 +2504,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2534,10 +2534,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2549,7 +2549,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>1</col>
@@ -2569,9 +2569,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2596,9 +2596,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2623,9 +2623,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId3"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2650,9 +2650,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId4"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -21754,16 +21754,38 @@
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="58">
-      <c r="B13" s="28" t="n"/>
-      <c r="C13" s="29" t="n"/>
-      <c r="D13" s="29" t="n"/>
-      <c r="E13" s="29" t="n"/>
-      <c r="F13" s="30" t="n"/>
-      <c r="G13" s="29" t="n"/>
-      <c r="H13" s="29" t="n"/>
-      <c r="I13" s="29" t="n"/>
-      <c r="J13" s="31" t="n"/>
-      <c r="K13" s="32" t="n"/>
+      <c r="B13" s="28" t="n">
+        <v>46182</v>
+      </c>
+      <c r="C13" s="29" t="n">
+        <v>26546838</v>
+      </c>
+      <c r="D13" s="29" t="n">
+        <v>22668073</v>
+      </c>
+      <c r="E13" s="29" t="n">
+        <v>3878765</v>
+      </c>
+      <c r="F13" s="30" t="n">
+        <v>0.1711</v>
+      </c>
+      <c r="G13" s="29" t="n">
+        <v>19003537</v>
+      </c>
+      <c r="H13" s="29" t="n">
+        <v>5010088</v>
+      </c>
+      <c r="I13" s="29" t="n">
+        <v>1148042</v>
+      </c>
+      <c r="J13" s="31" t="n">
+        <v>32.78</v>
+      </c>
+      <c r="K13" s="32" t="inlineStr">
+        <is>
+          <t>Auto weekly snapshot</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="58">
       <c r="B14" s="28" t="n"/>
@@ -23489,7 +23511,7 @@
         </is>
       </c>
       <c r="C5" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="D5" s="64" t="inlineStr">
         <is>
@@ -23508,7 +23530,7 @@
       </c>
       <c r="D6" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-06-08</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-06-09</t>
         </is>
       </c>
     </row>
@@ -23553,11 +23575,11 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>25.4743</v>
+        <v>25.4864</v>
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-06-08</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-06-09</t>
         </is>
       </c>
     </row>
@@ -25165,7 +25187,7 @@
         </is>
       </c>
       <c r="G38" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H38" s="34" t="inlineStr">
         <is>
@@ -25173,7 +25195,7 @@
         </is>
       </c>
       <c r="I38" t="n">
-        <v>22.83</v>
+        <v>22.799999</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="58">
@@ -25197,7 +25219,7 @@
         </is>
       </c>
       <c r="E39" s="33" t="n">
-        <v>1.1</v>
+        <v>1.106</v>
       </c>
       <c r="F39" s="34" t="inlineStr">
         <is>
@@ -25205,7 +25227,7 @@
         </is>
       </c>
       <c r="G39" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H39" s="34" t="inlineStr">
         <is>
@@ -25245,7 +25267,7 @@
         </is>
       </c>
       <c r="G40" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H40" s="34" t="inlineStr">
         <is>
@@ -25253,7 +25275,7 @@
         </is>
       </c>
       <c r="I40" t="n">
-        <v>770.090027</v>
+        <v>757.73999</v>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="58">
@@ -25285,7 +25307,7 @@
         </is>
       </c>
       <c r="G41" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H41" s="34" t="inlineStr">
         <is>
@@ -25293,7 +25315,7 @@
         </is>
       </c>
       <c r="I41" t="n">
-        <v>20.84</v>
+        <v>20.200001</v>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="58">
@@ -25325,7 +25347,7 @@
         </is>
       </c>
       <c r="G42" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H42" s="34" t="inlineStr">
         <is>
@@ -25333,7 +25355,7 @@
         </is>
       </c>
       <c r="I42" t="n">
-        <v>221.789993</v>
+        <v>218.070007</v>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="58">
@@ -25365,7 +25387,7 @@
         </is>
       </c>
       <c r="G43" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H43" s="34" t="inlineStr">
         <is>
@@ -25405,7 +25427,7 @@
         </is>
       </c>
       <c r="G44" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H44" s="34" t="inlineStr">
         <is>
@@ -25445,7 +25467,7 @@
         </is>
       </c>
       <c r="G45" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H45" s="34" t="inlineStr">
         <is>
@@ -25485,7 +25507,7 @@
         </is>
       </c>
       <c r="G46" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H46" s="34" t="inlineStr">
         <is>
@@ -25562,7 +25584,7 @@
         </is>
       </c>
       <c r="G48" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H48" s="34" t="inlineStr">
         <is>
@@ -25602,7 +25624,7 @@
         </is>
       </c>
       <c r="G49" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H49" s="34" t="inlineStr">
         <is>
@@ -25642,7 +25664,7 @@
         </is>
       </c>
       <c r="G50" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H50" s="34" t="inlineStr">
         <is>
@@ -25682,7 +25704,7 @@
         </is>
       </c>
       <c r="G51" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H51" s="34" t="inlineStr">
         <is>
@@ -25722,7 +25744,7 @@
         </is>
       </c>
       <c r="G52" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H52" s="34" t="inlineStr">
         <is>
@@ -25762,7 +25784,7 @@
         </is>
       </c>
       <c r="G53" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H53" s="34" t="inlineStr">
         <is>
@@ -25802,7 +25824,7 @@
         </is>
       </c>
       <c r="G54" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H54" s="34" t="inlineStr">
         <is>
@@ -25842,7 +25864,7 @@
         </is>
       </c>
       <c r="G55" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H55" s="34" t="inlineStr">
         <is>
@@ -25882,7 +25904,7 @@
         </is>
       </c>
       <c r="G56" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H56" s="34" t="inlineStr">
         <is>
@@ -25922,7 +25944,7 @@
         </is>
       </c>
       <c r="G57" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H57" s="34" t="inlineStr">
         <is>
@@ -25962,7 +25984,7 @@
         </is>
       </c>
       <c r="G58" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H58" s="34" t="inlineStr">
         <is>
@@ -26002,7 +26024,7 @@
         </is>
       </c>
       <c r="G59" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H59" s="34" t="inlineStr">
         <is>
@@ -26034,7 +26056,7 @@
         </is>
       </c>
       <c r="E60" s="33" t="n">
-        <v>159.29</v>
+        <v>154.76</v>
       </c>
       <c r="F60" s="34" t="inlineStr">
         <is>
@@ -26042,7 +26064,7 @@
         </is>
       </c>
       <c r="G60" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H60" s="34" t="inlineStr">
         <is>
@@ -26050,7 +26072,7 @@
         </is>
       </c>
       <c r="I60" t="n">
-        <v>159.289993</v>
+        <v>154.759995</v>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="58">
@@ -26074,7 +26096,7 @@
         </is>
       </c>
       <c r="E61" s="33" t="n">
-        <v>248.05</v>
+        <v>244.99</v>
       </c>
       <c r="F61" s="34" t="inlineStr">
         <is>
@@ -26082,7 +26104,7 @@
         </is>
       </c>
       <c r="G61" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H61" s="34" t="inlineStr">
         <is>
@@ -26090,7 +26112,7 @@
         </is>
       </c>
       <c r="I61" t="n">
-        <v>248.050003</v>
+        <v>244.990005</v>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="58">
@@ -26114,7 +26136,7 @@
         </is>
       </c>
       <c r="E62" s="33" t="n">
-        <v>492.97</v>
+        <v>492.17</v>
       </c>
       <c r="F62" s="34" t="inlineStr">
         <is>
@@ -26122,7 +26144,7 @@
         </is>
       </c>
       <c r="G62" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H62" s="34" t="inlineStr">
         <is>
@@ -26130,7 +26152,7 @@
         </is>
       </c>
       <c r="I62" t="n">
-        <v>492.970001</v>
+        <v>492.170013</v>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1" s="58">
@@ -26154,7 +26176,7 @@
         </is>
       </c>
       <c r="E63" s="33" t="n">
-        <v>168.555</v>
+        <v>165.66</v>
       </c>
       <c r="F63" s="34" t="inlineStr">
         <is>
@@ -26162,7 +26184,7 @@
         </is>
       </c>
       <c r="G63" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H63" s="34" t="inlineStr">
         <is>
@@ -26170,7 +26192,7 @@
         </is>
       </c>
       <c r="I63" t="n">
-        <v>168.554993</v>
+        <v>165.660004</v>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="58">
@@ -26194,7 +26216,7 @@
         </is>
       </c>
       <c r="E64" s="33" t="n">
-        <v>58.315</v>
+        <v>56.88</v>
       </c>
       <c r="F64" s="34" t="inlineStr">
         <is>
@@ -26202,7 +26224,7 @@
         </is>
       </c>
       <c r="G64" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H64" s="34" t="inlineStr">
         <is>
@@ -26210,7 +26232,7 @@
         </is>
       </c>
       <c r="I64" t="n">
-        <v>58.314999</v>
+        <v>56.880001</v>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1" s="58">
@@ -26234,7 +26256,7 @@
         </is>
       </c>
       <c r="E65" s="33" t="n">
-        <v>186.91</v>
+        <v>185.64</v>
       </c>
       <c r="F65" s="34" t="inlineStr">
         <is>
@@ -26242,7 +26264,7 @@
         </is>
       </c>
       <c r="G65" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H65" s="34" t="inlineStr">
         <is>
@@ -26250,7 +26272,7 @@
         </is>
       </c>
       <c r="I65" t="n">
-        <v>186.910004</v>
+        <v>185.639999</v>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1" s="58">
@@ -26274,7 +26296,7 @@
         </is>
       </c>
       <c r="E66" s="33" t="n">
-        <v>145.38</v>
+        <v>143.04</v>
       </c>
       <c r="F66" s="34" t="inlineStr">
         <is>
@@ -26282,7 +26304,7 @@
         </is>
       </c>
       <c r="G66" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H66" s="34" t="inlineStr">
         <is>
@@ -26290,7 +26312,7 @@
         </is>
       </c>
       <c r="I66" t="n">
-        <v>145.380005</v>
+        <v>143.039993</v>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1" s="58">
@@ -26314,7 +26336,7 @@
         </is>
       </c>
       <c r="E67" s="33" t="n">
-        <v>163.69</v>
+        <v>160.35</v>
       </c>
       <c r="F67" s="34" t="inlineStr">
         <is>
@@ -26322,7 +26344,7 @@
         </is>
       </c>
       <c r="G67" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H67" s="34" t="inlineStr">
         <is>
@@ -26330,7 +26352,7 @@
         </is>
       </c>
       <c r="I67" t="n">
-        <v>163.690002</v>
+        <v>160.350006</v>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1" s="58">
@@ -26354,7 +26376,7 @@
         </is>
       </c>
       <c r="E68" s="33" t="n">
-        <v>2102.01</v>
+        <v>2108.06</v>
       </c>
       <c r="F68" s="34" t="inlineStr">
         <is>
@@ -26362,7 +26384,7 @@
         </is>
       </c>
       <c r="G68" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H68" s="34" t="inlineStr">
         <is>
@@ -26370,7 +26392,7 @@
         </is>
       </c>
       <c r="I68" t="n">
-        <v>2102.01001</v>
+        <v>2108.060059</v>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="58">
@@ -26394,7 +26416,7 @@
         </is>
       </c>
       <c r="E69" s="33" t="n">
-        <v>1165.962</v>
+        <v>1149.15</v>
       </c>
       <c r="F69" s="34" t="inlineStr">
         <is>
@@ -26402,7 +26424,7 @@
         </is>
       </c>
       <c r="G69" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H69" s="34" t="inlineStr">
         <is>
@@ -26410,7 +26432,7 @@
         </is>
       </c>
       <c r="I69" t="n">
-        <v>1165.962036</v>
+        <v>1149.150024</v>
       </c>
     </row>
     <row r="70" ht="15" customHeight="1" s="58">
@@ -26434,7 +26456,7 @@
         </is>
       </c>
       <c r="E70" s="33" t="n">
-        <v>92.55</v>
+        <v>91.37</v>
       </c>
       <c r="F70" s="34" t="inlineStr">
         <is>
@@ -26442,7 +26464,7 @@
         </is>
       </c>
       <c r="G70" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H70" s="34" t="inlineStr">
         <is>
@@ -26450,7 +26472,7 @@
         </is>
       </c>
       <c r="I70" t="n">
-        <v>92.550003</v>
+        <v>91.370003</v>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1" s="58">
@@ -26474,7 +26496,7 @@
         </is>
       </c>
       <c r="E71" s="33" t="n">
-        <v>1567.97</v>
+        <v>1559.18</v>
       </c>
       <c r="F71" s="34" t="inlineStr">
         <is>
@@ -26482,7 +26504,7 @@
         </is>
       </c>
       <c r="G71" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H71" s="34" t="inlineStr">
         <is>
@@ -26490,7 +26512,7 @@
         </is>
       </c>
       <c r="I71" t="n">
-        <v>1567.969971</v>
+        <v>1559.180054</v>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1" s="58">
@@ -26514,7 +26536,7 @@
         </is>
       </c>
       <c r="E72" s="33" t="n">
-        <v>112.89</v>
+        <v>110.14</v>
       </c>
       <c r="F72" s="34" t="inlineStr">
         <is>
@@ -26522,7 +26544,7 @@
         </is>
       </c>
       <c r="G72" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H72" s="34" t="inlineStr">
         <is>
@@ -26530,7 +26552,7 @@
         </is>
       </c>
       <c r="I72" t="n">
-        <v>112.889999</v>
+        <v>110.139999</v>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1" s="58">
@@ -26554,7 +26576,7 @@
         </is>
       </c>
       <c r="E73" s="33" t="n">
-        <v>208.65</v>
+        <v>208.64</v>
       </c>
       <c r="F73" s="34" t="inlineStr">
         <is>
@@ -26562,7 +26584,7 @@
         </is>
       </c>
       <c r="G73" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H73" s="34" t="inlineStr">
         <is>
@@ -26570,7 +26592,7 @@
         </is>
       </c>
       <c r="I73" t="n">
-        <v>208.649994</v>
+        <v>208.639999</v>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1" s="58">
@@ -26594,7 +26616,7 @@
         </is>
       </c>
       <c r="E74" s="33" t="n">
-        <v>89.04300000000001</v>
+        <v>88.81999999999999</v>
       </c>
       <c r="F74" s="34" t="inlineStr">
         <is>
@@ -26602,7 +26624,7 @@
         </is>
       </c>
       <c r="G74" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H74" s="34" t="inlineStr">
         <is>
@@ -26610,7 +26632,7 @@
         </is>
       </c>
       <c r="I74" t="n">
-        <v>89.042503</v>
+        <v>88.81999999999999</v>
       </c>
     </row>
     <row r="75" ht="15" customHeight="1" s="58">
@@ -26634,7 +26656,7 @@
         </is>
       </c>
       <c r="E75" s="33" t="n">
-        <v>103.09</v>
+        <v>99.89</v>
       </c>
       <c r="F75" s="34" t="inlineStr">
         <is>
@@ -26642,7 +26664,7 @@
         </is>
       </c>
       <c r="G75" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H75" s="34" t="inlineStr">
         <is>
@@ -26650,7 +26672,7 @@
         </is>
       </c>
       <c r="I75" t="n">
-        <v>103.089996</v>
+        <v>99.889999</v>
       </c>
     </row>
     <row r="76" ht="15" customHeight="1" s="58">
@@ -26674,7 +26696,7 @@
         </is>
       </c>
       <c r="E76" s="33" t="n">
-        <v>376.65</v>
+        <v>374.69</v>
       </c>
       <c r="F76" s="34" t="inlineStr">
         <is>
@@ -26682,7 +26704,7 @@
         </is>
       </c>
       <c r="G76" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H76" s="34" t="inlineStr">
         <is>
@@ -26690,7 +26712,7 @@
         </is>
       </c>
       <c r="I76" t="n">
-        <v>376.649994</v>
+        <v>374.690002</v>
       </c>
     </row>
     <row r="77" ht="15" customHeight="1" s="58">
@@ -26714,7 +26736,7 @@
         </is>
       </c>
       <c r="E77" s="33" t="n">
-        <v>403.78</v>
+        <v>408.95</v>
       </c>
       <c r="F77" s="34" t="inlineStr">
         <is>
@@ -26722,7 +26744,7 @@
         </is>
       </c>
       <c r="G77" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H77" s="34" t="inlineStr">
         <is>
@@ -26730,7 +26752,7 @@
         </is>
       </c>
       <c r="I77" t="n">
-        <v>403.779999</v>
+        <v>408.950012</v>
       </c>
     </row>
     <row r="78" ht="15" customHeight="1" s="58">
@@ -26754,7 +26776,7 @@
         </is>
       </c>
       <c r="E78" s="33" t="n">
-        <v>54.68</v>
+        <v>54.98</v>
       </c>
       <c r="F78" s="34" t="inlineStr">
         <is>
@@ -26762,7 +26784,7 @@
         </is>
       </c>
       <c r="G78" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H78" s="34" t="inlineStr">
         <is>
@@ -26770,7 +26792,7 @@
         </is>
       </c>
       <c r="I78" t="n">
-        <v>54.68</v>
+        <v>54.98</v>
       </c>
     </row>
     <row r="79" ht="15" customHeight="1" s="58">
@@ -26794,7 +26816,7 @@
         </is>
       </c>
       <c r="E79" s="33" t="n">
-        <v>88.2</v>
+        <v>87.42</v>
       </c>
       <c r="F79" s="34" t="inlineStr">
         <is>
@@ -26802,7 +26824,7 @@
         </is>
       </c>
       <c r="G79" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H79" s="34" t="inlineStr">
         <is>
@@ -26810,7 +26832,7 @@
         </is>
       </c>
       <c r="I79" t="n">
-        <v>88.199997</v>
+        <v>87.41999800000001</v>
       </c>
     </row>
     <row r="80" ht="15" customHeight="1" s="58">
@@ -26834,7 +26856,7 @@
         </is>
       </c>
       <c r="E80" s="33" t="n">
-        <v>314.785</v>
+        <v>301.54</v>
       </c>
       <c r="F80" s="34" t="inlineStr">
         <is>
@@ -26842,7 +26864,7 @@
         </is>
       </c>
       <c r="G80" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H80" s="34" t="inlineStr">
         <is>
@@ -26850,7 +26872,7 @@
         </is>
       </c>
       <c r="I80" t="n">
-        <v>314.785004</v>
+        <v>301.540009</v>
       </c>
     </row>
     <row r="81" ht="15" customHeight="1" s="58">
@@ -26874,7 +26896,7 @@
         </is>
       </c>
       <c r="E81" s="33" t="n">
-        <v>160.43</v>
+        <v>162.11</v>
       </c>
       <c r="F81" s="34" t="inlineStr">
         <is>
@@ -26882,7 +26904,7 @@
         </is>
       </c>
       <c r="G81" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H81" s="34" t="inlineStr">
         <is>
@@ -26890,7 +26912,7 @@
         </is>
       </c>
       <c r="I81" t="n">
-        <v>160.429993</v>
+        <v>162.110001</v>
       </c>
     </row>
     <row r="82" ht="15" customHeight="1" s="58">
@@ -26914,7 +26936,7 @@
         </is>
       </c>
       <c r="E82" s="33" t="n">
-        <v>591.4450000000001</v>
+        <v>585.39</v>
       </c>
       <c r="F82" s="34" t="inlineStr">
         <is>
@@ -26922,7 +26944,7 @@
         </is>
       </c>
       <c r="G82" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H82" s="34" t="inlineStr">
         <is>
@@ -26930,7 +26952,7 @@
         </is>
       </c>
       <c r="I82" t="n">
-        <v>591.445007</v>
+        <v>585.3900149999999</v>
       </c>
     </row>
     <row r="83" ht="15" customHeight="1" s="58">
@@ -26954,7 +26976,7 @@
         </is>
       </c>
       <c r="E83" s="33" t="n">
-        <v>146.695</v>
+        <v>147.99</v>
       </c>
       <c r="F83" s="34" t="inlineStr">
         <is>
@@ -26962,7 +26984,7 @@
         </is>
       </c>
       <c r="G83" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H83" s="34" t="inlineStr">
         <is>
@@ -26970,7 +26992,7 @@
         </is>
       </c>
       <c r="I83" t="n">
-        <v>146.695007</v>
+        <v>147.990005</v>
       </c>
     </row>
     <row r="84" ht="15" customHeight="1" s="58">
@@ -26994,7 +27016,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>64.62</v>
+        <v>62.33</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -27002,7 +27024,7 @@
         </is>
       </c>
       <c r="G84" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H84" s="34" t="inlineStr">
         <is>
@@ -27010,7 +27032,7 @@
         </is>
       </c>
       <c r="I84" t="n">
-        <v>62.978049</v>
+        <v>62.997935</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="58">
@@ -27034,7 +27056,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>603.88</v>
+        <v>597.37</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -27042,7 +27064,7 @@
         </is>
       </c>
       <c r="G85" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H85" s="34" t="inlineStr">
         <is>
@@ -27050,7 +27072,7 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>589.937146</v>
+        <v>600.2251659999999</v>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="58">
@@ -27074,7 +27096,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>64015</v>
+        <v>62812</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -27082,7 +27104,7 @@
         </is>
       </c>
       <c r="G86" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H86" s="34" t="inlineStr">
         <is>
@@ -27090,7 +27112,7 @@
         </is>
       </c>
       <c r="I86" t="n">
-        <v>61869.050744</v>
+        <v>62897.354246</v>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="58">
@@ -27114,7 +27136,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.006915</v>
+        <v>0.006634</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -27122,7 +27144,7 @@
         </is>
       </c>
       <c r="G87" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H87" s="34" t="inlineStr">
         <is>
@@ -27130,7 +27152,7 @@
         </is>
       </c>
       <c r="I87" t="n">
-        <v>0.006701</v>
+        <v>0.006825</v>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="58">
@@ -27154,7 +27176,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.01133</v>
+        <v>0.011288</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -27162,7 +27184,7 @@
         </is>
       </c>
       <c r="G88" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H88" s="34" t="inlineStr">
         <is>
@@ -27170,7 +27192,7 @@
         </is>
       </c>
       <c r="I88" t="n">
-        <v>0.011517</v>
+        <v>0.011121</v>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="58">
@@ -27194,7 +27216,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>67.38</v>
+        <v>65.84999999999999</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -27202,7 +27224,7 @@
         </is>
       </c>
       <c r="G89" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H89" s="34" t="inlineStr">
         <is>
@@ -27210,7 +27232,7 @@
         </is>
       </c>
       <c r="I89" t="n">
-        <v>64.86742700000001</v>
+        <v>65.54274599999999</v>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="58">
@@ -27234,7 +27256,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>1.7</v>
+        <v>1.66</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -27242,7 +27264,7 @@
         </is>
       </c>
       <c r="G90" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H90" s="34" t="inlineStr">
         <is>
@@ -27250,7 +27272,7 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>1.635721</v>
+        <v>1.647569</v>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="58">
@@ -27282,7 +27304,7 @@
         </is>
       </c>
       <c r="G91" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H91" s="34" t="inlineStr">
         <is>
@@ -27314,7 +27336,7 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
-        <v>0.013725</v>
+        <v>0.013586</v>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
@@ -27322,7 +27344,7 @@
         </is>
       </c>
       <c r="G92" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H92" s="34" t="inlineStr">
         <is>
@@ -27330,7 +27352,7 @@
         </is>
       </c>
       <c r="I92" t="n">
-        <v>0.012786</v>
+        <v>0.012934</v>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="58">
@@ -27354,7 +27376,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>2.753159</v>
+        <v>2.64433</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -27362,7 +27384,7 @@
         </is>
       </c>
       <c r="G93" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H93" s="34" t="inlineStr">
         <is>
@@ -27370,7 +27392,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>2.686915</v>
+        <v>2.697433</v>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="58">
@@ -27394,7 +27416,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>25.082961</v>
+        <v>24.289554</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -27402,7 +27424,7 @@
         </is>
       </c>
       <c r="G94" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H94" s="34" t="inlineStr">
         <is>
@@ -27410,7 +27432,7 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>24.454453</v>
+        <v>24.582074</v>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="58">
@@ -27434,7 +27456,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.112806</v>
+        <v>0.110297</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -27442,7 +27464,7 @@
         </is>
       </c>
       <c r="G95" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H95" s="34" t="inlineStr">
         <is>
@@ -27450,7 +27472,7 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>0.115522</v>
+        <v>0.112477</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="58">
@@ -27474,7 +27496,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>19795.1864</v>
+        <v>19581.7886</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -27482,7 +27504,7 @@
         </is>
       </c>
       <c r="G96" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H96" s="34" t="inlineStr">
         <is>
@@ -27490,7 +27512,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>19338.139633</v>
+        <v>19675.38093</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="58">
@@ -27514,7 +27536,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2098411.7</v>
+        <v>2058977.36</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -27522,7 +27544,7 @@
         </is>
       </c>
       <c r="G97" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H97" s="34" t="inlineStr">
         <is>
@@ -27530,7 +27552,7 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>2028067.483392</v>
+        <v>2061775.272181</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="58">
@@ -27554,7 +27576,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>2.843173</v>
+        <v>2.791446</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -27562,7 +27584,7 @@
         </is>
       </c>
       <c r="G98" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H98" s="34" t="inlineStr">
         <is>
@@ -27570,7 +27592,7 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>2.766248</v>
+        <v>2.795793</v>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="58">
@@ -27594,7 +27616,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>55579.1456</v>
+        <v>54778.3302</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -27602,7 +27624,7 @@
         </is>
       </c>
       <c r="G99" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H99" s="34" t="inlineStr">
         <is>
@@ -27610,7 +27632,7 @@
         </is>
       </c>
       <c r="I99" t="n">
-        <v>53244.248293</v>
+        <v>54963.687363</v>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="58">
@@ -27634,7 +27656,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>25.257285</v>
+        <v>25.403812</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -27642,7 +27664,7 @@
         </is>
       </c>
       <c r="G100" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H100" s="34" t="inlineStr">
         <is>
@@ -27650,7 +27672,7 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>25.05189</v>
+        <v>25.167651</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="58">
@@ -27674,7 +27696,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>64015</v>
+        <v>62812</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -27682,7 +27704,7 @@
         </is>
       </c>
       <c r="G101" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H101" s="34" t="inlineStr">
         <is>
@@ -27690,7 +27712,7 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>61869.050744</v>
+        <v>62897.354246</v>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="58">
@@ -27714,7 +27736,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>17.07</v>
+        <v>18.13</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -27722,7 +27744,7 @@
         </is>
       </c>
       <c r="G102" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H102" s="34" t="inlineStr">
         <is>
@@ -27730,7 +27752,7 @@
         </is>
       </c>
       <c r="I102" t="n">
-        <v>16.380939</v>
+        <v>16.414197</v>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="58">
@@ -27828,7 +27850,7 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
-        <v>0.006915</v>
+        <v>0.006634</v>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
@@ -27836,7 +27858,7 @@
         </is>
       </c>
       <c r="G105" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H105" s="34" t="inlineStr">
         <is>
@@ -27844,7 +27866,7 @@
         </is>
       </c>
       <c r="I105" t="n">
-        <v>0.006701</v>
+        <v>0.006825</v>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="58">
@@ -27868,7 +27890,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>67.38</v>
+        <v>65.84999999999999</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>
@@ -27876,7 +27898,7 @@
         </is>
       </c>
       <c r="G106" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H106" s="34" t="inlineStr">
         <is>
@@ -27884,7 +27906,7 @@
         </is>
       </c>
       <c r="I106" t="n">
-        <v>64.86742700000001</v>
+        <v>65.54274599999999</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="58">
@@ -27916,7 +27938,7 @@
         </is>
       </c>
       <c r="G107" s="28" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="H107" s="34" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Weekly dashboard update — 2026-06-09
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-42660" yWindow="-540" windowWidth="32460" windowHeight="17180" tabRatio="500" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Realized" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Realized" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Prices" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Reference" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="AsOfDate">'FX &amp; Assumptions'!$C$5</definedName>
@@ -697,14 +697,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -726,8 +726,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -752,10 +752,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -764,10 +764,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4F81BD"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+              <a:ln w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -777,10 +777,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="C0504D"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -790,10 +790,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="9BBB59"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -803,10 +803,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="8064A2"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -816,10 +816,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4BACC6"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -829,10 +829,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="F79646"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -842,14 +842,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -875,14 +875,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -908,14 +908,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -941,14 +941,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -974,14 +974,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1007,14 +1007,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1038,16 +1038,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1142,16 +1142,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1172,10 +1172,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1187,14 +1187,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1216,8 +1216,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1242,10 +1242,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1254,10 +1254,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4672A8"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1267,10 +1267,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="AB4744"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1280,10 +1280,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="8AA64F"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1293,10 +1293,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="725990"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1306,10 +1306,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4299B0"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1319,10 +1319,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="DC853E"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1332,10 +1332,10 @@
             <idx val="6"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="93A9CE"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1345,10 +1345,10 @@
             <idx val="7"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="D09493"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1358,10 +1358,10 @@
             <idx val="8"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="B8CD97"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1371,14 +1371,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1405,14 +1405,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1439,14 +1439,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1473,14 +1473,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1507,14 +1507,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1541,14 +1541,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1575,14 +1575,14 @@
             <dLbl>
               <idx val="6"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1609,14 +1609,14 @@
             <dLbl>
               <idx val="7"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1643,14 +1643,14 @@
             <dLbl>
               <idx val="8"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1675,16 +1675,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1791,16 +1791,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1821,10 +1821,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1836,14 +1836,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1865,8 +1865,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1893,10 +1893,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1904,16 +1904,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2016,7 +2016,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2025,9 +2025,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2059,7 +2059,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2073,7 +2073,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2082,9 +2082,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2109,16 +2109,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2139,10 +2139,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2154,14 +2154,14 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -2183,8 +2183,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -2200,10 +2200,10 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2211,16 +2211,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2411,7 +2411,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2420,9 +2420,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2454,7 +2454,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2468,7 +2468,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2477,9 +2477,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2504,16 +2504,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2534,10 +2534,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2549,7 +2549,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>1</col>
@@ -2569,9 +2569,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2596,9 +2596,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+          <c:chart r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2623,9 +2623,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+          <c:chart r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2650,9 +2650,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+          <c:chart r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -21758,28 +21758,28 @@
         <v>46182</v>
       </c>
       <c r="C13" s="29" t="n">
-        <v>26546838</v>
+        <v>25610409</v>
       </c>
       <c r="D13" s="29" t="n">
-        <v>22668073</v>
+        <v>22675070</v>
       </c>
       <c r="E13" s="29" t="n">
-        <v>3878765</v>
+        <v>2935339</v>
       </c>
       <c r="F13" s="30" t="n">
-        <v>0.1711</v>
+        <v>0.1295</v>
       </c>
       <c r="G13" s="29" t="n">
-        <v>19003537</v>
+        <v>18067456</v>
       </c>
       <c r="H13" s="29" t="n">
-        <v>5010088</v>
+        <v>5003719</v>
       </c>
       <c r="I13" s="29" t="n">
-        <v>1148042</v>
+        <v>1150834</v>
       </c>
       <c r="J13" s="31" t="n">
-        <v>32.78</v>
+        <v>32.83</v>
       </c>
       <c r="K13" s="32" t="inlineStr">
         <is>
@@ -23526,7 +23526,7 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>32.78</v>
+        <v>32.83</v>
       </c>
       <c r="D6" s="64" t="inlineStr">
         <is>
@@ -23575,7 +23575,7 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>25.4864</v>
+        <v>25.5458</v>
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
@@ -23694,27 +23694,27 @@
         </is>
       </c>
       <c r="E5" s="33" t="n">
+        <v>23.3473</v>
+      </c>
+      <c r="F5" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G5" s="28" t="n">
+        <v>46178</v>
+      </c>
+      <c r="H5" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
         <v>26.0771</v>
       </c>
-      <c r="F5" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G5" s="28" t="n">
-        <v>46177</v>
-      </c>
-      <c r="H5" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I5" t="n">
-        <v>26.6433</v>
-      </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
@@ -23739,7 +23739,7 @@
         </is>
       </c>
       <c r="E6" s="33" t="n">
-        <v>10.6859</v>
+        <v>10.6865</v>
       </c>
       <c r="F6" s="34" t="inlineStr">
         <is>
@@ -23747,7 +23747,7 @@
         </is>
       </c>
       <c r="G6" s="28" t="n">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="H6" s="34" t="inlineStr">
         <is>
@@ -23759,7 +23759,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
@@ -23784,27 +23784,27 @@
         </is>
       </c>
       <c r="E7" s="33" t="n">
+        <v>7.1091</v>
+      </c>
+      <c r="F7" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G7" s="28" t="n">
+        <v>46178</v>
+      </c>
+      <c r="H7" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
         <v>7.1186</v>
       </c>
-      <c r="F7" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G7" s="28" t="n">
-        <v>46177</v>
-      </c>
-      <c r="H7" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I7" t="n">
-        <v>7.1237</v>
-      </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
@@ -23829,27 +23829,27 @@
         </is>
       </c>
       <c r="E8" s="33" t="n">
+        <v>9.393700000000001</v>
+      </c>
+      <c r="F8" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G8" s="28" t="n">
+        <v>46178</v>
+      </c>
+      <c r="H8" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
         <v>9.7468</v>
       </c>
-      <c r="F8" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G8" s="28" t="n">
-        <v>46177</v>
-      </c>
-      <c r="H8" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I8" t="n">
-        <v>9.7875</v>
-      </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
@@ -23874,27 +23874,27 @@
         </is>
       </c>
       <c r="E9" s="33" t="n">
+        <v>9.1631</v>
+      </c>
+      <c r="F9" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G9" s="28" t="n">
+        <v>46181</v>
+      </c>
+      <c r="H9" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
         <v>9.320600000000001</v>
       </c>
-      <c r="F9" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G9" s="28" t="n">
-        <v>46178</v>
-      </c>
-      <c r="H9" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I9" t="n">
-        <v>9.4649</v>
-      </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
@@ -23919,27 +23919,27 @@
         </is>
       </c>
       <c r="E10" s="33" t="n">
+        <v>13.5827</v>
+      </c>
+      <c r="F10" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G10" s="28" t="n">
+        <v>46178</v>
+      </c>
+      <c r="H10" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
         <v>13.6486</v>
       </c>
-      <c r="F10" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G10" s="28" t="n">
-        <v>46177</v>
-      </c>
-      <c r="H10" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I10" t="n">
-        <v>13.4306</v>
-      </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
@@ -23964,27 +23964,27 @@
         </is>
       </c>
       <c r="E11" s="33" t="n">
+        <v>12.9039</v>
+      </c>
+      <c r="F11" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G11" s="28" t="n">
+        <v>46181</v>
+      </c>
+      <c r="H11" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
         <v>13.2022</v>
       </c>
-      <c r="F11" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G11" s="28" t="n">
-        <v>46178</v>
-      </c>
-      <c r="H11" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I11" t="n">
-        <v>13.3664</v>
-      </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
@@ -24009,27 +24009,27 @@
         </is>
       </c>
       <c r="E12" s="33" t="n">
+        <v>26.0378</v>
+      </c>
+      <c r="F12" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G12" s="28" t="n">
+        <v>46181</v>
+      </c>
+      <c r="H12" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
         <v>26.689</v>
       </c>
-      <c r="F12" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G12" s="28" t="n">
-        <v>46178</v>
-      </c>
-      <c r="H12" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I12" t="n">
-        <v>27.1532</v>
-      </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
@@ -24054,27 +24054,27 @@
         </is>
       </c>
       <c r="E13" s="33" t="n">
+        <v>35.7675</v>
+      </c>
+      <c r="F13" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G13" s="28" t="n">
+        <v>46181</v>
+      </c>
+      <c r="H13" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
         <v>36.2424</v>
       </c>
-      <c r="F13" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G13" s="28" t="n">
-        <v>46178</v>
-      </c>
-      <c r="H13" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I13" t="n">
-        <v>36.5235</v>
-      </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
@@ -24099,27 +24099,27 @@
         </is>
       </c>
       <c r="E14" s="33" t="n">
+        <v>25.2435</v>
+      </c>
+      <c r="F14" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G14" s="28" t="n">
+        <v>46181</v>
+      </c>
+      <c r="H14" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
         <v>25.4991</v>
       </c>
-      <c r="F14" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G14" s="28" t="n">
-        <v>46178</v>
-      </c>
-      <c r="H14" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I14" t="n">
-        <v>25.5684</v>
-      </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
@@ -24144,27 +24144,27 @@
         </is>
       </c>
       <c r="E15" s="33" t="n">
+        <v>14.8572</v>
+      </c>
+      <c r="F15" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G15" s="28" t="n">
+        <v>46177</v>
+      </c>
+      <c r="H15" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
         <v>14.3709</v>
       </c>
-      <c r="F15" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G15" s="28" t="n">
-        <v>46175</v>
-      </c>
-      <c r="H15" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I15" t="n">
-        <v>14.8616</v>
-      </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-02</t>
         </is>
       </c>
     </row>
@@ -24189,27 +24189,27 @@
         </is>
       </c>
       <c r="E16" s="33" t="n">
+        <v>80.3703</v>
+      </c>
+      <c r="F16" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G16" s="28" t="n">
+        <v>46181</v>
+      </c>
+      <c r="H16" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
         <v>81.4024</v>
       </c>
-      <c r="F16" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G16" s="28" t="n">
-        <v>46178</v>
-      </c>
-      <c r="H16" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I16" t="n">
-        <v>81.99809999999999</v>
-      </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
@@ -24234,27 +24234,27 @@
         </is>
       </c>
       <c r="E17" s="33" t="n">
+        <v>52.898</v>
+      </c>
+      <c r="F17" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G17" s="28" t="n">
+        <v>46181</v>
+      </c>
+      <c r="H17" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
         <v>53.4695</v>
       </c>
-      <c r="F17" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G17" s="28" t="n">
-        <v>46178</v>
-      </c>
-      <c r="H17" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I17" t="n">
-        <v>53.6077</v>
-      </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
@@ -24279,27 +24279,27 @@
         </is>
       </c>
       <c r="E18" s="33" t="n">
+        <v>16.4116</v>
+      </c>
+      <c r="F18" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G18" s="28" t="n">
+        <v>46181</v>
+      </c>
+      <c r="H18" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
         <v>16.4291</v>
       </c>
-      <c r="F18" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G18" s="28" t="n">
-        <v>46178</v>
-      </c>
-      <c r="H18" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I18" t="n">
-        <v>16.4146</v>
-      </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
@@ -24324,27 +24324,27 @@
         </is>
       </c>
       <c r="E19" s="33" t="n">
+        <v>23.4026</v>
+      </c>
+      <c r="F19" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G19" s="28" t="n">
+        <v>46181</v>
+      </c>
+      <c r="H19" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
         <v>23.4013</v>
       </c>
-      <c r="F19" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G19" s="28" t="n">
-        <v>46178</v>
-      </c>
-      <c r="H19" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I19" t="n">
-        <v>23.4009</v>
-      </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
@@ -24369,27 +24369,27 @@
         </is>
       </c>
       <c r="E20" s="33" t="n">
+        <v>40.5739</v>
+      </c>
+      <c r="F20" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G20" s="28" t="n">
+        <v>46178</v>
+      </c>
+      <c r="H20" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
         <v>41.6601</v>
       </c>
-      <c r="F20" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G20" s="28" t="n">
-        <v>46177</v>
-      </c>
-      <c r="H20" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I20" t="n">
-        <v>41.7733</v>
-      </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
@@ -24414,27 +24414,27 @@
         </is>
       </c>
       <c r="E21" s="33" t="n">
+        <v>13.241</v>
+      </c>
+      <c r="F21" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G21" s="28" t="n">
+        <v>46181</v>
+      </c>
+      <c r="H21" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
         <v>13.3947</v>
       </c>
-      <c r="F21" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G21" s="28" t="n">
-        <v>46178</v>
-      </c>
-      <c r="H21" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I21" t="n">
-        <v>13.6591</v>
-      </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
@@ -24459,27 +24459,27 @@
         </is>
       </c>
       <c r="E22" s="33" t="n">
+        <v>13.2668</v>
+      </c>
+      <c r="F22" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G22" s="28" t="n">
+        <v>46178</v>
+      </c>
+      <c r="H22" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
         <v>13.1535</v>
       </c>
-      <c r="F22" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G22" s="28" t="n">
-        <v>46177</v>
-      </c>
-      <c r="H22" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I22" t="n">
-        <v>12.6846</v>
-      </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
@@ -24504,27 +24504,27 @@
         </is>
       </c>
       <c r="E23" s="33" t="n">
+        <v>12.3035</v>
+      </c>
+      <c r="F23" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G23" s="28" t="n">
+        <v>46181</v>
+      </c>
+      <c r="H23" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
         <v>12.4665</v>
       </c>
-      <c r="F23" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G23" s="28" t="n">
-        <v>46178</v>
-      </c>
-      <c r="H23" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I23" t="n">
-        <v>12.5147</v>
-      </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
@@ -24549,27 +24549,27 @@
         </is>
       </c>
       <c r="E24" s="33" t="n">
+        <v>11.9931</v>
+      </c>
+      <c r="F24" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G24" s="28" t="n">
+        <v>46178</v>
+      </c>
+      <c r="H24" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
         <v>12.0868</v>
       </c>
-      <c r="F24" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G24" s="28" t="n">
-        <v>46177</v>
-      </c>
-      <c r="H24" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I24" t="n">
-        <v>12.3129</v>
-      </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
@@ -24594,27 +24594,27 @@
         </is>
       </c>
       <c r="E25" s="33" t="n">
+        <v>9.8523</v>
+      </c>
+      <c r="F25" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G25" s="28" t="n">
+        <v>46181</v>
+      </c>
+      <c r="H25" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
         <v>10.0147</v>
       </c>
-      <c r="F25" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G25" s="28" t="n">
-        <v>46178</v>
-      </c>
-      <c r="H25" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I25" t="n">
-        <v>10.0259</v>
-      </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
@@ -24639,27 +24639,27 @@
         </is>
       </c>
       <c r="E26" s="33" t="n">
+        <v>13.8268</v>
+      </c>
+      <c r="F26" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G26" s="28" t="n">
+        <v>46181</v>
+      </c>
+      <c r="H26" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
         <v>14.0583</v>
       </c>
-      <c r="F26" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G26" s="28" t="n">
-        <v>46178</v>
-      </c>
-      <c r="H26" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I26" t="n">
-        <v>14.078</v>
-      </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
@@ -24684,27 +24684,27 @@
         </is>
       </c>
       <c r="E27" s="33" t="n">
+        <v>16.8474</v>
+      </c>
+      <c r="F27" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G27" s="28" t="n">
+        <v>46181</v>
+      </c>
+      <c r="H27" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
         <v>17.105</v>
       </c>
-      <c r="F27" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G27" s="28" t="n">
-        <v>46178</v>
-      </c>
-      <c r="H27" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I27" t="n">
-        <v>17.1468</v>
-      </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
@@ -24729,27 +24729,27 @@
         </is>
       </c>
       <c r="E28" s="33" t="n">
+        <v>19.1156</v>
+      </c>
+      <c r="F28" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G28" s="28" t="n">
+        <v>46181</v>
+      </c>
+      <c r="H28" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
         <v>19.8791</v>
       </c>
-      <c r="F28" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G28" s="28" t="n">
-        <v>46178</v>
-      </c>
-      <c r="H28" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I28" t="n">
-        <v>19.8865</v>
-      </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
@@ -24774,27 +24774,27 @@
         </is>
       </c>
       <c r="E29" s="33" t="n">
+        <v>23.8964</v>
+      </c>
+      <c r="F29" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G29" s="28" t="n">
+        <v>46178</v>
+      </c>
+      <c r="H29" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
         <v>27.8357</v>
       </c>
-      <c r="F29" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G29" s="28" t="n">
-        <v>46177</v>
-      </c>
-      <c r="H29" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I29" t="n">
-        <v>29.2852</v>
-      </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
@@ -24819,27 +24819,27 @@
         </is>
       </c>
       <c r="E30" s="33" t="n">
+        <v>36.6591</v>
+      </c>
+      <c r="F30" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G30" s="28" t="n">
+        <v>46178</v>
+      </c>
+      <c r="H30" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
         <v>38.836</v>
       </c>
-      <c r="F30" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G30" s="28" t="n">
-        <v>46177</v>
-      </c>
-      <c r="H30" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I30" t="n">
-        <v>39.0534</v>
-      </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
@@ -24864,27 +24864,27 @@
         </is>
       </c>
       <c r="E31" s="33" t="n">
+        <v>12.7623</v>
+      </c>
+      <c r="F31" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G31" s="28" t="n">
+        <v>46181</v>
+      </c>
+      <c r="H31" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
         <v>12.9367</v>
       </c>
-      <c r="F31" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G31" s="28" t="n">
-        <v>46178</v>
-      </c>
-      <c r="H31" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I31" t="n">
-        <v>13.0307</v>
-      </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
@@ -24909,7 +24909,7 @@
         </is>
       </c>
       <c r="E32" s="33" t="n">
-        <v>21.7047</v>
+        <v>21.7053</v>
       </c>
       <c r="F32" s="34" t="inlineStr">
         <is>
@@ -24917,7 +24917,7 @@
         </is>
       </c>
       <c r="G32" s="28" t="n">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="H32" s="34" t="inlineStr">
         <is>
@@ -24929,7 +24929,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
@@ -24954,27 +24954,27 @@
         </is>
       </c>
       <c r="E33" s="33" t="n">
+        <v>12.3354</v>
+      </c>
+      <c r="F33" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G33" s="28" t="n">
+        <v>46181</v>
+      </c>
+      <c r="H33" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
         <v>12.5235</v>
       </c>
-      <c r="F33" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G33" s="28" t="n">
-        <v>46178</v>
-      </c>
-      <c r="H33" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I33" t="n">
-        <v>12.5995</v>
-      </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
@@ -24999,27 +24999,27 @@
         </is>
       </c>
       <c r="E34" s="33" t="n">
+        <v>16.2041</v>
+      </c>
+      <c r="F34" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G34" s="28" t="n">
+        <v>46181</v>
+      </c>
+      <c r="H34" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
         <v>16.203</v>
       </c>
-      <c r="F34" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G34" s="28" t="n">
-        <v>46178</v>
-      </c>
-      <c r="H34" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I34" t="n">
-        <v>16.2028</v>
-      </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
@@ -25044,27 +25044,27 @@
         </is>
       </c>
       <c r="E35" s="33" t="n">
+        <v>27.8538</v>
+      </c>
+      <c r="F35" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G35" s="28" t="n">
+        <v>46178</v>
+      </c>
+      <c r="H35" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
         <v>28.936</v>
       </c>
-      <c r="F35" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G35" s="28" t="n">
-        <v>46177</v>
-      </c>
-      <c r="H35" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I35" t="n">
-        <v>28.8772</v>
-      </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
@@ -25089,27 +25089,27 @@
         </is>
       </c>
       <c r="E36" s="33" t="n">
+        <v>9.978999999999999</v>
+      </c>
+      <c r="F36" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G36" s="28" t="n">
+        <v>46181</v>
+      </c>
+      <c r="H36" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
         <v>10.032</v>
       </c>
-      <c r="F36" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G36" s="28" t="n">
-        <v>46178</v>
-      </c>
-      <c r="H36" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I36" t="n">
-        <v>9.992800000000001</v>
-      </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
@@ -25134,27 +25134,27 @@
         </is>
       </c>
       <c r="E37" s="33" t="n">
+        <v>22.348</v>
+      </c>
+      <c r="F37" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G37" s="28" t="n">
+        <v>46181</v>
+      </c>
+      <c r="H37" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
         <v>22.6458</v>
       </c>
-      <c r="F37" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G37" s="28" t="n">
-        <v>46178</v>
-      </c>
-      <c r="H37" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I37" t="n">
-        <v>22.7858</v>
-      </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
@@ -25459,7 +25459,7 @@
         </is>
       </c>
       <c r="E45" s="33" t="n">
-        <v>0.45</v>
+        <v>0.44</v>
       </c>
       <c r="F45" s="34" t="inlineStr">
         <is>
@@ -25475,7 +25475,7 @@
         </is>
       </c>
       <c r="I45" t="n">
-        <v>0.45</v>
+        <v>0.44</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="58">
@@ -25499,7 +25499,7 @@
         </is>
       </c>
       <c r="E46" s="33" t="n">
-        <v>0.3</v>
+        <v>0.29</v>
       </c>
       <c r="F46" s="34" t="inlineStr">
         <is>
@@ -25515,7 +25515,7 @@
         </is>
       </c>
       <c r="I46" t="n">
-        <v>0.3</v>
+        <v>0.29</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" s="58">
@@ -25616,7 +25616,7 @@
         </is>
       </c>
       <c r="E49" s="33" t="n">
-        <v>64.5</v>
+        <v>63.75</v>
       </c>
       <c r="F49" s="34" t="inlineStr">
         <is>
@@ -25632,7 +25632,7 @@
         </is>
       </c>
       <c r="I49" t="n">
-        <v>67</v>
+        <v>64.5</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="58">
@@ -25696,7 +25696,7 @@
         </is>
       </c>
       <c r="E51" s="33" t="n">
-        <v>15.2</v>
+        <v>15.3</v>
       </c>
       <c r="F51" s="34" t="inlineStr">
         <is>
@@ -25712,7 +25712,7 @@
         </is>
       </c>
       <c r="I51" t="n">
-        <v>15.2</v>
+        <v>15.3</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" s="58">
@@ -25736,7 +25736,7 @@
         </is>
       </c>
       <c r="E52" s="33" t="n">
-        <v>13.3</v>
+        <v>13.5</v>
       </c>
       <c r="F52" s="34" t="inlineStr">
         <is>
@@ -25816,7 +25816,7 @@
         </is>
       </c>
       <c r="E54" s="33" t="n">
-        <v>21.2</v>
+        <v>20.7</v>
       </c>
       <c r="F54" s="34" t="inlineStr">
         <is>
@@ -25832,7 +25832,7 @@
         </is>
       </c>
       <c r="I54" t="n">
-        <v>21.200001</v>
+        <v>20.700001</v>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="58">
@@ -25896,7 +25896,7 @@
         </is>
       </c>
       <c r="E56" s="33" t="n">
-        <v>4.82</v>
+        <v>4.76</v>
       </c>
       <c r="F56" s="34" t="inlineStr">
         <is>
@@ -25912,7 +25912,7 @@
         </is>
       </c>
       <c r="I56" t="n">
-        <v>4.82</v>
+        <v>4.76</v>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1" s="58">
@@ -25936,7 +25936,7 @@
         </is>
       </c>
       <c r="E57" s="33" t="n">
-        <v>2.64</v>
+        <v>2.58</v>
       </c>
       <c r="F57" s="34" t="inlineStr">
         <is>
@@ -25952,7 +25952,7 @@
         </is>
       </c>
       <c r="I57" t="n">
-        <v>2.64</v>
+        <v>2.58</v>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="58">
@@ -25976,7 +25976,7 @@
         </is>
       </c>
       <c r="E58" s="33" t="n">
-        <v>12.3</v>
+        <v>12.4</v>
       </c>
       <c r="F58" s="34" t="inlineStr">
         <is>
@@ -25992,7 +25992,7 @@
         </is>
       </c>
       <c r="I58" t="n">
-        <v>12.3</v>
+        <v>12.4</v>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="58">
@@ -26016,7 +26016,7 @@
         </is>
       </c>
       <c r="E59" s="33" t="n">
-        <v>17.4</v>
+        <v>16.8</v>
       </c>
       <c r="F59" s="34" t="inlineStr">
         <is>
@@ -26032,7 +26032,7 @@
         </is>
       </c>
       <c r="I59" t="n">
-        <v>17.4</v>
+        <v>16.799999</v>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1" s="58">
@@ -27016,7 +27016,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>62.33</v>
+        <v>62.5</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -27032,7 +27032,7 @@
         </is>
       </c>
       <c r="I84" t="n">
-        <v>62.997935</v>
+        <v>63.789122</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="58">
@@ -27056,7 +27056,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>597.37</v>
+        <v>597.47</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -27072,7 +27072,7 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>600.2251659999999</v>
+        <v>598.971959</v>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="58">
@@ -27096,7 +27096,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>62812</v>
+        <v>62719</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -27112,7 +27112,7 @@
         </is>
       </c>
       <c r="I86" t="n">
-        <v>62897.354246</v>
+        <v>62917.361877</v>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="58">
@@ -27136,7 +27136,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.006634</v>
+        <v>0.006772</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -27152,7 +27152,7 @@
         </is>
       </c>
       <c r="I87" t="n">
-        <v>0.006825</v>
+        <v>0.006867</v>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="58">
@@ -27176,7 +27176,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.011288</v>
+        <v>0.011151</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -27192,7 +27192,7 @@
         </is>
       </c>
       <c r="I88" t="n">
-        <v>0.011121</v>
+        <v>0.011091</v>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="58">
@@ -27216,7 +27216,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>65.84999999999999</v>
+        <v>66.29000000000001</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -27232,7 +27232,7 @@
         </is>
       </c>
       <c r="I89" t="n">
-        <v>65.54274599999999</v>
+        <v>66.163312</v>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="58">
@@ -27256,7 +27256,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>1.66</v>
+        <v>1.67</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -27272,7 +27272,7 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>1.647569</v>
+        <v>1.674318</v>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="58">
@@ -27336,7 +27336,7 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
-        <v>0.013586</v>
+        <v>0.013957</v>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
@@ -27352,7 +27352,7 @@
         </is>
       </c>
       <c r="I92" t="n">
-        <v>0.012934</v>
+        <v>0.01372</v>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="58">
@@ -27376,7 +27376,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>2.64433</v>
+        <v>2.650793</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -27392,7 +27392,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>2.697433</v>
+        <v>2.717743</v>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="58">
@@ -27416,7 +27416,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>24.289554</v>
+        <v>24.859401</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -27432,7 +27432,7 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>24.582074</v>
+        <v>24.780238</v>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="58">
@@ -27456,7 +27456,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.110297</v>
+        <v>0.112706</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -27472,7 +27472,7 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>0.112477</v>
+        <v>0.112702</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="58">
@@ -27496,7 +27496,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>19581.7886</v>
+        <v>19614.9401</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -27512,7 +27512,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>19675.38093</v>
+        <v>19664.249425</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="58">
@@ -27536,7 +27536,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2058977.36</v>
+        <v>2059064.77</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -27552,7 +27552,7 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>2061775.272181</v>
+        <v>2065576.99041</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="58">
@@ -27576,7 +27576,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>2.791446</v>
+        <v>2.814811</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -27592,7 +27592,7 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>2.795793</v>
+        <v>2.823931</v>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="58">
@@ -27616,7 +27616,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>54778.3302</v>
+        <v>55107.7814</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -27632,7 +27632,7 @@
         </is>
       </c>
       <c r="I99" t="n">
-        <v>54963.687363</v>
+        <v>54952.28728</v>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="58">
@@ -27656,7 +27656,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>25.403812</v>
+        <v>25.339639</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -27672,7 +27672,7 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>25.167651</v>
+        <v>25.246098</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="58">
@@ -27696,7 +27696,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>62812</v>
+        <v>62719</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -27712,7 +27712,7 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>62897.354246</v>
+        <v>62917.361877</v>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="58">
@@ -27736,7 +27736,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>18.13</v>
+        <v>18.01</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -27752,7 +27752,7 @@
         </is>
       </c>
       <c r="I102" t="n">
-        <v>16.414197</v>
+        <v>16.895152</v>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="58">
@@ -27850,7 +27850,7 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
-        <v>0.006634</v>
+        <v>0.006772</v>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
@@ -27866,7 +27866,7 @@
         </is>
       </c>
       <c r="I105" t="n">
-        <v>0.006825</v>
+        <v>0.006867</v>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="58">
@@ -27890,7 +27890,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>65.84999999999999</v>
+        <v>66.29000000000001</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>
@@ -27906,7 +27906,7 @@
         </is>
       </c>
       <c r="I106" t="n">
-        <v>65.54274599999999</v>
+        <v>66.163312</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="58">

</xml_diff>

<commit_message>
Daily dashboard update — 2026-06-10
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-42660" yWindow="-540" windowWidth="32460" windowHeight="17180" tabRatio="500" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Realized" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Prices" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Reference" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Realized" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="AsOfDate">'FX &amp; Assumptions'!$C$5</definedName>
@@ -697,14 +697,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -726,8 +726,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -752,10 +752,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -764,10 +764,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4F81BD"/>
               </a:solidFill>
-              <a:ln w="0">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -777,10 +777,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="C0504D"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -790,10 +790,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="9BBB59"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -803,10 +803,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="8064A2"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -816,10 +816,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4BACC6"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -829,10 +829,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="F79646"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -842,14 +842,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -875,14 +875,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -908,14 +908,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -941,14 +941,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -974,14 +974,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1007,14 +1007,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1038,16 +1038,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1142,16 +1142,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1172,10 +1172,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1187,14 +1187,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1216,8 +1216,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1242,10 +1242,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1254,10 +1254,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4672A8"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1267,10 +1267,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="AB4744"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1280,10 +1280,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="8AA64F"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1293,10 +1293,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="725990"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1306,10 +1306,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4299B0"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1319,10 +1319,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="DC853E"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1332,10 +1332,10 @@
             <idx val="6"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="93A9CE"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1345,10 +1345,10 @@
             <idx val="7"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="D09493"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1358,10 +1358,10 @@
             <idx val="8"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="B8CD97"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1371,14 +1371,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1405,14 +1405,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1439,14 +1439,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1473,14 +1473,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1507,14 +1507,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1541,14 +1541,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1575,14 +1575,14 @@
             <dLbl>
               <idx val="6"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1609,14 +1609,14 @@
             <dLbl>
               <idx val="7"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1643,14 +1643,14 @@
             <dLbl>
               <idx val="8"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1675,16 +1675,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1791,16 +1791,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1821,10 +1821,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1836,14 +1836,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1865,8 +1865,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1893,10 +1893,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1904,16 +1904,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2016,7 +2016,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2025,9 +2025,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2059,7 +2059,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="9360">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2073,7 +2073,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2082,9 +2082,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2109,16 +2109,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2139,10 +2139,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2154,14 +2154,14 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -2183,8 +2183,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -2200,10 +2200,10 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2211,16 +2211,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2411,7 +2411,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2420,9 +2420,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2454,7 +2454,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="9360">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2468,7 +2468,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2477,9 +2477,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2504,16 +2504,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2534,10 +2534,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2549,7 +2549,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>1</col>
@@ -2569,9 +2569,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2596,9 +2596,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2623,9 +2623,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId3"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2650,9 +2650,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId4"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -21788,16 +21788,38 @@
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="58">
-      <c r="B14" s="28" t="n"/>
-      <c r="C14" s="29" t="n"/>
-      <c r="D14" s="29" t="n"/>
-      <c r="E14" s="29" t="n"/>
-      <c r="F14" s="30" t="n"/>
-      <c r="G14" s="29" t="n"/>
-      <c r="H14" s="29" t="n"/>
-      <c r="I14" s="29" t="n"/>
-      <c r="J14" s="31" t="n"/>
-      <c r="K14" s="32" t="n"/>
+      <c r="B14" s="28" t="n">
+        <v>46183</v>
+      </c>
+      <c r="C14" s="29" t="n">
+        <v>25569671</v>
+      </c>
+      <c r="D14" s="29" t="n">
+        <v>22685359</v>
+      </c>
+      <c r="E14" s="29" t="n">
+        <v>2884312</v>
+      </c>
+      <c r="F14" s="30" t="n">
+        <v>0.1271</v>
+      </c>
+      <c r="G14" s="29" t="n">
+        <v>18067456</v>
+      </c>
+      <c r="H14" s="29" t="n">
+        <v>4972541</v>
+      </c>
+      <c r="I14" s="29" t="n">
+        <v>1139248</v>
+      </c>
+      <c r="J14" s="31" t="n">
+        <v>32.92</v>
+      </c>
+      <c r="K14" s="32" t="inlineStr">
+        <is>
+          <t>Auto weekly snapshot</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="58">
       <c r="B15" s="28" t="n"/>
@@ -23511,7 +23533,7 @@
         </is>
       </c>
       <c r="C5" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="D5" s="64" t="inlineStr">
         <is>
@@ -23526,11 +23548,11 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>32.82</v>
+        <v>32.92</v>
       </c>
       <c r="D6" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-06-09</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-06-10</t>
         </is>
       </c>
     </row>
@@ -23575,11 +23597,11 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>25.5494</v>
+        <v>25.5831</v>
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-06-09</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-06-10</t>
         </is>
       </c>
     </row>
@@ -25187,7 +25209,7 @@
         </is>
       </c>
       <c r="G38" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H38" s="34" t="inlineStr">
         <is>
@@ -25227,7 +25249,7 @@
         </is>
       </c>
       <c r="G39" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H39" s="34" t="inlineStr">
         <is>
@@ -25267,7 +25289,7 @@
         </is>
       </c>
       <c r="G40" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H40" s="34" t="inlineStr">
         <is>
@@ -25307,7 +25329,7 @@
         </is>
       </c>
       <c r="G41" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H41" s="34" t="inlineStr">
         <is>
@@ -25347,7 +25369,7 @@
         </is>
       </c>
       <c r="G42" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H42" s="34" t="inlineStr">
         <is>
@@ -25387,7 +25409,7 @@
         </is>
       </c>
       <c r="G43" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H43" s="34" t="inlineStr">
         <is>
@@ -25427,7 +25449,7 @@
         </is>
       </c>
       <c r="G44" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H44" s="34" t="inlineStr">
         <is>
@@ -25467,7 +25489,7 @@
         </is>
       </c>
       <c r="G45" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H45" s="34" t="inlineStr">
         <is>
@@ -25507,7 +25529,7 @@
         </is>
       </c>
       <c r="G46" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H46" s="34" t="inlineStr">
         <is>
@@ -25584,7 +25606,7 @@
         </is>
       </c>
       <c r="G48" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H48" s="34" t="inlineStr">
         <is>
@@ -25624,7 +25646,7 @@
         </is>
       </c>
       <c r="G49" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H49" s="34" t="inlineStr">
         <is>
@@ -25664,7 +25686,7 @@
         </is>
       </c>
       <c r="G50" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H50" s="34" t="inlineStr">
         <is>
@@ -25704,7 +25726,7 @@
         </is>
       </c>
       <c r="G51" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H51" s="34" t="inlineStr">
         <is>
@@ -25744,7 +25766,7 @@
         </is>
       </c>
       <c r="G52" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H52" s="34" t="inlineStr">
         <is>
@@ -25784,7 +25806,7 @@
         </is>
       </c>
       <c r="G53" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H53" s="34" t="inlineStr">
         <is>
@@ -25824,7 +25846,7 @@
         </is>
       </c>
       <c r="G54" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H54" s="34" t="inlineStr">
         <is>
@@ -25864,7 +25886,7 @@
         </is>
       </c>
       <c r="G55" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H55" s="34" t="inlineStr">
         <is>
@@ -25904,7 +25926,7 @@
         </is>
       </c>
       <c r="G56" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H56" s="34" t="inlineStr">
         <is>
@@ -25944,7 +25966,7 @@
         </is>
       </c>
       <c r="G57" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H57" s="34" t="inlineStr">
         <is>
@@ -25984,7 +26006,7 @@
         </is>
       </c>
       <c r="G58" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H58" s="34" t="inlineStr">
         <is>
@@ -26024,7 +26046,7 @@
         </is>
       </c>
       <c r="G59" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H59" s="34" t="inlineStr">
         <is>
@@ -26056,7 +26078,7 @@
         </is>
       </c>
       <c r="E60" s="33" t="n">
-        <v>154.76</v>
+        <v>164.57</v>
       </c>
       <c r="F60" s="34" t="inlineStr">
         <is>
@@ -26064,7 +26086,7 @@
         </is>
       </c>
       <c r="G60" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H60" s="34" t="inlineStr">
         <is>
@@ -26072,7 +26094,7 @@
         </is>
       </c>
       <c r="I60" t="n">
-        <v>154.759995</v>
+        <v>164.570007</v>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="58">
@@ -26096,7 +26118,7 @@
         </is>
       </c>
       <c r="E61" s="33" t="n">
-        <v>244.99</v>
+        <v>237.88</v>
       </c>
       <c r="F61" s="34" t="inlineStr">
         <is>
@@ -26104,7 +26126,7 @@
         </is>
       </c>
       <c r="G61" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H61" s="34" t="inlineStr">
         <is>
@@ -26112,7 +26134,7 @@
         </is>
       </c>
       <c r="I61" t="n">
-        <v>244.990005</v>
+        <v>237.880005</v>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="58">
@@ -26136,7 +26158,7 @@
         </is>
       </c>
       <c r="E62" s="33" t="n">
-        <v>492.17</v>
+        <v>499.21</v>
       </c>
       <c r="F62" s="34" t="inlineStr">
         <is>
@@ -26144,7 +26166,7 @@
         </is>
       </c>
       <c r="G62" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H62" s="34" t="inlineStr">
         <is>
@@ -26152,7 +26174,7 @@
         </is>
       </c>
       <c r="I62" t="n">
-        <v>492.170013</v>
+        <v>499.209991</v>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1" s="58">
@@ -26176,7 +26198,7 @@
         </is>
       </c>
       <c r="E63" s="33" t="n">
-        <v>165.66</v>
+        <v>164.07</v>
       </c>
       <c r="F63" s="34" t="inlineStr">
         <is>
@@ -26184,7 +26206,7 @@
         </is>
       </c>
       <c r="G63" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H63" s="34" t="inlineStr">
         <is>
@@ -26192,7 +26214,7 @@
         </is>
       </c>
       <c r="I63" t="n">
-        <v>165.660004</v>
+        <v>164.070007</v>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="58">
@@ -26216,7 +26238,7 @@
         </is>
       </c>
       <c r="E64" s="33" t="n">
-        <v>56.88</v>
+        <v>53.51</v>
       </c>
       <c r="F64" s="34" t="inlineStr">
         <is>
@@ -26224,7 +26246,7 @@
         </is>
       </c>
       <c r="G64" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H64" s="34" t="inlineStr">
         <is>
@@ -26232,7 +26254,7 @@
         </is>
       </c>
       <c r="I64" t="n">
-        <v>56.880001</v>
+        <v>53.509998</v>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1" s="58">
@@ -26256,7 +26278,7 @@
         </is>
       </c>
       <c r="E65" s="33" t="n">
-        <v>185.64</v>
+        <v>184.05</v>
       </c>
       <c r="F65" s="34" t="inlineStr">
         <is>
@@ -26264,7 +26286,7 @@
         </is>
       </c>
       <c r="G65" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H65" s="34" t="inlineStr">
         <is>
@@ -26272,7 +26294,7 @@
         </is>
       </c>
       <c r="I65" t="n">
-        <v>185.639999</v>
+        <v>184.050003</v>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1" s="58">
@@ -26296,7 +26318,7 @@
         </is>
       </c>
       <c r="E66" s="33" t="n">
-        <v>143.04</v>
+        <v>138.39</v>
       </c>
       <c r="F66" s="34" t="inlineStr">
         <is>
@@ -26304,7 +26326,7 @@
         </is>
       </c>
       <c r="G66" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H66" s="34" t="inlineStr">
         <is>
@@ -26312,7 +26334,7 @@
         </is>
       </c>
       <c r="I66" t="n">
-        <v>143.039993</v>
+        <v>138.389999</v>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1" s="58">
@@ -26336,7 +26358,7 @@
         </is>
       </c>
       <c r="E67" s="33" t="n">
-        <v>160.35</v>
+        <v>157.4</v>
       </c>
       <c r="F67" s="34" t="inlineStr">
         <is>
@@ -26344,7 +26366,7 @@
         </is>
       </c>
       <c r="G67" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H67" s="34" t="inlineStr">
         <is>
@@ -26352,7 +26374,7 @@
         </is>
       </c>
       <c r="I67" t="n">
-        <v>160.350006</v>
+        <v>157.399994</v>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1" s="58">
@@ -26376,7 +26398,7 @@
         </is>
       </c>
       <c r="E68" s="33" t="n">
-        <v>2108.06</v>
+        <v>2139.37</v>
       </c>
       <c r="F68" s="34" t="inlineStr">
         <is>
@@ -26384,7 +26406,7 @@
         </is>
       </c>
       <c r="G68" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H68" s="34" t="inlineStr">
         <is>
@@ -26392,7 +26414,7 @@
         </is>
       </c>
       <c r="I68" t="n">
-        <v>2108.060059</v>
+        <v>2139.370117</v>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="58">
@@ -26416,7 +26438,7 @@
         </is>
       </c>
       <c r="E69" s="33" t="n">
-        <v>1149.15</v>
+        <v>1144.68</v>
       </c>
       <c r="F69" s="34" t="inlineStr">
         <is>
@@ -26424,7 +26446,7 @@
         </is>
       </c>
       <c r="G69" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H69" s="34" t="inlineStr">
         <is>
@@ -26432,7 +26454,7 @@
         </is>
       </c>
       <c r="I69" t="n">
-        <v>1149.150024</v>
+        <v>1144.680054</v>
       </c>
     </row>
     <row r="70" ht="15" customHeight="1" s="58">
@@ -26456,7 +26478,7 @@
         </is>
       </c>
       <c r="E70" s="33" t="n">
-        <v>91.37</v>
+        <v>91.47</v>
       </c>
       <c r="F70" s="34" t="inlineStr">
         <is>
@@ -26464,7 +26486,7 @@
         </is>
       </c>
       <c r="G70" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H70" s="34" t="inlineStr">
         <is>
@@ -26472,7 +26494,7 @@
         </is>
       </c>
       <c r="I70" t="n">
-        <v>91.370003</v>
+        <v>91.470001</v>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1" s="58">
@@ -26496,7 +26518,7 @@
         </is>
       </c>
       <c r="E71" s="33" t="n">
-        <v>1559.18</v>
+        <v>1531.98</v>
       </c>
       <c r="F71" s="34" t="inlineStr">
         <is>
@@ -26504,7 +26526,7 @@
         </is>
       </c>
       <c r="G71" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H71" s="34" t="inlineStr">
         <is>
@@ -26512,7 +26534,7 @@
         </is>
       </c>
       <c r="I71" t="n">
-        <v>1559.180054</v>
+        <v>1531.97998</v>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1" s="58">
@@ -26536,7 +26558,7 @@
         </is>
       </c>
       <c r="E72" s="33" t="n">
-        <v>110.14</v>
+        <v>109.8</v>
       </c>
       <c r="F72" s="34" t="inlineStr">
         <is>
@@ -26544,7 +26566,7 @@
         </is>
       </c>
       <c r="G72" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H72" s="34" t="inlineStr">
         <is>
@@ -26552,7 +26574,7 @@
         </is>
       </c>
       <c r="I72" t="n">
-        <v>110.139999</v>
+        <v>109.800003</v>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1" s="58">
@@ -26576,7 +26598,7 @@
         </is>
       </c>
       <c r="E73" s="33" t="n">
-        <v>208.64</v>
+        <v>208.19</v>
       </c>
       <c r="F73" s="34" t="inlineStr">
         <is>
@@ -26584,7 +26606,7 @@
         </is>
       </c>
       <c r="G73" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H73" s="34" t="inlineStr">
         <is>
@@ -26592,7 +26614,7 @@
         </is>
       </c>
       <c r="I73" t="n">
-        <v>208.639999</v>
+        <v>208.190002</v>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1" s="58">
@@ -26616,7 +26638,7 @@
         </is>
       </c>
       <c r="E74" s="33" t="n">
-        <v>88.81999999999999</v>
+        <v>89.31999999999999</v>
       </c>
       <c r="F74" s="34" t="inlineStr">
         <is>
@@ -26624,7 +26646,7 @@
         </is>
       </c>
       <c r="G74" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H74" s="34" t="inlineStr">
         <is>
@@ -26632,7 +26654,7 @@
         </is>
       </c>
       <c r="I74" t="n">
-        <v>88.81999999999999</v>
+        <v>89.31999999999999</v>
       </c>
     </row>
     <row r="75" ht="15" customHeight="1" s="58">
@@ -26656,7 +26678,7 @@
         </is>
       </c>
       <c r="E75" s="33" t="n">
-        <v>99.89</v>
+        <v>97.94</v>
       </c>
       <c r="F75" s="34" t="inlineStr">
         <is>
@@ -26664,7 +26686,7 @@
         </is>
       </c>
       <c r="G75" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H75" s="34" t="inlineStr">
         <is>
@@ -26672,7 +26694,7 @@
         </is>
       </c>
       <c r="I75" t="n">
-        <v>99.889999</v>
+        <v>97.94000200000001</v>
       </c>
     </row>
     <row r="76" ht="15" customHeight="1" s="58">
@@ -26696,7 +26718,7 @@
         </is>
       </c>
       <c r="E76" s="33" t="n">
-        <v>374.69</v>
+        <v>369.21</v>
       </c>
       <c r="F76" s="34" t="inlineStr">
         <is>
@@ -26704,7 +26726,7 @@
         </is>
       </c>
       <c r="G76" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H76" s="34" t="inlineStr">
         <is>
@@ -26712,7 +26734,7 @@
         </is>
       </c>
       <c r="I76" t="n">
-        <v>374.690002</v>
+        <v>369.209991</v>
       </c>
     </row>
     <row r="77" ht="15" customHeight="1" s="58">
@@ -26736,7 +26758,7 @@
         </is>
       </c>
       <c r="E77" s="33" t="n">
-        <v>408.95</v>
+        <v>396.68</v>
       </c>
       <c r="F77" s="34" t="inlineStr">
         <is>
@@ -26744,7 +26766,7 @@
         </is>
       </c>
       <c r="G77" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H77" s="34" t="inlineStr">
         <is>
@@ -26752,7 +26774,7 @@
         </is>
       </c>
       <c r="I77" t="n">
-        <v>408.950012</v>
+        <v>396.679993</v>
       </c>
     </row>
     <row r="78" ht="15" customHeight="1" s="58">
@@ -26776,7 +26798,7 @@
         </is>
       </c>
       <c r="E78" s="33" t="n">
-        <v>54.98</v>
+        <v>53.19</v>
       </c>
       <c r="F78" s="34" t="inlineStr">
         <is>
@@ -26784,7 +26806,7 @@
         </is>
       </c>
       <c r="G78" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H78" s="34" t="inlineStr">
         <is>
@@ -26792,7 +26814,7 @@
         </is>
       </c>
       <c r="I78" t="n">
-        <v>54.98</v>
+        <v>53.189999</v>
       </c>
     </row>
     <row r="79" ht="15" customHeight="1" s="58">
@@ -26816,7 +26838,7 @@
         </is>
       </c>
       <c r="E79" s="33" t="n">
-        <v>87.42</v>
+        <v>88.03</v>
       </c>
       <c r="F79" s="34" t="inlineStr">
         <is>
@@ -26824,7 +26846,7 @@
         </is>
       </c>
       <c r="G79" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H79" s="34" t="inlineStr">
         <is>
@@ -26832,7 +26854,7 @@
         </is>
       </c>
       <c r="I79" t="n">
-        <v>87.41999800000001</v>
+        <v>88.029999</v>
       </c>
     </row>
     <row r="80" ht="15" customHeight="1" s="58">
@@ -26856,7 +26878,7 @@
         </is>
       </c>
       <c r="E80" s="33" t="n">
-        <v>301.54</v>
+        <v>290.55</v>
       </c>
       <c r="F80" s="34" t="inlineStr">
         <is>
@@ -26864,7 +26886,7 @@
         </is>
       </c>
       <c r="G80" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H80" s="34" t="inlineStr">
         <is>
@@ -26872,7 +26894,7 @@
         </is>
       </c>
       <c r="I80" t="n">
-        <v>301.540009</v>
+        <v>290.549988</v>
       </c>
     </row>
     <row r="81" ht="15" customHeight="1" s="58">
@@ -26896,7 +26918,7 @@
         </is>
       </c>
       <c r="E81" s="33" t="n">
-        <v>162.11</v>
+        <v>155.5</v>
       </c>
       <c r="F81" s="34" t="inlineStr">
         <is>
@@ -26904,7 +26926,7 @@
         </is>
       </c>
       <c r="G81" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H81" s="34" t="inlineStr">
         <is>
@@ -26936,7 +26958,7 @@
         </is>
       </c>
       <c r="E82" s="33" t="n">
-        <v>585.39</v>
+        <v>584.59</v>
       </c>
       <c r="F82" s="34" t="inlineStr">
         <is>
@@ -26944,7 +26966,7 @@
         </is>
       </c>
       <c r="G82" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H82" s="34" t="inlineStr">
         <is>
@@ -26952,7 +26974,7 @@
         </is>
       </c>
       <c r="I82" t="n">
-        <v>585.3900149999999</v>
+        <v>584.590027</v>
       </c>
     </row>
     <row r="83" ht="15" customHeight="1" s="58">
@@ -26976,7 +26998,7 @@
         </is>
       </c>
       <c r="E83" s="33" t="n">
-        <v>147.99</v>
+        <v>153.5</v>
       </c>
       <c r="F83" s="34" t="inlineStr">
         <is>
@@ -26984,7 +27006,7 @@
         </is>
       </c>
       <c r="G83" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H83" s="34" t="inlineStr">
         <is>
@@ -27016,7 +27038,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>62.45</v>
+        <v>62.35</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -27024,7 +27046,7 @@
         </is>
       </c>
       <c r="G84" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H84" s="34" t="inlineStr">
         <is>
@@ -27032,7 +27054,7 @@
         </is>
       </c>
       <c r="I84" t="n">
-        <v>63.949352</v>
+        <v>62.329354</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="58">
@@ -27056,7 +27078,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>597.78</v>
+        <v>592.63</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -27064,7 +27086,7 @@
         </is>
       </c>
       <c r="G85" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H85" s="34" t="inlineStr">
         <is>
@@ -27072,7 +27094,7 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>599.648747</v>
+        <v>597.762508</v>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="58">
@@ -27096,7 +27118,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>62699</v>
+        <v>61800</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -27104,7 +27126,7 @@
         </is>
       </c>
       <c r="G86" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H86" s="34" t="inlineStr">
         <is>
@@ -27112,7 +27134,7 @@
         </is>
       </c>
       <c r="I86" t="n">
-        <v>63013.341652</v>
+        <v>62789.444621</v>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="58">
@@ -27136,7 +27158,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.00676</v>
+        <v>0.006775</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -27144,7 +27166,7 @@
         </is>
       </c>
       <c r="G87" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H87" s="34" t="inlineStr">
         <is>
@@ -27152,7 +27174,7 @@
         </is>
       </c>
       <c r="I87" t="n">
-        <v>0.006891</v>
+        <v>0.006634</v>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="58">
@@ -27176,7 +27198,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.011164</v>
+        <v>0.010668</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -27184,7 +27206,7 @@
         </is>
       </c>
       <c r="G88" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H88" s="34" t="inlineStr">
         <is>
@@ -27192,7 +27214,7 @@
         </is>
       </c>
       <c r="I88" t="n">
-        <v>0.011091</v>
+        <v>0.011288</v>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="58">
@@ -27216,7 +27238,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>66.28</v>
+        <v>65.16</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -27224,7 +27246,7 @@
         </is>
       </c>
       <c r="G89" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H89" s="34" t="inlineStr">
         <is>
@@ -27232,7 +27254,7 @@
         </is>
       </c>
       <c r="I89" t="n">
-        <v>66.30426</v>
+        <v>65.863608</v>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="58">
@@ -27256,7 +27278,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>1.67</v>
+        <v>1.66</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -27264,7 +27286,7 @@
         </is>
       </c>
       <c r="G90" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H90" s="34" t="inlineStr">
         <is>
@@ -27272,7 +27294,7 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>1.679132</v>
+        <v>1.65999</v>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="58">
@@ -27304,7 +27326,7 @@
         </is>
       </c>
       <c r="G91" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H91" s="34" t="inlineStr">
         <is>
@@ -27336,7 +27358,7 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
-        <v>0.013957</v>
+        <v>0.013958</v>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
@@ -27344,7 +27366,7 @@
         </is>
       </c>
       <c r="G92" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H92" s="34" t="inlineStr">
         <is>
@@ -27352,7 +27374,7 @@
         </is>
       </c>
       <c r="I92" t="n">
-        <v>0.013481</v>
+        <v>0.013586</v>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="58">
@@ -27376,7 +27398,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>2.647294</v>
+        <v>2.66675</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -27384,7 +27406,7 @@
         </is>
       </c>
       <c r="G93" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H93" s="34" t="inlineStr">
         <is>
@@ -27392,7 +27414,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>2.72702</v>
+        <v>2.656061</v>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="58">
@@ -27416,7 +27438,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>24.851731</v>
+        <v>24.839161</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -27424,7 +27446,7 @@
         </is>
       </c>
       <c r="G94" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H94" s="34" t="inlineStr">
         <is>
@@ -27432,7 +27454,7 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>24.825418</v>
+        <v>24.417084</v>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="58">
@@ -27456,7 +27478,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.112821</v>
+        <v>0.110648</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -27464,7 +27486,7 @@
         </is>
       </c>
       <c r="G95" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H95" s="34" t="inlineStr">
         <is>
@@ -27472,7 +27494,7 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>0.112643</v>
+        <v>0.110792</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="58">
@@ -27496,7 +27518,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>19619.1396</v>
+        <v>19509.3796</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -27504,7 +27526,7 @@
         </is>
       </c>
       <c r="G96" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H96" s="34" t="inlineStr">
         <is>
@@ -27512,7 +27534,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>19680.471886</v>
+        <v>19678.341771</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="58">
@@ -27536,7 +27558,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2057781.18</v>
+        <v>2034456</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -27544,7 +27566,7 @@
         </is>
       </c>
       <c r="G97" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H97" s="34" t="inlineStr">
         <is>
@@ -27552,7 +27574,7 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>2068097.873032</v>
+        <v>2067028.516916</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="58">
@@ -27576,7 +27598,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>2.811657</v>
+        <v>2.792571</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -27584,7 +27606,7 @@
         </is>
       </c>
       <c r="G98" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H98" s="34" t="inlineStr">
         <is>
@@ -27592,7 +27614,7 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>2.827604</v>
+        <v>2.803584</v>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="58">
@@ -27616,7 +27638,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>55053.5808</v>
+        <v>54024.0244</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -27624,7 +27646,7 @@
         </is>
       </c>
       <c r="G99" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H99" s="34" t="inlineStr">
         <is>
@@ -27632,7 +27654,7 @@
         </is>
       </c>
       <c r="I99" t="n">
-        <v>55022.018108</v>
+        <v>54980.911477</v>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="58">
@@ -27656,7 +27678,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>25.330968</v>
+        <v>25.108578</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -27664,7 +27686,7 @@
         </is>
       </c>
       <c r="G100" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H100" s="34" t="inlineStr">
         <is>
@@ -27672,7 +27694,7 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>25.238416</v>
+        <v>25.512299</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="58">
@@ -27696,7 +27718,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>62699</v>
+        <v>61800</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -27704,7 +27726,7 @@
         </is>
       </c>
       <c r="G101" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H101" s="34" t="inlineStr">
         <is>
@@ -27712,7 +27734,7 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>63013.341652</v>
+        <v>62789.444621</v>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="58">
@@ -27736,7 +27758,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>18.04</v>
+        <v>18.87</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -27744,7 +27766,7 @@
         </is>
       </c>
       <c r="G102" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H102" s="34" t="inlineStr">
         <is>
@@ -27752,7 +27774,7 @@
         </is>
       </c>
       <c r="I102" t="n">
-        <v>16.937123</v>
+        <v>18.148664</v>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="58">
@@ -27850,7 +27872,7 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
-        <v>0.00676</v>
+        <v>0.006775</v>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
@@ -27858,7 +27880,7 @@
         </is>
       </c>
       <c r="G105" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H105" s="34" t="inlineStr">
         <is>
@@ -27866,7 +27888,7 @@
         </is>
       </c>
       <c r="I105" t="n">
-        <v>0.006891</v>
+        <v>0.006634</v>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="58">
@@ -27890,7 +27912,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>66.28</v>
+        <v>65.16</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>
@@ -27898,7 +27920,7 @@
         </is>
       </c>
       <c r="G106" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H106" s="34" t="inlineStr">
         <is>
@@ -27906,7 +27928,7 @@
         </is>
       </c>
       <c r="I106" t="n">
-        <v>66.30426</v>
+        <v>65.863608</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="58">
@@ -27938,7 +27960,7 @@
         </is>
       </c>
       <c r="G107" s="28" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="H107" s="34" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Weekly dashboard update — 2026-06-10
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-42660" yWindow="-540" windowWidth="32460" windowHeight="17180" tabRatio="500" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Realized" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Realized" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Prices" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Reference" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="AsOfDate">'FX &amp; Assumptions'!$C$5</definedName>
@@ -697,14 +697,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -726,8 +726,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -752,10 +752,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -764,10 +764,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4F81BD"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+              <a:ln w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -777,10 +777,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="C0504D"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -790,10 +790,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="9BBB59"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -803,10 +803,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="8064A2"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -816,10 +816,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4BACC6"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -829,10 +829,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="F79646"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -842,14 +842,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -875,14 +875,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -908,14 +908,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -941,14 +941,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -974,14 +974,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1007,14 +1007,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1038,16 +1038,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1142,16 +1142,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1172,10 +1172,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1187,14 +1187,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1216,8 +1216,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1242,10 +1242,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1254,10 +1254,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4672A8"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1267,10 +1267,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="AB4744"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1280,10 +1280,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="8AA64F"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1293,10 +1293,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="725990"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1306,10 +1306,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4299B0"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1319,10 +1319,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="DC853E"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1332,10 +1332,10 @@
             <idx val="6"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="93A9CE"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1345,10 +1345,10 @@
             <idx val="7"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="D09493"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1358,10 +1358,10 @@
             <idx val="8"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="B8CD97"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1371,14 +1371,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1405,14 +1405,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1439,14 +1439,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1473,14 +1473,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1507,14 +1507,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1541,14 +1541,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1575,14 +1575,14 @@
             <dLbl>
               <idx val="6"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1609,14 +1609,14 @@
             <dLbl>
               <idx val="7"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1643,14 +1643,14 @@
             <dLbl>
               <idx val="8"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1675,16 +1675,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1791,16 +1791,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1821,10 +1821,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1836,14 +1836,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1865,8 +1865,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1893,10 +1893,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1904,16 +1904,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2016,7 +2016,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2025,9 +2025,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2059,7 +2059,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2073,7 +2073,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2082,9 +2082,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2109,16 +2109,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2139,10 +2139,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2154,14 +2154,14 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -2183,8 +2183,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -2200,10 +2200,10 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2211,16 +2211,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2411,7 +2411,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2420,9 +2420,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2454,7 +2454,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2468,7 +2468,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2477,9 +2477,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2504,16 +2504,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2534,10 +2534,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2549,7 +2549,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>1</col>
@@ -2569,9 +2569,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2596,9 +2596,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+          <c:chart r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2623,9 +2623,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+          <c:chart r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2650,9 +2650,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+          <c:chart r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -21792,28 +21792,28 @@
         <v>46183</v>
       </c>
       <c r="C14" s="29" t="n">
-        <v>25569671</v>
+        <v>25855668</v>
       </c>
       <c r="D14" s="29" t="n">
-        <v>22685359</v>
+        <v>22680627</v>
       </c>
       <c r="E14" s="29" t="n">
-        <v>2884312</v>
+        <v>3175041</v>
       </c>
       <c r="F14" s="30" t="n">
-        <v>0.1271</v>
+        <v>0.14</v>
       </c>
       <c r="G14" s="29" t="n">
-        <v>18067456</v>
+        <v>18380456</v>
       </c>
       <c r="H14" s="29" t="n">
-        <v>4972541</v>
+        <v>4952801</v>
       </c>
       <c r="I14" s="29" t="n">
-        <v>1139248</v>
+        <v>1133148</v>
       </c>
       <c r="J14" s="31" t="n">
-        <v>32.92</v>
+        <v>32.88</v>
       </c>
       <c r="K14" s="32" t="inlineStr">
         <is>
@@ -23548,7 +23548,7 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>32.92</v>
+        <v>32.88</v>
       </c>
       <c r="D6" s="64" t="inlineStr">
         <is>
@@ -23597,7 +23597,7 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>25.5831</v>
+        <v>25.5617</v>
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
@@ -23716,27 +23716,27 @@
         </is>
       </c>
       <c r="E5" s="33" t="n">
+        <v>24.4495</v>
+      </c>
+      <c r="F5" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G5" s="28" t="n">
+        <v>46181</v>
+      </c>
+      <c r="H5" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
         <v>23.3473</v>
       </c>
-      <c r="F5" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G5" s="28" t="n">
-        <v>46178</v>
-      </c>
-      <c r="H5" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I5" t="n">
-        <v>26.0771</v>
-      </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
@@ -23761,27 +23761,27 @@
         </is>
       </c>
       <c r="E6" s="33" t="n">
+        <v>10.6868</v>
+      </c>
+      <c r="F6" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G6" s="28" t="n">
+        <v>46182</v>
+      </c>
+      <c r="H6" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
         <v>10.6865</v>
       </c>
-      <c r="F6" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G6" s="28" t="n">
-        <v>46181</v>
-      </c>
-      <c r="H6" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I6" t="n">
-        <v>10.6859</v>
-      </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
     </row>
@@ -23806,27 +23806,27 @@
         </is>
       </c>
       <c r="E7" s="33" t="n">
+        <v>7.0857</v>
+      </c>
+      <c r="F7" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G7" s="28" t="n">
+        <v>46181</v>
+      </c>
+      <c r="H7" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
         <v>7.1091</v>
       </c>
-      <c r="F7" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G7" s="28" t="n">
-        <v>46178</v>
-      </c>
-      <c r="H7" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I7" t="n">
-        <v>7.1186</v>
-      </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
@@ -23851,27 +23851,27 @@
         </is>
       </c>
       <c r="E8" s="33" t="n">
+        <v>9.2986</v>
+      </c>
+      <c r="F8" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G8" s="28" t="n">
+        <v>46181</v>
+      </c>
+      <c r="H8" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
         <v>9.393700000000001</v>
       </c>
-      <c r="F8" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G8" s="28" t="n">
-        <v>46178</v>
-      </c>
-      <c r="H8" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I8" t="n">
-        <v>9.7468</v>
-      </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
@@ -23896,27 +23896,27 @@
         </is>
       </c>
       <c r="E9" s="33" t="n">
+        <v>9.2889</v>
+      </c>
+      <c r="F9" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G9" s="28" t="n">
+        <v>46182</v>
+      </c>
+      <c r="H9" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
         <v>9.1631</v>
       </c>
-      <c r="F9" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G9" s="28" t="n">
-        <v>46181</v>
-      </c>
-      <c r="H9" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I9" t="n">
-        <v>9.320600000000001</v>
-      </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
     </row>
@@ -23941,27 +23941,27 @@
         </is>
       </c>
       <c r="E10" s="33" t="n">
+        <v>13.0438</v>
+      </c>
+      <c r="F10" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G10" s="28" t="n">
+        <v>46181</v>
+      </c>
+      <c r="H10" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
         <v>13.5827</v>
       </c>
-      <c r="F10" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G10" s="28" t="n">
-        <v>46178</v>
-      </c>
-      <c r="H10" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I10" t="n">
-        <v>13.6486</v>
-      </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
@@ -23986,27 +23986,27 @@
         </is>
       </c>
       <c r="E11" s="33" t="n">
+        <v>13.1546</v>
+      </c>
+      <c r="F11" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G11" s="28" t="n">
+        <v>46182</v>
+      </c>
+      <c r="H11" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
         <v>12.9039</v>
       </c>
-      <c r="F11" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G11" s="28" t="n">
-        <v>46181</v>
-      </c>
-      <c r="H11" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I11" t="n">
-        <v>13.2022</v>
-      </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
     </row>
@@ -24031,27 +24031,27 @@
         </is>
       </c>
       <c r="E12" s="33" t="n">
+        <v>26.6235</v>
+      </c>
+      <c r="F12" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G12" s="28" t="n">
+        <v>46182</v>
+      </c>
+      <c r="H12" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
         <v>26.0378</v>
       </c>
-      <c r="F12" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G12" s="28" t="n">
-        <v>46181</v>
-      </c>
-      <c r="H12" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I12" t="n">
-        <v>26.689</v>
-      </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
     </row>
@@ -24076,27 +24076,27 @@
         </is>
       </c>
       <c r="E13" s="33" t="n">
+        <v>36.2939</v>
+      </c>
+      <c r="F13" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G13" s="28" t="n">
+        <v>46182</v>
+      </c>
+      <c r="H13" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
         <v>35.7675</v>
       </c>
-      <c r="F13" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G13" s="28" t="n">
-        <v>46181</v>
-      </c>
-      <c r="H13" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I13" t="n">
-        <v>36.2424</v>
-      </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
     </row>
@@ -24121,27 +24121,27 @@
         </is>
       </c>
       <c r="E14" s="33" t="n">
+        <v>25.3708</v>
+      </c>
+      <c r="F14" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G14" s="28" t="n">
+        <v>46182</v>
+      </c>
+      <c r="H14" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
         <v>25.2435</v>
       </c>
-      <c r="F14" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G14" s="28" t="n">
-        <v>46181</v>
-      </c>
-      <c r="H14" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I14" t="n">
-        <v>25.4991</v>
-      </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
     </row>
@@ -24166,27 +24166,27 @@
         </is>
       </c>
       <c r="E15" s="33" t="n">
+        <v>14.8466</v>
+      </c>
+      <c r="F15" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G15" s="28" t="n">
+        <v>46178</v>
+      </c>
+      <c r="H15" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
         <v>14.8572</v>
       </c>
-      <c r="F15" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G15" s="28" t="n">
-        <v>46177</v>
-      </c>
-      <c r="H15" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I15" t="n">
-        <v>14.3709</v>
-      </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
@@ -24211,27 +24211,27 @@
         </is>
       </c>
       <c r="E16" s="33" t="n">
+        <v>81.4269</v>
+      </c>
+      <c r="F16" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G16" s="28" t="n">
+        <v>46182</v>
+      </c>
+      <c r="H16" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
         <v>80.3703</v>
       </c>
-      <c r="F16" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G16" s="28" t="n">
-        <v>46181</v>
-      </c>
-      <c r="H16" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I16" t="n">
-        <v>81.4024</v>
-      </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
     </row>
@@ -24256,27 +24256,27 @@
         </is>
       </c>
       <c r="E17" s="33" t="n">
+        <v>53.1377</v>
+      </c>
+      <c r="F17" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G17" s="28" t="n">
+        <v>46182</v>
+      </c>
+      <c r="H17" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
         <v>52.898</v>
       </c>
-      <c r="F17" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G17" s="28" t="n">
-        <v>46181</v>
-      </c>
-      <c r="H17" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I17" t="n">
-        <v>53.4695</v>
-      </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
     </row>
@@ -24301,27 +24301,27 @@
         </is>
       </c>
       <c r="E18" s="33" t="n">
+        <v>16.4125</v>
+      </c>
+      <c r="F18" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G18" s="28" t="n">
+        <v>46182</v>
+      </c>
+      <c r="H18" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
         <v>16.4116</v>
       </c>
-      <c r="F18" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G18" s="28" t="n">
-        <v>46181</v>
-      </c>
-      <c r="H18" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I18" t="n">
-        <v>16.4291</v>
-      </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
     </row>
@@ -24346,27 +24346,27 @@
         </is>
       </c>
       <c r="E19" s="33" t="n">
+        <v>23.4031</v>
+      </c>
+      <c r="F19" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G19" s="28" t="n">
+        <v>46182</v>
+      </c>
+      <c r="H19" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
         <v>23.4026</v>
       </c>
-      <c r="F19" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G19" s="28" t="n">
-        <v>46181</v>
-      </c>
-      <c r="H19" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I19" t="n">
-        <v>23.4013</v>
-      </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
     </row>
@@ -24391,27 +24391,27 @@
         </is>
       </c>
       <c r="E20" s="33" t="n">
+        <v>40.6754</v>
+      </c>
+      <c r="F20" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G20" s="28" t="n">
+        <v>46181</v>
+      </c>
+      <c r="H20" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
         <v>40.5739</v>
       </c>
-      <c r="F20" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G20" s="28" t="n">
-        <v>46178</v>
-      </c>
-      <c r="H20" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I20" t="n">
-        <v>41.6601</v>
-      </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
@@ -24436,27 +24436,27 @@
         </is>
       </c>
       <c r="E21" s="33" t="n">
+        <v>13.3598</v>
+      </c>
+      <c r="F21" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G21" s="28" t="n">
+        <v>46182</v>
+      </c>
+      <c r="H21" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
         <v>13.241</v>
       </c>
-      <c r="F21" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G21" s="28" t="n">
-        <v>46181</v>
-      </c>
-      <c r="H21" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I21" t="n">
-        <v>13.3947</v>
-      </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
     </row>
@@ -24481,27 +24481,27 @@
         </is>
       </c>
       <c r="E22" s="33" t="n">
+        <v>13.215</v>
+      </c>
+      <c r="F22" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G22" s="28" t="n">
+        <v>46181</v>
+      </c>
+      <c r="H22" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
         <v>13.2668</v>
       </c>
-      <c r="F22" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G22" s="28" t="n">
-        <v>46178</v>
-      </c>
-      <c r="H22" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I22" t="n">
-        <v>13.1535</v>
-      </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
@@ -24526,27 +24526,27 @@
         </is>
       </c>
       <c r="E23" s="33" t="n">
+        <v>12.3772</v>
+      </c>
+      <c r="F23" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G23" s="28" t="n">
+        <v>46182</v>
+      </c>
+      <c r="H23" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
         <v>12.3035</v>
       </c>
-      <c r="F23" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G23" s="28" t="n">
-        <v>46181</v>
-      </c>
-      <c r="H23" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I23" t="n">
-        <v>12.4665</v>
-      </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
     </row>
@@ -24571,27 +24571,27 @@
         </is>
       </c>
       <c r="E24" s="33" t="n">
+        <v>11.827</v>
+      </c>
+      <c r="F24" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G24" s="28" t="n">
+        <v>46181</v>
+      </c>
+      <c r="H24" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
         <v>11.9931</v>
       </c>
-      <c r="F24" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G24" s="28" t="n">
-        <v>46178</v>
-      </c>
-      <c r="H24" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I24" t="n">
-        <v>12.0868</v>
-      </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
@@ -24616,27 +24616,27 @@
         </is>
       </c>
       <c r="E25" s="33" t="n">
+        <v>9.9245</v>
+      </c>
+      <c r="F25" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G25" s="28" t="n">
+        <v>46182</v>
+      </c>
+      <c r="H25" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
         <v>9.8523</v>
       </c>
-      <c r="F25" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G25" s="28" t="n">
-        <v>46181</v>
-      </c>
-      <c r="H25" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I25" t="n">
-        <v>10.0147</v>
-      </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
     </row>
@@ -24661,27 +24661,27 @@
         </is>
       </c>
       <c r="E26" s="33" t="n">
+        <v>13.9301</v>
+      </c>
+      <c r="F26" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G26" s="28" t="n">
+        <v>46182</v>
+      </c>
+      <c r="H26" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
         <v>13.8268</v>
       </c>
-      <c r="F26" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G26" s="28" t="n">
-        <v>46181</v>
-      </c>
-      <c r="H26" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I26" t="n">
-        <v>14.0583</v>
-      </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
     </row>
@@ -24706,27 +24706,27 @@
         </is>
       </c>
       <c r="E27" s="33" t="n">
+        <v>16.8932</v>
+      </c>
+      <c r="F27" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G27" s="28" t="n">
+        <v>46182</v>
+      </c>
+      <c r="H27" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
         <v>16.8474</v>
       </c>
-      <c r="F27" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G27" s="28" t="n">
-        <v>46181</v>
-      </c>
-      <c r="H27" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I27" t="n">
-        <v>17.105</v>
-      </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
     </row>
@@ -24751,27 +24751,27 @@
         </is>
       </c>
       <c r="E28" s="33" t="n">
+        <v>19.2336</v>
+      </c>
+      <c r="F28" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G28" s="28" t="n">
+        <v>46182</v>
+      </c>
+      <c r="H28" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
         <v>19.1156</v>
       </c>
-      <c r="F28" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G28" s="28" t="n">
-        <v>46181</v>
-      </c>
-      <c r="H28" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I28" t="n">
-        <v>19.8791</v>
-      </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
     </row>
@@ -24796,27 +24796,27 @@
         </is>
       </c>
       <c r="E29" s="33" t="n">
+        <v>25.2898</v>
+      </c>
+      <c r="F29" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G29" s="28" t="n">
+        <v>46181</v>
+      </c>
+      <c r="H29" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
         <v>23.8964</v>
       </c>
-      <c r="F29" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G29" s="28" t="n">
-        <v>46178</v>
-      </c>
-      <c r="H29" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I29" t="n">
-        <v>27.8357</v>
-      </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
@@ -24841,27 +24841,27 @@
         </is>
       </c>
       <c r="E30" s="33" t="n">
+        <v>37.4218</v>
+      </c>
+      <c r="F30" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G30" s="28" t="n">
+        <v>46181</v>
+      </c>
+      <c r="H30" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
         <v>36.6591</v>
       </c>
-      <c r="F30" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G30" s="28" t="n">
-        <v>46178</v>
-      </c>
-      <c r="H30" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I30" t="n">
-        <v>38.836</v>
-      </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
@@ -24886,27 +24886,27 @@
         </is>
       </c>
       <c r="E31" s="33" t="n">
+        <v>12.9477</v>
+      </c>
+      <c r="F31" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G31" s="28" t="n">
+        <v>46182</v>
+      </c>
+      <c r="H31" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
         <v>12.7623</v>
       </c>
-      <c r="F31" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G31" s="28" t="n">
-        <v>46181</v>
-      </c>
-      <c r="H31" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I31" t="n">
-        <v>12.9367</v>
-      </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
     </row>
@@ -24931,27 +24931,27 @@
         </is>
       </c>
       <c r="E32" s="33" t="n">
+        <v>21.7055</v>
+      </c>
+      <c r="F32" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G32" s="28" t="n">
+        <v>46182</v>
+      </c>
+      <c r="H32" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
         <v>21.7053</v>
       </c>
-      <c r="F32" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G32" s="28" t="n">
-        <v>46181</v>
-      </c>
-      <c r="H32" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I32" t="n">
-        <v>21.7047</v>
-      </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
     </row>
@@ -24976,27 +24976,27 @@
         </is>
       </c>
       <c r="E33" s="33" t="n">
+        <v>12.5043</v>
+      </c>
+      <c r="F33" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G33" s="28" t="n">
+        <v>46182</v>
+      </c>
+      <c r="H33" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
         <v>12.3354</v>
       </c>
-      <c r="F33" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G33" s="28" t="n">
-        <v>46181</v>
-      </c>
-      <c r="H33" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I33" t="n">
-        <v>12.5235</v>
-      </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
     </row>
@@ -25021,27 +25021,27 @@
         </is>
       </c>
       <c r="E34" s="33" t="n">
+        <v>16.2045</v>
+      </c>
+      <c r="F34" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G34" s="28" t="n">
+        <v>46182</v>
+      </c>
+      <c r="H34" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
         <v>16.2041</v>
       </c>
-      <c r="F34" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G34" s="28" t="n">
-        <v>46181</v>
-      </c>
-      <c r="H34" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I34" t="n">
-        <v>16.203</v>
-      </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
     </row>
@@ -25066,27 +25066,27 @@
         </is>
       </c>
       <c r="E35" s="33" t="n">
+        <v>28.1255</v>
+      </c>
+      <c r="F35" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G35" s="28" t="n">
+        <v>46181</v>
+      </c>
+      <c r="H35" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
         <v>27.8538</v>
       </c>
-      <c r="F35" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G35" s="28" t="n">
-        <v>46178</v>
-      </c>
-      <c r="H35" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I35" t="n">
-        <v>28.936</v>
-      </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
@@ -25111,27 +25111,27 @@
         </is>
       </c>
       <c r="E36" s="33" t="n">
+        <v>9.9649</v>
+      </c>
+      <c r="F36" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G36" s="28" t="n">
+        <v>46182</v>
+      </c>
+      <c r="H36" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
         <v>9.978999999999999</v>
       </c>
-      <c r="F36" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G36" s="28" t="n">
-        <v>46181</v>
-      </c>
-      <c r="H36" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I36" t="n">
-        <v>10.032</v>
-      </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
     </row>
@@ -25156,27 +25156,27 @@
         </is>
       </c>
       <c r="E37" s="33" t="n">
+        <v>22.5842</v>
+      </c>
+      <c r="F37" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G37" s="28" t="n">
+        <v>46182</v>
+      </c>
+      <c r="H37" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
         <v>22.348</v>
       </c>
-      <c r="F37" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G37" s="28" t="n">
-        <v>46181</v>
-      </c>
-      <c r="H37" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I37" t="n">
-        <v>22.6458</v>
-      </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
     </row>
@@ -25217,7 +25217,7 @@
         </is>
       </c>
       <c r="I38" t="n">
-        <v>22.799999</v>
+        <v>22.82</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="58">
@@ -25257,7 +25257,7 @@
         </is>
       </c>
       <c r="I39" t="n">
-        <v>1.106</v>
+        <v>1.076</v>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="58">
@@ -25297,7 +25297,7 @@
         </is>
       </c>
       <c r="I40" t="n">
-        <v>757.73999</v>
+        <v>772.830017</v>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="58">
@@ -25337,7 +25337,7 @@
         </is>
       </c>
       <c r="I41" t="n">
-        <v>20.200001</v>
+        <v>21.110001</v>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="58">
@@ -25377,7 +25377,7 @@
         </is>
       </c>
       <c r="I42" t="n">
-        <v>218.070007</v>
+        <v>218.100006</v>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="58">
@@ -25441,7 +25441,7 @@
         </is>
       </c>
       <c r="E44" s="33" t="n">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="F44" s="34" t="inlineStr">
         <is>
@@ -25457,7 +25457,7 @@
         </is>
       </c>
       <c r="I44" t="n">
-        <v>174.5</v>
+        <v>170</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="58">
@@ -25638,7 +25638,7 @@
         </is>
       </c>
       <c r="E49" s="33" t="n">
-        <v>63.75</v>
+        <v>63</v>
       </c>
       <c r="F49" s="34" t="inlineStr">
         <is>
@@ -25654,7 +25654,7 @@
         </is>
       </c>
       <c r="I49" t="n">
-        <v>64.5</v>
+        <v>63.75</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="58">
@@ -25678,7 +25678,7 @@
         </is>
       </c>
       <c r="E50" s="33" t="n">
-        <v>9.4</v>
+        <v>9.25</v>
       </c>
       <c r="F50" s="34" t="inlineStr">
         <is>
@@ -25758,7 +25758,7 @@
         </is>
       </c>
       <c r="E52" s="33" t="n">
-        <v>13.5</v>
+        <v>13.4</v>
       </c>
       <c r="F52" s="34" t="inlineStr">
         <is>
@@ -25774,7 +25774,7 @@
         </is>
       </c>
       <c r="I52" t="n">
-        <v>13.3</v>
+        <v>13.4</v>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1" s="58">
@@ -25798,7 +25798,7 @@
         </is>
       </c>
       <c r="E53" s="33" t="n">
-        <v>5.7</v>
+        <v>5.35</v>
       </c>
       <c r="F53" s="34" t="inlineStr">
         <is>
@@ -25814,7 +25814,7 @@
         </is>
       </c>
       <c r="I53" t="n">
-        <v>5.7</v>
+        <v>5.35</v>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="58">
@@ -25838,7 +25838,7 @@
         </is>
       </c>
       <c r="E54" s="33" t="n">
-        <v>20.7</v>
+        <v>20.1</v>
       </c>
       <c r="F54" s="34" t="inlineStr">
         <is>
@@ -25854,7 +25854,7 @@
         </is>
       </c>
       <c r="I54" t="n">
-        <v>20.700001</v>
+        <v>20.1</v>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="58">
@@ -25878,7 +25878,7 @@
         </is>
       </c>
       <c r="E55" s="33" t="n">
-        <v>3.52</v>
+        <v>3.5</v>
       </c>
       <c r="F55" s="34" t="inlineStr">
         <is>
@@ -25958,7 +25958,7 @@
         </is>
       </c>
       <c r="E57" s="33" t="n">
-        <v>2.58</v>
+        <v>2.54</v>
       </c>
       <c r="F57" s="34" t="inlineStr">
         <is>
@@ -25974,7 +25974,7 @@
         </is>
       </c>
       <c r="I57" t="n">
-        <v>2.58</v>
+        <v>2.54</v>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="58">
@@ -25998,7 +25998,7 @@
         </is>
       </c>
       <c r="E58" s="33" t="n">
-        <v>12.4</v>
+        <v>12.1</v>
       </c>
       <c r="F58" s="34" t="inlineStr">
         <is>
@@ -26014,7 +26014,7 @@
         </is>
       </c>
       <c r="I58" t="n">
-        <v>12.4</v>
+        <v>12.1</v>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="58">
@@ -26038,7 +26038,7 @@
         </is>
       </c>
       <c r="E59" s="33" t="n">
-        <v>16.8</v>
+        <v>16.6</v>
       </c>
       <c r="F59" s="34" t="inlineStr">
         <is>
@@ -26054,7 +26054,7 @@
         </is>
       </c>
       <c r="I59" t="n">
-        <v>16.799999</v>
+        <v>16.6</v>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1" s="58">
@@ -26094,7 +26094,7 @@
         </is>
       </c>
       <c r="I60" t="n">
-        <v>164.570007</v>
+        <v>154.759995</v>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="58">
@@ -26134,7 +26134,7 @@
         </is>
       </c>
       <c r="I61" t="n">
-        <v>237.880005</v>
+        <v>244.990005</v>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="58">
@@ -26174,7 +26174,7 @@
         </is>
       </c>
       <c r="I62" t="n">
-        <v>499.209991</v>
+        <v>492.170013</v>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1" s="58">
@@ -26214,7 +26214,7 @@
         </is>
       </c>
       <c r="I63" t="n">
-        <v>164.070007</v>
+        <v>165.660004</v>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="58">
@@ -26254,7 +26254,7 @@
         </is>
       </c>
       <c r="I64" t="n">
-        <v>53.509998</v>
+        <v>56.880001</v>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1" s="58">
@@ -26294,7 +26294,7 @@
         </is>
       </c>
       <c r="I65" t="n">
-        <v>184.050003</v>
+        <v>185.639999</v>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1" s="58">
@@ -26334,7 +26334,7 @@
         </is>
       </c>
       <c r="I66" t="n">
-        <v>138.389999</v>
+        <v>143.039993</v>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1" s="58">
@@ -26374,7 +26374,7 @@
         </is>
       </c>
       <c r="I67" t="n">
-        <v>157.399994</v>
+        <v>160.350006</v>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1" s="58">
@@ -26414,7 +26414,7 @@
         </is>
       </c>
       <c r="I68" t="n">
-        <v>2139.370117</v>
+        <v>2108.060059</v>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="58">
@@ -26454,7 +26454,7 @@
         </is>
       </c>
       <c r="I69" t="n">
-        <v>1144.680054</v>
+        <v>1149.150024</v>
       </c>
     </row>
     <row r="70" ht="15" customHeight="1" s="58">
@@ -26494,7 +26494,7 @@
         </is>
       </c>
       <c r="I70" t="n">
-        <v>91.470001</v>
+        <v>91.370003</v>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1" s="58">
@@ -26534,7 +26534,7 @@
         </is>
       </c>
       <c r="I71" t="n">
-        <v>1531.97998</v>
+        <v>1559.180054</v>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1" s="58">
@@ -26574,7 +26574,7 @@
         </is>
       </c>
       <c r="I72" t="n">
-        <v>109.800003</v>
+        <v>110.139999</v>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1" s="58">
@@ -26614,7 +26614,7 @@
         </is>
       </c>
       <c r="I73" t="n">
-        <v>208.190002</v>
+        <v>208.639999</v>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1" s="58">
@@ -26654,7 +26654,7 @@
         </is>
       </c>
       <c r="I74" t="n">
-        <v>89.31999999999999</v>
+        <v>88.81999999999999</v>
       </c>
     </row>
     <row r="75" ht="15" customHeight="1" s="58">
@@ -26694,7 +26694,7 @@
         </is>
       </c>
       <c r="I75" t="n">
-        <v>97.94000200000001</v>
+        <v>99.889999</v>
       </c>
     </row>
     <row r="76" ht="15" customHeight="1" s="58">
@@ -26734,7 +26734,7 @@
         </is>
       </c>
       <c r="I76" t="n">
-        <v>369.209991</v>
+        <v>374.690002</v>
       </c>
     </row>
     <row r="77" ht="15" customHeight="1" s="58">
@@ -26774,7 +26774,7 @@
         </is>
       </c>
       <c r="I77" t="n">
-        <v>396.679993</v>
+        <v>408.950012</v>
       </c>
     </row>
     <row r="78" ht="15" customHeight="1" s="58">
@@ -26814,7 +26814,7 @@
         </is>
       </c>
       <c r="I78" t="n">
-        <v>53.189999</v>
+        <v>54.98</v>
       </c>
     </row>
     <row r="79" ht="15" customHeight="1" s="58">
@@ -26854,7 +26854,7 @@
         </is>
       </c>
       <c r="I79" t="n">
-        <v>88.029999</v>
+        <v>87.41999800000001</v>
       </c>
     </row>
     <row r="80" ht="15" customHeight="1" s="58">
@@ -26894,7 +26894,7 @@
         </is>
       </c>
       <c r="I80" t="n">
-        <v>290.549988</v>
+        <v>301.540009</v>
       </c>
     </row>
     <row r="81" ht="15" customHeight="1" s="58">
@@ -26974,7 +26974,7 @@
         </is>
       </c>
       <c r="I82" t="n">
-        <v>584.590027</v>
+        <v>585.3900149999999</v>
       </c>
     </row>
     <row r="83" ht="15" customHeight="1" s="58">
@@ -27038,7 +27038,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>62.35</v>
+        <v>61.83</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -27054,7 +27054,7 @@
         </is>
       </c>
       <c r="I84" t="n">
-        <v>62.329354</v>
+        <v>62.321831</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="58">
@@ -27078,7 +27078,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>592.63</v>
+        <v>589</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -27094,7 +27094,7 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>597.762508</v>
+        <v>596.983376</v>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="58">
@@ -27118,7 +27118,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>61800</v>
+        <v>61645</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -27134,7 +27134,7 @@
         </is>
       </c>
       <c r="I86" t="n">
-        <v>62789.444621</v>
+        <v>62538.72489</v>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="58">
@@ -27158,7 +27158,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.006775</v>
+        <v>0.006677</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -27174,7 +27174,7 @@
         </is>
       </c>
       <c r="I87" t="n">
-        <v>0.006634</v>
+        <v>0.006752</v>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="58">
@@ -27198,7 +27198,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.010668</v>
+        <v>0.010176</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -27214,7 +27214,7 @@
         </is>
       </c>
       <c r="I88" t="n">
-        <v>0.011288</v>
+        <v>0.01115</v>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="58">
@@ -27238,7 +27238,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>65.16</v>
+        <v>64.27</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -27254,7 +27254,7 @@
         </is>
       </c>
       <c r="I89" t="n">
-        <v>65.863608</v>
+        <v>66.029038</v>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="58">
@@ -27278,7 +27278,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>1.66</v>
+        <v>1.65</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -27294,7 +27294,7 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>1.65999</v>
+        <v>1.669154</v>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="58">
@@ -27358,7 +27358,7 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
-        <v>0.013958</v>
+        <v>0.013447</v>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
@@ -27374,7 +27374,7 @@
         </is>
       </c>
       <c r="I92" t="n">
-        <v>0.013586</v>
+        <v>0.014016</v>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="58">
@@ -27398,7 +27398,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>2.66675</v>
+        <v>2.613039</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -27414,7 +27414,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>2.656061</v>
+        <v>2.645742</v>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="58">
@@ -27438,7 +27438,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>24.839161</v>
+        <v>24.618407</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -27454,7 +27454,7 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>24.417084</v>
+        <v>24.78948</v>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="58">
@@ -27478,7 +27478,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.110648</v>
+        <v>0.109527</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -27494,7 +27494,7 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>0.110792</v>
+        <v>0.112555</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="58">
@@ -27518,7 +27518,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>19509.3796</v>
+        <v>19366.32</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -27534,7 +27534,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>19678.341771</v>
+        <v>19628.813399</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="58">
@@ -27558,7 +27558,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2034456</v>
+        <v>2026887.6</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -27574,7 +27574,7 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>2067028.516916</v>
+        <v>2056273.274367</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="58">
@@ -27598,7 +27598,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>2.792571</v>
+        <v>2.760013</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -27614,7 +27614,7 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>2.803584</v>
+        <v>2.81425</v>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="58">
@@ -27638,7 +27638,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>54024.0244</v>
+        <v>53851.1928</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -27654,7 +27654,7 @@
         </is>
       </c>
       <c r="I99" t="n">
-        <v>54980.911477</v>
+        <v>55041.450241</v>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="58">
@@ -27678,7 +27678,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>25.108578</v>
+        <v>24.657764</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -27694,7 +27694,7 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>25.512299</v>
+        <v>25.346541</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="58">
@@ -27718,7 +27718,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>61800</v>
+        <v>61645</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -27734,7 +27734,7 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>62789.444621</v>
+        <v>62538.72489</v>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="58">
@@ -27758,7 +27758,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>18.87</v>
+        <v>18.12</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -27774,7 +27774,7 @@
         </is>
       </c>
       <c r="I102" t="n">
-        <v>18.148664</v>
+        <v>18.003893</v>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="58">
@@ -27872,7 +27872,7 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
-        <v>0.006775</v>
+        <v>0.006677</v>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
@@ -27888,7 +27888,7 @@
         </is>
       </c>
       <c r="I105" t="n">
-        <v>0.006634</v>
+        <v>0.006752</v>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="58">
@@ -27912,7 +27912,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>65.16</v>
+        <v>64.27</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>
@@ -27928,7 +27928,7 @@
         </is>
       </c>
       <c r="I106" t="n">
-        <v>65.863608</v>
+        <v>66.029038</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="58">

</xml_diff>

<commit_message>
Daily dashboard update — 2026-06-11
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-42660" yWindow="-540" windowWidth="32460" windowHeight="17180" tabRatio="500" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Realized" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Prices" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Reference" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Realized" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="AsOfDate">'FX &amp; Assumptions'!$C$5</definedName>
@@ -697,14 +697,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -726,8 +726,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -752,10 +752,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -764,10 +764,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4F81BD"/>
               </a:solidFill>
-              <a:ln w="0">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -777,10 +777,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="C0504D"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -790,10 +790,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="9BBB59"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -803,10 +803,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="8064A2"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -816,10 +816,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4BACC6"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -829,10 +829,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="F79646"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -842,14 +842,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -875,14 +875,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -908,14 +908,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -941,14 +941,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -974,14 +974,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1007,14 +1007,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1038,16 +1038,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1142,16 +1142,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1172,10 +1172,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1187,14 +1187,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1216,8 +1216,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1242,10 +1242,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1254,10 +1254,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4672A8"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1267,10 +1267,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="AB4744"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1280,10 +1280,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="8AA64F"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1293,10 +1293,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="725990"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1306,10 +1306,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4299B0"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1319,10 +1319,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="DC853E"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1332,10 +1332,10 @@
             <idx val="6"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="93A9CE"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1345,10 +1345,10 @@
             <idx val="7"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="D09493"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1358,10 +1358,10 @@
             <idx val="8"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="B8CD97"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1371,14 +1371,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1405,14 +1405,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1439,14 +1439,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1473,14 +1473,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1507,14 +1507,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1541,14 +1541,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1575,14 +1575,14 @@
             <dLbl>
               <idx val="6"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1609,14 +1609,14 @@
             <dLbl>
               <idx val="7"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1643,14 +1643,14 @@
             <dLbl>
               <idx val="8"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1675,16 +1675,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1791,16 +1791,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1821,10 +1821,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1836,14 +1836,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1865,8 +1865,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1893,10 +1893,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1904,16 +1904,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2016,7 +2016,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2025,9 +2025,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2059,7 +2059,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="9360">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2073,7 +2073,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2082,9 +2082,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2109,16 +2109,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2139,10 +2139,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2154,14 +2154,14 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -2183,8 +2183,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -2200,10 +2200,10 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2211,16 +2211,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2411,7 +2411,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2420,9 +2420,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2454,7 +2454,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="9360">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2468,7 +2468,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2477,9 +2477,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2504,16 +2504,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2534,10 +2534,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2549,7 +2549,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>1</col>
@@ -2569,9 +2569,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2596,9 +2596,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2623,9 +2623,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId3"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2650,9 +2650,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId4"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -21822,16 +21822,38 @@
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="58">
-      <c r="B15" s="28" t="n"/>
-      <c r="C15" s="29" t="n"/>
-      <c r="D15" s="29" t="n"/>
-      <c r="E15" s="29" t="n"/>
-      <c r="F15" s="30" t="n"/>
-      <c r="G15" s="29" t="n"/>
-      <c r="H15" s="29" t="n"/>
-      <c r="I15" s="29" t="n"/>
-      <c r="J15" s="31" t="n"/>
-      <c r="K15" s="32" t="n"/>
+      <c r="B15" s="28" t="n">
+        <v>46184</v>
+      </c>
+      <c r="C15" s="29" t="n">
+        <v>25754859</v>
+      </c>
+      <c r="D15" s="29" t="n">
+        <v>22678562</v>
+      </c>
+      <c r="E15" s="29" t="n">
+        <v>3076297</v>
+      </c>
+      <c r="F15" s="30" t="n">
+        <v>0.1356</v>
+      </c>
+      <c r="G15" s="29" t="n">
+        <v>18380456</v>
+      </c>
+      <c r="H15" s="29" t="n">
+        <v>4869188</v>
+      </c>
+      <c r="I15" s="29" t="n">
+        <v>1136964</v>
+      </c>
+      <c r="J15" s="31" t="n">
+        <v>32.86</v>
+      </c>
+      <c r="K15" s="32" t="inlineStr">
+        <is>
+          <t>Auto weekly snapshot</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="58">
       <c r="B16" s="28" t="n"/>
@@ -23533,7 +23555,7 @@
         </is>
       </c>
       <c r="C5" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="D5" s="64" t="inlineStr">
         <is>
@@ -23548,11 +23570,11 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>32.88</v>
+        <v>32.86</v>
       </c>
       <c r="D6" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-06-10</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-06-11</t>
         </is>
       </c>
     </row>
@@ -23597,11 +23619,11 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>25.5806</v>
+        <v>25.5601</v>
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-06-10</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-06-11</t>
         </is>
       </c>
     </row>
@@ -25201,7 +25223,7 @@
         </is>
       </c>
       <c r="E38" s="33" t="n">
-        <v>22.83</v>
+        <v>23.16</v>
       </c>
       <c r="F38" s="34" t="inlineStr">
         <is>
@@ -25209,7 +25231,7 @@
         </is>
       </c>
       <c r="G38" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H38" s="34" t="inlineStr">
         <is>
@@ -25217,7 +25239,7 @@
         </is>
       </c>
       <c r="I38" t="n">
-        <v>22.82</v>
+        <v>23.16</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="58">
@@ -25241,7 +25263,7 @@
         </is>
       </c>
       <c r="E39" s="33" t="n">
-        <v>1.106</v>
+        <v>1.076</v>
       </c>
       <c r="F39" s="34" t="inlineStr">
         <is>
@@ -25249,7 +25271,7 @@
         </is>
       </c>
       <c r="G39" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H39" s="34" t="inlineStr">
         <is>
@@ -25257,7 +25279,7 @@
         </is>
       </c>
       <c r="I39" t="n">
-        <v>1.076</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="58">
@@ -25281,7 +25303,7 @@
         </is>
       </c>
       <c r="E40" s="33" t="n">
-        <v>770.09</v>
+        <v>753.37</v>
       </c>
       <c r="F40" s="34" t="inlineStr">
         <is>
@@ -25289,7 +25311,7 @@
         </is>
       </c>
       <c r="G40" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H40" s="34" t="inlineStr">
         <is>
@@ -25297,7 +25319,7 @@
         </is>
       </c>
       <c r="I40" t="n">
-        <v>772.830017</v>
+        <v>753.369995</v>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="58">
@@ -25321,7 +25343,7 @@
         </is>
       </c>
       <c r="E41" s="33" t="n">
-        <v>20.84</v>
+        <v>20.4</v>
       </c>
       <c r="F41" s="34" t="inlineStr">
         <is>
@@ -25329,7 +25351,7 @@
         </is>
       </c>
       <c r="G41" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H41" s="34" t="inlineStr">
         <is>
@@ -25337,7 +25359,7 @@
         </is>
       </c>
       <c r="I41" t="n">
-        <v>21.110001</v>
+        <v>20.4</v>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="58">
@@ -25361,7 +25383,7 @@
         </is>
       </c>
       <c r="E42" s="33" t="n">
-        <v>221.79</v>
+        <v>218.03</v>
       </c>
       <c r="F42" s="34" t="inlineStr">
         <is>
@@ -25369,7 +25391,7 @@
         </is>
       </c>
       <c r="G42" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H42" s="34" t="inlineStr">
         <is>
@@ -25377,7 +25399,7 @@
         </is>
       </c>
       <c r="I42" t="n">
-        <v>218.100006</v>
+        <v>218.029999</v>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="58">
@@ -25409,7 +25431,7 @@
         </is>
       </c>
       <c r="G43" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H43" s="34" t="inlineStr">
         <is>
@@ -25449,7 +25471,7 @@
         </is>
       </c>
       <c r="G44" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H44" s="34" t="inlineStr">
         <is>
@@ -25489,7 +25511,7 @@
         </is>
       </c>
       <c r="G45" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H45" s="34" t="inlineStr">
         <is>
@@ -25529,7 +25551,7 @@
         </is>
       </c>
       <c r="G46" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H46" s="34" t="inlineStr">
         <is>
@@ -25606,7 +25628,7 @@
         </is>
       </c>
       <c r="G48" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H48" s="34" t="inlineStr">
         <is>
@@ -25646,7 +25668,7 @@
         </is>
       </c>
       <c r="G49" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H49" s="34" t="inlineStr">
         <is>
@@ -25686,7 +25708,7 @@
         </is>
       </c>
       <c r="G50" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H50" s="34" t="inlineStr">
         <is>
@@ -25726,7 +25748,7 @@
         </is>
       </c>
       <c r="G51" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H51" s="34" t="inlineStr">
         <is>
@@ -25766,7 +25788,7 @@
         </is>
       </c>
       <c r="G52" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H52" s="34" t="inlineStr">
         <is>
@@ -25806,7 +25828,7 @@
         </is>
       </c>
       <c r="G53" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H53" s="34" t="inlineStr">
         <is>
@@ -25846,7 +25868,7 @@
         </is>
       </c>
       <c r="G54" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H54" s="34" t="inlineStr">
         <is>
@@ -25886,7 +25908,7 @@
         </is>
       </c>
       <c r="G55" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H55" s="34" t="inlineStr">
         <is>
@@ -25926,7 +25948,7 @@
         </is>
       </c>
       <c r="G56" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H56" s="34" t="inlineStr">
         <is>
@@ -25966,7 +25988,7 @@
         </is>
       </c>
       <c r="G57" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H57" s="34" t="inlineStr">
         <is>
@@ -26006,7 +26028,7 @@
         </is>
       </c>
       <c r="G58" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H58" s="34" t="inlineStr">
         <is>
@@ -26046,7 +26068,7 @@
         </is>
       </c>
       <c r="G59" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H59" s="34" t="inlineStr">
         <is>
@@ -26078,7 +26100,7 @@
         </is>
       </c>
       <c r="E60" s="33" t="n">
-        <v>170.34</v>
+        <v>157.43</v>
       </c>
       <c r="F60" s="34" t="inlineStr">
         <is>
@@ -26086,7 +26108,7 @@
         </is>
       </c>
       <c r="G60" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H60" s="34" t="inlineStr">
         <is>
@@ -26094,7 +26116,7 @@
         </is>
       </c>
       <c r="I60" t="n">
-        <v>170.339996</v>
+        <v>157.429993</v>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="58">
@@ -26118,7 +26140,7 @@
         </is>
       </c>
       <c r="E61" s="33" t="n">
-        <v>235.61</v>
+        <v>233.38</v>
       </c>
       <c r="F61" s="34" t="inlineStr">
         <is>
@@ -26126,7 +26148,7 @@
         </is>
       </c>
       <c r="G61" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H61" s="34" t="inlineStr">
         <is>
@@ -26134,7 +26156,7 @@
         </is>
       </c>
       <c r="I61" t="n">
-        <v>235.610001</v>
+        <v>233.380005</v>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="58">
@@ -26158,7 +26180,7 @@
         </is>
       </c>
       <c r="E62" s="33" t="n">
-        <v>532.24</v>
+        <v>497.01</v>
       </c>
       <c r="F62" s="34" t="inlineStr">
         <is>
@@ -26166,7 +26188,7 @@
         </is>
       </c>
       <c r="G62" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H62" s="34" t="inlineStr">
         <is>
@@ -26174,7 +26196,7 @@
         </is>
       </c>
       <c r="I62" t="n">
-        <v>532.23999</v>
+        <v>497.01001</v>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1" s="58">
@@ -26198,7 +26220,7 @@
         </is>
       </c>
       <c r="E63" s="33" t="n">
-        <v>164.83</v>
+        <v>157.87</v>
       </c>
       <c r="F63" s="34" t="inlineStr">
         <is>
@@ -26206,7 +26228,7 @@
         </is>
       </c>
       <c r="G63" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H63" s="34" t="inlineStr">
         <is>
@@ -26214,7 +26236,7 @@
         </is>
       </c>
       <c r="I63" t="n">
-        <v>164.830002</v>
+        <v>157.869995</v>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="58">
@@ -26238,7 +26260,7 @@
         </is>
       </c>
       <c r="E64" s="33" t="n">
-        <v>52.9</v>
+        <v>50.57</v>
       </c>
       <c r="F64" s="34" t="inlineStr">
         <is>
@@ -26246,7 +26268,7 @@
         </is>
       </c>
       <c r="G64" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H64" s="34" t="inlineStr">
         <is>
@@ -26254,7 +26276,7 @@
         </is>
       </c>
       <c r="I64" t="n">
-        <v>52.900002</v>
+        <v>50.57</v>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1" s="58">
@@ -26278,7 +26300,7 @@
         </is>
       </c>
       <c r="E65" s="33" t="n">
-        <v>188.19</v>
+        <v>178.45</v>
       </c>
       <c r="F65" s="34" t="inlineStr">
         <is>
@@ -26286,7 +26308,7 @@
         </is>
       </c>
       <c r="G65" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H65" s="34" t="inlineStr">
         <is>
@@ -26294,7 +26316,7 @@
         </is>
       </c>
       <c r="I65" t="n">
-        <v>188.190002</v>
+        <v>178.449997</v>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1" s="58">
@@ -26318,7 +26340,7 @@
         </is>
       </c>
       <c r="E66" s="33" t="n">
-        <v>140.69</v>
+        <v>138.88</v>
       </c>
       <c r="F66" s="34" t="inlineStr">
         <is>
@@ -26326,7 +26348,7 @@
         </is>
       </c>
       <c r="G66" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H66" s="34" t="inlineStr">
         <is>
@@ -26334,7 +26356,7 @@
         </is>
       </c>
       <c r="I66" t="n">
-        <v>140.690002</v>
+        <v>138.880005</v>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1" s="58">
@@ -26358,7 +26380,7 @@
         </is>
       </c>
       <c r="E67" s="33" t="n">
-        <v>156.71</v>
+        <v>154.91</v>
       </c>
       <c r="F67" s="34" t="inlineStr">
         <is>
@@ -26366,7 +26388,7 @@
         </is>
       </c>
       <c r="G67" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H67" s="34" t="inlineStr">
         <is>
@@ -26374,7 +26396,7 @@
         </is>
       </c>
       <c r="I67" t="n">
-        <v>156.710007</v>
+        <v>154.910004</v>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1" s="58">
@@ -26398,7 +26420,7 @@
         </is>
       </c>
       <c r="E68" s="33" t="n">
-        <v>2278.63</v>
+        <v>2135.64</v>
       </c>
       <c r="F68" s="34" t="inlineStr">
         <is>
@@ -26406,7 +26428,7 @@
         </is>
       </c>
       <c r="G68" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H68" s="34" t="inlineStr">
         <is>
@@ -26414,7 +26436,7 @@
         </is>
       </c>
       <c r="I68" t="n">
-        <v>2278.629883</v>
+        <v>2135.639893</v>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="58">
@@ -26438,7 +26460,7 @@
         </is>
       </c>
       <c r="E69" s="33" t="n">
-        <v>1155.5</v>
+        <v>1136.37</v>
       </c>
       <c r="F69" s="34" t="inlineStr">
         <is>
@@ -26446,7 +26468,7 @@
         </is>
       </c>
       <c r="G69" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H69" s="34" t="inlineStr">
         <is>
@@ -26454,7 +26476,7 @@
         </is>
       </c>
       <c r="I69" t="n">
-        <v>1144.680054</v>
+        <v>1136.369995</v>
       </c>
     </row>
     <row r="70" ht="15" customHeight="1" s="58">
@@ -26478,7 +26500,7 @@
         </is>
       </c>
       <c r="E70" s="33" t="n">
-        <v>92.05</v>
+        <v>87.91</v>
       </c>
       <c r="F70" s="34" t="inlineStr">
         <is>
@@ -26486,7 +26508,7 @@
         </is>
       </c>
       <c r="G70" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H70" s="34" t="inlineStr">
         <is>
@@ -26494,7 +26516,7 @@
         </is>
       </c>
       <c r="I70" t="n">
-        <v>92.050003</v>
+        <v>87.910004</v>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1" s="58">
@@ -26518,7 +26540,7 @@
         </is>
       </c>
       <c r="E71" s="33" t="n">
-        <v>1553.96</v>
+        <v>1473.04</v>
       </c>
       <c r="F71" s="34" t="inlineStr">
         <is>
@@ -26526,7 +26548,7 @@
         </is>
       </c>
       <c r="G71" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H71" s="34" t="inlineStr">
         <is>
@@ -26534,7 +26556,7 @@
         </is>
       </c>
       <c r="I71" t="n">
-        <v>1553.959961</v>
+        <v>1473.040039</v>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1" s="58">
@@ -26558,7 +26580,7 @@
         </is>
       </c>
       <c r="E72" s="33" t="n">
-        <v>112.45</v>
+        <v>109.08</v>
       </c>
       <c r="F72" s="34" t="inlineStr">
         <is>
@@ -26566,7 +26588,7 @@
         </is>
       </c>
       <c r="G72" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H72" s="34" t="inlineStr">
         <is>
@@ -26574,7 +26596,7 @@
         </is>
       </c>
       <c r="I72" t="n">
-        <v>112.449997</v>
+        <v>109.080002</v>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1" s="58">
@@ -26598,7 +26620,7 @@
         </is>
       </c>
       <c r="E73" s="33" t="n">
-        <v>206.165</v>
+        <v>200.42</v>
       </c>
       <c r="F73" s="34" t="inlineStr">
         <is>
@@ -26606,7 +26628,7 @@
         </is>
       </c>
       <c r="G73" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H73" s="34" t="inlineStr">
         <is>
@@ -26614,7 +26636,7 @@
         </is>
       </c>
       <c r="I73" t="n">
-        <v>206.164993</v>
+        <v>200.419998</v>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1" s="58">
@@ -26638,7 +26660,7 @@
         </is>
       </c>
       <c r="E74" s="33" t="n">
-        <v>91.55500000000001</v>
+        <v>87.56999999999999</v>
       </c>
       <c r="F74" s="34" t="inlineStr">
         <is>
@@ -26646,7 +26668,7 @@
         </is>
       </c>
       <c r="G74" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H74" s="34" t="inlineStr">
         <is>
@@ -26654,7 +26676,7 @@
         </is>
       </c>
       <c r="I74" t="n">
-        <v>91.55500000000001</v>
+        <v>87.56999999999999</v>
       </c>
     </row>
     <row r="75" ht="15" customHeight="1" s="58">
@@ -26678,7 +26700,7 @@
         </is>
       </c>
       <c r="E75" s="33" t="n">
-        <v>98.2</v>
+        <v>95</v>
       </c>
       <c r="F75" s="34" t="inlineStr">
         <is>
@@ -26686,7 +26708,7 @@
         </is>
       </c>
       <c r="G75" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H75" s="34" t="inlineStr">
         <is>
@@ -26694,7 +26716,7 @@
         </is>
       </c>
       <c r="I75" t="n">
-        <v>98.199997</v>
+        <v>97.94000200000001</v>
       </c>
     </row>
     <row r="76" ht="15" customHeight="1" s="58">
@@ -26718,7 +26740,7 @@
         </is>
       </c>
       <c r="E76" s="33" t="n">
-        <v>368.47</v>
+        <v>347.59</v>
       </c>
       <c r="F76" s="34" t="inlineStr">
         <is>
@@ -26726,7 +26748,7 @@
         </is>
       </c>
       <c r="G76" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H76" s="34" t="inlineStr">
         <is>
@@ -26734,7 +26756,7 @@
         </is>
       </c>
       <c r="I76" t="n">
-        <v>368.470001</v>
+        <v>347.589996</v>
       </c>
     </row>
     <row r="77" ht="15" customHeight="1" s="58">
@@ -26758,7 +26780,7 @@
         </is>
       </c>
       <c r="E77" s="33" t="n">
-        <v>390.05</v>
+        <v>381.59</v>
       </c>
       <c r="F77" s="34" t="inlineStr">
         <is>
@@ -26766,7 +26788,7 @@
         </is>
       </c>
       <c r="G77" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H77" s="34" t="inlineStr">
         <is>
@@ -26774,7 +26796,7 @@
         </is>
       </c>
       <c r="I77" t="n">
-        <v>390.049988</v>
+        <v>381.589996</v>
       </c>
     </row>
     <row r="78" ht="15" customHeight="1" s="58">
@@ -26798,7 +26820,7 @@
         </is>
       </c>
       <c r="E78" s="33" t="n">
-        <v>53.615</v>
+        <v>51.97</v>
       </c>
       <c r="F78" s="34" t="inlineStr">
         <is>
@@ -26806,7 +26828,7 @@
         </is>
       </c>
       <c r="G78" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H78" s="34" t="inlineStr">
         <is>
@@ -26814,7 +26836,7 @@
         </is>
       </c>
       <c r="I78" t="n">
-        <v>53.615002</v>
+        <v>51.970001</v>
       </c>
     </row>
     <row r="79" ht="15" customHeight="1" s="58">
@@ -26838,7 +26860,7 @@
         </is>
       </c>
       <c r="E79" s="33" t="n">
-        <v>86.88</v>
+        <v>85.13</v>
       </c>
       <c r="F79" s="34" t="inlineStr">
         <is>
@@ -26846,7 +26868,7 @@
         </is>
       </c>
       <c r="G79" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H79" s="34" t="inlineStr">
         <is>
@@ -26854,7 +26876,7 @@
         </is>
       </c>
       <c r="I79" t="n">
-        <v>86.879997</v>
+        <v>85.129997</v>
       </c>
     </row>
     <row r="80" ht="15" customHeight="1" s="58">
@@ -26878,7 +26900,7 @@
         </is>
       </c>
       <c r="E80" s="33" t="n">
-        <v>289.98</v>
+        <v>291.58</v>
       </c>
       <c r="F80" s="34" t="inlineStr">
         <is>
@@ -26886,7 +26908,7 @@
         </is>
       </c>
       <c r="G80" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H80" s="34" t="inlineStr">
         <is>
@@ -26894,7 +26916,7 @@
         </is>
       </c>
       <c r="I80" t="n">
-        <v>289.980011</v>
+        <v>291.579987</v>
       </c>
     </row>
     <row r="81" ht="15" customHeight="1" s="58">
@@ -26918,7 +26940,7 @@
         </is>
       </c>
       <c r="E81" s="33" t="n">
-        <v>158.67</v>
+        <v>153.97</v>
       </c>
       <c r="F81" s="34" t="inlineStr">
         <is>
@@ -26926,7 +26948,7 @@
         </is>
       </c>
       <c r="G81" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H81" s="34" t="inlineStr">
         <is>
@@ -26934,7 +26956,7 @@
         </is>
       </c>
       <c r="I81" t="n">
-        <v>158.669998</v>
+        <v>153.970001</v>
       </c>
     </row>
     <row r="82" ht="15" customHeight="1" s="58">
@@ -26958,7 +26980,7 @@
         </is>
       </c>
       <c r="E82" s="33" t="n">
-        <v>583.42</v>
+        <v>570.98</v>
       </c>
       <c r="F82" s="34" t="inlineStr">
         <is>
@@ -26966,7 +26988,7 @@
         </is>
       </c>
       <c r="G82" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H82" s="34" t="inlineStr">
         <is>
@@ -26974,7 +26996,7 @@
         </is>
       </c>
       <c r="I82" t="n">
-        <v>583.4198</v>
+        <v>570.97998</v>
       </c>
     </row>
     <row r="83" ht="15" customHeight="1" s="58">
@@ -26998,7 +27020,7 @@
         </is>
       </c>
       <c r="E83" s="33" t="n">
-        <v>144.75</v>
+        <v>139.99</v>
       </c>
       <c r="F83" s="34" t="inlineStr">
         <is>
@@ -27006,7 +27028,7 @@
         </is>
       </c>
       <c r="G83" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H83" s="34" t="inlineStr">
         <is>
@@ -27014,7 +27036,7 @@
         </is>
       </c>
       <c r="I83" t="n">
-        <v>153.5</v>
+        <v>139.990005</v>
       </c>
     </row>
     <row r="84" ht="15" customHeight="1" s="58">
@@ -27038,7 +27060,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>62.68</v>
+        <v>62.21</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -27046,7 +27068,7 @@
         </is>
       </c>
       <c r="G84" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H84" s="34" t="inlineStr">
         <is>
@@ -27054,7 +27076,7 @@
         </is>
       </c>
       <c r="I84" t="n">
-        <v>60.877799</v>
+        <v>62.344047</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="58">
@@ -27078,7 +27100,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>591.79</v>
+        <v>591.73</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -27086,7 +27108,7 @@
         </is>
       </c>
       <c r="G85" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H85" s="34" t="inlineStr">
         <is>
@@ -27094,7 +27116,7 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>587.036671</v>
+        <v>592.50805</v>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="58">
@@ -27118,7 +27140,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>61950</v>
+        <v>62104</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -27126,7 +27148,7 @@
         </is>
       </c>
       <c r="G86" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H86" s="34" t="inlineStr">
         <is>
@@ -27134,7 +27156,7 @@
         </is>
       </c>
       <c r="I86" t="n">
-        <v>61401.309315</v>
+        <v>61796.727025</v>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="58">
@@ -27158,7 +27180,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.006681</v>
+        <v>0.006445</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -27166,7 +27188,7 @@
         </is>
       </c>
       <c r="G87" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H87" s="34" t="inlineStr">
         <is>
@@ -27174,7 +27196,7 @@
         </is>
       </c>
       <c r="I87" t="n">
-        <v>0.006668</v>
+        <v>0.006782</v>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="58">
@@ -27198,7 +27220,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.010243</v>
+        <v>0.010345</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -27206,7 +27228,7 @@
         </is>
       </c>
       <c r="G88" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H88" s="34" t="inlineStr">
         <is>
@@ -27214,7 +27236,7 @@
         </is>
       </c>
       <c r="I88" t="n">
-        <v>0.010795</v>
+        <v>0.010714</v>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="58">
@@ -27238,7 +27260,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>64.91</v>
+        <v>64.20999999999999</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -27246,7 +27268,7 @@
         </is>
       </c>
       <c r="G89" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H89" s="34" t="inlineStr">
         <is>
@@ -27254,7 +27276,7 @@
         </is>
       </c>
       <c r="I89" t="n">
-        <v>64.84906100000001</v>
+        <v>65.086533</v>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="58">
@@ -27278,7 +27300,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>1.67</v>
+        <v>1.65</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -27286,7 +27308,7 @@
         </is>
       </c>
       <c r="G90" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H90" s="34" t="inlineStr">
         <is>
@@ -27294,7 +27316,7 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>1.637659</v>
+        <v>1.655745</v>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="58">
@@ -27326,7 +27348,7 @@
         </is>
       </c>
       <c r="G91" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H91" s="34" t="inlineStr">
         <is>
@@ -27358,7 +27380,7 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
-        <v>0.013732</v>
+        <v>0.013486</v>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
@@ -27366,7 +27388,7 @@
         </is>
       </c>
       <c r="G92" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H92" s="34" t="inlineStr">
         <is>
@@ -27374,7 +27396,7 @@
         </is>
       </c>
       <c r="I92" t="n">
-        <v>0.013667</v>
+        <v>0.013957</v>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="58">
@@ -27398,7 +27420,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>2.635168</v>
+        <v>2.572347</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -27406,7 +27428,7 @@
         </is>
       </c>
       <c r="G93" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H93" s="34" t="inlineStr">
         <is>
@@ -27414,7 +27436,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>2.610185</v>
+        <v>2.665431</v>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="58">
@@ -27438,7 +27460,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>24.727799</v>
+        <v>24.248774</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -27446,7 +27468,7 @@
         </is>
       </c>
       <c r="G94" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H94" s="34" t="inlineStr">
         <is>
@@ -27454,7 +27476,7 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>24.325458</v>
+        <v>24.790295</v>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="58">
@@ -27478,7 +27500,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.110943</v>
+        <v>0.108889</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -27486,7 +27508,7 @@
         </is>
       </c>
       <c r="G95" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H95" s="34" t="inlineStr">
         <is>
@@ -27494,7 +27516,7 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>0.111469</v>
+        <v>0.110444</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="58">
@@ -27518,7 +27540,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>19458.0552</v>
+        <v>19444.2478</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -27526,7 +27548,7 @@
         </is>
       </c>
       <c r="G96" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H96" s="34" t="inlineStr">
         <is>
@@ -27534,7 +27556,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>19301.765755</v>
+        <v>19469.814527</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="58">
@@ -27558,7 +27580,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2036916</v>
+        <v>2040737.44</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -27566,7 +27588,7 @@
         </is>
       </c>
       <c r="G97" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H97" s="34" t="inlineStr">
         <is>
@@ -27574,7 +27596,7 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>2018875.050278</v>
+        <v>2030640.450055</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="58">
@@ -27598,7 +27620,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>2.770469</v>
+        <v>2.758236</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -27606,7 +27628,7 @@
         </is>
       </c>
       <c r="G98" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H98" s="34" t="inlineStr">
         <is>
@@ -27614,7 +27636,7 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>2.783676</v>
+        <v>2.787017</v>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="58">
@@ -27638,7 +27660,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>54041.8968</v>
+        <v>53865.0978</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -27646,7 +27668,7 @@
         </is>
       </c>
       <c r="G99" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H99" s="34" t="inlineStr">
         <is>
@@ -27654,7 +27676,7 @@
         </is>
       </c>
       <c r="I99" t="n">
-        <v>53987.547529</v>
+        <v>53899.43744</v>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="58">
@@ -27678,7 +27700,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>24.806217</v>
+        <v>24.734806</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -27686,7 +27708,7 @@
         </is>
       </c>
       <c r="G100" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H100" s="34" t="inlineStr">
         <is>
@@ -27694,7 +27716,7 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>25.257457</v>
+        <v>25.062992</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="58">
@@ -27718,7 +27740,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>61950</v>
+        <v>62104</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -27726,7 +27748,7 @@
         </is>
       </c>
       <c r="G101" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H101" s="34" t="inlineStr">
         <is>
@@ -27734,7 +27756,7 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>61401.309315</v>
+        <v>61796.727025</v>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="58">
@@ -27758,7 +27780,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>18.04</v>
+        <v>17.71</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -27766,7 +27788,7 @@
         </is>
       </c>
       <c r="G102" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H102" s="34" t="inlineStr">
         <is>
@@ -27774,7 +27796,7 @@
         </is>
       </c>
       <c r="I102" t="n">
-        <v>17.614897</v>
+        <v>18.86456</v>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="58">
@@ -27872,7 +27894,7 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
-        <v>0.006681</v>
+        <v>0.006445</v>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
@@ -27880,7 +27902,7 @@
         </is>
       </c>
       <c r="G105" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H105" s="34" t="inlineStr">
         <is>
@@ -27888,7 +27910,7 @@
         </is>
       </c>
       <c r="I105" t="n">
-        <v>0.006668</v>
+        <v>0.006782</v>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="58">
@@ -27912,7 +27934,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>64.91</v>
+        <v>64.20999999999999</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>
@@ -27920,7 +27942,7 @@
         </is>
       </c>
       <c r="G106" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H106" s="34" t="inlineStr">
         <is>
@@ -27928,7 +27950,7 @@
         </is>
       </c>
       <c r="I106" t="n">
-        <v>64.84906100000001</v>
+        <v>65.086533</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="58">
@@ -27960,7 +27982,7 @@
         </is>
       </c>
       <c r="G107" s="28" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="H107" s="34" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Weekly dashboard update — 2026-06-11
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-42660" yWindow="-540" windowWidth="32460" windowHeight="17180" tabRatio="500" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Realized" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Realized" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Prices" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Reference" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="AsOfDate">'FX &amp; Assumptions'!$C$5</definedName>
@@ -697,14 +697,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -726,8 +726,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -752,10 +752,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -764,10 +764,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4F81BD"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+              <a:ln w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -777,10 +777,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="C0504D"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -790,10 +790,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="9BBB59"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -803,10 +803,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="8064A2"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -816,10 +816,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4BACC6"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -829,10 +829,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="F79646"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -842,14 +842,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -875,14 +875,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -908,14 +908,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -941,14 +941,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -974,14 +974,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1007,14 +1007,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1038,16 +1038,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1142,16 +1142,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1172,10 +1172,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1187,14 +1187,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1216,8 +1216,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1242,10 +1242,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1254,10 +1254,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4672A8"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1267,10 +1267,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="AB4744"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1280,10 +1280,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="8AA64F"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1293,10 +1293,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="725990"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1306,10 +1306,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4299B0"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1319,10 +1319,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="DC853E"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1332,10 +1332,10 @@
             <idx val="6"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="93A9CE"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1345,10 +1345,10 @@
             <idx val="7"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="D09493"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1358,10 +1358,10 @@
             <idx val="8"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="B8CD97"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1371,14 +1371,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1405,14 +1405,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1439,14 +1439,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1473,14 +1473,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1507,14 +1507,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1541,14 +1541,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1575,14 +1575,14 @@
             <dLbl>
               <idx val="6"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1609,14 +1609,14 @@
             <dLbl>
               <idx val="7"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1643,14 +1643,14 @@
             <dLbl>
               <idx val="8"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1675,16 +1675,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1791,16 +1791,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1821,10 +1821,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1836,14 +1836,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1865,8 +1865,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1893,10 +1893,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1904,16 +1904,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2016,7 +2016,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2025,9 +2025,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2059,7 +2059,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2073,7 +2073,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2082,9 +2082,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2109,16 +2109,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2139,10 +2139,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2154,14 +2154,14 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -2183,8 +2183,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -2200,10 +2200,10 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2211,16 +2211,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2411,7 +2411,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2420,9 +2420,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2454,7 +2454,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2468,7 +2468,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2477,9 +2477,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2504,16 +2504,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2534,10 +2534,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2549,7 +2549,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>1</col>
@@ -2569,9 +2569,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2596,9 +2596,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+          <c:chart r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2623,9 +2623,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+          <c:chart r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2650,9 +2650,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+          <c:chart r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -21826,28 +21826,28 @@
         <v>46184</v>
       </c>
       <c r="C15" s="29" t="n">
-        <v>25754859</v>
+        <v>25715762</v>
       </c>
       <c r="D15" s="29" t="n">
-        <v>22678562</v>
+        <v>22691872</v>
       </c>
       <c r="E15" s="29" t="n">
-        <v>3076297</v>
+        <v>3023890</v>
       </c>
       <c r="F15" s="30" t="n">
-        <v>0.1356</v>
+        <v>0.1333</v>
       </c>
       <c r="G15" s="29" t="n">
-        <v>18380456</v>
+        <v>18286893</v>
       </c>
       <c r="H15" s="29" t="n">
-        <v>4869188</v>
+        <v>4907650</v>
       </c>
       <c r="I15" s="29" t="n">
-        <v>1136964</v>
+        <v>1149975</v>
       </c>
       <c r="J15" s="31" t="n">
-        <v>32.86</v>
+        <v>32.98</v>
       </c>
       <c r="K15" s="32" t="inlineStr">
         <is>
@@ -23570,7 +23570,7 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>32.86</v>
+        <v>32.98</v>
       </c>
       <c r="D6" s="64" t="inlineStr">
         <is>
@@ -23619,7 +23619,7 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>25.5601</v>
+        <v>25.5975</v>
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
@@ -23738,27 +23738,27 @@
         </is>
       </c>
       <c r="E5" s="33" t="n">
+        <v>23.9719</v>
+      </c>
+      <c r="F5" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G5" s="28" t="n">
+        <v>46182</v>
+      </c>
+      <c r="H5" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
         <v>24.4495</v>
       </c>
-      <c r="F5" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G5" s="28" t="n">
-        <v>46181</v>
-      </c>
-      <c r="H5" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I5" t="n">
-        <v>23.3473</v>
-      </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
     </row>
@@ -23783,27 +23783,27 @@
         </is>
       </c>
       <c r="E6" s="33" t="n">
+        <v>10.687</v>
+      </c>
+      <c r="F6" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G6" s="28" t="n">
+        <v>46183</v>
+      </c>
+      <c r="H6" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
         <v>10.6868</v>
       </c>
-      <c r="F6" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G6" s="28" t="n">
-        <v>46182</v>
-      </c>
-      <c r="H6" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I6" t="n">
-        <v>10.6865</v>
-      </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
     </row>
@@ -23828,27 +23828,27 @@
         </is>
       </c>
       <c r="E7" s="33" t="n">
+        <v>7.0939</v>
+      </c>
+      <c r="F7" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G7" s="28" t="n">
+        <v>46182</v>
+      </c>
+      <c r="H7" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
         <v>7.0857</v>
       </c>
-      <c r="F7" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G7" s="28" t="n">
-        <v>46181</v>
-      </c>
-      <c r="H7" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I7" t="n">
-        <v>7.1091</v>
-      </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
     </row>
@@ -23873,27 +23873,27 @@
         </is>
       </c>
       <c r="E8" s="33" t="n">
+        <v>9.4916</v>
+      </c>
+      <c r="F8" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G8" s="28" t="n">
+        <v>46182</v>
+      </c>
+      <c r="H8" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
         <v>9.2986</v>
       </c>
-      <c r="F8" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G8" s="28" t="n">
-        <v>46181</v>
-      </c>
-      <c r="H8" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I8" t="n">
-        <v>9.393700000000001</v>
-      </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
     </row>
@@ -23918,27 +23918,27 @@
         </is>
       </c>
       <c r="E9" s="33" t="n">
+        <v>9.1568</v>
+      </c>
+      <c r="F9" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G9" s="28" t="n">
+        <v>46183</v>
+      </c>
+      <c r="H9" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
         <v>9.2889</v>
       </c>
-      <c r="F9" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G9" s="28" t="n">
-        <v>46182</v>
-      </c>
-      <c r="H9" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I9" t="n">
-        <v>9.1631</v>
-      </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
     </row>
@@ -23963,27 +23963,27 @@
         </is>
       </c>
       <c r="E10" s="33" t="n">
+        <v>13.2756</v>
+      </c>
+      <c r="F10" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G10" s="28" t="n">
+        <v>46182</v>
+      </c>
+      <c r="H10" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
         <v>13.0438</v>
       </c>
-      <c r="F10" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G10" s="28" t="n">
-        <v>46181</v>
-      </c>
-      <c r="H10" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I10" t="n">
-        <v>13.5827</v>
-      </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
     </row>
@@ -24008,27 +24008,27 @@
         </is>
       </c>
       <c r="E11" s="33" t="n">
+        <v>12.894</v>
+      </c>
+      <c r="F11" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G11" s="28" t="n">
+        <v>46183</v>
+      </c>
+      <c r="H11" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
         <v>13.1546</v>
       </c>
-      <c r="F11" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G11" s="28" t="n">
-        <v>46182</v>
-      </c>
-      <c r="H11" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I11" t="n">
-        <v>12.9039</v>
-      </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
     </row>
@@ -24053,27 +24053,27 @@
         </is>
       </c>
       <c r="E12" s="33" t="n">
+        <v>25.8795</v>
+      </c>
+      <c r="F12" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G12" s="28" t="n">
+        <v>46183</v>
+      </c>
+      <c r="H12" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
         <v>26.6235</v>
       </c>
-      <c r="F12" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G12" s="28" t="n">
-        <v>46182</v>
-      </c>
-      <c r="H12" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I12" t="n">
-        <v>26.0378</v>
-      </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
     </row>
@@ -24098,27 +24098,27 @@
         </is>
       </c>
       <c r="E13" s="33" t="n">
+        <v>35.8529</v>
+      </c>
+      <c r="F13" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G13" s="28" t="n">
+        <v>46183</v>
+      </c>
+      <c r="H13" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
         <v>36.2939</v>
       </c>
-      <c r="F13" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G13" s="28" t="n">
-        <v>46182</v>
-      </c>
-      <c r="H13" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I13" t="n">
-        <v>35.7675</v>
-      </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
     </row>
@@ -24143,27 +24143,27 @@
         </is>
       </c>
       <c r="E14" s="33" t="n">
+        <v>25.1917</v>
+      </c>
+      <c r="F14" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G14" s="28" t="n">
+        <v>46183</v>
+      </c>
+      <c r="H14" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
         <v>25.3708</v>
       </c>
-      <c r="F14" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G14" s="28" t="n">
-        <v>46182</v>
-      </c>
-      <c r="H14" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I14" t="n">
-        <v>25.2435</v>
-      </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
     </row>
@@ -24188,27 +24188,27 @@
         </is>
       </c>
       <c r="E15" s="33" t="n">
+        <v>14.8604</v>
+      </c>
+      <c r="F15" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G15" s="28" t="n">
+        <v>46181</v>
+      </c>
+      <c r="H15" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
         <v>14.8466</v>
       </c>
-      <c r="F15" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G15" s="28" t="n">
-        <v>46178</v>
-      </c>
-      <c r="H15" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I15" t="n">
-        <v>14.8572</v>
-      </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
@@ -24233,27 +24233,27 @@
         </is>
       </c>
       <c r="E16" s="33" t="n">
+        <v>80.4905</v>
+      </c>
+      <c r="F16" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G16" s="28" t="n">
+        <v>46183</v>
+      </c>
+      <c r="H16" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
         <v>81.4269</v>
       </c>
-      <c r="F16" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G16" s="28" t="n">
-        <v>46182</v>
-      </c>
-      <c r="H16" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I16" t="n">
-        <v>80.3703</v>
-      </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
     </row>
@@ -24278,27 +24278,27 @@
         </is>
       </c>
       <c r="E17" s="33" t="n">
+        <v>52.7619</v>
+      </c>
+      <c r="F17" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G17" s="28" t="n">
+        <v>46183</v>
+      </c>
+      <c r="H17" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
         <v>53.1377</v>
       </c>
-      <c r="F17" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G17" s="28" t="n">
-        <v>46182</v>
-      </c>
-      <c r="H17" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I17" t="n">
-        <v>52.898</v>
-      </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
     </row>
@@ -24323,27 +24323,27 @@
         </is>
       </c>
       <c r="E18" s="33" t="n">
+        <v>16.4301</v>
+      </c>
+      <c r="F18" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G18" s="28" t="n">
+        <v>46183</v>
+      </c>
+      <c r="H18" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
         <v>16.4125</v>
       </c>
-      <c r="F18" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G18" s="28" t="n">
-        <v>46182</v>
-      </c>
-      <c r="H18" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I18" t="n">
-        <v>16.4116</v>
-      </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
     </row>
@@ -24368,27 +24368,27 @@
         </is>
       </c>
       <c r="E19" s="33" t="n">
+        <v>23.4039</v>
+      </c>
+      <c r="F19" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G19" s="28" t="n">
+        <v>46183</v>
+      </c>
+      <c r="H19" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
         <v>23.4031</v>
       </c>
-      <c r="F19" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G19" s="28" t="n">
-        <v>46182</v>
-      </c>
-      <c r="H19" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I19" t="n">
-        <v>23.4026</v>
-      </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
     </row>
@@ -24413,27 +24413,27 @@
         </is>
       </c>
       <c r="E20" s="33" t="n">
+        <v>40.563</v>
+      </c>
+      <c r="F20" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G20" s="28" t="n">
+        <v>46182</v>
+      </c>
+      <c r="H20" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
         <v>40.6754</v>
       </c>
-      <c r="F20" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G20" s="28" t="n">
-        <v>46181</v>
-      </c>
-      <c r="H20" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I20" t="n">
-        <v>40.5739</v>
-      </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
     </row>
@@ -24458,27 +24458,27 @@
         </is>
       </c>
       <c r="E21" s="33" t="n">
+        <v>13.3396</v>
+      </c>
+      <c r="F21" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G21" s="28" t="n">
+        <v>46183</v>
+      </c>
+      <c r="H21" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
         <v>13.3598</v>
       </c>
-      <c r="F21" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G21" s="28" t="n">
-        <v>46182</v>
-      </c>
-      <c r="H21" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I21" t="n">
-        <v>13.241</v>
-      </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
     </row>
@@ -24503,27 +24503,27 @@
         </is>
       </c>
       <c r="E22" s="33" t="n">
+        <v>13.2159</v>
+      </c>
+      <c r="F22" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G22" s="28" t="n">
+        <v>46182</v>
+      </c>
+      <c r="H22" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
         <v>13.215</v>
       </c>
-      <c r="F22" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G22" s="28" t="n">
-        <v>46181</v>
-      </c>
-      <c r="H22" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I22" t="n">
-        <v>13.2668</v>
-      </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
     </row>
@@ -24548,27 +24548,27 @@
         </is>
       </c>
       <c r="E23" s="33" t="n">
+        <v>12.2493</v>
+      </c>
+      <c r="F23" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G23" s="28" t="n">
+        <v>46183</v>
+      </c>
+      <c r="H23" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
         <v>12.3772</v>
       </c>
-      <c r="F23" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G23" s="28" t="n">
-        <v>46182</v>
-      </c>
-      <c r="H23" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I23" t="n">
-        <v>12.3035</v>
-      </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
     </row>
@@ -24593,27 +24593,27 @@
         </is>
       </c>
       <c r="E24" s="33" t="n">
+        <v>11.8802</v>
+      </c>
+      <c r="F24" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G24" s="28" t="n">
+        <v>46182</v>
+      </c>
+      <c r="H24" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
         <v>11.827</v>
       </c>
-      <c r="F24" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G24" s="28" t="n">
-        <v>46181</v>
-      </c>
-      <c r="H24" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I24" t="n">
-        <v>11.9931</v>
-      </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
     </row>
@@ -24638,27 +24638,27 @@
         </is>
       </c>
       <c r="E25" s="33" t="n">
+        <v>9.9718</v>
+      </c>
+      <c r="F25" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G25" s="28" t="n">
+        <v>46183</v>
+      </c>
+      <c r="H25" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
         <v>9.9245</v>
       </c>
-      <c r="F25" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G25" s="28" t="n">
-        <v>46182</v>
-      </c>
-      <c r="H25" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I25" t="n">
-        <v>9.8523</v>
-      </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
     </row>
@@ -24683,27 +24683,27 @@
         </is>
       </c>
       <c r="E26" s="33" t="n">
+        <v>14.002</v>
+      </c>
+      <c r="F26" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G26" s="28" t="n">
+        <v>46183</v>
+      </c>
+      <c r="H26" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
         <v>13.9301</v>
       </c>
-      <c r="F26" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G26" s="28" t="n">
-        <v>46182</v>
-      </c>
-      <c r="H26" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I26" t="n">
-        <v>13.8268</v>
-      </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
     </row>
@@ -24728,27 +24728,27 @@
         </is>
       </c>
       <c r="E27" s="33" t="n">
+        <v>16.7307</v>
+      </c>
+      <c r="F27" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G27" s="28" t="n">
+        <v>46183</v>
+      </c>
+      <c r="H27" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
         <v>16.8932</v>
       </c>
-      <c r="F27" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G27" s="28" t="n">
-        <v>46182</v>
-      </c>
-      <c r="H27" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I27" t="n">
-        <v>16.8474</v>
-      </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
     </row>
@@ -24773,27 +24773,27 @@
         </is>
       </c>
       <c r="E28" s="33" t="n">
+        <v>18.5085</v>
+      </c>
+      <c r="F28" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G28" s="28" t="n">
+        <v>46183</v>
+      </c>
+      <c r="H28" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
         <v>19.2336</v>
       </c>
-      <c r="F28" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G28" s="28" t="n">
-        <v>46182</v>
-      </c>
-      <c r="H28" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I28" t="n">
-        <v>19.1156</v>
-      </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
     </row>
@@ -24818,27 +24818,27 @@
         </is>
       </c>
       <c r="E29" s="33" t="n">
+        <v>25.0651</v>
+      </c>
+      <c r="F29" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G29" s="28" t="n">
+        <v>46182</v>
+      </c>
+      <c r="H29" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
         <v>25.2898</v>
       </c>
-      <c r="F29" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G29" s="28" t="n">
-        <v>46181</v>
-      </c>
-      <c r="H29" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I29" t="n">
-        <v>23.8964</v>
-      </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
     </row>
@@ -24863,27 +24863,27 @@
         </is>
       </c>
       <c r="E30" s="33" t="n">
+        <v>36.0558</v>
+      </c>
+      <c r="F30" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G30" s="28" t="n">
+        <v>46182</v>
+      </c>
+      <c r="H30" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
         <v>37.4218</v>
       </c>
-      <c r="F30" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G30" s="28" t="n">
-        <v>46181</v>
-      </c>
-      <c r="H30" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I30" t="n">
-        <v>36.6591</v>
-      </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
     </row>
@@ -24908,27 +24908,27 @@
         </is>
       </c>
       <c r="E31" s="33" t="n">
+        <v>12.7851</v>
+      </c>
+      <c r="F31" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G31" s="28" t="n">
+        <v>46183</v>
+      </c>
+      <c r="H31" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
         <v>12.9477</v>
       </c>
-      <c r="F31" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G31" s="28" t="n">
-        <v>46182</v>
-      </c>
-      <c r="H31" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I31" t="n">
-        <v>12.7623</v>
-      </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
     </row>
@@ -24953,27 +24953,27 @@
         </is>
       </c>
       <c r="E32" s="33" t="n">
+        <v>21.7057</v>
+      </c>
+      <c r="F32" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G32" s="28" t="n">
+        <v>46183</v>
+      </c>
+      <c r="H32" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
         <v>21.7055</v>
       </c>
-      <c r="F32" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G32" s="28" t="n">
-        <v>46182</v>
-      </c>
-      <c r="H32" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I32" t="n">
-        <v>21.7053</v>
-      </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
     </row>
@@ -24998,27 +24998,27 @@
         </is>
       </c>
       <c r="E33" s="33" t="n">
+        <v>12.3702</v>
+      </c>
+      <c r="F33" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G33" s="28" t="n">
+        <v>46183</v>
+      </c>
+      <c r="H33" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
         <v>12.5043</v>
       </c>
-      <c r="F33" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G33" s="28" t="n">
-        <v>46182</v>
-      </c>
-      <c r="H33" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I33" t="n">
-        <v>12.3354</v>
-      </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
     </row>
@@ -25043,27 +25043,27 @@
         </is>
       </c>
       <c r="E34" s="33" t="n">
+        <v>16.205</v>
+      </c>
+      <c r="F34" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G34" s="28" t="n">
+        <v>46183</v>
+      </c>
+      <c r="H34" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
         <v>16.2045</v>
       </c>
-      <c r="F34" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G34" s="28" t="n">
-        <v>46182</v>
-      </c>
-      <c r="H34" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I34" t="n">
-        <v>16.2041</v>
-      </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
     </row>
@@ -25088,27 +25088,27 @@
         </is>
       </c>
       <c r="E35" s="33" t="n">
+        <v>27.6474</v>
+      </c>
+      <c r="F35" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G35" s="28" t="n">
+        <v>46182</v>
+      </c>
+      <c r="H35" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
         <v>28.1255</v>
       </c>
-      <c r="F35" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G35" s="28" t="n">
-        <v>46181</v>
-      </c>
-      <c r="H35" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I35" t="n">
-        <v>27.8538</v>
-      </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
     </row>
@@ -25133,27 +25133,27 @@
         </is>
       </c>
       <c r="E36" s="33" t="n">
+        <v>9.995900000000001</v>
+      </c>
+      <c r="F36" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G36" s="28" t="n">
+        <v>46183</v>
+      </c>
+      <c r="H36" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
         <v>9.9649</v>
       </c>
-      <c r="F36" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G36" s="28" t="n">
-        <v>46182</v>
-      </c>
-      <c r="H36" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I36" t="n">
-        <v>9.978999999999999</v>
-      </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
     </row>
@@ -25178,27 +25178,27 @@
         </is>
       </c>
       <c r="E37" s="33" t="n">
+        <v>22.3085</v>
+      </c>
+      <c r="F37" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G37" s="28" t="n">
+        <v>46183</v>
+      </c>
+      <c r="H37" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
         <v>22.5842</v>
       </c>
-      <c r="F37" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G37" s="28" t="n">
-        <v>46182</v>
-      </c>
-      <c r="H37" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I37" t="n">
-        <v>22.348</v>
-      </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
     </row>
@@ -25263,7 +25263,7 @@
         </is>
       </c>
       <c r="E39" s="33" t="n">
-        <v>1.076</v>
+        <v>1.08</v>
       </c>
       <c r="F39" s="34" t="inlineStr">
         <is>
@@ -25463,7 +25463,7 @@
         </is>
       </c>
       <c r="E44" s="33" t="n">
-        <v>169</v>
+        <v>168.5</v>
       </c>
       <c r="F44" s="34" t="inlineStr">
         <is>
@@ -25479,7 +25479,7 @@
         </is>
       </c>
       <c r="I44" t="n">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="58">
@@ -25503,7 +25503,7 @@
         </is>
       </c>
       <c r="E45" s="33" t="n">
-        <v>0.44</v>
+        <v>0.45</v>
       </c>
       <c r="F45" s="34" t="inlineStr">
         <is>
@@ -25519,7 +25519,7 @@
         </is>
       </c>
       <c r="I45" t="n">
-        <v>0.44</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="58">
@@ -25660,7 +25660,7 @@
         </is>
       </c>
       <c r="E49" s="33" t="n">
-        <v>63</v>
+        <v>62.75</v>
       </c>
       <c r="F49" s="34" t="inlineStr">
         <is>
@@ -25676,7 +25676,7 @@
         </is>
       </c>
       <c r="I49" t="n">
-        <v>63.75</v>
+        <v>63</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="58">
@@ -25740,7 +25740,7 @@
         </is>
       </c>
       <c r="E51" s="33" t="n">
-        <v>15.3</v>
+        <v>15.1</v>
       </c>
       <c r="F51" s="34" t="inlineStr">
         <is>
@@ -25756,7 +25756,7 @@
         </is>
       </c>
       <c r="I51" t="n">
-        <v>15.3</v>
+        <v>15.1</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" s="58">
@@ -25820,7 +25820,7 @@
         </is>
       </c>
       <c r="E53" s="33" t="n">
-        <v>5.35</v>
+        <v>5.45</v>
       </c>
       <c r="F53" s="34" t="inlineStr">
         <is>
@@ -25836,7 +25836,7 @@
         </is>
       </c>
       <c r="I53" t="n">
-        <v>5.35</v>
+        <v>5.45</v>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="58">
@@ -25860,7 +25860,7 @@
         </is>
       </c>
       <c r="E54" s="33" t="n">
-        <v>20.1</v>
+        <v>19.9</v>
       </c>
       <c r="F54" s="34" t="inlineStr">
         <is>
@@ -25876,7 +25876,7 @@
         </is>
       </c>
       <c r="I54" t="n">
-        <v>20.1</v>
+        <v>19.9</v>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="58">
@@ -25900,7 +25900,7 @@
         </is>
       </c>
       <c r="E55" s="33" t="n">
-        <v>3.5</v>
+        <v>3.54</v>
       </c>
       <c r="F55" s="34" t="inlineStr">
         <is>
@@ -25916,7 +25916,7 @@
         </is>
       </c>
       <c r="I55" t="n">
-        <v>3.52</v>
+        <v>3.54</v>
       </c>
     </row>
     <row r="56" ht="15" customHeight="1" s="58">
@@ -25940,7 +25940,7 @@
         </is>
       </c>
       <c r="E56" s="33" t="n">
-        <v>4.76</v>
+        <v>4.8</v>
       </c>
       <c r="F56" s="34" t="inlineStr">
         <is>
@@ -25956,7 +25956,7 @@
         </is>
       </c>
       <c r="I56" t="n">
-        <v>4.76</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1" s="58">
@@ -25980,7 +25980,7 @@
         </is>
       </c>
       <c r="E57" s="33" t="n">
-        <v>2.54</v>
+        <v>2.56</v>
       </c>
       <c r="F57" s="34" t="inlineStr">
         <is>
@@ -25996,7 +25996,7 @@
         </is>
       </c>
       <c r="I57" t="n">
-        <v>2.54</v>
+        <v>2.56</v>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="58">
@@ -26020,7 +26020,7 @@
         </is>
       </c>
       <c r="E58" s="33" t="n">
-        <v>12.1</v>
+        <v>11.9</v>
       </c>
       <c r="F58" s="34" t="inlineStr">
         <is>
@@ -26036,7 +26036,7 @@
         </is>
       </c>
       <c r="I58" t="n">
-        <v>12.1</v>
+        <v>11.9</v>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="58">
@@ -26060,7 +26060,7 @@
         </is>
       </c>
       <c r="E59" s="33" t="n">
-        <v>16.6</v>
+        <v>16.5</v>
       </c>
       <c r="F59" s="34" t="inlineStr">
         <is>
@@ -26100,7 +26100,7 @@
         </is>
       </c>
       <c r="E60" s="33" t="n">
-        <v>157.43</v>
+        <v>165.23</v>
       </c>
       <c r="F60" s="34" t="inlineStr">
         <is>
@@ -26116,7 +26116,7 @@
         </is>
       </c>
       <c r="I60" t="n">
-        <v>157.429993</v>
+        <v>165.229996</v>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="58">
@@ -26140,7 +26140,7 @@
         </is>
       </c>
       <c r="E61" s="33" t="n">
-        <v>233.38</v>
+        <v>221.2</v>
       </c>
       <c r="F61" s="34" t="inlineStr">
         <is>
@@ -26156,7 +26156,7 @@
         </is>
       </c>
       <c r="I61" t="n">
-        <v>233.380005</v>
+        <v>221.199997</v>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="58">
@@ -26180,7 +26180,7 @@
         </is>
       </c>
       <c r="E62" s="33" t="n">
-        <v>497.01</v>
+        <v>525.395</v>
       </c>
       <c r="F62" s="34" t="inlineStr">
         <is>
@@ -26196,7 +26196,7 @@
         </is>
       </c>
       <c r="I62" t="n">
-        <v>497.01001</v>
+        <v>525.39502</v>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1" s="58">
@@ -26220,7 +26220,7 @@
         </is>
       </c>
       <c r="E63" s="33" t="n">
-        <v>157.87</v>
+        <v>161.115</v>
       </c>
       <c r="F63" s="34" t="inlineStr">
         <is>
@@ -26236,7 +26236,7 @@
         </is>
       </c>
       <c r="I63" t="n">
-        <v>157.869995</v>
+        <v>161.115005</v>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="58">
@@ -26260,7 +26260,7 @@
         </is>
       </c>
       <c r="E64" s="33" t="n">
-        <v>50.57</v>
+        <v>51.89</v>
       </c>
       <c r="F64" s="34" t="inlineStr">
         <is>
@@ -26276,7 +26276,7 @@
         </is>
       </c>
       <c r="I64" t="n">
-        <v>50.57</v>
+        <v>51.889999</v>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1" s="58">
@@ -26300,7 +26300,7 @@
         </is>
       </c>
       <c r="E65" s="33" t="n">
-        <v>178.45</v>
+        <v>185.04</v>
       </c>
       <c r="F65" s="34" t="inlineStr">
         <is>
@@ -26316,7 +26316,7 @@
         </is>
       </c>
       <c r="I65" t="n">
-        <v>178.449997</v>
+        <v>185.039993</v>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1" s="58">
@@ -26340,7 +26340,7 @@
         </is>
       </c>
       <c r="E66" s="33" t="n">
-        <v>138.88</v>
+        <v>143</v>
       </c>
       <c r="F66" s="34" t="inlineStr">
         <is>
@@ -26380,7 +26380,7 @@
         </is>
       </c>
       <c r="E67" s="33" t="n">
-        <v>154.91</v>
+        <v>147.57</v>
       </c>
       <c r="F67" s="34" t="inlineStr">
         <is>
@@ -26396,7 +26396,7 @@
         </is>
       </c>
       <c r="I67" t="n">
-        <v>154.910004</v>
+        <v>147.570007</v>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1" s="58">
@@ -26420,7 +26420,7 @@
         </is>
       </c>
       <c r="E68" s="33" t="n">
-        <v>2135.64</v>
+        <v>2290.77</v>
       </c>
       <c r="F68" s="34" t="inlineStr">
         <is>
@@ -26436,7 +26436,7 @@
         </is>
       </c>
       <c r="I68" t="n">
-        <v>2135.639893</v>
+        <v>2290.77002</v>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="58">
@@ -26460,7 +26460,7 @@
         </is>
       </c>
       <c r="E69" s="33" t="n">
-        <v>1136.37</v>
+        <v>1166</v>
       </c>
       <c r="F69" s="34" t="inlineStr">
         <is>
@@ -26476,7 +26476,7 @@
         </is>
       </c>
       <c r="I69" t="n">
-        <v>1136.369995</v>
+        <v>1166.000244</v>
       </c>
     </row>
     <row r="70" ht="15" customHeight="1" s="58">
@@ -26500,7 +26500,7 @@
         </is>
       </c>
       <c r="E70" s="33" t="n">
-        <v>87.91</v>
+        <v>89.40000000000001</v>
       </c>
       <c r="F70" s="34" t="inlineStr">
         <is>
@@ -26516,7 +26516,7 @@
         </is>
       </c>
       <c r="I70" t="n">
-        <v>87.910004</v>
+        <v>89.400002</v>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1" s="58">
@@ -26540,7 +26540,7 @@
         </is>
       </c>
       <c r="E71" s="33" t="n">
-        <v>1473.04</v>
+        <v>1517.43</v>
       </c>
       <c r="F71" s="34" t="inlineStr">
         <is>
@@ -26556,7 +26556,7 @@
         </is>
       </c>
       <c r="I71" t="n">
-        <v>1473.040039</v>
+        <v>1517.430054</v>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1" s="58">
@@ -26580,7 +26580,7 @@
         </is>
       </c>
       <c r="E72" s="33" t="n">
-        <v>109.08</v>
+        <v>107.475</v>
       </c>
       <c r="F72" s="34" t="inlineStr">
         <is>
@@ -26596,7 +26596,7 @@
         </is>
       </c>
       <c r="I72" t="n">
-        <v>109.080002</v>
+        <v>107.474998</v>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1" s="58">
@@ -26620,7 +26620,7 @@
         </is>
       </c>
       <c r="E73" s="33" t="n">
-        <v>200.42</v>
+        <v>200.085</v>
       </c>
       <c r="F73" s="34" t="inlineStr">
         <is>
@@ -26636,7 +26636,7 @@
         </is>
       </c>
       <c r="I73" t="n">
-        <v>200.419998</v>
+        <v>200.085007</v>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1" s="58">
@@ -26660,7 +26660,7 @@
         </is>
       </c>
       <c r="E74" s="33" t="n">
-        <v>87.56999999999999</v>
+        <v>86.72</v>
       </c>
       <c r="F74" s="34" t="inlineStr">
         <is>
@@ -26676,7 +26676,7 @@
         </is>
       </c>
       <c r="I74" t="n">
-        <v>87.56999999999999</v>
+        <v>86.720001</v>
       </c>
     </row>
     <row r="75" ht="15" customHeight="1" s="58">
@@ -26700,7 +26700,7 @@
         </is>
       </c>
       <c r="E75" s="33" t="n">
-        <v>95</v>
+        <v>96.065</v>
       </c>
       <c r="F75" s="34" t="inlineStr">
         <is>
@@ -26716,7 +26716,7 @@
         </is>
       </c>
       <c r="I75" t="n">
-        <v>97.94000200000001</v>
+        <v>96.06500200000001</v>
       </c>
     </row>
     <row r="76" ht="15" customHeight="1" s="58">
@@ -26740,7 +26740,7 @@
         </is>
       </c>
       <c r="E76" s="33" t="n">
-        <v>347.59</v>
+        <v>362.65</v>
       </c>
       <c r="F76" s="34" t="inlineStr">
         <is>
@@ -26756,7 +26756,7 @@
         </is>
       </c>
       <c r="I76" t="n">
-        <v>347.589996</v>
+        <v>362.649994</v>
       </c>
     </row>
     <row r="77" ht="15" customHeight="1" s="58">
@@ -26780,7 +26780,7 @@
         </is>
       </c>
       <c r="E77" s="33" t="n">
-        <v>381.59</v>
+        <v>384.819</v>
       </c>
       <c r="F77" s="34" t="inlineStr">
         <is>
@@ -26796,7 +26796,7 @@
         </is>
       </c>
       <c r="I77" t="n">
-        <v>381.589996</v>
+        <v>384.819397</v>
       </c>
     </row>
     <row r="78" ht="15" customHeight="1" s="58">
@@ -26820,7 +26820,7 @@
         </is>
       </c>
       <c r="E78" s="33" t="n">
-        <v>51.97</v>
+        <v>51.57</v>
       </c>
       <c r="F78" s="34" t="inlineStr">
         <is>
@@ -26836,7 +26836,7 @@
         </is>
       </c>
       <c r="I78" t="n">
-        <v>51.970001</v>
+        <v>51.57</v>
       </c>
     </row>
     <row r="79" ht="15" customHeight="1" s="58">
@@ -26860,7 +26860,7 @@
         </is>
       </c>
       <c r="E79" s="33" t="n">
-        <v>85.13</v>
+        <v>89.14</v>
       </c>
       <c r="F79" s="34" t="inlineStr">
         <is>
@@ -26876,7 +26876,7 @@
         </is>
       </c>
       <c r="I79" t="n">
-        <v>85.129997</v>
+        <v>89.139999</v>
       </c>
     </row>
     <row r="80" ht="15" customHeight="1" s="58">
@@ -26900,7 +26900,7 @@
         </is>
       </c>
       <c r="E80" s="33" t="n">
-        <v>291.58</v>
+        <v>290.175</v>
       </c>
       <c r="F80" s="34" t="inlineStr">
         <is>
@@ -26916,7 +26916,7 @@
         </is>
       </c>
       <c r="I80" t="n">
-        <v>291.579987</v>
+        <v>290.174988</v>
       </c>
     </row>
     <row r="81" ht="15" customHeight="1" s="58">
@@ -26940,7 +26940,7 @@
         </is>
       </c>
       <c r="E81" s="33" t="n">
-        <v>153.97</v>
+        <v>154.73</v>
       </c>
       <c r="F81" s="34" t="inlineStr">
         <is>
@@ -26956,7 +26956,7 @@
         </is>
       </c>
       <c r="I81" t="n">
-        <v>153.970001</v>
+        <v>154.729996</v>
       </c>
     </row>
     <row r="82" ht="15" customHeight="1" s="58">
@@ -26980,7 +26980,7 @@
         </is>
       </c>
       <c r="E82" s="33" t="n">
-        <v>570.98</v>
+        <v>559.11</v>
       </c>
       <c r="F82" s="34" t="inlineStr">
         <is>
@@ -26996,7 +26996,7 @@
         </is>
       </c>
       <c r="I82" t="n">
-        <v>570.97998</v>
+        <v>559.1099850000001</v>
       </c>
     </row>
     <row r="83" ht="15" customHeight="1" s="58">
@@ -27020,7 +27020,7 @@
         </is>
       </c>
       <c r="E83" s="33" t="n">
-        <v>139.99</v>
+        <v>132</v>
       </c>
       <c r="F83" s="34" t="inlineStr">
         <is>
@@ -27060,7 +27060,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>62.21</v>
+        <v>62.9</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -27076,7 +27076,7 @@
         </is>
       </c>
       <c r="I84" t="n">
-        <v>62.344047</v>
+        <v>62.874274</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="58">
@@ -27100,7 +27100,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>591.73</v>
+        <v>597.67</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -27116,7 +27116,7 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>592.50805</v>
+        <v>593.679272</v>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="58">
@@ -27140,7 +27140,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>62104</v>
+        <v>62621</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -27156,7 +27156,7 @@
         </is>
       </c>
       <c r="I86" t="n">
-        <v>61796.727025</v>
+        <v>62241.829933</v>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="58">
@@ -27180,7 +27180,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.006445</v>
+        <v>0.006622</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -27196,7 +27196,7 @@
         </is>
       </c>
       <c r="I87" t="n">
-        <v>0.006782</v>
+        <v>0.006649</v>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="58">
@@ -27220,7 +27220,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.010345</v>
+        <v>0.010312</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -27236,7 +27236,7 @@
         </is>
       </c>
       <c r="I88" t="n">
-        <v>0.010714</v>
+        <v>0.010324</v>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="58">
@@ -27260,7 +27260,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>64.20999999999999</v>
+        <v>65.15000000000001</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -27276,7 +27276,7 @@
         </is>
       </c>
       <c r="I89" t="n">
-        <v>65.086533</v>
+        <v>64.99431199999999</v>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="58">
@@ -27300,7 +27300,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>1.65</v>
+        <v>1.71</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -27316,7 +27316,7 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>1.655745</v>
+        <v>1.674416</v>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="58">
@@ -27380,7 +27380,7 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
-        <v>0.013486</v>
+        <v>0.013575</v>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
@@ -27396,7 +27396,7 @@
         </is>
       </c>
       <c r="I92" t="n">
-        <v>0.013957</v>
+        <v>0.013841</v>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="58">
@@ -27420,7 +27420,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>2.572347</v>
+        <v>2.65522</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -27436,7 +27436,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>2.665431</v>
+        <v>2.649782</v>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="58">
@@ -27460,7 +27460,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>24.248774</v>
+        <v>24.603509</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -27476,7 +27476,7 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>24.790295</v>
+        <v>24.900178</v>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="58">
@@ -27500,7 +27500,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.108889</v>
+        <v>0.109976</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -27516,7 +27516,7 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>0.110444</v>
+        <v>0.111493</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="58">
@@ -27540,7 +27540,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>19444.2478</v>
+        <v>19711.1566</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -27556,7 +27556,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>19469.814527</v>
+        <v>19579.542394</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="58">
@@ -27580,7 +27580,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2040737.44</v>
+        <v>2065240.58</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -27596,7 +27596,7 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>2030640.450055</v>
+        <v>2052735.551204</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="58">
@@ -27620,7 +27620,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>2.758236</v>
+        <v>2.795781</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -27636,7 +27636,7 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>2.787017</v>
+        <v>2.787246</v>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="58">
@@ -27660,7 +27660,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>53865.0978</v>
+        <v>54079.9444</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -27676,7 +27676,7 @@
         </is>
       </c>
       <c r="I99" t="n">
-        <v>53899.43744</v>
+        <v>54357.657188</v>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="58">
@@ -27700,7 +27700,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>24.734806</v>
+        <v>25.169347</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -27716,7 +27716,7 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>25.062992</v>
+        <v>24.981841</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="58">
@@ -27740,7 +27740,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>62104</v>
+        <v>62621</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -27756,7 +27756,7 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>61796.727025</v>
+        <v>62241.829933</v>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="58">
@@ -27796,7 +27796,7 @@
         </is>
       </c>
       <c r="I102" t="n">
-        <v>18.86456</v>
+        <v>18.027189</v>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="58">
@@ -27894,7 +27894,7 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
-        <v>0.006445</v>
+        <v>0.006622</v>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
@@ -27910,7 +27910,7 @@
         </is>
       </c>
       <c r="I105" t="n">
-        <v>0.006782</v>
+        <v>0.006649</v>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="58">
@@ -27934,7 +27934,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>64.20999999999999</v>
+        <v>65.15000000000001</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>
@@ -27950,7 +27950,7 @@
         </is>
       </c>
       <c r="I106" t="n">
-        <v>65.086533</v>
+        <v>64.99431199999999</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="58">

</xml_diff>

<commit_message>
Daily dashboard update — 2026-06-12
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-42660" yWindow="-540" windowWidth="32460" windowHeight="17180" tabRatio="500" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Realized" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Prices" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Reference" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Realized" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="AsOfDate">'FX &amp; Assumptions'!$C$5</definedName>
@@ -697,14 +697,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -726,8 +726,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -752,10 +752,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -764,10 +764,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4F81BD"/>
               </a:solidFill>
-              <a:ln w="0">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -777,10 +777,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="C0504D"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -790,10 +790,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="9BBB59"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -803,10 +803,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="8064A2"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -816,10 +816,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4BACC6"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -829,10 +829,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="F79646"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -842,14 +842,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -875,14 +875,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -908,14 +908,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -941,14 +941,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -974,14 +974,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1007,14 +1007,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1038,16 +1038,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1142,16 +1142,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1172,10 +1172,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1187,14 +1187,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1216,8 +1216,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1242,10 +1242,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1254,10 +1254,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4672A8"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1267,10 +1267,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="AB4744"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1280,10 +1280,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="8AA64F"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1293,10 +1293,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="725990"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1306,10 +1306,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4299B0"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1319,10 +1319,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="DC853E"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1332,10 +1332,10 @@
             <idx val="6"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="93A9CE"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1345,10 +1345,10 @@
             <idx val="7"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="D09493"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1358,10 +1358,10 @@
             <idx val="8"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="B8CD97"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1371,14 +1371,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1405,14 +1405,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1439,14 +1439,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1473,14 +1473,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1507,14 +1507,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1541,14 +1541,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1575,14 +1575,14 @@
             <dLbl>
               <idx val="6"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1609,14 +1609,14 @@
             <dLbl>
               <idx val="7"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1643,14 +1643,14 @@
             <dLbl>
               <idx val="8"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1675,16 +1675,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1791,16 +1791,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1821,10 +1821,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1836,14 +1836,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1865,8 +1865,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1893,10 +1893,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1904,16 +1904,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2016,7 +2016,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2025,9 +2025,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2059,7 +2059,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="9360">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2073,7 +2073,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2082,9 +2082,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2109,16 +2109,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2139,10 +2139,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2154,14 +2154,14 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -2183,8 +2183,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -2200,10 +2200,10 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2211,16 +2211,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2411,7 +2411,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2420,9 +2420,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2454,7 +2454,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="9360">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2468,7 +2468,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2477,9 +2477,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2504,16 +2504,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2534,10 +2534,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2549,7 +2549,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>1</col>
@@ -2569,9 +2569,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2596,9 +2596,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2623,9 +2623,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId3"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2650,9 +2650,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId4"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -21860,28 +21860,28 @@
         <v>46185</v>
       </c>
       <c r="C16" s="29" t="n">
-        <v>25712637</v>
+        <v>25786746</v>
       </c>
       <c r="D16" s="29" t="n">
-        <v>22692689</v>
+        <v>22669464</v>
       </c>
       <c r="E16" s="29" t="n">
-        <v>3019948</v>
+        <v>3117282</v>
       </c>
       <c r="F16" s="30" t="n">
-        <v>0.1331</v>
+        <v>0.1375</v>
       </c>
       <c r="G16" s="29" t="n">
         <v>18286893</v>
       </c>
       <c r="H16" s="29" t="n">
-        <v>4905581</v>
+        <v>4982077</v>
       </c>
       <c r="I16" s="29" t="n">
-        <v>1149224</v>
+        <v>1154627</v>
       </c>
       <c r="J16" s="31" t="n">
-        <v>32.99</v>
+        <v>32.78</v>
       </c>
       <c r="K16" s="32" t="inlineStr">
         <is>
@@ -23592,7 +23592,7 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>32.99</v>
+        <v>32.78</v>
       </c>
       <c r="D6" s="64" t="inlineStr">
         <is>
@@ -23641,7 +23641,7 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>25.5918</v>
+        <v>25.5284</v>
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
@@ -25245,7 +25245,7 @@
         </is>
       </c>
       <c r="E38" s="33" t="n">
-        <v>23.16</v>
+        <v>23.23</v>
       </c>
       <c r="F38" s="34" t="inlineStr">
         <is>
@@ -25261,7 +25261,7 @@
         </is>
       </c>
       <c r="I38" t="n">
-        <v>23.16</v>
+        <v>23.23</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="58">
@@ -25301,7 +25301,7 @@
         </is>
       </c>
       <c r="I39" t="n">
-        <v>1.08</v>
+        <v>1.084</v>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="58">
@@ -25325,7 +25325,7 @@
         </is>
       </c>
       <c r="E40" s="33" t="n">
-        <v>753.37</v>
+        <v>746.08</v>
       </c>
       <c r="F40" s="34" t="inlineStr">
         <is>
@@ -25341,7 +25341,7 @@
         </is>
       </c>
       <c r="I40" t="n">
-        <v>753.369995</v>
+        <v>746.080017</v>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="58">
@@ -25365,7 +25365,7 @@
         </is>
       </c>
       <c r="E41" s="33" t="n">
-        <v>20.4</v>
+        <v>20.37</v>
       </c>
       <c r="F41" s="34" t="inlineStr">
         <is>
@@ -25381,7 +25381,7 @@
         </is>
       </c>
       <c r="I41" t="n">
-        <v>20.4</v>
+        <v>20.370001</v>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="58">
@@ -25405,7 +25405,7 @@
         </is>
       </c>
       <c r="E42" s="33" t="n">
-        <v>218.03</v>
+        <v>218.31</v>
       </c>
       <c r="F42" s="34" t="inlineStr">
         <is>
@@ -25421,7 +25421,7 @@
         </is>
       </c>
       <c r="I42" t="n">
-        <v>218.029999</v>
+        <v>218.309998</v>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="58">
@@ -25541,7 +25541,7 @@
         </is>
       </c>
       <c r="I45" t="n">
-        <v>0.44</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="58">
@@ -25778,7 +25778,7 @@
         </is>
       </c>
       <c r="I51" t="n">
-        <v>15.3</v>
+        <v>15.1</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" s="58">
@@ -25858,7 +25858,7 @@
         </is>
       </c>
       <c r="I53" t="n">
-        <v>5.35</v>
+        <v>5.45</v>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="58">
@@ -25898,7 +25898,7 @@
         </is>
       </c>
       <c r="I54" t="n">
-        <v>20.1</v>
+        <v>19.9</v>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="58">
@@ -25938,7 +25938,7 @@
         </is>
       </c>
       <c r="I55" t="n">
-        <v>3.5</v>
+        <v>3.54</v>
       </c>
     </row>
     <row r="56" ht="15" customHeight="1" s="58">
@@ -25978,7 +25978,7 @@
         </is>
       </c>
       <c r="I56" t="n">
-        <v>4.76</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1" s="58">
@@ -26018,7 +26018,7 @@
         </is>
       </c>
       <c r="I57" t="n">
-        <v>2.54</v>
+        <v>2.56</v>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="58">
@@ -26058,7 +26058,7 @@
         </is>
       </c>
       <c r="I58" t="n">
-        <v>12.1</v>
+        <v>11.9</v>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="58">
@@ -26122,7 +26122,7 @@
         </is>
       </c>
       <c r="E60" s="33" t="n">
-        <v>161.95</v>
+        <v>173.57</v>
       </c>
       <c r="F60" s="34" t="inlineStr">
         <is>
@@ -26138,7 +26138,7 @@
         </is>
       </c>
       <c r="I60" t="n">
-        <v>161.949997</v>
+        <v>173.570007</v>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="58">
@@ -26162,7 +26162,7 @@
         </is>
       </c>
       <c r="E61" s="33" t="n">
-        <v>222.31</v>
+        <v>218.8</v>
       </c>
       <c r="F61" s="34" t="inlineStr">
         <is>
@@ -26178,7 +26178,7 @@
         </is>
       </c>
       <c r="I61" t="n">
-        <v>222.309998</v>
+        <v>218.800003</v>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="58">
@@ -26202,7 +26202,7 @@
         </is>
       </c>
       <c r="E62" s="33" t="n">
-        <v>526.335</v>
+        <v>552.64</v>
       </c>
       <c r="F62" s="34" t="inlineStr">
         <is>
@@ -26218,7 +26218,7 @@
         </is>
       </c>
       <c r="I62" t="n">
-        <v>526.335022</v>
+        <v>552.6400149999999</v>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1" s="58">
@@ -26242,7 +26242,7 @@
         </is>
       </c>
       <c r="E63" s="33" t="n">
-        <v>158.07</v>
+        <v>162.93</v>
       </c>
       <c r="F63" s="34" t="inlineStr">
         <is>
@@ -26258,7 +26258,7 @@
         </is>
       </c>
       <c r="I63" t="n">
-        <v>158.070007</v>
+        <v>162.929993</v>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="58">
@@ -26282,7 +26282,7 @@
         </is>
       </c>
       <c r="E64" s="33" t="n">
-        <v>51.695</v>
+        <v>54.93</v>
       </c>
       <c r="F64" s="34" t="inlineStr">
         <is>
@@ -26298,7 +26298,7 @@
         </is>
       </c>
       <c r="I64" t="n">
-        <v>51.695</v>
+        <v>54.93</v>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1" s="58">
@@ -26322,7 +26322,7 @@
         </is>
       </c>
       <c r="E65" s="33" t="n">
-        <v>186.95</v>
+        <v>198.94</v>
       </c>
       <c r="F65" s="34" t="inlineStr">
         <is>
@@ -26338,7 +26338,7 @@
         </is>
       </c>
       <c r="I65" t="n">
-        <v>186.949997</v>
+        <v>198.940002</v>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1" s="58">
@@ -26362,7 +26362,7 @@
         </is>
       </c>
       <c r="E66" s="33" t="n">
-        <v>143.43</v>
+        <v>145.06</v>
       </c>
       <c r="F66" s="34" t="inlineStr">
         <is>
@@ -26378,7 +26378,7 @@
         </is>
       </c>
       <c r="I66" t="n">
-        <v>143.429993</v>
+        <v>145.059998</v>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1" s="58">
@@ -26402,7 +26402,7 @@
         </is>
       </c>
       <c r="E67" s="33" t="n">
-        <v>147.565</v>
+        <v>148.81</v>
       </c>
       <c r="F67" s="34" t="inlineStr">
         <is>
@@ -26418,7 +26418,7 @@
         </is>
       </c>
       <c r="I67" t="n">
-        <v>147.565002</v>
+        <v>148.809998</v>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1" s="58">
@@ -26442,7 +26442,7 @@
         </is>
       </c>
       <c r="E68" s="33" t="n">
-        <v>2297.585</v>
+        <v>2411.64</v>
       </c>
       <c r="F68" s="34" t="inlineStr">
         <is>
@@ -26458,7 +26458,7 @@
         </is>
       </c>
       <c r="I68" t="n">
-        <v>2297.584961</v>
+        <v>2411.639893</v>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="58">
@@ -26482,7 +26482,7 @@
         </is>
       </c>
       <c r="E69" s="33" t="n">
-        <v>1155</v>
+        <v>1160.95</v>
       </c>
       <c r="F69" s="34" t="inlineStr">
         <is>
@@ -26498,7 +26498,7 @@
         </is>
       </c>
       <c r="I69" t="n">
-        <v>1136.369995</v>
+        <v>1160.949951</v>
       </c>
     </row>
     <row r="70" ht="15" customHeight="1" s="58">
@@ -26522,7 +26522,7 @@
         </is>
       </c>
       <c r="E70" s="33" t="n">
-        <v>89.125</v>
+        <v>92.94</v>
       </c>
       <c r="F70" s="34" t="inlineStr">
         <is>
@@ -26538,7 +26538,7 @@
         </is>
       </c>
       <c r="I70" t="n">
-        <v>87.910004</v>
+        <v>92.94000200000001</v>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1" s="58">
@@ -26562,7 +26562,7 @@
         </is>
       </c>
       <c r="E71" s="33" t="n">
-        <v>1517.97</v>
+        <v>1589.55</v>
       </c>
       <c r="F71" s="34" t="inlineStr">
         <is>
@@ -26578,7 +26578,7 @@
         </is>
       </c>
       <c r="I71" t="n">
-        <v>1517.969971</v>
+        <v>1589.550049</v>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1" s="58">
@@ -26602,7 +26602,7 @@
         </is>
       </c>
       <c r="E72" s="33" t="n">
-        <v>108.195</v>
+        <v>110.58</v>
       </c>
       <c r="F72" s="34" t="inlineStr">
         <is>
@@ -26618,7 +26618,7 @@
         </is>
       </c>
       <c r="I72" t="n">
-        <v>108.195</v>
+        <v>110.580002</v>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1" s="58">
@@ -26642,7 +26642,7 @@
         </is>
       </c>
       <c r="E73" s="33" t="n">
-        <v>200.06</v>
+        <v>204.87</v>
       </c>
       <c r="F73" s="34" t="inlineStr">
         <is>
@@ -26658,7 +26658,7 @@
         </is>
       </c>
       <c r="I73" t="n">
-        <v>200.059998</v>
+        <v>204.869995</v>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1" s="58">
@@ -26682,7 +26682,7 @@
         </is>
       </c>
       <c r="E74" s="33" t="n">
-        <v>87.58</v>
+        <v>89.88</v>
       </c>
       <c r="F74" s="34" t="inlineStr">
         <is>
@@ -26698,7 +26698,7 @@
         </is>
       </c>
       <c r="I74" t="n">
-        <v>87.58000199999999</v>
+        <v>89.879997</v>
       </c>
     </row>
     <row r="75" ht="15" customHeight="1" s="58">
@@ -26722,7 +26722,7 @@
         </is>
       </c>
       <c r="E75" s="33" t="n">
-        <v>95.41</v>
+        <v>97.66</v>
       </c>
       <c r="F75" s="34" t="inlineStr">
         <is>
@@ -26738,7 +26738,7 @@
         </is>
       </c>
       <c r="I75" t="n">
-        <v>95.410004</v>
+        <v>97.660004</v>
       </c>
     </row>
     <row r="76" ht="15" customHeight="1" s="58">
@@ -26762,7 +26762,7 @@
         </is>
       </c>
       <c r="E76" s="33" t="n">
-        <v>359.6</v>
+        <v>381.4</v>
       </c>
       <c r="F76" s="34" t="inlineStr">
         <is>
@@ -26778,7 +26778,7 @@
         </is>
       </c>
       <c r="I76" t="n">
-        <v>359.600006</v>
+        <v>381.399994</v>
       </c>
     </row>
     <row r="77" ht="15" customHeight="1" s="58">
@@ -26802,7 +26802,7 @@
         </is>
       </c>
       <c r="E77" s="33" t="n">
-        <v>384.25</v>
+        <v>399.15</v>
       </c>
       <c r="F77" s="34" t="inlineStr">
         <is>
@@ -26818,7 +26818,7 @@
         </is>
       </c>
       <c r="I77" t="n">
-        <v>381.589996</v>
+        <v>399.149994</v>
       </c>
     </row>
     <row r="78" ht="15" customHeight="1" s="58">
@@ -26842,7 +26842,7 @@
         </is>
       </c>
       <c r="E78" s="33" t="n">
-        <v>51.15</v>
+        <v>51</v>
       </c>
       <c r="F78" s="34" t="inlineStr">
         <is>
@@ -26858,7 +26858,7 @@
         </is>
       </c>
       <c r="I78" t="n">
-        <v>51.150002</v>
+        <v>51.970001</v>
       </c>
     </row>
     <row r="79" ht="15" customHeight="1" s="58">
@@ -26882,7 +26882,7 @@
         </is>
       </c>
       <c r="E79" s="33" t="n">
-        <v>90.065</v>
+        <v>92.95999999999999</v>
       </c>
       <c r="F79" s="34" t="inlineStr">
         <is>
@@ -26898,7 +26898,7 @@
         </is>
       </c>
       <c r="I79" t="n">
-        <v>90.06500200000001</v>
+        <v>92.959999</v>
       </c>
     </row>
     <row r="80" ht="15" customHeight="1" s="58">
@@ -26922,7 +26922,7 @@
         </is>
       </c>
       <c r="E80" s="33" t="n">
-        <v>293.245</v>
+        <v>295.63</v>
       </c>
       <c r="F80" s="34" t="inlineStr">
         <is>
@@ -26938,7 +26938,7 @@
         </is>
       </c>
       <c r="I80" t="n">
-        <v>293.244995</v>
+        <v>295.630005</v>
       </c>
     </row>
     <row r="81" ht="15" customHeight="1" s="58">
@@ -26962,7 +26962,7 @@
         </is>
       </c>
       <c r="E81" s="33" t="n">
-        <v>153.07</v>
+        <v>160.43</v>
       </c>
       <c r="F81" s="34" t="inlineStr">
         <is>
@@ -26978,7 +26978,7 @@
         </is>
       </c>
       <c r="I81" t="n">
-        <v>153.070007</v>
+        <v>160.429993</v>
       </c>
     </row>
     <row r="82" ht="15" customHeight="1" s="58">
@@ -27002,7 +27002,7 @@
         </is>
       </c>
       <c r="E82" s="33" t="n">
-        <v>558.1900000000001</v>
+        <v>568.4299999999999</v>
       </c>
       <c r="F82" s="34" t="inlineStr">
         <is>
@@ -27018,7 +27018,7 @@
         </is>
       </c>
       <c r="I82" t="n">
-        <v>558.190002</v>
+        <v>568.429993</v>
       </c>
     </row>
     <row r="83" ht="15" customHeight="1" s="58">
@@ -27042,7 +27042,7 @@
         </is>
       </c>
       <c r="E83" s="33" t="n">
-        <v>122.26</v>
+        <v>122.34</v>
       </c>
       <c r="F83" s="34" t="inlineStr">
         <is>
@@ -27058,7 +27058,7 @@
         </is>
       </c>
       <c r="I83" t="n">
-        <v>122.260002</v>
+        <v>122.339996</v>
       </c>
     </row>
     <row r="84" ht="15" customHeight="1" s="58">
@@ -27082,7 +27082,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>63.09</v>
+        <v>63.96</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -27098,7 +27098,7 @@
         </is>
       </c>
       <c r="I84" t="n">
-        <v>62.611744</v>
+        <v>62.224742</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="58">
@@ -27122,7 +27122,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>597.95</v>
+        <v>601.4299999999999</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -27138,7 +27138,7 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>593.162188</v>
+        <v>591.367193</v>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="58">
@@ -27162,7 +27162,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>62511</v>
+        <v>63283</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -27178,7 +27178,7 @@
         </is>
       </c>
       <c r="I86" t="n">
-        <v>62258.562598</v>
+        <v>62102.478221</v>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="58">
@@ -27202,7 +27202,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.006626</v>
+        <v>0.006732</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -27218,7 +27218,7 @@
         </is>
       </c>
       <c r="I87" t="n">
-        <v>0.00658</v>
+        <v>0.006445</v>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="58">
@@ -27242,7 +27242,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.010232</v>
+        <v>0.010342</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -27258,7 +27258,7 @@
         </is>
       </c>
       <c r="I88" t="n">
-        <v>0.010075</v>
+        <v>0.010348</v>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="58">
@@ -27282,7 +27282,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>65.33</v>
+        <v>66.48</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -27298,7 +27298,7 @@
         </is>
       </c>
       <c r="I89" t="n">
-        <v>64.72349699999999</v>
+        <v>64.218192</v>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="58">
@@ -27322,7 +27322,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>1.71</v>
+        <v>1.74</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -27338,7 +27338,7 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>1.659099</v>
+        <v>1.652761</v>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="58">
@@ -27402,7 +27402,7 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
-        <v>0.013538</v>
+        <v>0.013764</v>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
@@ -27418,7 +27418,7 @@
         </is>
       </c>
       <c r="I92" t="n">
-        <v>0.013694</v>
+        <v>0.013483</v>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="58">
@@ -27442,7 +27442,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>2.645765</v>
+        <v>2.705628</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -27458,7 +27458,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>2.615126</v>
+        <v>2.566067</v>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="58">
@@ -27482,7 +27482,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>24.613311</v>
+        <v>24.531733</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -27498,7 +27498,7 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>24.444824</v>
+        <v>24.195297</v>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="58">
@@ -27522,7 +27522,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.10988</v>
+        <v>0.112923</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -27538,7 +27538,7 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>0.110713</v>
+        <v>0.108688</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="58">
@@ -27562,7 +27562,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>19726.3705</v>
+        <v>19714.8754</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -27578,7 +27578,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>19568.420574</v>
+        <v>19385.016583</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="58">
@@ -27602,7 +27602,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2062237.89</v>
+        <v>2074416.74</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -27618,7 +27618,7 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>2053909.980124</v>
+        <v>2035719.236083</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="58">
@@ -27642,7 +27642,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>2.792735</v>
+        <v>2.809672</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -27658,7 +27658,7 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>2.776927</v>
+        <v>2.752047</v>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="58">
@@ -27682,7 +27682,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>54047.517</v>
+        <v>54461.6754</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -27698,7 +27698,7 @@
         </is>
       </c>
       <c r="I99" t="n">
-        <v>54078.794087</v>
+        <v>53728.723039</v>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="58">
@@ -27722,7 +27722,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>25.156228</v>
+        <v>25.230307</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -27738,7 +27738,7 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>24.951689</v>
+        <v>24.674611</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="58">
@@ -27762,7 +27762,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>62511</v>
+        <v>63283</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -27778,7 +27778,7 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>62258.562598</v>
+        <v>62102.478221</v>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="58">
@@ -27802,7 +27802,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>17.6</v>
+        <v>17.69</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -27818,7 +27818,7 @@
         </is>
       </c>
       <c r="I102" t="n">
-        <v>17.817585</v>
+        <v>17.702621</v>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="58">
@@ -27916,7 +27916,7 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
-        <v>0.006626</v>
+        <v>0.006732</v>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
@@ -27932,7 +27932,7 @@
         </is>
       </c>
       <c r="I105" t="n">
-        <v>0.00658</v>
+        <v>0.006445</v>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="58">
@@ -27956,7 +27956,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>65.33</v>
+        <v>66.48</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>
@@ -27972,7 +27972,7 @@
         </is>
       </c>
       <c r="I106" t="n">
-        <v>64.72349699999999</v>
+        <v>64.218192</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="58">

</xml_diff>

<commit_message>
Weekly dashboard update — 2026-06-12
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-42660" yWindow="-540" windowWidth="32460" windowHeight="17180" tabRatio="500" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Realized" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Realized" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Prices" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Reference" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="AsOfDate">'FX &amp; Assumptions'!$C$5</definedName>
@@ -697,14 +697,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -726,8 +726,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -752,10 +752,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -764,10 +764,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4F81BD"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+              <a:ln w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -777,10 +777,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="C0504D"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -790,10 +790,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="9BBB59"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -803,10 +803,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="8064A2"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -816,10 +816,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4BACC6"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -829,10 +829,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="F79646"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -842,14 +842,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -875,14 +875,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -908,14 +908,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -941,14 +941,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -974,14 +974,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1007,14 +1007,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1038,16 +1038,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1142,16 +1142,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1172,10 +1172,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1187,14 +1187,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1216,8 +1216,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1242,10 +1242,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1254,10 +1254,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4672A8"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1267,10 +1267,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="AB4744"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1280,10 +1280,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="8AA64F"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1293,10 +1293,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="725990"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1306,10 +1306,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4299B0"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1319,10 +1319,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="DC853E"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1332,10 +1332,10 @@
             <idx val="6"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="93A9CE"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1345,10 +1345,10 @@
             <idx val="7"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="D09493"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1358,10 +1358,10 @@
             <idx val="8"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="B8CD97"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1371,14 +1371,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1405,14 +1405,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1439,14 +1439,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1473,14 +1473,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1507,14 +1507,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1541,14 +1541,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1575,14 +1575,14 @@
             <dLbl>
               <idx val="6"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1609,14 +1609,14 @@
             <dLbl>
               <idx val="7"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1643,14 +1643,14 @@
             <dLbl>
               <idx val="8"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1675,16 +1675,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1791,16 +1791,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1821,10 +1821,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1836,14 +1836,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1865,8 +1865,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1893,10 +1893,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1904,16 +1904,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2016,7 +2016,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2025,9 +2025,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2059,7 +2059,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2073,7 +2073,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2082,9 +2082,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2109,16 +2109,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2139,10 +2139,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2154,14 +2154,14 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -2183,8 +2183,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -2200,10 +2200,10 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2211,16 +2211,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2411,7 +2411,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2420,9 +2420,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2454,7 +2454,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2468,7 +2468,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2477,9 +2477,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2504,16 +2504,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2534,10 +2534,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2549,7 +2549,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>1</col>
@@ -2569,9 +2569,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2596,9 +2596,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+          <c:chart r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2623,9 +2623,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+          <c:chart r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2650,9 +2650,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+          <c:chart r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -21860,28 +21860,28 @@
         <v>46185</v>
       </c>
       <c r="C16" s="29" t="n">
-        <v>25786746</v>
+        <v>25590702</v>
       </c>
       <c r="D16" s="29" t="n">
-        <v>22669464</v>
+        <v>22662084</v>
       </c>
       <c r="E16" s="29" t="n">
-        <v>3117282</v>
+        <v>2928619</v>
       </c>
       <c r="F16" s="30" t="n">
-        <v>0.1375</v>
+        <v>0.1292</v>
       </c>
       <c r="G16" s="29" t="n">
-        <v>18286893</v>
+        <v>18073880</v>
       </c>
       <c r="H16" s="29" t="n">
-        <v>4982077</v>
+        <v>4998877</v>
       </c>
       <c r="I16" s="29" t="n">
-        <v>1154627</v>
+        <v>1155978</v>
       </c>
       <c r="J16" s="31" t="n">
-        <v>32.78</v>
+        <v>32.72</v>
       </c>
       <c r="K16" s="32" t="inlineStr">
         <is>
@@ -23592,7 +23592,7 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>32.78</v>
+        <v>32.72</v>
       </c>
       <c r="D6" s="64" t="inlineStr">
         <is>
@@ -23641,7 +23641,7 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>25.5284</v>
+        <v>25.4878</v>
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
@@ -23760,27 +23760,27 @@
         </is>
       </c>
       <c r="E5" s="33" t="n">
+        <v>23.4501</v>
+      </c>
+      <c r="F5" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G5" s="28" t="n">
+        <v>46183</v>
+      </c>
+      <c r="H5" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
         <v>23.9719</v>
       </c>
-      <c r="F5" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G5" s="28" t="n">
-        <v>46182</v>
-      </c>
-      <c r="H5" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I5" t="n">
-        <v>24.4495</v>
-      </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
     </row>
@@ -23805,27 +23805,27 @@
         </is>
       </c>
       <c r="E6" s="33" t="n">
+        <v>10.6872</v>
+      </c>
+      <c r="F6" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G6" s="28" t="n">
+        <v>46184</v>
+      </c>
+      <c r="H6" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
         <v>10.687</v>
       </c>
-      <c r="F6" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G6" s="28" t="n">
-        <v>46183</v>
-      </c>
-      <c r="H6" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I6" t="n">
-        <v>10.6868</v>
-      </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
     </row>
@@ -23850,27 +23850,27 @@
         </is>
       </c>
       <c r="E7" s="33" t="n">
+        <v>7.0666</v>
+      </c>
+      <c r="F7" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G7" s="28" t="n">
+        <v>46183</v>
+      </c>
+      <c r="H7" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
         <v>7.0939</v>
       </c>
-      <c r="F7" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G7" s="28" t="n">
-        <v>46182</v>
-      </c>
-      <c r="H7" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I7" t="n">
-        <v>7.0857</v>
-      </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
     </row>
@@ -23895,27 +23895,27 @@
         </is>
       </c>
       <c r="E8" s="33" t="n">
+        <v>9.3483</v>
+      </c>
+      <c r="F8" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G8" s="28" t="n">
+        <v>46183</v>
+      </c>
+      <c r="H8" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
         <v>9.4916</v>
       </c>
-      <c r="F8" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G8" s="28" t="n">
-        <v>46182</v>
-      </c>
-      <c r="H8" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I8" t="n">
-        <v>9.2986</v>
-      </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
     </row>
@@ -23940,27 +23940,27 @@
         </is>
       </c>
       <c r="E9" s="33" t="n">
+        <v>9.2189</v>
+      </c>
+      <c r="F9" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G9" s="28" t="n">
+        <v>46184</v>
+      </c>
+      <c r="H9" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
         <v>9.1568</v>
       </c>
-      <c r="F9" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G9" s="28" t="n">
-        <v>46183</v>
-      </c>
-      <c r="H9" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I9" t="n">
-        <v>9.2889</v>
-      </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
     </row>
@@ -23985,27 +23985,27 @@
         </is>
       </c>
       <c r="E10" s="33" t="n">
+        <v>12.9779</v>
+      </c>
+      <c r="F10" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G10" s="28" t="n">
+        <v>46183</v>
+      </c>
+      <c r="H10" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
         <v>13.2756</v>
       </c>
-      <c r="F10" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G10" s="28" t="n">
-        <v>46182</v>
-      </c>
-      <c r="H10" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I10" t="n">
-        <v>13.0438</v>
-      </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
     </row>
@@ -24030,27 +24030,27 @@
         </is>
       </c>
       <c r="E11" s="33" t="n">
+        <v>13.0418</v>
+      </c>
+      <c r="F11" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G11" s="28" t="n">
+        <v>46184</v>
+      </c>
+      <c r="H11" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
         <v>12.894</v>
       </c>
-      <c r="F11" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G11" s="28" t="n">
-        <v>46183</v>
-      </c>
-      <c r="H11" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I11" t="n">
-        <v>13.1546</v>
-      </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
     </row>
@@ -24075,27 +24075,27 @@
         </is>
       </c>
       <c r="E12" s="33" t="n">
+        <v>26.2924</v>
+      </c>
+      <c r="F12" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G12" s="28" t="n">
+        <v>46184</v>
+      </c>
+      <c r="H12" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
         <v>25.8795</v>
       </c>
-      <c r="F12" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G12" s="28" t="n">
-        <v>46183</v>
-      </c>
-      <c r="H12" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I12" t="n">
-        <v>26.6235</v>
-      </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
     </row>
@@ -24120,27 +24120,27 @@
         </is>
       </c>
       <c r="E13" s="33" t="n">
+        <v>36.0361</v>
+      </c>
+      <c r="F13" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G13" s="28" t="n">
+        <v>46184</v>
+      </c>
+      <c r="H13" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
         <v>35.8529</v>
       </c>
-      <c r="F13" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G13" s="28" t="n">
-        <v>46183</v>
-      </c>
-      <c r="H13" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I13" t="n">
-        <v>36.2939</v>
-      </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
     </row>
@@ -24165,27 +24165,27 @@
         </is>
       </c>
       <c r="E14" s="33" t="n">
+        <v>25.2656</v>
+      </c>
+      <c r="F14" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G14" s="28" t="n">
+        <v>46184</v>
+      </c>
+      <c r="H14" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
         <v>25.1917</v>
       </c>
-      <c r="F14" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G14" s="28" t="n">
-        <v>46183</v>
-      </c>
-      <c r="H14" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I14" t="n">
-        <v>25.3708</v>
-      </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
     </row>
@@ -24210,27 +24210,27 @@
         </is>
       </c>
       <c r="E15" s="33" t="n">
+        <v>15.0551</v>
+      </c>
+      <c r="F15" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G15" s="28" t="n">
+        <v>46182</v>
+      </c>
+      <c r="H15" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
         <v>14.8604</v>
       </c>
-      <c r="F15" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G15" s="28" t="n">
-        <v>46181</v>
-      </c>
-      <c r="H15" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I15" t="n">
-        <v>14.8466</v>
-      </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
     </row>
@@ -24255,27 +24255,27 @@
         </is>
       </c>
       <c r="E16" s="33" t="n">
+        <v>80.91589999999999</v>
+      </c>
+      <c r="F16" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G16" s="28" t="n">
+        <v>46184</v>
+      </c>
+      <c r="H16" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
         <v>80.4905</v>
       </c>
-      <c r="F16" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G16" s="28" t="n">
-        <v>46183</v>
-      </c>
-      <c r="H16" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I16" t="n">
-        <v>81.4269</v>
-      </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
     </row>
@@ -24300,27 +24300,27 @@
         </is>
       </c>
       <c r="E17" s="33" t="n">
+        <v>52.8716</v>
+      </c>
+      <c r="F17" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G17" s="28" t="n">
+        <v>46184</v>
+      </c>
+      <c r="H17" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
         <v>52.7619</v>
       </c>
-      <c r="F17" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G17" s="28" t="n">
-        <v>46183</v>
-      </c>
-      <c r="H17" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I17" t="n">
-        <v>53.1377</v>
-      </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
     </row>
@@ -24345,27 +24345,27 @@
         </is>
       </c>
       <c r="E18" s="33" t="n">
+        <v>16.4428</v>
+      </c>
+      <c r="F18" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G18" s="28" t="n">
+        <v>46184</v>
+      </c>
+      <c r="H18" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
         <v>16.4301</v>
       </c>
-      <c r="F18" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G18" s="28" t="n">
-        <v>46183</v>
-      </c>
-      <c r="H18" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I18" t="n">
-        <v>16.4125</v>
-      </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
     </row>
@@ -24390,27 +24390,27 @@
         </is>
       </c>
       <c r="E19" s="33" t="n">
+        <v>23.4043</v>
+      </c>
+      <c r="F19" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G19" s="28" t="n">
+        <v>46184</v>
+      </c>
+      <c r="H19" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
         <v>23.4039</v>
       </c>
-      <c r="F19" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G19" s="28" t="n">
-        <v>46183</v>
-      </c>
-      <c r="H19" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I19" t="n">
-        <v>23.4031</v>
-      </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
     </row>
@@ -24435,27 +24435,27 @@
         </is>
       </c>
       <c r="E20" s="33" t="n">
+        <v>39.919</v>
+      </c>
+      <c r="F20" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G20" s="28" t="n">
+        <v>46183</v>
+      </c>
+      <c r="H20" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
         <v>40.563</v>
       </c>
-      <c r="F20" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G20" s="28" t="n">
-        <v>46182</v>
-      </c>
-      <c r="H20" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I20" t="n">
-        <v>40.6754</v>
-      </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
     </row>
@@ -24480,27 +24480,27 @@
         </is>
       </c>
       <c r="E21" s="33" t="n">
+        <v>13.2943</v>
+      </c>
+      <c r="F21" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G21" s="28" t="n">
+        <v>46184</v>
+      </c>
+      <c r="H21" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
         <v>13.3396</v>
       </c>
-      <c r="F21" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G21" s="28" t="n">
-        <v>46183</v>
-      </c>
-      <c r="H21" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I21" t="n">
-        <v>13.3598</v>
-      </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
     </row>
@@ -24525,27 +24525,27 @@
         </is>
       </c>
       <c r="E22" s="33" t="n">
+        <v>13.3451</v>
+      </c>
+      <c r="F22" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G22" s="28" t="n">
+        <v>46183</v>
+      </c>
+      <c r="H22" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
         <v>13.2159</v>
       </c>
-      <c r="F22" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G22" s="28" t="n">
-        <v>46182</v>
-      </c>
-      <c r="H22" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I22" t="n">
-        <v>13.215</v>
-      </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
     </row>
@@ -24570,27 +24570,27 @@
         </is>
       </c>
       <c r="E23" s="33" t="n">
+        <v>12.299</v>
+      </c>
+      <c r="F23" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G23" s="28" t="n">
+        <v>46184</v>
+      </c>
+      <c r="H23" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
         <v>12.2493</v>
       </c>
-      <c r="F23" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G23" s="28" t="n">
-        <v>46183</v>
-      </c>
-      <c r="H23" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I23" t="n">
-        <v>12.3772</v>
-      </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
     </row>
@@ -24615,27 +24615,27 @@
         </is>
       </c>
       <c r="E24" s="33" t="n">
+        <v>11.6527</v>
+      </c>
+      <c r="F24" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G24" s="28" t="n">
+        <v>46183</v>
+      </c>
+      <c r="H24" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
         <v>11.8802</v>
       </c>
-      <c r="F24" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G24" s="28" t="n">
-        <v>46182</v>
-      </c>
-      <c r="H24" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I24" t="n">
-        <v>11.827</v>
-      </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
     </row>
@@ -24660,27 +24660,27 @@
         </is>
       </c>
       <c r="E25" s="33" t="n">
+        <v>9.909700000000001</v>
+      </c>
+      <c r="F25" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G25" s="28" t="n">
+        <v>46184</v>
+      </c>
+      <c r="H25" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
         <v>9.9718</v>
       </c>
-      <c r="F25" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G25" s="28" t="n">
-        <v>46183</v>
-      </c>
-      <c r="H25" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I25" t="n">
-        <v>9.9245</v>
-      </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
     </row>
@@ -24705,27 +24705,27 @@
         </is>
       </c>
       <c r="E26" s="33" t="n">
+        <v>13.909</v>
+      </c>
+      <c r="F26" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G26" s="28" t="n">
+        <v>46184</v>
+      </c>
+      <c r="H26" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
         <v>14.002</v>
       </c>
-      <c r="F26" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G26" s="28" t="n">
-        <v>46183</v>
-      </c>
-      <c r="H26" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I26" t="n">
-        <v>13.9301</v>
-      </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
     </row>
@@ -24750,27 +24750,27 @@
         </is>
       </c>
       <c r="E27" s="33" t="n">
+        <v>16.7383</v>
+      </c>
+      <c r="F27" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G27" s="28" t="n">
+        <v>46184</v>
+      </c>
+      <c r="H27" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
         <v>16.7307</v>
       </c>
-      <c r="F27" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G27" s="28" t="n">
-        <v>46183</v>
-      </c>
-      <c r="H27" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I27" t="n">
-        <v>16.8932</v>
-      </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
     </row>
@@ -24795,27 +24795,27 @@
         </is>
       </c>
       <c r="E28" s="33" t="n">
+        <v>18.1673</v>
+      </c>
+      <c r="F28" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G28" s="28" t="n">
+        <v>46184</v>
+      </c>
+      <c r="H28" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
         <v>18.5085</v>
       </c>
-      <c r="F28" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G28" s="28" t="n">
-        <v>46183</v>
-      </c>
-      <c r="H28" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I28" t="n">
-        <v>19.2336</v>
-      </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
     </row>
@@ -24840,27 +24840,27 @@
         </is>
       </c>
       <c r="E29" s="33" t="n">
+        <v>24.2974</v>
+      </c>
+      <c r="F29" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G29" s="28" t="n">
+        <v>46183</v>
+      </c>
+      <c r="H29" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
         <v>25.0651</v>
       </c>
-      <c r="F29" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G29" s="28" t="n">
-        <v>46182</v>
-      </c>
-      <c r="H29" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I29" t="n">
-        <v>25.2898</v>
-      </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
     </row>
@@ -24885,27 +24885,27 @@
         </is>
       </c>
       <c r="E30" s="33" t="n">
+        <v>36.0272</v>
+      </c>
+      <c r="F30" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G30" s="28" t="n">
+        <v>46183</v>
+      </c>
+      <c r="H30" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
         <v>36.0558</v>
       </c>
-      <c r="F30" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G30" s="28" t="n">
-        <v>46182</v>
-      </c>
-      <c r="H30" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I30" t="n">
-        <v>37.4218</v>
-      </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
     </row>
@@ -24930,27 +24930,27 @@
         </is>
       </c>
       <c r="E31" s="33" t="n">
+        <v>12.8526</v>
+      </c>
+      <c r="F31" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G31" s="28" t="n">
+        <v>46184</v>
+      </c>
+      <c r="H31" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
         <v>12.7851</v>
       </c>
-      <c r="F31" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G31" s="28" t="n">
-        <v>46183</v>
-      </c>
-      <c r="H31" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I31" t="n">
-        <v>12.9477</v>
-      </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
     </row>
@@ -24975,27 +24975,27 @@
         </is>
       </c>
       <c r="E32" s="33" t="n">
+        <v>21.7059</v>
+      </c>
+      <c r="F32" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G32" s="28" t="n">
+        <v>46184</v>
+      </c>
+      <c r="H32" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
         <v>21.7057</v>
       </c>
-      <c r="F32" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G32" s="28" t="n">
-        <v>46183</v>
-      </c>
-      <c r="H32" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I32" t="n">
-        <v>21.7055</v>
-      </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
     </row>
@@ -25020,27 +25020,27 @@
         </is>
       </c>
       <c r="E33" s="33" t="n">
+        <v>12.4116</v>
+      </c>
+      <c r="F33" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G33" s="28" t="n">
+        <v>46184</v>
+      </c>
+      <c r="H33" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
         <v>12.3702</v>
       </c>
-      <c r="F33" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G33" s="28" t="n">
-        <v>46183</v>
-      </c>
-      <c r="H33" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I33" t="n">
-        <v>12.5043</v>
-      </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
     </row>
@@ -25065,27 +25065,27 @@
         </is>
       </c>
       <c r="E34" s="33" t="n">
+        <v>16.2054</v>
+      </c>
+      <c r="F34" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G34" s="28" t="n">
+        <v>46184</v>
+      </c>
+      <c r="H34" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
         <v>16.205</v>
       </c>
-      <c r="F34" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G34" s="28" t="n">
-        <v>46183</v>
-      </c>
-      <c r="H34" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I34" t="n">
-        <v>16.2045</v>
-      </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
     </row>
@@ -25110,27 +25110,27 @@
         </is>
       </c>
       <c r="E35" s="33" t="n">
+        <v>26.542</v>
+      </c>
+      <c r="F35" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G35" s="28" t="n">
+        <v>46183</v>
+      </c>
+      <c r="H35" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
         <v>27.6474</v>
       </c>
-      <c r="F35" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G35" s="28" t="n">
-        <v>46182</v>
-      </c>
-      <c r="H35" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I35" t="n">
-        <v>28.1255</v>
-      </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
     </row>
@@ -25155,27 +25155,27 @@
         </is>
       </c>
       <c r="E36" s="33" t="n">
+        <v>10.0297</v>
+      </c>
+      <c r="F36" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G36" s="28" t="n">
+        <v>46184</v>
+      </c>
+      <c r="H36" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
         <v>9.995900000000001</v>
       </c>
-      <c r="F36" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G36" s="28" t="n">
-        <v>46183</v>
-      </c>
-      <c r="H36" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I36" t="n">
-        <v>9.9649</v>
-      </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
     </row>
@@ -25200,27 +25200,27 @@
         </is>
       </c>
       <c r="E37" s="33" t="n">
+        <v>22.4356</v>
+      </c>
+      <c r="F37" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G37" s="28" t="n">
+        <v>46184</v>
+      </c>
+      <c r="H37" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
         <v>22.3085</v>
       </c>
-      <c r="F37" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G37" s="28" t="n">
-        <v>46183</v>
-      </c>
-      <c r="H37" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I37" t="n">
-        <v>22.5842</v>
-      </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
     </row>
@@ -25285,7 +25285,7 @@
         </is>
       </c>
       <c r="E39" s="33" t="n">
-        <v>1.08</v>
+        <v>1.084</v>
       </c>
       <c r="F39" s="34" t="inlineStr">
         <is>
@@ -25485,7 +25485,7 @@
         </is>
       </c>
       <c r="E44" s="33" t="n">
-        <v>168.5</v>
+        <v>172.5</v>
       </c>
       <c r="F44" s="34" t="inlineStr">
         <is>
@@ -25501,7 +25501,7 @@
         </is>
       </c>
       <c r="I44" t="n">
-        <v>169</v>
+        <v>168.5</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="58">
@@ -25565,7 +25565,7 @@
         </is>
       </c>
       <c r="E46" s="33" t="n">
-        <v>0.29</v>
+        <v>0.3</v>
       </c>
       <c r="F46" s="34" t="inlineStr">
         <is>
@@ -25581,7 +25581,7 @@
         </is>
       </c>
       <c r="I46" t="n">
-        <v>0.29</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" s="58">
@@ -25682,7 +25682,7 @@
         </is>
       </c>
       <c r="E49" s="33" t="n">
-        <v>62.75</v>
+        <v>64</v>
       </c>
       <c r="F49" s="34" t="inlineStr">
         <is>
@@ -25698,7 +25698,7 @@
         </is>
       </c>
       <c r="I49" t="n">
-        <v>63</v>
+        <v>62.75</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="58">
@@ -25722,7 +25722,7 @@
         </is>
       </c>
       <c r="E50" s="33" t="n">
-        <v>9.25</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="F50" s="34" t="inlineStr">
         <is>
@@ -25738,7 +25738,7 @@
         </is>
       </c>
       <c r="I50" t="n">
-        <v>9.4</v>
+        <v>9.300000000000001</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="58">
@@ -25762,7 +25762,7 @@
         </is>
       </c>
       <c r="E51" s="33" t="n">
-        <v>15.1</v>
+        <v>15.3</v>
       </c>
       <c r="F51" s="34" t="inlineStr">
         <is>
@@ -25778,7 +25778,7 @@
         </is>
       </c>
       <c r="I51" t="n">
-        <v>15.1</v>
+        <v>15.3</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" s="58">
@@ -25842,7 +25842,7 @@
         </is>
       </c>
       <c r="E53" s="33" t="n">
-        <v>5.45</v>
+        <v>5.55</v>
       </c>
       <c r="F53" s="34" t="inlineStr">
         <is>
@@ -25858,7 +25858,7 @@
         </is>
       </c>
       <c r="I53" t="n">
-        <v>5.45</v>
+        <v>5.55</v>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="58">
@@ -25882,7 +25882,7 @@
         </is>
       </c>
       <c r="E54" s="33" t="n">
-        <v>19.9</v>
+        <v>20.4</v>
       </c>
       <c r="F54" s="34" t="inlineStr">
         <is>
@@ -25898,7 +25898,7 @@
         </is>
       </c>
       <c r="I54" t="n">
-        <v>19.9</v>
+        <v>20.4</v>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="58">
@@ -25962,7 +25962,7 @@
         </is>
       </c>
       <c r="E56" s="33" t="n">
-        <v>4.8</v>
+        <v>4.84</v>
       </c>
       <c r="F56" s="34" t="inlineStr">
         <is>
@@ -25978,7 +25978,7 @@
         </is>
       </c>
       <c r="I56" t="n">
-        <v>4.8</v>
+        <v>4.84</v>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1" s="58">
@@ -26002,7 +26002,7 @@
         </is>
       </c>
       <c r="E57" s="33" t="n">
-        <v>2.56</v>
+        <v>2.62</v>
       </c>
       <c r="F57" s="34" t="inlineStr">
         <is>
@@ -26018,7 +26018,7 @@
         </is>
       </c>
       <c r="I57" t="n">
-        <v>2.56</v>
+        <v>2.62</v>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="58">
@@ -26042,7 +26042,7 @@
         </is>
       </c>
       <c r="E58" s="33" t="n">
-        <v>11.9</v>
+        <v>12.1</v>
       </c>
       <c r="F58" s="34" t="inlineStr">
         <is>
@@ -26058,7 +26058,7 @@
         </is>
       </c>
       <c r="I58" t="n">
-        <v>11.9</v>
+        <v>12.1</v>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="58">
@@ -26082,7 +26082,7 @@
         </is>
       </c>
       <c r="E59" s="33" t="n">
-        <v>16.5</v>
+        <v>17.3</v>
       </c>
       <c r="F59" s="34" t="inlineStr">
         <is>
@@ -26098,7 +26098,7 @@
         </is>
       </c>
       <c r="I59" t="n">
-        <v>16.6</v>
+        <v>17.299999</v>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1" s="58">
@@ -26458,7 +26458,7 @@
         </is>
       </c>
       <c r="I68" t="n">
-        <v>2411.639893</v>
+        <v>241.164001</v>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="58">
@@ -27082,7 +27082,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>63.96</v>
+        <v>64.58</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -27098,7 +27098,7 @@
         </is>
       </c>
       <c r="I84" t="n">
-        <v>62.224742</v>
+        <v>62.582573</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="58">
@@ -27122,7 +27122,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>601.4299999999999</v>
+        <v>605.21</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -27138,7 +27138,7 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>591.367193</v>
+        <v>598.298346</v>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="58">
@@ -27162,7 +27162,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>63283</v>
+        <v>63399</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -27178,7 +27178,7 @@
         </is>
       </c>
       <c r="I86" t="n">
-        <v>62102.478221</v>
+        <v>62745.349742</v>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="58">
@@ -27202,7 +27202,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.006732</v>
+        <v>0.006731</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -27218,7 +27218,7 @@
         </is>
       </c>
       <c r="I87" t="n">
-        <v>0.006445</v>
+        <v>0.006639</v>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="58">
@@ -27242,7 +27242,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.010342</v>
+        <v>0.010462</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -27258,7 +27258,7 @@
         </is>
       </c>
       <c r="I88" t="n">
-        <v>0.010348</v>
+        <v>0.010154</v>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="58">
@@ -27282,7 +27282,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>66.48</v>
+        <v>66.70999999999999</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -27298,7 +27298,7 @@
         </is>
       </c>
       <c r="I89" t="n">
-        <v>64.218192</v>
+        <v>65.064046</v>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="58">
@@ -27322,7 +27322,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>1.74</v>
+        <v>2.12</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -27338,7 +27338,7 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>1.652761</v>
+        <v>1.68872</v>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="58">
@@ -27402,7 +27402,7 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
-        <v>0.013764</v>
+        <v>0.01399</v>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
@@ -27418,7 +27418,7 @@
         </is>
       </c>
       <c r="I92" t="n">
-        <v>0.013483</v>
+        <v>0.013617</v>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="58">
@@ -27442,7 +27442,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>2.705628</v>
+        <v>2.748251</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -27458,7 +27458,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>2.566067</v>
+        <v>2.634178</v>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="58">
@@ -27482,7 +27482,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>24.531733</v>
+        <v>24.69434</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -27498,7 +27498,7 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>24.195297</v>
+        <v>24.404913</v>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="58">
@@ -27522,7 +27522,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.112923</v>
+        <v>0.110852</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -27538,7 +27538,7 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>0.108688</v>
+        <v>0.110087</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="58">
@@ -27562,7 +27562,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>19714.8754</v>
+        <v>19802.4712</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -27578,7 +27578,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>19385.016583</v>
+        <v>19576.321865</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="58">
@@ -27602,7 +27602,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2074416.74</v>
+        <v>2074415.28</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -27618,7 +27618,7 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>2035719.236083</v>
+        <v>2053027.843561</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="58">
@@ -27642,7 +27642,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>2.809672</v>
+        <v>2.840227</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -27658,7 +27658,7 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>2.752047</v>
+        <v>2.76436</v>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="58">
@@ -27682,7 +27682,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>54461.6754</v>
+        <v>54469.9656</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -27698,7 +27698,7 @@
         </is>
       </c>
       <c r="I99" t="n">
-        <v>53728.723039</v>
+        <v>53879.464691</v>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="58">
@@ -27722,7 +27722,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>25.230307</v>
+        <v>25.102457</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -27738,7 +27738,7 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>24.674611</v>
+        <v>24.980636</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="58">
@@ -27762,7 +27762,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>63283</v>
+        <v>63399</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -27778,7 +27778,7 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>62102.478221</v>
+        <v>62745.349742</v>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="58">
@@ -27802,7 +27802,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>17.69</v>
+        <v>17.58</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -27818,7 +27818,7 @@
         </is>
       </c>
       <c r="I102" t="n">
-        <v>17.702621</v>
+        <v>17.805535</v>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="58">
@@ -27916,7 +27916,7 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
-        <v>0.006732</v>
+        <v>0.006731</v>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
@@ -27932,7 +27932,7 @@
         </is>
       </c>
       <c r="I105" t="n">
-        <v>0.006445</v>
+        <v>0.006639</v>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="58">
@@ -27956,7 +27956,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>66.48</v>
+        <v>66.70999999999999</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>
@@ -27972,7 +27972,7 @@
         </is>
       </c>
       <c r="I106" t="n">
-        <v>64.218192</v>
+        <v>65.064046</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="58">

</xml_diff>

<commit_message>
Daily dashboard update — 2026-06-13
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-42660" yWindow="-540" windowWidth="32460" windowHeight="17180" tabRatio="500" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Realized" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Prices" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Reference" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Realized" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="AsOfDate">'FX &amp; Assumptions'!$C$5</definedName>
@@ -697,14 +697,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -726,8 +726,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -752,10 +752,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -764,10 +764,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4F81BD"/>
               </a:solidFill>
-              <a:ln w="0">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -777,10 +777,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="C0504D"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -790,10 +790,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="9BBB59"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -803,10 +803,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="8064A2"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -816,10 +816,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4BACC6"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -829,10 +829,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="F79646"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -842,14 +842,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -875,14 +875,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -908,14 +908,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -941,14 +941,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -974,14 +974,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1007,14 +1007,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1038,16 +1038,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1142,16 +1142,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1172,10 +1172,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1187,14 +1187,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1216,8 +1216,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1242,10 +1242,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1254,10 +1254,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4672A8"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1267,10 +1267,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="AB4744"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1280,10 +1280,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="8AA64F"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1293,10 +1293,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="725990"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1306,10 +1306,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4299B0"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1319,10 +1319,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="DC853E"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1332,10 +1332,10 @@
             <idx val="6"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="93A9CE"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1345,10 +1345,10 @@
             <idx val="7"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="D09493"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1358,10 +1358,10 @@
             <idx val="8"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="B8CD97"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1371,14 +1371,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1405,14 +1405,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1439,14 +1439,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1473,14 +1473,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1507,14 +1507,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1541,14 +1541,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1575,14 +1575,14 @@
             <dLbl>
               <idx val="6"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1609,14 +1609,14 @@
             <dLbl>
               <idx val="7"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1643,14 +1643,14 @@
             <dLbl>
               <idx val="8"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1675,16 +1675,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1791,16 +1791,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1821,10 +1821,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1836,14 +1836,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1865,8 +1865,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1893,10 +1893,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1904,16 +1904,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2016,7 +2016,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2025,9 +2025,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2059,7 +2059,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="9360">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2073,7 +2073,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2082,9 +2082,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2109,16 +2109,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2139,10 +2139,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2154,14 +2154,14 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -2183,8 +2183,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -2200,10 +2200,10 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2211,16 +2211,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2411,7 +2411,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2420,9 +2420,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2454,7 +2454,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="9360">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2468,7 +2468,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2477,9 +2477,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2504,16 +2504,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2534,10 +2534,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2549,7 +2549,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>1</col>
@@ -2569,9 +2569,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2596,9 +2596,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2623,9 +2623,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId3"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2650,9 +2650,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId4"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -12648,7 +12648,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:K111"/>
+  <dimension ref="A2:K112"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="58" min="1" max="1"/>
@@ -18611,6 +18611,61 @@
       </c>
       <c r="K111" s="39">
         <f>IF(J111="THB",1,IF(J111="SGD",SGDTHB,FXRate))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112">
+        <f>B112&amp;"|"&amp;C112&amp;"|"&amp;D112</f>
+        <v/>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Mutual Fund</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>K-GTECHRMF</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>K Asset</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>Thematic</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>RMF</t>
+        </is>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="K112">
+        <f>IF(J112="THB",1,FXRate)</f>
         <v/>
       </c>
     </row>
@@ -18697,19 +18752,19 @@
     </row>
     <row r="8" ht="42" customHeight="1" s="58">
       <c r="B8" s="60">
-        <f>'MF - Lots'!P167+'Equities - Lots'!M53+'Crypto - Lots'!K32+'Unit Trust (SGD)'!M16</f>
+        <f>'MF - Lots'!P168+'Equities - Lots'!M53+'Crypto - Lots'!K32+'Unit Trust (SGD)'!M16</f>
         <v/>
       </c>
       <c r="C8" s="55" t="n"/>
       <c r="D8" s="56" t="n"/>
       <c r="F8" s="60">
-        <f>'MF - Lots'!O167+'Equities - Lots'!L53+'Crypto - Lots'!J32+'Unit Trust (SGD)'!L16</f>
+        <f>'MF - Lots'!O168+'Equities - Lots'!L53+'Crypto - Lots'!J32+'Unit Trust (SGD)'!L16</f>
         <v/>
       </c>
       <c r="G8" s="55" t="n"/>
       <c r="H8" s="56" t="n"/>
       <c r="J8" s="60">
-        <f>'MF - Lots'!Q167+'Equities - Lots'!N53+'Crypto - Lots'!L32+'Unit Trust (SGD)'!N16</f>
+        <f>'MF - Lots'!Q168+'Equities - Lots'!N53+'Crypto - Lots'!L32+'Unit Trust (SGD)'!N16</f>
         <v/>
       </c>
       <c r="K8" s="55" t="n"/>
@@ -18740,7 +18795,7 @@
     </row>
     <row r="11" ht="42" customHeight="1" s="58">
       <c r="B11" s="62">
-        <f>IFERROR(('MF - Lots'!Q167+'Equities - Lots'!N53+'Crypto - Lots'!L32+'Unit Trust (SGD)'!N16)/('MF - Lots'!O167+'Equities - Lots'!L53+'Crypto - Lots'!J32+'Unit Trust (SGD)'!L16),0)</f>
+        <f>IFERROR(('MF - Lots'!Q168+'Equities - Lots'!N53+'Crypto - Lots'!L32+'Unit Trust (SGD)'!N16)/('MF - Lots'!O168+'Equities - Lots'!L53+'Crypto - Lots'!J32+'Unit Trust (SGD)'!L16),0)</f>
         <v/>
       </c>
       <c r="C11" s="55" t="n"/>
@@ -21478,11 +21533,11 @@
         <v/>
       </c>
       <c r="C5" s="10">
-        <f>'MF - Lots'!P167+'Equities - Lots'!M53+'Crypto - Lots'!K32</f>
+        <f>'MF - Lots'!P168+'Equities - Lots'!M53+'Crypto - Lots'!K32</f>
         <v/>
       </c>
       <c r="D5" s="10">
-        <f>'MF - Lots'!O167+'Equities - Lots'!L53+'Crypto - Lots'!J32</f>
+        <f>'MF - Lots'!O168+'Equities - Lots'!L53+'Crypto - Lots'!J32</f>
         <v/>
       </c>
       <c r="E5" s="10">
@@ -21494,7 +21549,7 @@
         <v/>
       </c>
       <c r="G5" s="10">
-        <f>'MF - Lots'!P167</f>
+        <f>'MF - Lots'!P168</f>
         <v/>
       </c>
       <c r="H5" s="10">
@@ -21890,16 +21945,38 @@
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="58">
-      <c r="B17" s="28" t="n"/>
-      <c r="C17" s="29" t="n"/>
-      <c r="D17" s="29" t="n"/>
-      <c r="E17" s="29" t="n"/>
-      <c r="F17" s="30" t="n"/>
-      <c r="G17" s="29" t="n"/>
-      <c r="H17" s="29" t="n"/>
-      <c r="I17" s="29" t="n"/>
-      <c r="J17" s="31" t="n"/>
-      <c r="K17" s="32" t="n"/>
+      <c r="B17" s="28" t="n">
+        <v>46186</v>
+      </c>
+      <c r="C17" s="29" t="n">
+        <v>25663598</v>
+      </c>
+      <c r="D17" s="29" t="n">
+        <v>22757166</v>
+      </c>
+      <c r="E17" s="29" t="n">
+        <v>2906433</v>
+      </c>
+      <c r="F17" s="30" t="n">
+        <v>0.1277</v>
+      </c>
+      <c r="G17" s="29" t="n">
+        <v>18174259</v>
+      </c>
+      <c r="H17" s="29" t="n">
+        <v>4952962</v>
+      </c>
+      <c r="I17" s="29" t="n">
+        <v>1156514</v>
+      </c>
+      <c r="J17" s="31" t="n">
+        <v>32.68</v>
+      </c>
+      <c r="K17" s="32" t="inlineStr">
+        <is>
+          <t>Auto weekly snapshot</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="58">
       <c r="B18" s="28" t="n"/>
@@ -23577,7 +23654,7 @@
         </is>
       </c>
       <c r="C5" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="D5" s="64" t="inlineStr">
         <is>
@@ -23592,11 +23669,11 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>32.73</v>
+        <v>32.68</v>
       </c>
       <c r="D6" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-06-12</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-06-13</t>
         </is>
       </c>
     </row>
@@ -23641,11 +23718,11 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>25.5051</v>
+        <v>25.4608</v>
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-06-12</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-06-13</t>
         </is>
       </c>
     </row>
@@ -25245,7 +25322,7 @@
         </is>
       </c>
       <c r="E38" s="33" t="n">
-        <v>23.23</v>
+        <v>23.36</v>
       </c>
       <c r="F38" s="34" t="inlineStr">
         <is>
@@ -25253,7 +25330,7 @@
         </is>
       </c>
       <c r="G38" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H38" s="34" t="inlineStr">
         <is>
@@ -25261,7 +25338,7 @@
         </is>
       </c>
       <c r="I38" t="n">
-        <v>23.23</v>
+        <v>23.360001</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="58">
@@ -25293,7 +25370,7 @@
         </is>
       </c>
       <c r="G39" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H39" s="34" t="inlineStr">
         <is>
@@ -25301,7 +25378,7 @@
         </is>
       </c>
       <c r="I39" t="n">
-        <v>1.084</v>
+        <v>1.079</v>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="58">
@@ -25325,7 +25402,7 @@
         </is>
       </c>
       <c r="E40" s="33" t="n">
-        <v>746.08</v>
+        <v>764.1</v>
       </c>
       <c r="F40" s="34" t="inlineStr">
         <is>
@@ -25333,7 +25410,7 @@
         </is>
       </c>
       <c r="G40" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H40" s="34" t="inlineStr">
         <is>
@@ -25341,7 +25418,7 @@
         </is>
       </c>
       <c r="I40" t="n">
-        <v>746.080017</v>
+        <v>764.099976</v>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="58">
@@ -25365,7 +25442,7 @@
         </is>
       </c>
       <c r="E41" s="33" t="n">
-        <v>20.37</v>
+        <v>20.94</v>
       </c>
       <c r="F41" s="34" t="inlineStr">
         <is>
@@ -25373,7 +25450,7 @@
         </is>
       </c>
       <c r="G41" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H41" s="34" t="inlineStr">
         <is>
@@ -25381,7 +25458,7 @@
         </is>
       </c>
       <c r="I41" t="n">
-        <v>20.370001</v>
+        <v>20.940001</v>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="58">
@@ -25405,7 +25482,7 @@
         </is>
       </c>
       <c r="E42" s="33" t="n">
-        <v>218.31</v>
+        <v>218.66</v>
       </c>
       <c r="F42" s="34" t="inlineStr">
         <is>
@@ -25413,7 +25490,7 @@
         </is>
       </c>
       <c r="G42" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H42" s="34" t="inlineStr">
         <is>
@@ -25421,7 +25498,7 @@
         </is>
       </c>
       <c r="I42" t="n">
-        <v>218.309998</v>
+        <v>218.660004</v>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="58">
@@ -25453,7 +25530,7 @@
         </is>
       </c>
       <c r="G43" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H43" s="34" t="inlineStr">
         <is>
@@ -25493,7 +25570,7 @@
         </is>
       </c>
       <c r="G44" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H44" s="34" t="inlineStr">
         <is>
@@ -25533,7 +25610,7 @@
         </is>
       </c>
       <c r="G45" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H45" s="34" t="inlineStr">
         <is>
@@ -25573,7 +25650,7 @@
         </is>
       </c>
       <c r="G46" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H46" s="34" t="inlineStr">
         <is>
@@ -25650,7 +25727,7 @@
         </is>
       </c>
       <c r="G48" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H48" s="34" t="inlineStr">
         <is>
@@ -25690,7 +25767,7 @@
         </is>
       </c>
       <c r="G49" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H49" s="34" t="inlineStr">
         <is>
@@ -25730,7 +25807,7 @@
         </is>
       </c>
       <c r="G50" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H50" s="34" t="inlineStr">
         <is>
@@ -25770,7 +25847,7 @@
         </is>
       </c>
       <c r="G51" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H51" s="34" t="inlineStr">
         <is>
@@ -25810,7 +25887,7 @@
         </is>
       </c>
       <c r="G52" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H52" s="34" t="inlineStr">
         <is>
@@ -25850,7 +25927,7 @@
         </is>
       </c>
       <c r="G53" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H53" s="34" t="inlineStr">
         <is>
@@ -25890,7 +25967,7 @@
         </is>
       </c>
       <c r="G54" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H54" s="34" t="inlineStr">
         <is>
@@ -25930,7 +26007,7 @@
         </is>
       </c>
       <c r="G55" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H55" s="34" t="inlineStr">
         <is>
@@ -25970,7 +26047,7 @@
         </is>
       </c>
       <c r="G56" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H56" s="34" t="inlineStr">
         <is>
@@ -26010,7 +26087,7 @@
         </is>
       </c>
       <c r="G57" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H57" s="34" t="inlineStr">
         <is>
@@ -26050,7 +26127,7 @@
         </is>
       </c>
       <c r="G58" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H58" s="34" t="inlineStr">
         <is>
@@ -26090,7 +26167,7 @@
         </is>
       </c>
       <c r="G59" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H59" s="34" t="inlineStr">
         <is>
@@ -26122,7 +26199,7 @@
         </is>
       </c>
       <c r="E60" s="33" t="n">
-        <v>178.695</v>
+        <v>180.12</v>
       </c>
       <c r="F60" s="34" t="inlineStr">
         <is>
@@ -26130,7 +26207,7 @@
         </is>
       </c>
       <c r="G60" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H60" s="34" t="inlineStr">
         <is>
@@ -26138,7 +26215,7 @@
         </is>
       </c>
       <c r="I60" t="n">
-        <v>178.695007</v>
+        <v>180.119995</v>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="58">
@@ -26162,7 +26239,7 @@
         </is>
       </c>
       <c r="E61" s="33" t="n">
-        <v>202</v>
+        <v>204.02</v>
       </c>
       <c r="F61" s="34" t="inlineStr">
         <is>
@@ -26170,7 +26247,7 @@
         </is>
       </c>
       <c r="G61" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H61" s="34" t="inlineStr">
         <is>
@@ -26178,7 +26255,7 @@
         </is>
       </c>
       <c r="I61" t="n">
-        <v>218.800003</v>
+        <v>204.020004</v>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="58">
@@ -26202,7 +26279,7 @@
         </is>
       </c>
       <c r="E62" s="33" t="n">
-        <v>553.76</v>
+        <v>567.25</v>
       </c>
       <c r="F62" s="34" t="inlineStr">
         <is>
@@ -26210,7 +26287,7 @@
         </is>
       </c>
       <c r="G62" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H62" s="34" t="inlineStr">
         <is>
@@ -26218,7 +26295,7 @@
         </is>
       </c>
       <c r="I62" t="n">
-        <v>553.76001</v>
+        <v>552.6400149999999</v>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1" s="58">
@@ -26242,7 +26319,7 @@
         </is>
       </c>
       <c r="E63" s="33" t="n">
-        <v>164.345</v>
+        <v>164.09</v>
       </c>
       <c r="F63" s="34" t="inlineStr">
         <is>
@@ -26250,7 +26327,7 @@
         </is>
       </c>
       <c r="G63" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H63" s="34" t="inlineStr">
         <is>
@@ -26258,7 +26335,7 @@
         </is>
       </c>
       <c r="I63" t="n">
-        <v>164.345001</v>
+        <v>164.089996</v>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="58">
@@ -26282,7 +26359,7 @@
         </is>
       </c>
       <c r="E64" s="33" t="n">
-        <v>54.84</v>
+        <v>54.59</v>
       </c>
       <c r="F64" s="34" t="inlineStr">
         <is>
@@ -26290,7 +26367,7 @@
         </is>
       </c>
       <c r="G64" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H64" s="34" t="inlineStr">
         <is>
@@ -26298,7 +26375,7 @@
         </is>
       </c>
       <c r="I64" t="n">
-        <v>54.839901</v>
+        <v>54.59</v>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1" s="58">
@@ -26322,7 +26399,7 @@
         </is>
       </c>
       <c r="E65" s="33" t="n">
-        <v>198.09</v>
+        <v>197.45</v>
       </c>
       <c r="F65" s="34" t="inlineStr">
         <is>
@@ -26330,7 +26407,7 @@
         </is>
       </c>
       <c r="G65" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H65" s="34" t="inlineStr">
         <is>
@@ -26338,7 +26415,7 @@
         </is>
       </c>
       <c r="I65" t="n">
-        <v>198.089996</v>
+        <v>197.449997</v>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1" s="58">
@@ -26362,7 +26439,7 @@
         </is>
       </c>
       <c r="E66" s="33" t="n">
-        <v>144.86</v>
+        <v>146.3</v>
       </c>
       <c r="F66" s="34" t="inlineStr">
         <is>
@@ -26370,7 +26447,7 @@
         </is>
       </c>
       <c r="G66" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H66" s="34" t="inlineStr">
         <is>
@@ -26378,7 +26455,7 @@
         </is>
       </c>
       <c r="I66" t="n">
-        <v>144.860001</v>
+        <v>146.300003</v>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1" s="58">
@@ -26402,7 +26479,7 @@
         </is>
       </c>
       <c r="E67" s="33" t="n">
-        <v>145.02</v>
+        <v>148.17</v>
       </c>
       <c r="F67" s="34" t="inlineStr">
         <is>
@@ -26410,7 +26487,7 @@
         </is>
       </c>
       <c r="G67" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H67" s="34" t="inlineStr">
         <is>
@@ -26418,7 +26495,7 @@
         </is>
       </c>
       <c r="I67" t="n">
-        <v>145.020004</v>
+        <v>148.169998</v>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1" s="58">
@@ -26442,7 +26519,7 @@
         </is>
       </c>
       <c r="E68" s="33" t="n">
-        <v>248.85</v>
+        <v>254.54</v>
       </c>
       <c r="F68" s="34" t="inlineStr">
         <is>
@@ -26450,7 +26527,7 @@
         </is>
       </c>
       <c r="G68" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H68" s="34" t="inlineStr">
         <is>
@@ -26458,7 +26535,7 @@
         </is>
       </c>
       <c r="I68" t="n">
-        <v>248.850006</v>
+        <v>254.539993</v>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="58">
@@ -26482,7 +26559,7 @@
         </is>
       </c>
       <c r="E69" s="33" t="n">
-        <v>1155.14</v>
+        <v>1133</v>
       </c>
       <c r="F69" s="34" t="inlineStr">
         <is>
@@ -26490,7 +26567,7 @@
         </is>
       </c>
       <c r="G69" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H69" s="34" t="inlineStr">
         <is>
@@ -26498,7 +26575,7 @@
         </is>
       </c>
       <c r="I69" t="n">
-        <v>1155.140015</v>
+        <v>1160.949951</v>
       </c>
     </row>
     <row r="70" ht="15" customHeight="1" s="58">
@@ -26522,7 +26599,7 @@
         </is>
       </c>
       <c r="E70" s="33" t="n">
-        <v>93.84999999999999</v>
+        <v>95.23999999999999</v>
       </c>
       <c r="F70" s="34" t="inlineStr">
         <is>
@@ -26530,7 +26607,7 @@
         </is>
       </c>
       <c r="G70" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H70" s="34" t="inlineStr">
         <is>
@@ -26538,7 +26615,7 @@
         </is>
       </c>
       <c r="I70" t="n">
-        <v>93.849998</v>
+        <v>95.239998</v>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1" s="58">
@@ -26562,7 +26639,7 @@
         </is>
       </c>
       <c r="E71" s="33" t="n">
-        <v>1578.61</v>
+        <v>1577.32</v>
       </c>
       <c r="F71" s="34" t="inlineStr">
         <is>
@@ -26570,7 +26647,7 @@
         </is>
       </c>
       <c r="G71" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H71" s="34" t="inlineStr">
         <is>
@@ -26578,7 +26655,7 @@
         </is>
       </c>
       <c r="I71" t="n">
-        <v>1578.609985</v>
+        <v>1577.319946</v>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1" s="58">
@@ -26602,7 +26679,7 @@
         </is>
       </c>
       <c r="E72" s="33" t="n">
-        <v>109.51</v>
+        <v>111.05</v>
       </c>
       <c r="F72" s="34" t="inlineStr">
         <is>
@@ -26610,7 +26687,7 @@
         </is>
       </c>
       <c r="G72" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H72" s="34" t="inlineStr">
         <is>
@@ -26618,7 +26695,7 @@
         </is>
       </c>
       <c r="I72" t="n">
-        <v>109.510002</v>
+        <v>111.050003</v>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1" s="58">
@@ -26642,7 +26719,7 @@
         </is>
       </c>
       <c r="E73" s="33" t="n">
-        <v>205.895</v>
+        <v>205.19</v>
       </c>
       <c r="F73" s="34" t="inlineStr">
         <is>
@@ -26650,7 +26727,7 @@
         </is>
       </c>
       <c r="G73" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H73" s="34" t="inlineStr">
         <is>
@@ -26658,7 +26735,7 @@
         </is>
       </c>
       <c r="I73" t="n">
-        <v>205.895004</v>
+        <v>205.190002</v>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1" s="58">
@@ -26682,7 +26759,7 @@
         </is>
       </c>
       <c r="E74" s="33" t="n">
-        <v>90.56999999999999</v>
+        <v>91.45999999999999</v>
       </c>
       <c r="F74" s="34" t="inlineStr">
         <is>
@@ -26690,7 +26767,7 @@
         </is>
       </c>
       <c r="G74" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H74" s="34" t="inlineStr">
         <is>
@@ -26698,7 +26775,7 @@
         </is>
       </c>
       <c r="I74" t="n">
-        <v>90.56999999999999</v>
+        <v>91.459999</v>
       </c>
     </row>
     <row r="75" ht="15" customHeight="1" s="58">
@@ -26722,7 +26799,7 @@
         </is>
       </c>
       <c r="E75" s="33" t="n">
-        <v>97.93000000000001</v>
+        <v>98.59</v>
       </c>
       <c r="F75" s="34" t="inlineStr">
         <is>
@@ -26730,7 +26807,7 @@
         </is>
       </c>
       <c r="G75" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H75" s="34" t="inlineStr">
         <is>
@@ -26738,7 +26815,7 @@
         </is>
       </c>
       <c r="I75" t="n">
-        <v>97.93000000000001</v>
+        <v>98.589996</v>
       </c>
     </row>
     <row r="76" ht="15" customHeight="1" s="58">
@@ -26762,7 +26839,7 @@
         </is>
       </c>
       <c r="E76" s="33" t="n">
-        <v>398.2</v>
+        <v>403.2</v>
       </c>
       <c r="F76" s="34" t="inlineStr">
         <is>
@@ -26770,7 +26847,7 @@
         </is>
       </c>
       <c r="G76" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H76" s="34" t="inlineStr">
         <is>
@@ -26778,7 +26855,7 @@
         </is>
       </c>
       <c r="I76" t="n">
-        <v>398.200012</v>
+        <v>403.200012</v>
       </c>
     </row>
     <row r="77" ht="15" customHeight="1" s="58">
@@ -26802,7 +26879,7 @@
         </is>
       </c>
       <c r="E77" s="33" t="n">
-        <v>397.17</v>
+        <v>406.43</v>
       </c>
       <c r="F77" s="34" t="inlineStr">
         <is>
@@ -26810,7 +26887,7 @@
         </is>
       </c>
       <c r="G77" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H77" s="34" t="inlineStr">
         <is>
@@ -26818,7 +26895,7 @@
         </is>
       </c>
       <c r="I77" t="n">
-        <v>397.170013</v>
+        <v>406.429993</v>
       </c>
     </row>
     <row r="78" ht="15" customHeight="1" s="58">
@@ -26842,7 +26919,7 @@
         </is>
       </c>
       <c r="E78" s="33" t="n">
-        <v>50.505</v>
+        <v>50.25</v>
       </c>
       <c r="F78" s="34" t="inlineStr">
         <is>
@@ -26850,7 +26927,7 @@
         </is>
       </c>
       <c r="G78" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H78" s="34" t="inlineStr">
         <is>
@@ -26858,7 +26935,7 @@
         </is>
       </c>
       <c r="I78" t="n">
-        <v>50.505001</v>
+        <v>51</v>
       </c>
     </row>
     <row r="79" ht="15" customHeight="1" s="58">
@@ -26882,7 +26959,7 @@
         </is>
       </c>
       <c r="E79" s="33" t="n">
-        <v>95.405</v>
+        <v>95.5</v>
       </c>
       <c r="F79" s="34" t="inlineStr">
         <is>
@@ -26890,7 +26967,7 @@
         </is>
       </c>
       <c r="G79" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H79" s="34" t="inlineStr">
         <is>
@@ -26898,7 +26975,7 @@
         </is>
       </c>
       <c r="I79" t="n">
-        <v>95.404999</v>
+        <v>92.959999</v>
       </c>
     </row>
     <row r="80" ht="15" customHeight="1" s="58">
@@ -26922,7 +26999,7 @@
         </is>
       </c>
       <c r="E80" s="33" t="n">
-        <v>292.835</v>
+        <v>291.13</v>
       </c>
       <c r="F80" s="34" t="inlineStr">
         <is>
@@ -26930,7 +27007,7 @@
         </is>
       </c>
       <c r="G80" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H80" s="34" t="inlineStr">
         <is>
@@ -26938,7 +27015,7 @@
         </is>
       </c>
       <c r="I80" t="n">
-        <v>292.834991</v>
+        <v>291.130005</v>
       </c>
     </row>
     <row r="81" ht="15" customHeight="1" s="58">
@@ -26962,7 +27039,7 @@
         </is>
       </c>
       <c r="E81" s="33" t="n">
-        <v>159.86</v>
+        <v>159.78</v>
       </c>
       <c r="F81" s="34" t="inlineStr">
         <is>
@@ -26970,7 +27047,7 @@
         </is>
       </c>
       <c r="G81" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H81" s="34" t="inlineStr">
         <is>
@@ -26978,7 +27055,7 @@
         </is>
       </c>
       <c r="I81" t="n">
-        <v>159.860001</v>
+        <v>159.779999</v>
       </c>
     </row>
     <row r="82" ht="15" customHeight="1" s="58">
@@ -27002,7 +27079,7 @@
         </is>
       </c>
       <c r="E82" s="33" t="n">
-        <v>564.63</v>
+        <v>566.98</v>
       </c>
       <c r="F82" s="34" t="inlineStr">
         <is>
@@ -27010,7 +27087,7 @@
         </is>
       </c>
       <c r="G82" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H82" s="34" t="inlineStr">
         <is>
@@ -27018,7 +27095,7 @@
         </is>
       </c>
       <c r="I82" t="n">
-        <v>564.630005</v>
+        <v>566.97998</v>
       </c>
     </row>
     <row r="83" ht="15" customHeight="1" s="58">
@@ -27042,7 +27119,7 @@
         </is>
       </c>
       <c r="E83" s="33" t="n">
-        <v>133.05</v>
+        <v>130</v>
       </c>
       <c r="F83" s="34" t="inlineStr">
         <is>
@@ -27050,7 +27127,7 @@
         </is>
       </c>
       <c r="G83" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H83" s="34" t="inlineStr">
         <is>
@@ -27058,7 +27135,7 @@
         </is>
       </c>
       <c r="I83" t="n">
-        <v>133.050003</v>
+        <v>122.339996</v>
       </c>
     </row>
     <row r="84" ht="15" customHeight="1" s="58">
@@ -27082,7 +27159,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>64.13</v>
+        <v>64.48999999999999</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -27090,7 +27167,7 @@
         </is>
       </c>
       <c r="G84" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H84" s="34" t="inlineStr">
         <is>
@@ -27098,7 +27175,7 @@
         </is>
       </c>
       <c r="I84" t="n">
-        <v>63.051864</v>
+        <v>63.972226</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="58">
@@ -27122,7 +27199,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>606.25</v>
+        <v>604.1900000000001</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -27130,7 +27207,7 @@
         </is>
       </c>
       <c r="G85" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H85" s="34" t="inlineStr">
         <is>
@@ -27138,7 +27215,7 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>598.289931</v>
+        <v>601.595419</v>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="58">
@@ -27162,7 +27239,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>63373</v>
+        <v>63612</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -27170,7 +27247,7 @@
         </is>
       </c>
       <c r="G86" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H86" s="34" t="inlineStr">
         <is>
@@ -27178,7 +27255,7 @@
         </is>
       </c>
       <c r="I86" t="n">
-        <v>62707.589789</v>
+        <v>63325.221691</v>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="58">
@@ -27202,7 +27279,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.006727</v>
+        <v>0.006742</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -27210,7 +27287,7 @@
         </is>
       </c>
       <c r="G87" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H87" s="34" t="inlineStr">
         <is>
@@ -27218,7 +27295,7 @@
         </is>
       </c>
       <c r="I87" t="n">
-        <v>0.006648</v>
+        <v>0.006733</v>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="58">
@@ -27242,7 +27319,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.010374</v>
+        <v>0.010354</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -27250,7 +27327,7 @@
         </is>
       </c>
       <c r="G88" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H88" s="34" t="inlineStr">
         <is>
@@ -27258,7 +27335,7 @@
         </is>
       </c>
       <c r="I88" t="n">
-        <v>0.010339</v>
+        <v>0.010342</v>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="58">
@@ -27282,7 +27359,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>66.8</v>
+        <v>67.12</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -27290,7 +27367,7 @@
         </is>
       </c>
       <c r="G89" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H89" s="34" t="inlineStr">
         <is>
@@ -27298,7 +27375,7 @@
         </is>
       </c>
       <c r="I89" t="n">
-        <v>65.087233</v>
+        <v>66.485958</v>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="58">
@@ -27322,7 +27399,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>2.02</v>
+        <v>2.23</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -27330,7 +27407,7 @@
         </is>
       </c>
       <c r="G90" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H90" s="34" t="inlineStr">
         <is>
@@ -27338,7 +27415,7 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>1.704082</v>
+        <v>1.743307</v>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="58">
@@ -27370,7 +27447,7 @@
         </is>
       </c>
       <c r="G91" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H91" s="34" t="inlineStr">
         <is>
@@ -27402,7 +27479,7 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
-        <v>0.013846</v>
+        <v>0.013935</v>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
@@ -27410,7 +27487,7 @@
         </is>
       </c>
       <c r="G92" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H92" s="34" t="inlineStr">
         <is>
@@ -27418,7 +27495,7 @@
         </is>
       </c>
       <c r="I92" t="n">
-        <v>0.013601</v>
+        <v>0.013802</v>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="58">
@@ -27442,7 +27519,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>2.722416</v>
+        <v>2.756329</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -27450,7 +27527,7 @@
         </is>
       </c>
       <c r="G93" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H93" s="34" t="inlineStr">
         <is>
@@ -27458,7 +27535,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>2.644435</v>
+        <v>2.705184</v>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="58">
@@ -27482,7 +27559,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>24.634169</v>
+        <v>24.617844</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -27490,7 +27567,7 @@
         </is>
       </c>
       <c r="G94" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H94" s="34" t="inlineStr">
         <is>
@@ -27498,7 +27575,7 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>24.424056</v>
+        <v>24.463114</v>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="58">
@@ -27522,7 +27599,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.110875</v>
+        <v>0.11056</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -27530,7 +27607,7 @@
         </is>
       </c>
       <c r="G95" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H95" s="34" t="inlineStr">
         <is>
@@ -27538,7 +27615,7 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>0.109194</v>
+        <v>0.112576</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="58">
@@ -27562,7 +27639,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>19842.5625</v>
+        <v>19744.9292</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -27570,7 +27647,7 @@
         </is>
       </c>
       <c r="G96" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H96" s="34" t="inlineStr">
         <is>
@@ -27578,7 +27655,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>19582.029449</v>
+        <v>19660.138294</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="58">
@@ -27602,7 +27679,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2074198.29</v>
+        <v>2078840.16</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -27610,7 +27687,7 @@
         </is>
       </c>
       <c r="G97" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H97" s="34" t="inlineStr">
         <is>
@@ -27618,7 +27695,7 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>2052419.413803</v>
+        <v>2069468.244861</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="58">
@@ -27642,7 +27719,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>2.857427</v>
+        <v>2.821232</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -27650,7 +27727,7 @@
         </is>
       </c>
       <c r="G98" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H98" s="34" t="inlineStr">
         <is>
@@ -27658,7 +27735,7 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>2.77278</v>
+        <v>2.80571</v>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="58">
@@ -27682,7 +27759,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>54474.5028</v>
+        <v>54484.096</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -27690,7 +27767,7 @@
         </is>
       </c>
       <c r="G99" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H99" s="34" t="inlineStr">
         <is>
@@ -27698,7 +27775,7 @@
         </is>
       </c>
       <c r="I99" t="n">
-        <v>53680.79957</v>
+        <v>54343.335909</v>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="58">
@@ -27722,7 +27799,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>25.140633</v>
+        <v>25.226672</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -27730,7 +27807,7 @@
         </is>
       </c>
       <c r="G100" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H100" s="34" t="inlineStr">
         <is>
@@ -27738,7 +27815,7 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>25.061582</v>
+        <v>25.153329</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="58">
@@ -27762,7 +27839,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>63373</v>
+        <v>63612</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -27770,7 +27847,7 @@
         </is>
       </c>
       <c r="G101" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H101" s="34" t="inlineStr">
         <is>
@@ -27778,7 +27855,7 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>62707.589789</v>
+        <v>63325.221691</v>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="58">
@@ -27802,7 +27879,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>17.58</v>
+        <v>17.33</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -27810,7 +27887,7 @@
         </is>
       </c>
       <c r="G102" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H102" s="34" t="inlineStr">
         <is>
@@ -27818,7 +27895,7 @@
         </is>
       </c>
       <c r="I102" t="n">
-        <v>17.784835</v>
+        <v>17.691923</v>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="58">
@@ -27916,7 +27993,7 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
-        <v>0.006727</v>
+        <v>0.006742</v>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
@@ -27924,7 +28001,7 @@
         </is>
       </c>
       <c r="G105" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H105" s="34" t="inlineStr">
         <is>
@@ -27932,7 +28009,7 @@
         </is>
       </c>
       <c r="I105" t="n">
-        <v>0.006648</v>
+        <v>0.006733</v>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="58">
@@ -27956,7 +28033,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>66.8</v>
+        <v>67.12</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>
@@ -27964,7 +28041,7 @@
         </is>
       </c>
       <c r="G106" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H106" s="34" t="inlineStr">
         <is>
@@ -27972,7 +28049,7 @@
         </is>
       </c>
       <c r="I106" t="n">
-        <v>65.087233</v>
+        <v>66.485958</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="58">
@@ -28004,7 +28081,7 @@
         </is>
       </c>
       <c r="G107" s="28" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="H107" s="34" t="inlineStr">
         <is>
@@ -28020,7 +28097,45 @@
         <f>B108&amp;"|"&amp;C108&amp;"|"&amp;D108</f>
         <v/>
       </c>
-      <c r="G108" s="47" t="n"/>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Mutual Fund</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>K-GTECHRMF</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>K Asset</t>
+        </is>
+      </c>
+      <c r="E108" t="n">
+        <v>23.5969</v>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G108" s="47" t="n">
+        <v>46182</v>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I108" t="n">
+        <v>23.8653</v>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109">
@@ -28049,7 +28164,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:S167"/>
+  <dimension ref="A2:S168"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" style="58" min="1" max="1"/>
@@ -39543,41 +39658,114 @@
       <c r="S166" s="35" t="n"/>
     </row>
     <row r="167" ht="15" customHeight="1" s="58">
-      <c r="A167" s="13" t="inlineStr">
+      <c r="A167" t="n">
+        <v>163</v>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>K Asset</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>K-GTECHRMF</t>
+        </is>
+      </c>
+      <c r="D167">
+        <f>IFERROR(INDEX(Reference!$E:$E,MATCH("Mutual Fund|"&amp;C167&amp;"|"&amp;B167,Reference!$A:$A,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E167">
+        <f>IFERROR(INDEX(Reference!$H:$H,MATCH("Mutual Fund|"&amp;C167&amp;"|"&amp;B167,Reference!$A:$A,0)),"")</f>
+        <v/>
+      </c>
+      <c r="F167">
+        <f>IFERROR(INDEX(Reference!$G:$G,MATCH("Mutual Fund|"&amp;C167&amp;"|"&amp;B167,Reference!$A:$A,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G167">
+        <f>IFERROR(INDEX(Reference!$I:$I,MATCH("Mutual Fund|"&amp;C167&amp;"|"&amp;B167,Reference!$A:$A,0)),"")</f>
+        <v/>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="I167" t="n">
+        <v>2026</v>
+      </c>
+      <c r="J167" t="inlineStr">
+        <is>
+          <t>2037</t>
+        </is>
+      </c>
+      <c r="K167">
+        <f>IFERROR(IF(H167="","",(AsOfDate-H167)/365.25),"")</f>
+        <v/>
+      </c>
+      <c r="L167" t="n">
+        <v>4253.8891</v>
+      </c>
+      <c r="M167" t="n">
+        <v>23.5079</v>
+      </c>
+      <c r="N167">
+        <f>IFERROR(INDEX(Prices!$E:$E,MATCH("Mutual Fund|"&amp;C167&amp;"|"&amp;B167,Prices!$A:$A,0)),0)</f>
+        <v/>
+      </c>
+      <c r="O167" t="n">
+        <v>100000</v>
+      </c>
+      <c r="P167">
+        <f>L167*N167</f>
+        <v/>
+      </c>
+      <c r="Q167">
+        <f>P167-O167</f>
+        <v/>
+      </c>
+      <c r="R167">
+        <f>IFERROR(Q167/O167,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="13" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B167" s="43" t="n"/>
-      <c r="C167" s="43" t="n"/>
-      <c r="D167" s="43" t="n"/>
-      <c r="E167" s="43" t="n"/>
-      <c r="F167" s="43" t="n"/>
-      <c r="G167" s="43" t="n"/>
-      <c r="H167" s="43" t="n"/>
-      <c r="I167" s="43" t="n"/>
-      <c r="J167" s="43" t="n"/>
-      <c r="K167" s="43" t="n"/>
-      <c r="L167" s="43" t="n"/>
-      <c r="M167" s="43" t="n"/>
-      <c r="N167" s="43" t="n"/>
-      <c r="O167" s="14">
-        <f>SUM(O5:O166)</f>
-        <v/>
-      </c>
-      <c r="P167" s="14">
-        <f>SUM(P5:P166)</f>
-        <v/>
-      </c>
-      <c r="Q167" s="14">
-        <f>SUM(Q5:Q166)</f>
-        <v/>
-      </c>
-      <c r="R167" s="15">
-        <f>IFERROR(Q167/O167,0)</f>
-        <v/>
-      </c>
-      <c r="S167" s="43" t="n"/>
+      <c r="B168" s="43" t="n"/>
+      <c r="C168" s="43" t="n"/>
+      <c r="D168" s="43" t="n"/>
+      <c r="E168" s="43" t="n"/>
+      <c r="F168" s="43" t="n"/>
+      <c r="G168" s="43" t="n"/>
+      <c r="H168" s="43" t="n"/>
+      <c r="I168" s="43" t="n"/>
+      <c r="J168" s="43" t="n"/>
+      <c r="K168" s="43" t="n"/>
+      <c r="L168" s="43" t="n"/>
+      <c r="M168" s="43" t="n"/>
+      <c r="N168" s="43" t="n"/>
+      <c r="O168" s="14">
+        <f>SUM(O5:O167)</f>
+        <v/>
+      </c>
+      <c r="P168" s="14">
+        <f>SUM(P5:P167)</f>
+        <v/>
+      </c>
+      <c r="Q168" s="14">
+        <f>SUM(Q5:Q167)</f>
+        <v/>
+      </c>
+      <c r="R168" s="15">
+        <f>IFERROR(Q168/O168,0)</f>
+        <v/>
+      </c>
+      <c r="S168" s="43" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:S166"/>

</xml_diff>

<commit_message>
Daily dashboard update — 2026-06-14
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -21979,16 +21979,38 @@
       </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="58">
-      <c r="B18" s="28" t="n"/>
-      <c r="C18" s="29" t="n"/>
-      <c r="D18" s="29" t="n"/>
-      <c r="E18" s="29" t="n"/>
-      <c r="F18" s="30" t="n"/>
-      <c r="G18" s="29" t="n"/>
-      <c r="H18" s="29" t="n"/>
-      <c r="I18" s="29" t="n"/>
-      <c r="J18" s="31" t="n"/>
-      <c r="K18" s="32" t="n"/>
+      <c r="B18" s="28" t="n">
+        <v>46187</v>
+      </c>
+      <c r="C18" s="29" t="n">
+        <v>25676441</v>
+      </c>
+      <c r="D18" s="29" t="n">
+        <v>22757166</v>
+      </c>
+      <c r="E18" s="29" t="n">
+        <v>2919275</v>
+      </c>
+      <c r="F18" s="30" t="n">
+        <v>0.1283</v>
+      </c>
+      <c r="G18" s="29" t="n">
+        <v>18174259</v>
+      </c>
+      <c r="H18" s="29" t="n">
+        <v>4952962</v>
+      </c>
+      <c r="I18" s="29" t="n">
+        <v>1170589</v>
+      </c>
+      <c r="J18" s="31" t="n">
+        <v>32.68</v>
+      </c>
+      <c r="K18" s="32" t="inlineStr">
+        <is>
+          <t>Auto weekly snapshot</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="58">
       <c r="B19" s="28" t="n"/>
@@ -23654,7 +23676,7 @@
         </is>
       </c>
       <c r="C5" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="D5" s="64" t="inlineStr">
         <is>
@@ -23673,7 +23695,7 @@
       </c>
       <c r="D6" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-06-13</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-06-14</t>
         </is>
       </c>
     </row>
@@ -23722,7 +23744,7 @@
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-06-13</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-06-14</t>
         </is>
       </c>
     </row>
@@ -25330,7 +25352,7 @@
         </is>
       </c>
       <c r="G38" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H38" s="34" t="inlineStr">
         <is>
@@ -25362,7 +25384,7 @@
         </is>
       </c>
       <c r="E39" s="33" t="n">
-        <v>1.084</v>
+        <v>1.079</v>
       </c>
       <c r="F39" s="34" t="inlineStr">
         <is>
@@ -25370,7 +25392,7 @@
         </is>
       </c>
       <c r="G39" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H39" s="34" t="inlineStr">
         <is>
@@ -25410,7 +25432,7 @@
         </is>
       </c>
       <c r="G40" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H40" s="34" t="inlineStr">
         <is>
@@ -25450,7 +25472,7 @@
         </is>
       </c>
       <c r="G41" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H41" s="34" t="inlineStr">
         <is>
@@ -25490,7 +25512,7 @@
         </is>
       </c>
       <c r="G42" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H42" s="34" t="inlineStr">
         <is>
@@ -25530,7 +25552,7 @@
         </is>
       </c>
       <c r="G43" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H43" s="34" t="inlineStr">
         <is>
@@ -25570,7 +25592,7 @@
         </is>
       </c>
       <c r="G44" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H44" s="34" t="inlineStr">
         <is>
@@ -25610,7 +25632,7 @@
         </is>
       </c>
       <c r="G45" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H45" s="34" t="inlineStr">
         <is>
@@ -25650,7 +25672,7 @@
         </is>
       </c>
       <c r="G46" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H46" s="34" t="inlineStr">
         <is>
@@ -25727,7 +25749,7 @@
         </is>
       </c>
       <c r="G48" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H48" s="34" t="inlineStr">
         <is>
@@ -25767,7 +25789,7 @@
         </is>
       </c>
       <c r="G49" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H49" s="34" t="inlineStr">
         <is>
@@ -25807,7 +25829,7 @@
         </is>
       </c>
       <c r="G50" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H50" s="34" t="inlineStr">
         <is>
@@ -25847,7 +25869,7 @@
         </is>
       </c>
       <c r="G51" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H51" s="34" t="inlineStr">
         <is>
@@ -25887,7 +25909,7 @@
         </is>
       </c>
       <c r="G52" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H52" s="34" t="inlineStr">
         <is>
@@ -25927,7 +25949,7 @@
         </is>
       </c>
       <c r="G53" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H53" s="34" t="inlineStr">
         <is>
@@ -25967,7 +25989,7 @@
         </is>
       </c>
       <c r="G54" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H54" s="34" t="inlineStr">
         <is>
@@ -26007,7 +26029,7 @@
         </is>
       </c>
       <c r="G55" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H55" s="34" t="inlineStr">
         <is>
@@ -26047,7 +26069,7 @@
         </is>
       </c>
       <c r="G56" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H56" s="34" t="inlineStr">
         <is>
@@ -26087,7 +26109,7 @@
         </is>
       </c>
       <c r="G57" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H57" s="34" t="inlineStr">
         <is>
@@ -26127,7 +26149,7 @@
         </is>
       </c>
       <c r="G58" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H58" s="34" t="inlineStr">
         <is>
@@ -26167,7 +26189,7 @@
         </is>
       </c>
       <c r="G59" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H59" s="34" t="inlineStr">
         <is>
@@ -26207,7 +26229,7 @@
         </is>
       </c>
       <c r="G60" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H60" s="34" t="inlineStr">
         <is>
@@ -26247,7 +26269,7 @@
         </is>
       </c>
       <c r="G61" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H61" s="34" t="inlineStr">
         <is>
@@ -26287,7 +26309,7 @@
         </is>
       </c>
       <c r="G62" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H62" s="34" t="inlineStr">
         <is>
@@ -26327,7 +26349,7 @@
         </is>
       </c>
       <c r="G63" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H63" s="34" t="inlineStr">
         <is>
@@ -26367,7 +26389,7 @@
         </is>
       </c>
       <c r="G64" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H64" s="34" t="inlineStr">
         <is>
@@ -26407,7 +26429,7 @@
         </is>
       </c>
       <c r="G65" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H65" s="34" t="inlineStr">
         <is>
@@ -26447,7 +26469,7 @@
         </is>
       </c>
       <c r="G66" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H66" s="34" t="inlineStr">
         <is>
@@ -26487,7 +26509,7 @@
         </is>
       </c>
       <c r="G67" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H67" s="34" t="inlineStr">
         <is>
@@ -26527,7 +26549,7 @@
         </is>
       </c>
       <c r="G68" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H68" s="34" t="inlineStr">
         <is>
@@ -26567,7 +26589,7 @@
         </is>
       </c>
       <c r="G69" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H69" s="34" t="inlineStr">
         <is>
@@ -26607,7 +26629,7 @@
         </is>
       </c>
       <c r="G70" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H70" s="34" t="inlineStr">
         <is>
@@ -26647,7 +26669,7 @@
         </is>
       </c>
       <c r="G71" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H71" s="34" t="inlineStr">
         <is>
@@ -26687,7 +26709,7 @@
         </is>
       </c>
       <c r="G72" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H72" s="34" t="inlineStr">
         <is>
@@ -26727,7 +26749,7 @@
         </is>
       </c>
       <c r="G73" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H73" s="34" t="inlineStr">
         <is>
@@ -26767,7 +26789,7 @@
         </is>
       </c>
       <c r="G74" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H74" s="34" t="inlineStr">
         <is>
@@ -26807,7 +26829,7 @@
         </is>
       </c>
       <c r="G75" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H75" s="34" t="inlineStr">
         <is>
@@ -26847,7 +26869,7 @@
         </is>
       </c>
       <c r="G76" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H76" s="34" t="inlineStr">
         <is>
@@ -26887,7 +26909,7 @@
         </is>
       </c>
       <c r="G77" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H77" s="34" t="inlineStr">
         <is>
@@ -26927,7 +26949,7 @@
         </is>
       </c>
       <c r="G78" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H78" s="34" t="inlineStr">
         <is>
@@ -26967,7 +26989,7 @@
         </is>
       </c>
       <c r="G79" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H79" s="34" t="inlineStr">
         <is>
@@ -27007,7 +27029,7 @@
         </is>
       </c>
       <c r="G80" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H80" s="34" t="inlineStr">
         <is>
@@ -27047,7 +27069,7 @@
         </is>
       </c>
       <c r="G81" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H81" s="34" t="inlineStr">
         <is>
@@ -27087,7 +27109,7 @@
         </is>
       </c>
       <c r="G82" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H82" s="34" t="inlineStr">
         <is>
@@ -27127,7 +27149,7 @@
         </is>
       </c>
       <c r="G83" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H83" s="34" t="inlineStr">
         <is>
@@ -27159,7 +27181,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>64.48999999999999</v>
+        <v>67.48999999999999</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -27167,7 +27189,7 @@
         </is>
       </c>
       <c r="G84" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H84" s="34" t="inlineStr">
         <is>
@@ -27175,7 +27197,7 @@
         </is>
       </c>
       <c r="I84" t="n">
-        <v>63.972226</v>
+        <v>64.454099</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="58">
@@ -27199,7 +27221,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>604.1900000000001</v>
+        <v>609.92</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -27207,7 +27229,7 @@
         </is>
       </c>
       <c r="G85" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H85" s="34" t="inlineStr">
         <is>
@@ -27215,7 +27237,7 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>601.595419</v>
+        <v>604.300021</v>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="58">
@@ -27239,7 +27261,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>63612</v>
+        <v>64603</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -27247,7 +27269,7 @@
         </is>
       </c>
       <c r="G86" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H86" s="34" t="inlineStr">
         <is>
@@ -27255,7 +27277,7 @@
         </is>
       </c>
       <c r="I86" t="n">
-        <v>63325.221691</v>
+        <v>63626.823745</v>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="58">
@@ -27279,7 +27301,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.006742</v>
+        <v>0.006806</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -27287,7 +27309,7 @@
         </is>
       </c>
       <c r="G87" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H87" s="34" t="inlineStr">
         <is>
@@ -27295,7 +27317,7 @@
         </is>
       </c>
       <c r="I87" t="n">
-        <v>0.006733</v>
+        <v>0.006747</v>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="58">
@@ -27319,7 +27341,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.010354</v>
+        <v>0.010593</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -27327,7 +27349,7 @@
         </is>
       </c>
       <c r="G88" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H88" s="34" t="inlineStr">
         <is>
@@ -27335,7 +27357,7 @@
         </is>
       </c>
       <c r="I88" t="n">
-        <v>0.010342</v>
+        <v>0.010357</v>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="58">
@@ -27359,7 +27381,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>67.12</v>
+        <v>68.98</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -27367,7 +27389,7 @@
         </is>
       </c>
       <c r="G89" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H89" s="34" t="inlineStr">
         <is>
@@ -27375,7 +27397,7 @@
         </is>
       </c>
       <c r="I89" t="n">
-        <v>66.485958</v>
+        <v>67.093678</v>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="58">
@@ -27399,7 +27421,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>2.23</v>
+        <v>2.1</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -27407,7 +27429,7 @@
         </is>
       </c>
       <c r="G90" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H90" s="34" t="inlineStr">
         <is>
@@ -27415,7 +27437,7 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>1.743307</v>
+        <v>2.221388</v>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="58">
@@ -27447,7 +27469,7 @@
         </is>
       </c>
       <c r="G91" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H91" s="34" t="inlineStr">
         <is>
@@ -27479,23 +27501,23 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
+        <v>0.013966</v>
+      </c>
+      <c r="F92" s="34" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G92" s="28" t="n">
+        <v>46187</v>
+      </c>
+      <c r="H92" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I92" t="n">
         <v>0.013935</v>
-      </c>
-      <c r="F92" s="34" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="G92" s="28" t="n">
-        <v>46186</v>
-      </c>
-      <c r="H92" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I92" t="n">
-        <v>0.013802</v>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="58">
@@ -27519,7 +27541,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>2.756329</v>
+        <v>2.763192</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -27527,7 +27549,7 @@
         </is>
       </c>
       <c r="G93" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H93" s="34" t="inlineStr">
         <is>
@@ -27535,7 +27557,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>2.705184</v>
+        <v>2.756343</v>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="58">
@@ -27559,7 +27581,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>24.617844</v>
+        <v>25.108926</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -27567,7 +27589,7 @@
         </is>
       </c>
       <c r="G94" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H94" s="34" t="inlineStr">
         <is>
@@ -27575,7 +27597,7 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>24.463114</v>
+        <v>24.625157</v>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="58">
@@ -27599,7 +27621,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.11056</v>
+        <v>0.112009</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -27607,7 +27629,7 @@
         </is>
       </c>
       <c r="G95" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H95" s="34" t="inlineStr">
         <is>
@@ -27615,7 +27637,7 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>0.112576</v>
+        <v>0.110457</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="58">
@@ -27639,7 +27661,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>19744.9292</v>
+        <v>19932.1856</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -27647,7 +27669,7 @@
         </is>
       </c>
       <c r="G96" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H96" s="34" t="inlineStr">
         <is>
@@ -27655,7 +27677,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>19660.138294</v>
+        <v>19748.524686</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="58">
@@ -27679,7 +27701,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2078840.16</v>
+        <v>2111226.04</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -27687,7 +27709,7 @@
         </is>
       </c>
       <c r="G97" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H97" s="34" t="inlineStr">
         <is>
@@ -27695,7 +27717,7 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>2069468.244861</v>
+        <v>2079324.599992</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="58">
@@ -27719,7 +27741,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>2.821232</v>
+        <v>2.871526</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -27727,7 +27749,7 @@
         </is>
       </c>
       <c r="G98" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H98" s="34" t="inlineStr">
         <is>
@@ -27735,7 +27757,7 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>2.80571</v>
+        <v>2.82132</v>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="58">
@@ -27759,7 +27781,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>54484.096</v>
+        <v>55084.1008</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -27767,7 +27789,7 @@
         </is>
       </c>
       <c r="G99" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H99" s="34" t="inlineStr">
         <is>
@@ -27775,7 +27797,7 @@
         </is>
       </c>
       <c r="I99" t="n">
-        <v>54343.335909</v>
+        <v>54488.861432</v>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="58">
@@ -27799,7 +27821,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>25.226672</v>
+        <v>25.033828</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -27807,7 +27829,7 @@
         </is>
       </c>
       <c r="G100" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H100" s="34" t="inlineStr">
         <is>
@@ -27815,7 +27837,7 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>25.153329</v>
+        <v>25.226661</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="58">
@@ -27839,7 +27861,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>63612</v>
+        <v>64603</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -27847,7 +27869,7 @@
         </is>
       </c>
       <c r="G101" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H101" s="34" t="inlineStr">
         <is>
@@ -27855,7 +27877,7 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>63325.221691</v>
+        <v>63626.823745</v>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="58">
@@ -27879,7 +27901,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>17.33</v>
+        <v>17.64</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -27887,7 +27909,7 @@
         </is>
       </c>
       <c r="G102" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H102" s="34" t="inlineStr">
         <is>
@@ -27895,7 +27917,7 @@
         </is>
       </c>
       <c r="I102" t="n">
-        <v>17.691923</v>
+        <v>17.337864</v>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="58">
@@ -27993,7 +28015,7 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
-        <v>0.006742</v>
+        <v>0.006806</v>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
@@ -28001,7 +28023,7 @@
         </is>
       </c>
       <c r="G105" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H105" s="34" t="inlineStr">
         <is>
@@ -28009,7 +28031,7 @@
         </is>
       </c>
       <c r="I105" t="n">
-        <v>0.006733</v>
+        <v>0.006747</v>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="58">
@@ -28033,7 +28055,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>67.12</v>
+        <v>68.98</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>
@@ -28041,7 +28063,7 @@
         </is>
       </c>
       <c r="G106" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H106" s="34" t="inlineStr">
         <is>
@@ -28049,7 +28071,7 @@
         </is>
       </c>
       <c r="I106" t="n">
-        <v>66.485958</v>
+        <v>67.093678</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="58">
@@ -28081,7 +28103,7 @@
         </is>
       </c>
       <c r="G107" s="28" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="H107" s="34" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Daily dashboard update — 2026-06-15
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -22013,16 +22013,38 @@
       </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="58">
-      <c r="B19" s="28" t="n"/>
-      <c r="C19" s="29" t="n"/>
-      <c r="D19" s="29" t="n"/>
-      <c r="E19" s="29" t="n"/>
-      <c r="F19" s="30" t="n"/>
-      <c r="G19" s="29" t="n"/>
-      <c r="H19" s="29" t="n"/>
-      <c r="I19" s="29" t="n"/>
-      <c r="J19" s="31" t="n"/>
-      <c r="K19" s="32" t="n"/>
+      <c r="B19" s="28" t="n">
+        <v>46188</v>
+      </c>
+      <c r="C19" s="29" t="n">
+        <v>26314955</v>
+      </c>
+      <c r="D19" s="29" t="n">
+        <v>22743230</v>
+      </c>
+      <c r="E19" s="29" t="n">
+        <v>3571726</v>
+      </c>
+      <c r="F19" s="30" t="n">
+        <v>0.157</v>
+      </c>
+      <c r="G19" s="29" t="n">
+        <v>18819830</v>
+      </c>
+      <c r="H19" s="29" t="n">
+        <v>4939693</v>
+      </c>
+      <c r="I19" s="29" t="n">
+        <v>1178204</v>
+      </c>
+      <c r="J19" s="31" t="n">
+        <v>32.55</v>
+      </c>
+      <c r="K19" s="32" t="inlineStr">
+        <is>
+          <t>Auto weekly snapshot</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="58">
       <c r="B20" s="28" t="n"/>
@@ -23676,7 +23698,7 @@
         </is>
       </c>
       <c r="C5" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="D5" s="64" t="inlineStr">
         <is>
@@ -23691,11 +23713,11 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>32.68</v>
+        <v>32.55</v>
       </c>
       <c r="D6" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-06-14</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-06-15</t>
         </is>
       </c>
     </row>
@@ -23740,11 +23762,11 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>25.4608</v>
+        <v>25.4349</v>
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-06-14</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-06-15</t>
         </is>
       </c>
     </row>
@@ -23859,27 +23881,27 @@
         </is>
       </c>
       <c r="E5" s="33" t="n">
+        <v>25.5328</v>
+      </c>
+      <c r="F5" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G5" s="28" t="n">
+        <v>46184</v>
+      </c>
+      <c r="H5" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
         <v>23.4501</v>
       </c>
-      <c r="F5" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G5" s="28" t="n">
-        <v>46183</v>
-      </c>
-      <c r="H5" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I5" t="n">
-        <v>23.9719</v>
-      </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
     </row>
@@ -23904,27 +23926,27 @@
         </is>
       </c>
       <c r="E6" s="33" t="n">
+        <v>10.6873</v>
+      </c>
+      <c r="F6" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G6" s="28" t="n">
+        <v>46185</v>
+      </c>
+      <c r="H6" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
         <v>10.6872</v>
       </c>
-      <c r="F6" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G6" s="28" t="n">
-        <v>46184</v>
-      </c>
-      <c r="H6" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I6" t="n">
-        <v>10.687</v>
-      </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>
@@ -23949,27 +23971,27 @@
         </is>
       </c>
       <c r="E7" s="33" t="n">
+        <v>7.0558</v>
+      </c>
+      <c r="F7" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G7" s="28" t="n">
+        <v>46184</v>
+      </c>
+      <c r="H7" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
         <v>7.0666</v>
       </c>
-      <c r="F7" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G7" s="28" t="n">
-        <v>46183</v>
-      </c>
-      <c r="H7" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I7" t="n">
-        <v>7.0939</v>
-      </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
     </row>
@@ -23994,27 +24016,27 @@
         </is>
       </c>
       <c r="E8" s="33" t="n">
+        <v>9.4458</v>
+      </c>
+      <c r="F8" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G8" s="28" t="n">
+        <v>46184</v>
+      </c>
+      <c r="H8" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
         <v>9.3483</v>
       </c>
-      <c r="F8" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G8" s="28" t="n">
-        <v>46183</v>
-      </c>
-      <c r="H8" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I8" t="n">
-        <v>9.4916</v>
-      </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
     </row>
@@ -24039,27 +24061,27 @@
         </is>
       </c>
       <c r="E9" s="33" t="n">
+        <v>9.285500000000001</v>
+      </c>
+      <c r="F9" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G9" s="28" t="n">
+        <v>46185</v>
+      </c>
+      <c r="H9" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
         <v>9.2189</v>
       </c>
-      <c r="F9" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G9" s="28" t="n">
-        <v>46184</v>
-      </c>
-      <c r="H9" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I9" t="n">
-        <v>9.1568</v>
-      </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>
@@ -24084,27 +24106,27 @@
         </is>
       </c>
       <c r="E10" s="33" t="n">
+        <v>12.9605</v>
+      </c>
+      <c r="F10" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G10" s="28" t="n">
+        <v>46184</v>
+      </c>
+      <c r="H10" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
         <v>12.9779</v>
       </c>
-      <c r="F10" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G10" s="28" t="n">
-        <v>46183</v>
-      </c>
-      <c r="H10" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I10" t="n">
-        <v>13.2756</v>
-      </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
     </row>
@@ -24129,27 +24151,27 @@
         </is>
       </c>
       <c r="E11" s="33" t="n">
+        <v>13.2722</v>
+      </c>
+      <c r="F11" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G11" s="28" t="n">
+        <v>46185</v>
+      </c>
+      <c r="H11" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
         <v>13.0418</v>
       </c>
-      <c r="F11" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G11" s="28" t="n">
-        <v>46184</v>
-      </c>
-      <c r="H11" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I11" t="n">
-        <v>12.894</v>
-      </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>
@@ -24174,27 +24196,27 @@
         </is>
       </c>
       <c r="E12" s="33" t="n">
+        <v>26.8895</v>
+      </c>
+      <c r="F12" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G12" s="28" t="n">
+        <v>46185</v>
+      </c>
+      <c r="H12" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
         <v>26.2924</v>
       </c>
-      <c r="F12" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G12" s="28" t="n">
-        <v>46184</v>
-      </c>
-      <c r="H12" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I12" t="n">
-        <v>25.8795</v>
-      </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>
@@ -24219,27 +24241,27 @@
         </is>
       </c>
       <c r="E13" s="33" t="n">
+        <v>36.5289</v>
+      </c>
+      <c r="F13" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G13" s="28" t="n">
+        <v>46185</v>
+      </c>
+      <c r="H13" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
         <v>36.0361</v>
       </c>
-      <c r="F13" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G13" s="28" t="n">
-        <v>46184</v>
-      </c>
-      <c r="H13" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I13" t="n">
-        <v>35.8529</v>
-      </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>
@@ -24264,27 +24286,27 @@
         </is>
       </c>
       <c r="E14" s="33" t="n">
+        <v>25.535</v>
+      </c>
+      <c r="F14" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G14" s="28" t="n">
+        <v>46185</v>
+      </c>
+      <c r="H14" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
         <v>25.2656</v>
       </c>
-      <c r="F14" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G14" s="28" t="n">
-        <v>46184</v>
-      </c>
-      <c r="H14" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I14" t="n">
-        <v>25.1917</v>
-      </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>
@@ -24309,27 +24331,27 @@
         </is>
       </c>
       <c r="E15" s="33" t="n">
+        <v>14.919</v>
+      </c>
+      <c r="F15" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G15" s="28" t="n">
+        <v>46183</v>
+      </c>
+      <c r="H15" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
         <v>15.0551</v>
       </c>
-      <c r="F15" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G15" s="28" t="n">
-        <v>46182</v>
-      </c>
-      <c r="H15" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I15" t="n">
-        <v>14.8604</v>
-      </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
     </row>
@@ -24354,27 +24376,27 @@
         </is>
       </c>
       <c r="E16" s="33" t="n">
+        <v>81.94029999999999</v>
+      </c>
+      <c r="F16" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G16" s="28" t="n">
+        <v>46185</v>
+      </c>
+      <c r="H16" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
         <v>80.91589999999999</v>
       </c>
-      <c r="F16" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G16" s="28" t="n">
-        <v>46184</v>
-      </c>
-      <c r="H16" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I16" t="n">
-        <v>80.4905</v>
-      </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>
@@ -24399,27 +24421,27 @@
         </is>
       </c>
       <c r="E17" s="33" t="n">
+        <v>53.4365</v>
+      </c>
+      <c r="F17" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G17" s="28" t="n">
+        <v>46185</v>
+      </c>
+      <c r="H17" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
         <v>52.8716</v>
       </c>
-      <c r="F17" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G17" s="28" t="n">
-        <v>46184</v>
-      </c>
-      <c r="H17" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I17" t="n">
-        <v>52.7619</v>
-      </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>
@@ -24444,27 +24466,27 @@
         </is>
       </c>
       <c r="E18" s="33" t="n">
+        <v>16.4623</v>
+      </c>
+      <c r="F18" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G18" s="28" t="n">
+        <v>46185</v>
+      </c>
+      <c r="H18" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
         <v>16.4428</v>
       </c>
-      <c r="F18" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G18" s="28" t="n">
-        <v>46184</v>
-      </c>
-      <c r="H18" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I18" t="n">
-        <v>16.4301</v>
-      </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>
@@ -24489,27 +24511,27 @@
         </is>
       </c>
       <c r="E19" s="33" t="n">
+        <v>23.4045</v>
+      </c>
+      <c r="F19" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G19" s="28" t="n">
+        <v>46185</v>
+      </c>
+      <c r="H19" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
         <v>23.4043</v>
       </c>
-      <c r="F19" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G19" s="28" t="n">
-        <v>46184</v>
-      </c>
-      <c r="H19" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I19" t="n">
-        <v>23.4039</v>
-      </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>
@@ -24534,27 +24556,27 @@
         </is>
       </c>
       <c r="E20" s="33" t="n">
+        <v>40.574</v>
+      </c>
+      <c r="F20" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G20" s="28" t="n">
+        <v>46184</v>
+      </c>
+      <c r="H20" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
         <v>39.919</v>
       </c>
-      <c r="F20" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G20" s="28" t="n">
-        <v>46183</v>
-      </c>
-      <c r="H20" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I20" t="n">
-        <v>40.563</v>
-      </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
     </row>
@@ -24579,27 +24601,27 @@
         </is>
       </c>
       <c r="E21" s="33" t="n">
+        <v>13.5289</v>
+      </c>
+      <c r="F21" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G21" s="28" t="n">
+        <v>46185</v>
+      </c>
+      <c r="H21" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
         <v>13.2943</v>
       </c>
-      <c r="F21" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G21" s="28" t="n">
-        <v>46184</v>
-      </c>
-      <c r="H21" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I21" t="n">
-        <v>13.3396</v>
-      </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>
@@ -24624,27 +24646,27 @@
         </is>
       </c>
       <c r="E22" s="33" t="n">
+        <v>13.2862</v>
+      </c>
+      <c r="F22" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G22" s="28" t="n">
+        <v>46184</v>
+      </c>
+      <c r="H22" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
         <v>13.3451</v>
       </c>
-      <c r="F22" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G22" s="28" t="n">
-        <v>46183</v>
-      </c>
-      <c r="H22" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I22" t="n">
-        <v>13.2159</v>
-      </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
     </row>
@@ -24669,27 +24691,27 @@
         </is>
       </c>
       <c r="E23" s="33" t="n">
+        <v>12.4646</v>
+      </c>
+      <c r="F23" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G23" s="28" t="n">
+        <v>46185</v>
+      </c>
+      <c r="H23" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
         <v>12.299</v>
       </c>
-      <c r="F23" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G23" s="28" t="n">
-        <v>46184</v>
-      </c>
-      <c r="H23" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I23" t="n">
-        <v>12.2493</v>
-      </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>
@@ -24714,27 +24736,27 @@
         </is>
       </c>
       <c r="E24" s="33" t="n">
+        <v>11.56</v>
+      </c>
+      <c r="F24" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G24" s="28" t="n">
+        <v>46184</v>
+      </c>
+      <c r="H24" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
         <v>11.6527</v>
       </c>
-      <c r="F24" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G24" s="28" t="n">
-        <v>46183</v>
-      </c>
-      <c r="H24" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I24" t="n">
-        <v>11.8802</v>
-      </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
     </row>
@@ -24759,27 +24781,27 @@
         </is>
       </c>
       <c r="E25" s="33" t="n">
+        <v>9.825200000000001</v>
+      </c>
+      <c r="F25" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G25" s="28" t="n">
+        <v>46185</v>
+      </c>
+      <c r="H25" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
         <v>9.909700000000001</v>
       </c>
-      <c r="F25" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G25" s="28" t="n">
-        <v>46184</v>
-      </c>
-      <c r="H25" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I25" t="n">
-        <v>9.9718</v>
-      </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>
@@ -24804,27 +24826,27 @@
         </is>
       </c>
       <c r="E26" s="33" t="n">
+        <v>13.7868</v>
+      </c>
+      <c r="F26" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G26" s="28" t="n">
+        <v>46185</v>
+      </c>
+      <c r="H26" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
         <v>13.909</v>
       </c>
-      <c r="F26" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G26" s="28" t="n">
-        <v>46184</v>
-      </c>
-      <c r="H26" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I26" t="n">
-        <v>14.002</v>
-      </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>
@@ -24849,27 +24871,27 @@
         </is>
       </c>
       <c r="E27" s="33" t="n">
+        <v>17.0399</v>
+      </c>
+      <c r="F27" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G27" s="28" t="n">
+        <v>46185</v>
+      </c>
+      <c r="H27" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
         <v>16.7383</v>
       </c>
-      <c r="F27" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G27" s="28" t="n">
-        <v>46184</v>
-      </c>
-      <c r="H27" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I27" t="n">
-        <v>16.7307</v>
-      </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>
@@ -24894,27 +24916,27 @@
         </is>
       </c>
       <c r="E28" s="33" t="n">
+        <v>18.7544</v>
+      </c>
+      <c r="F28" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G28" s="28" t="n">
+        <v>46185</v>
+      </c>
+      <c r="H28" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
         <v>18.1673</v>
       </c>
-      <c r="F28" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G28" s="28" t="n">
-        <v>46184</v>
-      </c>
-      <c r="H28" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I28" t="n">
-        <v>18.5085</v>
-      </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>
@@ -24939,27 +24961,27 @@
         </is>
       </c>
       <c r="E29" s="33" t="n">
+        <v>27.104</v>
+      </c>
+      <c r="F29" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G29" s="28" t="n">
+        <v>46184</v>
+      </c>
+      <c r="H29" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
         <v>24.2974</v>
       </c>
-      <c r="F29" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G29" s="28" t="n">
-        <v>46183</v>
-      </c>
-      <c r="H29" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I29" t="n">
-        <v>25.0651</v>
-      </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
     </row>
@@ -24984,27 +25006,27 @@
         </is>
       </c>
       <c r="E30" s="33" t="n">
+        <v>36.9119</v>
+      </c>
+      <c r="F30" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G30" s="28" t="n">
+        <v>46184</v>
+      </c>
+      <c r="H30" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
         <v>36.0272</v>
       </c>
-      <c r="F30" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G30" s="28" t="n">
-        <v>46183</v>
-      </c>
-      <c r="H30" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I30" t="n">
-        <v>36.0558</v>
-      </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
     </row>
@@ -25029,27 +25051,27 @@
         </is>
       </c>
       <c r="E31" s="33" t="n">
+        <v>13.0229</v>
+      </c>
+      <c r="F31" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G31" s="28" t="n">
+        <v>46185</v>
+      </c>
+      <c r="H31" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
         <v>12.8526</v>
       </c>
-      <c r="F31" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G31" s="28" t="n">
-        <v>46184</v>
-      </c>
-      <c r="H31" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I31" t="n">
-        <v>12.7851</v>
-      </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>
@@ -25074,27 +25096,27 @@
         </is>
       </c>
       <c r="E32" s="33" t="n">
+        <v>21.706</v>
+      </c>
+      <c r="F32" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G32" s="28" t="n">
+        <v>46185</v>
+      </c>
+      <c r="H32" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
         <v>21.7059</v>
       </c>
-      <c r="F32" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G32" s="28" t="n">
-        <v>46184</v>
-      </c>
-      <c r="H32" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I32" t="n">
-        <v>21.7057</v>
-      </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>
@@ -25119,27 +25141,27 @@
         </is>
       </c>
       <c r="E33" s="33" t="n">
+        <v>12.5506</v>
+      </c>
+      <c r="F33" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G33" s="28" t="n">
+        <v>46185</v>
+      </c>
+      <c r="H33" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
         <v>12.4116</v>
       </c>
-      <c r="F33" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G33" s="28" t="n">
-        <v>46184</v>
-      </c>
-      <c r="H33" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I33" t="n">
-        <v>12.3702</v>
-      </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>
@@ -25164,27 +25186,27 @@
         </is>
       </c>
       <c r="E34" s="33" t="n">
+        <v>16.2056</v>
+      </c>
+      <c r="F34" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G34" s="28" t="n">
+        <v>46185</v>
+      </c>
+      <c r="H34" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
         <v>16.2054</v>
       </c>
-      <c r="F34" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G34" s="28" t="n">
-        <v>46184</v>
-      </c>
-      <c r="H34" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I34" t="n">
-        <v>16.205</v>
-      </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>
@@ -25209,27 +25231,27 @@
         </is>
       </c>
       <c r="E35" s="33" t="n">
+        <v>27.4092</v>
+      </c>
+      <c r="F35" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G35" s="28" t="n">
+        <v>46184</v>
+      </c>
+      <c r="H35" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
         <v>26.542</v>
       </c>
-      <c r="F35" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G35" s="28" t="n">
-        <v>46183</v>
-      </c>
-      <c r="H35" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I35" t="n">
-        <v>27.6474</v>
-      </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
     </row>
@@ -25254,27 +25276,27 @@
         </is>
       </c>
       <c r="E36" s="33" t="n">
+        <v>10.079</v>
+      </c>
+      <c r="F36" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G36" s="28" t="n">
+        <v>46185</v>
+      </c>
+      <c r="H36" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
         <v>10.0297</v>
       </c>
-      <c r="F36" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G36" s="28" t="n">
-        <v>46184</v>
-      </c>
-      <c r="H36" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I36" t="n">
-        <v>9.995900000000001</v>
-      </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>
@@ -25299,27 +25321,27 @@
         </is>
       </c>
       <c r="E37" s="33" t="n">
+        <v>22.7488</v>
+      </c>
+      <c r="F37" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G37" s="28" t="n">
+        <v>46185</v>
+      </c>
+      <c r="H37" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
         <v>22.4356</v>
       </c>
-      <c r="F37" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G37" s="28" t="n">
-        <v>46184</v>
-      </c>
-      <c r="H37" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I37" t="n">
-        <v>22.3085</v>
-      </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>
@@ -25352,7 +25374,7 @@
         </is>
       </c>
       <c r="G38" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H38" s="34" t="inlineStr">
         <is>
@@ -25392,7 +25414,7 @@
         </is>
       </c>
       <c r="G39" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H39" s="34" t="inlineStr">
         <is>
@@ -25432,7 +25454,7 @@
         </is>
       </c>
       <c r="G40" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H40" s="34" t="inlineStr">
         <is>
@@ -25472,7 +25494,7 @@
         </is>
       </c>
       <c r="G41" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H41" s="34" t="inlineStr">
         <is>
@@ -25512,7 +25534,7 @@
         </is>
       </c>
       <c r="G42" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H42" s="34" t="inlineStr">
         <is>
@@ -25552,7 +25574,7 @@
         </is>
       </c>
       <c r="G43" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H43" s="34" t="inlineStr">
         <is>
@@ -25592,7 +25614,7 @@
         </is>
       </c>
       <c r="G44" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H44" s="34" t="inlineStr">
         <is>
@@ -25632,7 +25654,7 @@
         </is>
       </c>
       <c r="G45" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H45" s="34" t="inlineStr">
         <is>
@@ -25672,7 +25694,7 @@
         </is>
       </c>
       <c r="G46" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H46" s="34" t="inlineStr">
         <is>
@@ -25749,7 +25771,7 @@
         </is>
       </c>
       <c r="G48" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H48" s="34" t="inlineStr">
         <is>
@@ -25789,7 +25811,7 @@
         </is>
       </c>
       <c r="G49" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H49" s="34" t="inlineStr">
         <is>
@@ -25829,7 +25851,7 @@
         </is>
       </c>
       <c r="G50" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H50" s="34" t="inlineStr">
         <is>
@@ -25869,7 +25891,7 @@
         </is>
       </c>
       <c r="G51" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H51" s="34" t="inlineStr">
         <is>
@@ -25909,7 +25931,7 @@
         </is>
       </c>
       <c r="G52" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H52" s="34" t="inlineStr">
         <is>
@@ -25949,7 +25971,7 @@
         </is>
       </c>
       <c r="G53" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H53" s="34" t="inlineStr">
         <is>
@@ -25989,7 +26011,7 @@
         </is>
       </c>
       <c r="G54" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H54" s="34" t="inlineStr">
         <is>
@@ -26029,7 +26051,7 @@
         </is>
       </c>
       <c r="G55" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H55" s="34" t="inlineStr">
         <is>
@@ -26069,7 +26091,7 @@
         </is>
       </c>
       <c r="G56" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H56" s="34" t="inlineStr">
         <is>
@@ -26109,7 +26131,7 @@
         </is>
       </c>
       <c r="G57" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H57" s="34" t="inlineStr">
         <is>
@@ -26149,7 +26171,7 @@
         </is>
       </c>
       <c r="G58" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H58" s="34" t="inlineStr">
         <is>
@@ -26189,7 +26211,7 @@
         </is>
       </c>
       <c r="G59" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H59" s="34" t="inlineStr">
         <is>
@@ -26229,7 +26251,7 @@
         </is>
       </c>
       <c r="G60" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H60" s="34" t="inlineStr">
         <is>
@@ -26269,7 +26291,7 @@
         </is>
       </c>
       <c r="G61" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H61" s="34" t="inlineStr">
         <is>
@@ -26309,7 +26331,7 @@
         </is>
       </c>
       <c r="G62" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H62" s="34" t="inlineStr">
         <is>
@@ -26349,7 +26371,7 @@
         </is>
       </c>
       <c r="G63" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H63" s="34" t="inlineStr">
         <is>
@@ -26389,7 +26411,7 @@
         </is>
       </c>
       <c r="G64" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H64" s="34" t="inlineStr">
         <is>
@@ -26429,7 +26451,7 @@
         </is>
       </c>
       <c r="G65" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H65" s="34" t="inlineStr">
         <is>
@@ -26469,7 +26491,7 @@
         </is>
       </c>
       <c r="G66" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H66" s="34" t="inlineStr">
         <is>
@@ -26509,7 +26531,7 @@
         </is>
       </c>
       <c r="G67" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H67" s="34" t="inlineStr">
         <is>
@@ -26549,7 +26571,7 @@
         </is>
       </c>
       <c r="G68" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H68" s="34" t="inlineStr">
         <is>
@@ -26589,7 +26611,7 @@
         </is>
       </c>
       <c r="G69" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H69" s="34" t="inlineStr">
         <is>
@@ -26629,7 +26651,7 @@
         </is>
       </c>
       <c r="G70" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H70" s="34" t="inlineStr">
         <is>
@@ -26669,7 +26691,7 @@
         </is>
       </c>
       <c r="G71" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H71" s="34" t="inlineStr">
         <is>
@@ -26709,7 +26731,7 @@
         </is>
       </c>
       <c r="G72" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H72" s="34" t="inlineStr">
         <is>
@@ -26749,7 +26771,7 @@
         </is>
       </c>
       <c r="G73" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H73" s="34" t="inlineStr">
         <is>
@@ -26789,7 +26811,7 @@
         </is>
       </c>
       <c r="G74" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H74" s="34" t="inlineStr">
         <is>
@@ -26829,7 +26851,7 @@
         </is>
       </c>
       <c r="G75" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H75" s="34" t="inlineStr">
         <is>
@@ -26869,7 +26891,7 @@
         </is>
       </c>
       <c r="G76" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H76" s="34" t="inlineStr">
         <is>
@@ -26909,7 +26931,7 @@
         </is>
       </c>
       <c r="G77" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H77" s="34" t="inlineStr">
         <is>
@@ -26949,7 +26971,7 @@
         </is>
       </c>
       <c r="G78" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H78" s="34" t="inlineStr">
         <is>
@@ -26989,7 +27011,7 @@
         </is>
       </c>
       <c r="G79" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H79" s="34" t="inlineStr">
         <is>
@@ -27029,7 +27051,7 @@
         </is>
       </c>
       <c r="G80" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H80" s="34" t="inlineStr">
         <is>
@@ -27069,7 +27091,7 @@
         </is>
       </c>
       <c r="G81" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H81" s="34" t="inlineStr">
         <is>
@@ -27109,7 +27131,7 @@
         </is>
       </c>
       <c r="G82" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H82" s="34" t="inlineStr">
         <is>
@@ -27149,7 +27171,7 @@
         </is>
       </c>
       <c r="G83" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H83" s="34" t="inlineStr">
         <is>
@@ -27181,7 +27203,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>67.48999999999999</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -27189,7 +27211,7 @@
         </is>
       </c>
       <c r="G84" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H84" s="34" t="inlineStr">
         <is>
@@ -27197,7 +27219,7 @@
         </is>
       </c>
       <c r="I84" t="n">
-        <v>64.454099</v>
+        <v>67.473827</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="58">
@@ -27221,7 +27243,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>609.92</v>
+        <v>613.5700000000001</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -27229,7 +27251,7 @@
         </is>
       </c>
       <c r="G85" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H85" s="34" t="inlineStr">
         <is>
@@ -27237,7 +27259,7 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>604.300021</v>
+        <v>609.785544</v>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="58">
@@ -27261,7 +27283,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>64603</v>
+        <v>65397</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -27269,7 +27291,7 @@
         </is>
       </c>
       <c r="G86" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H86" s="34" t="inlineStr">
         <is>
@@ -27277,7 +27299,7 @@
         </is>
       </c>
       <c r="I86" t="n">
-        <v>63626.823745</v>
+        <v>64587.277657</v>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="58">
@@ -27301,7 +27323,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.006806</v>
+        <v>0.006865</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -27309,7 +27331,7 @@
         </is>
       </c>
       <c r="G87" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H87" s="34" t="inlineStr">
         <is>
@@ -27317,7 +27339,7 @@
         </is>
       </c>
       <c r="I87" t="n">
-        <v>0.006747</v>
+        <v>0.006802</v>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="58">
@@ -27341,7 +27363,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.010593</v>
+        <v>0.01079</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -27349,7 +27371,7 @@
         </is>
       </c>
       <c r="G88" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H88" s="34" t="inlineStr">
         <is>
@@ -27357,7 +27379,7 @@
         </is>
       </c>
       <c r="I88" t="n">
-        <v>0.010357</v>
+        <v>0.010617</v>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="58">
@@ -27381,7 +27403,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>68.98</v>
+        <v>70.78</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -27389,7 +27411,7 @@
         </is>
       </c>
       <c r="G89" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H89" s="34" t="inlineStr">
         <is>
@@ -27397,7 +27419,7 @@
         </is>
       </c>
       <c r="I89" t="n">
-        <v>67.093678</v>
+        <v>68.959726</v>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="58">
@@ -27421,7 +27443,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>2.1</v>
+        <v>2.04</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -27429,7 +27451,7 @@
         </is>
       </c>
       <c r="G90" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H90" s="34" t="inlineStr">
         <is>
@@ -27437,7 +27459,7 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>2.221388</v>
+        <v>2.10347</v>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="58">
@@ -27469,7 +27491,7 @@
         </is>
       </c>
       <c r="G91" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H91" s="34" t="inlineStr">
         <is>
@@ -27501,7 +27523,7 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
-        <v>0.013966</v>
+        <v>0.014121</v>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
@@ -27509,7 +27531,7 @@
         </is>
       </c>
       <c r="G92" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H92" s="34" t="inlineStr">
         <is>
@@ -27517,7 +27539,7 @@
         </is>
       </c>
       <c r="I92" t="n">
-        <v>0.013935</v>
+        <v>0.013981</v>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="58">
@@ -27541,7 +27563,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>2.763192</v>
+        <v>2.767043</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -27549,7 +27571,7 @@
         </is>
       </c>
       <c r="G93" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H93" s="34" t="inlineStr">
         <is>
@@ -27557,7 +27579,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>2.756343</v>
+        <v>2.752933</v>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="58">
@@ -27581,7 +27603,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>25.108926</v>
+        <v>25.650149</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -27589,7 +27611,7 @@
         </is>
       </c>
       <c r="G94" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H94" s="34" t="inlineStr">
         <is>
@@ -27597,7 +27619,7 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>24.625157</v>
+        <v>25.001496</v>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="58">
@@ -27621,7 +27643,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.112009</v>
+        <v>0.113693</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -27629,7 +27651,7 @@
         </is>
       </c>
       <c r="G95" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H95" s="34" t="inlineStr">
         <is>
@@ -27637,7 +27659,7 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>0.110457</v>
+        <v>0.111563</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="58">
@@ -27661,7 +27683,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>19932.1856</v>
+        <v>19971.7035</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -27669,7 +27691,7 @@
         </is>
       </c>
       <c r="G96" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H96" s="34" t="inlineStr">
         <is>
@@ -27677,7 +27699,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>19748.524686</v>
+        <v>19848.519455</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="58">
@@ -27701,7 +27723,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2111226.04</v>
+        <v>2128672.35</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -27709,7 +27731,7 @@
         </is>
       </c>
       <c r="G97" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H97" s="34" t="inlineStr">
         <is>
@@ -27717,7 +27739,7 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>2079324.599992</v>
+        <v>2102315.887721</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="58">
@@ -27741,7 +27763,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>2.871526</v>
+        <v>2.878624</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -27749,7 +27771,7 @@
         </is>
       </c>
       <c r="G98" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H98" s="34" t="inlineStr">
         <is>
@@ -27757,7 +27779,7 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>2.82132</v>
+        <v>2.859995</v>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="58">
@@ -27781,7 +27803,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>55084.1008</v>
+        <v>55711.929</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -27789,7 +27811,7 @@
         </is>
       </c>
       <c r="G99" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H99" s="34" t="inlineStr">
         <is>
@@ -27797,7 +27819,7 @@
         </is>
       </c>
       <c r="I99" t="n">
-        <v>54488.861432</v>
+        <v>54854.917991</v>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="58">
@@ -27821,7 +27843,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>25.033828</v>
+        <v>25.06018</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -27829,7 +27851,7 @@
         </is>
       </c>
       <c r="G100" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H100" s="34" t="inlineStr">
         <is>
@@ -27837,7 +27859,7 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>25.226661</v>
+        <v>24.934249</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="58">
@@ -27861,7 +27883,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>64603</v>
+        <v>65397</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -27869,7 +27891,7 @@
         </is>
       </c>
       <c r="G101" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H101" s="34" t="inlineStr">
         <is>
@@ -27877,7 +27899,7 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>63626.823745</v>
+        <v>64587.277657</v>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="58">
@@ -27901,7 +27923,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>17.64</v>
+        <v>17.91</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -27909,7 +27931,7 @@
         </is>
       </c>
       <c r="G102" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H102" s="34" t="inlineStr">
         <is>
@@ -27917,7 +27939,7 @@
         </is>
       </c>
       <c r="I102" t="n">
-        <v>17.337864</v>
+        <v>17.64308</v>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="58">
@@ -28015,7 +28037,7 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
-        <v>0.006806</v>
+        <v>0.006865</v>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
@@ -28023,7 +28045,7 @@
         </is>
       </c>
       <c r="G105" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H105" s="34" t="inlineStr">
         <is>
@@ -28031,7 +28053,7 @@
         </is>
       </c>
       <c r="I105" t="n">
-        <v>0.006747</v>
+        <v>0.006802</v>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="58">
@@ -28055,7 +28077,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>68.98</v>
+        <v>70.78</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>
@@ -28063,7 +28085,7 @@
         </is>
       </c>
       <c r="G106" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H106" s="34" t="inlineStr">
         <is>
@@ -28071,7 +28093,7 @@
         </is>
       </c>
       <c r="I106" t="n">
-        <v>67.093678</v>
+        <v>68.959726</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="58">
@@ -28103,7 +28125,7 @@
         </is>
       </c>
       <c r="G107" s="28" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="H107" s="34" t="inlineStr">
         <is>
@@ -28135,27 +28157,27 @@
         </is>
       </c>
       <c r="E108" t="n">
+        <v>22.8715</v>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G108" s="47" t="n">
+        <v>46183</v>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I108" t="n">
         <v>23.5969</v>
       </c>
-      <c r="F108" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G108" s="47" t="n">
-        <v>46182</v>
-      </c>
-      <c r="H108" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I108" t="n">
-        <v>23.8653</v>
-      </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily dashboard update (backstop) — 2026-06-16
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-42660" yWindow="-540" windowWidth="32460" windowHeight="17180" tabRatio="500" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Realized" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Realized" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Prices" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Reference" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="AsOfDate">'FX &amp; Assumptions'!$C$5</definedName>
@@ -697,14 +697,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -726,8 +726,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -752,10 +752,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -764,10 +764,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4F81BD"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+              <a:ln w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -777,10 +777,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="C0504D"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -790,10 +790,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="9BBB59"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -803,10 +803,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="8064A2"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -816,10 +816,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4BACC6"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -829,10 +829,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="F79646"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -842,14 +842,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -875,14 +875,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -908,14 +908,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -941,14 +941,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -974,14 +974,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1007,14 +1007,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1038,16 +1038,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1142,16 +1142,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1172,10 +1172,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1187,14 +1187,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1216,8 +1216,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1242,10 +1242,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1254,10 +1254,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4672A8"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1267,10 +1267,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="AB4744"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1280,10 +1280,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="8AA64F"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1293,10 +1293,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="725990"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1306,10 +1306,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4299B0"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1319,10 +1319,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="DC853E"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1332,10 +1332,10 @@
             <idx val="6"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="93A9CE"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1345,10 +1345,10 @@
             <idx val="7"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="D09493"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1358,10 +1358,10 @@
             <idx val="8"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="B8CD97"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1371,14 +1371,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1405,14 +1405,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1439,14 +1439,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1473,14 +1473,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1507,14 +1507,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1541,14 +1541,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1575,14 +1575,14 @@
             <dLbl>
               <idx val="6"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1609,14 +1609,14 @@
             <dLbl>
               <idx val="7"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1643,14 +1643,14 @@
             <dLbl>
               <idx val="8"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1675,16 +1675,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1791,16 +1791,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1821,10 +1821,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1836,14 +1836,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1865,8 +1865,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1893,10 +1893,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1904,16 +1904,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2016,7 +2016,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2025,9 +2025,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2059,7 +2059,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2073,7 +2073,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2082,9 +2082,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2109,16 +2109,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2139,10 +2139,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2154,14 +2154,14 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -2183,8 +2183,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -2200,10 +2200,10 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2211,16 +2211,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2411,7 +2411,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2420,9 +2420,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2454,7 +2454,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2468,7 +2468,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2477,9 +2477,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2504,16 +2504,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2534,10 +2534,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2549,7 +2549,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>1</col>
@@ -2569,9 +2569,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2596,9 +2596,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+          <c:chart r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2623,9 +2623,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+          <c:chart r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2650,9 +2650,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+          <c:chart r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -22047,16 +22047,38 @@
       </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="58">
-      <c r="B20" s="28" t="n"/>
-      <c r="C20" s="29" t="n"/>
-      <c r="D20" s="29" t="n"/>
-      <c r="E20" s="29" t="n"/>
-      <c r="F20" s="30" t="n"/>
-      <c r="G20" s="29" t="n"/>
-      <c r="H20" s="29" t="n"/>
-      <c r="I20" s="29" t="n"/>
-      <c r="J20" s="31" t="n"/>
-      <c r="K20" s="32" t="n"/>
+      <c r="B20" s="28" t="n">
+        <v>46189</v>
+      </c>
+      <c r="C20" s="29" t="n">
+        <v>26427197</v>
+      </c>
+      <c r="D20" s="29" t="n">
+        <v>22739234</v>
+      </c>
+      <c r="E20" s="29" t="n">
+        <v>3687963</v>
+      </c>
+      <c r="F20" s="30" t="n">
+        <v>0.1622</v>
+      </c>
+      <c r="G20" s="29" t="n">
+        <v>18819830</v>
+      </c>
+      <c r="H20" s="29" t="n">
+        <v>5027209</v>
+      </c>
+      <c r="I20" s="29" t="n">
+        <v>1209366</v>
+      </c>
+      <c r="J20" s="31" t="n">
+        <v>32.53</v>
+      </c>
+      <c r="K20" s="32" t="inlineStr">
+        <is>
+          <t>Auto weekly snapshot</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="58">
       <c r="B21" s="28" t="n"/>
@@ -23698,7 +23720,7 @@
         </is>
       </c>
       <c r="C5" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="D5" s="64" t="inlineStr">
         <is>
@@ -23713,11 +23735,11 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>32.55</v>
+        <v>32.53</v>
       </c>
       <c r="D6" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-06-15</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-06-16</t>
         </is>
       </c>
     </row>
@@ -23762,11 +23784,11 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>25.4349</v>
+        <v>25.375</v>
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-06-15</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-06-16</t>
         </is>
       </c>
     </row>
@@ -25374,7 +25396,7 @@
         </is>
       </c>
       <c r="G38" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H38" s="34" t="inlineStr">
         <is>
@@ -25406,7 +25428,7 @@
         </is>
       </c>
       <c r="E39" s="33" t="n">
-        <v>1.079</v>
+        <v>1.066</v>
       </c>
       <c r="F39" s="34" t="inlineStr">
         <is>
@@ -25414,7 +25436,7 @@
         </is>
       </c>
       <c r="G39" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H39" s="34" t="inlineStr">
         <is>
@@ -25422,7 +25444,7 @@
         </is>
       </c>
       <c r="I39" t="n">
-        <v>1.079</v>
+        <v>1.066</v>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="58">
@@ -25454,7 +25476,7 @@
         </is>
       </c>
       <c r="G40" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H40" s="34" t="inlineStr">
         <is>
@@ -25494,7 +25516,7 @@
         </is>
       </c>
       <c r="G41" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H41" s="34" t="inlineStr">
         <is>
@@ -25534,7 +25556,7 @@
         </is>
       </c>
       <c r="G42" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H42" s="34" t="inlineStr">
         <is>
@@ -25566,7 +25588,7 @@
         </is>
       </c>
       <c r="E43" s="33" t="n">
-        <v>5.45</v>
+        <v>5.35</v>
       </c>
       <c r="F43" s="34" t="inlineStr">
         <is>
@@ -25574,7 +25596,7 @@
         </is>
       </c>
       <c r="G43" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H43" s="34" t="inlineStr">
         <is>
@@ -25582,7 +25604,7 @@
         </is>
       </c>
       <c r="I43" t="n">
-        <v>5.45</v>
+        <v>5.35</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="58">
@@ -25614,7 +25636,7 @@
         </is>
       </c>
       <c r="G44" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H44" s="34" t="inlineStr">
         <is>
@@ -25654,7 +25676,7 @@
         </is>
       </c>
       <c r="G45" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H45" s="34" t="inlineStr">
         <is>
@@ -25686,7 +25708,7 @@
         </is>
       </c>
       <c r="E46" s="33" t="n">
-        <v>0.3</v>
+        <v>0.29</v>
       </c>
       <c r="F46" s="34" t="inlineStr">
         <is>
@@ -25694,7 +25716,7 @@
         </is>
       </c>
       <c r="G46" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H46" s="34" t="inlineStr">
         <is>
@@ -25702,7 +25724,7 @@
         </is>
       </c>
       <c r="I46" t="n">
-        <v>0.3</v>
+        <v>0.29</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" s="58">
@@ -25771,7 +25793,7 @@
         </is>
       </c>
       <c r="G48" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H48" s="34" t="inlineStr">
         <is>
@@ -25803,23 +25825,23 @@
         </is>
       </c>
       <c r="E49" s="33" t="n">
+        <v>65</v>
+      </c>
+      <c r="F49" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G49" s="28" t="n">
+        <v>46189</v>
+      </c>
+      <c r="H49" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
         <v>64</v>
-      </c>
-      <c r="F49" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G49" s="28" t="n">
-        <v>46188</v>
-      </c>
-      <c r="H49" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I49" t="n">
-        <v>62.75</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="58">
@@ -25843,7 +25865,7 @@
         </is>
       </c>
       <c r="E50" s="33" t="n">
-        <v>9.300000000000001</v>
+        <v>9.4</v>
       </c>
       <c r="F50" s="34" t="inlineStr">
         <is>
@@ -25851,7 +25873,7 @@
         </is>
       </c>
       <c r="G50" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H50" s="34" t="inlineStr">
         <is>
@@ -25859,7 +25881,7 @@
         </is>
       </c>
       <c r="I50" t="n">
-        <v>9.300000000000001</v>
+        <v>9.4</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="58">
@@ -25883,7 +25905,7 @@
         </is>
       </c>
       <c r="E51" s="33" t="n">
-        <v>15.3</v>
+        <v>15.4</v>
       </c>
       <c r="F51" s="34" t="inlineStr">
         <is>
@@ -25891,7 +25913,7 @@
         </is>
       </c>
       <c r="G51" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H51" s="34" t="inlineStr">
         <is>
@@ -25899,7 +25921,7 @@
         </is>
       </c>
       <c r="I51" t="n">
-        <v>15.3</v>
+        <v>15.4</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" s="58">
@@ -25923,7 +25945,7 @@
         </is>
       </c>
       <c r="E52" s="33" t="n">
-        <v>13.4</v>
+        <v>13.3</v>
       </c>
       <c r="F52" s="34" t="inlineStr">
         <is>
@@ -25931,7 +25953,7 @@
         </is>
       </c>
       <c r="G52" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H52" s="34" t="inlineStr">
         <is>
@@ -25939,7 +25961,7 @@
         </is>
       </c>
       <c r="I52" t="n">
-        <v>13.4</v>
+        <v>13.3</v>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1" s="58">
@@ -25963,7 +25985,7 @@
         </is>
       </c>
       <c r="E53" s="33" t="n">
-        <v>5.55</v>
+        <v>5.45</v>
       </c>
       <c r="F53" s="34" t="inlineStr">
         <is>
@@ -25971,7 +25993,7 @@
         </is>
       </c>
       <c r="G53" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H53" s="34" t="inlineStr">
         <is>
@@ -25979,7 +26001,7 @@
         </is>
       </c>
       <c r="I53" t="n">
-        <v>5.55</v>
+        <v>5.45</v>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="58">
@@ -26003,7 +26025,7 @@
         </is>
       </c>
       <c r="E54" s="33" t="n">
-        <v>20.4</v>
+        <v>21.7</v>
       </c>
       <c r="F54" s="34" t="inlineStr">
         <is>
@@ -26011,7 +26033,7 @@
         </is>
       </c>
       <c r="G54" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H54" s="34" t="inlineStr">
         <is>
@@ -26019,7 +26041,7 @@
         </is>
       </c>
       <c r="I54" t="n">
-        <v>20.4</v>
+        <v>21.700001</v>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="58">
@@ -26051,7 +26073,7 @@
         </is>
       </c>
       <c r="G55" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H55" s="34" t="inlineStr">
         <is>
@@ -26091,7 +26113,7 @@
         </is>
       </c>
       <c r="G56" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H56" s="34" t="inlineStr">
         <is>
@@ -26123,7 +26145,7 @@
         </is>
       </c>
       <c r="E57" s="33" t="n">
-        <v>2.62</v>
+        <v>2.68</v>
       </c>
       <c r="F57" s="34" t="inlineStr">
         <is>
@@ -26131,7 +26153,7 @@
         </is>
       </c>
       <c r="G57" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H57" s="34" t="inlineStr">
         <is>
@@ -26139,7 +26161,7 @@
         </is>
       </c>
       <c r="I57" t="n">
-        <v>2.62</v>
+        <v>2.68</v>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="58">
@@ -26163,7 +26185,7 @@
         </is>
       </c>
       <c r="E58" s="33" t="n">
-        <v>12.1</v>
+        <v>12.2</v>
       </c>
       <c r="F58" s="34" t="inlineStr">
         <is>
@@ -26171,7 +26193,7 @@
         </is>
       </c>
       <c r="G58" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H58" s="34" t="inlineStr">
         <is>
@@ -26203,7 +26225,7 @@
         </is>
       </c>
       <c r="E59" s="33" t="n">
-        <v>17.3</v>
+        <v>18</v>
       </c>
       <c r="F59" s="34" t="inlineStr">
         <is>
@@ -26211,7 +26233,7 @@
         </is>
       </c>
       <c r="G59" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H59" s="34" t="inlineStr">
         <is>
@@ -26243,7 +26265,7 @@
         </is>
       </c>
       <c r="E60" s="33" t="n">
-        <v>180.12</v>
+        <v>189.455</v>
       </c>
       <c r="F60" s="34" t="inlineStr">
         <is>
@@ -26251,7 +26273,7 @@
         </is>
       </c>
       <c r="G60" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H60" s="34" t="inlineStr">
         <is>
@@ -26259,7 +26281,7 @@
         </is>
       </c>
       <c r="I60" t="n">
-        <v>180.119995</v>
+        <v>189.455002</v>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="58">
@@ -26283,7 +26305,7 @@
         </is>
       </c>
       <c r="E61" s="33" t="n">
-        <v>204.02</v>
+        <v>207.155</v>
       </c>
       <c r="F61" s="34" t="inlineStr">
         <is>
@@ -26291,7 +26313,7 @@
         </is>
       </c>
       <c r="G61" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H61" s="34" t="inlineStr">
         <is>
@@ -26299,7 +26321,7 @@
         </is>
       </c>
       <c r="I61" t="n">
-        <v>204.020004</v>
+        <v>207.154999</v>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="58">
@@ -26323,7 +26345,7 @@
         </is>
       </c>
       <c r="E62" s="33" t="n">
-        <v>567.25</v>
+        <v>588.51</v>
       </c>
       <c r="F62" s="34" t="inlineStr">
         <is>
@@ -26331,7 +26353,7 @@
         </is>
       </c>
       <c r="G62" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H62" s="34" t="inlineStr">
         <is>
@@ -26339,7 +26361,7 @@
         </is>
       </c>
       <c r="I62" t="n">
-        <v>552.6400149999999</v>
+        <v>588.51001</v>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1" s="58">
@@ -26363,7 +26385,7 @@
         </is>
       </c>
       <c r="E63" s="33" t="n">
-        <v>164.09</v>
+        <v>167.35</v>
       </c>
       <c r="F63" s="34" t="inlineStr">
         <is>
@@ -26371,7 +26393,7 @@
         </is>
       </c>
       <c r="G63" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H63" s="34" t="inlineStr">
         <is>
@@ -26379,7 +26401,7 @@
         </is>
       </c>
       <c r="I63" t="n">
-        <v>164.089996</v>
+        <v>167.350006</v>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="58">
@@ -26403,7 +26425,7 @@
         </is>
       </c>
       <c r="E64" s="33" t="n">
-        <v>54.59</v>
+        <v>52.56</v>
       </c>
       <c r="F64" s="34" t="inlineStr">
         <is>
@@ -26411,7 +26433,7 @@
         </is>
       </c>
       <c r="G64" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H64" s="34" t="inlineStr">
         <is>
@@ -26419,7 +26441,7 @@
         </is>
       </c>
       <c r="I64" t="n">
-        <v>54.59</v>
+        <v>52.560001</v>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1" s="58">
@@ -26443,7 +26465,7 @@
         </is>
       </c>
       <c r="E65" s="33" t="n">
-        <v>197.45</v>
+        <v>211.14</v>
       </c>
       <c r="F65" s="34" t="inlineStr">
         <is>
@@ -26451,7 +26473,7 @@
         </is>
       </c>
       <c r="G65" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H65" s="34" t="inlineStr">
         <is>
@@ -26459,7 +26481,7 @@
         </is>
       </c>
       <c r="I65" t="n">
-        <v>197.449997</v>
+        <v>211.139999</v>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1" s="58">
@@ -26483,7 +26505,7 @@
         </is>
       </c>
       <c r="E66" s="33" t="n">
-        <v>146.3</v>
+        <v>148.268</v>
       </c>
       <c r="F66" s="34" t="inlineStr">
         <is>
@@ -26491,7 +26513,7 @@
         </is>
       </c>
       <c r="G66" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H66" s="34" t="inlineStr">
         <is>
@@ -26499,7 +26521,7 @@
         </is>
       </c>
       <c r="I66" t="n">
-        <v>146.300003</v>
+        <v>148.267502</v>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1" s="58">
@@ -26523,7 +26545,7 @@
         </is>
       </c>
       <c r="E67" s="33" t="n">
-        <v>148.17</v>
+        <v>142.605</v>
       </c>
       <c r="F67" s="34" t="inlineStr">
         <is>
@@ -26531,7 +26553,7 @@
         </is>
       </c>
       <c r="G67" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H67" s="34" t="inlineStr">
         <is>
@@ -26539,7 +26561,7 @@
         </is>
       </c>
       <c r="I67" t="n">
-        <v>148.169998</v>
+        <v>142.604996</v>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1" s="58">
@@ -26563,7 +26585,7 @@
         </is>
       </c>
       <c r="E68" s="33" t="n">
-        <v>254.54</v>
+        <v>255.22</v>
       </c>
       <c r="F68" s="34" t="inlineStr">
         <is>
@@ -26571,7 +26593,7 @@
         </is>
       </c>
       <c r="G68" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H68" s="34" t="inlineStr">
         <is>
@@ -26579,7 +26601,7 @@
         </is>
       </c>
       <c r="I68" t="n">
-        <v>254.539993</v>
+        <v>255.220001</v>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="58">
@@ -26603,7 +26625,7 @@
         </is>
       </c>
       <c r="E69" s="33" t="n">
-        <v>1133</v>
+        <v>1125.85</v>
       </c>
       <c r="F69" s="34" t="inlineStr">
         <is>
@@ -26611,7 +26633,7 @@
         </is>
       </c>
       <c r="G69" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H69" s="34" t="inlineStr">
         <is>
@@ -26619,7 +26641,7 @@
         </is>
       </c>
       <c r="I69" t="n">
-        <v>1160.949951</v>
+        <v>1125.849976</v>
       </c>
     </row>
     <row r="70" ht="15" customHeight="1" s="58">
@@ -26643,7 +26665,7 @@
         </is>
       </c>
       <c r="E70" s="33" t="n">
-        <v>95.23999999999999</v>
+        <v>100.67</v>
       </c>
       <c r="F70" s="34" t="inlineStr">
         <is>
@@ -26651,7 +26673,7 @@
         </is>
       </c>
       <c r="G70" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H70" s="34" t="inlineStr">
         <is>
@@ -26659,7 +26681,7 @@
         </is>
       </c>
       <c r="I70" t="n">
-        <v>95.239998</v>
+        <v>100.669998</v>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1" s="58">
@@ -26683,7 +26705,7 @@
         </is>
       </c>
       <c r="E71" s="33" t="n">
-        <v>1577.32</v>
+        <v>1652.85</v>
       </c>
       <c r="F71" s="34" t="inlineStr">
         <is>
@@ -26691,7 +26713,7 @@
         </is>
       </c>
       <c r="G71" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H71" s="34" t="inlineStr">
         <is>
@@ -26699,7 +26721,7 @@
         </is>
       </c>
       <c r="I71" t="n">
-        <v>1577.319946</v>
+        <v>1652.849976</v>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1" s="58">
@@ -26723,7 +26745,7 @@
         </is>
       </c>
       <c r="E72" s="33" t="n">
-        <v>111.05</v>
+        <v>111.855</v>
       </c>
       <c r="F72" s="34" t="inlineStr">
         <is>
@@ -26731,7 +26753,7 @@
         </is>
       </c>
       <c r="G72" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H72" s="34" t="inlineStr">
         <is>
@@ -26739,7 +26761,7 @@
         </is>
       </c>
       <c r="I72" t="n">
-        <v>111.050003</v>
+        <v>111.855003</v>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1" s="58">
@@ -26763,7 +26785,7 @@
         </is>
       </c>
       <c r="E73" s="33" t="n">
-        <v>205.19</v>
+        <v>212.24</v>
       </c>
       <c r="F73" s="34" t="inlineStr">
         <is>
@@ -26771,7 +26793,7 @@
         </is>
       </c>
       <c r="G73" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H73" s="34" t="inlineStr">
         <is>
@@ -26779,7 +26801,7 @@
         </is>
       </c>
       <c r="I73" t="n">
-        <v>205.190002</v>
+        <v>212.240005</v>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1" s="58">
@@ -26803,7 +26825,7 @@
         </is>
       </c>
       <c r="E74" s="33" t="n">
-        <v>91.45999999999999</v>
+        <v>93.515</v>
       </c>
       <c r="F74" s="34" t="inlineStr">
         <is>
@@ -26811,7 +26833,7 @@
         </is>
       </c>
       <c r="G74" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H74" s="34" t="inlineStr">
         <is>
@@ -26819,7 +26841,7 @@
         </is>
       </c>
       <c r="I74" t="n">
-        <v>91.459999</v>
+        <v>93.514999</v>
       </c>
     </row>
     <row r="75" ht="15" customHeight="1" s="58">
@@ -26843,7 +26865,7 @@
         </is>
       </c>
       <c r="E75" s="33" t="n">
-        <v>98.59</v>
+        <v>101.215</v>
       </c>
       <c r="F75" s="34" t="inlineStr">
         <is>
@@ -26851,7 +26873,7 @@
         </is>
       </c>
       <c r="G75" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H75" s="34" t="inlineStr">
         <is>
@@ -26859,7 +26881,7 @@
         </is>
       </c>
       <c r="I75" t="n">
-        <v>98.589996</v>
+        <v>101.214996</v>
       </c>
     </row>
     <row r="76" ht="15" customHeight="1" s="58">
@@ -26883,7 +26905,7 @@
         </is>
       </c>
       <c r="E76" s="33" t="n">
-        <v>403.2</v>
+        <v>433.11</v>
       </c>
       <c r="F76" s="34" t="inlineStr">
         <is>
@@ -26891,7 +26913,7 @@
         </is>
       </c>
       <c r="G76" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H76" s="34" t="inlineStr">
         <is>
@@ -26899,7 +26921,7 @@
         </is>
       </c>
       <c r="I76" t="n">
-        <v>403.200012</v>
+        <v>433.109985</v>
       </c>
     </row>
     <row r="77" ht="15" customHeight="1" s="58">
@@ -26923,7 +26945,7 @@
         </is>
       </c>
       <c r="E77" s="33" t="n">
-        <v>406.43</v>
+        <v>409.76</v>
       </c>
       <c r="F77" s="34" t="inlineStr">
         <is>
@@ -26931,7 +26953,7 @@
         </is>
       </c>
       <c r="G77" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H77" s="34" t="inlineStr">
         <is>
@@ -26939,7 +26961,7 @@
         </is>
       </c>
       <c r="I77" t="n">
-        <v>406.429993</v>
+        <v>409.760101</v>
       </c>
     </row>
     <row r="78" ht="15" customHeight="1" s="58">
@@ -26963,7 +26985,7 @@
         </is>
       </c>
       <c r="E78" s="33" t="n">
-        <v>50.25</v>
+        <v>51.15</v>
       </c>
       <c r="F78" s="34" t="inlineStr">
         <is>
@@ -26971,7 +26993,7 @@
         </is>
       </c>
       <c r="G78" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H78" s="34" t="inlineStr">
         <is>
@@ -26979,7 +27001,7 @@
         </is>
       </c>
       <c r="I78" t="n">
-        <v>51</v>
+        <v>51.150002</v>
       </c>
     </row>
     <row r="79" ht="15" customHeight="1" s="58">
@@ -27003,23 +27025,23 @@
         </is>
       </c>
       <c r="E79" s="33" t="n">
+        <v>97.5</v>
+      </c>
+      <c r="F79" s="34" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G79" s="28" t="n">
+        <v>46189</v>
+      </c>
+      <c r="H79" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I79" t="n">
         <v>95.5</v>
-      </c>
-      <c r="F79" s="34" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="G79" s="28" t="n">
-        <v>46188</v>
-      </c>
-      <c r="H79" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I79" t="n">
-        <v>92.959999</v>
       </c>
     </row>
     <row r="80" ht="15" customHeight="1" s="58">
@@ -27043,7 +27065,7 @@
         </is>
       </c>
       <c r="E80" s="33" t="n">
-        <v>291.13</v>
+        <v>296.2</v>
       </c>
       <c r="F80" s="34" t="inlineStr">
         <is>
@@ -27051,7 +27073,7 @@
         </is>
       </c>
       <c r="G80" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H80" s="34" t="inlineStr">
         <is>
@@ -27059,7 +27081,7 @@
         </is>
       </c>
       <c r="I80" t="n">
-        <v>291.130005</v>
+        <v>296.200012</v>
       </c>
     </row>
     <row r="81" ht="15" customHeight="1" s="58">
@@ -27083,7 +27105,7 @@
         </is>
       </c>
       <c r="E81" s="33" t="n">
-        <v>159.78</v>
+        <v>170.7</v>
       </c>
       <c r="F81" s="34" t="inlineStr">
         <is>
@@ -27091,7 +27113,7 @@
         </is>
       </c>
       <c r="G81" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H81" s="34" t="inlineStr">
         <is>
@@ -27099,7 +27121,7 @@
         </is>
       </c>
       <c r="I81" t="n">
-        <v>159.779999</v>
+        <v>170.699997</v>
       </c>
     </row>
     <row r="82" ht="15" customHeight="1" s="58">
@@ -27123,7 +27145,7 @@
         </is>
       </c>
       <c r="E82" s="33" t="n">
-        <v>566.98</v>
+        <v>594.6799999999999</v>
       </c>
       <c r="F82" s="34" t="inlineStr">
         <is>
@@ -27131,7 +27153,7 @@
         </is>
       </c>
       <c r="G82" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H82" s="34" t="inlineStr">
         <is>
@@ -27139,7 +27161,7 @@
         </is>
       </c>
       <c r="I82" t="n">
-        <v>566.97998</v>
+        <v>594.679993</v>
       </c>
     </row>
     <row r="83" ht="15" customHeight="1" s="58">
@@ -27163,7 +27185,7 @@
         </is>
       </c>
       <c r="E83" s="33" t="n">
-        <v>130</v>
+        <v>109.99</v>
       </c>
       <c r="F83" s="34" t="inlineStr">
         <is>
@@ -27171,7 +27193,7 @@
         </is>
       </c>
       <c r="G83" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H83" s="34" t="inlineStr">
         <is>
@@ -27179,7 +27201,7 @@
         </is>
       </c>
       <c r="I83" t="n">
-        <v>122.339996</v>
+        <v>109.990097</v>
       </c>
     </row>
     <row r="84" ht="15" customHeight="1" s="58">
@@ -27203,7 +27225,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>68.09999999999999</v>
+        <v>75.73</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -27211,7 +27233,7 @@
         </is>
       </c>
       <c r="G84" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H84" s="34" t="inlineStr">
         <is>
@@ -27219,7 +27241,7 @@
         </is>
       </c>
       <c r="I84" t="n">
-        <v>67.473827</v>
+        <v>65.556043</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="58">
@@ -27243,7 +27265,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>613.5700000000001</v>
+        <v>622.8099999999999</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -27251,7 +27273,7 @@
         </is>
       </c>
       <c r="G85" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H85" s="34" t="inlineStr">
         <is>
@@ -27259,7 +27281,7 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>609.785544</v>
+        <v>604.099198</v>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="58">
@@ -27283,7 +27305,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>65397</v>
+        <v>66787</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -27291,7 +27313,7 @@
         </is>
       </c>
       <c r="G86" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H86" s="34" t="inlineStr">
         <is>
@@ -27299,7 +27321,7 @@
         </is>
       </c>
       <c r="I86" t="n">
-        <v>64587.277657</v>
+        <v>63754.471854</v>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="58">
@@ -27323,7 +27345,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.006865</v>
+        <v>0.007369</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -27331,7 +27353,7 @@
         </is>
       </c>
       <c r="G87" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H87" s="34" t="inlineStr">
         <is>
@@ -27339,7 +27361,7 @@
         </is>
       </c>
       <c r="I87" t="n">
-        <v>0.006802</v>
+        <v>0.006501</v>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="58">
@@ -27363,7 +27385,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.01079</v>
+        <v>0.011464</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -27371,7 +27393,7 @@
         </is>
       </c>
       <c r="G88" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H88" s="34" t="inlineStr">
         <is>
@@ -27379,7 +27401,7 @@
         </is>
       </c>
       <c r="I88" t="n">
-        <v>0.010617</v>
+        <v>0.010382</v>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="58">
@@ -27403,7 +27425,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>70.78</v>
+        <v>75.45999999999999</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -27411,7 +27433,7 @@
         </is>
       </c>
       <c r="G89" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H89" s="34" t="inlineStr">
         <is>
@@ -27419,7 +27441,7 @@
         </is>
       </c>
       <c r="I89" t="n">
-        <v>68.959726</v>
+        <v>67.364605</v>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="58">
@@ -27443,7 +27465,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>2.04</v>
+        <v>2</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -27451,7 +27473,7 @@
         </is>
       </c>
       <c r="G90" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H90" s="34" t="inlineStr">
         <is>
@@ -27459,7 +27481,7 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>2.10347</v>
+        <v>1.97687</v>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="58">
@@ -27491,7 +27513,7 @@
         </is>
       </c>
       <c r="G91" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H91" s="34" t="inlineStr">
         <is>
@@ -27523,7 +27545,7 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
-        <v>0.014121</v>
+        <v>0.01642</v>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
@@ -27531,7 +27553,7 @@
         </is>
       </c>
       <c r="G92" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H92" s="34" t="inlineStr">
         <is>
@@ -27539,7 +27561,7 @@
         </is>
       </c>
       <c r="I92" t="n">
-        <v>0.013981</v>
+        <v>0.013468</v>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="58">
@@ -27563,7 +27585,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>2.767043</v>
+        <v>2.881377</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -27571,7 +27593,7 @@
         </is>
       </c>
       <c r="G93" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H93" s="34" t="inlineStr">
         <is>
@@ -27579,7 +27601,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>2.752933</v>
+        <v>2.663097</v>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="58">
@@ -27603,7 +27625,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>25.650149</v>
+        <v>26.320478</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -27611,7 +27633,7 @@
         </is>
       </c>
       <c r="G94" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H94" s="34" t="inlineStr">
         <is>
@@ -27619,7 +27641,7 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>25.001496</v>
+        <v>24.345992</v>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="58">
@@ -27643,7 +27665,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.113693</v>
+        <v>0.116758</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -27651,7 +27673,7 @@
         </is>
       </c>
       <c r="G95" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H95" s="34" t="inlineStr">
         <is>
@@ -27659,7 +27681,7 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>0.111563</v>
+        <v>0.108153</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="58">
@@ -27683,7 +27705,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>19971.7035</v>
+        <v>20260.0093</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -27691,7 +27713,7 @@
         </is>
       </c>
       <c r="G96" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H96" s="34" t="inlineStr">
         <is>
@@ -27699,7 +27721,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>19848.519455</v>
+        <v>19651.346896</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="58">
@@ -27723,7 +27745,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2128672.35</v>
+        <v>2172581.11</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -27731,7 +27753,7 @@
         </is>
       </c>
       <c r="G97" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H97" s="34" t="inlineStr">
         <is>
@@ -27739,7 +27761,7 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>2102315.887721</v>
+        <v>2073932.9694</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="58">
@@ -27763,7 +27785,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>2.878624</v>
+        <v>2.908377</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -27771,7 +27793,7 @@
         </is>
       </c>
       <c r="G98" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H98" s="34" t="inlineStr">
         <is>
@@ -27779,7 +27801,7 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>2.859995</v>
+        <v>2.807326</v>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="58">
@@ -27803,7 +27825,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>55711.929</v>
+        <v>59507.129</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -27811,7 +27833,7 @@
         </is>
       </c>
       <c r="G99" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H99" s="34" t="inlineStr">
         <is>
@@ -27819,7 +27841,7 @@
         </is>
       </c>
       <c r="I99" t="n">
-        <v>54854.917991</v>
+        <v>54015.191291</v>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="58">
@@ -27843,7 +27865,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>25.06018</v>
+        <v>25.347278</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -27851,7 +27873,7 @@
         </is>
       </c>
       <c r="G100" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H100" s="34" t="inlineStr">
         <is>
@@ -27859,7 +27881,7 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>24.934249</v>
+        <v>24.738972</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="58">
@@ -27883,7 +27905,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>65397</v>
+        <v>66787</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -27891,7 +27913,7 @@
         </is>
       </c>
       <c r="G101" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H101" s="34" t="inlineStr">
         <is>
@@ -27899,7 +27921,7 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>64587.277657</v>
+        <v>63754.471854</v>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="58">
@@ -27923,7 +27945,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>17.91</v>
+        <v>18.26</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -27931,7 +27953,7 @@
         </is>
       </c>
       <c r="G102" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H102" s="34" t="inlineStr">
         <is>
@@ -27939,7 +27961,7 @@
         </is>
       </c>
       <c r="I102" t="n">
-        <v>17.64308</v>
+        <v>17.304945</v>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="58">
@@ -28037,7 +28059,7 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
-        <v>0.006865</v>
+        <v>0.007369</v>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
@@ -28045,7 +28067,7 @@
         </is>
       </c>
       <c r="G105" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H105" s="34" t="inlineStr">
         <is>
@@ -28053,7 +28075,7 @@
         </is>
       </c>
       <c r="I105" t="n">
-        <v>0.006802</v>
+        <v>0.006501</v>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="58">
@@ -28077,7 +28099,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>70.78</v>
+        <v>75.45999999999999</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>
@@ -28085,7 +28107,7 @@
         </is>
       </c>
       <c r="G106" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H106" s="34" t="inlineStr">
         <is>
@@ -28093,7 +28115,7 @@
         </is>
       </c>
       <c r="I106" t="n">
-        <v>68.959726</v>
+        <v>67.364605</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="58">
@@ -28125,7 +28147,7 @@
         </is>
       </c>
       <c r="G107" s="28" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="H107" s="34" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Daily dashboard update — 2026-06-16
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-42660" yWindow="-540" windowWidth="32460" windowHeight="17180" tabRatio="500" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Realized" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Prices" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Reference" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Realized" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="AsOfDate">'FX &amp; Assumptions'!$C$5</definedName>
@@ -697,14 +697,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -726,8 +726,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -752,10 +752,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -764,10 +764,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4F81BD"/>
               </a:solidFill>
-              <a:ln w="0">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -777,10 +777,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="C0504D"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -790,10 +790,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="9BBB59"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -803,10 +803,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="8064A2"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -816,10 +816,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4BACC6"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -829,10 +829,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="F79646"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -842,14 +842,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -875,14 +875,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -908,14 +908,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -941,14 +941,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -974,14 +974,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1007,14 +1007,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1038,16 +1038,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1142,16 +1142,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1172,10 +1172,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1187,14 +1187,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1216,8 +1216,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1242,10 +1242,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1254,10 +1254,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4672A8"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1267,10 +1267,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="AB4744"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1280,10 +1280,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="8AA64F"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1293,10 +1293,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="725990"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1306,10 +1306,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4299B0"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1319,10 +1319,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="DC853E"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1332,10 +1332,10 @@
             <idx val="6"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="93A9CE"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1345,10 +1345,10 @@
             <idx val="7"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="D09493"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1358,10 +1358,10 @@
             <idx val="8"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="B8CD97"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1371,14 +1371,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1405,14 +1405,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1439,14 +1439,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1473,14 +1473,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1507,14 +1507,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1541,14 +1541,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1575,14 +1575,14 @@
             <dLbl>
               <idx val="6"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1609,14 +1609,14 @@
             <dLbl>
               <idx val="7"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1643,14 +1643,14 @@
             <dLbl>
               <idx val="8"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1675,16 +1675,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1791,16 +1791,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1821,10 +1821,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1836,14 +1836,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1865,8 +1865,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1893,10 +1893,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1904,16 +1904,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2016,7 +2016,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2025,9 +2025,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2059,7 +2059,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="9360">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2073,7 +2073,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2082,9 +2082,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2109,16 +2109,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2139,10 +2139,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2154,14 +2154,14 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -2183,8 +2183,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -2200,10 +2200,10 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2211,16 +2211,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2411,7 +2411,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2420,9 +2420,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2454,7 +2454,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="9360">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2468,7 +2468,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2477,9 +2477,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2504,16 +2504,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2534,10 +2534,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2549,7 +2549,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>1</col>
@@ -2569,9 +2569,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2596,9 +2596,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2623,9 +2623,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId3"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2650,9 +2650,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId4"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -22051,28 +22051,28 @@
         <v>46189</v>
       </c>
       <c r="C20" s="29" t="n">
-        <v>26427197</v>
+        <v>26416936</v>
       </c>
       <c r="D20" s="29" t="n">
-        <v>22739234</v>
+        <v>22740625</v>
       </c>
       <c r="E20" s="29" t="n">
-        <v>3687963</v>
+        <v>3676311</v>
       </c>
       <c r="F20" s="30" t="n">
-        <v>0.1622</v>
+        <v>0.1617</v>
       </c>
       <c r="G20" s="29" t="n">
         <v>18819830</v>
       </c>
       <c r="H20" s="29" t="n">
-        <v>5027209</v>
+        <v>5027896</v>
       </c>
       <c r="I20" s="29" t="n">
-        <v>1209366</v>
+        <v>1197790</v>
       </c>
       <c r="J20" s="31" t="n">
-        <v>32.53</v>
+        <v>32.54</v>
       </c>
       <c r="K20" s="32" t="inlineStr">
         <is>
@@ -23735,7 +23735,7 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>32.53</v>
+        <v>32.54</v>
       </c>
       <c r="D6" s="64" t="inlineStr">
         <is>
@@ -23784,7 +23784,7 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>25.375</v>
+        <v>25.3866</v>
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
@@ -25404,7 +25404,7 @@
         </is>
       </c>
       <c r="I38" t="n">
-        <v>23.360001</v>
+        <v>23.52</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="58">
@@ -25524,7 +25524,7 @@
         </is>
       </c>
       <c r="I41" t="n">
-        <v>20.940001</v>
+        <v>21.75</v>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="58">
@@ -25564,7 +25564,7 @@
         </is>
       </c>
       <c r="I42" t="n">
-        <v>218.660004</v>
+        <v>220.389999</v>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="58">
@@ -26265,7 +26265,7 @@
         </is>
       </c>
       <c r="E60" s="33" t="n">
-        <v>189.455</v>
+        <v>191.6</v>
       </c>
       <c r="F60" s="34" t="inlineStr">
         <is>
@@ -26281,7 +26281,7 @@
         </is>
       </c>
       <c r="I60" t="n">
-        <v>189.455002</v>
+        <v>191.600006</v>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="58">
@@ -26305,7 +26305,7 @@
         </is>
       </c>
       <c r="E61" s="33" t="n">
-        <v>207.155</v>
+        <v>206.36</v>
       </c>
       <c r="F61" s="34" t="inlineStr">
         <is>
@@ -26321,7 +26321,7 @@
         </is>
       </c>
       <c r="I61" t="n">
-        <v>207.154999</v>
+        <v>206.360001</v>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="58">
@@ -26345,7 +26345,7 @@
         </is>
       </c>
       <c r="E62" s="33" t="n">
-        <v>588.51</v>
+        <v>585.78</v>
       </c>
       <c r="F62" s="34" t="inlineStr">
         <is>
@@ -26361,7 +26361,7 @@
         </is>
       </c>
       <c r="I62" t="n">
-        <v>588.51001</v>
+        <v>585.780029</v>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1" s="58">
@@ -26385,7 +26385,7 @@
         </is>
       </c>
       <c r="E63" s="33" t="n">
-        <v>167.35</v>
+        <v>165.94</v>
       </c>
       <c r="F63" s="34" t="inlineStr">
         <is>
@@ -26401,7 +26401,7 @@
         </is>
       </c>
       <c r="I63" t="n">
-        <v>167.350006</v>
+        <v>165.940002</v>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="58">
@@ -26425,7 +26425,7 @@
         </is>
       </c>
       <c r="E64" s="33" t="n">
-        <v>52.56</v>
+        <v>52.395</v>
       </c>
       <c r="F64" s="34" t="inlineStr">
         <is>
@@ -26441,7 +26441,7 @@
         </is>
       </c>
       <c r="I64" t="n">
-        <v>52.560001</v>
+        <v>52.395</v>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1" s="58">
@@ -26465,7 +26465,7 @@
         </is>
       </c>
       <c r="E65" s="33" t="n">
-        <v>211.14</v>
+        <v>211.45</v>
       </c>
       <c r="F65" s="34" t="inlineStr">
         <is>
@@ -26481,7 +26481,7 @@
         </is>
       </c>
       <c r="I65" t="n">
-        <v>211.139999</v>
+        <v>211.449997</v>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1" s="58">
@@ -26505,7 +26505,7 @@
         </is>
       </c>
       <c r="E66" s="33" t="n">
-        <v>148.268</v>
+        <v>149.49</v>
       </c>
       <c r="F66" s="34" t="inlineStr">
         <is>
@@ -26521,7 +26521,7 @@
         </is>
       </c>
       <c r="I66" t="n">
-        <v>148.267502</v>
+        <v>149.490005</v>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1" s="58">
@@ -26545,7 +26545,7 @@
         </is>
       </c>
       <c r="E67" s="33" t="n">
-        <v>142.605</v>
+        <v>142.77</v>
       </c>
       <c r="F67" s="34" t="inlineStr">
         <is>
@@ -26561,7 +26561,7 @@
         </is>
       </c>
       <c r="I67" t="n">
-        <v>142.604996</v>
+        <v>142.770004</v>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1" s="58">
@@ -26585,7 +26585,7 @@
         </is>
       </c>
       <c r="E68" s="33" t="n">
-        <v>255.22</v>
+        <v>256.42</v>
       </c>
       <c r="F68" s="34" t="inlineStr">
         <is>
@@ -26601,7 +26601,7 @@
         </is>
       </c>
       <c r="I68" t="n">
-        <v>255.220001</v>
+        <v>256.420013</v>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="58">
@@ -26625,7 +26625,7 @@
         </is>
       </c>
       <c r="E69" s="33" t="n">
-        <v>1125.85</v>
+        <v>1129.35</v>
       </c>
       <c r="F69" s="34" t="inlineStr">
         <is>
@@ -26641,7 +26641,7 @@
         </is>
       </c>
       <c r="I69" t="n">
-        <v>1125.849976</v>
+        <v>1129.349976</v>
       </c>
     </row>
     <row r="70" ht="15" customHeight="1" s="58">
@@ -26665,7 +26665,7 @@
         </is>
       </c>
       <c r="E70" s="33" t="n">
-        <v>100.67</v>
+        <v>100.32</v>
       </c>
       <c r="F70" s="34" t="inlineStr">
         <is>
@@ -26681,7 +26681,7 @@
         </is>
       </c>
       <c r="I70" t="n">
-        <v>100.669998</v>
+        <v>100.32</v>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1" s="58">
@@ -26705,7 +26705,7 @@
         </is>
       </c>
       <c r="E71" s="33" t="n">
-        <v>1652.85</v>
+        <v>1652.29</v>
       </c>
       <c r="F71" s="34" t="inlineStr">
         <is>
@@ -26721,7 +26721,7 @@
         </is>
       </c>
       <c r="I71" t="n">
-        <v>1652.849976</v>
+        <v>1652.290039</v>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1" s="58">
@@ -26745,7 +26745,7 @@
         </is>
       </c>
       <c r="E72" s="33" t="n">
-        <v>111.855</v>
+        <v>110.81</v>
       </c>
       <c r="F72" s="34" t="inlineStr">
         <is>
@@ -26761,7 +26761,7 @@
         </is>
       </c>
       <c r="I72" t="n">
-        <v>111.855003</v>
+        <v>110.809998</v>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1" s="58">
@@ -26785,7 +26785,7 @@
         </is>
       </c>
       <c r="E73" s="33" t="n">
-        <v>212.24</v>
+        <v>212.45</v>
       </c>
       <c r="F73" s="34" t="inlineStr">
         <is>
@@ -26801,7 +26801,7 @@
         </is>
       </c>
       <c r="I73" t="n">
-        <v>212.240005</v>
+        <v>212.449997</v>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1" s="58">
@@ -26825,7 +26825,7 @@
         </is>
       </c>
       <c r="E74" s="33" t="n">
-        <v>93.515</v>
+        <v>92.97</v>
       </c>
       <c r="F74" s="34" t="inlineStr">
         <is>
@@ -26841,7 +26841,7 @@
         </is>
       </c>
       <c r="I74" t="n">
-        <v>93.514999</v>
+        <v>92.970001</v>
       </c>
     </row>
     <row r="75" ht="15" customHeight="1" s="58">
@@ -26865,7 +26865,7 @@
         </is>
       </c>
       <c r="E75" s="33" t="n">
-        <v>101.215</v>
+        <v>101.28</v>
       </c>
       <c r="F75" s="34" t="inlineStr">
         <is>
@@ -26881,7 +26881,7 @@
         </is>
       </c>
       <c r="I75" t="n">
-        <v>101.214996</v>
+        <v>101.279999</v>
       </c>
     </row>
     <row r="76" ht="15" customHeight="1" s="58">
@@ -26905,7 +26905,7 @@
         </is>
       </c>
       <c r="E76" s="33" t="n">
-        <v>433.11</v>
+        <v>432.41</v>
       </c>
       <c r="F76" s="34" t="inlineStr">
         <is>
@@ -26921,7 +26921,7 @@
         </is>
       </c>
       <c r="I76" t="n">
-        <v>433.109985</v>
+        <v>432.410004</v>
       </c>
     </row>
     <row r="77" ht="15" customHeight="1" s="58">
@@ -26945,7 +26945,7 @@
         </is>
       </c>
       <c r="E77" s="33" t="n">
-        <v>409.76</v>
+        <v>411.15</v>
       </c>
       <c r="F77" s="34" t="inlineStr">
         <is>
@@ -26961,7 +26961,7 @@
         </is>
       </c>
       <c r="I77" t="n">
-        <v>409.760101</v>
+        <v>411.149994</v>
       </c>
     </row>
     <row r="78" ht="15" customHeight="1" s="58">
@@ -26985,7 +26985,7 @@
         </is>
       </c>
       <c r="E78" s="33" t="n">
-        <v>51.15</v>
+        <v>51.66</v>
       </c>
       <c r="F78" s="34" t="inlineStr">
         <is>
@@ -27001,7 +27001,7 @@
         </is>
       </c>
       <c r="I78" t="n">
-        <v>51.150002</v>
+        <v>51.66</v>
       </c>
     </row>
     <row r="79" ht="15" customHeight="1" s="58">
@@ -27025,7 +27025,7 @@
         </is>
       </c>
       <c r="E79" s="33" t="n">
-        <v>97.5</v>
+        <v>96.89</v>
       </c>
       <c r="F79" s="34" t="inlineStr">
         <is>
@@ -27041,7 +27041,7 @@
         </is>
       </c>
       <c r="I79" t="n">
-        <v>95.5</v>
+        <v>96.889999</v>
       </c>
     </row>
     <row r="80" ht="15" customHeight="1" s="58">
@@ -27065,7 +27065,7 @@
         </is>
       </c>
       <c r="E80" s="33" t="n">
-        <v>296.2</v>
+        <v>296.42</v>
       </c>
       <c r="F80" s="34" t="inlineStr">
         <is>
@@ -27081,7 +27081,7 @@
         </is>
       </c>
       <c r="I80" t="n">
-        <v>296.200012</v>
+        <v>296.420013</v>
       </c>
     </row>
     <row r="81" ht="15" customHeight="1" s="58">
@@ -27105,7 +27105,7 @@
         </is>
       </c>
       <c r="E81" s="33" t="n">
-        <v>170.7</v>
+        <v>169.62</v>
       </c>
       <c r="F81" s="34" t="inlineStr">
         <is>
@@ -27121,7 +27121,7 @@
         </is>
       </c>
       <c r="I81" t="n">
-        <v>170.699997</v>
+        <v>169.619995</v>
       </c>
     </row>
     <row r="82" ht="15" customHeight="1" s="58">
@@ -27145,7 +27145,7 @@
         </is>
       </c>
       <c r="E82" s="33" t="n">
-        <v>594.6799999999999</v>
+        <v>593.48</v>
       </c>
       <c r="F82" s="34" t="inlineStr">
         <is>
@@ -27161,7 +27161,7 @@
         </is>
       </c>
       <c r="I82" t="n">
-        <v>594.679993</v>
+        <v>593.47998</v>
       </c>
     </row>
     <row r="83" ht="15" customHeight="1" s="58">
@@ -27185,7 +27185,7 @@
         </is>
       </c>
       <c r="E83" s="33" t="n">
-        <v>109.99</v>
+        <v>110</v>
       </c>
       <c r="F83" s="34" t="inlineStr">
         <is>
@@ -27201,7 +27201,7 @@
         </is>
       </c>
       <c r="I83" t="n">
-        <v>109.990097</v>
+        <v>130</v>
       </c>
     </row>
     <row r="84" ht="15" customHeight="1" s="58">
@@ -27225,7 +27225,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>75.73</v>
+        <v>73.84</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -27241,7 +27241,7 @@
         </is>
       </c>
       <c r="I84" t="n">
-        <v>65.556043</v>
+        <v>68.104428</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="58">
@@ -27265,7 +27265,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>622.8099999999999</v>
+        <v>617.1</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -27281,7 +27281,7 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>604.099198</v>
+        <v>613.567738</v>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="58">
@@ -27305,7 +27305,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>66787</v>
+        <v>66335</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -27321,7 +27321,7 @@
         </is>
       </c>
       <c r="I86" t="n">
-        <v>63754.471854</v>
+        <v>65396.650356</v>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="58">
@@ -27345,7 +27345,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.007369</v>
+        <v>0.00712</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -27361,7 +27361,7 @@
         </is>
       </c>
       <c r="I87" t="n">
-        <v>0.006501</v>
+        <v>0.006866</v>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="58">
@@ -27385,7 +27385,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.011464</v>
+        <v>0.011422</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -27401,7 +27401,7 @@
         </is>
       </c>
       <c r="I88" t="n">
-        <v>0.010382</v>
+        <v>0.010802</v>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="58">
@@ -27425,7 +27425,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>75.45999999999999</v>
+        <v>74.18000000000001</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -27441,7 +27441,7 @@
         </is>
       </c>
       <c r="I89" t="n">
-        <v>67.364605</v>
+        <v>70.774581</v>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="58">
@@ -27465,7 +27465,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>2</v>
+        <v>1.99</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -27481,7 +27481,7 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>1.97687</v>
+        <v>2.04956</v>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="58">
@@ -27545,7 +27545,7 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
-        <v>0.01642</v>
+        <v>0.016021</v>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
@@ -27561,7 +27561,7 @@
         </is>
       </c>
       <c r="I92" t="n">
-        <v>0.013468</v>
+        <v>0.014121</v>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="58">
@@ -27585,7 +27585,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>2.881377</v>
+        <v>2.811261</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -27601,7 +27601,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>2.663097</v>
+        <v>2.766373</v>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="58">
@@ -27625,7 +27625,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>26.320478</v>
+        <v>25.782809</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -27641,7 +27641,7 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>24.345992</v>
+        <v>25.707333</v>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="58">
@@ -27665,7 +27665,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.116758</v>
+        <v>0.114032</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -27681,7 +27681,7 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>0.108153</v>
+        <v>0.113817</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="58">
@@ -27705,7 +27705,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>20260.0093</v>
+        <v>20080.434</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -27721,7 +27721,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>19651.346896</v>
+        <v>19965.494209</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="58">
@@ -27745,7 +27745,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2172581.11</v>
+        <v>2158540.9</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -27761,7 +27761,7 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>2073932.9694</v>
+        <v>2128007.002575</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="58">
@@ -27785,7 +27785,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>2.908377</v>
+        <v>2.861307</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -27801,7 +27801,7 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>2.807326</v>
+        <v>2.880897</v>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="58">
@@ -27825,7 +27825,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>59507.129</v>
+        <v>58401.165</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -27841,7 +27841,7 @@
         </is>
       </c>
       <c r="I99" t="n">
-        <v>54015.191291</v>
+        <v>55694.466891</v>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="58">
@@ -27865,7 +27865,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>25.347278</v>
+        <v>25.266789</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -27881,7 +27881,7 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>24.738972</v>
+        <v>25.053858</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="58">
@@ -27905,7 +27905,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>66787</v>
+        <v>66335</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -27921,7 +27921,7 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>63754.471854</v>
+        <v>65396.650356</v>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="58">
@@ -27945,7 +27945,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>18.26</v>
+        <v>18.02</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -27961,7 +27961,7 @@
         </is>
       </c>
       <c r="I102" t="n">
-        <v>17.304945</v>
+        <v>17.9002</v>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="58">
@@ -28059,7 +28059,7 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
-        <v>0.007369</v>
+        <v>0.00712</v>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
@@ -28075,7 +28075,7 @@
         </is>
       </c>
       <c r="I105" t="n">
-        <v>0.006501</v>
+        <v>0.006866</v>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="58">
@@ -28099,7 +28099,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>75.45999999999999</v>
+        <v>74.18000000000001</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>
@@ -28115,7 +28115,7 @@
         </is>
       </c>
       <c r="I106" t="n">
-        <v>67.364605</v>
+        <v>70.774581</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="58">

</xml_diff>

<commit_message>
Daily dashboard update (backstop) — 2026-06-17
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-42660" yWindow="-540" windowWidth="32460" windowHeight="17180" tabRatio="500" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Realized" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Realized" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Prices" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Reference" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="AsOfDate">'FX &amp; Assumptions'!$C$5</definedName>
@@ -697,14 +697,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -726,8 +726,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -752,10 +752,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -764,10 +764,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4F81BD"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+              <a:ln w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -777,10 +777,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="C0504D"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -790,10 +790,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="9BBB59"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -803,10 +803,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="8064A2"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -816,10 +816,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4BACC6"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -829,10 +829,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="F79646"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -842,14 +842,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -875,14 +875,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -908,14 +908,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -941,14 +941,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -974,14 +974,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1007,14 +1007,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1038,16 +1038,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1142,16 +1142,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1172,10 +1172,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1187,14 +1187,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1216,8 +1216,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1242,10 +1242,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1254,10 +1254,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4672A8"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1267,10 +1267,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="AB4744"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1280,10 +1280,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="8AA64F"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1293,10 +1293,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="725990"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1306,10 +1306,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4299B0"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1319,10 +1319,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="DC853E"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1332,10 +1332,10 @@
             <idx val="6"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="93A9CE"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1345,10 +1345,10 @@
             <idx val="7"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="D09493"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1358,10 +1358,10 @@
             <idx val="8"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="B8CD97"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1371,14 +1371,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1405,14 +1405,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1439,14 +1439,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1473,14 +1473,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1507,14 +1507,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1541,14 +1541,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1575,14 +1575,14 @@
             <dLbl>
               <idx val="6"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1609,14 +1609,14 @@
             <dLbl>
               <idx val="7"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1643,14 +1643,14 @@
             <dLbl>
               <idx val="8"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1675,16 +1675,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1791,16 +1791,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1821,10 +1821,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1836,14 +1836,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1865,8 +1865,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1893,10 +1893,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1904,16 +1904,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2016,7 +2016,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2025,9 +2025,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2059,7 +2059,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2073,7 +2073,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2082,9 +2082,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2109,16 +2109,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2139,10 +2139,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2154,14 +2154,14 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -2183,8 +2183,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -2200,10 +2200,10 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2211,16 +2211,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2411,7 +2411,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2420,9 +2420,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2454,7 +2454,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2468,7 +2468,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2477,9 +2477,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2504,16 +2504,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2534,10 +2534,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2549,7 +2549,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>1</col>
@@ -2569,9 +2569,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2596,9 +2596,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+          <c:chart r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2623,9 +2623,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+          <c:chart r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2650,9 +2650,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+          <c:chart r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -22081,16 +22081,38 @@
       </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="58">
-      <c r="B21" s="28" t="n"/>
-      <c r="C21" s="29" t="n"/>
-      <c r="D21" s="29" t="n"/>
-      <c r="E21" s="29" t="n"/>
-      <c r="F21" s="30" t="n"/>
-      <c r="G21" s="29" t="n"/>
-      <c r="H21" s="29" t="n"/>
-      <c r="I21" s="29" t="n"/>
-      <c r="J21" s="31" t="n"/>
-      <c r="K21" s="32" t="n"/>
+      <c r="B21" s="28" t="n">
+        <v>46190</v>
+      </c>
+      <c r="C21" s="29" t="n">
+        <v>26404449</v>
+      </c>
+      <c r="D21" s="29" t="n">
+        <v>22738651</v>
+      </c>
+      <c r="E21" s="29" t="n">
+        <v>3665798</v>
+      </c>
+      <c r="F21" s="30" t="n">
+        <v>0.1612</v>
+      </c>
+      <c r="G21" s="29" t="n">
+        <v>18859011</v>
+      </c>
+      <c r="H21" s="29" t="n">
+        <v>4978471</v>
+      </c>
+      <c r="I21" s="29" t="n">
+        <v>1188979</v>
+      </c>
+      <c r="J21" s="31" t="n">
+        <v>32.54</v>
+      </c>
+      <c r="K21" s="32" t="inlineStr">
+        <is>
+          <t>Auto weekly snapshot</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="58">
       <c r="B22" s="28" t="n"/>
@@ -23720,7 +23742,7 @@
         </is>
       </c>
       <c r="C5" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="D5" s="64" t="inlineStr">
         <is>
@@ -23739,7 +23761,7 @@
       </c>
       <c r="D6" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-06-16</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-06-17</t>
         </is>
       </c>
     </row>
@@ -23784,11 +23806,11 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>25.3866</v>
+        <v>25.327</v>
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-06-16</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-06-17</t>
         </is>
       </c>
     </row>
@@ -23903,27 +23925,27 @@
         </is>
       </c>
       <c r="E5" s="33" t="n">
+        <v>25.8262</v>
+      </c>
+      <c r="F5" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G5" s="28" t="n">
+        <v>46185</v>
+      </c>
+      <c r="H5" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
         <v>25.5328</v>
       </c>
-      <c r="F5" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G5" s="28" t="n">
-        <v>46184</v>
-      </c>
-      <c r="H5" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I5" t="n">
-        <v>23.4501</v>
-      </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>
@@ -23948,27 +23970,27 @@
         </is>
       </c>
       <c r="E6" s="33" t="n">
+        <v>10.6878</v>
+      </c>
+      <c r="F6" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G6" s="28" t="n">
+        <v>46188</v>
+      </c>
+      <c r="H6" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
         <v>10.6873</v>
       </c>
-      <c r="F6" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G6" s="28" t="n">
-        <v>46185</v>
-      </c>
-      <c r="H6" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I6" t="n">
-        <v>10.6872</v>
-      </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
     </row>
@@ -23993,27 +24015,27 @@
         </is>
       </c>
       <c r="E7" s="33" t="n">
+        <v>7.1641</v>
+      </c>
+      <c r="F7" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G7" s="28" t="n">
+        <v>46185</v>
+      </c>
+      <c r="H7" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
         <v>7.0558</v>
       </c>
-      <c r="F7" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G7" s="28" t="n">
-        <v>46184</v>
-      </c>
-      <c r="H7" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I7" t="n">
-        <v>7.0666</v>
-      </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>
@@ -24038,27 +24060,27 @@
         </is>
       </c>
       <c r="E8" s="33" t="n">
+        <v>9.5237</v>
+      </c>
+      <c r="F8" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G8" s="28" t="n">
+        <v>46185</v>
+      </c>
+      <c r="H8" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
         <v>9.4458</v>
       </c>
-      <c r="F8" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G8" s="28" t="n">
-        <v>46184</v>
-      </c>
-      <c r="H8" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I8" t="n">
-        <v>9.3483</v>
-      </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>
@@ -24083,27 +24105,27 @@
         </is>
       </c>
       <c r="E9" s="33" t="n">
+        <v>9.372999999999999</v>
+      </c>
+      <c r="F9" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G9" s="28" t="n">
+        <v>46188</v>
+      </c>
+      <c r="H9" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
         <v>9.285500000000001</v>
       </c>
-      <c r="F9" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G9" s="28" t="n">
-        <v>46185</v>
-      </c>
-      <c r="H9" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I9" t="n">
-        <v>9.2189</v>
-      </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
     </row>
@@ -24128,27 +24150,27 @@
         </is>
       </c>
       <c r="E10" s="33" t="n">
+        <v>13.2399</v>
+      </c>
+      <c r="F10" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G10" s="28" t="n">
+        <v>46185</v>
+      </c>
+      <c r="H10" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
         <v>12.9605</v>
       </c>
-      <c r="F10" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G10" s="28" t="n">
-        <v>46184</v>
-      </c>
-      <c r="H10" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I10" t="n">
-        <v>12.9779</v>
-      </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>
@@ -24173,27 +24195,27 @@
         </is>
       </c>
       <c r="E11" s="33" t="n">
+        <v>13.2787</v>
+      </c>
+      <c r="F11" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G11" s="28" t="n">
+        <v>46188</v>
+      </c>
+      <c r="H11" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
         <v>13.2722</v>
       </c>
-      <c r="F11" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G11" s="28" t="n">
-        <v>46185</v>
-      </c>
-      <c r="H11" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I11" t="n">
-        <v>13.0418</v>
-      </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
     </row>
@@ -24218,27 +24240,27 @@
         </is>
       </c>
       <c r="E12" s="33" t="n">
+        <v>26.987</v>
+      </c>
+      <c r="F12" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G12" s="28" t="n">
+        <v>46188</v>
+      </c>
+      <c r="H12" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
         <v>26.8895</v>
       </c>
-      <c r="F12" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G12" s="28" t="n">
-        <v>46185</v>
-      </c>
-      <c r="H12" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I12" t="n">
-        <v>26.2924</v>
-      </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
     </row>
@@ -24263,27 +24285,27 @@
         </is>
       </c>
       <c r="E13" s="33" t="n">
+        <v>36.4884</v>
+      </c>
+      <c r="F13" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G13" s="28" t="n">
+        <v>46188</v>
+      </c>
+      <c r="H13" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
         <v>36.5289</v>
       </c>
-      <c r="F13" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G13" s="28" t="n">
-        <v>46185</v>
-      </c>
-      <c r="H13" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I13" t="n">
-        <v>36.0361</v>
-      </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
     </row>
@@ -24308,27 +24330,27 @@
         </is>
       </c>
       <c r="E14" s="33" t="n">
+        <v>25.5415</v>
+      </c>
+      <c r="F14" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G14" s="28" t="n">
+        <v>46188</v>
+      </c>
+      <c r="H14" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
         <v>25.535</v>
       </c>
-      <c r="F14" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G14" s="28" t="n">
-        <v>46185</v>
-      </c>
-      <c r="H14" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I14" t="n">
-        <v>25.2656</v>
-      </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
     </row>
@@ -24353,27 +24375,27 @@
         </is>
       </c>
       <c r="E15" s="33" t="n">
+        <v>15.0939</v>
+      </c>
+      <c r="F15" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G15" s="28" t="n">
+        <v>46184</v>
+      </c>
+      <c r="H15" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
         <v>14.919</v>
       </c>
-      <c r="F15" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G15" s="28" t="n">
-        <v>46183</v>
-      </c>
-      <c r="H15" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I15" t="n">
-        <v>15.0551</v>
-      </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
     </row>
@@ -24398,27 +24420,27 @@
         </is>
       </c>
       <c r="E16" s="33" t="n">
+        <v>81.8086</v>
+      </c>
+      <c r="F16" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G16" s="28" t="n">
+        <v>46188</v>
+      </c>
+      <c r="H16" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
         <v>81.94029999999999</v>
       </c>
-      <c r="F16" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G16" s="28" t="n">
-        <v>46185</v>
-      </c>
-      <c r="H16" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I16" t="n">
-        <v>80.91589999999999</v>
-      </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
     </row>
@@ -24443,27 +24465,27 @@
         </is>
       </c>
       <c r="E17" s="33" t="n">
+        <v>53.5038</v>
+      </c>
+      <c r="F17" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G17" s="28" t="n">
+        <v>46188</v>
+      </c>
+      <c r="H17" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
         <v>53.4365</v>
       </c>
-      <c r="F17" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G17" s="28" t="n">
-        <v>46185</v>
-      </c>
-      <c r="H17" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I17" t="n">
-        <v>52.8716</v>
-      </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
     </row>
@@ -24488,27 +24510,27 @@
         </is>
       </c>
       <c r="E18" s="33" t="n">
+        <v>16.5024</v>
+      </c>
+      <c r="F18" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G18" s="28" t="n">
+        <v>46188</v>
+      </c>
+      <c r="H18" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
         <v>16.4623</v>
       </c>
-      <c r="F18" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G18" s="28" t="n">
-        <v>46185</v>
-      </c>
-      <c r="H18" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I18" t="n">
-        <v>16.4428</v>
-      </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
     </row>
@@ -24533,27 +24555,27 @@
         </is>
       </c>
       <c r="E19" s="33" t="n">
+        <v>23.4061</v>
+      </c>
+      <c r="F19" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G19" s="28" t="n">
+        <v>46188</v>
+      </c>
+      <c r="H19" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
         <v>23.4045</v>
       </c>
-      <c r="F19" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G19" s="28" t="n">
-        <v>46185</v>
-      </c>
-      <c r="H19" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I19" t="n">
-        <v>23.4043</v>
-      </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
     </row>
@@ -24578,27 +24600,27 @@
         </is>
       </c>
       <c r="E20" s="33" t="n">
+        <v>40.7663</v>
+      </c>
+      <c r="F20" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G20" s="28" t="n">
+        <v>46185</v>
+      </c>
+      <c r="H20" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
         <v>40.574</v>
       </c>
-      <c r="F20" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G20" s="28" t="n">
-        <v>46184</v>
-      </c>
-      <c r="H20" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I20" t="n">
-        <v>39.919</v>
-      </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>
@@ -24623,27 +24645,27 @@
         </is>
       </c>
       <c r="E21" s="33" t="n">
+        <v>13.6767</v>
+      </c>
+      <c r="F21" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G21" s="28" t="n">
+        <v>46188</v>
+      </c>
+      <c r="H21" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
         <v>13.5289</v>
       </c>
-      <c r="F21" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G21" s="28" t="n">
-        <v>46185</v>
-      </c>
-      <c r="H21" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I21" t="n">
-        <v>13.2943</v>
-      </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
     </row>
@@ -24668,27 +24690,27 @@
         </is>
       </c>
       <c r="E22" s="33" t="n">
+        <v>13.3532</v>
+      </c>
+      <c r="F22" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G22" s="28" t="n">
+        <v>46185</v>
+      </c>
+      <c r="H22" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
         <v>13.2862</v>
       </c>
-      <c r="F22" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G22" s="28" t="n">
-        <v>46184</v>
-      </c>
-      <c r="H22" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I22" t="n">
-        <v>13.3451</v>
-      </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>
@@ -24713,27 +24735,27 @@
         </is>
       </c>
       <c r="E23" s="33" t="n">
+        <v>12.4628</v>
+      </c>
+      <c r="F23" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G23" s="28" t="n">
+        <v>46188</v>
+      </c>
+      <c r="H23" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
         <v>12.4646</v>
       </c>
-      <c r="F23" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G23" s="28" t="n">
-        <v>46185</v>
-      </c>
-      <c r="H23" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I23" t="n">
-        <v>12.299</v>
-      </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
     </row>
@@ -24758,27 +24780,27 @@
         </is>
       </c>
       <c r="E24" s="33" t="n">
+        <v>11.7378</v>
+      </c>
+      <c r="F24" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G24" s="28" t="n">
+        <v>46185</v>
+      </c>
+      <c r="H24" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
         <v>11.56</v>
       </c>
-      <c r="F24" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G24" s="28" t="n">
-        <v>46184</v>
-      </c>
-      <c r="H24" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I24" t="n">
-        <v>11.6527</v>
-      </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>
@@ -24803,27 +24825,27 @@
         </is>
       </c>
       <c r="E25" s="33" t="n">
+        <v>9.921799999999999</v>
+      </c>
+      <c r="F25" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G25" s="28" t="n">
+        <v>46188</v>
+      </c>
+      <c r="H25" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
         <v>9.825200000000001</v>
       </c>
-      <c r="F25" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G25" s="28" t="n">
-        <v>46185</v>
-      </c>
-      <c r="H25" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I25" t="n">
-        <v>9.909700000000001</v>
-      </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
     </row>
@@ -24848,27 +24870,27 @@
         </is>
       </c>
       <c r="E26" s="33" t="n">
+        <v>13.9253</v>
+      </c>
+      <c r="F26" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G26" s="28" t="n">
+        <v>46188</v>
+      </c>
+      <c r="H26" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
         <v>13.7868</v>
       </c>
-      <c r="F26" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G26" s="28" t="n">
-        <v>46185</v>
-      </c>
-      <c r="H26" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I26" t="n">
-        <v>13.909</v>
-      </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
     </row>
@@ -24893,27 +24915,27 @@
         </is>
       </c>
       <c r="E27" s="33" t="n">
+        <v>17.1935</v>
+      </c>
+      <c r="F27" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G27" s="28" t="n">
+        <v>46188</v>
+      </c>
+      <c r="H27" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
         <v>17.0399</v>
       </c>
-      <c r="F27" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G27" s="28" t="n">
-        <v>46185</v>
-      </c>
-      <c r="H27" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I27" t="n">
-        <v>16.7383</v>
-      </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
     </row>
@@ -24938,27 +24960,27 @@
         </is>
       </c>
       <c r="E28" s="33" t="n">
+        <v>19.2686</v>
+      </c>
+      <c r="F28" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G28" s="28" t="n">
+        <v>46188</v>
+      </c>
+      <c r="H28" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
         <v>18.7544</v>
       </c>
-      <c r="F28" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G28" s="28" t="n">
-        <v>46185</v>
-      </c>
-      <c r="H28" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I28" t="n">
-        <v>18.1673</v>
-      </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
     </row>
@@ -24983,27 +25005,27 @@
         </is>
       </c>
       <c r="E29" s="33" t="n">
+        <v>26.8484</v>
+      </c>
+      <c r="F29" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G29" s="28" t="n">
+        <v>46185</v>
+      </c>
+      <c r="H29" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
         <v>27.104</v>
       </c>
-      <c r="F29" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G29" s="28" t="n">
-        <v>46184</v>
-      </c>
-      <c r="H29" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I29" t="n">
-        <v>24.2974</v>
-      </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>
@@ -25028,27 +25050,27 @@
         </is>
       </c>
       <c r="E30" s="33" t="n">
+        <v>39.1699</v>
+      </c>
+      <c r="F30" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G30" s="28" t="n">
+        <v>46185</v>
+      </c>
+      <c r="H30" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
         <v>36.9119</v>
       </c>
-      <c r="F30" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G30" s="28" t="n">
-        <v>46184</v>
-      </c>
-      <c r="H30" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I30" t="n">
-        <v>36.0272</v>
-      </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>
@@ -25073,27 +25095,27 @@
         </is>
       </c>
       <c r="E31" s="33" t="n">
+        <v>13.0122</v>
+      </c>
+      <c r="F31" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G31" s="28" t="n">
+        <v>46188</v>
+      </c>
+      <c r="H31" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
         <v>13.0229</v>
       </c>
-      <c r="F31" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G31" s="28" t="n">
-        <v>46185</v>
-      </c>
-      <c r="H31" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I31" t="n">
-        <v>12.8526</v>
-      </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
     </row>
@@ -25118,27 +25140,27 @@
         </is>
       </c>
       <c r="E32" s="33" t="n">
+        <v>21.7065</v>
+      </c>
+      <c r="F32" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G32" s="28" t="n">
+        <v>46188</v>
+      </c>
+      <c r="H32" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
         <v>21.706</v>
       </c>
-      <c r="F32" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G32" s="28" t="n">
-        <v>46185</v>
-      </c>
-      <c r="H32" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I32" t="n">
-        <v>21.7059</v>
-      </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
     </row>
@@ -25163,27 +25185,27 @@
         </is>
       </c>
       <c r="E33" s="33" t="n">
+        <v>12.5219</v>
+      </c>
+      <c r="F33" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G33" s="28" t="n">
+        <v>46188</v>
+      </c>
+      <c r="H33" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
         <v>12.5506</v>
       </c>
-      <c r="F33" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G33" s="28" t="n">
-        <v>46185</v>
-      </c>
-      <c r="H33" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I33" t="n">
-        <v>12.4116</v>
-      </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
     </row>
@@ -25208,27 +25230,27 @@
         </is>
       </c>
       <c r="E34" s="33" t="n">
+        <v>16.2066</v>
+      </c>
+      <c r="F34" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G34" s="28" t="n">
+        <v>46188</v>
+      </c>
+      <c r="H34" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
         <v>16.2056</v>
       </c>
-      <c r="F34" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G34" s="28" t="n">
-        <v>46185</v>
-      </c>
-      <c r="H34" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I34" t="n">
-        <v>16.2054</v>
-      </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
     </row>
@@ -25253,27 +25275,27 @@
         </is>
       </c>
       <c r="E35" s="33" t="n">
+        <v>27.2155</v>
+      </c>
+      <c r="F35" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G35" s="28" t="n">
+        <v>46185</v>
+      </c>
+      <c r="H35" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
         <v>27.4092</v>
       </c>
-      <c r="F35" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G35" s="28" t="n">
-        <v>46184</v>
-      </c>
-      <c r="H35" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I35" t="n">
-        <v>26.542</v>
-      </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>
@@ -25298,27 +25320,27 @@
         </is>
       </c>
       <c r="E36" s="33" t="n">
+        <v>10.1561</v>
+      </c>
+      <c r="F36" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G36" s="28" t="n">
+        <v>46188</v>
+      </c>
+      <c r="H36" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
         <v>10.079</v>
       </c>
-      <c r="F36" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G36" s="28" t="n">
-        <v>46185</v>
-      </c>
-      <c r="H36" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I36" t="n">
-        <v>10.0297</v>
-      </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
     </row>
@@ -25343,27 +25365,27 @@
         </is>
       </c>
       <c r="E37" s="33" t="n">
+        <v>22.7039</v>
+      </c>
+      <c r="F37" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G37" s="28" t="n">
+        <v>46188</v>
+      </c>
+      <c r="H37" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
         <v>22.7488</v>
       </c>
-      <c r="F37" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G37" s="28" t="n">
-        <v>46185</v>
-      </c>
-      <c r="H37" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I37" t="n">
-        <v>22.4356</v>
-      </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
     </row>
@@ -25388,7 +25410,7 @@
         </is>
       </c>
       <c r="E38" s="33" t="n">
-        <v>23.36</v>
+        <v>23.52</v>
       </c>
       <c r="F38" s="34" t="inlineStr">
         <is>
@@ -25396,7 +25418,7 @@
         </is>
       </c>
       <c r="G38" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H38" s="34" t="inlineStr">
         <is>
@@ -25440,7 +25462,7 @@
       </c>
       <c r="H39" s="34" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="I39" t="n">
@@ -25476,7 +25498,7 @@
         </is>
       </c>
       <c r="G40" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H40" s="34" t="inlineStr">
         <is>
@@ -25508,7 +25530,7 @@
         </is>
       </c>
       <c r="E41" s="33" t="n">
-        <v>20.94</v>
+        <v>21.75</v>
       </c>
       <c r="F41" s="34" t="inlineStr">
         <is>
@@ -25516,7 +25538,7 @@
         </is>
       </c>
       <c r="G41" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H41" s="34" t="inlineStr">
         <is>
@@ -25524,7 +25546,7 @@
         </is>
       </c>
       <c r="I41" t="n">
-        <v>21.75</v>
+        <v>20.940001</v>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="58">
@@ -25548,7 +25570,7 @@
         </is>
       </c>
       <c r="E42" s="33" t="n">
-        <v>218.66</v>
+        <v>220.39</v>
       </c>
       <c r="F42" s="34" t="inlineStr">
         <is>
@@ -25556,7 +25578,7 @@
         </is>
       </c>
       <c r="G42" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H42" s="34" t="inlineStr">
         <is>
@@ -25596,7 +25618,7 @@
         </is>
       </c>
       <c r="G43" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H43" s="34" t="inlineStr">
         <is>
@@ -25628,23 +25650,23 @@
         </is>
       </c>
       <c r="E44" s="33" t="n">
+        <v>175.5</v>
+      </c>
+      <c r="F44" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G44" s="28" t="n">
+        <v>46190</v>
+      </c>
+      <c r="H44" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
         <v>172.5</v>
-      </c>
-      <c r="F44" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G44" s="28" t="n">
-        <v>46189</v>
-      </c>
-      <c r="H44" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I44" t="n">
-        <v>168.5</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="58">
@@ -25668,7 +25690,7 @@
         </is>
       </c>
       <c r="E45" s="33" t="n">
-        <v>0.45</v>
+        <v>0.44</v>
       </c>
       <c r="F45" s="34" t="inlineStr">
         <is>
@@ -25676,7 +25698,7 @@
         </is>
       </c>
       <c r="G45" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H45" s="34" t="inlineStr">
         <is>
@@ -25684,7 +25706,7 @@
         </is>
       </c>
       <c r="I45" t="n">
-        <v>0.45</v>
+        <v>0.44</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="58">
@@ -25716,7 +25738,7 @@
         </is>
       </c>
       <c r="G46" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H46" s="34" t="inlineStr">
         <is>
@@ -25793,7 +25815,7 @@
         </is>
       </c>
       <c r="G48" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H48" s="34" t="inlineStr">
         <is>
@@ -25825,23 +25847,23 @@
         </is>
       </c>
       <c r="E49" s="33" t="n">
+        <v>64.25</v>
+      </c>
+      <c r="F49" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G49" s="28" t="n">
+        <v>46190</v>
+      </c>
+      <c r="H49" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
         <v>65</v>
-      </c>
-      <c r="F49" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G49" s="28" t="n">
-        <v>46189</v>
-      </c>
-      <c r="H49" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I49" t="n">
-        <v>64</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="58">
@@ -25865,7 +25887,7 @@
         </is>
       </c>
       <c r="E50" s="33" t="n">
-        <v>9.4</v>
+        <v>9.5</v>
       </c>
       <c r="F50" s="34" t="inlineStr">
         <is>
@@ -25873,7 +25895,7 @@
         </is>
       </c>
       <c r="G50" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H50" s="34" t="inlineStr">
         <is>
@@ -25905,7 +25927,7 @@
         </is>
       </c>
       <c r="E51" s="33" t="n">
-        <v>15.4</v>
+        <v>15.6</v>
       </c>
       <c r="F51" s="34" t="inlineStr">
         <is>
@@ -25913,7 +25935,7 @@
         </is>
       </c>
       <c r="G51" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H51" s="34" t="inlineStr">
         <is>
@@ -25921,7 +25943,7 @@
         </is>
       </c>
       <c r="I51" t="n">
-        <v>15.4</v>
+        <v>15.6</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" s="58">
@@ -25945,7 +25967,7 @@
         </is>
       </c>
       <c r="E52" s="33" t="n">
-        <v>13.3</v>
+        <v>13.4</v>
       </c>
       <c r="F52" s="34" t="inlineStr">
         <is>
@@ -25953,7 +25975,7 @@
         </is>
       </c>
       <c r="G52" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H52" s="34" t="inlineStr">
         <is>
@@ -25961,7 +25983,7 @@
         </is>
       </c>
       <c r="I52" t="n">
-        <v>13.3</v>
+        <v>13.4</v>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1" s="58">
@@ -25993,7 +26015,7 @@
         </is>
       </c>
       <c r="G53" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H53" s="34" t="inlineStr">
         <is>
@@ -26025,7 +26047,7 @@
         </is>
       </c>
       <c r="E54" s="33" t="n">
-        <v>21.7</v>
+        <v>21.8</v>
       </c>
       <c r="F54" s="34" t="inlineStr">
         <is>
@@ -26033,7 +26055,7 @@
         </is>
       </c>
       <c r="G54" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H54" s="34" t="inlineStr">
         <is>
@@ -26041,7 +26063,7 @@
         </is>
       </c>
       <c r="I54" t="n">
-        <v>21.700001</v>
+        <v>21.799999</v>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="58">
@@ -26073,7 +26095,7 @@
         </is>
       </c>
       <c r="G55" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H55" s="34" t="inlineStr">
         <is>
@@ -26105,7 +26127,7 @@
         </is>
       </c>
       <c r="E56" s="33" t="n">
-        <v>4.84</v>
+        <v>4.86</v>
       </c>
       <c r="F56" s="34" t="inlineStr">
         <is>
@@ -26113,7 +26135,7 @@
         </is>
       </c>
       <c r="G56" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H56" s="34" t="inlineStr">
         <is>
@@ -26121,7 +26143,7 @@
         </is>
       </c>
       <c r="I56" t="n">
-        <v>4.84</v>
+        <v>4.86</v>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1" s="58">
@@ -26145,7 +26167,7 @@
         </is>
       </c>
       <c r="E57" s="33" t="n">
-        <v>2.68</v>
+        <v>2.64</v>
       </c>
       <c r="F57" s="34" t="inlineStr">
         <is>
@@ -26153,7 +26175,7 @@
         </is>
       </c>
       <c r="G57" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H57" s="34" t="inlineStr">
         <is>
@@ -26161,7 +26183,7 @@
         </is>
       </c>
       <c r="I57" t="n">
-        <v>2.68</v>
+        <v>2.64</v>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="58">
@@ -26185,7 +26207,7 @@
         </is>
       </c>
       <c r="E58" s="33" t="n">
-        <v>12.2</v>
+        <v>12.3</v>
       </c>
       <c r="F58" s="34" t="inlineStr">
         <is>
@@ -26193,7 +26215,7 @@
         </is>
       </c>
       <c r="G58" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H58" s="34" t="inlineStr">
         <is>
@@ -26201,7 +26223,7 @@
         </is>
       </c>
       <c r="I58" t="n">
-        <v>12.1</v>
+        <v>12.3</v>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="58">
@@ -26233,7 +26255,7 @@
         </is>
       </c>
       <c r="G59" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H59" s="34" t="inlineStr">
         <is>
@@ -26265,7 +26287,7 @@
         </is>
       </c>
       <c r="E60" s="33" t="n">
-        <v>191.6</v>
+        <v>180.475</v>
       </c>
       <c r="F60" s="34" t="inlineStr">
         <is>
@@ -26273,7 +26295,7 @@
         </is>
       </c>
       <c r="G60" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H60" s="34" t="inlineStr">
         <is>
@@ -26281,7 +26303,7 @@
         </is>
       </c>
       <c r="I60" t="n">
-        <v>191.600006</v>
+        <v>180.475006</v>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="58">
@@ -26305,7 +26327,7 @@
         </is>
       </c>
       <c r="E61" s="33" t="n">
-        <v>206.36</v>
+        <v>206.95</v>
       </c>
       <c r="F61" s="34" t="inlineStr">
         <is>
@@ -26313,7 +26335,7 @@
         </is>
       </c>
       <c r="G61" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H61" s="34" t="inlineStr">
         <is>
@@ -26321,7 +26343,7 @@
         </is>
       </c>
       <c r="I61" t="n">
-        <v>206.360001</v>
+        <v>206.949997</v>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="58">
@@ -26345,7 +26367,7 @@
         </is>
       </c>
       <c r="E62" s="33" t="n">
-        <v>585.78</v>
+        <v>577.88</v>
       </c>
       <c r="F62" s="34" t="inlineStr">
         <is>
@@ -26353,7 +26375,7 @@
         </is>
       </c>
       <c r="G62" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H62" s="34" t="inlineStr">
         <is>
@@ -26361,7 +26383,7 @@
         </is>
       </c>
       <c r="I62" t="n">
-        <v>585.780029</v>
+        <v>577.880005</v>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1" s="58">
@@ -26385,7 +26407,7 @@
         </is>
       </c>
       <c r="E63" s="33" t="n">
-        <v>165.94</v>
+        <v>163.458</v>
       </c>
       <c r="F63" s="34" t="inlineStr">
         <is>
@@ -26393,7 +26415,7 @@
         </is>
       </c>
       <c r="G63" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H63" s="34" t="inlineStr">
         <is>
@@ -26401,7 +26423,7 @@
         </is>
       </c>
       <c r="I63" t="n">
-        <v>165.940002</v>
+        <v>163.457993</v>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="58">
@@ -26425,7 +26447,7 @@
         </is>
       </c>
       <c r="E64" s="33" t="n">
-        <v>52.395</v>
+        <v>51.7</v>
       </c>
       <c r="F64" s="34" t="inlineStr">
         <is>
@@ -26433,7 +26455,7 @@
         </is>
       </c>
       <c r="G64" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H64" s="34" t="inlineStr">
         <is>
@@ -26441,7 +26463,7 @@
         </is>
       </c>
       <c r="I64" t="n">
-        <v>52.395</v>
+        <v>51.700001</v>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1" s="58">
@@ -26465,7 +26487,7 @@
         </is>
       </c>
       <c r="E65" s="33" t="n">
-        <v>211.45</v>
+        <v>206.005</v>
       </c>
       <c r="F65" s="34" t="inlineStr">
         <is>
@@ -26473,7 +26495,7 @@
         </is>
       </c>
       <c r="G65" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H65" s="34" t="inlineStr">
         <is>
@@ -26481,7 +26503,7 @@
         </is>
       </c>
       <c r="I65" t="n">
-        <v>211.449997</v>
+        <v>206.005005</v>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1" s="58">
@@ -26505,7 +26527,7 @@
         </is>
       </c>
       <c r="E66" s="33" t="n">
-        <v>149.49</v>
+        <v>145.73</v>
       </c>
       <c r="F66" s="34" t="inlineStr">
         <is>
@@ -26513,7 +26535,7 @@
         </is>
       </c>
       <c r="G66" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H66" s="34" t="inlineStr">
         <is>
@@ -26521,7 +26543,7 @@
         </is>
       </c>
       <c r="I66" t="n">
-        <v>149.490005</v>
+        <v>145.729996</v>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1" s="58">
@@ -26545,7 +26567,7 @@
         </is>
       </c>
       <c r="E67" s="33" t="n">
-        <v>142.77</v>
+        <v>143.41</v>
       </c>
       <c r="F67" s="34" t="inlineStr">
         <is>
@@ -26553,7 +26575,7 @@
         </is>
       </c>
       <c r="G67" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H67" s="34" t="inlineStr">
         <is>
@@ -26561,7 +26583,7 @@
         </is>
       </c>
       <c r="I67" t="n">
-        <v>142.770004</v>
+        <v>143.410004</v>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1" s="58">
@@ -26585,7 +26607,7 @@
         </is>
       </c>
       <c r="E68" s="33" t="n">
-        <v>256.42</v>
+        <v>241.69</v>
       </c>
       <c r="F68" s="34" t="inlineStr">
         <is>
@@ -26593,7 +26615,7 @@
         </is>
       </c>
       <c r="G68" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H68" s="34" t="inlineStr">
         <is>
@@ -26601,7 +26623,7 @@
         </is>
       </c>
       <c r="I68" t="n">
-        <v>256.420013</v>
+        <v>241.690002</v>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="58">
@@ -26625,7 +26647,7 @@
         </is>
       </c>
       <c r="E69" s="33" t="n">
-        <v>1129.35</v>
+        <v>1126.47</v>
       </c>
       <c r="F69" s="34" t="inlineStr">
         <is>
@@ -26633,7 +26655,7 @@
         </is>
       </c>
       <c r="G69" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H69" s="34" t="inlineStr">
         <is>
@@ -26641,7 +26663,7 @@
         </is>
       </c>
       <c r="I69" t="n">
-        <v>1129.349976</v>
+        <v>1126.469971</v>
       </c>
     </row>
     <row r="70" ht="15" customHeight="1" s="58">
@@ -26665,7 +26687,7 @@
         </is>
       </c>
       <c r="E70" s="33" t="n">
-        <v>100.32</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="F70" s="34" t="inlineStr">
         <is>
@@ -26673,7 +26695,7 @@
         </is>
       </c>
       <c r="G70" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H70" s="34" t="inlineStr">
         <is>
@@ -26681,7 +26703,7 @@
         </is>
       </c>
       <c r="I70" t="n">
-        <v>100.32</v>
+        <v>97.099998</v>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1" s="58">
@@ -26705,7 +26727,7 @@
         </is>
       </c>
       <c r="E71" s="33" t="n">
-        <v>1652.29</v>
+        <v>1543.38</v>
       </c>
       <c r="F71" s="34" t="inlineStr">
         <is>
@@ -26713,7 +26735,7 @@
         </is>
       </c>
       <c r="G71" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H71" s="34" t="inlineStr">
         <is>
@@ -26721,7 +26743,7 @@
         </is>
       </c>
       <c r="I71" t="n">
-        <v>1652.290039</v>
+        <v>1543.380005</v>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1" s="58">
@@ -26745,7 +26767,7 @@
         </is>
       </c>
       <c r="E72" s="33" t="n">
-        <v>110.81</v>
+        <v>108.36</v>
       </c>
       <c r="F72" s="34" t="inlineStr">
         <is>
@@ -26753,7 +26775,7 @@
         </is>
       </c>
       <c r="G72" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H72" s="34" t="inlineStr">
         <is>
@@ -26761,7 +26783,7 @@
         </is>
       </c>
       <c r="I72" t="n">
-        <v>110.809998</v>
+        <v>108.360001</v>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1" s="58">
@@ -26785,7 +26807,7 @@
         </is>
       </c>
       <c r="E73" s="33" t="n">
-        <v>212.45</v>
+        <v>208.965</v>
       </c>
       <c r="F73" s="34" t="inlineStr">
         <is>
@@ -26793,7 +26815,7 @@
         </is>
       </c>
       <c r="G73" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H73" s="34" t="inlineStr">
         <is>
@@ -26801,7 +26823,7 @@
         </is>
       </c>
       <c r="I73" t="n">
-        <v>212.449997</v>
+        <v>208.964996</v>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1" s="58">
@@ -26825,7 +26847,7 @@
         </is>
       </c>
       <c r="E74" s="33" t="n">
-        <v>92.97</v>
+        <v>90.09</v>
       </c>
       <c r="F74" s="34" t="inlineStr">
         <is>
@@ -26833,7 +26855,7 @@
         </is>
       </c>
       <c r="G74" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H74" s="34" t="inlineStr">
         <is>
@@ -26841,7 +26863,7 @@
         </is>
       </c>
       <c r="I74" t="n">
-        <v>92.970001</v>
+        <v>90.089996</v>
       </c>
     </row>
     <row r="75" ht="15" customHeight="1" s="58">
@@ -26865,7 +26887,7 @@
         </is>
       </c>
       <c r="E75" s="33" t="n">
-        <v>101.28</v>
+        <v>97.51000000000001</v>
       </c>
       <c r="F75" s="34" t="inlineStr">
         <is>
@@ -26873,7 +26895,7 @@
         </is>
       </c>
       <c r="G75" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H75" s="34" t="inlineStr">
         <is>
@@ -26881,7 +26903,7 @@
         </is>
       </c>
       <c r="I75" t="n">
-        <v>101.279999</v>
+        <v>97.510002</v>
       </c>
     </row>
     <row r="76" ht="15" customHeight="1" s="58">
@@ -26905,7 +26927,7 @@
         </is>
       </c>
       <c r="E76" s="33" t="n">
-        <v>432.41</v>
+        <v>422.65</v>
       </c>
       <c r="F76" s="34" t="inlineStr">
         <is>
@@ -26913,7 +26935,7 @@
         </is>
       </c>
       <c r="G76" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H76" s="34" t="inlineStr">
         <is>
@@ -26921,7 +26943,7 @@
         </is>
       </c>
       <c r="I76" t="n">
-        <v>432.410004</v>
+        <v>422.649994</v>
       </c>
     </row>
     <row r="77" ht="15" customHeight="1" s="58">
@@ -26945,7 +26967,7 @@
         </is>
       </c>
       <c r="E77" s="33" t="n">
-        <v>411.15</v>
+        <v>405.22</v>
       </c>
       <c r="F77" s="34" t="inlineStr">
         <is>
@@ -26953,7 +26975,7 @@
         </is>
       </c>
       <c r="G77" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H77" s="34" t="inlineStr">
         <is>
@@ -26961,7 +26983,7 @@
         </is>
       </c>
       <c r="I77" t="n">
-        <v>411.149994</v>
+        <v>405.220001</v>
       </c>
     </row>
     <row r="78" ht="15" customHeight="1" s="58">
@@ -26985,7 +27007,7 @@
         </is>
       </c>
       <c r="E78" s="33" t="n">
-        <v>51.66</v>
+        <v>52.82</v>
       </c>
       <c r="F78" s="34" t="inlineStr">
         <is>
@@ -26993,7 +27015,7 @@
         </is>
       </c>
       <c r="G78" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H78" s="34" t="inlineStr">
         <is>
@@ -27001,7 +27023,7 @@
         </is>
       </c>
       <c r="I78" t="n">
-        <v>51.66</v>
+        <v>52.82</v>
       </c>
     </row>
     <row r="79" ht="15" customHeight="1" s="58">
@@ -27025,7 +27047,7 @@
         </is>
       </c>
       <c r="E79" s="33" t="n">
-        <v>96.89</v>
+        <v>97.419</v>
       </c>
       <c r="F79" s="34" t="inlineStr">
         <is>
@@ -27033,7 +27055,7 @@
         </is>
       </c>
       <c r="G79" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H79" s="34" t="inlineStr">
         <is>
@@ -27041,7 +27063,7 @@
         </is>
       </c>
       <c r="I79" t="n">
-        <v>96.889999</v>
+        <v>97.41860200000001</v>
       </c>
     </row>
     <row r="80" ht="15" customHeight="1" s="58">
@@ -27065,7 +27087,7 @@
         </is>
       </c>
       <c r="E80" s="33" t="n">
-        <v>296.42</v>
+        <v>299.535</v>
       </c>
       <c r="F80" s="34" t="inlineStr">
         <is>
@@ -27073,7 +27095,7 @@
         </is>
       </c>
       <c r="G80" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H80" s="34" t="inlineStr">
         <is>
@@ -27081,7 +27103,7 @@
         </is>
       </c>
       <c r="I80" t="n">
-        <v>296.420013</v>
+        <v>299.535004</v>
       </c>
     </row>
     <row r="81" ht="15" customHeight="1" s="58">
@@ -27105,7 +27127,7 @@
         </is>
       </c>
       <c r="E81" s="33" t="n">
-        <v>169.62</v>
+        <v>171.1</v>
       </c>
       <c r="F81" s="34" t="inlineStr">
         <is>
@@ -27113,7 +27135,7 @@
         </is>
       </c>
       <c r="G81" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H81" s="34" t="inlineStr">
         <is>
@@ -27121,7 +27143,7 @@
         </is>
       </c>
       <c r="I81" t="n">
-        <v>169.619995</v>
+        <v>171.100006</v>
       </c>
     </row>
     <row r="82" ht="15" customHeight="1" s="58">
@@ -27157,7 +27179,7 @@
       </c>
       <c r="H82" s="34" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="I82" t="n">
@@ -27185,7 +27207,7 @@
         </is>
       </c>
       <c r="E83" s="33" t="n">
-        <v>110</v>
+        <v>96.79000000000001</v>
       </c>
       <c r="F83" s="34" t="inlineStr">
         <is>
@@ -27193,7 +27215,7 @@
         </is>
       </c>
       <c r="G83" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H83" s="34" t="inlineStr">
         <is>
@@ -27201,7 +27223,7 @@
         </is>
       </c>
       <c r="I83" t="n">
-        <v>130</v>
+        <v>96.790001</v>
       </c>
     </row>
     <row r="84" ht="15" customHeight="1" s="58">
@@ -27225,7 +27247,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>73.84</v>
+        <v>76.12</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -27233,7 +27255,7 @@
         </is>
       </c>
       <c r="G84" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H84" s="34" t="inlineStr">
         <is>
@@ -27241,7 +27263,7 @@
         </is>
       </c>
       <c r="I84" t="n">
-        <v>68.104428</v>
+        <v>75.770287</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="58">
@@ -27265,7 +27287,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>617.1</v>
+        <v>606.98</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -27273,7 +27295,7 @@
         </is>
       </c>
       <c r="G85" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H85" s="34" t="inlineStr">
         <is>
@@ -27281,7 +27303,7 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>613.567738</v>
+        <v>622.44403</v>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="58">
@@ -27305,7 +27327,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>66335</v>
+        <v>65784</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -27313,7 +27335,7 @@
         </is>
       </c>
       <c r="G86" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H86" s="34" t="inlineStr">
         <is>
@@ -27321,7 +27343,7 @@
         </is>
       </c>
       <c r="I86" t="n">
-        <v>65396.650356</v>
+        <v>66778.095833</v>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="58">
@@ -27345,7 +27367,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.00712</v>
+        <v>0.007143</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -27353,7 +27375,7 @@
         </is>
       </c>
       <c r="G87" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H87" s="34" t="inlineStr">
         <is>
@@ -27361,7 +27383,7 @@
         </is>
       </c>
       <c r="I87" t="n">
-        <v>0.006866</v>
+        <v>0.007378</v>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="58">
@@ -27385,7 +27407,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.011422</v>
+        <v>0.011146</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -27393,7 +27415,7 @@
         </is>
       </c>
       <c r="G88" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H88" s="34" t="inlineStr">
         <is>
@@ -27401,7 +27423,7 @@
         </is>
       </c>
       <c r="I88" t="n">
-        <v>0.010802</v>
+        <v>0.011425</v>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="58">
@@ -27425,7 +27447,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>74.18000000000001</v>
+        <v>73.73999999999999</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -27433,7 +27455,7 @@
         </is>
       </c>
       <c r="G89" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H89" s="34" t="inlineStr">
         <is>
@@ -27441,7 +27463,7 @@
         </is>
       </c>
       <c r="I89" t="n">
-        <v>70.774581</v>
+        <v>75.468017</v>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="58">
@@ -27465,7 +27487,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>1.99</v>
+        <v>1.9</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -27473,7 +27495,7 @@
         </is>
       </c>
       <c r="G90" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H90" s="34" t="inlineStr">
         <is>
@@ -27481,7 +27503,7 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>2.04956</v>
+        <v>2.008537</v>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="58">
@@ -27513,7 +27535,7 @@
         </is>
       </c>
       <c r="G91" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H91" s="34" t="inlineStr">
         <is>
@@ -27545,7 +27567,7 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
-        <v>0.016021</v>
+        <v>0.018617</v>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
@@ -27553,7 +27575,7 @@
         </is>
       </c>
       <c r="G92" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H92" s="34" t="inlineStr">
         <is>
@@ -27561,7 +27583,7 @@
         </is>
       </c>
       <c r="I92" t="n">
-        <v>0.014121</v>
+        <v>0.016358</v>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="58">
@@ -27585,7 +27607,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>2.811261</v>
+        <v>2.789622</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -27593,7 +27615,7 @@
         </is>
       </c>
       <c r="G93" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H93" s="34" t="inlineStr">
         <is>
@@ -27601,7 +27623,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>2.766373</v>
+        <v>2.882494</v>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="58">
@@ -27625,7 +27647,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>25.782809</v>
+        <v>25.745388</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -27633,7 +27655,7 @@
         </is>
       </c>
       <c r="G94" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H94" s="34" t="inlineStr">
         <is>
@@ -27641,7 +27663,7 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>25.707333</v>
+        <v>26.350781</v>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="58">
@@ -27665,7 +27687,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.114032</v>
+        <v>0.114195</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -27673,7 +27695,7 @@
         </is>
       </c>
       <c r="G95" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H95" s="34" t="inlineStr">
         <is>
@@ -27681,7 +27703,7 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>0.113817</v>
+        <v>0.116825</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="58">
@@ -27705,7 +27727,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>20080.434</v>
+        <v>19751.1292</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -27713,7 +27735,7 @@
         </is>
       </c>
       <c r="G96" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H96" s="34" t="inlineStr">
         <is>
@@ -27721,7 +27743,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>19965.494209</v>
+        <v>20254.328726</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="58">
@@ -27745,7 +27767,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2158540.9</v>
+        <v>2140611.36</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -27753,7 +27775,7 @@
         </is>
       </c>
       <c r="G97" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H97" s="34" t="inlineStr">
         <is>
@@ -27761,7 +27783,7 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>2128007.002575</v>
+        <v>2172959.238391</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="58">
@@ -27785,7 +27807,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>2.861307</v>
+        <v>2.844712</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -27793,7 +27815,7 @@
         </is>
       </c>
       <c r="G98" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H98" s="34" t="inlineStr">
         <is>
@@ -27801,7 +27823,7 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>2.880897</v>
+        <v>2.909689</v>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="58">
@@ -27825,7 +27847,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>58401.165</v>
+        <v>58353.0058</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -27833,7 +27855,7 @@
         </is>
       </c>
       <c r="G99" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H99" s="34" t="inlineStr">
         <is>
@@ -27841,7 +27863,7 @@
         </is>
       </c>
       <c r="I99" t="n">
-        <v>55694.466891</v>
+        <v>59517.718886</v>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="58">
@@ -27865,7 +27887,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>25.266789</v>
+        <v>25.089088</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -27873,7 +27895,7 @@
         </is>
       </c>
       <c r="G100" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H100" s="34" t="inlineStr">
         <is>
@@ -27881,7 +27903,7 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>25.053858</v>
+        <v>25.388902</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="58">
@@ -27905,7 +27927,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>66335</v>
+        <v>65784</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -27913,7 +27935,7 @@
         </is>
       </c>
       <c r="G101" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H101" s="34" t="inlineStr">
         <is>
@@ -27921,7 +27943,7 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>65396.650356</v>
+        <v>66778.095833</v>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="58">
@@ -27945,7 +27967,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>18.02</v>
+        <v>17.67</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -27953,7 +27975,7 @@
         </is>
       </c>
       <c r="G102" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H102" s="34" t="inlineStr">
         <is>
@@ -27961,7 +27983,7 @@
         </is>
       </c>
       <c r="I102" t="n">
-        <v>17.9002</v>
+        <v>18.267948</v>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="58">
@@ -28059,7 +28081,7 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
-        <v>0.00712</v>
+        <v>0.007143</v>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
@@ -28067,7 +28089,7 @@
         </is>
       </c>
       <c r="G105" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H105" s="34" t="inlineStr">
         <is>
@@ -28075,7 +28097,7 @@
         </is>
       </c>
       <c r="I105" t="n">
-        <v>0.006866</v>
+        <v>0.007378</v>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="58">
@@ -28099,7 +28121,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>74.18000000000001</v>
+        <v>73.73999999999999</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>
@@ -28107,7 +28129,7 @@
         </is>
       </c>
       <c r="G106" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H106" s="34" t="inlineStr">
         <is>
@@ -28115,7 +28137,7 @@
         </is>
       </c>
       <c r="I106" t="n">
-        <v>70.774581</v>
+        <v>75.468017</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="58">
@@ -28147,7 +28169,7 @@
         </is>
       </c>
       <c r="G107" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H107" s="34" t="inlineStr">
         <is>
@@ -28179,27 +28201,27 @@
         </is>
       </c>
       <c r="E108" t="n">
+        <v>23.7132</v>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G108" s="47" t="n">
+        <v>46184</v>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I108" t="n">
         <v>22.8715</v>
       </c>
-      <c r="F108" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G108" s="47" t="n">
-        <v>46183</v>
-      </c>
-      <c r="H108" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I108" t="n">
-        <v>23.5969</v>
-      </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily dashboard update — 2026-06-17
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-42660" yWindow="-540" windowWidth="32460" windowHeight="17180" tabRatio="500" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Realized" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Prices" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Reference" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Realized" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="AsOfDate">'FX &amp; Assumptions'!$C$5</definedName>
@@ -697,14 +697,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -726,8 +726,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -752,10 +752,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -764,10 +764,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4F81BD"/>
               </a:solidFill>
-              <a:ln w="0">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -777,10 +777,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="C0504D"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -790,10 +790,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="9BBB59"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -803,10 +803,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="8064A2"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -816,10 +816,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4BACC6"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -829,10 +829,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="F79646"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -842,14 +842,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -875,14 +875,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -908,14 +908,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -941,14 +941,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -974,14 +974,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1007,14 +1007,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1038,16 +1038,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1142,16 +1142,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1172,10 +1172,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1187,14 +1187,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1216,8 +1216,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1242,10 +1242,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1254,10 +1254,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4672A8"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1267,10 +1267,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="AB4744"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1280,10 +1280,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="8AA64F"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1293,10 +1293,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="725990"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1306,10 +1306,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4299B0"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1319,10 +1319,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="DC853E"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1332,10 +1332,10 @@
             <idx val="6"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="93A9CE"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1345,10 +1345,10 @@
             <idx val="7"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="D09493"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1358,10 +1358,10 @@
             <idx val="8"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="B8CD97"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1371,14 +1371,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1405,14 +1405,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1439,14 +1439,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1473,14 +1473,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1507,14 +1507,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1541,14 +1541,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1575,14 +1575,14 @@
             <dLbl>
               <idx val="6"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1609,14 +1609,14 @@
             <dLbl>
               <idx val="7"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1643,14 +1643,14 @@
             <dLbl>
               <idx val="8"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1675,16 +1675,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1791,16 +1791,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1821,10 +1821,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1836,14 +1836,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1865,8 +1865,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1893,10 +1893,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1904,16 +1904,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2016,7 +2016,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2025,9 +2025,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2059,7 +2059,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="9360">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2073,7 +2073,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2082,9 +2082,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2109,16 +2109,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2139,10 +2139,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2154,14 +2154,14 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -2183,8 +2183,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -2200,10 +2200,10 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2211,16 +2211,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2411,7 +2411,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2420,9 +2420,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2454,7 +2454,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="9360">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2468,7 +2468,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2477,9 +2477,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2504,16 +2504,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2534,10 +2534,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2549,7 +2549,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>1</col>
@@ -2569,9 +2569,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2596,9 +2596,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2623,9 +2623,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId3"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2650,9 +2650,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId4"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -22085,28 +22085,28 @@
         <v>46190</v>
       </c>
       <c r="C21" s="29" t="n">
-        <v>26404449</v>
+        <v>26398175</v>
       </c>
       <c r="D21" s="29" t="n">
-        <v>22738651</v>
+        <v>22737189</v>
       </c>
       <c r="E21" s="29" t="n">
-        <v>3665798</v>
+        <v>3660986</v>
       </c>
       <c r="F21" s="30" t="n">
-        <v>0.1612</v>
+        <v>0.161</v>
       </c>
       <c r="G21" s="29" t="n">
         <v>18859011</v>
       </c>
       <c r="H21" s="29" t="n">
-        <v>4978471</v>
+        <v>4958993</v>
       </c>
       <c r="I21" s="29" t="n">
-        <v>1188979</v>
+        <v>1183061</v>
       </c>
       <c r="J21" s="31" t="n">
-        <v>32.54</v>
+        <v>32.51</v>
       </c>
       <c r="K21" s="32" t="inlineStr">
         <is>
@@ -23757,7 +23757,7 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>32.54</v>
+        <v>32.51</v>
       </c>
       <c r="D6" s="64" t="inlineStr">
         <is>
@@ -23806,7 +23806,7 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>25.327</v>
+        <v>25.374</v>
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
@@ -25410,7 +25410,7 @@
         </is>
       </c>
       <c r="E38" s="33" t="n">
-        <v>23.52</v>
+        <v>23.28</v>
       </c>
       <c r="F38" s="34" t="inlineStr">
         <is>
@@ -25426,7 +25426,7 @@
         </is>
       </c>
       <c r="I38" t="n">
-        <v>23.52</v>
+        <v>23.280001</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="58">
@@ -25458,15 +25458,15 @@
         </is>
       </c>
       <c r="G39" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H39" s="34" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I39" t="n">
-        <v>1.066</v>
+        <v>1.078</v>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="58">
@@ -25490,7 +25490,7 @@
         </is>
       </c>
       <c r="E40" s="33" t="n">
-        <v>764.1</v>
+        <v>793.24</v>
       </c>
       <c r="F40" s="34" t="inlineStr">
         <is>
@@ -25506,7 +25506,7 @@
         </is>
       </c>
       <c r="I40" t="n">
-        <v>764.099976</v>
+        <v>793.23999</v>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="58">
@@ -25530,7 +25530,7 @@
         </is>
       </c>
       <c r="E41" s="33" t="n">
-        <v>21.75</v>
+        <v>21.78</v>
       </c>
       <c r="F41" s="34" t="inlineStr">
         <is>
@@ -25546,7 +25546,7 @@
         </is>
       </c>
       <c r="I41" t="n">
-        <v>20.940001</v>
+        <v>21.780001</v>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="58">
@@ -25570,7 +25570,7 @@
         </is>
       </c>
       <c r="E42" s="33" t="n">
-        <v>220.39</v>
+        <v>218.09</v>
       </c>
       <c r="F42" s="34" t="inlineStr">
         <is>
@@ -25586,7 +25586,7 @@
         </is>
       </c>
       <c r="I42" t="n">
-        <v>220.389999</v>
+        <v>218.089996</v>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="58">
@@ -26287,7 +26287,7 @@
         </is>
       </c>
       <c r="E60" s="33" t="n">
-        <v>180.475</v>
+        <v>176.845</v>
       </c>
       <c r="F60" s="34" t="inlineStr">
         <is>
@@ -26303,7 +26303,7 @@
         </is>
       </c>
       <c r="I60" t="n">
-        <v>180.475006</v>
+        <v>176.845001</v>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="58">
@@ -26327,7 +26327,7 @@
         </is>
       </c>
       <c r="E61" s="33" t="n">
-        <v>206.95</v>
+        <v>207.32</v>
       </c>
       <c r="F61" s="34" t="inlineStr">
         <is>
@@ -26343,7 +26343,7 @@
         </is>
       </c>
       <c r="I61" t="n">
-        <v>206.949997</v>
+        <v>207.320007</v>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="58">
@@ -26367,7 +26367,7 @@
         </is>
       </c>
       <c r="E62" s="33" t="n">
-        <v>577.88</v>
+        <v>568.23</v>
       </c>
       <c r="F62" s="34" t="inlineStr">
         <is>
@@ -26383,7 +26383,7 @@
         </is>
       </c>
       <c r="I62" t="n">
-        <v>577.880005</v>
+        <v>568.22998</v>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1" s="58">
@@ -26407,7 +26407,7 @@
         </is>
       </c>
       <c r="E63" s="33" t="n">
-        <v>163.458</v>
+        <v>160.76</v>
       </c>
       <c r="F63" s="34" t="inlineStr">
         <is>
@@ -26423,7 +26423,7 @@
         </is>
       </c>
       <c r="I63" t="n">
-        <v>163.457993</v>
+        <v>160.759995</v>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="58">
@@ -26447,7 +26447,7 @@
         </is>
       </c>
       <c r="E64" s="33" t="n">
-        <v>51.7</v>
+        <v>50.26</v>
       </c>
       <c r="F64" s="34" t="inlineStr">
         <is>
@@ -26463,7 +26463,7 @@
         </is>
       </c>
       <c r="I64" t="n">
-        <v>51.700001</v>
+        <v>50.259998</v>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1" s="58">
@@ -26487,7 +26487,7 @@
         </is>
       </c>
       <c r="E65" s="33" t="n">
-        <v>206.005</v>
+        <v>205.91</v>
       </c>
       <c r="F65" s="34" t="inlineStr">
         <is>
@@ -26503,7 +26503,7 @@
         </is>
       </c>
       <c r="I65" t="n">
-        <v>206.005005</v>
+        <v>205.910004</v>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1" s="58">
@@ -26527,7 +26527,7 @@
         </is>
       </c>
       <c r="E66" s="33" t="n">
-        <v>145.73</v>
+        <v>147.02</v>
       </c>
       <c r="F66" s="34" t="inlineStr">
         <is>
@@ -26543,7 +26543,7 @@
         </is>
       </c>
       <c r="I66" t="n">
-        <v>145.729996</v>
+        <v>147.020004</v>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1" s="58">
@@ -26567,7 +26567,7 @@
         </is>
       </c>
       <c r="E67" s="33" t="n">
-        <v>143.41</v>
+        <v>142.24</v>
       </c>
       <c r="F67" s="34" t="inlineStr">
         <is>
@@ -26583,7 +26583,7 @@
         </is>
       </c>
       <c r="I67" t="n">
-        <v>143.410004</v>
+        <v>142.240005</v>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1" s="58">
@@ -26607,7 +26607,7 @@
         </is>
       </c>
       <c r="E68" s="33" t="n">
-        <v>241.69</v>
+        <v>237.33</v>
       </c>
       <c r="F68" s="34" t="inlineStr">
         <is>
@@ -26623,7 +26623,7 @@
         </is>
       </c>
       <c r="I68" t="n">
-        <v>241.690002</v>
+        <v>237.330002</v>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="58">
@@ -26647,7 +26647,7 @@
         </is>
       </c>
       <c r="E69" s="33" t="n">
-        <v>1126.47</v>
+        <v>1122.5</v>
       </c>
       <c r="F69" s="34" t="inlineStr">
         <is>
@@ -26663,7 +26663,7 @@
         </is>
       </c>
       <c r="I69" t="n">
-        <v>1126.469971</v>
+        <v>1129.349976</v>
       </c>
     </row>
     <row r="70" ht="15" customHeight="1" s="58">
@@ -26687,7 +26687,7 @@
         </is>
       </c>
       <c r="E70" s="33" t="n">
-        <v>97.09999999999999</v>
+        <v>95.63</v>
       </c>
       <c r="F70" s="34" t="inlineStr">
         <is>
@@ -26703,7 +26703,7 @@
         </is>
       </c>
       <c r="I70" t="n">
-        <v>97.099998</v>
+        <v>95.629997</v>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1" s="58">
@@ -26727,7 +26727,7 @@
         </is>
       </c>
       <c r="E71" s="33" t="n">
-        <v>1543.38</v>
+        <v>1498.77</v>
       </c>
       <c r="F71" s="34" t="inlineStr">
         <is>
@@ -26743,7 +26743,7 @@
         </is>
       </c>
       <c r="I71" t="n">
-        <v>1543.380005</v>
+        <v>1498.77002</v>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1" s="58">
@@ -26767,7 +26767,7 @@
         </is>
       </c>
       <c r="E72" s="33" t="n">
-        <v>108.36</v>
+        <v>109.22</v>
       </c>
       <c r="F72" s="34" t="inlineStr">
         <is>
@@ -26783,7 +26783,7 @@
         </is>
       </c>
       <c r="I72" t="n">
-        <v>108.360001</v>
+        <v>109.220001</v>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1" s="58">
@@ -26807,7 +26807,7 @@
         </is>
       </c>
       <c r="E73" s="33" t="n">
-        <v>208.965</v>
+        <v>207.41</v>
       </c>
       <c r="F73" s="34" t="inlineStr">
         <is>
@@ -26823,7 +26823,7 @@
         </is>
       </c>
       <c r="I73" t="n">
-        <v>208.964996</v>
+        <v>207.410004</v>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1" s="58">
@@ -26847,7 +26847,7 @@
         </is>
       </c>
       <c r="E74" s="33" t="n">
-        <v>90.09</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="F74" s="34" t="inlineStr">
         <is>
@@ -26863,7 +26863,7 @@
         </is>
       </c>
       <c r="I74" t="n">
-        <v>90.089996</v>
+        <v>89.599998</v>
       </c>
     </row>
     <row r="75" ht="15" customHeight="1" s="58">
@@ -26887,7 +26887,7 @@
         </is>
       </c>
       <c r="E75" s="33" t="n">
-        <v>97.51000000000001</v>
+        <v>96.56</v>
       </c>
       <c r="F75" s="34" t="inlineStr">
         <is>
@@ -26903,7 +26903,7 @@
         </is>
       </c>
       <c r="I75" t="n">
-        <v>97.510002</v>
+        <v>96.55999799999999</v>
       </c>
     </row>
     <row r="76" ht="15" customHeight="1" s="58">
@@ -26927,7 +26927,7 @@
         </is>
       </c>
       <c r="E76" s="33" t="n">
-        <v>422.65</v>
+        <v>409.35</v>
       </c>
       <c r="F76" s="34" t="inlineStr">
         <is>
@@ -26943,7 +26943,7 @@
         </is>
       </c>
       <c r="I76" t="n">
-        <v>422.649994</v>
+        <v>409.350006</v>
       </c>
     </row>
     <row r="77" ht="15" customHeight="1" s="58">
@@ -26967,7 +26967,7 @@
         </is>
       </c>
       <c r="E77" s="33" t="n">
-        <v>405.22</v>
+        <v>404.66</v>
       </c>
       <c r="F77" s="34" t="inlineStr">
         <is>
@@ -26983,7 +26983,7 @@
         </is>
       </c>
       <c r="I77" t="n">
-        <v>405.220001</v>
+        <v>404.660004</v>
       </c>
     </row>
     <row r="78" ht="15" customHeight="1" s="58">
@@ -27007,7 +27007,7 @@
         </is>
       </c>
       <c r="E78" s="33" t="n">
-        <v>52.82</v>
+        <v>52.76</v>
       </c>
       <c r="F78" s="34" t="inlineStr">
         <is>
@@ -27023,7 +27023,7 @@
         </is>
       </c>
       <c r="I78" t="n">
-        <v>52.82</v>
+        <v>52.759998</v>
       </c>
     </row>
     <row r="79" ht="15" customHeight="1" s="58">
@@ -27047,7 +27047,7 @@
         </is>
       </c>
       <c r="E79" s="33" t="n">
-        <v>97.419</v>
+        <v>96.78</v>
       </c>
       <c r="F79" s="34" t="inlineStr">
         <is>
@@ -27063,7 +27063,7 @@
         </is>
       </c>
       <c r="I79" t="n">
-        <v>97.41860200000001</v>
+        <v>96.779999</v>
       </c>
     </row>
     <row r="80" ht="15" customHeight="1" s="58">
@@ -27087,7 +27087,7 @@
         </is>
       </c>
       <c r="E80" s="33" t="n">
-        <v>299.535</v>
+        <v>299.24</v>
       </c>
       <c r="F80" s="34" t="inlineStr">
         <is>
@@ -27103,7 +27103,7 @@
         </is>
       </c>
       <c r="I80" t="n">
-        <v>299.535004</v>
+        <v>299.23999</v>
       </c>
     </row>
     <row r="81" ht="15" customHeight="1" s="58">
@@ -27127,7 +27127,7 @@
         </is>
       </c>
       <c r="E81" s="33" t="n">
-        <v>171.1</v>
+        <v>169.27</v>
       </c>
       <c r="F81" s="34" t="inlineStr">
         <is>
@@ -27143,7 +27143,7 @@
         </is>
       </c>
       <c r="I81" t="n">
-        <v>171.100006</v>
+        <v>169.270004</v>
       </c>
     </row>
     <row r="82" ht="15" customHeight="1" s="58">
@@ -27167,7 +27167,7 @@
         </is>
       </c>
       <c r="E82" s="33" t="n">
-        <v>593.48</v>
+        <v>600.21</v>
       </c>
       <c r="F82" s="34" t="inlineStr">
         <is>
@@ -27175,15 +27175,15 @@
         </is>
       </c>
       <c r="G82" s="28" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="H82" s="34" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I82" t="n">
-        <v>593.47998</v>
+        <v>600.210022</v>
       </c>
     </row>
     <row r="83" ht="15" customHeight="1" s="58">
@@ -27207,7 +27207,7 @@
         </is>
       </c>
       <c r="E83" s="33" t="n">
-        <v>96.79000000000001</v>
+        <v>91.98999999999999</v>
       </c>
       <c r="F83" s="34" t="inlineStr">
         <is>
@@ -27223,7 +27223,7 @@
         </is>
       </c>
       <c r="I83" t="n">
-        <v>96.790001</v>
+        <v>91.989998</v>
       </c>
     </row>
     <row r="84" ht="15" customHeight="1" s="58">
@@ -27247,7 +27247,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>76.12</v>
+        <v>76.13</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -27263,7 +27263,7 @@
         </is>
       </c>
       <c r="I84" t="n">
-        <v>75.770287</v>
+        <v>73.921914</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="58">
@@ -27287,7 +27287,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>606.98</v>
+        <v>603.33</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -27303,7 +27303,7 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>622.44403</v>
+        <v>617.3147740000001</v>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="58">
@@ -27327,7 +27327,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>65784</v>
+        <v>65522</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -27343,7 +27343,7 @@
         </is>
       </c>
       <c r="I86" t="n">
-        <v>66778.095833</v>
+        <v>66354.39950100001</v>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="58">
@@ -27367,7 +27367,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.007143</v>
+        <v>0.007159</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -27383,7 +27383,7 @@
         </is>
       </c>
       <c r="I87" t="n">
-        <v>0.007378</v>
+        <v>0.007116</v>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="58">
@@ -27407,7 +27407,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.011146</v>
+        <v>0.011297</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -27423,7 +27423,7 @@
         </is>
       </c>
       <c r="I88" t="n">
-        <v>0.011425</v>
+        <v>0.011434</v>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="58">
@@ -27447,7 +27447,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>73.73999999999999</v>
+        <v>73.31999999999999</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -27463,7 +27463,7 @@
         </is>
       </c>
       <c r="I89" t="n">
-        <v>75.468017</v>
+        <v>74.175377</v>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="58">
@@ -27503,7 +27503,7 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>2.008537</v>
+        <v>1.986521</v>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="58">
@@ -27567,7 +27567,7 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
-        <v>0.018617</v>
+        <v>0.018253</v>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
@@ -27583,7 +27583,7 @@
         </is>
       </c>
       <c r="I92" t="n">
-        <v>0.016358</v>
+        <v>0.016036</v>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="58">
@@ -27607,7 +27607,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>2.789622</v>
+        <v>2.797258</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -27623,7 +27623,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>2.882494</v>
+        <v>2.809108</v>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="58">
@@ -27647,7 +27647,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>25.745388</v>
+        <v>26.05618</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -27663,7 +27663,7 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>26.350781</v>
+        <v>25.756446</v>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="58">
@@ -27687,7 +27687,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.114195</v>
+        <v>0.11331</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -27703,7 +27703,7 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>0.116825</v>
+        <v>0.113973</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="58">
@@ -27727,7 +27727,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>19751.1292</v>
+        <v>19614.2583</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -27743,7 +27743,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>20254.328726</v>
+        <v>20068.903314</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="58">
@@ -27767,7 +27767,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2140611.36</v>
+        <v>2130120.22</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -27783,7 +27783,7 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>2172959.238391</v>
+        <v>2157181.527783</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="58">
@@ -27807,7 +27807,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>2.844712</v>
+        <v>2.830873</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -27823,7 +27823,7 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>2.909689</v>
+        <v>2.858493</v>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="58">
@@ -27847,7 +27847,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>58353.0058</v>
+        <v>58009.5436</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -27863,7 +27863,7 @@
         </is>
       </c>
       <c r="I99" t="n">
-        <v>59517.718886</v>
+        <v>58346.787202</v>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="58">
@@ -27887,7 +27887,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>25.089088</v>
+        <v>25.038877</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -27903,7 +27903,7 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>25.388902</v>
+        <v>25.244738</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="58">
@@ -27927,7 +27927,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>65784</v>
+        <v>65522</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -27943,7 +27943,7 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>66778.095833</v>
+        <v>66354.39950100001</v>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="58">
@@ -27967,7 +27967,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>17.67</v>
+        <v>17.79</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -27983,7 +27983,7 @@
         </is>
       </c>
       <c r="I102" t="n">
-        <v>18.267948</v>
+        <v>18.020095</v>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="58">
@@ -28081,7 +28081,7 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
-        <v>0.007143</v>
+        <v>0.007159</v>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
@@ -28097,7 +28097,7 @@
         </is>
       </c>
       <c r="I105" t="n">
-        <v>0.007378</v>
+        <v>0.007116</v>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="58">
@@ -28121,7 +28121,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>73.73999999999999</v>
+        <v>73.31999999999999</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>
@@ -28137,7 +28137,7 @@
         </is>
       </c>
       <c r="I106" t="n">
-        <v>75.468017</v>
+        <v>74.175377</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="58">

</xml_diff>

<commit_message>
Daily dashboard update — 2026-06-18
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -22115,16 +22115,38 @@
       </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="58">
-      <c r="B22" s="28" t="n"/>
-      <c r="C22" s="29" t="n"/>
-      <c r="D22" s="29" t="n"/>
-      <c r="E22" s="29" t="n"/>
-      <c r="F22" s="30" t="n"/>
-      <c r="G22" s="29" t="n"/>
-      <c r="H22" s="29" t="n"/>
-      <c r="I22" s="29" t="n"/>
-      <c r="J22" s="31" t="n"/>
-      <c r="K22" s="32" t="n"/>
+      <c r="B22" s="28" t="n">
+        <v>46191</v>
+      </c>
+      <c r="C22" s="29" t="n">
+        <v>26830180</v>
+      </c>
+      <c r="D22" s="29" t="n">
+        <v>22751797</v>
+      </c>
+      <c r="E22" s="29" t="n">
+        <v>4078383</v>
+      </c>
+      <c r="F22" s="30" t="n">
+        <v>0.1793</v>
+      </c>
+      <c r="G22" s="29" t="n">
+        <v>19307529</v>
+      </c>
+      <c r="H22" s="29" t="n">
+        <v>4952110</v>
+      </c>
+      <c r="I22" s="29" t="n">
+        <v>1176365</v>
+      </c>
+      <c r="J22" s="31" t="n">
+        <v>32.65</v>
+      </c>
+      <c r="K22" s="32" t="inlineStr">
+        <is>
+          <t>Auto weekly snapshot</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="58">
       <c r="B23" s="28" t="n"/>
@@ -23742,7 +23764,7 @@
         </is>
       </c>
       <c r="C5" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="D5" s="64" t="inlineStr">
         <is>
@@ -23757,11 +23779,11 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>32.51</v>
+        <v>32.65</v>
       </c>
       <c r="D6" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-06-17</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-06-18</t>
         </is>
       </c>
     </row>
@@ -23806,11 +23828,11 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>25.374</v>
+        <v>25.3898</v>
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-06-17</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-06-18</t>
         </is>
       </c>
     </row>
@@ -23925,27 +23947,27 @@
         </is>
       </c>
       <c r="E5" s="33" t="n">
+        <v>27.7204</v>
+      </c>
+      <c r="F5" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G5" s="28" t="n">
+        <v>46188</v>
+      </c>
+      <c r="H5" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
         <v>25.8262</v>
       </c>
-      <c r="F5" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G5" s="28" t="n">
-        <v>46185</v>
-      </c>
-      <c r="H5" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I5" t="n">
-        <v>25.5328</v>
-      </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
     </row>
@@ -23970,27 +23992,27 @@
         </is>
       </c>
       <c r="E6" s="33" t="n">
+        <v>10.688</v>
+      </c>
+      <c r="F6" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G6" s="28" t="n">
+        <v>46189</v>
+      </c>
+      <c r="H6" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
         <v>10.6878</v>
       </c>
-      <c r="F6" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G6" s="28" t="n">
-        <v>46188</v>
-      </c>
-      <c r="H6" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I6" t="n">
-        <v>10.6873</v>
-      </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -24015,27 +24037,27 @@
         </is>
       </c>
       <c r="E7" s="33" t="n">
+        <v>7.2207</v>
+      </c>
+      <c r="F7" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G7" s="28" t="n">
+        <v>46188</v>
+      </c>
+      <c r="H7" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
         <v>7.1641</v>
       </c>
-      <c r="F7" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G7" s="28" t="n">
-        <v>46185</v>
-      </c>
-      <c r="H7" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I7" t="n">
-        <v>7.0558</v>
-      </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
     </row>
@@ -24060,27 +24082,27 @@
         </is>
       </c>
       <c r="E8" s="33" t="n">
+        <v>9.8744</v>
+      </c>
+      <c r="F8" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G8" s="28" t="n">
+        <v>46188</v>
+      </c>
+      <c r="H8" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
         <v>9.5237</v>
       </c>
-      <c r="F8" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G8" s="28" t="n">
-        <v>46185</v>
-      </c>
-      <c r="H8" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I8" t="n">
-        <v>9.4458</v>
-      </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
     </row>
@@ -24105,27 +24127,27 @@
         </is>
       </c>
       <c r="E9" s="33" t="n">
+        <v>9.332100000000001</v>
+      </c>
+      <c r="F9" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G9" s="28" t="n">
+        <v>46189</v>
+      </c>
+      <c r="H9" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
         <v>9.372999999999999</v>
       </c>
-      <c r="F9" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G9" s="28" t="n">
-        <v>46188</v>
-      </c>
-      <c r="H9" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I9" t="n">
-        <v>9.285500000000001</v>
-      </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -24150,27 +24172,27 @@
         </is>
       </c>
       <c r="E10" s="33" t="n">
+        <v>13.7411</v>
+      </c>
+      <c r="F10" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G10" s="28" t="n">
+        <v>46188</v>
+      </c>
+      <c r="H10" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
         <v>13.2399</v>
       </c>
-      <c r="F10" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G10" s="28" t="n">
-        <v>46185</v>
-      </c>
-      <c r="H10" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I10" t="n">
-        <v>12.9605</v>
-      </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
     </row>
@@ -24195,27 +24217,27 @@
         </is>
       </c>
       <c r="E11" s="33" t="n">
+        <v>13.3095</v>
+      </c>
+      <c r="F11" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G11" s="28" t="n">
+        <v>46189</v>
+      </c>
+      <c r="H11" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
         <v>13.2787</v>
       </c>
-      <c r="F11" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G11" s="28" t="n">
-        <v>46188</v>
-      </c>
-      <c r="H11" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I11" t="n">
-        <v>13.2722</v>
-      </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -24240,27 +24262,27 @@
         </is>
       </c>
       <c r="E12" s="33" t="n">
+        <v>26.703</v>
+      </c>
+      <c r="F12" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G12" s="28" t="n">
+        <v>46189</v>
+      </c>
+      <c r="H12" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
         <v>26.987</v>
       </c>
-      <c r="F12" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G12" s="28" t="n">
-        <v>46188</v>
-      </c>
-      <c r="H12" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I12" t="n">
-        <v>26.8895</v>
-      </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -24285,27 +24307,27 @@
         </is>
       </c>
       <c r="E13" s="33" t="n">
+        <v>36.4324</v>
+      </c>
+      <c r="F13" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G13" s="28" t="n">
+        <v>46189</v>
+      </c>
+      <c r="H13" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
         <v>36.4884</v>
       </c>
-      <c r="F13" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G13" s="28" t="n">
-        <v>46188</v>
-      </c>
-      <c r="H13" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I13" t="n">
-        <v>36.5289</v>
-      </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -24330,27 +24352,27 @@
         </is>
       </c>
       <c r="E14" s="33" t="n">
+        <v>25.5798</v>
+      </c>
+      <c r="F14" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G14" s="28" t="n">
+        <v>46189</v>
+      </c>
+      <c r="H14" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
         <v>25.5415</v>
       </c>
-      <c r="F14" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G14" s="28" t="n">
-        <v>46188</v>
-      </c>
-      <c r="H14" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I14" t="n">
-        <v>25.535</v>
-      </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -24375,27 +24397,27 @@
         </is>
       </c>
       <c r="E15" s="33" t="n">
+        <v>15.0377</v>
+      </c>
+      <c r="F15" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G15" s="28" t="n">
+        <v>46185</v>
+      </c>
+      <c r="H15" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
         <v>15.0939</v>
       </c>
-      <c r="F15" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G15" s="28" t="n">
-        <v>46184</v>
-      </c>
-      <c r="H15" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I15" t="n">
-        <v>14.919</v>
-      </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>
@@ -24420,27 +24442,27 @@
         </is>
       </c>
       <c r="E16" s="33" t="n">
+        <v>81.7367</v>
+      </c>
+      <c r="F16" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G16" s="28" t="n">
+        <v>46189</v>
+      </c>
+      <c r="H16" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
         <v>81.8086</v>
       </c>
-      <c r="F16" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G16" s="28" t="n">
-        <v>46188</v>
-      </c>
-      <c r="H16" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I16" t="n">
-        <v>81.94029999999999</v>
-      </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -24465,27 +24487,27 @@
         </is>
       </c>
       <c r="E17" s="33" t="n">
+        <v>53.5816</v>
+      </c>
+      <c r="F17" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G17" s="28" t="n">
+        <v>46189</v>
+      </c>
+      <c r="H17" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
         <v>53.5038</v>
       </c>
-      <c r="F17" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G17" s="28" t="n">
-        <v>46188</v>
-      </c>
-      <c r="H17" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I17" t="n">
-        <v>53.4365</v>
-      </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -24510,27 +24532,27 @@
         </is>
       </c>
       <c r="E18" s="33" t="n">
+        <v>16.4959</v>
+      </c>
+      <c r="F18" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G18" s="28" t="n">
+        <v>46189</v>
+      </c>
+      <c r="H18" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
         <v>16.5024</v>
       </c>
-      <c r="F18" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G18" s="28" t="n">
-        <v>46188</v>
-      </c>
-      <c r="H18" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I18" t="n">
-        <v>16.4623</v>
-      </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -24555,27 +24577,27 @@
         </is>
       </c>
       <c r="E19" s="33" t="n">
+        <v>23.4068</v>
+      </c>
+      <c r="F19" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G19" s="28" t="n">
+        <v>46189</v>
+      </c>
+      <c r="H19" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
         <v>23.4061</v>
       </c>
-      <c r="F19" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G19" s="28" t="n">
-        <v>46188</v>
-      </c>
-      <c r="H19" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I19" t="n">
-        <v>23.4045</v>
-      </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -24600,27 +24622,27 @@
         </is>
       </c>
       <c r="E20" s="33" t="n">
+        <v>41.4428</v>
+      </c>
+      <c r="F20" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G20" s="28" t="n">
+        <v>46188</v>
+      </c>
+      <c r="H20" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
         <v>40.7663</v>
       </c>
-      <c r="F20" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G20" s="28" t="n">
-        <v>46185</v>
-      </c>
-      <c r="H20" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I20" t="n">
-        <v>40.574</v>
-      </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
     </row>
@@ -24645,27 +24667,27 @@
         </is>
       </c>
       <c r="E21" s="33" t="n">
+        <v>13.5882</v>
+      </c>
+      <c r="F21" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G21" s="28" t="n">
+        <v>46189</v>
+      </c>
+      <c r="H21" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
         <v>13.6767</v>
       </c>
-      <c r="F21" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G21" s="28" t="n">
-        <v>46188</v>
-      </c>
-      <c r="H21" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I21" t="n">
-        <v>13.5289</v>
-      </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -24690,27 +24712,27 @@
         </is>
       </c>
       <c r="E22" s="33" t="n">
+        <v>13.2398</v>
+      </c>
+      <c r="F22" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G22" s="28" t="n">
+        <v>46188</v>
+      </c>
+      <c r="H22" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
         <v>13.3532</v>
       </c>
-      <c r="F22" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G22" s="28" t="n">
-        <v>46185</v>
-      </c>
-      <c r="H22" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I22" t="n">
-        <v>13.2862</v>
-      </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
     </row>
@@ -24735,27 +24757,27 @@
         </is>
       </c>
       <c r="E23" s="33" t="n">
+        <v>12.477</v>
+      </c>
+      <c r="F23" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G23" s="28" t="n">
+        <v>46189</v>
+      </c>
+      <c r="H23" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
         <v>12.4628</v>
       </c>
-      <c r="F23" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G23" s="28" t="n">
-        <v>46188</v>
-      </c>
-      <c r="H23" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I23" t="n">
-        <v>12.4646</v>
-      </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -24780,27 +24802,27 @@
         </is>
       </c>
       <c r="E24" s="33" t="n">
+        <v>12.0412</v>
+      </c>
+      <c r="F24" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G24" s="28" t="n">
+        <v>46188</v>
+      </c>
+      <c r="H24" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
         <v>11.7378</v>
       </c>
-      <c r="F24" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G24" s="28" t="n">
-        <v>46185</v>
-      </c>
-      <c r="H24" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I24" t="n">
-        <v>11.56</v>
-      </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
     </row>
@@ -24825,27 +24847,27 @@
         </is>
       </c>
       <c r="E25" s="33" t="n">
+        <v>9.928100000000001</v>
+      </c>
+      <c r="F25" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G25" s="28" t="n">
+        <v>46189</v>
+      </c>
+      <c r="H25" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
         <v>9.921799999999999</v>
       </c>
-      <c r="F25" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G25" s="28" t="n">
-        <v>46188</v>
-      </c>
-      <c r="H25" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I25" t="n">
-        <v>9.825200000000001</v>
-      </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -24870,27 +24892,27 @@
         </is>
       </c>
       <c r="E26" s="33" t="n">
+        <v>13.9345</v>
+      </c>
+      <c r="F26" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G26" s="28" t="n">
+        <v>46189</v>
+      </c>
+      <c r="H26" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
         <v>13.9253</v>
       </c>
-      <c r="F26" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G26" s="28" t="n">
-        <v>46188</v>
-      </c>
-      <c r="H26" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I26" t="n">
-        <v>13.7868</v>
-      </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -24915,27 +24937,27 @@
         </is>
       </c>
       <c r="E27" s="33" t="n">
+        <v>17.2282</v>
+      </c>
+      <c r="F27" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G27" s="28" t="n">
+        <v>46189</v>
+      </c>
+      <c r="H27" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
         <v>17.1935</v>
       </c>
-      <c r="F27" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G27" s="28" t="n">
-        <v>46188</v>
-      </c>
-      <c r="H27" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I27" t="n">
-        <v>17.0399</v>
-      </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -24960,27 +24982,27 @@
         </is>
       </c>
       <c r="E28" s="33" t="n">
+        <v>19.3198</v>
+      </c>
+      <c r="F28" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G28" s="28" t="n">
+        <v>46189</v>
+      </c>
+      <c r="H28" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
         <v>19.2686</v>
       </c>
-      <c r="F28" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G28" s="28" t="n">
-        <v>46188</v>
-      </c>
-      <c r="H28" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I28" t="n">
-        <v>18.7544</v>
-      </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -25005,27 +25027,27 @@
         </is>
       </c>
       <c r="E29" s="33" t="n">
+        <v>28.7079</v>
+      </c>
+      <c r="F29" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G29" s="28" t="n">
+        <v>46188</v>
+      </c>
+      <c r="H29" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
         <v>26.8484</v>
       </c>
-      <c r="F29" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G29" s="28" t="n">
-        <v>46185</v>
-      </c>
-      <c r="H29" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I29" t="n">
-        <v>27.104</v>
-      </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
     </row>
@@ -25050,27 +25072,27 @@
         </is>
       </c>
       <c r="E30" s="33" t="n">
+        <v>40.5797</v>
+      </c>
+      <c r="F30" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G30" s="28" t="n">
+        <v>46188</v>
+      </c>
+      <c r="H30" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
         <v>39.1699</v>
       </c>
-      <c r="F30" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G30" s="28" t="n">
-        <v>46185</v>
-      </c>
-      <c r="H30" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I30" t="n">
-        <v>36.9119</v>
-      </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
     </row>
@@ -25095,27 +25117,27 @@
         </is>
       </c>
       <c r="E31" s="33" t="n">
+        <v>12.9887</v>
+      </c>
+      <c r="F31" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G31" s="28" t="n">
+        <v>46189</v>
+      </c>
+      <c r="H31" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
         <v>13.0122</v>
       </c>
-      <c r="F31" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G31" s="28" t="n">
-        <v>46188</v>
-      </c>
-      <c r="H31" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I31" t="n">
-        <v>13.0229</v>
-      </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -25140,27 +25162,27 @@
         </is>
       </c>
       <c r="E32" s="33" t="n">
+        <v>21.7067</v>
+      </c>
+      <c r="F32" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G32" s="28" t="n">
+        <v>46189</v>
+      </c>
+      <c r="H32" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
         <v>21.7065</v>
       </c>
-      <c r="F32" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G32" s="28" t="n">
-        <v>46188</v>
-      </c>
-      <c r="H32" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I32" t="n">
-        <v>21.706</v>
-      </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -25185,27 +25207,27 @@
         </is>
       </c>
       <c r="E33" s="33" t="n">
+        <v>12.5343</v>
+      </c>
+      <c r="F33" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G33" s="28" t="n">
+        <v>46189</v>
+      </c>
+      <c r="H33" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
         <v>12.5219</v>
       </c>
-      <c r="F33" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G33" s="28" t="n">
-        <v>46188</v>
-      </c>
-      <c r="H33" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I33" t="n">
-        <v>12.5506</v>
-      </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -25230,27 +25252,27 @@
         </is>
       </c>
       <c r="E34" s="33" t="n">
+        <v>16.207</v>
+      </c>
+      <c r="F34" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G34" s="28" t="n">
+        <v>46189</v>
+      </c>
+      <c r="H34" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
         <v>16.2066</v>
       </c>
-      <c r="F34" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G34" s="28" t="n">
-        <v>46188</v>
-      </c>
-      <c r="H34" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I34" t="n">
-        <v>16.2056</v>
-      </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -25275,27 +25297,27 @@
         </is>
       </c>
       <c r="E35" s="33" t="n">
+        <v>27.8097</v>
+      </c>
+      <c r="F35" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G35" s="28" t="n">
+        <v>46188</v>
+      </c>
+      <c r="H35" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
         <v>27.2155</v>
       </c>
-      <c r="F35" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G35" s="28" t="n">
-        <v>46185</v>
-      </c>
-      <c r="H35" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I35" t="n">
-        <v>27.4092</v>
-      </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
     </row>
@@ -25320,27 +25342,27 @@
         </is>
       </c>
       <c r="E36" s="33" t="n">
+        <v>10.1449</v>
+      </c>
+      <c r="F36" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G36" s="28" t="n">
+        <v>46189</v>
+      </c>
+      <c r="H36" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
         <v>10.1561</v>
       </c>
-      <c r="F36" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G36" s="28" t="n">
-        <v>46188</v>
-      </c>
-      <c r="H36" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I36" t="n">
-        <v>10.079</v>
-      </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -25365,27 +25387,27 @@
         </is>
       </c>
       <c r="E37" s="33" t="n">
+        <v>22.698</v>
+      </c>
+      <c r="F37" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G37" s="28" t="n">
+        <v>46189</v>
+      </c>
+      <c r="H37" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
         <v>22.7039</v>
       </c>
-      <c r="F37" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G37" s="28" t="n">
-        <v>46188</v>
-      </c>
-      <c r="H37" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I37" t="n">
-        <v>22.7488</v>
-      </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -25410,7 +25432,7 @@
         </is>
       </c>
       <c r="E38" s="33" t="n">
-        <v>23.28</v>
+        <v>23.24</v>
       </c>
       <c r="F38" s="34" t="inlineStr">
         <is>
@@ -25418,7 +25440,7 @@
         </is>
       </c>
       <c r="G38" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H38" s="34" t="inlineStr">
         <is>
@@ -25426,7 +25448,7 @@
         </is>
       </c>
       <c r="I38" t="n">
-        <v>23.280001</v>
+        <v>23.24</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="58">
@@ -25450,7 +25472,7 @@
         </is>
       </c>
       <c r="E39" s="33" t="n">
-        <v>1.066</v>
+        <v>1.078</v>
       </c>
       <c r="F39" s="34" t="inlineStr">
         <is>
@@ -25458,7 +25480,7 @@
         </is>
       </c>
       <c r="G39" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H39" s="34" t="inlineStr">
         <is>
@@ -25466,7 +25488,7 @@
         </is>
       </c>
       <c r="I39" t="n">
-        <v>1.078</v>
+        <v>1.083</v>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="58">
@@ -25490,7 +25512,7 @@
         </is>
       </c>
       <c r="E40" s="33" t="n">
-        <v>793.24</v>
+        <v>784.6900000000001</v>
       </c>
       <c r="F40" s="34" t="inlineStr">
         <is>
@@ -25498,7 +25520,7 @@
         </is>
       </c>
       <c r="G40" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H40" s="34" t="inlineStr">
         <is>
@@ -25506,7 +25528,7 @@
         </is>
       </c>
       <c r="I40" t="n">
-        <v>793.23999</v>
+        <v>784.690002</v>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="58">
@@ -25530,7 +25552,7 @@
         </is>
       </c>
       <c r="E41" s="33" t="n">
-        <v>21.78</v>
+        <v>21.87</v>
       </c>
       <c r="F41" s="34" t="inlineStr">
         <is>
@@ -25538,7 +25560,7 @@
         </is>
       </c>
       <c r="G41" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H41" s="34" t="inlineStr">
         <is>
@@ -25546,7 +25568,7 @@
         </is>
       </c>
       <c r="I41" t="n">
-        <v>21.780001</v>
+        <v>21.870001</v>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="58">
@@ -25570,7 +25592,7 @@
         </is>
       </c>
       <c r="E42" s="33" t="n">
-        <v>218.09</v>
+        <v>216</v>
       </c>
       <c r="F42" s="34" t="inlineStr">
         <is>
@@ -25578,7 +25600,7 @@
         </is>
       </c>
       <c r="G42" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H42" s="34" t="inlineStr">
         <is>
@@ -25610,7 +25632,7 @@
         </is>
       </c>
       <c r="E43" s="33" t="n">
-        <v>5.35</v>
+        <v>5.4</v>
       </c>
       <c r="F43" s="34" t="inlineStr">
         <is>
@@ -25618,7 +25640,7 @@
         </is>
       </c>
       <c r="G43" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H43" s="34" t="inlineStr">
         <is>
@@ -25626,7 +25648,7 @@
         </is>
       </c>
       <c r="I43" t="n">
-        <v>5.35</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="58">
@@ -25650,23 +25672,23 @@
         </is>
       </c>
       <c r="E44" s="33" t="n">
+        <v>174</v>
+      </c>
+      <c r="F44" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G44" s="28" t="n">
+        <v>46191</v>
+      </c>
+      <c r="H44" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
         <v>175.5</v>
-      </c>
-      <c r="F44" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G44" s="28" t="n">
-        <v>46190</v>
-      </c>
-      <c r="H44" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I44" t="n">
-        <v>172.5</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="58">
@@ -25690,7 +25712,7 @@
         </is>
       </c>
       <c r="E45" s="33" t="n">
-        <v>0.44</v>
+        <v>0.45</v>
       </c>
       <c r="F45" s="34" t="inlineStr">
         <is>
@@ -25698,7 +25720,7 @@
         </is>
       </c>
       <c r="G45" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H45" s="34" t="inlineStr">
         <is>
@@ -25706,7 +25728,7 @@
         </is>
       </c>
       <c r="I45" t="n">
-        <v>0.44</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="58">
@@ -25730,7 +25752,7 @@
         </is>
       </c>
       <c r="E46" s="33" t="n">
-        <v>0.29</v>
+        <v>0.3</v>
       </c>
       <c r="F46" s="34" t="inlineStr">
         <is>
@@ -25738,7 +25760,7 @@
         </is>
       </c>
       <c r="G46" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H46" s="34" t="inlineStr">
         <is>
@@ -25746,7 +25768,7 @@
         </is>
       </c>
       <c r="I46" t="n">
-        <v>0.29</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" s="58">
@@ -25815,7 +25837,7 @@
         </is>
       </c>
       <c r="G48" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H48" s="34" t="inlineStr">
         <is>
@@ -25855,7 +25877,7 @@
         </is>
       </c>
       <c r="G49" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H49" s="34" t="inlineStr">
         <is>
@@ -25887,7 +25909,7 @@
         </is>
       </c>
       <c r="E50" s="33" t="n">
-        <v>9.5</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="F50" s="34" t="inlineStr">
         <is>
@@ -25895,7 +25917,7 @@
         </is>
       </c>
       <c r="G50" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H50" s="34" t="inlineStr">
         <is>
@@ -25903,7 +25925,7 @@
         </is>
       </c>
       <c r="I50" t="n">
-        <v>9.4</v>
+        <v>9.800000000000001</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="58">
@@ -25927,7 +25949,7 @@
         </is>
       </c>
       <c r="E51" s="33" t="n">
-        <v>15.6</v>
+        <v>15.9</v>
       </c>
       <c r="F51" s="34" t="inlineStr">
         <is>
@@ -25935,7 +25957,7 @@
         </is>
       </c>
       <c r="G51" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H51" s="34" t="inlineStr">
         <is>
@@ -25943,7 +25965,7 @@
         </is>
       </c>
       <c r="I51" t="n">
-        <v>15.6</v>
+        <v>15.9</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" s="58">
@@ -25967,7 +25989,7 @@
         </is>
       </c>
       <c r="E52" s="33" t="n">
-        <v>13.4</v>
+        <v>13.6</v>
       </c>
       <c r="F52" s="34" t="inlineStr">
         <is>
@@ -25975,7 +25997,7 @@
         </is>
       </c>
       <c r="G52" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H52" s="34" t="inlineStr">
         <is>
@@ -25983,7 +26005,7 @@
         </is>
       </c>
       <c r="I52" t="n">
-        <v>13.4</v>
+        <v>13.6</v>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1" s="58">
@@ -26007,7 +26029,7 @@
         </is>
       </c>
       <c r="E53" s="33" t="n">
-        <v>5.45</v>
+        <v>5.6</v>
       </c>
       <c r="F53" s="34" t="inlineStr">
         <is>
@@ -26015,7 +26037,7 @@
         </is>
       </c>
       <c r="G53" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H53" s="34" t="inlineStr">
         <is>
@@ -26023,7 +26045,7 @@
         </is>
       </c>
       <c r="I53" t="n">
-        <v>5.45</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="58">
@@ -26047,7 +26069,7 @@
         </is>
       </c>
       <c r="E54" s="33" t="n">
-        <v>21.8</v>
+        <v>22.7</v>
       </c>
       <c r="F54" s="34" t="inlineStr">
         <is>
@@ -26055,7 +26077,7 @@
         </is>
       </c>
       <c r="G54" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H54" s="34" t="inlineStr">
         <is>
@@ -26063,7 +26085,7 @@
         </is>
       </c>
       <c r="I54" t="n">
-        <v>21.799999</v>
+        <v>22.700001</v>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="58">
@@ -26087,7 +26109,7 @@
         </is>
       </c>
       <c r="E55" s="33" t="n">
-        <v>3.54</v>
+        <v>3.5</v>
       </c>
       <c r="F55" s="34" t="inlineStr">
         <is>
@@ -26095,7 +26117,7 @@
         </is>
       </c>
       <c r="G55" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H55" s="34" t="inlineStr">
         <is>
@@ -26127,7 +26149,7 @@
         </is>
       </c>
       <c r="E56" s="33" t="n">
-        <v>4.86</v>
+        <v>4.88</v>
       </c>
       <c r="F56" s="34" t="inlineStr">
         <is>
@@ -26135,7 +26157,7 @@
         </is>
       </c>
       <c r="G56" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H56" s="34" t="inlineStr">
         <is>
@@ -26143,7 +26165,7 @@
         </is>
       </c>
       <c r="I56" t="n">
-        <v>4.86</v>
+        <v>4.88</v>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1" s="58">
@@ -26167,7 +26189,7 @@
         </is>
       </c>
       <c r="E57" s="33" t="n">
-        <v>2.64</v>
+        <v>2.7</v>
       </c>
       <c r="F57" s="34" t="inlineStr">
         <is>
@@ -26175,7 +26197,7 @@
         </is>
       </c>
       <c r="G57" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H57" s="34" t="inlineStr">
         <is>
@@ -26183,7 +26205,7 @@
         </is>
       </c>
       <c r="I57" t="n">
-        <v>2.64</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="58">
@@ -26207,7 +26229,7 @@
         </is>
       </c>
       <c r="E58" s="33" t="n">
-        <v>12.3</v>
+        <v>12.4</v>
       </c>
       <c r="F58" s="34" t="inlineStr">
         <is>
@@ -26215,7 +26237,7 @@
         </is>
       </c>
       <c r="G58" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H58" s="34" t="inlineStr">
         <is>
@@ -26223,7 +26245,7 @@
         </is>
       </c>
       <c r="I58" t="n">
-        <v>12.3</v>
+        <v>12.4</v>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="58">
@@ -26247,7 +26269,7 @@
         </is>
       </c>
       <c r="E59" s="33" t="n">
-        <v>18</v>
+        <v>19.2</v>
       </c>
       <c r="F59" s="34" t="inlineStr">
         <is>
@@ -26255,7 +26277,7 @@
         </is>
       </c>
       <c r="G59" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H59" s="34" t="inlineStr">
         <is>
@@ -26263,7 +26285,7 @@
         </is>
       </c>
       <c r="I59" t="n">
-        <v>17.299999</v>
+        <v>19.200001</v>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1" s="58">
@@ -26287,7 +26309,7 @@
         </is>
       </c>
       <c r="E60" s="33" t="n">
-        <v>176.845</v>
+        <v>175.445</v>
       </c>
       <c r="F60" s="34" t="inlineStr">
         <is>
@@ -26295,7 +26317,7 @@
         </is>
       </c>
       <c r="G60" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H60" s="34" t="inlineStr">
         <is>
@@ -26303,7 +26325,7 @@
         </is>
       </c>
       <c r="I60" t="n">
-        <v>176.845001</v>
+        <v>175.445007</v>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="58">
@@ -26327,7 +26349,7 @@
         </is>
       </c>
       <c r="E61" s="33" t="n">
-        <v>207.32</v>
+        <v>196.28</v>
       </c>
       <c r="F61" s="34" t="inlineStr">
         <is>
@@ -26335,7 +26357,7 @@
         </is>
       </c>
       <c r="G61" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H61" s="34" t="inlineStr">
         <is>
@@ -26343,7 +26365,7 @@
         </is>
       </c>
       <c r="I61" t="n">
-        <v>207.320007</v>
+        <v>196.279999</v>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="58">
@@ -26367,7 +26389,7 @@
         </is>
       </c>
       <c r="E62" s="33" t="n">
-        <v>568.23</v>
+        <v>592.92</v>
       </c>
       <c r="F62" s="34" t="inlineStr">
         <is>
@@ -26375,7 +26397,7 @@
         </is>
       </c>
       <c r="G62" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H62" s="34" t="inlineStr">
         <is>
@@ -26383,7 +26405,7 @@
         </is>
       </c>
       <c r="I62" t="n">
-        <v>568.22998</v>
+        <v>592.919983</v>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1" s="58">
@@ -26407,7 +26429,7 @@
         </is>
       </c>
       <c r="E63" s="33" t="n">
-        <v>160.76</v>
+        <v>160.27</v>
       </c>
       <c r="F63" s="34" t="inlineStr">
         <is>
@@ -26415,7 +26437,7 @@
         </is>
       </c>
       <c r="G63" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H63" s="34" t="inlineStr">
         <is>
@@ -26423,7 +26445,7 @@
         </is>
       </c>
       <c r="I63" t="n">
-        <v>160.759995</v>
+        <v>160.270004</v>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="58">
@@ -26447,7 +26469,7 @@
         </is>
       </c>
       <c r="E64" s="33" t="n">
-        <v>50.26</v>
+        <v>47.78</v>
       </c>
       <c r="F64" s="34" t="inlineStr">
         <is>
@@ -26455,7 +26477,7 @@
         </is>
       </c>
       <c r="G64" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H64" s="34" t="inlineStr">
         <is>
@@ -26463,7 +26485,7 @@
         </is>
       </c>
       <c r="I64" t="n">
-        <v>50.259998</v>
+        <v>47.779999</v>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1" s="58">
@@ -26487,7 +26509,7 @@
         </is>
       </c>
       <c r="E65" s="33" t="n">
-        <v>205.91</v>
+        <v>205.08</v>
       </c>
       <c r="F65" s="34" t="inlineStr">
         <is>
@@ -26495,7 +26517,7 @@
         </is>
       </c>
       <c r="G65" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H65" s="34" t="inlineStr">
         <is>
@@ -26503,7 +26525,7 @@
         </is>
       </c>
       <c r="I65" t="n">
-        <v>205.910004</v>
+        <v>205.080002</v>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1" s="58">
@@ -26527,7 +26549,7 @@
         </is>
       </c>
       <c r="E66" s="33" t="n">
-        <v>147.02</v>
+        <v>144.14</v>
       </c>
       <c r="F66" s="34" t="inlineStr">
         <is>
@@ -26535,7 +26557,7 @@
         </is>
       </c>
       <c r="G66" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H66" s="34" t="inlineStr">
         <is>
@@ -26543,7 +26565,7 @@
         </is>
       </c>
       <c r="I66" t="n">
-        <v>147.020004</v>
+        <v>144.139999</v>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1" s="58">
@@ -26567,7 +26589,7 @@
         </is>
       </c>
       <c r="E67" s="33" t="n">
-        <v>142.24</v>
+        <v>133.58</v>
       </c>
       <c r="F67" s="34" t="inlineStr">
         <is>
@@ -26575,7 +26597,7 @@
         </is>
       </c>
       <c r="G67" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H67" s="34" t="inlineStr">
         <is>
@@ -26583,7 +26605,7 @@
         </is>
       </c>
       <c r="I67" t="n">
-        <v>142.240005</v>
+        <v>133.580002</v>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1" s="58">
@@ -26607,7 +26629,7 @@
         </is>
       </c>
       <c r="E68" s="33" t="n">
-        <v>237.33</v>
+        <v>238.73</v>
       </c>
       <c r="F68" s="34" t="inlineStr">
         <is>
@@ -26615,7 +26637,7 @@
         </is>
       </c>
       <c r="G68" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H68" s="34" t="inlineStr">
         <is>
@@ -26623,7 +26645,7 @@
         </is>
       </c>
       <c r="I68" t="n">
-        <v>237.330002</v>
+        <v>238.729996</v>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="58">
@@ -26647,23 +26669,23 @@
         </is>
       </c>
       <c r="E69" s="33" t="n">
+        <v>1112</v>
+      </c>
+      <c r="F69" s="34" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G69" s="28" t="n">
+        <v>46191</v>
+      </c>
+      <c r="H69" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I69" t="n">
         <v>1122.5</v>
-      </c>
-      <c r="F69" s="34" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="G69" s="28" t="n">
-        <v>46190</v>
-      </c>
-      <c r="H69" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I69" t="n">
-        <v>1129.349976</v>
       </c>
     </row>
     <row r="70" ht="15" customHeight="1" s="58">
@@ -26687,7 +26709,7 @@
         </is>
       </c>
       <c r="E70" s="33" t="n">
-        <v>95.63</v>
+        <v>94.11</v>
       </c>
       <c r="F70" s="34" t="inlineStr">
         <is>
@@ -26695,7 +26717,7 @@
         </is>
       </c>
       <c r="G70" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H70" s="34" t="inlineStr">
         <is>
@@ -26703,7 +26725,7 @@
         </is>
       </c>
       <c r="I70" t="n">
-        <v>95.629997</v>
+        <v>94.110001</v>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1" s="58">
@@ -26727,7 +26749,7 @@
         </is>
       </c>
       <c r="E71" s="33" t="n">
-        <v>1498.77</v>
+        <v>1448.21</v>
       </c>
       <c r="F71" s="34" t="inlineStr">
         <is>
@@ -26735,7 +26757,7 @@
         </is>
       </c>
       <c r="G71" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H71" s="34" t="inlineStr">
         <is>
@@ -26743,7 +26765,7 @@
         </is>
       </c>
       <c r="I71" t="n">
-        <v>1498.77002</v>
+        <v>1448.209961</v>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1" s="58">
@@ -26767,7 +26789,7 @@
         </is>
       </c>
       <c r="E72" s="33" t="n">
-        <v>109.22</v>
+        <v>106.96</v>
       </c>
       <c r="F72" s="34" t="inlineStr">
         <is>
@@ -26775,7 +26797,7 @@
         </is>
       </c>
       <c r="G72" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H72" s="34" t="inlineStr">
         <is>
@@ -26783,7 +26805,7 @@
         </is>
       </c>
       <c r="I72" t="n">
-        <v>109.220001</v>
+        <v>106.959999</v>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1" s="58">
@@ -26807,7 +26829,7 @@
         </is>
       </c>
       <c r="E73" s="33" t="n">
-        <v>207.41</v>
+        <v>204.65</v>
       </c>
       <c r="F73" s="34" t="inlineStr">
         <is>
@@ -26815,7 +26837,7 @@
         </is>
       </c>
       <c r="G73" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H73" s="34" t="inlineStr">
         <is>
@@ -26823,7 +26845,7 @@
         </is>
       </c>
       <c r="I73" t="n">
-        <v>207.410004</v>
+        <v>204.649994</v>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1" s="58">
@@ -26847,7 +26869,7 @@
         </is>
       </c>
       <c r="E74" s="33" t="n">
-        <v>89.59999999999999</v>
+        <v>84.52</v>
       </c>
       <c r="F74" s="34" t="inlineStr">
         <is>
@@ -26855,7 +26877,7 @@
         </is>
       </c>
       <c r="G74" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H74" s="34" t="inlineStr">
         <is>
@@ -26863,7 +26885,7 @@
         </is>
       </c>
       <c r="I74" t="n">
-        <v>89.599998</v>
+        <v>84.519997</v>
       </c>
     </row>
     <row r="75" ht="15" customHeight="1" s="58">
@@ -26887,7 +26909,7 @@
         </is>
       </c>
       <c r="E75" s="33" t="n">
-        <v>96.56</v>
+        <v>94.65000000000001</v>
       </c>
       <c r="F75" s="34" t="inlineStr">
         <is>
@@ -26895,7 +26917,7 @@
         </is>
       </c>
       <c r="G75" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H75" s="34" t="inlineStr">
         <is>
@@ -26903,7 +26925,7 @@
         </is>
       </c>
       <c r="I75" t="n">
-        <v>96.55999799999999</v>
+        <v>94.650002</v>
       </c>
     </row>
     <row r="76" ht="15" customHeight="1" s="58">
@@ -26927,7 +26949,7 @@
         </is>
       </c>
       <c r="E76" s="33" t="n">
-        <v>409.35</v>
+        <v>408.56</v>
       </c>
       <c r="F76" s="34" t="inlineStr">
         <is>
@@ -26935,7 +26957,7 @@
         </is>
       </c>
       <c r="G76" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H76" s="34" t="inlineStr">
         <is>
@@ -26943,7 +26965,7 @@
         </is>
       </c>
       <c r="I76" t="n">
-        <v>409.350006</v>
+        <v>408.559998</v>
       </c>
     </row>
     <row r="77" ht="15" customHeight="1" s="58">
@@ -26967,7 +26989,7 @@
         </is>
       </c>
       <c r="E77" s="33" t="n">
-        <v>404.66</v>
+        <v>396.38</v>
       </c>
       <c r="F77" s="34" t="inlineStr">
         <is>
@@ -26975,7 +26997,7 @@
         </is>
       </c>
       <c r="G77" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H77" s="34" t="inlineStr">
         <is>
@@ -26983,7 +27005,7 @@
         </is>
       </c>
       <c r="I77" t="n">
-        <v>404.660004</v>
+        <v>396.380005</v>
       </c>
     </row>
     <row r="78" ht="15" customHeight="1" s="58">
@@ -27007,7 +27029,7 @@
         </is>
       </c>
       <c r="E78" s="33" t="n">
-        <v>52.76</v>
+        <v>50.77</v>
       </c>
       <c r="F78" s="34" t="inlineStr">
         <is>
@@ -27015,7 +27037,7 @@
         </is>
       </c>
       <c r="G78" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H78" s="34" t="inlineStr">
         <is>
@@ -27023,7 +27045,7 @@
         </is>
       </c>
       <c r="I78" t="n">
-        <v>52.759998</v>
+        <v>50.77</v>
       </c>
     </row>
     <row r="79" ht="15" customHeight="1" s="58">
@@ -27047,7 +27069,7 @@
         </is>
       </c>
       <c r="E79" s="33" t="n">
-        <v>96.78</v>
+        <v>96.04000000000001</v>
       </c>
       <c r="F79" s="34" t="inlineStr">
         <is>
@@ -27055,7 +27077,7 @@
         </is>
       </c>
       <c r="G79" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H79" s="34" t="inlineStr">
         <is>
@@ -27063,7 +27085,7 @@
         </is>
       </c>
       <c r="I79" t="n">
-        <v>96.779999</v>
+        <v>96.040001</v>
       </c>
     </row>
     <row r="80" ht="15" customHeight="1" s="58">
@@ -27087,7 +27109,7 @@
         </is>
       </c>
       <c r="E80" s="33" t="n">
-        <v>299.24</v>
+        <v>295.95</v>
       </c>
       <c r="F80" s="34" t="inlineStr">
         <is>
@@ -27095,7 +27117,7 @@
         </is>
       </c>
       <c r="G80" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H80" s="34" t="inlineStr">
         <is>
@@ -27103,7 +27125,7 @@
         </is>
       </c>
       <c r="I80" t="n">
-        <v>299.23999</v>
+        <v>295.950012</v>
       </c>
     </row>
     <row r="81" ht="15" customHeight="1" s="58">
@@ -27127,7 +27149,7 @@
         </is>
       </c>
       <c r="E81" s="33" t="n">
-        <v>169.27</v>
+        <v>164.915</v>
       </c>
       <c r="F81" s="34" t="inlineStr">
         <is>
@@ -27135,7 +27157,7 @@
         </is>
       </c>
       <c r="G81" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H81" s="34" t="inlineStr">
         <is>
@@ -27143,7 +27165,7 @@
         </is>
       </c>
       <c r="I81" t="n">
-        <v>169.270004</v>
+        <v>164.914993</v>
       </c>
     </row>
     <row r="82" ht="15" customHeight="1" s="58">
@@ -27167,7 +27189,7 @@
         </is>
       </c>
       <c r="E82" s="33" t="n">
-        <v>600.21</v>
+        <v>567.58</v>
       </c>
       <c r="F82" s="34" t="inlineStr">
         <is>
@@ -27175,7 +27197,7 @@
         </is>
       </c>
       <c r="G82" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H82" s="34" t="inlineStr">
         <is>
@@ -27183,7 +27205,7 @@
         </is>
       </c>
       <c r="I82" t="n">
-        <v>600.210022</v>
+        <v>567.580017</v>
       </c>
     </row>
     <row r="83" ht="15" customHeight="1" s="58">
@@ -27207,7 +27229,7 @@
         </is>
       </c>
       <c r="E83" s="33" t="n">
-        <v>91.98999999999999</v>
+        <v>99.16</v>
       </c>
       <c r="F83" s="34" t="inlineStr">
         <is>
@@ -27215,7 +27237,7 @@
         </is>
       </c>
       <c r="G83" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H83" s="34" t="inlineStr">
         <is>
@@ -27223,7 +27245,7 @@
         </is>
       </c>
       <c r="I83" t="n">
-        <v>91.989998</v>
+        <v>99.160004</v>
       </c>
     </row>
     <row r="84" ht="15" customHeight="1" s="58">
@@ -27247,7 +27269,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>76.13</v>
+        <v>74.20999999999999</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -27255,7 +27277,7 @@
         </is>
       </c>
       <c r="G84" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H84" s="34" t="inlineStr">
         <is>
@@ -27263,7 +27285,7 @@
         </is>
       </c>
       <c r="I84" t="n">
-        <v>73.921914</v>
+        <v>76.154329</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="58">
@@ -27287,7 +27309,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>603.33</v>
+        <v>602.73</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -27295,7 +27317,7 @@
         </is>
       </c>
       <c r="G85" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H85" s="34" t="inlineStr">
         <is>
@@ -27303,7 +27325,7 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>617.3147740000001</v>
+        <v>603.383287</v>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="58">
@@ -27327,7 +27349,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>65522</v>
+        <v>64619</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -27335,7 +27357,7 @@
         </is>
       </c>
       <c r="G86" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H86" s="34" t="inlineStr">
         <is>
@@ -27343,7 +27365,7 @@
         </is>
       </c>
       <c r="I86" t="n">
-        <v>66354.39950100001</v>
+        <v>65537.478196</v>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="58">
@@ -27367,7 +27389,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.007159</v>
+        <v>0.006961</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -27375,7 +27397,7 @@
         </is>
       </c>
       <c r="G87" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H87" s="34" t="inlineStr">
         <is>
@@ -27383,7 +27405,7 @@
         </is>
       </c>
       <c r="I87" t="n">
-        <v>0.007116</v>
+        <v>0.007156</v>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="58">
@@ -27407,7 +27429,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.011297</v>
+        <v>0.011333</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -27415,7 +27437,7 @@
         </is>
       </c>
       <c r="G88" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H88" s="34" t="inlineStr">
         <is>
@@ -27423,7 +27445,7 @@
         </is>
       </c>
       <c r="I88" t="n">
-        <v>0.011434</v>
+        <v>0.0113</v>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="58">
@@ -27447,7 +27469,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>73.31999999999999</v>
+        <v>72.34999999999999</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -27455,7 +27477,7 @@
         </is>
       </c>
       <c r="G89" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H89" s="34" t="inlineStr">
         <is>
@@ -27463,7 +27485,7 @@
         </is>
       </c>
       <c r="I89" t="n">
-        <v>74.175377</v>
+        <v>73.334495</v>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="58">
@@ -27487,7 +27509,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>1.9</v>
+        <v>1.92</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -27495,7 +27517,7 @@
         </is>
       </c>
       <c r="G90" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H90" s="34" t="inlineStr">
         <is>
@@ -27503,7 +27525,7 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>1.986521</v>
+        <v>1.89794</v>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="58">
@@ -27535,7 +27557,7 @@
         </is>
       </c>
       <c r="G91" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H91" s="34" t="inlineStr">
         <is>
@@ -27567,7 +27589,7 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
-        <v>0.018253</v>
+        <v>0.017602</v>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
@@ -27575,7 +27597,7 @@
         </is>
       </c>
       <c r="G92" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H92" s="34" t="inlineStr">
         <is>
@@ -27583,7 +27605,7 @@
         </is>
       </c>
       <c r="I92" t="n">
-        <v>0.016036</v>
+        <v>0.018237</v>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="58">
@@ -27607,7 +27629,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>2.797258</v>
+        <v>2.843913</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -27615,7 +27637,7 @@
         </is>
       </c>
       <c r="G93" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H93" s="34" t="inlineStr">
         <is>
@@ -27623,7 +27645,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>2.809108</v>
+        <v>2.809242</v>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="58">
@@ -27647,7 +27669,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>26.05618</v>
+        <v>25.132142</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -27655,7 +27677,7 @@
         </is>
       </c>
       <c r="G94" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H94" s="34" t="inlineStr">
         <is>
@@ -27663,7 +27685,7 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>25.756446</v>
+        <v>26.172029</v>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="58">
@@ -27687,7 +27709,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.11331</v>
+        <v>0.114241</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -27695,7 +27717,7 @@
         </is>
       </c>
       <c r="G95" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H95" s="34" t="inlineStr">
         <is>
@@ -27703,7 +27725,7 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>0.113973</v>
+        <v>0.113777</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="58">
@@ -27727,7 +27749,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>19614.2583</v>
+        <v>19679.1345</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -27735,7 +27757,7 @@
         </is>
       </c>
       <c r="G96" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H96" s="34" t="inlineStr">
         <is>
@@ -27743,7 +27765,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>20068.903314</v>
+        <v>19700.464318</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="58">
@@ -27767,7 +27789,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2130120.22</v>
+        <v>2109810.35</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -27775,7 +27797,7 @@
         </is>
       </c>
       <c r="G97" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H97" s="34" t="inlineStr">
         <is>
@@ -27783,7 +27805,7 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>2157181.527783</v>
+        <v>2139798.663086</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="58">
@@ -27807,7 +27829,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>2.830873</v>
+        <v>2.814691</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -27815,7 +27837,7 @@
         </is>
       </c>
       <c r="G98" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H98" s="34" t="inlineStr">
         <is>
@@ -27823,7 +27845,7 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>2.858493</v>
+        <v>2.842868</v>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="58">
@@ -27847,7 +27869,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>58009.5436</v>
+        <v>57329.8085</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -27855,7 +27877,7 @@
         </is>
       </c>
       <c r="G99" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H99" s="34" t="inlineStr">
         <is>
@@ -27863,7 +27885,7 @@
         </is>
       </c>
       <c r="I99" t="n">
-        <v>58346.787202</v>
+        <v>58191.597022</v>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="58">
@@ -27887,7 +27909,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>25.038877</v>
+        <v>25.028217</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -27895,7 +27917,7 @@
         </is>
       </c>
       <c r="G100" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H100" s="34" t="inlineStr">
         <is>
@@ -27903,7 +27925,7 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>25.244738</v>
+        <v>25.153691</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="58">
@@ -27927,7 +27949,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>65522</v>
+        <v>64619</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -27935,7 +27957,7 @@
         </is>
       </c>
       <c r="G101" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H101" s="34" t="inlineStr">
         <is>
@@ -27943,7 +27965,7 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>66354.39950100001</v>
+        <v>65537.478196</v>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="58">
@@ -27967,7 +27989,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>17.79</v>
+        <v>17.59</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -27975,7 +27997,7 @@
         </is>
       </c>
       <c r="G102" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H102" s="34" t="inlineStr">
         <is>
@@ -27983,7 +28005,7 @@
         </is>
       </c>
       <c r="I102" t="n">
-        <v>18.020095</v>
+        <v>17.792892</v>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="58">
@@ -28081,7 +28103,7 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
-        <v>0.007159</v>
+        <v>0.006961</v>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
@@ -28089,7 +28111,7 @@
         </is>
       </c>
       <c r="G105" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H105" s="34" t="inlineStr">
         <is>
@@ -28097,7 +28119,7 @@
         </is>
       </c>
       <c r="I105" t="n">
-        <v>0.007116</v>
+        <v>0.007156</v>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="58">
@@ -28121,7 +28143,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>73.31999999999999</v>
+        <v>72.34999999999999</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>
@@ -28129,7 +28151,7 @@
         </is>
       </c>
       <c r="G106" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H106" s="34" t="inlineStr">
         <is>
@@ -28137,7 +28159,7 @@
         </is>
       </c>
       <c r="I106" t="n">
-        <v>74.175377</v>
+        <v>73.334495</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="58">
@@ -28169,7 +28191,7 @@
         </is>
       </c>
       <c r="G107" s="28" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="H107" s="34" t="inlineStr">
         <is>
@@ -28201,27 +28223,27 @@
         </is>
       </c>
       <c r="E108" t="n">
+        <v>23.9542</v>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G108" s="47" t="n">
+        <v>46185</v>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I108" t="n">
         <v>23.7132</v>
       </c>
-      <c r="F108" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G108" s="47" t="n">
-        <v>46184</v>
-      </c>
-      <c r="H108" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I108" t="n">
-        <v>22.8715</v>
-      </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily dashboard update — 2026-06-19
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -22149,16 +22149,38 @@
       </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="58">
-      <c r="B23" s="28" t="n"/>
-      <c r="C23" s="29" t="n"/>
-      <c r="D23" s="29" t="n"/>
-      <c r="E23" s="29" t="n"/>
-      <c r="F23" s="30" t="n"/>
-      <c r="G23" s="29" t="n"/>
-      <c r="H23" s="29" t="n"/>
-      <c r="I23" s="29" t="n"/>
-      <c r="J23" s="31" t="n"/>
-      <c r="K23" s="32" t="n"/>
+      <c r="B23" s="28" t="n">
+        <v>46192</v>
+      </c>
+      <c r="C23" s="29" t="n">
+        <v>26712406</v>
+      </c>
+      <c r="D23" s="29" t="n">
+        <v>22763316</v>
+      </c>
+      <c r="E23" s="29" t="n">
+        <v>3949090</v>
+      </c>
+      <c r="F23" s="30" t="n">
+        <v>0.1735</v>
+      </c>
+      <c r="G23" s="29" t="n">
+        <v>19130171</v>
+      </c>
+      <c r="H23" s="29" t="n">
+        <v>5031721</v>
+      </c>
+      <c r="I23" s="29" t="n">
+        <v>1149451</v>
+      </c>
+      <c r="J23" s="31" t="n">
+        <v>32.76</v>
+      </c>
+      <c r="K23" s="32" t="inlineStr">
+        <is>
+          <t>Auto weekly snapshot</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="58">
       <c r="B24" s="28" t="n"/>
@@ -23764,7 +23786,7 @@
         </is>
       </c>
       <c r="C5" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="D5" s="64" t="inlineStr">
         <is>
@@ -23779,11 +23801,11 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>32.65</v>
+        <v>32.76</v>
       </c>
       <c r="D6" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-06-18</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-06-19</t>
         </is>
       </c>
     </row>
@@ -23828,11 +23850,11 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>25.3898</v>
+        <v>25.4035</v>
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-06-18</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-06-19</t>
         </is>
       </c>
     </row>
@@ -23947,27 +23969,27 @@
         </is>
       </c>
       <c r="E5" s="33" t="n">
+        <v>26.3904</v>
+      </c>
+      <c r="F5" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G5" s="28" t="n">
+        <v>46189</v>
+      </c>
+      <c r="H5" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
         <v>27.7204</v>
       </c>
-      <c r="F5" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G5" s="28" t="n">
-        <v>46188</v>
-      </c>
-      <c r="H5" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I5" t="n">
-        <v>25.8262</v>
-      </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -23992,27 +24014,27 @@
         </is>
       </c>
       <c r="E6" s="33" t="n">
+        <v>10.6881</v>
+      </c>
+      <c r="F6" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G6" s="28" t="n">
+        <v>46190</v>
+      </c>
+      <c r="H6" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
         <v>10.688</v>
       </c>
-      <c r="F6" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G6" s="28" t="n">
-        <v>46189</v>
-      </c>
-      <c r="H6" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I6" t="n">
-        <v>10.6878</v>
-      </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
     </row>
@@ -24037,27 +24059,27 @@
         </is>
       </c>
       <c r="E7" s="33" t="n">
+        <v>7.2353</v>
+      </c>
+      <c r="F7" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G7" s="28" t="n">
+        <v>46189</v>
+      </c>
+      <c r="H7" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
         <v>7.2207</v>
       </c>
-      <c r="F7" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G7" s="28" t="n">
-        <v>46188</v>
-      </c>
-      <c r="H7" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I7" t="n">
-        <v>7.1641</v>
-      </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -24082,27 +24104,27 @@
         </is>
       </c>
       <c r="E8" s="33" t="n">
+        <v>9.8331</v>
+      </c>
+      <c r="F8" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G8" s="28" t="n">
+        <v>46189</v>
+      </c>
+      <c r="H8" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
         <v>9.8744</v>
       </c>
-      <c r="F8" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G8" s="28" t="n">
-        <v>46188</v>
-      </c>
-      <c r="H8" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I8" t="n">
-        <v>9.5237</v>
-      </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -24127,27 +24149,27 @@
         </is>
       </c>
       <c r="E9" s="33" t="n">
+        <v>9.472899999999999</v>
+      </c>
+      <c r="F9" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G9" s="28" t="n">
+        <v>46190</v>
+      </c>
+      <c r="H9" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
         <v>9.332100000000001</v>
       </c>
-      <c r="F9" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G9" s="28" t="n">
-        <v>46189</v>
-      </c>
-      <c r="H9" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I9" t="n">
-        <v>9.372999999999999</v>
-      </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
     </row>
@@ -24172,27 +24194,27 @@
         </is>
       </c>
       <c r="E10" s="33" t="n">
+        <v>13.8162</v>
+      </c>
+      <c r="F10" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G10" s="28" t="n">
+        <v>46189</v>
+      </c>
+      <c r="H10" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
         <v>13.7411</v>
       </c>
-      <c r="F10" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G10" s="28" t="n">
-        <v>46188</v>
-      </c>
-      <c r="H10" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I10" t="n">
-        <v>13.2399</v>
-      </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -24217,27 +24239,27 @@
         </is>
       </c>
       <c r="E11" s="33" t="n">
+        <v>13.4113</v>
+      </c>
+      <c r="F11" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G11" s="28" t="n">
+        <v>46190</v>
+      </c>
+      <c r="H11" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
         <v>13.3095</v>
       </c>
-      <c r="F11" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G11" s="28" t="n">
-        <v>46189</v>
-      </c>
-      <c r="H11" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I11" t="n">
-        <v>13.2787</v>
-      </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
     </row>
@@ -24262,27 +24284,27 @@
         </is>
       </c>
       <c r="E12" s="33" t="n">
+        <v>27.0928</v>
+      </c>
+      <c r="F12" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G12" s="28" t="n">
+        <v>46190</v>
+      </c>
+      <c r="H12" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
         <v>26.703</v>
       </c>
-      <c r="F12" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G12" s="28" t="n">
-        <v>46189</v>
-      </c>
-      <c r="H12" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I12" t="n">
-        <v>26.987</v>
-      </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
     </row>
@@ -24307,27 +24329,27 @@
         </is>
       </c>
       <c r="E13" s="33" t="n">
+        <v>36.3498</v>
+      </c>
+      <c r="F13" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G13" s="28" t="n">
+        <v>46190</v>
+      </c>
+      <c r="H13" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
         <v>36.4324</v>
       </c>
-      <c r="F13" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G13" s="28" t="n">
-        <v>46189</v>
-      </c>
-      <c r="H13" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I13" t="n">
-        <v>36.4884</v>
-      </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
     </row>
@@ -24352,27 +24374,27 @@
         </is>
       </c>
       <c r="E14" s="33" t="n">
+        <v>25.5786</v>
+      </c>
+      <c r="F14" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G14" s="28" t="n">
+        <v>46190</v>
+      </c>
+      <c r="H14" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
         <v>25.5798</v>
       </c>
-      <c r="F14" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G14" s="28" t="n">
-        <v>46189</v>
-      </c>
-      <c r="H14" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I14" t="n">
-        <v>25.5415</v>
-      </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
     </row>
@@ -24397,27 +24419,27 @@
         </is>
       </c>
       <c r="E15" s="33" t="n">
+        <v>14.9777</v>
+      </c>
+      <c r="F15" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G15" s="28" t="n">
+        <v>46188</v>
+      </c>
+      <c r="H15" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
         <v>15.0377</v>
       </c>
-      <c r="F15" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G15" s="28" t="n">
-        <v>46185</v>
-      </c>
-      <c r="H15" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I15" t="n">
-        <v>15.0939</v>
-      </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
     </row>
@@ -24442,27 +24464,27 @@
         </is>
       </c>
       <c r="E16" s="33" t="n">
+        <v>81.5475</v>
+      </c>
+      <c r="F16" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G16" s="28" t="n">
+        <v>46190</v>
+      </c>
+      <c r="H16" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
         <v>81.7367</v>
       </c>
-      <c r="F16" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G16" s="28" t="n">
-        <v>46189</v>
-      </c>
-      <c r="H16" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I16" t="n">
-        <v>81.8086</v>
-      </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
     </row>
@@ -24487,27 +24509,27 @@
         </is>
       </c>
       <c r="E17" s="33" t="n">
+        <v>53.5889</v>
+      </c>
+      <c r="F17" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G17" s="28" t="n">
+        <v>46190</v>
+      </c>
+      <c r="H17" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
         <v>53.5816</v>
       </c>
-      <c r="F17" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G17" s="28" t="n">
-        <v>46189</v>
-      </c>
-      <c r="H17" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I17" t="n">
-        <v>53.5038</v>
-      </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
     </row>
@@ -24532,27 +24554,27 @@
         </is>
       </c>
       <c r="E18" s="33" t="n">
+        <v>16.5015</v>
+      </c>
+      <c r="F18" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G18" s="28" t="n">
+        <v>46190</v>
+      </c>
+      <c r="H18" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
         <v>16.4959</v>
       </c>
-      <c r="F18" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G18" s="28" t="n">
-        <v>46189</v>
-      </c>
-      <c r="H18" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I18" t="n">
-        <v>16.5024</v>
-      </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
     </row>
@@ -24577,27 +24599,27 @@
         </is>
       </c>
       <c r="E19" s="33" t="n">
+        <v>23.4072</v>
+      </c>
+      <c r="F19" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G19" s="28" t="n">
+        <v>46190</v>
+      </c>
+      <c r="H19" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
         <v>23.4068</v>
       </c>
-      <c r="F19" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G19" s="28" t="n">
-        <v>46189</v>
-      </c>
-      <c r="H19" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I19" t="n">
-        <v>23.4061</v>
-      </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
     </row>
@@ -24622,27 +24644,27 @@
         </is>
       </c>
       <c r="E20" s="33" t="n">
+        <v>41.2001</v>
+      </c>
+      <c r="F20" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G20" s="28" t="n">
+        <v>46189</v>
+      </c>
+      <c r="H20" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
         <v>41.4428</v>
       </c>
-      <c r="F20" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G20" s="28" t="n">
-        <v>46188</v>
-      </c>
-      <c r="H20" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I20" t="n">
-        <v>40.7663</v>
-      </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -24667,27 +24689,27 @@
         </is>
       </c>
       <c r="E21" s="33" t="n">
+        <v>13.5424</v>
+      </c>
+      <c r="F21" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G21" s="28" t="n">
+        <v>46190</v>
+      </c>
+      <c r="H21" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
         <v>13.5882</v>
       </c>
-      <c r="F21" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G21" s="28" t="n">
-        <v>46189</v>
-      </c>
-      <c r="H21" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I21" t="n">
-        <v>13.6767</v>
-      </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
     </row>
@@ -24712,27 +24734,27 @@
         </is>
       </c>
       <c r="E22" s="33" t="n">
+        <v>13.1369</v>
+      </c>
+      <c r="F22" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G22" s="28" t="n">
+        <v>46189</v>
+      </c>
+      <c r="H22" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
         <v>13.2398</v>
       </c>
-      <c r="F22" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G22" s="28" t="n">
-        <v>46188</v>
-      </c>
-      <c r="H22" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I22" t="n">
-        <v>13.3532</v>
-      </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -24757,27 +24779,27 @@
         </is>
       </c>
       <c r="E23" s="33" t="n">
+        <v>12.5011</v>
+      </c>
+      <c r="F23" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G23" s="28" t="n">
+        <v>46190</v>
+      </c>
+      <c r="H23" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
         <v>12.477</v>
       </c>
-      <c r="F23" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G23" s="28" t="n">
-        <v>46189</v>
-      </c>
-      <c r="H23" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I23" t="n">
-        <v>12.4628</v>
-      </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
     </row>
@@ -24802,27 +24824,27 @@
         </is>
       </c>
       <c r="E24" s="33" t="n">
+        <v>12.0997</v>
+      </c>
+      <c r="F24" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G24" s="28" t="n">
+        <v>46189</v>
+      </c>
+      <c r="H24" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
         <v>12.0412</v>
       </c>
-      <c r="F24" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G24" s="28" t="n">
-        <v>46188</v>
-      </c>
-      <c r="H24" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I24" t="n">
-        <v>11.7378</v>
-      </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -24847,27 +24869,27 @@
         </is>
       </c>
       <c r="E25" s="33" t="n">
+        <v>9.900700000000001</v>
+      </c>
+      <c r="F25" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G25" s="28" t="n">
+        <v>46190</v>
+      </c>
+      <c r="H25" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
         <v>9.928100000000001</v>
       </c>
-      <c r="F25" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G25" s="28" t="n">
-        <v>46189</v>
-      </c>
-      <c r="H25" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I25" t="n">
-        <v>9.921799999999999</v>
-      </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
     </row>
@@ -24892,27 +24914,27 @@
         </is>
       </c>
       <c r="E26" s="33" t="n">
+        <v>13.8979</v>
+      </c>
+      <c r="F26" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G26" s="28" t="n">
+        <v>46190</v>
+      </c>
+      <c r="H26" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
         <v>13.9345</v>
       </c>
-      <c r="F26" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G26" s="28" t="n">
-        <v>46189</v>
-      </c>
-      <c r="H26" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I26" t="n">
-        <v>13.9253</v>
-      </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
     </row>
@@ -24937,27 +24959,27 @@
         </is>
       </c>
       <c r="E27" s="33" t="n">
+        <v>17.295</v>
+      </c>
+      <c r="F27" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G27" s="28" t="n">
+        <v>46190</v>
+      </c>
+      <c r="H27" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
         <v>17.2282</v>
       </c>
-      <c r="F27" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G27" s="28" t="n">
-        <v>46189</v>
-      </c>
-      <c r="H27" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I27" t="n">
-        <v>17.1935</v>
-      </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
     </row>
@@ -24982,27 +25004,27 @@
         </is>
       </c>
       <c r="E28" s="33" t="n">
+        <v>19.2269</v>
+      </c>
+      <c r="F28" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G28" s="28" t="n">
+        <v>46190</v>
+      </c>
+      <c r="H28" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
         <v>19.3198</v>
       </c>
-      <c r="F28" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G28" s="28" t="n">
-        <v>46189</v>
-      </c>
-      <c r="H28" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I28" t="n">
-        <v>19.2686</v>
-      </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
     </row>
@@ -25027,27 +25049,27 @@
         </is>
       </c>
       <c r="E29" s="33" t="n">
+        <v>27.9553</v>
+      </c>
+      <c r="F29" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G29" s="28" t="n">
+        <v>46189</v>
+      </c>
+      <c r="H29" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
         <v>28.7079</v>
       </c>
-      <c r="F29" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G29" s="28" t="n">
-        <v>46188</v>
-      </c>
-      <c r="H29" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I29" t="n">
-        <v>26.8484</v>
-      </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -25072,27 +25094,27 @@
         </is>
       </c>
       <c r="E30" s="33" t="n">
+        <v>39.515</v>
+      </c>
+      <c r="F30" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G30" s="28" t="n">
+        <v>46189</v>
+      </c>
+      <c r="H30" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
         <v>40.5797</v>
       </c>
-      <c r="F30" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G30" s="28" t="n">
-        <v>46188</v>
-      </c>
-      <c r="H30" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I30" t="n">
-        <v>39.1699</v>
-      </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -25117,27 +25139,27 @@
         </is>
       </c>
       <c r="E31" s="33" t="n">
+        <v>12.9833</v>
+      </c>
+      <c r="F31" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G31" s="28" t="n">
+        <v>46190</v>
+      </c>
+      <c r="H31" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
         <v>12.9887</v>
       </c>
-      <c r="F31" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G31" s="28" t="n">
-        <v>46189</v>
-      </c>
-      <c r="H31" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I31" t="n">
-        <v>13.0122</v>
-      </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
     </row>
@@ -25162,27 +25184,27 @@
         </is>
       </c>
       <c r="E32" s="33" t="n">
+        <v>21.7069</v>
+      </c>
+      <c r="F32" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G32" s="28" t="n">
+        <v>46190</v>
+      </c>
+      <c r="H32" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
         <v>21.7067</v>
       </c>
-      <c r="F32" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G32" s="28" t="n">
-        <v>46189</v>
-      </c>
-      <c r="H32" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I32" t="n">
-        <v>21.7065</v>
-      </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
     </row>
@@ -25207,27 +25229,27 @@
         </is>
       </c>
       <c r="E33" s="33" t="n">
+        <v>12.5135</v>
+      </c>
+      <c r="F33" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G33" s="28" t="n">
+        <v>46190</v>
+      </c>
+      <c r="H33" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
         <v>12.5343</v>
       </c>
-      <c r="F33" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G33" s="28" t="n">
-        <v>46189</v>
-      </c>
-      <c r="H33" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I33" t="n">
-        <v>12.5219</v>
-      </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
     </row>
@@ -25252,27 +25274,27 @@
         </is>
       </c>
       <c r="E34" s="33" t="n">
+        <v>16.2073</v>
+      </c>
+      <c r="F34" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G34" s="28" t="n">
+        <v>46190</v>
+      </c>
+      <c r="H34" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
         <v>16.207</v>
       </c>
-      <c r="F34" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G34" s="28" t="n">
-        <v>46189</v>
-      </c>
-      <c r="H34" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I34" t="n">
-        <v>16.2066</v>
-      </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
     </row>
@@ -25297,27 +25319,27 @@
         </is>
       </c>
       <c r="E35" s="33" t="n">
+        <v>27.843</v>
+      </c>
+      <c r="F35" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G35" s="28" t="n">
+        <v>46189</v>
+      </c>
+      <c r="H35" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
         <v>27.8097</v>
       </c>
-      <c r="F35" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G35" s="28" t="n">
-        <v>46188</v>
-      </c>
-      <c r="H35" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I35" t="n">
-        <v>27.2155</v>
-      </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -25342,27 +25364,27 @@
         </is>
       </c>
       <c r="E36" s="33" t="n">
+        <v>10.1966</v>
+      </c>
+      <c r="F36" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G36" s="28" t="n">
+        <v>46190</v>
+      </c>
+      <c r="H36" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
         <v>10.1449</v>
       </c>
-      <c r="F36" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G36" s="28" t="n">
-        <v>46189</v>
-      </c>
-      <c r="H36" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I36" t="n">
-        <v>10.1561</v>
-      </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
     </row>
@@ -25387,27 +25409,27 @@
         </is>
       </c>
       <c r="E37" s="33" t="n">
+        <v>22.686</v>
+      </c>
+      <c r="F37" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G37" s="28" t="n">
+        <v>46190</v>
+      </c>
+      <c r="H37" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
         <v>22.698</v>
       </c>
-      <c r="F37" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G37" s="28" t="n">
-        <v>46189</v>
-      </c>
-      <c r="H37" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I37" t="n">
-        <v>22.7039</v>
-      </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
     </row>
@@ -25432,7 +25454,7 @@
         </is>
       </c>
       <c r="E38" s="33" t="n">
-        <v>23.24</v>
+        <v>23.04</v>
       </c>
       <c r="F38" s="34" t="inlineStr">
         <is>
@@ -25440,7 +25462,7 @@
         </is>
       </c>
       <c r="G38" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H38" s="34" t="inlineStr">
         <is>
@@ -25448,7 +25470,7 @@
         </is>
       </c>
       <c r="I38" t="n">
-        <v>23.24</v>
+        <v>23.040001</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="58">
@@ -25472,7 +25494,7 @@
         </is>
       </c>
       <c r="E39" s="33" t="n">
-        <v>1.078</v>
+        <v>1.083</v>
       </c>
       <c r="F39" s="34" t="inlineStr">
         <is>
@@ -25480,7 +25502,7 @@
         </is>
       </c>
       <c r="G39" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H39" s="34" t="inlineStr">
         <is>
@@ -25488,7 +25510,7 @@
         </is>
       </c>
       <c r="I39" t="n">
-        <v>1.083</v>
+        <v>1.082</v>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="58">
@@ -25512,7 +25534,7 @@
         </is>
       </c>
       <c r="E40" s="33" t="n">
-        <v>784.6900000000001</v>
+        <v>792.59</v>
       </c>
       <c r="F40" s="34" t="inlineStr">
         <is>
@@ -25520,7 +25542,7 @@
         </is>
       </c>
       <c r="G40" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H40" s="34" t="inlineStr">
         <is>
@@ -25528,7 +25550,7 @@
         </is>
       </c>
       <c r="I40" t="n">
-        <v>784.690002</v>
+        <v>792.590027</v>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="58">
@@ -25552,7 +25574,7 @@
         </is>
       </c>
       <c r="E41" s="33" t="n">
-        <v>21.87</v>
+        <v>22.17</v>
       </c>
       <c r="F41" s="34" t="inlineStr">
         <is>
@@ -25560,7 +25582,7 @@
         </is>
       </c>
       <c r="G41" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H41" s="34" t="inlineStr">
         <is>
@@ -25568,7 +25590,7 @@
         </is>
       </c>
       <c r="I41" t="n">
-        <v>21.870001</v>
+        <v>22.17</v>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="58">
@@ -25592,7 +25614,7 @@
         </is>
       </c>
       <c r="E42" s="33" t="n">
-        <v>216</v>
+        <v>214.44</v>
       </c>
       <c r="F42" s="34" t="inlineStr">
         <is>
@@ -25600,7 +25622,7 @@
         </is>
       </c>
       <c r="G42" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H42" s="34" t="inlineStr">
         <is>
@@ -25608,7 +25630,7 @@
         </is>
       </c>
       <c r="I42" t="n">
-        <v>218.089996</v>
+        <v>214.440002</v>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="58">
@@ -25640,7 +25662,7 @@
         </is>
       </c>
       <c r="G43" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H43" s="34" t="inlineStr">
         <is>
@@ -25672,23 +25694,23 @@
         </is>
       </c>
       <c r="E44" s="33" t="n">
+        <v>176</v>
+      </c>
+      <c r="F44" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G44" s="28" t="n">
+        <v>46192</v>
+      </c>
+      <c r="H44" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
         <v>174</v>
-      </c>
-      <c r="F44" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G44" s="28" t="n">
-        <v>46191</v>
-      </c>
-      <c r="H44" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I44" t="n">
-        <v>175.5</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="58">
@@ -25712,7 +25734,7 @@
         </is>
       </c>
       <c r="E45" s="33" t="n">
-        <v>0.45</v>
+        <v>0.46</v>
       </c>
       <c r="F45" s="34" t="inlineStr">
         <is>
@@ -25720,7 +25742,7 @@
         </is>
       </c>
       <c r="G45" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H45" s="34" t="inlineStr">
         <is>
@@ -25728,7 +25750,7 @@
         </is>
       </c>
       <c r="I45" t="n">
-        <v>0.45</v>
+        <v>0.46</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="58">
@@ -25760,7 +25782,7 @@
         </is>
       </c>
       <c r="G46" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H46" s="34" t="inlineStr">
         <is>
@@ -25837,7 +25859,7 @@
         </is>
       </c>
       <c r="G48" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H48" s="34" t="inlineStr">
         <is>
@@ -25869,23 +25891,23 @@
         </is>
       </c>
       <c r="E49" s="33" t="n">
+        <v>63.5</v>
+      </c>
+      <c r="F49" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G49" s="28" t="n">
+        <v>46192</v>
+      </c>
+      <c r="H49" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
         <v>64.25</v>
-      </c>
-      <c r="F49" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G49" s="28" t="n">
-        <v>46191</v>
-      </c>
-      <c r="H49" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I49" t="n">
-        <v>65</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="58">
@@ -25909,7 +25931,7 @@
         </is>
       </c>
       <c r="E50" s="33" t="n">
-        <v>9.800000000000001</v>
+        <v>10.2</v>
       </c>
       <c r="F50" s="34" t="inlineStr">
         <is>
@@ -25917,7 +25939,7 @@
         </is>
       </c>
       <c r="G50" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H50" s="34" t="inlineStr">
         <is>
@@ -25925,7 +25947,7 @@
         </is>
       </c>
       <c r="I50" t="n">
-        <v>9.800000000000001</v>
+        <v>10.2</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="58">
@@ -25949,7 +25971,7 @@
         </is>
       </c>
       <c r="E51" s="33" t="n">
-        <v>15.9</v>
+        <v>15.8</v>
       </c>
       <c r="F51" s="34" t="inlineStr">
         <is>
@@ -25957,7 +25979,7 @@
         </is>
       </c>
       <c r="G51" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H51" s="34" t="inlineStr">
         <is>
@@ -25965,7 +25987,7 @@
         </is>
       </c>
       <c r="I51" t="n">
-        <v>15.9</v>
+        <v>15.8</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" s="58">
@@ -25997,7 +26019,7 @@
         </is>
       </c>
       <c r="G52" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H52" s="34" t="inlineStr">
         <is>
@@ -26029,7 +26051,7 @@
         </is>
       </c>
       <c r="E53" s="33" t="n">
-        <v>5.6</v>
+        <v>5.55</v>
       </c>
       <c r="F53" s="34" t="inlineStr">
         <is>
@@ -26037,7 +26059,7 @@
         </is>
       </c>
       <c r="G53" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H53" s="34" t="inlineStr">
         <is>
@@ -26045,7 +26067,7 @@
         </is>
       </c>
       <c r="I53" t="n">
-        <v>5.6</v>
+        <v>5.55</v>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="58">
@@ -26069,7 +26091,7 @@
         </is>
       </c>
       <c r="E54" s="33" t="n">
-        <v>22.7</v>
+        <v>21.9</v>
       </c>
       <c r="F54" s="34" t="inlineStr">
         <is>
@@ -26077,7 +26099,7 @@
         </is>
       </c>
       <c r="G54" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H54" s="34" t="inlineStr">
         <is>
@@ -26085,7 +26107,7 @@
         </is>
       </c>
       <c r="I54" t="n">
-        <v>22.700001</v>
+        <v>21.9</v>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="58">
@@ -26109,7 +26131,7 @@
         </is>
       </c>
       <c r="E55" s="33" t="n">
-        <v>3.5</v>
+        <v>3.48</v>
       </c>
       <c r="F55" s="34" t="inlineStr">
         <is>
@@ -26117,7 +26139,7 @@
         </is>
       </c>
       <c r="G55" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H55" s="34" t="inlineStr">
         <is>
@@ -26125,7 +26147,7 @@
         </is>
       </c>
       <c r="I55" t="n">
-        <v>3.54</v>
+        <v>3.48</v>
       </c>
     </row>
     <row r="56" ht="15" customHeight="1" s="58">
@@ -26149,7 +26171,7 @@
         </is>
       </c>
       <c r="E56" s="33" t="n">
-        <v>4.88</v>
+        <v>4.86</v>
       </c>
       <c r="F56" s="34" t="inlineStr">
         <is>
@@ -26157,7 +26179,7 @@
         </is>
       </c>
       <c r="G56" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H56" s="34" t="inlineStr">
         <is>
@@ -26165,7 +26187,7 @@
         </is>
       </c>
       <c r="I56" t="n">
-        <v>4.88</v>
+        <v>4.86</v>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1" s="58">
@@ -26189,7 +26211,7 @@
         </is>
       </c>
       <c r="E57" s="33" t="n">
-        <v>2.7</v>
+        <v>2.64</v>
       </c>
       <c r="F57" s="34" t="inlineStr">
         <is>
@@ -26197,7 +26219,7 @@
         </is>
       </c>
       <c r="G57" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H57" s="34" t="inlineStr">
         <is>
@@ -26205,7 +26227,7 @@
         </is>
       </c>
       <c r="I57" t="n">
-        <v>2.7</v>
+        <v>2.64</v>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="58">
@@ -26229,7 +26251,7 @@
         </is>
       </c>
       <c r="E58" s="33" t="n">
-        <v>12.4</v>
+        <v>12.3</v>
       </c>
       <c r="F58" s="34" t="inlineStr">
         <is>
@@ -26237,7 +26259,7 @@
         </is>
       </c>
       <c r="G58" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H58" s="34" t="inlineStr">
         <is>
@@ -26245,7 +26267,7 @@
         </is>
       </c>
       <c r="I58" t="n">
-        <v>12.4</v>
+        <v>12.3</v>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="58">
@@ -26269,7 +26291,7 @@
         </is>
       </c>
       <c r="E59" s="33" t="n">
-        <v>19.2</v>
+        <v>18.8</v>
       </c>
       <c r="F59" s="34" t="inlineStr">
         <is>
@@ -26277,7 +26299,7 @@
         </is>
       </c>
       <c r="G59" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H59" s="34" t="inlineStr">
         <is>
@@ -26285,7 +26307,7 @@
         </is>
       </c>
       <c r="I59" t="n">
-        <v>19.200001</v>
+        <v>18.799999</v>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1" s="58">
@@ -26309,7 +26331,7 @@
         </is>
       </c>
       <c r="E60" s="33" t="n">
-        <v>175.445</v>
+        <v>187.53</v>
       </c>
       <c r="F60" s="34" t="inlineStr">
         <is>
@@ -26317,7 +26339,7 @@
         </is>
       </c>
       <c r="G60" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H60" s="34" t="inlineStr">
         <is>
@@ -26325,7 +26347,7 @@
         </is>
       </c>
       <c r="I60" t="n">
-        <v>175.445007</v>
+        <v>187.529999</v>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="58">
@@ -26349,7 +26371,7 @@
         </is>
       </c>
       <c r="E61" s="33" t="n">
-        <v>196.28</v>
+        <v>195.16</v>
       </c>
       <c r="F61" s="34" t="inlineStr">
         <is>
@@ -26357,7 +26379,7 @@
         </is>
       </c>
       <c r="G61" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H61" s="34" t="inlineStr">
         <is>
@@ -26365,7 +26387,7 @@
         </is>
       </c>
       <c r="I61" t="n">
-        <v>196.279999</v>
+        <v>195.160004</v>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="58">
@@ -26389,7 +26411,7 @@
         </is>
       </c>
       <c r="E62" s="33" t="n">
-        <v>592.92</v>
+        <v>617.11</v>
       </c>
       <c r="F62" s="34" t="inlineStr">
         <is>
@@ -26397,7 +26419,7 @@
         </is>
       </c>
       <c r="G62" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H62" s="34" t="inlineStr">
         <is>
@@ -26405,7 +26427,7 @@
         </is>
       </c>
       <c r="I62" t="n">
-        <v>592.919983</v>
+        <v>617.1099850000001</v>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1" s="58">
@@ -26429,7 +26451,7 @@
         </is>
       </c>
       <c r="E63" s="33" t="n">
-        <v>160.27</v>
+        <v>165.29</v>
       </c>
       <c r="F63" s="34" t="inlineStr">
         <is>
@@ -26437,7 +26459,7 @@
         </is>
       </c>
       <c r="G63" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H63" s="34" t="inlineStr">
         <is>
@@ -26445,7 +26467,7 @@
         </is>
       </c>
       <c r="I63" t="n">
-        <v>160.270004</v>
+        <v>165.289993</v>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="58">
@@ -26469,7 +26491,7 @@
         </is>
       </c>
       <c r="E64" s="33" t="n">
-        <v>47.78</v>
+        <v>52.28</v>
       </c>
       <c r="F64" s="34" t="inlineStr">
         <is>
@@ -26477,7 +26499,7 @@
         </is>
       </c>
       <c r="G64" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H64" s="34" t="inlineStr">
         <is>
@@ -26485,7 +26507,7 @@
         </is>
       </c>
       <c r="I64" t="n">
-        <v>47.779999</v>
+        <v>52.279999</v>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1" s="58">
@@ -26509,7 +26531,7 @@
         </is>
       </c>
       <c r="E65" s="33" t="n">
-        <v>205.08</v>
+        <v>219.2</v>
       </c>
       <c r="F65" s="34" t="inlineStr">
         <is>
@@ -26517,7 +26539,7 @@
         </is>
       </c>
       <c r="G65" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H65" s="34" t="inlineStr">
         <is>
@@ -26525,7 +26547,7 @@
         </is>
       </c>
       <c r="I65" t="n">
-        <v>205.080002</v>
+        <v>219.199997</v>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1" s="58">
@@ -26549,7 +26571,7 @@
         </is>
       </c>
       <c r="E66" s="33" t="n">
-        <v>144.14</v>
+        <v>144.73</v>
       </c>
       <c r="F66" s="34" t="inlineStr">
         <is>
@@ -26557,7 +26579,7 @@
         </is>
       </c>
       <c r="G66" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H66" s="34" t="inlineStr">
         <is>
@@ -26565,7 +26587,7 @@
         </is>
       </c>
       <c r="I66" t="n">
-        <v>144.139999</v>
+        <v>144.729996</v>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1" s="58">
@@ -26589,7 +26611,7 @@
         </is>
       </c>
       <c r="E67" s="33" t="n">
-        <v>133.58</v>
+        <v>127.49</v>
       </c>
       <c r="F67" s="34" t="inlineStr">
         <is>
@@ -26597,7 +26619,7 @@
         </is>
       </c>
       <c r="G67" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H67" s="34" t="inlineStr">
         <is>
@@ -26605,7 +26627,7 @@
         </is>
       </c>
       <c r="I67" t="n">
-        <v>133.580002</v>
+        <v>127.489998</v>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1" s="58">
@@ -26629,7 +26651,7 @@
         </is>
       </c>
       <c r="E68" s="33" t="n">
-        <v>238.73</v>
+        <v>259.56</v>
       </c>
       <c r="F68" s="34" t="inlineStr">
         <is>
@@ -26637,7 +26659,7 @@
         </is>
       </c>
       <c r="G68" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H68" s="34" t="inlineStr">
         <is>
@@ -26645,7 +26667,7 @@
         </is>
       </c>
       <c r="I68" t="n">
-        <v>238.729996</v>
+        <v>259.559998</v>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="58">
@@ -26669,7 +26691,7 @@
         </is>
       </c>
       <c r="E69" s="33" t="n">
-        <v>1112</v>
+        <v>1098.57</v>
       </c>
       <c r="F69" s="34" t="inlineStr">
         <is>
@@ -26677,7 +26699,7 @@
         </is>
       </c>
       <c r="G69" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H69" s="34" t="inlineStr">
         <is>
@@ -26685,7 +26707,7 @@
         </is>
       </c>
       <c r="I69" t="n">
-        <v>1122.5</v>
+        <v>1098.569946</v>
       </c>
     </row>
     <row r="70" ht="15" customHeight="1" s="58">
@@ -26709,7 +26731,7 @@
         </is>
       </c>
       <c r="E70" s="33" t="n">
-        <v>94.11</v>
+        <v>99.77</v>
       </c>
       <c r="F70" s="34" t="inlineStr">
         <is>
@@ -26717,7 +26739,7 @@
         </is>
       </c>
       <c r="G70" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H70" s="34" t="inlineStr">
         <is>
@@ -26725,7 +26747,7 @@
         </is>
       </c>
       <c r="I70" t="n">
-        <v>94.110001</v>
+        <v>99.769997</v>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1" s="58">
@@ -26749,7 +26771,7 @@
         </is>
       </c>
       <c r="E71" s="33" t="n">
-        <v>1448.21</v>
+        <v>1563.7</v>
       </c>
       <c r="F71" s="34" t="inlineStr">
         <is>
@@ -26757,7 +26779,7 @@
         </is>
       </c>
       <c r="G71" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H71" s="34" t="inlineStr">
         <is>
@@ -26765,7 +26787,7 @@
         </is>
       </c>
       <c r="I71" t="n">
-        <v>1448.209961</v>
+        <v>1563.699951</v>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1" s="58">
@@ -26789,7 +26811,7 @@
         </is>
       </c>
       <c r="E72" s="33" t="n">
-        <v>106.96</v>
+        <v>108.44</v>
       </c>
       <c r="F72" s="34" t="inlineStr">
         <is>
@@ -26797,7 +26819,7 @@
         </is>
       </c>
       <c r="G72" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H72" s="34" t="inlineStr">
         <is>
@@ -26805,7 +26827,7 @@
         </is>
       </c>
       <c r="I72" t="n">
-        <v>106.959999</v>
+        <v>108.440002</v>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1" s="58">
@@ -26829,7 +26851,7 @@
         </is>
       </c>
       <c r="E73" s="33" t="n">
-        <v>204.65</v>
+        <v>210.69</v>
       </c>
       <c r="F73" s="34" t="inlineStr">
         <is>
@@ -26837,7 +26859,7 @@
         </is>
       </c>
       <c r="G73" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H73" s="34" t="inlineStr">
         <is>
@@ -26845,7 +26867,7 @@
         </is>
       </c>
       <c r="I73" t="n">
-        <v>204.649994</v>
+        <v>210.690002</v>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1" s="58">
@@ -26869,7 +26891,7 @@
         </is>
       </c>
       <c r="E74" s="33" t="n">
-        <v>84.52</v>
+        <v>88.94</v>
       </c>
       <c r="F74" s="34" t="inlineStr">
         <is>
@@ -26877,7 +26899,7 @@
         </is>
       </c>
       <c r="G74" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H74" s="34" t="inlineStr">
         <is>
@@ -26885,7 +26907,7 @@
         </is>
       </c>
       <c r="I74" t="n">
-        <v>84.519997</v>
+        <v>88.94000200000001</v>
       </c>
     </row>
     <row r="75" ht="15" customHeight="1" s="58">
@@ -26909,7 +26931,7 @@
         </is>
       </c>
       <c r="E75" s="33" t="n">
-        <v>94.65000000000001</v>
+        <v>98.42</v>
       </c>
       <c r="F75" s="34" t="inlineStr">
         <is>
@@ -26917,7 +26939,7 @@
         </is>
       </c>
       <c r="G75" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H75" s="34" t="inlineStr">
         <is>
@@ -26925,7 +26947,7 @@
         </is>
       </c>
       <c r="I75" t="n">
-        <v>94.650002</v>
+        <v>98.41999800000001</v>
       </c>
     </row>
     <row r="76" ht="15" customHeight="1" s="58">
@@ -26949,7 +26971,7 @@
         </is>
       </c>
       <c r="E76" s="33" t="n">
-        <v>408.56</v>
+        <v>437.92</v>
       </c>
       <c r="F76" s="34" t="inlineStr">
         <is>
@@ -26957,7 +26979,7 @@
         </is>
       </c>
       <c r="G76" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H76" s="34" t="inlineStr">
         <is>
@@ -26965,7 +26987,7 @@
         </is>
       </c>
       <c r="I76" t="n">
-        <v>408.559998</v>
+        <v>437.920013</v>
       </c>
     </row>
     <row r="77" ht="15" customHeight="1" s="58">
@@ -26989,7 +27011,7 @@
         </is>
       </c>
       <c r="E77" s="33" t="n">
-        <v>396.38</v>
+        <v>400.49</v>
       </c>
       <c r="F77" s="34" t="inlineStr">
         <is>
@@ -26997,7 +27019,7 @@
         </is>
       </c>
       <c r="G77" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H77" s="34" t="inlineStr">
         <is>
@@ -27005,7 +27027,7 @@
         </is>
       </c>
       <c r="I77" t="n">
-        <v>396.380005</v>
+        <v>400.48999</v>
       </c>
     </row>
     <row r="78" ht="15" customHeight="1" s="58">
@@ -27029,7 +27051,7 @@
         </is>
       </c>
       <c r="E78" s="33" t="n">
-        <v>50.77</v>
+        <v>51.45</v>
       </c>
       <c r="F78" s="34" t="inlineStr">
         <is>
@@ -27037,7 +27059,7 @@
         </is>
       </c>
       <c r="G78" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H78" s="34" t="inlineStr">
         <is>
@@ -27045,7 +27067,7 @@
         </is>
       </c>
       <c r="I78" t="n">
-        <v>50.77</v>
+        <v>51.450001</v>
       </c>
     </row>
     <row r="79" ht="15" customHeight="1" s="58">
@@ -27069,7 +27091,7 @@
         </is>
       </c>
       <c r="E79" s="33" t="n">
-        <v>96.04000000000001</v>
+        <v>95.55</v>
       </c>
       <c r="F79" s="34" t="inlineStr">
         <is>
@@ -27077,7 +27099,7 @@
         </is>
       </c>
       <c r="G79" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H79" s="34" t="inlineStr">
         <is>
@@ -27085,7 +27107,7 @@
         </is>
       </c>
       <c r="I79" t="n">
-        <v>96.040001</v>
+        <v>95.550003</v>
       </c>
     </row>
     <row r="80" ht="15" customHeight="1" s="58">
@@ -27109,7 +27131,7 @@
         </is>
       </c>
       <c r="E80" s="33" t="n">
-        <v>295.95</v>
+        <v>298.01</v>
       </c>
       <c r="F80" s="34" t="inlineStr">
         <is>
@@ -27117,7 +27139,7 @@
         </is>
       </c>
       <c r="G80" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H80" s="34" t="inlineStr">
         <is>
@@ -27125,7 +27147,7 @@
         </is>
       </c>
       <c r="I80" t="n">
-        <v>295.950012</v>
+        <v>298.01001</v>
       </c>
     </row>
     <row r="81" ht="15" customHeight="1" s="58">
@@ -27149,7 +27171,7 @@
         </is>
       </c>
       <c r="E81" s="33" t="n">
-        <v>164.915</v>
+        <v>163.26</v>
       </c>
       <c r="F81" s="34" t="inlineStr">
         <is>
@@ -27157,7 +27179,7 @@
         </is>
       </c>
       <c r="G81" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H81" s="34" t="inlineStr">
         <is>
@@ -27165,7 +27187,7 @@
         </is>
       </c>
       <c r="I81" t="n">
-        <v>164.914993</v>
+        <v>163.259995</v>
       </c>
     </row>
     <row r="82" ht="15" customHeight="1" s="58">
@@ -27189,7 +27211,7 @@
         </is>
       </c>
       <c r="E82" s="33" t="n">
-        <v>567.58</v>
+        <v>577.22</v>
       </c>
       <c r="F82" s="34" t="inlineStr">
         <is>
@@ -27197,7 +27219,7 @@
         </is>
       </c>
       <c r="G82" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H82" s="34" t="inlineStr">
         <is>
@@ -27205,7 +27227,7 @@
         </is>
       </c>
       <c r="I82" t="n">
-        <v>567.580017</v>
+        <v>577.219971</v>
       </c>
     </row>
     <row r="83" ht="15" customHeight="1" s="58">
@@ -27229,7 +27251,7 @@
         </is>
       </c>
       <c r="E83" s="33" t="n">
-        <v>99.16</v>
+        <v>100.51</v>
       </c>
       <c r="F83" s="34" t="inlineStr">
         <is>
@@ -27237,7 +27259,7 @@
         </is>
       </c>
       <c r="G83" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H83" s="34" t="inlineStr">
         <is>
@@ -27245,7 +27267,7 @@
         </is>
       </c>
       <c r="I83" t="n">
-        <v>99.160004</v>
+        <v>100.510002</v>
       </c>
     </row>
     <row r="84" ht="15" customHeight="1" s="58">
@@ -27269,7 +27291,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>74.20999999999999</v>
+        <v>75.47</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -27277,7 +27299,7 @@
         </is>
       </c>
       <c r="G84" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H84" s="34" t="inlineStr">
         <is>
@@ -27285,7 +27307,7 @@
         </is>
       </c>
       <c r="I84" t="n">
-        <v>76.154329</v>
+        <v>74.212987</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="58">
@@ -27309,7 +27331,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>602.73</v>
+        <v>580.45</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -27317,7 +27339,7 @@
         </is>
       </c>
       <c r="G85" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H85" s="34" t="inlineStr">
         <is>
@@ -27325,7 +27347,7 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>603.383287</v>
+        <v>602.725129</v>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="58">
@@ -27349,7 +27371,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>64619</v>
+        <v>62889</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -27357,7 +27379,7 @@
         </is>
       </c>
       <c r="G86" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H86" s="34" t="inlineStr">
         <is>
@@ -27365,7 +27387,7 @@
         </is>
       </c>
       <c r="I86" t="n">
-        <v>65537.478196</v>
+        <v>64619.242742</v>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="58">
@@ -27389,7 +27411,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.006961</v>
+        <v>0.006755</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -27397,7 +27419,7 @@
         </is>
       </c>
       <c r="G87" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H87" s="34" t="inlineStr">
         <is>
@@ -27405,7 +27427,7 @@
         </is>
       </c>
       <c r="I87" t="n">
-        <v>0.007156</v>
+        <v>0.006964</v>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="58">
@@ -27429,23 +27451,23 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
+        <v>0.01164</v>
+      </c>
+      <c r="F88" s="34" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G88" s="28" t="n">
+        <v>46192</v>
+      </c>
+      <c r="H88" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I88" t="n">
         <v>0.011333</v>
-      </c>
-      <c r="F88" s="34" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="G88" s="28" t="n">
-        <v>46191</v>
-      </c>
-      <c r="H88" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I88" t="n">
-        <v>0.0113</v>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="58">
@@ -27469,7 +27491,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>72.34999999999999</v>
+        <v>69.76000000000001</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -27477,7 +27499,7 @@
         </is>
       </c>
       <c r="G89" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H89" s="34" t="inlineStr">
         <is>
@@ -27485,7 +27507,7 @@
         </is>
       </c>
       <c r="I89" t="n">
-        <v>73.334495</v>
+        <v>72.355187</v>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="58">
@@ -27509,7 +27531,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>1.92</v>
+        <v>1.89</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -27517,7 +27539,7 @@
         </is>
       </c>
       <c r="G90" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H90" s="34" t="inlineStr">
         <is>
@@ -27525,7 +27547,7 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>1.89794</v>
+        <v>1.924387</v>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="58">
@@ -27557,7 +27579,7 @@
         </is>
       </c>
       <c r="G91" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H91" s="34" t="inlineStr">
         <is>
@@ -27589,7 +27611,7 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
-        <v>0.017602</v>
+        <v>0.01715</v>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
@@ -27597,7 +27619,7 @@
         </is>
       </c>
       <c r="G92" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H92" s="34" t="inlineStr">
         <is>
@@ -27605,7 +27627,7 @@
         </is>
       </c>
       <c r="I92" t="n">
-        <v>0.018237</v>
+        <v>0.017605</v>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="58">
@@ -27629,7 +27651,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>2.843913</v>
+        <v>2.811234</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -27637,7 +27659,7 @@
         </is>
       </c>
       <c r="G93" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H93" s="34" t="inlineStr">
         <is>
@@ -27645,7 +27667,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>2.809242</v>
+        <v>2.854145</v>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="58">
@@ -27669,7 +27691,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>25.132142</v>
+        <v>23.876143</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -27677,7 +27699,7 @@
         </is>
       </c>
       <c r="G94" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H94" s="34" t="inlineStr">
         <is>
@@ -27685,7 +27707,7 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>26.172029</v>
+        <v>25.210324</v>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="58">
@@ -27709,7 +27731,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.114241</v>
+        <v>0.114188</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -27717,7 +27739,7 @@
         </is>
       </c>
       <c r="G95" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H95" s="34" t="inlineStr">
         <is>
@@ -27725,7 +27747,7 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>0.113777</v>
+        <v>0.114627</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="58">
@@ -27749,7 +27771,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>19679.1345</v>
+        <v>19015.542</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -27757,7 +27779,7 @@
         </is>
       </c>
       <c r="G96" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H96" s="34" t="inlineStr">
         <is>
@@ -27765,7 +27787,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>19700.464318</v>
+        <v>19745.275231</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="58">
@@ -27789,7 +27811,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2109810.35</v>
+        <v>2060243.64</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -27797,7 +27819,7 @@
         </is>
       </c>
       <c r="G97" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H97" s="34" t="inlineStr">
         <is>
@@ -27805,7 +27827,7 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>2139798.663086</v>
+        <v>2116926.392244</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="58">
@@ -27829,7 +27851,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>2.814691</v>
+        <v>2.740374</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -27837,7 +27859,7 @@
         </is>
       </c>
       <c r="G98" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H98" s="34" t="inlineStr">
         <is>
@@ -27845,7 +27867,7 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>2.842868</v>
+        <v>2.824329</v>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="58">
@@ -27869,7 +27891,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>57329.8085</v>
+        <v>56000.5992</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -27877,7 +27899,7 @@
         </is>
       </c>
       <c r="G99" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H99" s="34" t="inlineStr">
         <is>
@@ -27885,7 +27907,7 @@
         </is>
       </c>
       <c r="I99" t="n">
-        <v>58191.597022</v>
+        <v>57523.137774</v>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="58">
@@ -27909,7 +27931,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>25.028217</v>
+        <v>24.804398</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -27917,7 +27939,7 @@
         </is>
       </c>
       <c r="G100" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H100" s="34" t="inlineStr">
         <is>
@@ -27925,7 +27947,7 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>25.153691</v>
+        <v>25.109343</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="58">
@@ -27949,7 +27971,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>64619</v>
+        <v>62889</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -27957,7 +27979,7 @@
         </is>
       </c>
       <c r="G101" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H101" s="34" t="inlineStr">
         <is>
@@ -27965,7 +27987,7 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>65537.478196</v>
+        <v>64619.242742</v>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="58">
@@ -27989,7 +28011,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>17.59</v>
+        <v>17.57</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -27997,7 +28019,7 @@
         </is>
       </c>
       <c r="G102" s="28" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="H102" s="34" t="inlineStr">
         <is>
@@ -28005,7 +28027,7 @@
         </is>
       </c>
       <c r="I102" t="n">
-        <v>17.79